<commit_message>
Datos al 2 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F3AD4DB-2D23-4CB2-82BF-97CC77E2AD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACA9261C-7B40-43B0-8EF8-B29D6E9EDEB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="767" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="202">
   <si>
     <t>Fecha</t>
   </si>
@@ -129,9 +129,6 @@
     <t>Marfeca</t>
   </si>
   <si>
-    <t>Cintillo</t>
-  </si>
-  <si>
     <t>SEPH</t>
   </si>
   <si>
@@ -306,312 +303,21 @@
     <t>Detención</t>
   </si>
   <si>
-    <t>Regidor</t>
-  </si>
-  <si>
-    <t>Reforma Electoral</t>
-  </si>
-  <si>
-    <t>Entrega De Apoyos</t>
-  </si>
-  <si>
-    <t>Atracción De Inversiones</t>
-  </si>
-  <si>
-    <t>Opacidad</t>
-  </si>
-  <si>
-    <t>Violencia Escolar</t>
-  </si>
-  <si>
-    <t>Reunión SMDIF</t>
-  </si>
-  <si>
     <t>Marcha 8M</t>
   </si>
   <si>
     <t>Disturbios</t>
   </si>
   <si>
-    <t>Indicación geográfica</t>
-  </si>
-  <si>
-    <t>Cabildos, donde más cometen violencia política a mujeres</t>
-  </si>
-  <si>
-    <t>Violencia Política De Género</t>
-  </si>
-  <si>
-    <t>Feria Ganadera en Pachuca espera 60 mil visitantes</t>
-  </si>
-  <si>
-    <t>OEEH</t>
-  </si>
-  <si>
-    <t>Expo feria</t>
-  </si>
-  <si>
-    <t>Se invertirán 104 mdp en Tulancingo</t>
-  </si>
-  <si>
     <t>Ruta de la Transformación</t>
   </si>
   <si>
-    <t>No les alcanza para comprar mariscos</t>
-  </si>
-  <si>
-    <t>El misterio en la Cueva del Chivo</t>
-  </si>
-  <si>
-    <t>Pierden su empleo 705 mil personas</t>
-  </si>
-  <si>
-    <t>Tasa de desocupación</t>
-  </si>
-  <si>
-    <t>Colectiva aclara términos básicos antes del 8M</t>
-  </si>
-  <si>
-    <t>IEEH considera viable propuesta de eliminar el PREP</t>
-  </si>
-  <si>
-    <t>Tradición musical</t>
-  </si>
-  <si>
-    <t>Cecultah</t>
-  </si>
-  <si>
-    <t>Concierto Sinfónico</t>
-  </si>
-  <si>
-    <t>Rutas en Metepec y Agua Blanca</t>
-  </si>
-  <si>
-    <t>ACTOPAN BUSCA REGISTRO PARA EL XIMBÓ</t>
-  </si>
-  <si>
-    <t>Cuando en una colonia se abre una zanja, se levanta una calle o se construye obra pública, hay algo que el pueblo sabe bien: esa obra no es del gobierno...</t>
-  </si>
-  <si>
-    <t>Ejecución de obras</t>
-  </si>
-  <si>
-    <t>Suben a 12, casos de sarampión</t>
-  </si>
-  <si>
-    <t>Sarampión</t>
-  </si>
-  <si>
-    <t>Registra el estado 641 llamadas diarias al 911 por violencia de pareja</t>
-  </si>
-  <si>
-    <t>Violencia De Género</t>
-  </si>
-  <si>
-    <t>Rossellini y los límites de la belleza</t>
-  </si>
-  <si>
-    <t>Espectáculos</t>
-  </si>
-  <si>
-    <t>Tuzobús: ven para mayo actualizaciones de unidades</t>
-  </si>
-  <si>
-    <t>Sitmah</t>
-  </si>
-  <si>
-    <t>Modernización Tuzobús</t>
-  </si>
-  <si>
-    <t>Arranca juicio contra uno por el crimen de Rosaura</t>
-  </si>
-  <si>
-    <t>Proceso Por Feminicidio</t>
-  </si>
-  <si>
-    <t>Indagan presunto abuso contra menores en escuela</t>
-  </si>
-  <si>
-    <t>"Somos de carne y hueso", dicen ministros a indígenas</t>
-  </si>
-  <si>
-    <t>Taddei valora el PREP y Claudia descarta negociar las listas VIP</t>
-  </si>
-  <si>
-    <t>París renueva su edificio más feo</t>
-  </si>
-  <si>
-    <t>RENUNCIA EL ABOGADO DEL FEMINICIDA DE ROSAURA</t>
-  </si>
-  <si>
-    <t>Van 69 mil viviendas para 16 municipios</t>
-  </si>
-  <si>
-    <t>Plan Nacional De Vivienda</t>
-  </si>
-  <si>
-    <t>APELA CNDH LAS TARIFAS AVALADAS EN LA CAPITAL POR EL CONGRESO</t>
-  </si>
-  <si>
-    <t>Inconstitucionalidad</t>
-  </si>
-  <si>
-    <t>Celebrarán la primera feria ganadera local</t>
-  </si>
-  <si>
-    <t>La última y nos vamos</t>
-  </si>
-  <si>
-    <t>Aumentaron en 2025 8.25% las picaduras a los ductos</t>
-  </si>
-  <si>
     <t>Huachicol</t>
   </si>
   <si>
-    <t>LOS JOÃO encienden</t>
-  </si>
-  <si>
-    <t>La Jornada Hidalgo</t>
-  </si>
-  <si>
-    <t>Exhiben hidalguenses desprotegidos abandono del consulado de NY</t>
-  </si>
-  <si>
-    <t>Atención A Migrantes</t>
-  </si>
-  <si>
-    <t>Es viable eliminar PREP de elecciones: presidenta del IEEH</t>
-  </si>
-  <si>
-    <t>TV Azteca va a concurso mercantil para pagar deuda</t>
-  </si>
-  <si>
-    <t>Pago de impuestos</t>
-  </si>
-  <si>
-    <t>Esperan 60 mil asistentes a la Expo Ganadera Hidalgo 2026</t>
-  </si>
-  <si>
-    <t>Es innegable que la percepción de inseguridad en la ciudadanía es más fuerte que el discurso oficial (…) Los golpes a los huachicoleros han sido relevantes, pero lo más grave es que esas acciones no inhiben la actuación de los grupos criminales”.</t>
-  </si>
-  <si>
-    <t>Destina gobierno estatal 104 mdp en obras y apoyos para Metepec y Agua Blanca</t>
-  </si>
-  <si>
-    <t>Atrae Pachuca inversión por 120 mdp en infraestructura educativa</t>
-  </si>
-  <si>
-    <t>Habrá rediseño de rutas del Tuzobús con llegada de nuevas unidades: Semot</t>
-  </si>
-  <si>
-    <t>Presentan La Ganadera Hidalgo Expo Feria 2026 en Pachuca</t>
-  </si>
-  <si>
-    <t>Escalan disputas en Ajacuba y mineral de la Reforma</t>
-  </si>
-  <si>
-    <t>Menchaca invierte en Metepec y Agua Blanca 104 millones</t>
-  </si>
-  <si>
-    <t>Gusano barrenador provoca caída de 30% en ventas ganaderas</t>
-  </si>
-  <si>
-    <t>Gusano barrenador</t>
-  </si>
-  <si>
-    <t>Abraham Mendoza</t>
-  </si>
-  <si>
-    <t>Pluris: ¿representación o privilegio?</t>
-  </si>
-  <si>
-    <t>Impulsan autoempleo para madres en Tepeji</t>
-  </si>
-  <si>
-    <t>Impulso a la mujer</t>
-  </si>
-  <si>
-    <t>Abogado de presunto feminicida de Rosaura renuncia durante audiencia</t>
-  </si>
-  <si>
-    <t>Regidora propone zonas de recuperación en bares de Pachuca</t>
-  </si>
-  <si>
-    <t>Vigilancia en bares</t>
-  </si>
-  <si>
-    <t>SSH confirma 2 casos de sarampión en Tula y Tlaxcoapan</t>
-  </si>
-  <si>
-    <t>Trabajar con vocación y transparencia, pide Edda Vita a DIF municipales del Valle del Mezquital</t>
-  </si>
-  <si>
-    <t>Emprenderán acción legal en contra de la persona que originó incendio en el Cerro del Xicuco</t>
-  </si>
-  <si>
-    <t>incendio</t>
-  </si>
-  <si>
-    <t>En Tlaxcoapan realizan plática informativa sobre sarampión</t>
-  </si>
-  <si>
-    <t>DIF de Ajacuba realiza entrega de lentes y apoyo sociales</t>
-  </si>
-  <si>
-    <t>IEEH aprueba plan estratégico institucional</t>
-  </si>
-  <si>
-    <t>¿Tu negocio crece, pero tu contabilidad no te sigue el ritmo?</t>
-  </si>
-  <si>
-    <t>Publicidad</t>
-  </si>
-  <si>
-    <t>Tendrá La Ganadera Hidalgo 2026 cartelera artística, charrería y toros en primera edición</t>
-  </si>
-  <si>
-    <t>Confirman dos casos de sarampión en la entidad</t>
-  </si>
-  <si>
-    <t>Habrá cierre en tramo de la glorieta 24 Horas de viernes a lunes por obras</t>
-  </si>
-  <si>
-    <t>Glorieta 24 Horas</t>
-  </si>
-  <si>
-    <t>Julio Menchaca transforma Metepec y Agua Blanca con más de 104 millones de pesos</t>
-  </si>
-  <si>
-    <t>Aseguran a sujeto por presuntos tocamientos a menor en Pachuca</t>
-  </si>
-  <si>
-    <t>Hidalgo registra la mayor reducción nacional en desempleo</t>
-  </si>
-  <si>
-    <t>Detectan dos nuevos casos de sarampión; suman 11 en 2026</t>
-  </si>
-  <si>
-    <t>Aseguradoras reportan el robo de 631 vehículos</t>
-  </si>
-  <si>
-    <t>Piden denunciar a grupos que comparten contenido íntimo</t>
-  </si>
-  <si>
-    <t>Violencia digital</t>
-  </si>
-  <si>
-    <t>Decomisan mil 100 litros de hidrocarburo en Singuilucan</t>
-  </si>
-  <si>
     <t>FGR</t>
   </si>
   <si>
-    <t>Combate Al Huachicol</t>
-  </si>
-  <si>
-    <t>Ahórrese las molestias que sienta por los cierres temporales en la Glorieta 24 Horas de Pachuca, debido a trabajos de pasos peatonales a la altura del Cenhies, tan necesarios para la protección de los habitantes</t>
-  </si>
-  <si>
     <t>Nivel</t>
   </si>
   <si>
@@ -619,6 +325,324 @@
   </si>
   <si>
     <t>PRI</t>
+  </si>
+  <si>
+    <t>Últimos días de rebaja en el pago del predial</t>
+  </si>
+  <si>
+    <t>Predial</t>
+  </si>
+  <si>
+    <t>La colectiva Aquelarre respalda iconoclasia</t>
+  </si>
+  <si>
+    <t>Hallan vestigios arqueológicos en tren a Querétaro</t>
+  </si>
+  <si>
+    <t>INAH</t>
+  </si>
+  <si>
+    <t>Tren México Querétaro</t>
+  </si>
+  <si>
+    <t>Hidalgo con 71.3% de informalidad laboral</t>
+  </si>
+  <si>
+    <t>Informalidad laboral</t>
+  </si>
+  <si>
+    <t>Biden deportó más hidalguenses que Trump</t>
+  </si>
+  <si>
+    <t>Deportaciones</t>
+  </si>
+  <si>
+    <t>AutoFest reúne a miles en Pachuca</t>
+  </si>
+  <si>
+    <t>Mercado Libre alista su expansión en Polo del Bienestar</t>
+  </si>
+  <si>
+    <t>Polos del Bienestar</t>
+  </si>
+  <si>
+    <t>Regresa el calor</t>
+  </si>
+  <si>
+    <t>Busca el PRD Hidalgo ir sin coalición</t>
+  </si>
+  <si>
+    <t>Alianzas Electorales</t>
+  </si>
+  <si>
+    <t>Héroe hidalguense con capa y sotana</t>
+  </si>
+  <si>
+    <t>Inicia registro para Beca Rita Cetina</t>
+  </si>
+  <si>
+    <t>Beca Rita Cetina</t>
+  </si>
+  <si>
+    <t>Cae la pobreza laboral en Hidalgo... y mejora ingreso por ingreso per cápita: Inegi</t>
+  </si>
+  <si>
+    <t>Índice De Pobreza</t>
+  </si>
+  <si>
+    <t>Aúlla en el Zócalo Shakira y 400 mil más mueven las caderas en CDMX</t>
+  </si>
+  <si>
+    <t>Inevitable hacer comparaciones</t>
+  </si>
+  <si>
+    <t>Los accidentes viales dejan 45 víctimas al día</t>
+  </si>
+  <si>
+    <t>Con videovigilancia buscan prevenir desastres</t>
+  </si>
+  <si>
+    <t>Prevención de incendios</t>
+  </si>
+  <si>
+    <t>Francis, Alemania y RU apuntan a Irán</t>
+  </si>
+  <si>
+    <t>Nuevo Poder Judicial en un año</t>
+  </si>
+  <si>
+    <t>Ellas los preferían neardentales</t>
+  </si>
+  <si>
+    <t>Pachuca mejora ingresos y otorga un aumento de sueldo a policías</t>
+  </si>
+  <si>
+    <t>Aumento salarial</t>
+  </si>
+  <si>
+    <t>Denuncias por tortura, en 3 demarcaciones</t>
+  </si>
+  <si>
+    <t>Tortura</t>
+  </si>
+  <si>
+    <t>SUMAN MÁS DE 300 QUERELLAS POR DELITOS DEL FUERO FEDERAL</t>
+  </si>
+  <si>
+    <t>Incidencia Delictiva</t>
+  </si>
+  <si>
+    <t>PERSONAS CON VIH SUFREN DESABASTO DE MEDICAMENTO</t>
+  </si>
+  <si>
+    <t>IMSS</t>
+  </si>
+  <si>
+    <t>Abasto De Medicamentos</t>
+  </si>
+  <si>
+    <t>Hidalgo, quinto lugar en robo de gas LP: Igavim</t>
+  </si>
+  <si>
+    <t>SALOMÓN, REY BLANQUIAZUL</t>
+  </si>
+  <si>
+    <t>EXHORTAN A ACLARAR TARIFAS DE LOS TAXIS</t>
+  </si>
+  <si>
+    <t>Aumento Tarifa De Transporte</t>
+  </si>
+  <si>
+    <t>ARSENAL SUEÑA CON LA PREMIER</t>
+  </si>
+  <si>
+    <t>Sheinbaum alcanza aprobación de 76.8% en febrero: encuesta</t>
+  </si>
+  <si>
+    <t>Aprobación Sheinbaum</t>
+  </si>
+  <si>
+    <t>ASF encuentra anomalías en $750 millones ejercidos por 30 municipios</t>
+  </si>
+  <si>
+    <t>Observaciones ASF</t>
+  </si>
+  <si>
+    <t>Entre el miedo y la presencia militar, Jalisco intenta regresar a la normalidad</t>
+  </si>
+  <si>
+    <t>Respaldo a la presidenta se mantiene en febrero</t>
+  </si>
+  <si>
+    <t>Está por cumplirse un año de la “supuesta” investigación de Ana Karen Parra, de la Comisión de Derechos Humanos de Hidalgo, sin avances. En contraste, cuando el Legislativo solicitó investigar por violencia política al presidente municipal de Epazoyucan, la respuesta fue inmediata”.</t>
+  </si>
+  <si>
+    <t>Exigen destitución de funcionario</t>
+  </si>
+  <si>
+    <t>Rinde frutos disciplina hacendaria con aumento salarial a policías de Pachuca</t>
+  </si>
+  <si>
+    <t>alcald</t>
+  </si>
+  <si>
+    <t>Acercan asesoría jurídica y psicológica a mujeres del estado</t>
+  </si>
+  <si>
+    <t>IHM</t>
+  </si>
+  <si>
+    <t>Registra Mineral de la Reforma 138 incendios desde principios de año</t>
+  </si>
+  <si>
+    <t>Control de incendios</t>
+  </si>
+  <si>
+    <t>Zunoticia</t>
+  </si>
+  <si>
+    <t>Rutas de la Transformación conectan con mujeres en territorio: IHM</t>
+  </si>
+  <si>
+    <t>Impulsa Sipinna acciones para prevenir y erradicar la violencia hacia adolescentes</t>
+  </si>
+  <si>
+    <t>Sipinna</t>
+  </si>
+  <si>
+    <t>Protección del menor</t>
+  </si>
+  <si>
+    <t>"Somos Huasteca" logra convenio para ofrecer tortilla a 20 pesos el kilo</t>
+  </si>
+  <si>
+    <t>Realizaron simulacro de código erio</t>
+  </si>
+  <si>
+    <t>Alcalde brinda audiencias en domingo de Atención Ciudadana</t>
+  </si>
+  <si>
+    <t>Atención a la ciudadanía</t>
+  </si>
+  <si>
+    <t>Partido Verde descarta fuga de alcaldes a Morena</t>
+  </si>
+  <si>
+    <t>Adhesión política</t>
+  </si>
+  <si>
+    <t>Grupo Bimbo promueve amparo contra Huejutla</t>
+  </si>
+  <si>
+    <t>Amparo</t>
+  </si>
+  <si>
+    <t>Más de 3 mil 500 cebaderos respaldan a Menchaca</t>
+  </si>
+  <si>
+    <t>Cebaderos</t>
+  </si>
+  <si>
+    <t>SEIINAC documenta 75 muertes violentas de mujeres en Hidalgo</t>
+  </si>
+  <si>
+    <t>Feminicidio</t>
+  </si>
+  <si>
+    <t>Policías de Pachuca reciben aumento del 15%</t>
+  </si>
+  <si>
+    <t>Medécigo anuncia inversión histórica en espacios públicos</t>
+  </si>
+  <si>
+    <t>Rehabilitación de espacios públicos</t>
+  </si>
+  <si>
+    <t>Sudáfrica en Pachuca: una oportunidad que trasciende el futbol</t>
+  </si>
+  <si>
+    <t>Policías rescatan a joven en riesgo en puente de Pachuca</t>
+  </si>
+  <si>
+    <t>Evitan suicidio</t>
+  </si>
+  <si>
+    <t>Claudia Sandoval toma protesta de nuevos delegados</t>
+  </si>
+  <si>
+    <t>Toma de protesta</t>
+  </si>
+  <si>
+    <t>Jorge Reyes: disciplina financiera que se traduce en inversión y seguridad para la capital</t>
+  </si>
+  <si>
+    <t>Cebaderos del Altiplano hidalguense cierran filas con el gobierno de Julio Menchaca</t>
+  </si>
+  <si>
+    <t>Hidalguenses representando a México conquistan plata en los Panamericanos de El Salvador</t>
+  </si>
+  <si>
+    <t>Inhide</t>
+  </si>
+  <si>
+    <t>Justa Deportiva</t>
+  </si>
+  <si>
+    <t>Zitlaly Zúñiga encabezó las faenas del pueblo en Ajacuba</t>
+  </si>
+  <si>
+    <t>Conmemora la Sección 15 del SNTE el 62 Aniversario de Educación Indígena</t>
+  </si>
+  <si>
+    <t>Conmemoración Aniversario</t>
+  </si>
+  <si>
+    <t>Entre sirenas, lágrimas y aplausos despidieron al paramédico de Cruz Roja</t>
+  </si>
+  <si>
+    <t>Jorge Reyes: Disciplina financiera que se traduce en inversión y seguridad para la capital</t>
+  </si>
+  <si>
+    <t>Financiamiento educativo, motor de desarrollo en Hidalgo</t>
+  </si>
+  <si>
+    <t>Financiamiento educativo</t>
+  </si>
+  <si>
+    <t>Durante marzo, 10% de descuento en el predial</t>
+  </si>
+  <si>
+    <t>Cuatro detenidos por fraude en juegos de azar en Pachuca</t>
+  </si>
+  <si>
+    <t>Rescata SSPH a hombre que estaba en puente de bulevar Colosio</t>
+  </si>
+  <si>
+    <t>Exigen renuncia del delegado de la FGR en Hidalgo</t>
+  </si>
+  <si>
+    <t>Exigen destitución de docente</t>
+  </si>
+  <si>
+    <t>Trump insta a Guardia Revolucionaria iraní a rendirse</t>
+  </si>
+  <si>
+    <t>Temas internacionales</t>
+  </si>
+  <si>
+    <t>Guerra de tiranos e intereses</t>
+  </si>
+  <si>
+    <t>Van contra tarifas excesivas de los taxis</t>
+  </si>
+  <si>
+    <t>Abusos taxistas</t>
+  </si>
+  <si>
+    <t>Presentan el Sistema de Consult de la Eslecciones</t>
+  </si>
+  <si>
+    <t>Sin datos</t>
   </si>
 </sst>
 </file>
@@ -730,7 +754,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -738,6 +762,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -800,8 +828,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J64" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J64" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J66" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J66" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1160,7 +1188,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -1204,18 +1232,18 @@
         <v>8</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
@@ -1227,13 +1255,13 @@
         <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J2" t="s">
         <v>17</v>
@@ -1241,109 +1269,109 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
-      </c>
-      <c r="C3" t="s">
-        <v>101</v>
+        <v>81</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>98</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>103</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s">
-        <v>42</v>
-      </c>
-      <c r="J3" t="s">
-        <v>192</v>
+      <c r="I3" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
-      </c>
-      <c r="C4" t="s">
-        <v>104</v>
+        <v>81</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>99</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>100</v>
       </c>
       <c r="G4" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
-      </c>
-      <c r="I4" t="s">
-        <v>42</v>
-      </c>
-      <c r="J4" t="s">
-        <v>26</v>
+        <v>11</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
-      </c>
-      <c r="C5" t="s">
-        <v>106</v>
+        <v>81</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>71</v>
       </c>
       <c r="G5" t="s">
-        <v>81</v>
+        <v>103</v>
       </c>
       <c r="H5" t="s">
-        <v>11</v>
-      </c>
-      <c r="I5" t="s">
-        <v>10</v>
-      </c>
-      <c r="J5" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
-      </c>
-      <c r="C6" t="s">
-        <v>107</v>
+        <v>81</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>104</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -1355,315 +1383,315 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
-      <c r="I6" t="s">
-        <v>10</v>
-      </c>
-      <c r="J6" t="s">
+      <c r="I6" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J6" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
-      </c>
-      <c r="C7" t="s">
-        <v>108</v>
+        <v>81</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>106</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>109</v>
+        <v>80</v>
       </c>
       <c r="H7" t="s">
-        <v>16</v>
-      </c>
-      <c r="I7" t="s">
-        <v>62</v>
-      </c>
-      <c r="J7" t="s">
-        <v>14</v>
+        <v>11</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B8" t="s">
         <v>82</v>
       </c>
-      <c r="C8" t="s">
-        <v>110</v>
+      <c r="C8" s="7" t="s">
+        <v>107</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="F8" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="G8" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
       </c>
-      <c r="I8" t="s">
-        <v>10</v>
-      </c>
-      <c r="J8" t="s">
-        <v>10</v>
+      <c r="I8" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
-      </c>
-      <c r="C9" t="s">
-        <v>111</v>
+        <v>82</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>109</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>52</v>
+        <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
-      <c r="I9" t="s">
-        <v>10</v>
-      </c>
-      <c r="J9" t="s">
+      <c r="I9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J9" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B10" t="s">
-        <v>83</v>
-      </c>
-      <c r="C10" t="s">
-        <v>112</v>
+        <v>82</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>110</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="F10" t="s">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="G10" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="H10" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" t="s">
-        <v>42</v>
-      </c>
-      <c r="J10" t="s">
-        <v>192</v>
+        <v>11</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B11" t="s">
-        <v>83</v>
-      </c>
-      <c r="C11" t="s">
-        <v>115</v>
+        <v>82</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>112</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>105</v>
+        <v>22</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
-      <c r="I11" t="s">
-        <v>42</v>
-      </c>
-      <c r="J11" t="s">
-        <v>26</v>
+      <c r="I11" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C12" t="s">
-        <v>116</v>
+        <v>82</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>113</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>28</v>
       </c>
       <c r="G12" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
-      <c r="I12" t="s">
-        <v>10</v>
-      </c>
-      <c r="J12" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I12" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B13" t="s">
         <v>83</v>
       </c>
-      <c r="C13" t="s">
-        <v>117</v>
+      <c r="C13" s="7" t="s">
+        <v>115</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="F13" t="s">
-        <v>2</v>
+        <v>71</v>
       </c>
       <c r="G13" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H13" t="s">
-        <v>11</v>
-      </c>
-      <c r="I13" t="s">
-        <v>42</v>
-      </c>
-      <c r="J13" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B14" t="s">
         <v>83</v>
       </c>
-      <c r="C14" t="s">
-        <v>119</v>
+      <c r="C14" s="7" t="s">
+        <v>117</v>
       </c>
       <c r="D14" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
       </c>
-      <c r="I14" t="s">
-        <v>42</v>
-      </c>
-      <c r="J14" t="s">
-        <v>192</v>
+      <c r="I14" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J14" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" t="s">
-        <v>121</v>
+        <v>83</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>118</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>122</v>
+        <v>80</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
-      <c r="I15" t="s">
-        <v>42</v>
-      </c>
-      <c r="J15" t="s">
-        <v>192</v>
+      <c r="I15" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J15" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B16" t="s">
-        <v>84</v>
-      </c>
-      <c r="C16" t="s">
-        <v>123</v>
+        <v>83</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>119</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -1675,126 +1703,126 @@
         <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>124</v>
+        <v>80</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
       </c>
-      <c r="I16" t="s">
-        <v>10</v>
-      </c>
-      <c r="J16" t="s">
+      <c r="I16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J16" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" t="s">
-        <v>125</v>
+        <v>83</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>120</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="F17" t="s">
-        <v>126</v>
+        <v>21</v>
       </c>
       <c r="G17" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
-      <c r="I17" t="s">
-        <v>42</v>
-      </c>
-      <c r="J17" t="s">
-        <v>192</v>
+      <c r="I17" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J17" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B18" t="s">
-        <v>84</v>
-      </c>
-      <c r="C18" t="s">
-        <v>128</v>
+        <v>83</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>122</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>74</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>129</v>
+        <v>80</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
-      <c r="I18" t="s">
-        <v>10</v>
-      </c>
-      <c r="J18" t="s">
+      <c r="I18" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J18" s="8" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
-      </c>
-      <c r="C19" t="s">
-        <v>130</v>
+        <v>83</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>123</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="G19" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="H19" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" t="s">
-        <v>42</v>
-      </c>
-      <c r="J19" t="s">
-        <v>192</v>
+        <v>11</v>
+      </c>
+      <c r="I19" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J19" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" t="s">
-        <v>131</v>
+        <v>83</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>124</v>
       </c>
       <c r="D20" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
         <v>10</v>
@@ -1803,382 +1831,382 @@
         <v>10</v>
       </c>
       <c r="G20" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
-      <c r="I20" t="s">
-        <v>10</v>
-      </c>
-      <c r="J20" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I20" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J20" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C21" t="s">
-        <v>132</v>
+        <v>83</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F21" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G21" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
       <c r="H21" t="s">
-        <v>11</v>
-      </c>
-      <c r="I21" t="s">
-        <v>62</v>
-      </c>
-      <c r="J21" t="s">
-        <v>14</v>
+        <v>27</v>
+      </c>
+      <c r="I21" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J21" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
-      </c>
-      <c r="C22" t="s">
-        <v>133</v>
+        <v>83</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>127</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F22" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G22" t="s">
-        <v>81</v>
+        <v>128</v>
       </c>
       <c r="H22" t="s">
-        <v>11</v>
-      </c>
-      <c r="I22" t="s">
-        <v>10</v>
-      </c>
-      <c r="J22" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J22" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
-      </c>
-      <c r="C23" t="s">
-        <v>134</v>
+        <v>83</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>129</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="G23" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
-      <c r="I23" t="s">
-        <v>10</v>
-      </c>
-      <c r="J23" t="s">
-        <v>10</v>
+      <c r="I23" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J23" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
-      </c>
-      <c r="C24" t="s">
-        <v>135</v>
+        <v>83</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>131</v>
       </c>
       <c r="D24" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E24" t="s">
         <v>14</v>
       </c>
       <c r="F24" t="s">
-        <v>14</v>
+        <v>132</v>
       </c>
       <c r="G24" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="H24" t="s">
-        <v>11</v>
-      </c>
-      <c r="I24" t="s">
-        <v>62</v>
-      </c>
-      <c r="J24" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J24" s="8" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B25" t="s">
-        <v>84</v>
-      </c>
-      <c r="C25" t="s">
-        <v>137</v>
+        <v>83</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>134</v>
       </c>
       <c r="D25" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E25" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="F25" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="G25" t="s">
-        <v>138</v>
+        <v>91</v>
       </c>
       <c r="H25" t="s">
         <v>16</v>
       </c>
-      <c r="I25" t="s">
-        <v>10</v>
-      </c>
-      <c r="J25" t="s">
-        <v>44</v>
+      <c r="I25" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J25" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
-      </c>
-      <c r="C26" t="s">
-        <v>139</v>
+        <v>83</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>135</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>103</v>
+        <v>22</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
-      <c r="I26" t="s">
-        <v>42</v>
-      </c>
-      <c r="J26" t="s">
-        <v>192</v>
+      <c r="I26" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J26" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B27" t="s">
-        <v>84</v>
-      </c>
-      <c r="C27" t="s">
-        <v>140</v>
+        <v>83</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>136</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="F27" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
       <c r="G27" t="s">
-        <v>22</v>
+        <v>137</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
       </c>
-      <c r="I27" t="s">
-        <v>10</v>
-      </c>
-      <c r="J27" t="s">
-        <v>10</v>
+      <c r="I27" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J27" s="8" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B28" t="s">
-        <v>84</v>
-      </c>
-      <c r="C28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>10</v>
+      </c>
+      <c r="F28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J28" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A29" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B29" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+      <c r="E29" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>140</v>
+      </c>
+      <c r="H29" t="s">
+        <v>27</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J29" s="8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A30" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B30" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="D28" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" t="s">
-        <v>18</v>
-      </c>
-      <c r="F28" t="s">
-        <v>18</v>
-      </c>
-      <c r="G28" t="s">
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>17</v>
+      </c>
+      <c r="F30" t="s">
+        <v>17</v>
+      </c>
+      <c r="G30" t="s">
         <v>142</v>
       </c>
-      <c r="H28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" t="s">
-        <v>42</v>
-      </c>
-      <c r="J28" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B29" t="s">
-        <v>84</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="H30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I30" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J30" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A31" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B31" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
-        <v>10</v>
-      </c>
-      <c r="F29" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" t="s">
-        <v>22</v>
-      </c>
-      <c r="H29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I29" t="s">
-        <v>10</v>
-      </c>
-      <c r="J29" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B30" t="s">
-        <v>144</v>
-      </c>
-      <c r="C30" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" t="s">
-        <v>13</v>
-      </c>
-      <c r="E30" t="s">
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
         <v>14</v>
       </c>
-      <c r="F30" t="s">
+      <c r="F31" t="s">
         <v>14</v>
       </c>
-      <c r="G30" t="s">
-        <v>146</v>
-      </c>
-      <c r="H30" t="s">
-        <v>16</v>
-      </c>
-      <c r="I30" t="s">
-        <v>62</v>
-      </c>
-      <c r="J30" t="s">
+      <c r="G31" t="s">
+        <v>89</v>
+      </c>
+      <c r="H31" t="s">
+        <v>11</v>
+      </c>
+      <c r="I31" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J31" s="8" t="s">
         <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B31" t="s">
-        <v>144</v>
-      </c>
-      <c r="C31" t="s">
-        <v>147</v>
-      </c>
-      <c r="D31" t="s">
-        <v>12</v>
-      </c>
-      <c r="E31" t="s">
-        <v>52</v>
-      </c>
-      <c r="F31" t="s">
-        <v>52</v>
-      </c>
-      <c r="G31" t="s">
-        <v>90</v>
-      </c>
-      <c r="H31" t="s">
-        <v>11</v>
-      </c>
-      <c r="I31" t="s">
-        <v>10</v>
-      </c>
-      <c r="J31" t="s">
-        <v>10</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B32" t="s">
+        <v>83</v>
+      </c>
+      <c r="C32" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="C32" t="s">
-        <v>148</v>
-      </c>
       <c r="D32" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E32" t="s">
         <v>14</v>
@@ -2187,123 +2215,123 @@
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
-      <c r="I32" t="s">
-        <v>62</v>
-      </c>
-      <c r="J32" t="s">
+      <c r="I32" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J32" s="8" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
-      </c>
-      <c r="C33" t="s">
-        <v>150</v>
+        <v>83</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>145</v>
       </c>
       <c r="D33" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="F33" t="s">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="G33" t="s">
-        <v>103</v>
+        <v>146</v>
       </c>
       <c r="H33" t="s">
-        <v>11</v>
-      </c>
-      <c r="I33" t="s">
-        <v>42</v>
-      </c>
-      <c r="J33" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+        <v>16</v>
+      </c>
+      <c r="I33" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J33" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B34" t="s">
-        <v>144</v>
-      </c>
-      <c r="C34" t="s">
-        <v>151</v>
+        <v>85</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>147</v>
       </c>
       <c r="D34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F34" t="s">
-        <v>18</v>
+        <v>148</v>
       </c>
       <c r="G34" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="H34" t="s">
-        <v>16</v>
-      </c>
-      <c r="I34" t="s">
-        <v>42</v>
-      </c>
-      <c r="J34" t="s">
-        <v>192</v>
+        <v>27</v>
+      </c>
+      <c r="I34" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J34" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B35" t="s">
-        <v>86</v>
-      </c>
-      <c r="C35" t="s">
-        <v>152</v>
+        <v>85</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>149</v>
       </c>
       <c r="D35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F35" t="s">
-        <v>26</v>
+        <v>150</v>
       </c>
       <c r="G35" t="s">
-        <v>105</v>
+        <v>90</v>
       </c>
       <c r="H35" t="s">
-        <v>27</v>
-      </c>
-      <c r="I35" t="s">
-        <v>42</v>
-      </c>
-      <c r="J35" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="I35" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J35" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B36" t="s">
-        <v>86</v>
-      </c>
-      <c r="C36" t="s">
-        <v>153</v>
+        <v>85</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>151</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
@@ -2312,318 +2340,318 @@
         <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="G36" t="s">
-        <v>92</v>
+        <v>152</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
-      <c r="I36" t="s">
-        <v>41</v>
-      </c>
-      <c r="J36" t="s">
+      <c r="I36" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J36" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
-      </c>
-      <c r="C37" t="s">
+        <v>153</v>
+      </c>
+      <c r="C37" s="7" t="s">
         <v>154</v>
       </c>
       <c r="D37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E37" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="F37" t="s">
-        <v>126</v>
+        <v>150</v>
       </c>
       <c r="G37" t="s">
-        <v>127</v>
+        <v>90</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
-      <c r="I37" t="s">
-        <v>42</v>
-      </c>
-      <c r="J37" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I37" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J37" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B38" t="s">
-        <v>86</v>
-      </c>
-      <c r="C38" t="s">
+        <v>153</v>
+      </c>
+      <c r="C38" s="7" t="s">
         <v>155</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F38" t="s">
-        <v>102</v>
+        <v>156</v>
       </c>
       <c r="G38" t="s">
-        <v>103</v>
+        <v>157</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
       </c>
-      <c r="I38" t="s">
-        <v>42</v>
-      </c>
-      <c r="J38" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="I38" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J38" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B39" t="s">
-        <v>33</v>
-      </c>
-      <c r="C39" t="s">
-        <v>156</v>
+        <v>153</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>158</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F39" t="s">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="G39" t="s">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="H39" t="s">
-        <v>16</v>
-      </c>
-      <c r="I39" t="s">
-        <v>41</v>
-      </c>
-      <c r="J39" t="s">
-        <v>17</v>
+        <v>11</v>
+      </c>
+      <c r="I39" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J39" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B40" t="s">
-        <v>33</v>
-      </c>
-      <c r="C40" t="s">
-        <v>157</v>
+        <v>153</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>159</v>
       </c>
       <c r="D40" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G40" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="H40" t="s">
-        <v>27</v>
-      </c>
-      <c r="I40" t="s">
-        <v>42</v>
-      </c>
-      <c r="J40" t="s">
-        <v>26</v>
+        <v>11</v>
+      </c>
+      <c r="I40" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J40" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B41" t="s">
-        <v>33</v>
-      </c>
-      <c r="C41" t="s">
-        <v>158</v>
+        <v>153</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>160</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>66</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>66</v>
+        <v>86</v>
       </c>
       <c r="G41" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H41" t="s">
-        <v>16</v>
-      </c>
-      <c r="I41" t="s">
-        <v>42</v>
-      </c>
-      <c r="J41" t="s">
-        <v>192</v>
+        <v>11</v>
+      </c>
+      <c r="I41" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J41" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B42" t="s">
-        <v>33</v>
-      </c>
-      <c r="C42" t="s">
-        <v>160</v>
+        <v>32</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>162</v>
       </c>
       <c r="D42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>28</v>
+        <v>64</v>
       </c>
       <c r="F42" t="s">
         <v>2</v>
       </c>
       <c r="G42" t="s">
-        <v>81</v>
+        <v>163</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
-      <c r="I42" t="s">
-        <v>10</v>
-      </c>
-      <c r="J42" t="s">
-        <v>10</v>
+      <c r="I42" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J42" s="8" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B43" t="s">
-        <v>33</v>
-      </c>
-      <c r="C43" t="s">
-        <v>161</v>
+        <v>32</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>164</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F43" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G43" t="s">
-        <v>90</v>
+        <v>165</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
-      <c r="I43" t="s">
-        <v>62</v>
-      </c>
-      <c r="J43" t="s">
-        <v>14</v>
+      <c r="I43" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J43" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B44" t="s">
-        <v>33</v>
-      </c>
-      <c r="C44" t="s">
-        <v>162</v>
+        <v>32</v>
+      </c>
+      <c r="C44" s="7" t="s">
+        <v>166</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G44" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="H44" t="s">
-        <v>27</v>
-      </c>
-      <c r="I44" t="s">
-        <v>41</v>
-      </c>
-      <c r="J44" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="I44" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J44" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B45" t="s">
-        <v>33</v>
-      </c>
-      <c r="C45" t="s">
-        <v>164</v>
+        <v>32</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>168</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="F45" t="s">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="G45" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
-      </c>
-      <c r="I45" t="s">
-        <v>10</v>
-      </c>
-      <c r="J45" t="s">
-        <v>10</v>
+        <v>16</v>
+      </c>
+      <c r="I45" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J45" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B46" t="s">
-        <v>33</v>
-      </c>
-      <c r="C46" t="s">
-        <v>165</v>
+        <v>32</v>
+      </c>
+      <c r="C46" s="7" t="s">
+        <v>170</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
@@ -2632,126 +2660,126 @@
         <v>17</v>
       </c>
       <c r="F46" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="G46" t="s">
-        <v>166</v>
+        <v>126</v>
       </c>
       <c r="H46" t="s">
-        <v>11</v>
-      </c>
-      <c r="I46" t="s">
-        <v>41</v>
-      </c>
-      <c r="J46" t="s">
+        <v>27</v>
+      </c>
+      <c r="I46" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J46" s="8" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B47" t="s">
-        <v>29</v>
-      </c>
-      <c r="C47" t="s">
-        <v>167</v>
+        <v>32</v>
+      </c>
+      <c r="C47" s="7" t="s">
+        <v>171</v>
       </c>
       <c r="D47" t="s">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
-        <v>15</v>
+        <v>86</v>
       </c>
       <c r="G47" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="H47" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" t="s">
-        <v>42</v>
-      </c>
-      <c r="J47" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="I47" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J47" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B48" t="s">
-        <v>29</v>
-      </c>
-      <c r="C48" t="s">
-        <v>168</v>
+        <v>32</v>
+      </c>
+      <c r="C48" s="7" t="s">
+        <v>173</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="F48" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G48" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
       </c>
-      <c r="I48" t="s">
-        <v>42</v>
-      </c>
-      <c r="J48" t="s">
-        <v>192</v>
+      <c r="I48" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J48" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B49" t="s">
         <v>29</v>
       </c>
-      <c r="C49" t="s">
-        <v>169</v>
+      <c r="C49" s="7" t="s">
+        <v>174</v>
       </c>
       <c r="D49" t="s">
         <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F49" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="G49" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
       </c>
-      <c r="I49" t="s">
-        <v>10</v>
-      </c>
-      <c r="J49" t="s">
-        <v>10</v>
+      <c r="I49" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J49" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B50" t="s">
         <v>29</v>
       </c>
-      <c r="C50" t="s">
-        <v>171</v>
+      <c r="C50" s="7" t="s">
+        <v>176</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -2760,30 +2788,30 @@
         <v>17</v>
       </c>
       <c r="F50" t="s">
+        <v>86</v>
+      </c>
+      <c r="G50" t="s">
+        <v>177</v>
+      </c>
+      <c r="H50" t="s">
+        <v>11</v>
+      </c>
+      <c r="I50" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J50" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="G50" t="s">
-        <v>120</v>
-      </c>
-      <c r="H50" t="s">
-        <v>11</v>
-      </c>
-      <c r="I50" t="s">
-        <v>41</v>
-      </c>
-      <c r="J50" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B51" t="s">
         <v>29</v>
       </c>
-      <c r="C51" t="s">
-        <v>172</v>
+      <c r="C51" s="7" t="s">
+        <v>178</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
@@ -2792,435 +2820,499 @@
         <v>17</v>
       </c>
       <c r="F51" t="s">
+        <v>86</v>
+      </c>
+      <c r="G51" t="s">
+        <v>126</v>
+      </c>
+      <c r="H51" t="s">
+        <v>27</v>
+      </c>
+      <c r="I51" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J51" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="G51" t="s">
-        <v>91</v>
-      </c>
-      <c r="H51" t="s">
-        <v>11</v>
-      </c>
-      <c r="I51" t="s">
-        <v>41</v>
-      </c>
-      <c r="J51" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    </row>
+    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B52" t="s">
         <v>29</v>
       </c>
-      <c r="C52" t="s">
-        <v>173</v>
+      <c r="C52" s="7" t="s">
+        <v>179</v>
       </c>
       <c r="D52" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E52" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="F52" t="s">
-        <v>52</v>
+        <v>26</v>
       </c>
       <c r="G52" t="s">
-        <v>90</v>
+        <v>167</v>
       </c>
       <c r="H52" t="s">
-        <v>11</v>
-      </c>
-      <c r="I52" t="s">
-        <v>10</v>
-      </c>
-      <c r="J52" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="I52" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J52" s="8" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B53" t="s">
         <v>29</v>
       </c>
-      <c r="C53" t="s">
-        <v>174</v>
+      <c r="C53" s="7" t="s">
+        <v>180</v>
       </c>
       <c r="D53" t="s">
-        <v>175</v>
+        <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F53" t="s">
-        <v>10</v>
+        <v>181</v>
       </c>
       <c r="G53" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="s">
-        <v>10</v>
-      </c>
-      <c r="J53" t="s">
-        <v>10</v>
+        <v>27</v>
+      </c>
+      <c r="I53" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J53" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B54" t="s">
-        <v>32</v>
-      </c>
-      <c r="C54" t="s">
-        <v>176</v>
+        <v>29</v>
+      </c>
+      <c r="C54" s="7" t="s">
+        <v>183</v>
       </c>
       <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>17</v>
+      </c>
+      <c r="F54" t="s">
+        <v>86</v>
+      </c>
+      <c r="G54" t="s">
+        <v>80</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+      <c r="I54" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J54" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A55" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B55" t="s">
+        <v>29</v>
+      </c>
+      <c r="C55" s="7" t="s">
+        <v>184</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" t="s">
+        <v>10</v>
+      </c>
+      <c r="G55" t="s">
+        <v>185</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J55" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A56" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B56" t="s">
+        <v>29</v>
+      </c>
+      <c r="C56" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>10</v>
+      </c>
+      <c r="G56" t="s">
+        <v>80</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J56" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B57" t="s">
+        <v>31</v>
+      </c>
+      <c r="C57" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D57" t="s">
         <v>13</v>
       </c>
-      <c r="E54" t="s">
-        <v>37</v>
-      </c>
-      <c r="F54" t="s">
-        <v>102</v>
-      </c>
-      <c r="G54" t="s">
-        <v>103</v>
-      </c>
-      <c r="H54" t="s">
-        <v>27</v>
-      </c>
-      <c r="I54" t="s">
-        <v>42</v>
-      </c>
-      <c r="J54" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B55" t="s">
-        <v>32</v>
-      </c>
-      <c r="C55" t="s">
-        <v>177</v>
-      </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>15</v>
-      </c>
-      <c r="F55" t="s">
-        <v>15</v>
-      </c>
-      <c r="G55" t="s">
-        <v>120</v>
-      </c>
-      <c r="H55" t="s">
-        <v>16</v>
-      </c>
-      <c r="I55" t="s">
-        <v>42</v>
-      </c>
-      <c r="J55" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A56" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B56" t="s">
-        <v>32</v>
-      </c>
-      <c r="C56" t="s">
-        <v>178</v>
-      </c>
-      <c r="D56" t="s">
-        <v>12</v>
-      </c>
-      <c r="E56" t="s">
-        <v>85</v>
-      </c>
-      <c r="F56" t="s">
-        <v>85</v>
-      </c>
-      <c r="G56" t="s">
-        <v>179</v>
-      </c>
-      <c r="H56" t="s">
-        <v>16</v>
-      </c>
-      <c r="I56" t="s">
-        <v>42</v>
-      </c>
-      <c r="J56" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A57" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B57" t="s">
-        <v>32</v>
-      </c>
-      <c r="C57" t="s">
-        <v>180</v>
-      </c>
-      <c r="D57" t="s">
-        <v>12</v>
-      </c>
       <c r="E57" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="F57" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="G57" t="s">
-        <v>105</v>
+        <v>126</v>
       </c>
       <c r="H57" t="s">
         <v>27</v>
       </c>
-      <c r="I57" t="s">
-        <v>42</v>
-      </c>
-      <c r="J57" t="s">
-        <v>26</v>
+      <c r="I57" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J57" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B58" t="s">
-        <v>32</v>
-      </c>
-      <c r="C58" t="s">
-        <v>181</v>
+        <v>31</v>
+      </c>
+      <c r="C58" s="7" t="s">
+        <v>188</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="F58" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="G58" t="s">
-        <v>88</v>
+        <v>189</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
       </c>
-      <c r="I58" t="s">
-        <v>41</v>
-      </c>
-      <c r="J58" t="s">
-        <v>17</v>
+      <c r="I58" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J58" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B59" t="s">
-        <v>32</v>
-      </c>
-      <c r="C59" t="s">
-        <v>182</v>
+        <v>31</v>
+      </c>
+      <c r="C59" s="7" t="s">
+        <v>190</v>
       </c>
       <c r="D59" t="s">
         <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="F59" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="G59" t="s">
-        <v>109</v>
+        <v>97</v>
       </c>
       <c r="H59" t="s">
-        <v>27</v>
-      </c>
-      <c r="I59" t="s">
-        <v>42</v>
-      </c>
-      <c r="J59" t="s">
-        <v>192</v>
+        <v>11</v>
+      </c>
+      <c r="I59" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J59" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B60" t="s">
-        <v>38</v>
-      </c>
-      <c r="C60" t="s">
-        <v>183</v>
+        <v>31</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>191</v>
       </c>
       <c r="D60" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F60" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="G60" t="s">
-        <v>120</v>
+        <v>87</v>
       </c>
       <c r="H60" t="s">
-        <v>16</v>
-      </c>
-      <c r="I60" t="s">
-        <v>42</v>
-      </c>
-      <c r="J60" t="s">
+        <v>11</v>
+      </c>
+      <c r="I60" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="J60" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A61" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B61" t="s">
+        <v>31</v>
+      </c>
+      <c r="C61" s="7" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A61" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B61" t="s">
-        <v>38</v>
-      </c>
-      <c r="C61" t="s">
-        <v>184</v>
-      </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F61" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G61" t="s">
-        <v>97</v>
+        <v>175</v>
       </c>
       <c r="H61" t="s">
         <v>11</v>
       </c>
-      <c r="I61" t="s">
-        <v>10</v>
-      </c>
-      <c r="J61" t="s">
-        <v>10</v>
+      <c r="I61" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="J61" s="8" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B62" t="s">
-        <v>38</v>
-      </c>
-      <c r="C62" t="s">
-        <v>185</v>
+        <v>37</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>193</v>
       </c>
       <c r="D62" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E62" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="F62" t="s">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="G62" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
       </c>
-      <c r="I62" t="s">
-        <v>10</v>
-      </c>
-      <c r="J62" t="s">
-        <v>44</v>
+      <c r="I62" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="J62" s="8" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B63" t="s">
-        <v>38</v>
-      </c>
-      <c r="C63" t="s">
-        <v>187</v>
+        <v>37</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>195</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F63" t="s">
-        <v>188</v>
+        <v>10</v>
       </c>
       <c r="G63" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
       </c>
-      <c r="I63" t="s">
-        <v>62</v>
-      </c>
-      <c r="J63" t="s">
-        <v>14</v>
+      <c r="I63" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J63" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
-        <v>46080</v>
+        <v>46083</v>
       </c>
       <c r="B64" t="s">
+        <v>37</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>197</v>
+      </c>
+      <c r="D64" t="s">
         <v>38</v>
       </c>
-      <c r="C64" t="s">
-        <v>190</v>
-      </c>
-      <c r="D64" t="s">
-        <v>39</v>
-      </c>
       <c r="E64" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="F64" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="G64" t="s">
-        <v>179</v>
+        <v>196</v>
       </c>
       <c r="H64" t="s">
-        <v>27</v>
-      </c>
-      <c r="I64" t="s">
-        <v>42</v>
-      </c>
-      <c r="J64" t="s">
-        <v>192</v>
+        <v>16</v>
+      </c>
+      <c r="I64" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J64" s="8" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A65" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B65" t="s">
+        <v>37</v>
+      </c>
+      <c r="C65" s="7" t="s">
+        <v>198</v>
+      </c>
+      <c r="D65" t="s">
+        <v>9</v>
+      </c>
+      <c r="E65" t="s">
+        <v>43</v>
+      </c>
+      <c r="F65" t="s">
+        <v>43</v>
+      </c>
+      <c r="G65" t="s">
+        <v>199</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J65" s="8" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A66" s="5">
+        <v>46083</v>
+      </c>
+      <c r="B66" t="s">
+        <v>37</v>
+      </c>
+      <c r="C66" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
+        <v>10</v>
+      </c>
+      <c r="G66" t="s">
+        <v>80</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="J66" s="8" t="s">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -3248,13 +3340,13 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s">
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>191</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -3262,7 +3354,7 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
         <v>17</v>
@@ -3276,24 +3368,24 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
         <v>20</v>
       </c>
       <c r="E3" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -3301,44 +3393,44 @@
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E7" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -3349,18 +3441,18 @@
         <v>10</v>
       </c>
       <c r="D8" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E8" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
         <v>28</v>
@@ -3371,38 +3463,38 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E10" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" t="s">
         <v>48</v>
       </c>
-      <c r="B11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D11" t="s">
-        <v>49</v>
-      </c>
       <c r="E11" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D12" t="s">
         <v>26</v>
@@ -3416,38 +3508,38 @@
         <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="E13" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s">
         <v>50</v>
       </c>
-      <c r="B14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D14" t="s">
-        <v>51</v>
-      </c>
       <c r="E14" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D15" t="s">
         <v>51</v>
-      </c>
-      <c r="B15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D15" t="s">
-        <v>52</v>
       </c>
       <c r="E15" t="s">
         <v>10</v>
@@ -3455,7 +3547,7 @@
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -3464,29 +3556,29 @@
         <v>19</v>
       </c>
       <c r="E16" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" t="s">
         <v>53</v>
-      </c>
-      <c r="B17" t="s">
-        <v>54</v>
       </c>
       <c r="D17" t="s">
         <v>23</v>
       </c>
       <c r="E17" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
         <v>55</v>
-      </c>
-      <c r="B18" t="s">
-        <v>56</v>
       </c>
       <c r="D18" t="s">
         <v>10</v>
@@ -3500,13 +3592,13 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D19" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E19" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -3514,27 +3606,27 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D20" t="s">
         <v>18</v>
       </c>
       <c r="E20" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E21" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -3553,30 +3645,30 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D23" t="s">
-        <v>193</v>
+        <v>95</v>
       </c>
       <c r="E23" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D24" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E24" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -3584,41 +3676,41 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E25" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D26" t="s">
         <v>25</v>
       </c>
       <c r="E26" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D27" t="s">
         <v>21</v>
       </c>
       <c r="E27" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
@@ -3626,94 +3718,94 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E28" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E29" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E30" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
         <v>15</v>
       </c>
       <c r="E31" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D32" t="s">
         <v>24</v>
       </c>
       <c r="E32" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D33" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E33" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D34" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -3721,13 +3813,13 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D35" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E35" t="s">
         <v>10</v>
@@ -3738,13 +3830,13 @@
         <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E36" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.35">
@@ -3752,38 +3844,38 @@
         <v>21</v>
       </c>
       <c r="B37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D37" t="s">
+        <v>54</v>
+      </c>
+      <c r="E37" t="s">
         <v>55</v>
-      </c>
-      <c r="E37" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D38" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E39" t="s">
         <v>10</v>
@@ -3791,30 +3883,30 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E40" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E41" t="s">
-        <v>192</v>
+        <v>94</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.35">
@@ -3822,10 +3914,10 @@
         <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E42" t="s">
         <v>10</v>
@@ -3836,26 +3928,26 @@
         <v>24</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D43" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E43" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
@@ -3863,7 +3955,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
@@ -3871,15 +3963,15 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B47" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>
@@ -3887,7 +3979,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B49" t="s">
         <v>10</v>
@@ -3895,26 +3987,26 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50" t="s">
         <v>77</v>
-      </c>
-      <c r="B50" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B51" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B52" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Portadas del 3 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C41459A-0FC4-4FC1-996A-03B3A0662D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF466669-4979-41D3-B271-76FC36FE9CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="192">
   <si>
     <t>Fecha</t>
   </si>
@@ -144,9 +144,6 @@
     <t>Policía municipal</t>
   </si>
   <si>
-    <t>Violencia digital</t>
-  </si>
-  <si>
     <t>Semot</t>
   </si>
   <si>
@@ -159,15 +156,9 @@
     <t>OEEH</t>
   </si>
   <si>
-    <t>Expo feria</t>
-  </si>
-  <si>
     <t>Plaza Juárez</t>
   </si>
   <si>
-    <t>Editorial</t>
-  </si>
-  <si>
     <t>Clasificación</t>
   </si>
   <si>
@@ -300,9 +291,6 @@
     <t>El Universal Hidalgo</t>
   </si>
   <si>
-    <t>Sitmah</t>
-  </si>
-  <si>
     <t>Milenio Hidalgo</t>
   </si>
   <si>
@@ -318,298 +306,313 @@
     <t>Alcalde</t>
   </si>
   <si>
-    <t>Ejecución de obras</t>
-  </si>
-  <si>
-    <t>Detención</t>
-  </si>
-  <si>
-    <t>Publicidad</t>
-  </si>
-  <si>
-    <t>Sarampión</t>
-  </si>
-  <si>
-    <t>Plan Nacional De Vivienda</t>
-  </si>
-  <si>
-    <t>Regidor</t>
-  </si>
-  <si>
     <t>Reforma Electoral</t>
   </si>
   <si>
-    <t>Pago de impuestos</t>
-  </si>
-  <si>
-    <t>Entrega De Apoyos</t>
-  </si>
-  <si>
-    <t>Huachicol</t>
-  </si>
-  <si>
-    <t>Combate Al Huachicol</t>
-  </si>
-  <si>
-    <t>Atracción De Inversiones</t>
-  </si>
-  <si>
-    <t>Glorieta 24 Horas</t>
-  </si>
-  <si>
     <t>Opacidad</t>
   </si>
   <si>
-    <t>Violencia Política De Género</t>
-  </si>
-  <si>
-    <t>Vigilancia en bares</t>
-  </si>
-  <si>
-    <t>Violencia De Género</t>
-  </si>
-  <si>
-    <t>Violencia Escolar</t>
-  </si>
-  <si>
-    <t>Reunión SMDIF</t>
-  </si>
-  <si>
-    <t>Marcha 8M</t>
-  </si>
-  <si>
-    <t>FGR</t>
-  </si>
-  <si>
-    <t>Espectáculos</t>
-  </si>
-  <si>
-    <t>Ruta de la Transformación</t>
-  </si>
-  <si>
-    <t>Disturbios</t>
-  </si>
-  <si>
-    <t>Gusano barrenador</t>
-  </si>
-  <si>
-    <t>Modernización Tuzobús</t>
-  </si>
-  <si>
-    <t>Cabildos, donde más cometen violencia política a mujeres</t>
-  </si>
-  <si>
-    <t>Feria Ganadera en Pachuca espera 60 mil visitantes</t>
-  </si>
-  <si>
-    <t>Se invertirán 104 mdp en Tulancingo</t>
-  </si>
-  <si>
-    <t>No les alcanza para comprar mariscos</t>
-  </si>
-  <si>
-    <t>El misterio en la Cueva del Chivo</t>
-  </si>
-  <si>
-    <t>Pierden su empleo 705 mil personas</t>
-  </si>
-  <si>
-    <t>Tasa de desocupación</t>
-  </si>
-  <si>
-    <t>Colectiva aclara términos básicos antes del 8M</t>
-  </si>
-  <si>
-    <t>IEEH considera viable propuesta de eliminar el PREP</t>
-  </si>
-  <si>
-    <t>Tradición musical</t>
-  </si>
-  <si>
-    <t>Cecultah</t>
-  </si>
-  <si>
-    <t>Concierto Sinfónico</t>
-  </si>
-  <si>
-    <t>Rutas en Metepec y Agua Blanca</t>
-  </si>
-  <si>
-    <t>ACTOPAN BUSCA REGISTRO PARA EL XIMBÓ</t>
-  </si>
-  <si>
-    <t>Indicación geográfica</t>
-  </si>
-  <si>
-    <t>Cuando en una colonia se abre una zanja, se levanta una calle o se construye obra pública, hay algo que el pueblo sabe bien: esa obra no es del gobierno...</t>
-  </si>
-  <si>
-    <t>Suben a 12, casos de sarampión</t>
-  </si>
-  <si>
-    <t>Registra el estado 641 llamadas diarias al 911 por violencia de pareja</t>
-  </si>
-  <si>
-    <t>Rossellini y los límites de la belleza</t>
-  </si>
-  <si>
-    <t>Tuzobús: ven para mayo actualizaciones de unidades</t>
-  </si>
-  <si>
-    <t>Arranca juicio contra uno por el crimen de Rosaura</t>
-  </si>
-  <si>
-    <t>Proceso Por Feminicidio</t>
-  </si>
-  <si>
-    <t>Indagan presunto abuso contra menores en escuela</t>
-  </si>
-  <si>
-    <t>"Somos de carne y hueso", dicen ministros a indígenas</t>
-  </si>
-  <si>
-    <t>Taddei valora el PREP y Claudia descarta negociar las listas VIP</t>
-  </si>
-  <si>
-    <t>París renueva su edificio más feo</t>
-  </si>
-  <si>
-    <t>RENUNCIA EL ABOGADO DEL FEMINICIDA  DE ROSAURA</t>
-  </si>
-  <si>
-    <t>Van 69 mil viviendas para 16 municipios</t>
-  </si>
-  <si>
-    <t>APELA CNDH LAS TARIFAS AVALADAS EN LA CAPITAL POR EL CONGRESO</t>
-  </si>
-  <si>
-    <t>Inconstitucionalidad</t>
-  </si>
-  <si>
-    <t>Celebrarán la primera feria  ganadera local</t>
-  </si>
-  <si>
-    <t>La última y nos vamos</t>
-  </si>
-  <si>
-    <t>Aumentaron en 2025 8.25% las picaduras a los ductos</t>
-  </si>
-  <si>
-    <t>LOS JOÃO encienden</t>
-  </si>
-  <si>
-    <t>Exhiben hidalguenses  desprotegidos abandono  del consulado de NY</t>
-  </si>
-  <si>
-    <t>Atención A Migrantes</t>
-  </si>
-  <si>
-    <t>Es viable eliminar PREP  de elecciones:  presidenta  del IEEH</t>
-  </si>
-  <si>
-    <t>TV Azteca va a concurso mercantil para pagar deuda</t>
-  </si>
-  <si>
-    <t>Esperan 60 mil asistentes a la Expo Ganadera Hidalgo 2026</t>
-  </si>
-  <si>
-    <t>Es innegable que la percepción de inseguridad en la ciudadanía es más fuerte que el discurso oficial  (…) Los golpes a los huachicoleros han sido relevantes, pero lo más grave es que esas acciones no  inhiben la actuación de los grupos criminales”.</t>
-  </si>
-  <si>
-    <t>Destina gobierno estatal 104 mdp en obras y apoyos  para Metepec y Agua Blanca</t>
-  </si>
-  <si>
-    <t>Atrae Pachuca inversión por 120  mdp en infraestructura educativa</t>
-  </si>
-  <si>
-    <t>Habrá rediseño de rutas del  Tuzobús con llegada de nuevas  unidades: Semot</t>
-  </si>
-  <si>
-    <t>Presentan La Ganadera Hidalgo  Expo Feria 2026 en Pachuca</t>
-  </si>
-  <si>
-    <t>Escalan disputas en Ajacuba y mineral de la Reforma</t>
-  </si>
-  <si>
-    <t>Menchaca invierte en Metepec y Agua Blanca 104 millones</t>
-  </si>
-  <si>
-    <t>Gusano barrenador provoca caída de 30% en ventas ganaderas</t>
-  </si>
-  <si>
-    <t>Abraham Mendoza</t>
-  </si>
-  <si>
-    <t>Pluris: ¿representación o privilegio?</t>
-  </si>
-  <si>
-    <t>Impulsan autoempleo para madres en Tepeji</t>
-  </si>
-  <si>
-    <t>Impulso a la mujer</t>
-  </si>
-  <si>
-    <t>Abogado de presunto feminicida de Rosaura renuncia durante audiencia</t>
-  </si>
-  <si>
-    <t>Regidora propone zonas de recuperación en bares de Pachuca</t>
-  </si>
-  <si>
-    <t>SSH confirma 2 casos de sarampión en Tula y Tlaxcoapan</t>
-  </si>
-  <si>
-    <t>Trabajar con vocación y transparencia, pide Edda Vita a DIF municipales del Valle del Mezquital</t>
-  </si>
-  <si>
-    <t>Emprenderán acción legal en contra de la persona que originó incendio en el Cerro del Xicuco</t>
-  </si>
-  <si>
-    <t>incendio</t>
-  </si>
-  <si>
-    <t>En Tlaxcoapan realizan plática informativa sobre sarampión</t>
-  </si>
-  <si>
-    <t>DIF de Ajacuba realiza entrega de lentes y apoyo sociales</t>
-  </si>
-  <si>
-    <t>IEEH aprueba plan estratégico institucional</t>
-  </si>
-  <si>
-    <t>¿Tu negocio crece, pero tu contabilidad no te sigue el ritmo?</t>
-  </si>
-  <si>
-    <t>Tendrá La Ganadera Hidalgo 2026 cartelera artística, charrería y toros en primera edición</t>
-  </si>
-  <si>
-    <t>Confirman dos casos de sarampión en la entidad</t>
-  </si>
-  <si>
-    <t>Habrá cierre en tramo de la glorieta 24 Horas de viernes a lunes por obras</t>
-  </si>
-  <si>
-    <t>Julio Menchaca transforma Metepec y Agua Blanca con más de 104 millones de pesos</t>
-  </si>
-  <si>
-    <t>Aseguran a sujeto por presuntos tocamientos a menor en Pachuca</t>
-  </si>
-  <si>
-    <t>Hidalgo registra la mayor reducción nacional en desempleo</t>
-  </si>
-  <si>
-    <t>Detectan dos nuevos casos de sarampión; suman 11 en 2026</t>
-  </si>
-  <si>
-    <t>Aseguradoras reportan el robo de 631 vehículos</t>
-  </si>
-  <si>
-    <t>Piden denunciar a grupos que comparten contenido íntimo</t>
-  </si>
-  <si>
-    <t>Decomisan mil 100 litros de hidrocarburo en Singuilucan</t>
-  </si>
-  <si>
-    <t>Ahórrese las molestias que sienta por los cierres temporales en la Glorieta 24 Horas de Pachuca, debido a trabajos de pasos peatonales a la altura del Cenhies, tan necesarios para la protección de los habitantes</t>
+    <t>Advierten que siguen las brechas de género</t>
+  </si>
+  <si>
+    <t>8m</t>
+  </si>
+  <si>
+    <t>Sepultan a El Mencho</t>
+  </si>
+  <si>
+    <t>El náhuatl la llevó al debate presidencial</t>
+  </si>
+  <si>
+    <t>Fuego simultáneo en cerros de Pachuca</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>Control de incendios</t>
+  </si>
+  <si>
+    <t>Remesas disminuyen al iniciar el presente año</t>
+  </si>
+  <si>
+    <t>Remesas</t>
+  </si>
+  <si>
+    <t>Transportistas en paro laboral por falta de pago</t>
+  </si>
+  <si>
+    <t>Paro laboral</t>
+  </si>
+  <si>
+    <t>Criterio</t>
+  </si>
+  <si>
+    <t>COMPITE SOLO UNA FIRMA POR LA RECOLECCIÓN  DE LA BASURA</t>
+  </si>
+  <si>
+    <t>Disposición de basura</t>
+  </si>
+  <si>
+    <t>Hidalgo, sitio dos nacional en casos por covid: Salud</t>
+  </si>
+  <si>
+    <t>Covid 19</t>
+  </si>
+  <si>
+    <t>Comienza la construcción de viviendas</t>
+  </si>
+  <si>
+    <t>CEVI</t>
+  </si>
+  <si>
+    <t>Huracán Priscilla</t>
+  </si>
+  <si>
+    <t>PRESENCIA EN 16 MUNICIPIOS  DEL NARCOMENUDEO: SESNSP</t>
+  </si>
+  <si>
+    <t>Incidencia Delictiva</t>
+  </si>
+  <si>
+    <t>¡Se prendió el cerro en Pachuca!</t>
+  </si>
+  <si>
+    <t>TUZOS BUSCAN REIVINDICACIÓN</t>
+  </si>
+  <si>
+    <t>VA POR OTRA  NOCHE ÉPICA</t>
+  </si>
+  <si>
+    <t>Sin beneficio predio de 5 mmdp; ni refinería, ni parque ecológico</t>
+  </si>
+  <si>
+    <t>Parque Ecológico Tula</t>
+  </si>
+  <si>
+    <t>Proyecto rechazado en Tula se llevará a cabo en Puebla</t>
+  </si>
+  <si>
+    <t>Requieren traslado más de 1,800 casas de 19 municipios</t>
+  </si>
+  <si>
+    <t>Reubicación de viviendas</t>
+  </si>
+  <si>
+    <t>Contaminación  más fuerte de  presa Endhó se  da en Hidalgo</t>
+  </si>
+  <si>
+    <t>CEAA</t>
+  </si>
+  <si>
+    <t>Presa Endhó</t>
+  </si>
+  <si>
+    <t>Garantizan 8 mmdp para  reparar daños por lluvias</t>
+  </si>
+  <si>
+    <t>Reportan la localización de  11 personas desaparecidas</t>
+  </si>
+  <si>
+    <t>Reunión Gabinete De Seguridad</t>
+  </si>
+  <si>
+    <t>Registra Pachuca 3 incendios forestales simultáneos</t>
+  </si>
+  <si>
+    <t>Elon Musk ya presagia los viajes a marte y vida eterna</t>
+  </si>
+  <si>
+    <t>Irán bloquea el flujo  de petróleo y amenaza  con incendiar buques</t>
+  </si>
+  <si>
+    <t>Temas internacionales</t>
+  </si>
+  <si>
+    <t>Crecen fraudes  en solicitudes  de créditos</t>
+  </si>
+  <si>
+    <t>Incendios provocan evacuaciones y mala calidad del aire</t>
+  </si>
+  <si>
+    <t>Incendios forestales</t>
+  </si>
+  <si>
+    <t>Transportistas  paran obras  del canal Viejo  Requena  por impago</t>
+  </si>
+  <si>
+    <t>EU intensifica operaciones aéreas en el Golfo de México</t>
+  </si>
+  <si>
+    <t>Gastarán 8.1 mil  mdp para reparar  daños de vaguada</t>
+  </si>
+  <si>
+    <t>La popularidad te lleva al cargo, pero no te enseña a gobernar. Y cuando un municipio se pierde, no solo  se pierde territorio, se pierde credibilidad, se pierde militancia, se pierde futuro. Morena gana batallas  electorales, pero no está consolidando hegemonía territorial”.</t>
+  </si>
+  <si>
+    <t>Trabajo partidista</t>
+  </si>
+  <si>
+    <t>Destinan más de 8 mil 115 mdp para reconstrucción tras lluvias  de octubre</t>
+  </si>
+  <si>
+    <t>Afectan tres incendios calidad del  aire en Pachuca</t>
+  </si>
+  <si>
+    <t>Incendios</t>
+  </si>
+  <si>
+    <t>Construirán viviendas de 61.7 metros  cuadrados para damnificados por  vaguada monzónica</t>
+  </si>
+  <si>
+    <t>Localizan a 11 personas con  ficha de búsqueda en Hidalgo</t>
+  </si>
+  <si>
+    <t>Zunoticia</t>
+  </si>
+  <si>
+    <t>Comuneros se manifestaron por falta de energía eléctrica</t>
+  </si>
+  <si>
+    <t>Secretario de Educación visita Huejutla y alcalde anuncia inversión para secundaria</t>
+  </si>
+  <si>
+    <t>Entrega de infraestructura escolar</t>
+  </si>
+  <si>
+    <t>Aumento en el precio del pollo golpea la economía de comerciantes</t>
+  </si>
+  <si>
+    <t>Alta demanda en expedición de fichas en el Cecyteh 17</t>
+  </si>
+  <si>
+    <t>Media superior</t>
+  </si>
+  <si>
+    <t>Preinscripciones</t>
+  </si>
+  <si>
+    <t>Más de 8 mil 115 mdp para reconstrucción de municipios afectados por las lluvias</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo y PT abren nuevo capítulo de negociación</t>
+  </si>
+  <si>
+    <t>Persecución política</t>
+  </si>
+  <si>
+    <t>Tres incendios ahúman Pachuca</t>
+  </si>
+  <si>
+    <t>Dignificar a la Policía es fortalecer a Pachuca</t>
+  </si>
+  <si>
+    <t>Aumento salarial</t>
+  </si>
+  <si>
+    <t>Pachuca lista programa integral de cultura vial</t>
+  </si>
+  <si>
+    <t>Cultura vial</t>
+  </si>
+  <si>
+    <t>Construirán mil 816 casas para familias que viven en zonas de riesgo</t>
+  </si>
+  <si>
+    <t>8 mil 115 millones de pesos para reconstrucción</t>
+  </si>
+  <si>
+    <t>Inicia la entrega de enseres domésticos a damnificados</t>
+  </si>
+  <si>
+    <t>Reconstrucción de caminos durante todo el año: Sheinbaum</t>
+  </si>
+  <si>
+    <t>Bacheo</t>
+  </si>
+  <si>
+    <t>Agilizarán obras y reforzarán seguridad en Pachuca rumbo al Mundial 2026</t>
+  </si>
+  <si>
+    <t>Mundial De Futbol</t>
+  </si>
+  <si>
+    <t>Avanza rehabilitación de carretera</t>
+  </si>
+  <si>
+    <t>Rehabilitación carretera</t>
+  </si>
+  <si>
+    <t>Gabinete de Seguridad atiende búsqueda de personas desaparecidas</t>
+  </si>
+  <si>
+    <t>Pachuca inicia auditoría estatal al ejercicio fiscal 2025</t>
+  </si>
+  <si>
+    <t>Auditorías</t>
+  </si>
+  <si>
+    <t>Destinarán más de 8 mil 115 mdp a la reconstrucción de municipios afectados por las lluvias</t>
+  </si>
+  <si>
+    <t>Incendio de milpa daña propiedad en Bojay</t>
+  </si>
+  <si>
+    <t>Más incendios en cerros de Pachuca; continúan activos</t>
+  </si>
+  <si>
+    <t>Tráfico, por gran crecimiento de la metrópoli de la Bella Airosa: SIpdus</t>
+  </si>
+  <si>
+    <t>Ordenamiento vial</t>
+  </si>
+  <si>
+    <t>Pachuca inicia auditoría estatal al Ejercicio Fiscal 2025</t>
+  </si>
+  <si>
+    <t>Alertan por página fraudulenta de boletos en Hidalgo</t>
+  </si>
+  <si>
+    <t>Alerta De Fraude</t>
+  </si>
+  <si>
+    <t>Más de 8 mil 115 millones de pesos serán destinados a la reconstrucción de municipios afectados por las lluvias</t>
+  </si>
+  <si>
+    <t>Ven diputados necesaria la reforma electoral</t>
+  </si>
+  <si>
+    <t>Incendios ahogan a Pachuca</t>
+  </si>
+  <si>
+    <t>En busca del ciudadano</t>
+  </si>
+  <si>
+    <t>Sancionan a 203 por maltrato a personas</t>
+  </si>
+  <si>
+    <t>Sanción por maltrato</t>
+  </si>
+  <si>
+    <t>Federación dará 71% para reconstrucción</t>
+  </si>
+  <si>
+    <t>SICT</t>
+  </si>
+  <si>
+    <t>Resaltan estrategias de seguridad</t>
+  </si>
+  <si>
+    <t>Inician reconstrucciones en municipios afectados</t>
+  </si>
+  <si>
+    <t>Reportaron cuatro incendios forestales activos en la entidad</t>
+  </si>
+  <si>
+    <t>Regidora denuncia contrato en lo ""oscurito"" con Cervecera Modelo</t>
+  </si>
+  <si>
+    <t>En una semana: Gobierno de Hidalgo localizó a 11 personas desaparecidad</t>
   </si>
 </sst>
 </file>
@@ -778,8 +781,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:I64" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2">
-  <autoFilter ref="A1:I64" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:I68" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2">
+  <autoFilter ref="A1:I68" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="1"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1125,7 +1128,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1168,135 +1171,135 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>120</v>
+        <v>93</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="H4" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B5" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="G5" t="s">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B6" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -1308,7 +1311,7 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
@@ -1320,145 +1323,145 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B7" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>124</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="H7" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>127</v>
+        <v>105</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>15</v>
       </c>
       <c r="G9" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" t="s">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
-      <c r="E10" t="s">
-        <v>37</v>
-      </c>
       <c r="F10" t="s">
-        <v>129</v>
+        <v>108</v>
       </c>
       <c r="G10" t="s">
-        <v>130</v>
+        <v>109</v>
       </c>
       <c r="H10" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>131</v>
+        <v>110</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="G11" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
@@ -1470,175 +1473,175 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B12" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>132</v>
+        <v>112</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>47</v>
+        <v>96</v>
       </c>
       <c r="G12" t="s">
-        <v>133</v>
+        <v>97</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B13" t="s">
+        <v>102</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" t="s">
-        <v>48</v>
-      </c>
-      <c r="F13" t="s">
-        <v>2</v>
-      </c>
-      <c r="G13" t="s">
-        <v>93</v>
-      </c>
-      <c r="H13" t="s">
-        <v>11</v>
-      </c>
-      <c r="I13" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B14" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>135</v>
+        <v>114</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>96</v>
+        <v>22</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B15" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>136</v>
+        <v>115</v>
       </c>
       <c r="D15" t="s">
         <v>13</v>
       </c>
       <c r="E15" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="H15" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B16" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>137</v>
+        <v>117</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F16" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Presidencia de la República</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B17" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="F17" t="s">
-        <v>87</v>
+        <v>108</v>
       </c>
       <c r="G17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
@@ -1648,135 +1651,135 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B18" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>139</v>
+        <v>120</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="F18" t="s">
-        <v>77</v>
+        <v>121</v>
       </c>
       <c r="G18" t="s">
-        <v>140</v>
+        <v>122</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B19" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>141</v>
+        <v>123</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="F19" t="s">
-        <v>31</v>
+        <v>86</v>
       </c>
       <c r="G19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H19" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B20" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>142</v>
+        <v>124</v>
       </c>
       <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>26</v>
+      </c>
+      <c r="F20" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" t="s">
+        <v>125</v>
+      </c>
+      <c r="H20" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B21" t="s">
+        <v>84</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D21" t="s">
         <v>9</v>
       </c>
-      <c r="E20" t="s">
-        <v>10</v>
-      </c>
-      <c r="F20" t="s">
-        <v>10</v>
-      </c>
-      <c r="G20" t="s">
-        <v>84</v>
-      </c>
-      <c r="H20" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B21" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D21" t="s">
-        <v>12</v>
-      </c>
       <c r="E21" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="F21" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B22" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>144</v>
+        <v>127</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
@@ -1788,37 +1791,37 @@
         <v>10</v>
       </c>
       <c r="G22" t="s">
+        <v>81</v>
+      </c>
+      <c r="H22" t="s">
+        <v>11</v>
+      </c>
+      <c r="I22" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B23" t="s">
         <v>84</v>
       </c>
-      <c r="H22" t="s">
-        <v>11</v>
-      </c>
-      <c r="I22" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A23" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B23" t="s">
-        <v>88</v>
-      </c>
       <c r="C23" s="6" t="s">
-        <v>145</v>
+        <v>128</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>77</v>
+        <v>10</v>
       </c>
       <c r="G23" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
@@ -1830,103 +1833,103 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B24" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>146</v>
+        <v>130</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>97</v>
+        <v>81</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B25" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>147</v>
+        <v>131</v>
       </c>
       <c r="D25" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E25" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>148</v>
+        <v>132</v>
       </c>
       <c r="H25" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B26" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>149</v>
+        <v>133</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>40</v>
+        <v>101</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -1938,7 +1941,7 @@
         <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>22</v>
+        <v>129</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
@@ -1950,238 +1953,238 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>151</v>
+        <v>135</v>
       </c>
       <c r="D28" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="F28" t="s">
-        <v>18</v>
+        <v>86</v>
       </c>
       <c r="G28" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="H28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B29" t="s">
+        <v>85</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" t="s">
+        <v>19</v>
+      </c>
+      <c r="G29" t="s">
+        <v>137</v>
+      </c>
+      <c r="H29" t="s">
         <v>16</v>
       </c>
-      <c r="I28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A29" s="5">
-        <v>46080</v>
-      </c>
-      <c r="B29" t="s">
-        <v>88</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
-        <v>10</v>
-      </c>
-      <c r="F29" t="s">
-        <v>10</v>
-      </c>
-      <c r="G29" t="s">
-        <v>22</v>
-      </c>
-      <c r="H29" t="s">
-        <v>11</v>
-      </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Partidos</v>
       </c>
     </row>
     <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B30" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="D30" t="s">
         <v>13</v>
       </c>
       <c r="E30" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="F30" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="G30" t="s">
-        <v>154</v>
+        <v>109</v>
       </c>
       <c r="H30" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B31" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>155</v>
+        <v>139</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="F31" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="G31" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B32" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="F32" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="G32" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="33" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="D33" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="F33" t="s">
-        <v>39</v>
+        <v>26</v>
       </c>
       <c r="G33" t="s">
-        <v>40</v>
+        <v>125</v>
       </c>
       <c r="H33" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B34" t="s">
-        <v>89</v>
+        <v>143</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="D34" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E34" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F34" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G34" t="s">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="H34" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="D35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F35" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G35" t="s">
-        <v>115</v>
+        <v>146</v>
       </c>
       <c r="H35" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2190,55 +2193,55 @@
     </row>
     <row r="36" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B36" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F36" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="G36" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B37" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="F37" t="s">
-        <v>87</v>
+        <v>149</v>
       </c>
       <c r="G37" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
@@ -2250,25 +2253,25 @@
     </row>
     <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B38" t="s">
-        <v>91</v>
+        <v>143</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="F38" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="G38" t="s">
-        <v>40</v>
+        <v>109</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -2278,345 +2281,345 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B39" t="s">
         <v>33</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>163</v>
+        <v>152</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F39" t="s">
-        <v>92</v>
+        <v>2</v>
       </c>
       <c r="G39" t="s">
-        <v>106</v>
+        <v>153</v>
       </c>
       <c r="H39" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B40" t="s">
         <v>33</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="D40" t="s">
         <v>9</v>
       </c>
       <c r="E40" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="F40" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="G40" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="H40" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B41" t="s">
         <v>33</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>69</v>
+        <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>117</v>
+        <v>156</v>
       </c>
       <c r="H41" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B42" t="s">
         <v>33</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F42" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G42" t="s">
-        <v>84</v>
+        <v>158</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Alcaldías</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B43" t="s">
         <v>33</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="F43" t="s">
-        <v>14</v>
+        <v>108</v>
       </c>
       <c r="G43" t="s">
-        <v>99</v>
+        <v>119</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B44" t="s">
         <v>33</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="G44" t="s">
-        <v>169</v>
+        <v>109</v>
       </c>
       <c r="H44" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B45" t="s">
         <v>33</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="F45" t="s">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="G45" t="s">
-        <v>140</v>
+        <v>109</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B46" t="s">
         <v>33</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F46" t="s">
-        <v>98</v>
+        <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>108</v>
+        <v>163</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B47" t="s">
         <v>29</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="D47" t="s">
         <v>30</v>
       </c>
       <c r="E47" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G47" t="s">
-        <v>96</v>
+        <v>165</v>
       </c>
       <c r="H47" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Alcaldías</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B48" t="s">
         <v>29</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>50</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G48" t="s">
-        <v>111</v>
+        <v>167</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="49" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B49" t="s">
         <v>29</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E49" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F49" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G49" t="s">
-        <v>175</v>
+        <v>125</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B50" t="s">
         <v>29</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -2625,10 +2628,10 @@
         <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>17</v>
+        <v>88</v>
       </c>
       <c r="G50" t="s">
-        <v>96</v>
+        <v>170</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
@@ -2640,55 +2643,55 @@
     </row>
     <row r="51" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B51" t="s">
         <v>29</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="F51" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="G51" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B52" t="s">
         <v>29</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
@@ -2700,16 +2703,16 @@
     </row>
     <row r="53" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B53" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>95</v>
+        <v>13</v>
       </c>
       <c r="E53" t="s">
         <v>10</v>
@@ -2718,7 +2721,7 @@
         <v>10</v>
       </c>
       <c r="G53" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
@@ -2730,28 +2733,28 @@
     </row>
     <row r="54" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B54" t="s">
         <v>32</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="D54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="F54" t="s">
-        <v>39</v>
+        <v>86</v>
       </c>
       <c r="G54" t="s">
-        <v>40</v>
+        <v>175</v>
       </c>
       <c r="H54" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2760,88 +2763,88 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B55" t="s">
         <v>32</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D55" t="s">
         <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F55" t="s">
-        <v>15</v>
+        <v>88</v>
       </c>
       <c r="G55" t="s">
-        <v>96</v>
+        <v>170</v>
       </c>
       <c r="H55" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Alcaldías</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B56" t="s">
         <v>32</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>90</v>
+        <v>37</v>
       </c>
       <c r="F56" t="s">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="G56" t="s">
-        <v>105</v>
+        <v>178</v>
       </c>
       <c r="H56" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B57" t="s">
         <v>32</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="F57" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="G57" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="H57" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2850,163 +2853,163 @@
     </row>
     <row r="58" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B58" t="s">
         <v>32</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>184</v>
+        <v>168</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F58" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="G58" t="s">
-        <v>94</v>
+        <v>125</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B59" t="s">
-        <v>32</v>
+        <v>83</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="D59" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E59" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="F59" t="s">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="G59" t="s">
-        <v>125</v>
+        <v>89</v>
       </c>
       <c r="H59" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B60" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="D60" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E60" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F60" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G60" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H60" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B61" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F61" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G61" t="s">
-        <v>116</v>
+        <v>89</v>
       </c>
       <c r="H61" t="s">
         <v>11</v>
       </c>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Presidencia de la República</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B62" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="D62" t="s">
         <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="F62" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="G62" t="s">
-        <v>35</v>
+        <v>184</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
       </c>
       <c r="I62" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Alcaldías</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B63" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
@@ -3015,10 +3018,10 @@
         <v>14</v>
       </c>
       <c r="F63" t="s">
-        <v>113</v>
+        <v>186</v>
       </c>
       <c r="G63" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
@@ -3028,32 +3031,152 @@
         <v>Presidencia de la República</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
-        <v>46080</v>
+        <v>46084</v>
       </c>
       <c r="B64" t="s">
-        <v>41</v>
+        <v>83</v>
       </c>
       <c r="C64" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D64" t="s">
+        <v>12</v>
+      </c>
+      <c r="E64" t="s">
+        <v>26</v>
+      </c>
+      <c r="F64" t="s">
+        <v>26</v>
+      </c>
+      <c r="G64" t="s">
+        <v>125</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B65" t="s">
+        <v>39</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D65" t="s">
+        <v>13</v>
+      </c>
+      <c r="E65" t="s">
+        <v>86</v>
+      </c>
+      <c r="F65" t="s">
+        <v>86</v>
+      </c>
+      <c r="G65" t="s">
+        <v>109</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B66" t="s">
+        <v>39</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>21</v>
+      </c>
+      <c r="F66" t="s">
+        <v>21</v>
+      </c>
+      <c r="G66" t="s">
+        <v>132</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B67" t="s">
+        <v>39</v>
+      </c>
+      <c r="C67" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="D64" t="s">
-        <v>42</v>
-      </c>
-      <c r="E64" t="s">
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>17</v>
+      </c>
+      <c r="F67" t="s">
+        <v>17</v>
+      </c>
+      <c r="G67" t="s">
         <v>90</v>
       </c>
-      <c r="F64" t="s">
-        <v>90</v>
-      </c>
-      <c r="G64" t="s">
-        <v>105</v>
-      </c>
-      <c r="H64" t="s">
+      <c r="H67" t="s">
+        <v>16</v>
+      </c>
+      <c r="I67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A68" s="5">
+        <v>46084</v>
+      </c>
+      <c r="B68" t="s">
+        <v>39</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" t="s">
+        <v>26</v>
+      </c>
+      <c r="F68" t="s">
+        <v>26</v>
+      </c>
+      <c r="G68" t="s">
+        <v>125</v>
+      </c>
+      <c r="H68" t="s">
         <v>27</v>
       </c>
-      <c r="I64" t="str">
+      <c r="I68" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
@@ -3081,7 +3204,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3089,7 +3212,7 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3097,20 +3220,20 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
@@ -3118,18 +3241,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3142,34 +3265,34 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B9" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B12" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3177,28 +3300,28 @@
         <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -3206,18 +3329,18 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B17" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3225,7 +3348,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3233,15 +3356,15 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3254,18 +3377,18 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B24" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3273,23 +3396,23 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B27" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -3297,63 +3420,63 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B29" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B30" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B31" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B32" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B33" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -3361,7 +3484,7 @@
         <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -3369,15 +3492,15 @@
         <v>21</v>
       </c>
       <c r="B37" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B38" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
@@ -3385,23 +3508,23 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B40" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B41" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3409,7 +3532,7 @@
         <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -3417,20 +3540,20 @@
         <v>24</v>
       </c>
       <c r="B43" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B44" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
@@ -3438,7 +3561,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
@@ -3446,15 +3569,15 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B47" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>
@@ -3462,7 +3585,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B49" t="s">
         <v>10</v>
@@ -3470,26 +3593,26 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B50" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B51" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B52" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reporte 4 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF466669-4979-41D3-B271-76FC36FE9CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09DCCDFF-2B47-402C-80EE-F84796C1EA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="582" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="505" uniqueCount="176">
   <si>
     <t>Fecha</t>
   </si>
@@ -126,12 +126,6 @@
     <t>Delegación</t>
   </si>
   <si>
-    <t>Marfeca</t>
-  </si>
-  <si>
-    <t>Cintillo</t>
-  </si>
-  <si>
     <t>SEPH</t>
   </si>
   <si>
@@ -153,12 +147,6 @@
     <t>Turismo</t>
   </si>
   <si>
-    <t>OEEH</t>
-  </si>
-  <si>
-    <t>Plaza Juárez</t>
-  </si>
-  <si>
     <t>Clasificación</t>
   </si>
   <si>
@@ -309,310 +297,274 @@
     <t>Reforma Electoral</t>
   </si>
   <si>
-    <t>Opacidad</t>
-  </si>
-  <si>
-    <t>Advierten que siguen las brechas de género</t>
-  </si>
-  <si>
     <t>8m</t>
   </si>
   <si>
-    <t>Sepultan a El Mencho</t>
-  </si>
-  <si>
-    <t>El náhuatl la llevó al debate presidencial</t>
-  </si>
-  <si>
-    <t>Fuego simultáneo en cerros de Pachuca</t>
-  </si>
-  <si>
-    <t>PC</t>
-  </si>
-  <si>
     <t>Control de incendios</t>
   </si>
   <si>
-    <t>Remesas disminuyen al iniciar el presente año</t>
-  </si>
-  <si>
-    <t>Remesas</t>
-  </si>
-  <si>
-    <t>Transportistas en paro laboral por falta de pago</t>
-  </si>
-  <si>
-    <t>Paro laboral</t>
-  </si>
-  <si>
     <t>Criterio</t>
   </si>
   <si>
-    <t>COMPITE SOLO UNA FIRMA POR LA RECOLECCIÓN  DE LA BASURA</t>
-  </si>
-  <si>
-    <t>Disposición de basura</t>
-  </si>
-  <si>
-    <t>Hidalgo, sitio dos nacional en casos por covid: Salud</t>
-  </si>
-  <si>
-    <t>Covid 19</t>
-  </si>
-  <si>
-    <t>Comienza la construcción de viviendas</t>
-  </si>
-  <si>
-    <t>CEVI</t>
-  </si>
-  <si>
-    <t>Huracán Priscilla</t>
-  </si>
-  <si>
-    <t>PRESENCIA EN 16 MUNICIPIOS  DEL NARCOMENUDEO: SESNSP</t>
-  </si>
-  <si>
-    <t>Incidencia Delictiva</t>
-  </si>
-  <si>
-    <t>¡Se prendió el cerro en Pachuca!</t>
-  </si>
-  <si>
-    <t>TUZOS BUSCAN REIVINDICACIÓN</t>
-  </si>
-  <si>
-    <t>VA POR OTRA  NOCHE ÉPICA</t>
-  </si>
-  <si>
-    <t>Sin beneficio predio de 5 mmdp; ni refinería, ni parque ecológico</t>
-  </si>
-  <si>
     <t>Parque Ecológico Tula</t>
   </si>
   <si>
-    <t>Proyecto rechazado en Tula se llevará a cabo en Puebla</t>
-  </si>
-  <si>
-    <t>Requieren traslado más de 1,800 casas de 19 municipios</t>
-  </si>
-  <si>
-    <t>Reubicación de viviendas</t>
-  </si>
-  <si>
-    <t>Contaminación  más fuerte de  presa Endhó se  da en Hidalgo</t>
-  </si>
-  <si>
-    <t>CEAA</t>
-  </si>
-  <si>
-    <t>Presa Endhó</t>
-  </si>
-  <si>
-    <t>Garantizan 8 mmdp para  reparar daños por lluvias</t>
-  </si>
-  <si>
-    <t>Reportan la localización de  11 personas desaparecidas</t>
-  </si>
-  <si>
-    <t>Reunión Gabinete De Seguridad</t>
-  </si>
-  <si>
-    <t>Registra Pachuca 3 incendios forestales simultáneos</t>
-  </si>
-  <si>
-    <t>Elon Musk ya presagia los viajes a marte y vida eterna</t>
-  </si>
-  <si>
-    <t>Irán bloquea el flujo  de petróleo y amenaza  con incendiar buques</t>
-  </si>
-  <si>
-    <t>Temas internacionales</t>
-  </si>
-  <si>
-    <t>Crecen fraudes  en solicitudes  de créditos</t>
-  </si>
-  <si>
-    <t>Incendios provocan evacuaciones y mala calidad del aire</t>
-  </si>
-  <si>
     <t>Incendios forestales</t>
   </si>
   <si>
-    <t>Transportistas  paran obras  del canal Viejo  Requena  por impago</t>
-  </si>
-  <si>
-    <t>EU intensifica operaciones aéreas en el Golfo de México</t>
-  </si>
-  <si>
-    <t>Gastarán 8.1 mil  mdp para reparar  daños de vaguada</t>
-  </si>
-  <si>
-    <t>La popularidad te lleva al cargo, pero no te enseña a gobernar. Y cuando un municipio se pierde, no solo  se pierde territorio, se pierde credibilidad, se pierde militancia, se pierde futuro. Morena gana batallas  electorales, pero no está consolidando hegemonía territorial”.</t>
-  </si>
-  <si>
-    <t>Trabajo partidista</t>
-  </si>
-  <si>
-    <t>Destinan más de 8 mil 115 mdp para reconstrucción tras lluvias  de octubre</t>
-  </si>
-  <si>
-    <t>Afectan tres incendios calidad del  aire en Pachuca</t>
-  </si>
-  <si>
-    <t>Incendios</t>
-  </si>
-  <si>
-    <t>Construirán viviendas de 61.7 metros  cuadrados para damnificados por  vaguada monzónica</t>
-  </si>
-  <si>
-    <t>Localizan a 11 personas con  ficha de búsqueda en Hidalgo</t>
-  </si>
-  <si>
     <t>Zunoticia</t>
   </si>
   <si>
-    <t>Comuneros se manifestaron por falta de energía eléctrica</t>
-  </si>
-  <si>
-    <t>Secretario de Educación visita Huejutla y alcalde anuncia inversión para secundaria</t>
-  </si>
-  <si>
-    <t>Entrega de infraestructura escolar</t>
-  </si>
-  <si>
-    <t>Aumento en el precio del pollo golpea la economía de comerciantes</t>
-  </si>
-  <si>
-    <t>Alta demanda en expedición de fichas en el Cecyteh 17</t>
-  </si>
-  <si>
-    <t>Media superior</t>
-  </si>
-  <si>
-    <t>Preinscripciones</t>
-  </si>
-  <si>
-    <t>Más de 8 mil 115 mdp para reconstrucción de municipios afectados por las lluvias</t>
-  </si>
-  <si>
-    <t>Gobierno de Hidalgo y PT abren nuevo capítulo de negociación</t>
-  </si>
-  <si>
-    <t>Persecución política</t>
-  </si>
-  <si>
-    <t>Tres incendios ahúman Pachuca</t>
-  </si>
-  <si>
-    <t>Dignificar a la Policía es fortalecer a Pachuca</t>
-  </si>
-  <si>
-    <t>Aumento salarial</t>
-  </si>
-  <si>
-    <t>Pachuca lista programa integral de cultura vial</t>
-  </si>
-  <si>
-    <t>Cultura vial</t>
-  </si>
-  <si>
-    <t>Construirán mil 816 casas para familias que viven en zonas de riesgo</t>
-  </si>
-  <si>
-    <t>8 mil 115 millones de pesos para reconstrucción</t>
-  </si>
-  <si>
-    <t>Inicia la entrega de enseres domésticos a damnificados</t>
-  </si>
-  <si>
-    <t>Reconstrucción de caminos durante todo el año: Sheinbaum</t>
-  </si>
-  <si>
-    <t>Bacheo</t>
-  </si>
-  <si>
-    <t>Agilizarán obras y reforzarán seguridad en Pachuca rumbo al Mundial 2026</t>
-  </si>
-  <si>
     <t>Mundial De Futbol</t>
   </si>
   <si>
-    <t>Avanza rehabilitación de carretera</t>
-  </si>
-  <si>
-    <t>Rehabilitación carretera</t>
-  </si>
-  <si>
-    <t>Gabinete de Seguridad atiende búsqueda de personas desaparecidas</t>
-  </si>
-  <si>
-    <t>Pachuca inicia auditoría estatal al ejercicio fiscal 2025</t>
-  </si>
-  <si>
-    <t>Auditorías</t>
-  </si>
-  <si>
-    <t>Destinarán más de 8 mil 115 mdp a la reconstrucción de municipios afectados por las lluvias</t>
-  </si>
-  <si>
-    <t>Incendio de milpa daña propiedad en Bojay</t>
-  </si>
-  <si>
-    <t>Más incendios en cerros de Pachuca; continúan activos</t>
-  </si>
-  <si>
-    <t>Tráfico, por gran crecimiento de la metrópoli de la Bella Airosa: SIpdus</t>
-  </si>
-  <si>
-    <t>Ordenamiento vial</t>
-  </si>
-  <si>
-    <t>Pachuca inicia auditoría estatal al Ejercicio Fiscal 2025</t>
-  </si>
-  <si>
-    <t>Alertan por página fraudulenta de boletos en Hidalgo</t>
-  </si>
-  <si>
-    <t>Alerta De Fraude</t>
-  </si>
-  <si>
-    <t>Más de 8 mil 115 millones de pesos serán destinados a la reconstrucción de municipios afectados por las lluvias</t>
-  </si>
-  <si>
-    <t>Ven diputados necesaria la reforma electoral</t>
-  </si>
-  <si>
-    <t>Incendios ahogan a Pachuca</t>
-  </si>
-  <si>
-    <t>En busca del ciudadano</t>
-  </si>
-  <si>
-    <t>Sancionan a 203 por maltrato a personas</t>
-  </si>
-  <si>
-    <t>Sanción por maltrato</t>
-  </si>
-  <si>
-    <t>Federación dará 71% para reconstrucción</t>
-  </si>
-  <si>
-    <t>SICT</t>
-  </si>
-  <si>
-    <t>Resaltan estrategias de seguridad</t>
-  </si>
-  <si>
-    <t>Inician reconstrucciones en municipios afectados</t>
-  </si>
-  <si>
-    <t>Reportaron cuatro incendios forestales activos en la entidad</t>
-  </si>
-  <si>
-    <t>Regidora denuncia contrato en lo ""oscurito"" con Cervecera Modelo</t>
-  </si>
-  <si>
-    <t>En una semana: Gobierno de Hidalgo localizó a 11 personas desaparecidad</t>
+    <t>Sofocan incendio en Cerro Gordo</t>
+  </si>
+  <si>
+    <t>Escala la guerra en Oriente Medio</t>
+  </si>
+  <si>
+    <t>Firman convenio para regular publicidad carretera</t>
+  </si>
+  <si>
+    <t>Ruta de la Transformación</t>
+  </si>
+  <si>
+    <t>Más de 41 mil tienen problemas auditivos</t>
+  </si>
+  <si>
+    <t>Blindarán el Reloj y sede de gobierno</t>
+  </si>
+  <si>
+    <t>Marcha 8M</t>
+  </si>
+  <si>
+    <t>Retiran anuncios publicitarios por contaminación visual</t>
+  </si>
+  <si>
+    <t>Firma De Convenio</t>
+  </si>
+  <si>
+    <t>En México, la historia reciente ha colocado a miles de mujeres en un lugar que jamás imaginaron ocupar: el de buscadoras. Son madres...</t>
+  </si>
+  <si>
+    <t>Personas desaparecidas</t>
+  </si>
+  <si>
+    <t>Huehuetla de fiesta</t>
+  </si>
+  <si>
+    <t>Carnavales</t>
+  </si>
+  <si>
+    <t>Presidenta levanta la Copa Fifa</t>
+  </si>
+  <si>
+    <t>Secretario de Gobierno se reúne con diputados en Congreso de la Unión</t>
+  </si>
+  <si>
+    <t>Reunión con diputados</t>
+  </si>
+  <si>
+    <t>CNDH denuncia cobros excesivos en municipios</t>
+  </si>
+  <si>
+    <t>Ven polo de desarrollo en predio de refinería fallida ubicado en Tula</t>
+  </si>
+  <si>
+    <t>Polos del Bienestar</t>
+  </si>
+  <si>
+    <t>Piden no abandonar vocación ecológica</t>
+  </si>
+  <si>
+    <t>GLPVEM</t>
+  </si>
+  <si>
+    <t>Van 28 mdp para bienestar e igual sustantiva</t>
+  </si>
+  <si>
+    <t>IHM</t>
+  </si>
+  <si>
+    <t>Impulso a la mujer</t>
+  </si>
+  <si>
+    <t>Las familias en precariedad son 7 de cada 10</t>
+  </si>
+  <si>
+    <t>Precariedad laboral</t>
+  </si>
+  <si>
+    <t>Sheinbaum levanta el trofeo con Bebeto</t>
+  </si>
+  <si>
+    <t>Registran alza de 17% en atenciones psicológicas entre los adolescentes</t>
+  </si>
+  <si>
+    <t>Inhjuve</t>
+  </si>
+  <si>
+    <t>atención</t>
+  </si>
+  <si>
+    <t>Hombre hiere a 2 mujeres y luego atenta contra su vida</t>
+  </si>
+  <si>
+    <t>Ataque Armado</t>
+  </si>
+  <si>
+    <t>Introducido hace un cuarto de siglo, el iPod vuelve a entusiasmar</t>
+  </si>
+  <si>
+    <t>Proponen regular servicios de animales de compañía</t>
+  </si>
+  <si>
+    <t>Iniciativa</t>
+  </si>
+  <si>
+    <t>Donald Trump oferta seguros y protección a naves marítimas</t>
+  </si>
+  <si>
+    <t>LA SEMARNATH  PREVÉ MÁS DE 200 INCENDIOS EN LA ENTIDAD</t>
+  </si>
+  <si>
+    <t>Firman convenio para erradicar la publicidad ilegal de la vía pública</t>
+  </si>
+  <si>
+    <t>A CUATRO AÑOS DEL PUENTE ATIRANTADO: POLÉMICA Y CRÍTICAS</t>
+  </si>
+  <si>
+    <t>Puente Atirantado</t>
+  </si>
+  <si>
+    <t>Jóvenes de Pachuca piden más  bibliotecas</t>
+  </si>
+  <si>
+    <t>Bibliotecas</t>
+  </si>
+  <si>
+    <t>¡Están de regreso!</t>
+  </si>
+  <si>
+    <t>INSTALARÁN VALLAS PARA LA MARCHA DEL 8 DE MARZO</t>
+  </si>
+  <si>
+    <t>Sombras y luces del mundial</t>
+  </si>
+  <si>
+    <t>Protegerán patrimonio ante marchas del 8M</t>
+  </si>
+  <si>
+    <t>Sheinbaum alista   entrega final de   reforma electoral</t>
+  </si>
+  <si>
+    <t>Cancela Trump posibilidad de diálogo con Irán</t>
+  </si>
+  <si>
+    <t>Firman convenio para proteger la imagen urbana</t>
+  </si>
+  <si>
+    <t>Salir a marchar y ocupar las calles sigue siendo tan necesario, no estamos cerca de  acabar con la discriminación y violencia. Aún el aborto voluntario sigue siendo un  delito, aún no hay un sistema de cuidados, la violencia sexual persiste, la desigualdad  salarial también y los feminicidios se siguen contabilizando”.</t>
+  </si>
+  <si>
+    <t>Firman convenio la contra contaminación visual; retiran 210 anuncios publicitarios</t>
+  </si>
+  <si>
+    <t>Atentan contra dos mujeres en  Chavarría; presunto agresor se  habría suicidado</t>
+  </si>
+  <si>
+    <t>Pronostican heladas en zonas montañosas y calor en gran parte del estado</t>
+  </si>
+  <si>
+    <t>Conagua</t>
+  </si>
+  <si>
+    <t>Alerta Meteorológica</t>
+  </si>
+  <si>
+    <t>Confirma Menchaca instalación de vallas en el marco del 8M</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo y SICT protegen imagen urbana</t>
+  </si>
+  <si>
+    <t>Paola Rojas en Huejutla el próximo 8 de marzo</t>
+  </si>
+  <si>
+    <t>Inauguran alcalde y presidenta del DIF lactario en registro de lo familiar</t>
+  </si>
+  <si>
+    <t>Iniciaron talleres en el centro cultural regional de la huasteca hidalguense</t>
+  </si>
+  <si>
+    <t>Taller Cultural</t>
+  </si>
+  <si>
+    <t>Develan placa de fundadores de la telesecundaria 65 de Lemontitla</t>
+  </si>
+  <si>
+    <t>CAPASHH mantiene atención a usuarios durante entrega-recepción</t>
+  </si>
+  <si>
+    <t>Agua</t>
+  </si>
+  <si>
+    <t>Atención a la ciudadanía</t>
+  </si>
+  <si>
+    <t>Lorena García, la alcaldesa que más crece en aprobación</t>
+  </si>
+  <si>
+    <t>Aprobación Alcalde</t>
+  </si>
+  <si>
+    <t>Tatiana Ángeles cierra filas con la 4T y manda mensaje a críticos</t>
+  </si>
+  <si>
+    <t>Respaldo gobernador</t>
+  </si>
+  <si>
+    <t>Hidalgo va contra la contaminación visual; retiran 200 anuncios</t>
+  </si>
+  <si>
+    <t>Ayuntamientos: entre recaudar y respetar la ley</t>
+  </si>
+  <si>
+    <t>Recaudación</t>
+  </si>
+  <si>
+    <t>Menchaca reorganiza dependencias; ahorro de 100 millones</t>
+  </si>
+  <si>
+    <t>Arrendamiento</t>
+  </si>
+  <si>
+    <t>Solo cinco partidos dan aguinaldos en Hidalgo</t>
+  </si>
+  <si>
+    <t>Aguinaldos</t>
+  </si>
+  <si>
+    <t>Hallan sin vida a presunto agresor de mujeres en Chavarría</t>
+  </si>
+  <si>
+    <t>Rescatan a perrita tras denuncias por descuido en Pachuca</t>
+  </si>
+  <si>
+    <t>Rescate Animal</t>
+  </si>
+  <si>
+    <t>Tuzos derrotan 2-1 a Necaxa en el estadio Hidalgo</t>
+  </si>
+  <si>
+    <t>Hallan sin vida da hombre que atacó a dos mujeres en Mineral de la Reforma</t>
+  </si>
+  <si>
+    <t>Julio Menchaca impulsa desarrollo y bienestar en Arenal con más de 80 millones de pesos</t>
+  </si>
+  <si>
+    <t>La luna de sangre tiño el cielo de la Bella Airosa</t>
   </si>
 </sst>
 </file>
@@ -1173,46 +1125,46 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B2" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -1221,7 +1173,7 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
@@ -1233,70 +1185,70 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B4" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>81</v>
+        <v>96</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B5" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>98</v>
@@ -1305,10 +1257,10 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G6" t="s">
         <v>99</v>
@@ -1318,27 +1270,27 @@
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F7" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G7" t="s">
         <v>101</v>
@@ -1348,120 +1300,120 @@
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B8" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" t="s">
+        <v>103</v>
+      </c>
+      <c r="H8" t="s">
+        <v>11</v>
+      </c>
+      <c r="I8" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B8" t="s">
-        <v>102</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G8" t="s">
-        <v>104</v>
-      </c>
-      <c r="H8" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="C9" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" t="s">
+        <v>10</v>
+      </c>
+      <c r="G9" t="s">
         <v>105</v>
       </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>106</v>
-      </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B10" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>86</v>
+        <v>14</v>
       </c>
       <c r="F10" t="s">
-        <v>108</v>
+        <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>92</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
@@ -1473,130 +1425,130 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B12" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D12" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>96</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D13" t="s">
+        <v>13</v>
+      </c>
+      <c r="E13" t="s">
+        <v>26</v>
+      </c>
+      <c r="F13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G13" t="s">
+        <v>111</v>
+      </c>
+      <c r="H13" t="s">
+        <v>11</v>
+      </c>
+      <c r="I13" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" t="s">
-        <v>10</v>
-      </c>
-      <c r="F13" t="s">
-        <v>10</v>
-      </c>
-      <c r="G13" t="s">
-        <v>22</v>
-      </c>
-      <c r="H13" t="s">
-        <v>11</v>
-      </c>
-      <c r="I13" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B14" t="s">
-        <v>102</v>
+        <v>80</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F14" t="s">
+        <v>113</v>
+      </c>
+      <c r="G14" t="s">
+        <v>89</v>
+      </c>
+      <c r="H14" t="s">
+        <v>11</v>
+      </c>
+      <c r="I14" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B15" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" t="s">
-        <v>10</v>
-      </c>
-      <c r="F14" t="s">
-        <v>10</v>
-      </c>
-      <c r="G14" t="s">
-        <v>22</v>
-      </c>
-      <c r="H14" t="s">
-        <v>11</v>
-      </c>
-      <c r="I14" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B15" t="s">
-        <v>84</v>
-      </c>
-      <c r="C15" s="6" t="s">
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" t="s">
         <v>115</v>
-      </c>
-      <c r="D15" t="s">
-        <v>13</v>
-      </c>
-      <c r="E15" t="s">
-        <v>14</v>
-      </c>
-      <c r="F15" t="s">
-        <v>14</v>
       </c>
       <c r="G15" t="s">
         <v>116</v>
       </c>
       <c r="H15" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B16" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>117</v>
@@ -1605,58 +1557,58 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" t="s">
+        <v>68</v>
+      </c>
+      <c r="G16" t="s">
+        <v>118</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+      <c r="I16" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" t="s">
+        <v>9</v>
+      </c>
+      <c r="E17" t="s">
         <v>14</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F17" t="s">
         <v>14</v>
       </c>
-      <c r="G16" t="s">
-        <v>116</v>
-      </c>
-      <c r="H16" t="s">
-        <v>11</v>
-      </c>
-      <c r="I16" t="str">
+      <c r="G17" t="s">
+        <v>92</v>
+      </c>
+      <c r="H17" t="s">
+        <v>11</v>
+      </c>
+      <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Presidencia de la República</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B17" t="s">
-        <v>84</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" t="s">
-        <v>86</v>
-      </c>
-      <c r="F17" t="s">
-        <v>108</v>
-      </c>
-      <c r="G17" t="s">
-        <v>119</v>
-      </c>
-      <c r="H17" t="s">
-        <v>11</v>
-      </c>
-      <c r="I17" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B18" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C18" s="6" t="s">
         <v>120</v>
@@ -1665,7 +1617,7 @@
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>86</v>
+        <v>20</v>
       </c>
       <c r="F18" t="s">
         <v>121</v>
@@ -1683,10 +1635,10 @@
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B19" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>123</v>
@@ -1695,91 +1647,91 @@
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>86</v>
+        <v>32</v>
       </c>
       <c r="G19" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="H19" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B20" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G20" t="s">
-        <v>125</v>
+        <v>77</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B21" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>126</v>
       </c>
       <c r="D21" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="F21" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="G21" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B22" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
@@ -1791,7 +1743,7 @@
         <v>10</v>
       </c>
       <c r="G22" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
@@ -1803,40 +1755,40 @@
     </row>
     <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B23" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F23" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="G23" t="s">
-        <v>129</v>
+        <v>90</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B24" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C24" s="6" t="s">
         <v>130</v>
@@ -1845,91 +1797,91 @@
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F24" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G24" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C25" s="6" t="s">
         <v>131</v>
       </c>
       <c r="D25" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E25" t="s">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="F25" t="s">
-        <v>10</v>
+        <v>82</v>
       </c>
       <c r="G25" t="s">
         <v>132</v>
       </c>
       <c r="H25" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C26" s="6" t="s">
         <v>133</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F26" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G26" t="s">
-        <v>101</v>
+        <v>134</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B27" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -1941,7 +1893,7 @@
         <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>129</v>
+        <v>22</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
@@ -1953,25 +1905,25 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B28" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="F28" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="G28" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H28" t="s">
         <v>11</v>
@@ -1981,57 +1933,57 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="29" spans="1:9" ht="90" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B29" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>137</v>
+        <v>22</v>
       </c>
       <c r="H29" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B30" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>138</v>
       </c>
       <c r="D30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="F30" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="G30" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
@@ -2043,76 +1995,76 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>139</v>
       </c>
       <c r="D31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="F31" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="G31" t="s">
+        <v>85</v>
+      </c>
+      <c r="H31" t="s">
+        <v>11</v>
+      </c>
+      <c r="I31" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B32" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="H31" t="s">
-        <v>11</v>
-      </c>
-      <c r="I31" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B32" t="s">
-        <v>87</v>
-      </c>
-      <c r="C32" s="6" t="s">
+      <c r="D32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" t="s">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" t="s">
+        <v>77</v>
+      </c>
+      <c r="H32" t="s">
+        <v>11</v>
+      </c>
+      <c r="I32" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B33" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D32" t="s">
-        <v>12</v>
-      </c>
-      <c r="E32" t="s">
-        <v>86</v>
-      </c>
-      <c r="F32" t="s">
-        <v>86</v>
-      </c>
-      <c r="G32" t="s">
-        <v>109</v>
-      </c>
-      <c r="H32" t="s">
-        <v>11</v>
-      </c>
-      <c r="I32" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B33" t="s">
-        <v>87</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>142</v>
-      </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E33" t="s">
         <v>26</v>
@@ -2121,67 +2073,67 @@
         <v>26</v>
       </c>
       <c r="G33" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="H33" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="34" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" ht="105" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B34" t="s">
-        <v>143</v>
+        <v>81</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="F34" t="s">
-        <v>10</v>
+        <v>46</v>
       </c>
       <c r="G34" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H34" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="35" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B35" t="s">
+        <v>83</v>
+      </c>
+      <c r="C35" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C35" s="6" t="s">
-        <v>145</v>
-      </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F35" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="G35" t="s">
-        <v>146</v>
+        <v>101</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
@@ -2193,85 +2145,85 @@
     </row>
     <row r="36" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B36" t="s">
-        <v>143</v>
+        <v>83</v>
       </c>
       <c r="C36" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" t="s">
+        <v>24</v>
+      </c>
+      <c r="G36" t="s">
+        <v>124</v>
+      </c>
+      <c r="H36" t="s">
+        <v>11</v>
+      </c>
+      <c r="I36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B37" t="s">
+        <v>83</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
+        <v>14</v>
+      </c>
+      <c r="F37" t="s">
+        <v>146</v>
+      </c>
+      <c r="G37" t="s">
         <v>147</v>
       </c>
-      <c r="D36" t="s">
-        <v>12</v>
-      </c>
-      <c r="E36" t="s">
-        <v>10</v>
-      </c>
-      <c r="F36" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" t="s">
-        <v>81</v>
-      </c>
-      <c r="H36" t="s">
-        <v>11</v>
-      </c>
-      <c r="I36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A37" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B37" t="s">
-        <v>143</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="D37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E37" t="s">
-        <v>31</v>
-      </c>
-      <c r="F37" t="s">
-        <v>149</v>
-      </c>
-      <c r="G37" t="s">
-        <v>150</v>
-      </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B38" t="s">
-        <v>143</v>
+        <v>83</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="F38" t="s">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="G38" t="s">
-        <v>109</v>
+        <v>99</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -2281,27 +2233,27 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B39" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F39" t="s">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="G39" t="s">
-        <v>153</v>
+        <v>101</v>
       </c>
       <c r="H39" t="s">
         <v>11</v>
@@ -2313,43 +2265,43 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B40" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D40" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F40" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="G40" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Alcaldías</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B41" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
@@ -2361,25 +2313,25 @@
         <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>156</v>
+        <v>77</v>
       </c>
       <c r="H41" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B42" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
@@ -2391,7 +2343,7 @@
         <v>17</v>
       </c>
       <c r="G42" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
@@ -2403,163 +2355,163 @@
     </row>
     <row r="43" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B43" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>86</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>108</v>
+        <v>10</v>
       </c>
       <c r="G43" t="s">
-        <v>119</v>
+        <v>77</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B44" t="s">
-        <v>33</v>
+        <v>91</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>86</v>
+        <v>156</v>
       </c>
       <c r="G44" t="s">
-        <v>109</v>
+        <v>157</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B45" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F45" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="G45" t="s">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
     </row>
     <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B46" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F46" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G46" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="47" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B47" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="D47" t="s">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="E47" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F47" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G47" t="s">
-        <v>165</v>
+        <v>101</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B48" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
@@ -2571,7 +2523,7 @@
         <v>17</v>
       </c>
       <c r="G48" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
@@ -2583,16 +2535,16 @@
     </row>
     <row r="49" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B49" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E49" t="s">
         <v>26</v>
@@ -2601,10 +2553,10 @@
         <v>26</v>
       </c>
       <c r="G49" t="s">
-        <v>125</v>
+        <v>166</v>
       </c>
       <c r="H49" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2613,55 +2565,55 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B50" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F50" t="s">
-        <v>88</v>
+        <v>10</v>
       </c>
       <c r="G50" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B51" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>86</v>
+        <v>24</v>
       </c>
       <c r="F51" t="s">
-        <v>86</v>
+        <v>24</v>
       </c>
       <c r="G51" t="s">
-        <v>109</v>
+        <v>124</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
@@ -2673,512 +2625,270 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>172</v>
+        <v>149</v>
       </c>
       <c r="D52" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E52" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F52" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G52" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46084</v>
+        <v>46085</v>
       </c>
       <c r="B53" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C53" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>17</v>
+      </c>
+      <c r="F53" t="s">
+        <v>17</v>
+      </c>
+      <c r="G53" t="s">
+        <v>171</v>
+      </c>
+      <c r="H53" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B54" t="s">
+        <v>30</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>10</v>
+      </c>
+      <c r="F54" t="s">
+        <v>10</v>
+      </c>
+      <c r="G54" t="s">
+        <v>22</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+      <c r="I54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B55" t="s">
+        <v>30</v>
+      </c>
+      <c r="C55" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="D53" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" t="s">
-        <v>10</v>
-      </c>
-      <c r="F53" t="s">
-        <v>10</v>
-      </c>
-      <c r="G53" t="s">
-        <v>97</v>
-      </c>
-      <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="str">
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>24</v>
+      </c>
+      <c r="F55" t="s">
+        <v>24</v>
+      </c>
+      <c r="G55" t="s">
+        <v>124</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="A56" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B56" t="s">
+        <v>30</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>26</v>
+      </c>
+      <c r="F56" t="s">
+        <v>26</v>
+      </c>
+      <c r="G56" t="s">
+        <v>96</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A57" s="5">
+        <v>46085</v>
+      </c>
+      <c r="B57" t="s">
+        <v>30</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>10</v>
+      </c>
+      <c r="F57" t="s">
+        <v>10</v>
+      </c>
+      <c r="G57" t="s">
+        <v>77</v>
+      </c>
+      <c r="H57" t="s">
+        <v>11</v>
+      </c>
+      <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A54" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B54" t="s">
-        <v>32</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="D54" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" t="s">
-        <v>86</v>
-      </c>
-      <c r="F54" t="s">
-        <v>86</v>
-      </c>
-      <c r="G54" t="s">
-        <v>175</v>
-      </c>
-      <c r="H54" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A55" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B55" t="s">
-        <v>32</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>17</v>
-      </c>
-      <c r="F55" t="s">
-        <v>88</v>
-      </c>
-      <c r="G55" t="s">
-        <v>170</v>
-      </c>
-      <c r="H55" t="s">
-        <v>11</v>
-      </c>
-      <c r="I55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A56" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B56" t="s">
-        <v>32</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="D56" t="s">
-        <v>12</v>
-      </c>
-      <c r="E56" t="s">
-        <v>37</v>
-      </c>
-      <c r="F56" t="s">
-        <v>38</v>
-      </c>
-      <c r="G56" t="s">
-        <v>178</v>
-      </c>
-      <c r="H56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" ht="45" x14ac:dyDescent="0.25">
-      <c r="A57" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B57" t="s">
-        <v>32</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D57" t="s">
-        <v>12</v>
-      </c>
-      <c r="E57" t="s">
-        <v>86</v>
-      </c>
-      <c r="F57" t="s">
-        <v>86</v>
-      </c>
-      <c r="G57" t="s">
-        <v>109</v>
-      </c>
-      <c r="H57" t="s">
-        <v>11</v>
-      </c>
-      <c r="I57" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B58" t="s">
-        <v>32</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="D58" t="s">
-        <v>12</v>
-      </c>
-      <c r="E58" t="s">
-        <v>26</v>
-      </c>
-      <c r="F58" t="s">
-        <v>26</v>
-      </c>
-      <c r="G58" t="s">
-        <v>125</v>
-      </c>
-      <c r="H58" t="s">
-        <v>11</v>
-      </c>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A58" s="5"/>
+      <c r="C58" s="6"/>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>No indexado</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A59" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B59" t="s">
-        <v>83</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D59" t="s">
-        <v>13</v>
-      </c>
-      <c r="E59" t="s">
-        <v>44</v>
-      </c>
-      <c r="F59" t="s">
-        <v>44</v>
-      </c>
-      <c r="G59" t="s">
-        <v>89</v>
-      </c>
-      <c r="H59" t="s">
-        <v>11</v>
-      </c>
+      <c r="A59" s="5"/>
+      <c r="C59" s="6"/>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>No indexado</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A60" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B60" t="s">
-        <v>83</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D60" t="s">
-        <v>9</v>
-      </c>
-      <c r="E60" t="s">
-        <v>10</v>
-      </c>
-      <c r="F60" t="s">
-        <v>10</v>
-      </c>
-      <c r="G60" t="s">
-        <v>97</v>
-      </c>
-      <c r="H60" t="s">
-        <v>11</v>
-      </c>
+      <c r="A60" s="5"/>
+      <c r="C60" s="6"/>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>No indexado</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A61" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B61" t="s">
-        <v>83</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="D61" t="s">
-        <v>12</v>
-      </c>
-      <c r="E61" t="s">
-        <v>14</v>
-      </c>
-      <c r="F61" t="s">
-        <v>14</v>
-      </c>
-      <c r="G61" t="s">
-        <v>89</v>
-      </c>
-      <c r="H61" t="s">
-        <v>11</v>
-      </c>
+      <c r="A61" s="5"/>
+      <c r="C61" s="6"/>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>No indexado</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A62" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B62" t="s">
-        <v>83</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="D62" t="s">
-        <v>12</v>
-      </c>
-      <c r="E62" t="s">
-        <v>17</v>
-      </c>
-      <c r="F62" t="s">
-        <v>34</v>
-      </c>
-      <c r="G62" t="s">
-        <v>184</v>
-      </c>
-      <c r="H62" t="s">
-        <v>11</v>
-      </c>
+      <c r="A62" s="5"/>
+      <c r="C62" s="6"/>
       <c r="I62" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>No indexado</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A63" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B63" t="s">
-        <v>83</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="D63" t="s">
-        <v>12</v>
-      </c>
-      <c r="E63" t="s">
-        <v>14</v>
-      </c>
-      <c r="F63" t="s">
-        <v>186</v>
-      </c>
-      <c r="G63" t="s">
-        <v>119</v>
-      </c>
-      <c r="H63" t="s">
-        <v>11</v>
-      </c>
+      <c r="A63" s="5"/>
+      <c r="C63" s="6"/>
       <c r="I63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>No indexado</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A64" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B64" t="s">
-        <v>83</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D64" t="s">
-        <v>12</v>
-      </c>
-      <c r="E64" t="s">
-        <v>26</v>
-      </c>
-      <c r="F64" t="s">
-        <v>26</v>
-      </c>
-      <c r="G64" t="s">
-        <v>125</v>
-      </c>
-      <c r="H64" t="s">
-        <v>11</v>
-      </c>
+      <c r="A64" s="5"/>
+      <c r="C64" s="6"/>
       <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>No indexado</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A65" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B65" t="s">
-        <v>39</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="D65" t="s">
-        <v>13</v>
-      </c>
-      <c r="E65" t="s">
-        <v>86</v>
-      </c>
-      <c r="F65" t="s">
-        <v>86</v>
-      </c>
-      <c r="G65" t="s">
-        <v>109</v>
-      </c>
-      <c r="H65" t="s">
-        <v>11</v>
-      </c>
+      <c r="A65" s="5"/>
+      <c r="C65" s="6"/>
       <c r="I65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A66" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B66" t="s">
-        <v>39</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D66" t="s">
-        <v>12</v>
-      </c>
-      <c r="E66" t="s">
-        <v>21</v>
-      </c>
-      <c r="F66" t="s">
-        <v>21</v>
-      </c>
-      <c r="G66" t="s">
-        <v>132</v>
-      </c>
-      <c r="H66" t="s">
-        <v>11</v>
-      </c>
+        <v>No indexado</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A66" s="5"/>
+      <c r="C66" s="6"/>
       <c r="I66" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A67" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B67" t="s">
-        <v>39</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D67" t="s">
-        <v>12</v>
-      </c>
-      <c r="E67" t="s">
-        <v>17</v>
-      </c>
-      <c r="F67" t="s">
-        <v>17</v>
-      </c>
-      <c r="G67" t="s">
-        <v>90</v>
-      </c>
-      <c r="H67" t="s">
-        <v>16</v>
-      </c>
+        <v>No indexado</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A67" s="5"/>
+      <c r="C67" s="6"/>
       <c r="I67" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A68" s="5">
-        <v>46084</v>
-      </c>
-      <c r="B68" t="s">
-        <v>39</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="D68" t="s">
-        <v>12</v>
-      </c>
-      <c r="E68" t="s">
-        <v>26</v>
-      </c>
-      <c r="F68" t="s">
-        <v>26</v>
-      </c>
-      <c r="G68" t="s">
-        <v>125</v>
-      </c>
-      <c r="H68" t="s">
-        <v>27</v>
-      </c>
+        <v>No indexado</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A68" s="5"/>
+      <c r="C68" s="6"/>
       <c r="I68" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>No indexado</v>
       </c>
     </row>
   </sheetData>
@@ -3204,7 +2914,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3212,7 +2922,7 @@
         <v>17</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3220,20 +2930,20 @@
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
@@ -3241,18 +2951,18 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B6" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3265,34 +2975,34 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B9" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3300,28 +3010,28 @@
         <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
@@ -3329,18 +3039,18 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B17" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3348,7 +3058,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3356,15 +3066,15 @@
         <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3377,18 +3087,18 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B24" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3396,23 +3106,23 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="B27" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
@@ -3420,63 +3130,63 @@
         <v>14</v>
       </c>
       <c r="B28" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B29" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="B30" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="B31" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="B33" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B34" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B35" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -3484,7 +3194,7 @@
         <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
@@ -3492,39 +3202,39 @@
         <v>21</v>
       </c>
       <c r="B37" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B39" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B41" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3532,7 +3242,7 @@
         <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
@@ -3540,20 +3250,20 @@
         <v>24</v>
       </c>
       <c r="B43" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B44" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
@@ -3561,7 +3271,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
@@ -3569,15 +3279,15 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B47" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>
@@ -3585,7 +3295,7 @@
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B49" t="s">
         <v>10</v>
@@ -3593,26 +3303,26 @@
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B50" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B51" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B52" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Homicidios 5 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DA2E339-E8DF-4A6D-86F4-639EEE850885}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77B54590-16EA-47EB-A757-CB68FCC126BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="186">
   <si>
     <t>Fecha</t>
   </si>
@@ -595,9 +595,6 @@
   </si>
   <si>
     <t>Muere trailero tras resistirse a un asalto</t>
-  </si>
-  <si>
-    <t>Homicidio</t>
   </si>
 </sst>
 </file>
@@ -1114,20 +1111,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
   <dimension ref="A1:I65"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.7109375" customWidth="1"/>
-    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.7265625" customWidth="1"/>
+    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1156,7 +1153,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
         <v>46086</v>
       </c>
@@ -1186,7 +1183,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
         <v>46086</v>
       </c>
@@ -1216,7 +1213,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
         <v>46086</v>
       </c>
@@ -1246,7 +1243,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
         <v>46086</v>
       </c>
@@ -1276,7 +1273,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
         <v>46086</v>
       </c>
@@ -1306,7 +1303,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
         <v>46086</v>
       </c>
@@ -1336,7 +1333,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
         <v>46086</v>
       </c>
@@ -1366,7 +1363,7 @@
         <v>Partidos</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
         <v>46086</v>
       </c>
@@ -1396,7 +1393,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
         <v>46086</v>
       </c>
@@ -1426,7 +1423,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
         <v>46086</v>
       </c>
@@ -1456,7 +1453,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
         <v>46086</v>
       </c>
@@ -1486,7 +1483,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
         <v>46086</v>
       </c>
@@ -1516,7 +1513,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
         <v>46086</v>
       </c>
@@ -1546,7 +1543,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
         <v>46086</v>
       </c>
@@ -1576,7 +1573,7 @@
         <v>Partidos</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
         <v>46086</v>
       </c>
@@ -1606,7 +1603,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
         <v>46086</v>
       </c>
@@ -1636,7 +1633,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
         <v>46086</v>
       </c>
@@ -1666,7 +1663,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
         <v>46086</v>
       </c>
@@ -1696,7 +1693,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>46086</v>
       </c>
@@ -1726,7 +1723,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
         <v>46086</v>
       </c>
@@ -1756,7 +1753,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
         <v>46086</v>
       </c>
@@ -1786,7 +1783,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
         <v>46086</v>
       </c>
@@ -1816,7 +1813,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
         <v>46086</v>
       </c>
@@ -1846,7 +1843,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
         <v>46086</v>
       </c>
@@ -1876,7 +1873,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
         <v>46086</v>
       </c>
@@ -1906,7 +1903,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
         <v>46086</v>
       </c>
@@ -1936,7 +1933,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>46086</v>
       </c>
@@ -1966,7 +1963,7 @@
         <v>Presidencia de la República</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
         <v>46086</v>
       </c>
@@ -1996,7 +1993,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
         <v>46086</v>
       </c>
@@ -2026,7 +2023,7 @@
         <v>Presidencia de la República</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
         <v>46086</v>
       </c>
@@ -2056,7 +2053,7 @@
         <v>Presidencia de la República</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
         <v>46086</v>
       </c>
@@ -2086,7 +2083,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
         <v>46086</v>
       </c>
@@ -2116,7 +2113,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>46086</v>
       </c>
@@ -2146,7 +2143,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>46086</v>
       </c>
@@ -2176,7 +2173,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
         <v>46086</v>
       </c>
@@ -2206,7 +2203,7 @@
         <v>Presidencia de la República</v>
       </c>
     </row>
-    <row r="37" spans="1:9" ht="75" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" ht="58" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
         <v>46086</v>
       </c>
@@ -2236,7 +2233,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="38" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
         <v>46086</v>
       </c>
@@ -2266,7 +2263,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="39" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
         <v>46086</v>
       </c>
@@ -2296,7 +2293,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="40" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
         <v>46086</v>
       </c>
@@ -2326,7 +2323,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="41" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
         <v>46086</v>
       </c>
@@ -2356,7 +2353,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="42" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
         <v>46086</v>
       </c>
@@ -2386,7 +2383,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
         <v>46086</v>
       </c>
@@ -2416,7 +2413,7 @@
         <v>Alcaldías</v>
       </c>
     </row>
-    <row r="44" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
         <v>46086</v>
       </c>
@@ -2446,7 +2443,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="45" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
         <v>46086</v>
       </c>
@@ -2476,7 +2473,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="46" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
         <v>46086</v>
       </c>
@@ -2506,7 +2503,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
         <v>46086</v>
       </c>
@@ -2536,7 +2533,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="48" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
         <v>46086</v>
       </c>
@@ -2566,7 +2563,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
         <v>46086</v>
       </c>
@@ -2596,7 +2593,7 @@
         <v>Partidos</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
         <v>46086</v>
       </c>
@@ -2626,7 +2623,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
         <v>46086</v>
       </c>
@@ -2656,7 +2653,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
         <v>46086</v>
       </c>
@@ -2686,7 +2683,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
         <v>46086</v>
       </c>
@@ -2716,7 +2713,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
         <v>46086</v>
       </c>
@@ -2746,7 +2743,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
         <v>46086</v>
       </c>
@@ -2776,7 +2773,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
         <v>46086</v>
       </c>
@@ -2806,7 +2803,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
         <v>46086</v>
       </c>
@@ -2836,7 +2833,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
         <v>46086</v>
       </c>
@@ -2866,7 +2863,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
         <v>46086</v>
       </c>
@@ -2896,7 +2893,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
         <v>46086</v>
       </c>
@@ -2926,7 +2923,7 @@
         <v>Alcaldías</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
         <v>46086</v>
       </c>
@@ -2956,7 +2953,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" ht="29" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
         <v>46086</v>
       </c>
@@ -2986,7 +2983,7 @@
         <v>Gobierno del estado</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
         <v>46086</v>
       </c>
@@ -3016,7 +3013,7 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
         <v>46086</v>
       </c>
@@ -3046,7 +3043,7 @@
         <v>Presidencia de la República</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
         <v>46086</v>
       </c>
@@ -3066,7 +3063,7 @@
         <v>24</v>
       </c>
       <c r="G65" t="s">
-        <v>186</v>
+        <v>119</v>
       </c>
       <c r="H65" t="s">
         <v>16</v>
@@ -3088,13 +3085,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8151DEFD-FF29-4969-B1FC-DF47C7CD743C}">
   <dimension ref="A1:B52"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -3102,7 +3099,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>17</v>
       </c>
@@ -3110,7 +3107,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -3118,7 +3115,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>39</v>
       </c>
@@ -3126,7 +3123,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -3134,7 +3131,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>41</v>
       </c>
@@ -3142,7 +3139,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -3150,7 +3147,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>28</v>
       </c>
@@ -3158,7 +3155,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>42</v>
       </c>
@@ -3166,7 +3163,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>43</v>
       </c>
@@ -3174,7 +3171,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>44</v>
       </c>
@@ -3182,7 +3179,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>45</v>
       </c>
@@ -3190,7 +3187,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -3198,7 +3195,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -3206,7 +3203,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>47</v>
       </c>
@@ -3214,7 +3211,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>48</v>
       </c>
@@ -3222,7 +3219,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>49</v>
       </c>
@@ -3230,7 +3227,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>51</v>
       </c>
@@ -3238,7 +3235,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -3246,7 +3243,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>23</v>
       </c>
@@ -3254,7 +3251,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>53</v>
       </c>
@@ -3262,7 +3259,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>10</v>
       </c>
@@ -3270,7 +3267,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>54</v>
       </c>
@@ -3278,7 +3275,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -3286,7 +3283,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>18</v>
       </c>
@@ -3294,7 +3291,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>56</v>
       </c>
@@ -3302,7 +3299,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>57</v>
       </c>
@@ -3310,7 +3307,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>14</v>
       </c>
@@ -3318,7 +3315,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>59</v>
       </c>
@@ -3326,7 +3323,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>60</v>
       </c>
@@ -3334,7 +3331,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>61</v>
       </c>
@@ -3342,7 +3339,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>62</v>
       </c>
@@ -3350,7 +3347,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>63</v>
       </c>
@@ -3358,7 +3355,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>64</v>
       </c>
@@ -3366,7 +3363,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>65</v>
       </c>
@@ -3374,7 +3371,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>25</v>
       </c>
@@ -3382,7 +3379,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>21</v>
       </c>
@@ -3390,7 +3387,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>33</v>
       </c>
@@ -3398,7 +3395,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>29</v>
       </c>
@@ -3406,7 +3403,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>66</v>
       </c>
@@ -3414,7 +3411,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>67</v>
       </c>
@@ -3422,7 +3419,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -3430,7 +3427,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>24</v>
       </c>
@@ -3438,7 +3435,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>68</v>
       </c>
@@ -3446,7 +3443,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>69</v>
       </c>
@@ -3454,7 +3451,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>70</v>
       </c>
@@ -3462,7 +3459,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>35</v>
       </c>
@@ -3470,7 +3467,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>71</v>
       </c>
@@ -3478,7 +3475,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>72</v>
       </c>
@@ -3486,7 +3483,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>73</v>
       </c>
@@ -3494,7 +3491,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>75</v>
       </c>
@@ -3502,7 +3499,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>76</v>
       </c>

</xml_diff>

<commit_message>
Reporte 9 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FF3096B-56DF-40C7-972E-7A531F5FCEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{353D8093-174A-4CF9-8434-AC0CE1DDE95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="552" uniqueCount="163">
   <si>
     <t>Fecha</t>
   </si>
@@ -105,9 +105,6 @@
     <t>Semarnath</t>
   </si>
   <si>
-    <t>Deportes</t>
-  </si>
-  <si>
     <t>Oficialía Mayor</t>
   </si>
   <si>
@@ -279,337 +276,256 @@
     <t>Zunoticia</t>
   </si>
   <si>
-    <t>Mundial De Futbol</t>
-  </si>
-  <si>
     <t>Marcha 8M</t>
   </si>
   <si>
-    <t>Vallas</t>
-  </si>
-  <si>
-    <t>Sarampión</t>
-  </si>
-  <si>
-    <t>Temas internacionales</t>
-  </si>
-  <si>
-    <t>Abasto De Agua</t>
-  </si>
-  <si>
-    <t>Gusano barrenador</t>
-  </si>
-  <si>
-    <t>Sitmah</t>
-  </si>
-  <si>
     <t>Nivel</t>
   </si>
   <si>
-    <t>Cierre de clínica afecta a casi 10 mil usuarios</t>
-  </si>
-  <si>
-    <t>Deficiencias Centro de Salud</t>
-  </si>
-  <si>
-    <t>Fallo de la SCJN abre paso a ejecución de sentencia</t>
-  </si>
-  <si>
-    <t>SICT</t>
-  </si>
-  <si>
-    <t>Tren México Querétaro</t>
-  </si>
-  <si>
-    <t>Hasta el lunes abrirán estación Plaza Juárez</t>
-  </si>
-  <si>
-    <t>Se siguen violentando nuestros derechos</t>
-  </si>
-  <si>
     <t>8M</t>
   </si>
   <si>
-    <t>Tarifa inicial de $55 y kilómetro extra $4.50</t>
-  </si>
-  <si>
-    <t>Aumento Tarifa De Transporte</t>
-  </si>
-  <si>
-    <t>Señalan a alcaldes por los altos costos en leyes de ingresos</t>
-  </si>
-  <si>
-    <t>Ley De Ingresos</t>
-  </si>
-  <si>
-    <t>Reloj acorazado</t>
-  </si>
-  <si>
-    <t>Recientemente se publicó una reforma a la Constitución Política de Hidalgo en materia del Tribunal de Justicia Administrativa. Puede...</t>
-  </si>
-  <si>
-    <t>Reforma De Ley</t>
-  </si>
-  <si>
-    <t>Realizan cercos epidemiológicos</t>
-  </si>
-  <si>
-    <t>Vacunación</t>
-  </si>
-  <si>
-    <t>Rutas de la Transformación en Acaxochitlán</t>
-  </si>
-  <si>
-    <t>Ruta de la Transformación</t>
-  </si>
-  <si>
-    <t>Crece en Hidalgo el emprendimiento</t>
-  </si>
-  <si>
-    <t>Emprendimiento</t>
-  </si>
-  <si>
-    <t>Aseh insta a empresas a cumplir o pagar</t>
-  </si>
-  <si>
-    <t>ASEH</t>
-  </si>
-  <si>
-    <t>Garantía de obra</t>
-  </si>
-  <si>
-    <t>CHARLYN PIDE SALARIOS JUSTOS</t>
-  </si>
-  <si>
-    <t>Olympia impulsa el pádel en Hidalgo</t>
-  </si>
-  <si>
-    <t>DIERON A LUZ CASI 500 MENORES DE 15 AÑOS</t>
-  </si>
-  <si>
-    <t>Embarazo adolescente</t>
-  </si>
-  <si>
-    <t>Ellas mueven a Hidalgo</t>
-  </si>
-  <si>
-    <t>2025: año con menos robo de vehículos en una década</t>
-  </si>
-  <si>
-    <t>Robo de vehículo</t>
-  </si>
-  <si>
-    <t>Robo de cableado: En túnel Real del Monte a Huasca pega con 380 mdp</t>
-  </si>
-  <si>
-    <t>Carretera Huasca</t>
-  </si>
-  <si>
-    <t>Maltrato animal: va uno más ante el MP por violencia contra mascotas</t>
-  </si>
-  <si>
-    <t>Maltrato animal</t>
-  </si>
-  <si>
-    <t>Aplicarán sanciones en predios abandonados</t>
-  </si>
-  <si>
-    <t>Prevención de incendios</t>
-  </si>
-  <si>
-    <t>La muerte se ensaña con el arte: Lobo Antunes y Pedro Friedeberg</t>
-  </si>
-  <si>
-    <t>Lookmaxxers, tribu digital de heterosexuales</t>
-  </si>
-  <si>
-    <t>Donald Trump encarga al senador Markwayne Mullin estrategia migratoria de EU</t>
-  </si>
-  <si>
-    <t>Candidaturas con filtro. Morena prevé pasarlas por la FGR y nada de despensas</t>
-  </si>
-  <si>
-    <t>Por vestigios ven posible modificar ruta del México-Querétaro</t>
-  </si>
-  <si>
-    <t>Menchaca busca proteger a mujeres policías con vallas</t>
-  </si>
-  <si>
-    <t>Piden incluir en código penal el protocolo de feminicidio</t>
-  </si>
-  <si>
-    <t>Perspectiva de género</t>
-  </si>
-  <si>
-    <t>Trump asegura que caída de Cuba será la cereza del pastel</t>
-  </si>
-  <si>
-    <t>Avanza construcción del Tren México-Querétaro en Hidalgo</t>
-  </si>
-  <si>
-    <t>Vivimos en un momento en donde la inmediatez de las noticias y los alcances de propagación de  información de todo tipo son extremos (…) Así construimos metáforas sobre los conflictos: desde la  buenitud, como aquellas personas bondadosas y positivas; y la malitud, los partidarios de la maldad. ¿Son  tan simplificables las relaciones entre personas, grupos y países?”.</t>
-  </si>
-  <si>
-    <t>Invierten más de 130 mdp en obras para Acaxochitlán</t>
-  </si>
-  <si>
-    <t>Suma Hidalgo 15 casos de sarampión en nueve municipios</t>
-  </si>
-  <si>
-    <t>Definen colectivas feministas itinerario de actividades y marcha del 8M en Pachuca</t>
-  </si>
-  <si>
-    <t>Incluyen a Hidalgo en programa federal de nuevas canchas por el mundial</t>
-  </si>
-  <si>
-    <t>Que los actuales dirigentes de la UCLA se hagan a un lado</t>
-  </si>
-  <si>
-    <t>Despojo</t>
-  </si>
-  <si>
-    <t>En Huautla, Sipdus pavimenta camino deTohuaco Amazintla</t>
-  </si>
-  <si>
     <t>Sipdus</t>
   </si>
   <si>
-    <t>Rehabilitación carretera</t>
-  </si>
-  <si>
-    <t>Brindan certeza jurídica a menor de edad en estado de vulnerabilidad</t>
-  </si>
-  <si>
-    <t>Protección del menor</t>
-  </si>
-  <si>
-    <t>Alcalde recorrió instalaciones deportivas</t>
-  </si>
-  <si>
-    <t>Alcalde</t>
-  </si>
-  <si>
-    <t>Recorrido por instalaciones</t>
-  </si>
-  <si>
-    <t>Inaugura secretario de Educación final de Mundialito de Futbol</t>
-  </si>
-  <si>
-    <t>Marcha del 8M será resguardada por 300 policías mujeres</t>
-  </si>
-  <si>
-    <t>Proponen tipificar el acecho y el acoso sexual en Hidalgo</t>
-  </si>
-  <si>
-    <t>PAN cuestiona gasto en vallas; pide destinar recursos a programas</t>
-  </si>
-  <si>
-    <t>Caasim recupera pozo clave para abastecer de agua a Pachuca</t>
-  </si>
-  <si>
-    <t>Caasim</t>
-  </si>
-  <si>
-    <t>Profepa detiene destrucción de bosque en Zacualtipán</t>
-  </si>
-  <si>
-    <t>Protección Biodiversidad</t>
-  </si>
-  <si>
-    <t>Juez obliga al Niño DIF garantizar tratamiento a menor</t>
-  </si>
-  <si>
-    <t>Hospital del Niño</t>
-  </si>
-  <si>
-    <t>Amparo</t>
-  </si>
-  <si>
-    <t>Editorial ¿Monumentos o mujeres?</t>
-  </si>
-  <si>
     <t>Marfeca</t>
   </si>
   <si>
-    <t>Claudia Sandoval escucha y atiende el día del Pueblo en Colonia Dendho</t>
-  </si>
-  <si>
-    <t>Atención a la ciudadanía</t>
-  </si>
-  <si>
-    <t>Acaxochitlán se fortalece con inversión de más de 130 mdp en infraestructura: Menchaca</t>
-  </si>
-  <si>
-    <t>Gobierno de Tlaxcoapan impulsa el deporte en jóvenes del Cobaeh Doxey</t>
-  </si>
-  <si>
-    <t>Impulso al deporte</t>
-  </si>
-  <si>
-    <t>Fortalecen servicios de rehabilitación con nuevo espacio en la UBR de Atotonilco de Tula</t>
-  </si>
-  <si>
-    <t>Rehabilitación UBR</t>
-  </si>
-  <si>
-    <t>La autonomía sindical abre caminos para nuevas generaciones del magisterio</t>
-  </si>
-  <si>
-    <t>Aparatoso accidente entre automóvil y camión deja 1 prensado en la Pachuca-Actopan</t>
-  </si>
-  <si>
-    <t>Accidente Carretero</t>
-  </si>
-  <si>
-    <t>Blindan Palacio de Gobierno y Reloj Monumental previo a movilizaciones del 8M</t>
-  </si>
-  <si>
-    <t>Colocan vallas en Reloj y Palacio de Gobierno previo al 8M</t>
-  </si>
-  <si>
-    <t>Hay seis casos activos de sarampión en la entidad</t>
-  </si>
-  <si>
-    <t>Llaman a ganaderos hidalguenses a prevenir gusano barrenador</t>
-  </si>
-  <si>
-    <t>Con inversión superior a los 130 mdp, Julio Menchaca fortalece la infraestructura en Acaxochitlán</t>
-  </si>
-  <si>
-    <t>Ballet de Pachuca presentará México en escena</t>
-  </si>
-  <si>
-    <t>Evento Cultural</t>
-  </si>
-  <si>
-    <t>Hidalgo invierte 130 mdp en Acaxochitlán</t>
-  </si>
-  <si>
-    <t>Hidalgo será sede de reunión de gabinetes de seguridad</t>
-  </si>
-  <si>
-    <t>Reunión Gabinetes De Seguridad</t>
-  </si>
-  <si>
-    <t>La guerra en Medio Oriente se extiende. Trump encendió el fuego que después puede resultar imposible apagarlo</t>
-  </si>
-  <si>
     <t>Editorial</t>
   </si>
   <si>
-    <t>Policía desmanteló tres puntos de venta de droga</t>
-  </si>
-  <si>
-    <t>Combate Al Narcomenudeo</t>
-  </si>
-  <si>
-    <t>Suman 33 muertes por sarampión en México</t>
-  </si>
-  <si>
-    <t>Salud</t>
-  </si>
-  <si>
     <t>Gabinete</t>
+  </si>
+  <si>
+    <t>Gastan hasta 100 mil pesos en limpiar pintas</t>
+  </si>
+  <si>
+    <t>Sube el precio del gas tipo LP en la entidad</t>
+  </si>
+  <si>
+    <t>Capacitan a mujeres para emprender</t>
+  </si>
+  <si>
+    <t>Marcha 8M reúne a miles; saldo blanco</t>
+  </si>
+  <si>
+    <t>Precio del petróleo supera 100 dólares</t>
+  </si>
+  <si>
+    <t>Exigen que termine violencia contra mujeres</t>
+  </si>
+  <si>
+    <t>Las calles se pintaron de morado en Hidalgo, miles de mujeres de todas las edades, estratos sociales y creencias se unieron en una sola voz</t>
+  </si>
+  <si>
+    <t>Incierto uso de urnas electrónicas</t>
+  </si>
+  <si>
+    <t>Suben víctimas por vaguada</t>
+  </si>
+  <si>
+    <t>Huracán Priscilla</t>
+  </si>
+  <si>
+    <t>PRD pide emitir alerta</t>
+  </si>
+  <si>
+    <t>Alerta de género</t>
+  </si>
+  <si>
+    <t>No pedimos permiso</t>
+  </si>
+  <si>
+    <t>MOSTRARON LA FUERZA VIOLETA</t>
+  </si>
+  <si>
+    <t>Hasta 7 asesinadas, pero sin feminicidios</t>
+  </si>
+  <si>
+    <t>Feminicidio</t>
+  </si>
+  <si>
+    <t>Lizzie vivió una espiral de violencia</t>
+  </si>
+  <si>
+    <t>Recaudan $268.8 millones por trámites vehiculares en 2 meses</t>
+  </si>
+  <si>
+    <t>Recaudación</t>
+  </si>
+  <si>
+    <t>Mujeres toman calles para exigir alto a la violencia</t>
+  </si>
+  <si>
+    <t>Reconoce CSP a mujeres en Fuerzas Armadas</t>
+  </si>
+  <si>
+    <t>Se manifiestan en el Día Internacional de la Mujer</t>
+  </si>
+  <si>
+    <t>En Hidalgo, las tres más recientes presidencias del Tribunal Superior de Justicia han sido de magistradas, antecedidas de la primera, hace casi 20 años”</t>
+  </si>
+  <si>
+    <t>Transcurre en paz marcha feminista por el 8M</t>
+  </si>
+  <si>
+    <t>Establecerán cabildos calendario oficial de sesiones para evitar inasistencias de ediles</t>
+  </si>
+  <si>
+    <t>Iniciativa</t>
+  </si>
+  <si>
+    <t>Inicia consulta para la restauración ecológica de la Presa Endhó</t>
+  </si>
+  <si>
+    <t>Medio ambiente</t>
+  </si>
+  <si>
+    <t>Presa Endhó</t>
+  </si>
+  <si>
+    <t>Exhiben a deudores alimentarios en tendederos de denuncia</t>
+  </si>
+  <si>
+    <t>Marchan mujeres por el 8M, exigen justicia por feminicidios en la Huasteca</t>
+  </si>
+  <si>
+    <t>Más de mil asistentes en conferencia magistral de Paola Rojas en Huejutla</t>
+  </si>
+  <si>
+    <t>Promueve Saderh productividad del campo</t>
+  </si>
+  <si>
+    <t>Impulso al agro</t>
+  </si>
+  <si>
+    <t>Protección Civil revisa que comercios cumplan las medidas de seguridad</t>
+  </si>
+  <si>
+    <t>Prevención De Riesgos</t>
+  </si>
+  <si>
+    <t>Cuasiparroquia "Sagrado Corazón de Jesús" celebró la fiesta del elote</t>
+  </si>
+  <si>
+    <t>Mujeres al volante: Maura García encuentra en el taxi una nueva ruta profesional</t>
+  </si>
+  <si>
+    <t>¡Se acabó el "mandadito"!</t>
+  </si>
+  <si>
+    <t>Supervisión de Transporte</t>
+  </si>
+  <si>
+    <t>Del abuso al feminicidio</t>
+  </si>
+  <si>
+    <t>"Hombres han tenido toda la historia de Hidalgo, ahora le toca a las mujeres"</t>
+  </si>
+  <si>
+    <t>8m</t>
+  </si>
+  <si>
+    <t>De mercenarios y plurinominales</t>
+  </si>
+  <si>
+    <t>La verdadera pregunta no es por qué marchan, sino por qué aún tienen que hacerlo</t>
+  </si>
+  <si>
+    <t>97 apos del PRI... y caben en una combi</t>
+  </si>
+  <si>
+    <t>PRI</t>
+  </si>
+  <si>
+    <t>Conmemoración Aniversario</t>
+  </si>
+  <si>
+    <t>Yo como que oí... Carolina Viggiano, tendedero de denuncias y Napoleón González</t>
+  </si>
+  <si>
+    <t>Despacho del Gobernador promueve prevención al acoso y hostigamiento</t>
+  </si>
+  <si>
+    <t>Cintillo</t>
+  </si>
+  <si>
+    <t>Claudia Sandoval celebra el carnaval de Tezoquipa, fortaleciendo tradiciones del pueblo</t>
+  </si>
+  <si>
+    <t>Carnavales</t>
+  </si>
+  <si>
+    <t>Miles marchan en Pachuca durante el 8M para exigir justicia y frenar la violencia contra las mujeres</t>
+  </si>
+  <si>
+    <t>Con carreras, caminatas y zumba conmemoran el 8M</t>
+  </si>
+  <si>
+    <t>8M en Pachuca: mujeres toman las calles para alzar la voz contra la violencia de género</t>
+  </si>
+  <si>
+    <t>Tienen homicidios en el estado alza marginal de 24% en una década</t>
+  </si>
+  <si>
+    <t>Homicidios</t>
+  </si>
+  <si>
+    <t>Caasim: más de $ 600 mil en robos</t>
+  </si>
+  <si>
+    <t>Robo de infraestructura</t>
+  </si>
+  <si>
+    <t>Exigen justicia para mujeres... presentes y ausentes</t>
+  </si>
+  <si>
+    <t>Amagan con paro en la UAEH si no hay acuerdos</t>
+  </si>
+  <si>
+    <t>Paro laboral</t>
+  </si>
+  <si>
+    <t>La esperanza de la vida sexual mejora para los adultos mayores</t>
+  </si>
+  <si>
+    <t>CJNG protagonizó más de 556 tiroteos en 2025 que superan los mil fallecidos</t>
+  </si>
+  <si>
+    <t>inseguridad</t>
+  </si>
+  <si>
+    <t>Tendederos y altares en el epicentro de las protestas</t>
+  </si>
+  <si>
+    <t>Competencia entre bancos bajará las comisiones, estiman</t>
+  </si>
+  <si>
+    <t>Plaza Juárez</t>
+  </si>
+  <si>
+    <t>Exigen las mujeres justicia e igualdad de derechos</t>
+  </si>
+  <si>
+    <t>Reportan saldo blanco en Hidalgo durante marchas por el 8M</t>
+  </si>
+  <si>
+    <t>El grito de las mujeres volvió a escucharse en las calles para exigir justicia ante miles de feminicidios y desapariciones y no podrá acallarse en tanto siga el terror para ellas</t>
+  </si>
+  <si>
+    <t>Elementos policiacos frustran intento de suicidio</t>
+  </si>
+  <si>
+    <t>Policía municipal</t>
+  </si>
+  <si>
+    <t>Evitan suicidio</t>
+  </si>
+  <si>
+    <t>Impiden la descarga de residuos en el Relleno Sanitario</t>
+  </si>
+  <si>
+    <t>Contaminación de río</t>
   </si>
 </sst>
 </file>
@@ -742,7 +658,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -754,10 +670,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -857,8 +772,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J64" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J64" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J57" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J57" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1224,7 +1139,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1268,37 +1183,37 @@
         <v>8</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="H2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1307,32 +1222,32 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1341,22 +1256,22 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
         <v>81</v>
@@ -1366,25 +1281,25 @@
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E5" t="s">
         <v>10</v>
@@ -1393,7 +1308,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
@@ -1409,59 +1324,59 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="D7" t="s">
         <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="H7" t="s">
         <v>11</v>
@@ -1475,95 +1390,95 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>101</v>
+        <v>92</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
@@ -1574,52 +1489,52 @@
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>106</v>
+        <v>96</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="F11" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="G11" t="s">
-        <v>107</v>
+        <v>97</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B12" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -1631,10 +1546,10 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="H12" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1647,25 +1562,25 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F13" t="s">
-        <v>111</v>
+        <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>112</v>
+        <v>79</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -1681,47 +1596,47 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G14" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H14" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>114</v>
+        <v>102</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -1733,7 +1648,7 @@
         <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
@@ -1747,98 +1662,98 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B16" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>115</v>
+        <v>103</v>
       </c>
       <c r="D16" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="F16" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="G16" t="s">
-        <v>116</v>
+        <v>104</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B17" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
       <c r="D17" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F17" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G17" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B18" t="s">
         <v>74</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
       <c r="D18" t="s">
         <v>13</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="F18" t="s">
-        <v>18</v>
+        <v>43</v>
       </c>
       <c r="G18" t="s">
-        <v>119</v>
+        <v>79</v>
       </c>
       <c r="H18" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1849,15 +1764,15 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B19" t="s">
         <v>74</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
@@ -1866,13 +1781,13 @@
         <v>14</v>
       </c>
       <c r="F19" t="s">
-        <v>92</v>
+        <v>14</v>
       </c>
       <c r="G19" t="s">
-        <v>121</v>
+        <v>81</v>
       </c>
       <c r="H19" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1883,86 +1798,86 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B20" t="s">
         <v>74</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>122</v>
+        <v>107</v>
       </c>
       <c r="D20" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E20" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G20" t="s">
-        <v>123</v>
+        <v>79</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B21" t="s">
         <v>74</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="F21" t="s">
-        <v>17</v>
+        <v>63</v>
       </c>
       <c r="G21" t="s">
-        <v>125</v>
+        <v>81</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="D22" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E22" t="s">
         <v>10</v>
@@ -1971,7 +1886,7 @@
         <v>10</v>
       </c>
       <c r="G22" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
@@ -1985,27 +1900,27 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="F23" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>111</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
@@ -2021,32 +1936,32 @@
     </row>
     <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B24" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>128</v>
+        <v>112</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F24" t="s">
-        <v>10</v>
+        <v>113</v>
       </c>
       <c r="G24" t="s">
-        <v>84</v>
+        <v>114</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2055,32 +1970,32 @@
     </row>
     <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B25" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2089,56 +2004,56 @@
     </row>
     <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F26" t="s">
-        <v>92</v>
+        <v>18</v>
       </c>
       <c r="G26" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="H26" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="D27" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G27" t="s">
         <v>81</v>
@@ -2148,75 +2063,75 @@
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>46090</v>
+      </c>
+      <c r="B28" t="s">
+        <v>78</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>58</v>
+      </c>
+      <c r="F28" t="s">
+        <v>58</v>
+      </c>
+      <c r="G28" t="s">
+        <v>119</v>
+      </c>
+      <c r="H28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B28" t="s">
-        <v>75</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="D28" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" t="s">
-        <v>39</v>
-      </c>
-      <c r="F28" t="s">
-        <v>39</v>
-      </c>
-      <c r="G28" t="s">
-        <v>133</v>
-      </c>
-      <c r="H28" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
       <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B29" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F29" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G29" t="s">
-        <v>71</v>
+        <v>121</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2225,96 +2140,96 @@
     </row>
     <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B30" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>135</v>
+        <v>122</v>
       </c>
       <c r="D30" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="G30" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="120" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B31" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>136</v>
+        <v>123</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F31" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="G31" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H31" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>137</v>
+        <v>124</v>
       </c>
       <c r="D32" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F32" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G32" t="s">
-        <v>107</v>
+        <v>125</v>
       </c>
       <c r="H32" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2322,105 +2237,105 @@
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F33" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G33" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B34" t="s">
+        <v>30</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" t="s">
+        <v>128</v>
+      </c>
+      <c r="H34" t="s">
+        <v>11</v>
+      </c>
+      <c r="I34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>46090</v>
+      </c>
+      <c r="B35" t="s">
+        <v>30</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35" t="s">
         <v>76</v>
       </c>
-      <c r="C34" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="D34" t="s">
-        <v>12</v>
-      </c>
-      <c r="E34" t="s">
-        <v>10</v>
-      </c>
-      <c r="F34" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" t="s">
-        <v>81</v>
-      </c>
-      <c r="H34" t="s">
-        <v>11</v>
-      </c>
-      <c r="I34" t="str">
+      <c r="H35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
-      </c>
-      <c r="J34" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A35" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B35" t="s">
-        <v>76</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" t="s">
-        <v>14</v>
-      </c>
-      <c r="F35" t="s">
-        <v>14</v>
-      </c>
-      <c r="G35" t="s">
-        <v>80</v>
-      </c>
-      <c r="H35" t="s">
-        <v>11</v>
-      </c>
-      <c r="I35" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2429,26 +2344,26 @@
     </row>
     <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B36" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" t="s">
         <v>79</v>
       </c>
-      <c r="C36" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s">
-        <v>10</v>
-      </c>
-      <c r="F36" t="s">
-        <v>10</v>
-      </c>
-      <c r="G36" t="s">
-        <v>142</v>
-      </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
@@ -2461,129 +2376,129 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B37" t="s">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="F37" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="G37" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="H37" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B38" t="s">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="F38" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G38" t="s">
-        <v>147</v>
+        <v>95</v>
       </c>
       <c r="H38" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="D39" t="s">
-        <v>12</v>
+        <v>136</v>
       </c>
       <c r="E39" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="F39" t="s">
-        <v>149</v>
+        <v>40</v>
       </c>
       <c r="G39" t="s">
-        <v>150</v>
+        <v>81</v>
       </c>
       <c r="H39" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>151</v>
+        <v>123</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F40" t="s">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="G40" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
@@ -2599,59 +2514,59 @@
     </row>
     <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B41" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>152</v>
+        <v>137</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>81</v>
+        <v>138</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B42" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="D42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
@@ -2665,132 +2580,132 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B43" t="s">
-        <v>31</v>
+        <v>83</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="F43" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="G43" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H43" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B44" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="D44" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E44" t="s">
-        <v>144</v>
+        <v>10</v>
       </c>
       <c r="F44" t="s">
-        <v>156</v>
+        <v>10</v>
       </c>
       <c r="G44" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="H44" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J44" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="5">
+        <v>46090</v>
+      </c>
+      <c r="B45" t="s">
+        <v>73</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D45" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" t="s">
+        <v>18</v>
+      </c>
+      <c r="G45" t="s">
+        <v>143</v>
+      </c>
+      <c r="H45" t="s">
+        <v>11</v>
+      </c>
+      <c r="I45" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J44" t="str">
+      <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B45" t="s">
-        <v>31</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="D45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E45" t="s">
-        <v>14</v>
-      </c>
-      <c r="F45" t="s">
-        <v>14</v>
-      </c>
-      <c r="G45" t="s">
-        <v>158</v>
-      </c>
-      <c r="H45" t="s">
-        <v>27</v>
-      </c>
-      <c r="I45" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J45" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B46" t="s">
-        <v>31</v>
+        <v>73</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>42</v>
+        <v>82</v>
       </c>
       <c r="F46" t="s">
-        <v>160</v>
+        <v>82</v>
       </c>
       <c r="G46" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
       <c r="H46" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2803,25 +2718,25 @@
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B47" t="s">
-        <v>31</v>
+        <v>73</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>162</v>
+        <v>146</v>
       </c>
       <c r="D47" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E47" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F47" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G47" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H47" t="s">
         <v>16</v>
@@ -2835,34 +2750,34 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B48" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>164</v>
+        <v>147</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="F48" t="s">
-        <v>149</v>
+        <v>64</v>
       </c>
       <c r="G48" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2871,100 +2786,100 @@
     </row>
     <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B49" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="D49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="F49" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="G49" t="s">
-        <v>107</v>
+        <v>70</v>
       </c>
       <c r="H49" t="s">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B50" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F50" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G50" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="H50" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B51" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F51" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G51" t="s">
-        <v>170</v>
+        <v>79</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2973,13 +2888,13 @@
     </row>
     <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B52" t="s">
-        <v>163</v>
+        <v>73</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>171</v>
+        <v>153</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
@@ -2991,7 +2906,7 @@
         <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
@@ -3005,18 +2920,18 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B53" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="D53" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E53" t="s">
         <v>10</v>
@@ -3025,7 +2940,7 @@
         <v>10</v>
       </c>
       <c r="G53" t="s">
-        <v>173</v>
+        <v>79</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
@@ -3041,25 +2956,25 @@
     </row>
     <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B54" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>174</v>
+        <v>156</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="F54" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="G54" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
@@ -3073,30 +2988,30 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B55" t="s">
-        <v>30</v>
+        <v>154</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>175</v>
+        <v>157</v>
       </c>
       <c r="D55" t="s">
-        <v>13</v>
+        <v>84</v>
       </c>
       <c r="E55" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F55" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G55" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H55" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3109,306 +3024,68 @@
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B56" t="s">
-        <v>30</v>
+        <v>154</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>176</v>
+        <v>158</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F56" t="s">
-        <v>15</v>
+        <v>159</v>
       </c>
       <c r="G56" t="s">
-        <v>83</v>
+        <v>160</v>
       </c>
       <c r="H56" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46087</v>
+        <v>46090</v>
       </c>
       <c r="B57" t="s">
-        <v>30</v>
+        <v>154</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>177</v>
+        <v>161</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="F57" t="s">
-        <v>59</v>
+        <v>159</v>
       </c>
       <c r="G57" t="s">
-        <v>86</v>
+        <v>162</v>
       </c>
       <c r="H57" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J57" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B58" t="s">
-        <v>30</v>
-      </c>
-      <c r="C58" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="D58" t="s">
-        <v>12</v>
-      </c>
-      <c r="E58" t="s">
-        <v>26</v>
-      </c>
-      <c r="F58" t="s">
-        <v>26</v>
-      </c>
-      <c r="G58" t="s">
-        <v>107</v>
-      </c>
-      <c r="H58" t="s">
-        <v>27</v>
-      </c>
-      <c r="I58" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J58" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B59" t="s">
-        <v>30</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D59" t="s">
-        <v>12</v>
-      </c>
-      <c r="E59" t="s">
-        <v>17</v>
-      </c>
-      <c r="F59" t="s">
-        <v>17</v>
-      </c>
-      <c r="G59" t="s">
-        <v>180</v>
-      </c>
-      <c r="H59" t="s">
-        <v>11</v>
-      </c>
-      <c r="I59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B60" t="s">
-        <v>30</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D60" t="s">
-        <v>13</v>
-      </c>
-      <c r="E60" t="s">
-        <v>26</v>
-      </c>
-      <c r="F60" t="s">
-        <v>26</v>
-      </c>
-      <c r="G60" t="s">
-        <v>107</v>
-      </c>
-      <c r="H60" t="s">
-        <v>11</v>
-      </c>
-      <c r="I60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A61" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B61" t="s">
-        <v>30</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="D61" t="s">
-        <v>12</v>
-      </c>
-      <c r="E61" t="s">
-        <v>26</v>
-      </c>
-      <c r="F61" t="s">
-        <v>26</v>
-      </c>
-      <c r="G61" t="s">
-        <v>183</v>
-      </c>
-      <c r="H61" t="s">
-        <v>11</v>
-      </c>
-      <c r="I61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A62" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B62" t="s">
-        <v>30</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="D62" t="s">
-        <v>185</v>
-      </c>
-      <c r="E62" t="s">
-        <v>10</v>
-      </c>
-      <c r="F62" t="s">
-        <v>10</v>
-      </c>
-      <c r="G62" t="s">
-        <v>84</v>
-      </c>
-      <c r="H62" t="s">
-        <v>16</v>
-      </c>
-      <c r="I62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B63" t="s">
-        <v>30</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D63" t="s">
-        <v>12</v>
-      </c>
-      <c r="E63" t="s">
-        <v>24</v>
-      </c>
-      <c r="F63" t="s">
-        <v>24</v>
-      </c>
-      <c r="G63" t="s">
-        <v>187</v>
-      </c>
-      <c r="H63" t="s">
-        <v>11</v>
-      </c>
-      <c r="I63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A64" s="5">
-        <v>46087</v>
-      </c>
-      <c r="B64" t="s">
-        <v>30</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="D64" t="s">
-        <v>12</v>
-      </c>
-      <c r="E64" t="s">
-        <v>14</v>
-      </c>
-      <c r="F64" t="s">
-        <v>189</v>
-      </c>
-      <c r="G64" t="s">
-        <v>83</v>
-      </c>
-      <c r="H64" t="s">
-        <v>16</v>
-      </c>
-      <c r="I64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
@@ -3437,27 +3114,27 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
         <v>67</v>
-      </c>
-      <c r="B2" t="s">
-        <v>68</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -3465,13 +3142,13 @@
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -3479,251 +3156,251 @@
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E7" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>190</v>
+        <v>41</v>
+      </c>
+      <c r="E8" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B10" t="s">
         <v>10</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E16" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B17" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E17" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E18" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" t="s">
         <v>47</v>
-      </c>
-      <c r="B20" t="s">
-        <v>48</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" t="s">
         <v>49</v>
       </c>
-      <c r="B21" t="s">
-        <v>50</v>
-      </c>
       <c r="D21" s="9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E21" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3731,27 +3408,27 @@
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D22" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E22" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E23" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -3765,49 +3442,49 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E26" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>50</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>34</v>
+        <v>49</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>190</v>
+        <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3815,23 +3492,23 @@
         <v>18</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -3839,55 +3516,55 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B32" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B33" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B34" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -3895,31 +3572,31 @@
         <v>21</v>
       </c>
       <c r="B38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B41" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -3927,28 +3604,28 @@
         <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B43" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B44" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
@@ -3956,7 +3633,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
@@ -3964,15 +3641,15 @@
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B47" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Reporte 11 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60FFC503-EBAE-4EC7-AA55-6CB94302C1AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AE7B0B-FBA6-4026-B3C8-F297DFB2F06B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="191">
   <si>
     <t>Fecha</t>
   </si>
@@ -285,331 +285,331 @@
     <t>Marfeca</t>
   </si>
   <si>
-    <t>Editorial</t>
-  </si>
-  <si>
     <t>Gabinete</t>
   </si>
   <si>
-    <t>Feminicidio</t>
-  </si>
-  <si>
     <t>Cintillo</t>
   </si>
   <si>
     <t>Plaza Juárez</t>
   </si>
   <si>
-    <t>Policía municipal</t>
-  </si>
-  <si>
-    <t>Se cumple una semana con mala calidad del aire</t>
-  </si>
-  <si>
-    <t>Calidad del aire</t>
-  </si>
-  <si>
-    <t>Familias solo reciben 20 litros de agua al adía</t>
-  </si>
-  <si>
-    <t>Abasto De Agua</t>
-  </si>
-  <si>
-    <t>Embajadora de Sudáfrica visitará Hidalgo</t>
-  </si>
-  <si>
     <t>Mundial De Futbol</t>
   </si>
   <si>
-    <t>Pachuca podría quedar sin mando coordinado</t>
-  </si>
-  <si>
     <t>Mando Coordinado</t>
   </si>
   <si>
-    <t>Piden terminar construcción de escuela</t>
-  </si>
-  <si>
-    <t>Exigencia de obra</t>
-  </si>
-  <si>
-    <t>Regreso a casa</t>
-  </si>
-  <si>
-    <t>Conservación de especies</t>
-  </si>
-  <si>
-    <t>SSPH reprueba el desempeño de Ayala Guarro</t>
-  </si>
-  <si>
-    <t>Avances contra la delincuencia</t>
-  </si>
-  <si>
-    <t>Reunión Gabinete De Seguridad</t>
-  </si>
-  <si>
-    <t>Capacitarán a aspirantes al 2027</t>
-  </si>
-  <si>
-    <t>Sucesión alcaldía</t>
-  </si>
-  <si>
-    <t>El partido Morena celebró el fin de semana pasado su Congreso Nacional para definir lineamientos con miras al proceso electoral de.</t>
-  </si>
-  <si>
-    <t>Congreso Nacional</t>
-  </si>
-  <si>
-    <t>UN HURACÁN SIN FUERZA REAL</t>
-  </si>
-  <si>
     <t>Deportes</t>
   </si>
   <si>
-    <t>BUSCA DAR EL PRIMER GOLPE EN CHAMPIONS</t>
-  </si>
-  <si>
-    <t>MULTARON A 18 POR TIRAR LA BASURA EN CALLES DE PACHUCA</t>
-  </si>
-  <si>
-    <t>Sanciones por basura</t>
-  </si>
-  <si>
-    <t>DESTITUYE CJMH A AGENTES POR ANOMALÍAS EN SU QUEHACER</t>
-  </si>
-  <si>
-    <t>CJMH</t>
-  </si>
-  <si>
-    <t>Destitución</t>
-  </si>
-  <si>
-    <t>REHABILITAN EL VIADUCTO NUEVO HIDALGO</t>
-  </si>
-  <si>
-    <t>Rehabilitación Vial</t>
-  </si>
-  <si>
-    <t>PODRÍAN QUITAR A AYALA GUARRO DE SP, ADVIERTE CRUZ</t>
-  </si>
-  <si>
-    <t>HALLAZGO DE 3 CADÁVERES, SIN HECHO ILÍCITO</t>
-  </si>
-  <si>
     <t>Localización de cuerpo</t>
   </si>
   <si>
-    <t>Hidalgo, en top 10 por alza en denuncias de extorsión</t>
-  </si>
-  <si>
-    <t>Extorsión</t>
-  </si>
-  <si>
-    <t>Encuentran cuerpos de 2 mujeres y un hombre</t>
-  </si>
-  <si>
-    <t>Nathaniel Campos asume la Secretaría de Seguridad</t>
-  </si>
-  <si>
-    <t>Nombramientos</t>
-  </si>
-  <si>
-    <t>Destinarán $8 millones para las zonas arqueológicas</t>
-  </si>
-  <si>
-    <t>Localizan con vida a 53 de 60 mujeres reportadas</t>
-  </si>
-  <si>
-    <t>Fiscalía de Género</t>
-  </si>
-  <si>
-    <t>Localización de persona</t>
-  </si>
-  <si>
-    <t>Feminicidio: Cierra estado con 15 casos en 2025 y lleva uno en el año</t>
-  </si>
-  <si>
-    <t>Diplomacia de Sudáfrica la capital del estado</t>
-  </si>
-  <si>
-    <t>México opta por blindar la gasolina en 24 pesos frente a volatilidad</t>
-  </si>
-  <si>
-    <t>Firma De Convenio</t>
-  </si>
-  <si>
-    <t>Estados Unidos procesa a 44 por violencia de izquierda</t>
-  </si>
-  <si>
-    <t>Temas internacionales</t>
-  </si>
-  <si>
-    <t>Elliot, el mando Nike que cuenta tenis en la calle</t>
-  </si>
-  <si>
-    <t>Localizan a 53 de 69 mujeres desaparecidas, durante 2026</t>
-  </si>
-  <si>
-    <t>Avanza construcción de torres de gobierno</t>
-  </si>
-  <si>
-    <t>Complejo Gubernamental</t>
-  </si>
-  <si>
-    <t>Cruz Neri amaga con sacar a Pachuca del mando coordinado</t>
-  </si>
-  <si>
-    <t>El orgullo de decir no: CSP defiende soberanía tras dichos de Trump</t>
-  </si>
-  <si>
-    <t>Si el partido guinda no cuida sus puertas, 2027 no será el año del cambio, sino el del reciclaje de cacicazgos bajo una estrella roja que no pregunta por apellidos ni expedientes judiciales”.</t>
-  </si>
-  <si>
-    <t>Amenaza Cruz Neri con destituir a secretario de Seguridad de Pachuca</t>
-  </si>
-  <si>
-    <t>Suma Auditoría Superior 4.5 mdp recuperados por multas de evaluación de desempeño</t>
-  </si>
-  <si>
-    <t>ASEH</t>
-  </si>
-  <si>
-    <t>Evaluación de desempeño</t>
-  </si>
-  <si>
-    <t>Reportan saldo blanco tras movilización del 8M; desplegaron a 376 policías</t>
-  </si>
-  <si>
-    <t>Siguen sin ser localizadas 15 mujeres reportadas como desaparecidas en 2026</t>
-  </si>
-  <si>
-    <t>Se manifestaron por falta de agua</t>
-  </si>
-  <si>
-    <t>Protesta Por Agua</t>
-  </si>
-  <si>
-    <t>Gabinete de Seguridad de Hidalgo reporta avances contra la delincuencia</t>
-  </si>
-  <si>
-    <t>Finalizan mantenimiento en la red de drenaje</t>
-  </si>
-  <si>
-    <t>Obras públicas</t>
-  </si>
-  <si>
-    <t>Reparación De Tubería</t>
-  </si>
-  <si>
-    <t>Detectan casos de virus Coxsackie en Huautla y Xochiatipan</t>
-  </si>
-  <si>
-    <t>Prevención De Enfermedades</t>
-  </si>
-  <si>
-    <t>Iniciativa para periodistas en Hidalgo genera alerta por posible censura</t>
-  </si>
-  <si>
-    <t>Ley de Protección a Periodistas</t>
-  </si>
-  <si>
-    <t>Descarta alcalde creación de autodefensas en Ixmiquilpan</t>
-  </si>
-  <si>
     <t>Alcalde</t>
   </si>
   <si>
-    <t>Guardias comunitarias</t>
-  </si>
-  <si>
-    <t>Me he cansado de hablar con Ayala Guarro""</t>
-  </si>
-  <si>
-    <t>Relevo en la policía de Tizayuca; llega nuevo mando coordinado</t>
-  </si>
-  <si>
-    <t>Lanzan ""Jefas Transformadoras""</t>
-  </si>
-  <si>
-    <t>Impulso a mujeres emprendedoras</t>
-  </si>
-  <si>
-    <t>Reportan 69 mujeres desaparecidas en 2026: 53 han sido localizadas con vida</t>
-  </si>
-  <si>
-    <t>400% más presupuesto. El reto: la realidad</t>
-  </si>
-  <si>
-    <t>Erradicación Violencia De Género</t>
-  </si>
-  <si>
-    <t>Bomberos de Atitalaquia atienden incendio en el Cardonal</t>
-  </si>
-  <si>
-    <t>Control de incendios</t>
-  </si>
-  <si>
-    <t>Desisten dos funcionarios que impugnaron incompatibilidad por doble cargo</t>
-  </si>
-  <si>
-    <t>Doble Plaza</t>
-  </si>
-  <si>
-    <t>Incremento a tarifa del transporte será condicionado a mejora del servicio: Semoth</t>
-  </si>
-  <si>
-    <t>Aumento Tarifa De Transporte</t>
-  </si>
-  <si>
-    <t>Hidalgo fortalece política pública para las mujeres con presupuesto histórico superior a mil 300 mdp</t>
-  </si>
-  <si>
-    <t>Mañanera de Hidalgo</t>
-  </si>
-  <si>
-    <t>16 ejemplares regresan a su hábitat tras proceso de atención en la Unidad de Rehabilitación de Fauna en Pachuca</t>
-  </si>
-  <si>
-    <t>Rehabilitación animal</t>
-  </si>
-  <si>
-    <t>Cabildo de Atitalaquia reconoce la historia de ""La Güera Rodríguez""</t>
-  </si>
-  <si>
-    <t>SSPH amaga con retirar Mando Coordinado en Pachuca; se reúne con alcalde</t>
-  </si>
-  <si>
-    <t>mando</t>
-  </si>
-  <si>
-    <t>Gabinete de Seguridad reporta avances contra la delincuencia</t>
-  </si>
-  <si>
-    <t>16 ejemplares regresan a su hábitat tras proceso de atención en la Unidad de Rehabilitación</t>
-  </si>
-  <si>
-    <t>Hidalgo invierte más de 7.5 millones de pesos en obras educativas en Pachuca</t>
-  </si>
-  <si>
-    <t>Infraestructura escolar</t>
-  </si>
-  <si>
-    <t>Encuentran si vida a tres personas en vivienda de Tolcayuca</t>
-  </si>
-  <si>
-    <t>Hidalgo fortalece política Pública para las mujeres con presupuesto histórico</t>
-  </si>
-  <si>
-    <t>Presupuesto de mil 300 mdp para apoyar a mujeres violentadas</t>
-  </si>
-  <si>
-    <t>Un muerto y un herido tras colapso de edificio</t>
-  </si>
-  <si>
-    <t>Encuentran a un bebé sin vida a orillas de un canal</t>
-  </si>
-  <si>
-    <t>Advierte Cruz Neri que se quitará apoyo a Mando Coordinado</t>
+    <t>Hidalgo, con 10 homicidios en febrero</t>
+  </si>
+  <si>
+    <t>Homicidios</t>
+  </si>
+  <si>
+    <t>Extraen material pétreo de río</t>
+  </si>
+  <si>
+    <t>Contaminación de río</t>
+  </si>
+  <si>
+    <t>Buscan instalar Polo de Bienestar en Sahagún</t>
+  </si>
+  <si>
+    <t>Polos del Bienestar</t>
+  </si>
+  <si>
+    <t>Insuficiente donación sanguínea en el IMS</t>
+  </si>
+  <si>
+    <t>IMSS</t>
+  </si>
+  <si>
+    <t>Donación de sangre</t>
+  </si>
+  <si>
+    <t>Campesinos piden terminar obra en el canal Tlamaco</t>
+  </si>
+  <si>
+    <t>Conagua</t>
+  </si>
+  <si>
+    <t>Obra inconclusa</t>
+  </si>
+  <si>
+    <t>Reconocen la Charrería como patrimonio del estado</t>
+  </si>
+  <si>
+    <t>Patrimonio cultural</t>
+  </si>
+  <si>
+    <t>Prevén visita presidencial para inaugurar nueva nave de Mercado Libre</t>
+  </si>
+  <si>
+    <t>Visita Sheinbaum</t>
+  </si>
+  <si>
+    <t>Avanza la industria en Hidalgo en 2025</t>
+  </si>
+  <si>
+    <t>Índice De Actividad Industrial</t>
+  </si>
+  <si>
+    <t>PATRIMONIO CULTURAL</t>
+  </si>
+  <si>
+    <t>Proponen capacitar a los choferes</t>
+  </si>
+  <si>
+    <t>Iniciativa</t>
+  </si>
+  <si>
+    <t>Poco interés en la donación de sangre</t>
+  </si>
+  <si>
+    <t>DOMINAN A SAN LUIS</t>
+  </si>
+  <si>
+    <t>GANAN, PERO  ¿A QUÉ COSTO?</t>
+  </si>
+  <si>
+    <t>APRUEBAN CREAR UNIDAD ESPECIAL CONTRA EXTORSIÓN</t>
+  </si>
+  <si>
+    <t>Prevención de Extorsión</t>
+  </si>
+  <si>
+    <t>VOLUNTARIOS PARTICIPAN EN REGENERACIÓN DE BOSQUES</t>
+  </si>
+  <si>
+    <t>Conservación Biodiversidad</t>
+  </si>
+  <si>
+    <t>La charrería ya es patrimonio cultural estatal</t>
+  </si>
+  <si>
+    <t>PARA SER REPARTIDOR,  TIENEN QUE INVERTIR HASTA 22 MIL PESOS</t>
+  </si>
+  <si>
+    <t>SERVICIOS DEL IHM AYUDARON A MARÍA A SUPERAR DUELOS</t>
+  </si>
+  <si>
+    <t>IHM</t>
+  </si>
+  <si>
+    <t>Apoyo A La Mujer</t>
+  </si>
+  <si>
+    <t>Caen líderes criminales y homicidios bajan 28% en el primer bimestre</t>
+  </si>
+  <si>
+    <t>Incidencia Delictiva</t>
+  </si>
+  <si>
+    <t>Demanda de riñones supera las donaciones</t>
+  </si>
+  <si>
+    <t>Donación De Órganos</t>
+  </si>
+  <si>
+    <t>Buscan creación de polo de desarrollo en el Altiplano</t>
+  </si>
+  <si>
+    <t>Ferrocarrileras ofrecen empleo</t>
+  </si>
+  <si>
+    <t>Proyectos Ferroviarios</t>
+  </si>
+  <si>
+    <t>Lloran en Perú a Bryce Echenique, su escritor más querido</t>
+  </si>
+  <si>
+    <t>Surcorea, Vietnam, India... todo Asia padece ya escasez</t>
+  </si>
+  <si>
+    <t>"Estar con y para México", ventaja de Banorte</t>
+  </si>
+  <si>
+    <t>Gobierno estatal y productores pactan tecnificar sus tierras</t>
+  </si>
+  <si>
+    <t>Tecnificación De Riego</t>
+  </si>
+  <si>
+    <t>Luz verde a reforma  para reforzar lucha   contra la extorsión</t>
+  </si>
+  <si>
+    <t>Diego Rivera   logra amparo   en juzgado   de Toluca</t>
+  </si>
+  <si>
+    <t>Amparo</t>
+  </si>
+  <si>
+    <t>Controlan fuga de combustible en Tlapacoya</t>
+  </si>
+  <si>
+    <t>Pemex</t>
+  </si>
+  <si>
+    <t>Fuga de hidrocarburo</t>
+  </si>
+  <si>
+    <t>Cuando ocurre una unión de hecho entre un menor y un adulto, hay toda  una comunidad o sociedad que la ha validado y normalizado. No es solo  responsabilidad de la familia nuclear y la persona agresora, sino de todo un  sistema que día a día acepta esta conducta”.</t>
+  </si>
+  <si>
+    <t>Erradicación matrimonio infantil</t>
+  </si>
+  <si>
+    <t>Impulsa Menchaca Tercer Polo de  Desarrollo en Sahagún</t>
+  </si>
+  <si>
+    <t>Sigue pendiente futuro de Ayala  Guarro en Seguridad de Pachuca</t>
+  </si>
+  <si>
+    <t>Descartan dictámenes periciales  relación con delincuencia de los  decesos en Tolcayuca</t>
+  </si>
+  <si>
+    <t>Visitará Hidalgo  embajadora de Sudáfrica</t>
+  </si>
+  <si>
+    <t>Julio Menchaca renueva compromiso de transformar a Hidalgo</t>
+  </si>
+  <si>
+    <t>Ruta de la Transformación</t>
+  </si>
+  <si>
+    <t>Llaman mantener pozos de agua en óptimas condiciones</t>
+  </si>
+  <si>
+    <t>Agua</t>
+  </si>
+  <si>
+    <t>Rehabilitación de pozo</t>
+  </si>
+  <si>
+    <t>Avanza Sipdus en la tecnificación del campo en Francisco I. Madero</t>
+  </si>
+  <si>
+    <t>Exhortan a prevenir golpes de calor ante las altas temperaturas</t>
+  </si>
+  <si>
+    <t>Golpe de calor</t>
+  </si>
+  <si>
+    <t>Las tres dudas políticas del PRI</t>
+  </si>
+  <si>
+    <t>PRI</t>
+  </si>
+  <si>
+    <t>Militancia Partidista</t>
+  </si>
+  <si>
+    <t>¿Ahuyentan inversiones?</t>
+  </si>
+  <si>
+    <t>Ley De Ingresos</t>
+  </si>
+  <si>
+    <t>Violencia a la baja en Hidalgo: homicidios disminuyen casi 30%</t>
+  </si>
+  <si>
+    <t>Trabajador hidalguense entre víctimas de derrumbe en CDMX</t>
+  </si>
+  <si>
+    <t>Menchaca pide a Tepeapulco aclarar observaciones</t>
+  </si>
+  <si>
+    <t>Observaciones ASEH</t>
+  </si>
+  <si>
+    <t>IEEH socializa reglas de postulación con partidos y ¿Segobh?</t>
+  </si>
+  <si>
+    <t>Reunión con partidos</t>
+  </si>
+  <si>
+    <t>Cae supuesto líder de ""Los Poshcos"" en Hidalgo</t>
+  </si>
+  <si>
+    <t>Combate a la delincuencia</t>
+  </si>
+  <si>
+    <t>Menchaca impulsa infraestructura en Tlanalapa con más de 67 mdp</t>
+  </si>
+  <si>
+    <t>Entrega Cristhian Martínez obra de más de 11 mdp</t>
+  </si>
+  <si>
+    <t>Entrega de obra</t>
+  </si>
+  <si>
+    <t>En Tepeapulco, Menchaca renueva compromiso de transformar a Hidalgo</t>
+  </si>
+  <si>
+    <t>Mi gobierno tiene disciplina financiera, no erogamos un peso sin estar debidamente comprobado</t>
+  </si>
+  <si>
+    <t>Disciplina financiera</t>
+  </si>
+  <si>
+    <t>Sin sanciones a policías por confrontación con manifestantes del 8M</t>
+  </si>
+  <si>
+    <t>Magisterio hidalguense fortalece la unidad</t>
+  </si>
+  <si>
+    <t>IEEH inaugura la 3a edición del Diplomado en violencia política de género</t>
+  </si>
+  <si>
+    <t>Violencia Política De Género</t>
+  </si>
+  <si>
+    <t>En Hidalgo, incidencia delictiva a la baja: reporte nacional</t>
+  </si>
+  <si>
+    <t>Renovación de la carpeta asfáltica desquicia la México-Pachuca</t>
+  </si>
+  <si>
+    <t>Desde Tepeapulco, Julio Menchaca renueva compromiso de transformar a Hidalgo</t>
+  </si>
+  <si>
+    <t>SSPH detiene a presunto líder del grupo delictivo ""Los Poshcos""</t>
+  </si>
+  <si>
+    <t>Fuga de oleoso causa alarma en sector de la capital</t>
+  </si>
+  <si>
+    <t>Yua viene muestra gastronómica de Santiago de Anaya</t>
+  </si>
+  <si>
+    <t>Festival Gastronómico</t>
+  </si>
+  <si>
+    <t>Reforzarán seguridad pública de Pachuca</t>
+  </si>
+  <si>
+    <t>Refuerzo De Seguridad</t>
+  </si>
+  <si>
+    <t>Crearán una unidad especializada contra la extorsión</t>
+  </si>
+  <si>
+    <t>Siempre es mejor atender los señalamientos a la seguridad en la capital, que entorpecer la coordinación que debe existir entre los mandos del estado</t>
+  </si>
+  <si>
+    <t>Anuncian inversión de 26 mdp para Ciudad Sahagún</t>
+  </si>
+  <si>
+    <t>Sheinbaum destacó la reducción del 44% de homicidios</t>
   </si>
 </sst>
 </file>
@@ -856,8 +856,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J65" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J65" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J64" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J64" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1223,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J65"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -1272,25 +1272,25 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B2" t="s">
         <v>71</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
@@ -1306,32 +1306,32 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B3" t="s">
         <v>71</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H3" t="s">
         <v>16</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1340,28 +1340,28 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B4" t="s">
         <v>71</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H4" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1369,132 +1369,132 @@
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B5" t="s">
         <v>71</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>23</v>
+        <v>97</v>
       </c>
       <c r="G5" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B6" t="s">
         <v>71</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>28</v>
+        <v>100</v>
       </c>
       <c r="G6" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="H6" t="s">
         <v>16</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F7" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H7" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B8" t="s">
         <v>72</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
         <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>95</v>
+        <v>105</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
@@ -1505,33 +1505,33 @@
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B9" t="s">
         <v>72</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>59</v>
       </c>
       <c r="G9" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H9" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1539,71 +1539,71 @@
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B10" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D10" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" t="s">
+        <v>38</v>
+      </c>
+      <c r="G10" t="s">
         <v>103</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F10" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" t="s">
-        <v>104</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B11" t="s">
         <v>72</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="G11" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1612,32 +1612,32 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F12" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="G12" t="s">
-        <v>108</v>
+        <v>98</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1646,13 +1646,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B13" t="s">
         <v>76</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1664,7 +1664,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>108</v>
+        <v>87</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -1678,64 +1678,64 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B14" t="s">
         <v>76</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B15" t="s">
         <v>76</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F15" t="s">
-        <v>113</v>
+        <v>25</v>
       </c>
       <c r="G15" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H15" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1743,135 +1743,135 @@
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B16" t="s">
         <v>76</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B17" t="s">
         <v>76</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="D17" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="F17" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="G17" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B18" t="s">
         <v>76</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>120</v>
       </c>
       <c r="D19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="F19" t="s">
-        <v>18</v>
+        <v>121</v>
       </c>
       <c r="G19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H19" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1882,18 +1882,18 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B20" t="s">
         <v>73</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E20" t="s">
         <v>18</v>
@@ -1902,10 +1902,10 @@
         <v>18</v>
       </c>
       <c r="G20" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="H20" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1918,32 +1918,32 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B21" t="s">
         <v>73</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F21" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="G21" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1952,168 +1952,168 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B22" t="s">
         <v>73</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="D22" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E22" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F22" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G22" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B23" t="s">
         <v>73</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F23" t="s">
-        <v>127</v>
+        <v>14</v>
       </c>
       <c r="G23" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H23" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B24" t="s">
         <v>73</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="H24" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B25" t="s">
         <v>73</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B26" t="s">
         <v>73</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>132</v>
+        <v>70</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2122,10 +2122,10 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C27" s="6" t="s">
         <v>133</v>
@@ -2134,10 +2134,10 @@
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="F27" t="s">
-        <v>10</v>
+        <v>80</v>
       </c>
       <c r="G27" t="s">
         <v>134</v>
@@ -2147,50 +2147,50 @@
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C28" s="6" t="s">
         <v>135</v>
       </c>
       <c r="D28" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E28" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F28" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G28" t="s">
-        <v>70</v>
+        <v>115</v>
       </c>
       <c r="H28" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B29" t="s">
         <v>74</v>
@@ -2202,156 +2202,156 @@
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F29" t="s">
-        <v>127</v>
+        <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="H29" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B30" t="s">
         <v>74</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
       </c>
       <c r="E30" t="s">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="F30" t="s">
-        <v>80</v>
+        <v>139</v>
       </c>
       <c r="G30" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B31" t="s">
         <v>74</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="F31" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="G31" t="s">
-        <v>95</v>
+        <v>142</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J31" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32" s="5">
+        <v>46092</v>
+      </c>
+      <c r="B32" t="s">
+        <v>75</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32" t="s">
+        <v>25</v>
+      </c>
+      <c r="F32" t="s">
+        <v>25</v>
+      </c>
+      <c r="G32" t="s">
+        <v>95</v>
+      </c>
+      <c r="H32" t="s">
+        <v>26</v>
+      </c>
+      <c r="I32" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J31" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A32" s="5">
-        <v>46091</v>
-      </c>
-      <c r="B32" t="s">
-        <v>74</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D32" t="s">
-        <v>12</v>
-      </c>
-      <c r="E32" t="s">
-        <v>14</v>
-      </c>
-      <c r="F32" t="s">
-        <v>14</v>
-      </c>
-      <c r="G32" t="s">
-        <v>70</v>
-      </c>
-      <c r="H32" t="s">
+      <c r="J32" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A33" s="5">
+        <v>46092</v>
+      </c>
+      <c r="B33" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" t="s">
+        <v>89</v>
+      </c>
+      <c r="G33" t="s">
+        <v>86</v>
+      </c>
+      <c r="H33" t="s">
         <v>11</v>
       </c>
-      <c r="I32" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J32" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A33" s="5">
-        <v>46091</v>
-      </c>
-      <c r="B33" t="s">
-        <v>74</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D33" t="s">
-        <v>12</v>
-      </c>
-      <c r="E33" t="s">
-        <v>19</v>
-      </c>
-      <c r="F33" t="s">
-        <v>19</v>
-      </c>
-      <c r="G33" t="s">
-        <v>104</v>
-      </c>
-      <c r="H33" t="s">
-        <v>16</v>
-      </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2360,25 +2360,25 @@
     </row>
     <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B34" t="s">
         <v>75</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="D34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F34" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="G34" t="s">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
@@ -2392,204 +2392,204 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B35" t="s">
         <v>75</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="F35" t="s">
-        <v>144</v>
+        <v>43</v>
       </c>
       <c r="G35" t="s">
-        <v>145</v>
+        <v>85</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D36" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E36" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F36" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G36" t="s">
-        <v>78</v>
+        <v>148</v>
       </c>
       <c r="H36" t="s">
+        <v>26</v>
+      </c>
+      <c r="I36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37" s="5">
+        <v>46092</v>
+      </c>
+      <c r="B37" t="s">
+        <v>77</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" t="s">
+        <v>150</v>
+      </c>
+      <c r="G37" t="s">
+        <v>151</v>
+      </c>
+      <c r="H37" t="s">
         <v>11</v>
       </c>
-      <c r="I36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A37" s="5">
-        <v>46091</v>
-      </c>
-      <c r="B37" t="s">
-        <v>75</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="D37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E37" t="s">
-        <v>18</v>
-      </c>
-      <c r="F37" t="s">
-        <v>127</v>
-      </c>
-      <c r="G37" t="s">
-        <v>128</v>
-      </c>
-      <c r="H37" t="s">
-        <v>16</v>
-      </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B38" t="s">
         <v>77</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="F38" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="G38" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="H38" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B39" t="s">
         <v>77</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F39" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G39" t="s">
-        <v>102</v>
+        <v>154</v>
       </c>
       <c r="H39" t="s">
         <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B40" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>17</v>
+        <v>156</v>
       </c>
       <c r="F40" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="G40" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Partidos</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2598,100 +2598,100 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="H41" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B42" t="s">
         <v>30</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="D42" t="s">
         <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F42" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="G42" t="s">
-        <v>157</v>
+        <v>91</v>
       </c>
       <c r="H42" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B43" t="s">
         <v>30</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>159</v>
+        <v>10</v>
       </c>
       <c r="G43" t="s">
-        <v>160</v>
+        <v>70</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2700,25 +2700,25 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B44" t="s">
         <v>30</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D44" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F44" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G44" t="s">
-        <v>95</v>
+        <v>163</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
@@ -2729,30 +2729,30 @@
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B45" t="s">
         <v>30</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F45" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G45" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
@@ -2768,62 +2768,62 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B46" t="s">
         <v>30</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F46" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="G46" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B47" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="D47" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="E47" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F47" t="s">
-        <v>127</v>
+        <v>25</v>
       </c>
       <c r="G47" t="s">
-        <v>128</v>
+        <v>148</v>
       </c>
       <c r="H47" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2831,132 +2831,132 @@
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B48" t="s">
-        <v>30</v>
+        <v>81</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D48" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>43</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>43</v>
+        <v>89</v>
       </c>
       <c r="G48" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B49" t="s">
         <v>81</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D49" t="s">
-        <v>85</v>
+        <v>13</v>
       </c>
       <c r="E49" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F49" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G49" t="s">
-        <v>169</v>
+        <v>148</v>
       </c>
       <c r="H49" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B50" t="s">
         <v>81</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>2</v>
+        <v>89</v>
       </c>
       <c r="G50" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H50" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B51" t="s">
         <v>81</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>150</v>
+        <v>174</v>
       </c>
       <c r="D51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F51" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="G51" t="s">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
@@ -2967,129 +2967,129 @@
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B52" t="s">
         <v>81</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>173</v>
+        <v>70</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B53" t="s">
         <v>81</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D53" t="s">
         <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="F53" t="s">
-        <v>2</v>
+        <v>45</v>
       </c>
       <c r="G53" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A54" s="5">
+        <v>46092</v>
+      </c>
+      <c r="B54" t="s">
+        <v>29</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D54" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" t="s">
+        <v>23</v>
+      </c>
+      <c r="F54" t="s">
+        <v>23</v>
+      </c>
+      <c r="G54" t="s">
+        <v>124</v>
+      </c>
+      <c r="H54" t="s">
+        <v>26</v>
+      </c>
+      <c r="I54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J53" t="str">
+      <c r="J54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A54" s="5">
-        <v>46091</v>
-      </c>
-      <c r="B54" t="s">
-        <v>81</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D54" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" t="s">
-        <v>17</v>
-      </c>
-      <c r="F54" t="s">
-        <v>17</v>
-      </c>
-      <c r="G54" t="s">
-        <v>177</v>
-      </c>
-      <c r="H54" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B55" t="s">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D55" t="s">
         <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F55" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G55" t="s">
         <v>70</v>
@@ -3099,7 +3099,7 @@
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3108,28 +3108,28 @@
     </row>
     <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B56" t="s">
         <v>29</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D56" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F56" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G56" t="s">
-        <v>180</v>
+        <v>148</v>
       </c>
       <c r="H56" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3137,12 +3137,12 @@
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B57" t="s">
         <v>29</v>
@@ -3154,13 +3154,13 @@
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F57" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G57" t="s">
-        <v>102</v>
+        <v>167</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
@@ -3171,12 +3171,12 @@
       </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B58" t="s">
         <v>29</v>
@@ -3188,29 +3188,29 @@
         <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F58" t="s">
-        <v>17</v>
+        <v>139</v>
       </c>
       <c r="G58" t="s">
-        <v>177</v>
+        <v>140</v>
       </c>
       <c r="H58" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B59" t="s">
         <v>29</v>
@@ -3222,16 +3222,16 @@
         <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="F59" t="s">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="G59" t="s">
         <v>184</v>
       </c>
       <c r="H59" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3244,93 +3244,93 @@
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B60" t="s">
-        <v>29</v>
+        <v>84</v>
       </c>
       <c r="C60" s="6" t="s">
         <v>185</v>
       </c>
       <c r="D60" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E60" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F60" t="s">
-        <v>2</v>
+        <v>89</v>
       </c>
       <c r="G60" t="s">
-        <v>119</v>
+        <v>186</v>
       </c>
       <c r="H60" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B61" t="s">
-        <v>29</v>
+        <v>84</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="F61" t="s">
-        <v>127</v>
+        <v>38</v>
       </c>
       <c r="G61" t="s">
-        <v>167</v>
+        <v>115</v>
       </c>
       <c r="H61" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B62" t="s">
+        <v>84</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>23</v>
+      </c>
+      <c r="F62" t="s">
+        <v>23</v>
+      </c>
+      <c r="G62" t="s">
         <v>86</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D62" t="s">
-        <v>13</v>
-      </c>
-      <c r="E62" t="s">
-        <v>18</v>
-      </c>
-      <c r="F62" t="s">
-        <v>127</v>
-      </c>
-      <c r="G62" t="s">
-        <v>167</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
@@ -3346,104 +3346,70 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B63" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D63" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E63" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F63" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G63" t="s">
-        <v>70</v>
+        <v>148</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
       </c>
       <c r="I63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
-        <v>46091</v>
+        <v>46092</v>
       </c>
       <c r="B64" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D64" t="s">
         <v>12</v>
       </c>
       <c r="E64" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F64" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G64" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="H64" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A65" s="5">
-        <v>46091</v>
-      </c>
-      <c r="B65" t="s">
-        <v>86</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D65" t="s">
-        <v>12</v>
-      </c>
-      <c r="E65" t="s">
-        <v>23</v>
-      </c>
-      <c r="F65" t="s">
-        <v>2</v>
-      </c>
-      <c r="G65" t="s">
-        <v>95</v>
-      </c>
-      <c r="H65" t="s">
-        <v>11</v>
-      </c>
-      <c r="I65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
       </c>
     </row>
   </sheetData>
@@ -3490,7 +3456,7 @@
         <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -3504,7 +3470,7 @@
         <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -3518,7 +3484,7 @@
         <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -3532,7 +3498,7 @@
         <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -3546,7 +3512,7 @@
         <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -3560,7 +3526,7 @@
         <v>41</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -3574,7 +3540,7 @@
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -3588,7 +3554,7 @@
         <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -3616,7 +3582,7 @@
         <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -3630,7 +3596,7 @@
         <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -3644,7 +3610,7 @@
         <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -3658,7 +3624,7 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -3672,7 +3638,7 @@
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -3686,7 +3652,7 @@
         <v>52</v>
       </c>
       <c r="E16" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -3700,7 +3666,7 @@
         <v>58</v>
       </c>
       <c r="E17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -3714,7 +3680,7 @@
         <v>59</v>
       </c>
       <c r="E18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -3728,7 +3694,7 @@
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -3742,7 +3708,7 @@
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -3756,7 +3722,7 @@
         <v>31</v>
       </c>
       <c r="E21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -3770,7 +3736,7 @@
         <v>28</v>
       </c>
       <c r="E22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -3784,7 +3750,7 @@
         <v>60</v>
       </c>
       <c r="E23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -3798,7 +3764,7 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -3812,7 +3778,7 @@
         <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -3826,7 +3792,7 @@
         <v>61</v>
       </c>
       <c r="E26" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -3840,7 +3806,7 @@
         <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Actualizo datos para reporte
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AE7B0B-FBA6-4026-B3C8-F297DFB2F06B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869E9C63-D6C3-433D-8114-6A50E7F7B5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="186">
   <si>
     <t>Fecha</t>
   </si>
@@ -273,15 +273,9 @@
     <t>Zunoticia</t>
   </si>
   <si>
-    <t>Marcha 8M</t>
-  </si>
-  <si>
     <t>Nivel</t>
   </si>
   <si>
-    <t>Sipdus</t>
-  </si>
-  <si>
     <t>Marfeca</t>
   </si>
   <si>
@@ -303,313 +297,304 @@
     <t>Deportes</t>
   </si>
   <si>
-    <t>Localización de cuerpo</t>
-  </si>
-  <si>
     <t>Alcalde</t>
   </si>
   <si>
-    <t>Hidalgo, con 10 homicidios en febrero</t>
-  </si>
-  <si>
-    <t>Homicidios</t>
-  </si>
-  <si>
-    <t>Extraen material pétreo de río</t>
-  </si>
-  <si>
-    <t>Contaminación de río</t>
-  </si>
-  <si>
-    <t>Buscan instalar Polo de Bienestar en Sahagún</t>
-  </si>
-  <si>
-    <t>Polos del Bienestar</t>
-  </si>
-  <si>
-    <t>Insuficiente donación sanguínea en el IMS</t>
-  </si>
-  <si>
-    <t>IMSS</t>
-  </si>
-  <si>
-    <t>Donación de sangre</t>
-  </si>
-  <si>
-    <t>Campesinos piden terminar obra en el canal Tlamaco</t>
-  </si>
-  <si>
-    <t>Conagua</t>
-  </si>
-  <si>
-    <t>Obra inconclusa</t>
-  </si>
-  <si>
-    <t>Reconocen la Charrería como patrimonio del estado</t>
-  </si>
-  <si>
-    <t>Patrimonio cultural</t>
-  </si>
-  <si>
-    <t>Prevén visita presidencial para inaugurar nueva nave de Mercado Libre</t>
-  </si>
-  <si>
-    <t>Visita Sheinbaum</t>
-  </si>
-  <si>
-    <t>Avanza la industria en Hidalgo en 2025</t>
-  </si>
-  <si>
     <t>Índice De Actividad Industrial</t>
   </si>
   <si>
-    <t>PATRIMONIO CULTURAL</t>
-  </si>
-  <si>
-    <t>Proponen capacitar a los choferes</t>
-  </si>
-  <si>
-    <t>Iniciativa</t>
-  </si>
-  <si>
-    <t>Poco interés en la donación de sangre</t>
-  </si>
-  <si>
-    <t>DOMINAN A SAN LUIS</t>
-  </si>
-  <si>
-    <t>GANAN, PERO  ¿A QUÉ COSTO?</t>
-  </si>
-  <si>
-    <t>APRUEBAN CREAR UNIDAD ESPECIAL CONTRA EXTORSIÓN</t>
-  </si>
-  <si>
-    <t>Prevención de Extorsión</t>
-  </si>
-  <si>
-    <t>VOLUNTARIOS PARTICIPAN EN REGENERACIÓN DE BOSQUES</t>
-  </si>
-  <si>
-    <t>Conservación Biodiversidad</t>
-  </si>
-  <si>
-    <t>La charrería ya es patrimonio cultural estatal</t>
-  </si>
-  <si>
-    <t>PARA SER REPARTIDOR,  TIENEN QUE INVERTIR HASTA 22 MIL PESOS</t>
-  </si>
-  <si>
-    <t>SERVICIOS DEL IHM AYUDARON A MARÍA A SUPERAR DUELOS</t>
-  </si>
-  <si>
-    <t>IHM</t>
-  </si>
-  <si>
     <t>Apoyo A La Mujer</t>
   </si>
   <si>
-    <t>Caen líderes criminales y homicidios bajan 28% en el primer bimestre</t>
-  </si>
-  <si>
-    <t>Incidencia Delictiva</t>
-  </si>
-  <si>
-    <t>Demanda de riñones supera las donaciones</t>
-  </si>
-  <si>
-    <t>Donación De Órganos</t>
-  </si>
-  <si>
-    <t>Buscan creación de polo de desarrollo en el Altiplano</t>
-  </si>
-  <si>
-    <t>Ferrocarrileras ofrecen empleo</t>
-  </si>
-  <si>
-    <t>Proyectos Ferroviarios</t>
-  </si>
-  <si>
-    <t>Lloran en Perú a Bryce Echenique, su escritor más querido</t>
-  </si>
-  <si>
-    <t>Surcorea, Vietnam, India... todo Asia padece ya escasez</t>
-  </si>
-  <si>
-    <t>"Estar con y para México", ventaja de Banorte</t>
-  </si>
-  <si>
-    <t>Gobierno estatal y productores pactan tecnificar sus tierras</t>
-  </si>
-  <si>
-    <t>Tecnificación De Riego</t>
-  </si>
-  <si>
-    <t>Luz verde a reforma  para reforzar lucha   contra la extorsión</t>
-  </si>
-  <si>
-    <t>Diego Rivera   logra amparo   en juzgado   de Toluca</t>
-  </si>
-  <si>
-    <t>Amparo</t>
-  </si>
-  <si>
-    <t>Controlan fuga de combustible en Tlapacoya</t>
-  </si>
-  <si>
-    <t>Pemex</t>
-  </si>
-  <si>
-    <t>Fuga de hidrocarburo</t>
-  </si>
-  <si>
-    <t>Cuando ocurre una unión de hecho entre un menor y un adulto, hay toda  una comunidad o sociedad que la ha validado y normalizado. No es solo  responsabilidad de la familia nuclear y la persona agresora, sino de todo un  sistema que día a día acepta esta conducta”.</t>
-  </si>
-  <si>
-    <t>Erradicación matrimonio infantil</t>
-  </si>
-  <si>
-    <t>Impulsa Menchaca Tercer Polo de  Desarrollo en Sahagún</t>
-  </si>
-  <si>
-    <t>Sigue pendiente futuro de Ayala  Guarro en Seguridad de Pachuca</t>
-  </si>
-  <si>
-    <t>Descartan dictámenes periciales  relación con delincuencia de los  decesos en Tolcayuca</t>
-  </si>
-  <si>
-    <t>Visitará Hidalgo  embajadora de Sudáfrica</t>
-  </si>
-  <si>
-    <t>Julio Menchaca renueva compromiso de transformar a Hidalgo</t>
-  </si>
-  <si>
-    <t>Ruta de la Transformación</t>
-  </si>
-  <si>
-    <t>Llaman mantener pozos de agua en óptimas condiciones</t>
-  </si>
-  <si>
-    <t>Agua</t>
-  </si>
-  <si>
-    <t>Rehabilitación de pozo</t>
-  </si>
-  <si>
-    <t>Avanza Sipdus en la tecnificación del campo en Francisco I. Madero</t>
-  </si>
-  <si>
-    <t>Exhortan a prevenir golpes de calor ante las altas temperaturas</t>
-  </si>
-  <si>
-    <t>Golpe de calor</t>
-  </si>
-  <si>
-    <t>Las tres dudas políticas del PRI</t>
-  </si>
-  <si>
-    <t>PRI</t>
-  </si>
-  <si>
-    <t>Militancia Partidista</t>
-  </si>
-  <si>
-    <t>¿Ahuyentan inversiones?</t>
-  </si>
-  <si>
-    <t>Ley De Ingresos</t>
-  </si>
-  <si>
-    <t>Violencia a la baja en Hidalgo: homicidios disminuyen casi 30%</t>
-  </si>
-  <si>
-    <t>Trabajador hidalguense entre víctimas de derrumbe en CDMX</t>
-  </si>
-  <si>
-    <t>Menchaca pide a Tepeapulco aclarar observaciones</t>
-  </si>
-  <si>
-    <t>Observaciones ASEH</t>
-  </si>
-  <si>
-    <t>IEEH socializa reglas de postulación con partidos y ¿Segobh?</t>
-  </si>
-  <si>
-    <t>Reunión con partidos</t>
-  </si>
-  <si>
-    <t>Cae supuesto líder de ""Los Poshcos"" en Hidalgo</t>
-  </si>
-  <si>
     <t>Combate a la delincuencia</t>
   </si>
   <si>
-    <t>Menchaca impulsa infraestructura en Tlanalapa con más de 67 mdp</t>
-  </si>
-  <si>
-    <t>Entrega Cristhian Martínez obra de más de 11 mdp</t>
-  </si>
-  <si>
-    <t>Entrega de obra</t>
-  </si>
-  <si>
-    <t>En Tepeapulco, Menchaca renueva compromiso de transformar a Hidalgo</t>
-  </si>
-  <si>
-    <t>Mi gobierno tiene disciplina financiera, no erogamos un peso sin estar debidamente comprobado</t>
-  </si>
-  <si>
-    <t>Disciplina financiera</t>
-  </si>
-  <si>
-    <t>Sin sanciones a policías por confrontación con manifestantes del 8M</t>
-  </si>
-  <si>
-    <t>Magisterio hidalguense fortalece la unidad</t>
-  </si>
-  <si>
-    <t>IEEH inaugura la 3a edición del Diplomado en violencia política de género</t>
-  </si>
-  <si>
-    <t>Violencia Política De Género</t>
-  </si>
-  <si>
-    <t>En Hidalgo, incidencia delictiva a la baja: reporte nacional</t>
-  </si>
-  <si>
-    <t>Renovación de la carpeta asfáltica desquicia la México-Pachuca</t>
-  </si>
-  <si>
-    <t>Desde Tepeapulco, Julio Menchaca renueva compromiso de transformar a Hidalgo</t>
-  </si>
-  <si>
-    <t>SSPH detiene a presunto líder del grupo delictivo ""Los Poshcos""</t>
-  </si>
-  <si>
-    <t>Fuga de oleoso causa alarma en sector de la capital</t>
-  </si>
-  <si>
-    <t>Yua viene muestra gastronómica de Santiago de Anaya</t>
-  </si>
-  <si>
-    <t>Festival Gastronómico</t>
-  </si>
-  <si>
-    <t>Reforzarán seguridad pública de Pachuca</t>
-  </si>
-  <si>
-    <t>Refuerzo De Seguridad</t>
-  </si>
-  <si>
-    <t>Crearán una unidad especializada contra la extorsión</t>
-  </si>
-  <si>
-    <t>Siempre es mejor atender los señalamientos a la seguridad en la capital, que entorpecer la coordinación que debe existir entre los mandos del estado</t>
-  </si>
-  <si>
-    <t>Anuncian inversión de 26 mdp para Ciudad Sahagún</t>
-  </si>
-  <si>
-    <t>Sheinbaum destacó la reducción del 44% de homicidios</t>
+    <t>La patineta ha salvado la vida de algunos skaters</t>
+  </si>
+  <si>
+    <t>Uso de pantallas debe regularse según la edad</t>
+  </si>
+  <si>
+    <t>Aseguran que aún hay trabas para las mujeres</t>
+  </si>
+  <si>
+    <t>Renovarán dirigencia del SNTE</t>
+  </si>
+  <si>
+    <t>Tiran en San Lázaro la reforma electoral</t>
+  </si>
+  <si>
+    <t>Reforma Electoral</t>
+  </si>
+  <si>
+    <t>Visibilizan violencia en adultos mayores</t>
+  </si>
+  <si>
+    <t>IAAMEH</t>
+  </si>
+  <si>
+    <t>Violentómetro</t>
+  </si>
+  <si>
+    <t>Movimiento Ciudadano exige 52 mil pesos para su representante</t>
+  </si>
+  <si>
+    <t>Presupuesto IEEH</t>
+  </si>
+  <si>
+    <t>Aumentan enfermedades respiratorias</t>
+  </si>
+  <si>
+    <t>IRAS</t>
+  </si>
+  <si>
+    <t>Votan contra la reforma electoral</t>
+  </si>
+  <si>
+    <t>Nueva Alianza Hidalgo, en riesgo</t>
+  </si>
+  <si>
+    <t>Fraude</t>
+  </si>
+  <si>
+    <t>Bienvenida Sudáfrica</t>
+  </si>
+  <si>
+    <t>La Reforma Electoral se podría analizar en tres planos: jurídico, político y electoral, y, por supuesto, rumbo al 2027. Jurídicamente, sí existe...</t>
+  </si>
+  <si>
+    <t>Pachuca.- La embajadora de Sudáfrica, Beryl Rose Sisulu, visitó Pachuca y recibió la bienvenida del gobernador Julio Menchaca. La diplomática hizo un recorrido por el estadio Hidalgo, donde la selección sudafricana entrenará durante el Mundial FIFA 2026.</t>
+  </si>
+  <si>
+    <t>REGRESAN TUZAS AL ESTADIO HIDALGO</t>
+  </si>
+  <si>
+    <t>LAS CASAS DEL MUNDIAL</t>
+  </si>
+  <si>
+    <t>SEIS EMPRESAS, CON CONTRATOS PESE A SANCIÓN</t>
+  </si>
+  <si>
+    <t>Inhabilitación de proveedores</t>
+  </si>
+  <si>
+    <t>FUERON PRIVADOS DE LA LIBERTAD 30 MENORES EN ENERO: SESNSP</t>
+  </si>
+  <si>
+    <t>Secuestros</t>
+  </si>
+  <si>
+    <t>Nuevo salón de Plenos será para mil asistentes</t>
+  </si>
+  <si>
+    <t>Junta de Gobierno</t>
+  </si>
+  <si>
+    <t>Salón De Plenos</t>
+  </si>
+  <si>
+    <t>SUDÁFRICA VE EN PACHUCA UN HOGAR</t>
+  </si>
+  <si>
+    <t>Coalición no está en riesgo por oposición: Rico Mercado</t>
+  </si>
+  <si>
+    <t>Alianzas Electorales</t>
+  </si>
+  <si>
+    <t>Sin cambio de placas 342 mil autos, a 2 años de iniciar programa</t>
+  </si>
+  <si>
+    <t>Reemplacamiento</t>
+  </si>
+  <si>
+    <t>Inauguración De Empresa</t>
+  </si>
+  <si>
+    <t>Por diversas irregularidades van 151 vehículos al corralón</t>
+  </si>
+  <si>
+    <t>Corralones</t>
+  </si>
+  <si>
+    <t>Confiscan autoridades celulares chips, droga...</t>
+  </si>
+  <si>
+    <t>Inspección Ceresos</t>
+  </si>
+  <si>
+    <t>Sí se avanza en seguridad, pero no se echan campanas al vuelo: Julio Menchaca</t>
+  </si>
+  <si>
+    <t>Morena activa el plan B, tras el timo del Verde y PT, sus aliados</t>
+  </si>
+  <si>
+    <t>Bienvenida. Sudáfrica resalta seguridad del país</t>
+  </si>
+  <si>
+    <t>Legisladores piden reforzar combate a la violencia de género</t>
+  </si>
+  <si>
+    <t>Erradicación Violencia De Género</t>
+  </si>
+  <si>
+    <t>PTAR acumula deuda de %100 millones por impuestos municipales</t>
+  </si>
+  <si>
+    <t>PTAR</t>
+  </si>
+  <si>
+    <t>Hidalgo y Sudáfrica se alistan para la Copa Mundial</t>
+  </si>
+  <si>
+    <t>Rechazan en San Lázaro reforma de Sheinbaum</t>
+  </si>
+  <si>
+    <t>La administración federal no perdió una reforma; compró estabilidad política y narrativa. En este tablero, el camino más corto hacia la consolidación requería, irónicamente, de una caída pública controlada”.</t>
+  </si>
+  <si>
+    <t>Lidera Hidalgo en crecimiento industrial</t>
+  </si>
+  <si>
+    <t>Se reúne Menchaca con embajadora de Sudáfrica rumbo al Mundial 2026</t>
+  </si>
+  <si>
+    <t>Podrían ampliar aforo del nuevo Salón de Plenos</t>
+  </si>
+  <si>
+    <t>Inaugura Grupo Indumil planta de blindaje en el Parque Industrial Platah</t>
+  </si>
+  <si>
+    <t>Xochiatipan se quedó sin energía eléctrica</t>
+  </si>
+  <si>
+    <t>CFE</t>
+  </si>
+  <si>
+    <t>Suministro eléctrico</t>
+  </si>
+  <si>
+    <t>Invierte gobierno 11 millones de pesos en campo huasteco</t>
+  </si>
+  <si>
+    <t>Entrega De Apoyos</t>
+  </si>
+  <si>
+    <t>Integra INE primer cabildo infantil Huejutla 2026</t>
+  </si>
+  <si>
+    <t>Cabildo Juvenil</t>
+  </si>
+  <si>
+    <t>Alcaldesa deja plantados a comités comunales</t>
+  </si>
+  <si>
+    <t>Mal desempeño de alcaldes</t>
+  </si>
+  <si>
+    <t>Adultos mayores enfrentan largas filas para cobrar pensiones</t>
+  </si>
+  <si>
+    <t>Pensión Del Bienestar</t>
+  </si>
+  <si>
+    <t>Sancionarán malas prácticas de quienes arrojen basura sobre el río de Colalambre</t>
+  </si>
+  <si>
+    <t>Sanciones por basura</t>
+  </si>
+  <si>
+    <t>Blindaje industrial en Hidalgo</t>
+  </si>
+  <si>
+    <t>Hidalgo lidera el crecimiento industrial del país</t>
+  </si>
+  <si>
+    <t>Comuneros del Mezquital ofrecen terrenos para nuevo Cereso</t>
+  </si>
+  <si>
+    <t>Construcción de Cereso</t>
+  </si>
+  <si>
+    <t>"Se puede caminar con el teléfono en la mano"</t>
+  </si>
+  <si>
+    <t>Una reforma enviada a morir</t>
+  </si>
+  <si>
+    <t>Editorial</t>
+  </si>
+  <si>
+    <t>Presidente del Congreso pide mantener el Mando Coordinado en Pachuca</t>
+  </si>
+  <si>
+    <t>Morena prepara candidaturas y deja abierta la puerta a alianzas</t>
+  </si>
+  <si>
+    <t>SSPH combate al delito en Ceresos del estado con revisiones permanentes</t>
+  </si>
+  <si>
+    <t>Bomberos de Atitalaquia imparten capacitación en emergencias con materiales peligrosos</t>
+  </si>
+  <si>
+    <t>Prevención De Riesgos</t>
+  </si>
+  <si>
+    <t>Embajadora de Sudáfrica constata la riqueza cultural, histórica y gastronómica de Hidalgo</t>
+  </si>
+  <si>
+    <t>El deporte también une al magisterio</t>
+  </si>
+  <si>
+    <t>En Tlaxcoapan realizan reunión con delegados y comisariados para prevenir incendios</t>
+  </si>
+  <si>
+    <t>Prevención de incendios</t>
+  </si>
+  <si>
+    <t>Gobierno de Tlahuelilpan, DIF municipal y fundaciones realizan jornadas de salud femenina</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo fortalece cooperación con Sudáfrica rumbo al Mundial 2026</t>
+  </si>
+  <si>
+    <t>Ya se alista la lluvia de pétalos en Mineral del Chico</t>
+  </si>
+  <si>
+    <t>Hidalgo, estado con más crecimiento industrial de México</t>
+  </si>
+  <si>
+    <t>Aseguran a cuatro personas de Los Polos, banda delictiva en Pachuca</t>
+  </si>
+  <si>
+    <t>Tuzas reciben a Tijuana en el Huracán</t>
+  </si>
+  <si>
+    <t>Hallan celulares, marihuana y 96 puntas en penal de Pachuca</t>
+  </si>
+  <si>
+    <t>Diputados rechazan iniciativa de reforma electoral</t>
+  </si>
+  <si>
+    <t>Selección de Italia vence 9-1 a México</t>
+  </si>
+  <si>
+    <t>Toman violentamente el Relleno sanitario Regional de Apan</t>
+  </si>
+  <si>
+    <t>Toma violenta</t>
+  </si>
+  <si>
+    <t>Hidalgo coopera con Sudáfrica rumbo al Mundial 2026</t>
+  </si>
+  <si>
+    <t>Blindan a fuerzas de seguridad</t>
+  </si>
+  <si>
+    <t>Industria. Con un crecimiento superior a 30%, el estado supera la media nacional</t>
+  </si>
+  <si>
+    <t>Donan unidad del tren ligero al Tec de Pachuca</t>
   </si>
 </sst>
 </file>
@@ -856,8 +841,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J64" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J64" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J69" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1223,7 +1208,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -1267,12 +1252,12 @@
         <v>8</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B2" t="s">
         <v>71</v>
@@ -1284,35 +1269,35 @@
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B3" t="s">
         <v>71</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
@@ -1324,10 +1309,10 @@
         <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1340,66 +1325,66 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B4" t="s">
         <v>71</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B5" t="s">
         <v>71</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>98</v>
+        <v>70</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1408,28 +1393,28 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B6" t="s">
         <v>71</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
         <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>100</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="H6" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1442,96 +1427,96 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B7" t="s">
         <v>71</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>97</v>
       </c>
       <c r="G7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="H7" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B8" t="s">
         <v>72</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="F8" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G8" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="H8" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B9" t="s">
         <v>72</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="F9" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="G9" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="H9" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1544,25 +1529,25 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B10" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="F10" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>103</v>
+        <v>95</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
@@ -1578,32 +1563,32 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B11" t="s">
         <v>72</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="F11" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="G11" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="H11" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Partidos</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1612,47 +1597,47 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B12" t="s">
         <v>72</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D12" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E12" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F12" t="s">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="G12" t="s">
-        <v>98</v>
+        <v>83</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B13" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1664,7 +1649,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -1678,83 +1663,83 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B15" t="s">
         <v>76</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>115</v>
+        <v>85</v>
       </c>
       <c r="H15" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B16" t="s">
         <v>76</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -1766,7 +1751,7 @@
         <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>117</v>
+        <v>83</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
@@ -1782,130 +1767,130 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B17" t="s">
         <v>76</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D17" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G17" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B18" t="s">
         <v>76</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F18" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G18" t="s">
-        <v>70</v>
+        <v>114</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B19" t="s">
         <v>76</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="F19" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="G19" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="H19" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D20" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E20" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="G20" t="s">
-        <v>124</v>
+        <v>83</v>
       </c>
       <c r="H20" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1918,59 +1903,59 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F21" t="s">
-        <v>97</v>
+        <v>2</v>
       </c>
       <c r="G21" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Partidos</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B22" t="s">
         <v>73</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D22" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E22" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="F22" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="G22" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
@@ -1981,71 +1966,71 @@
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B23" t="s">
         <v>73</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>128</v>
+        <v>183</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="F23" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="G23" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="H23" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B24" t="s">
         <v>73</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F24" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G24" t="s">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2054,236 +2039,236 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B25" t="s">
         <v>73</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F25" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G25" t="s">
-        <v>70</v>
+        <v>127</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B26" t="s">
         <v>73</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F26" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G26" t="s">
-        <v>70</v>
+        <v>89</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A27" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>59</v>
+      </c>
+      <c r="F27" t="s">
+        <v>59</v>
+      </c>
+      <c r="G27" t="s">
+        <v>87</v>
+      </c>
+      <c r="H27" t="s">
+        <v>26</v>
+      </c>
+      <c r="I27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A28" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B28" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" t="s">
+        <v>95</v>
+      </c>
+      <c r="H28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="5">
-        <v>46092</v>
-      </c>
-      <c r="B27" t="s">
-        <v>74</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="D27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" t="s">
-        <v>80</v>
-      </c>
-      <c r="F27" t="s">
-        <v>80</v>
-      </c>
-      <c r="G27" t="s">
-        <v>134</v>
-      </c>
-      <c r="H27" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="5">
-        <v>46092</v>
-      </c>
-      <c r="B28" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="D28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" t="s">
-        <v>25</v>
-      </c>
-      <c r="F28" t="s">
-        <v>25</v>
-      </c>
-      <c r="G28" t="s">
-        <v>115</v>
-      </c>
-      <c r="H28" t="s">
-        <v>26</v>
-      </c>
-      <c r="I28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D29" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E29" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="F29" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G29" t="s">
-        <v>137</v>
+        <v>83</v>
       </c>
       <c r="H29" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B30" t="s">
         <v>74</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D30" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="F30" t="s">
-        <v>139</v>
+        <v>38</v>
       </c>
       <c r="G30" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B31" t="s">
         <v>74</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="F31" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="G31" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2292,16 +2277,16 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B32" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="D32" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E32" t="s">
         <v>25</v>
@@ -2310,7 +2295,7 @@
         <v>25</v>
       </c>
       <c r="G32" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="H32" t="s">
         <v>26</v>
@@ -2324,98 +2309,98 @@
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F33" t="s">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="G33" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F34" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="H34" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B35" t="s">
         <v>75</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="F35" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="G35" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H35" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2428,16 +2413,16 @@
     </row>
     <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B36" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="D36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E36" t="s">
         <v>25</v>
@@ -2446,7 +2431,7 @@
         <v>25</v>
       </c>
       <c r="G36" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="H36" t="s">
         <v>26</v>
@@ -2462,32 +2447,32 @@
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F37" t="s">
-        <v>150</v>
+        <v>116</v>
       </c>
       <c r="G37" t="s">
-        <v>151</v>
+        <v>117</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2496,25 +2481,25 @@
     </row>
     <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B38" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="F38" t="s">
-        <v>80</v>
+        <v>59</v>
       </c>
       <c r="G38" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -2528,34 +2513,34 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B39" t="s">
         <v>77</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="D39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F39" t="s">
-        <v>17</v>
+        <v>143</v>
       </c>
       <c r="G39" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="H39" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2564,198 +2549,198 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B40" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>156</v>
+        <v>58</v>
       </c>
       <c r="F40" t="s">
-        <v>156</v>
+        <v>2</v>
       </c>
       <c r="G40" t="s">
-        <v>157</v>
+        <v>146</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B41" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
       </c>
       <c r="E41" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" t="s">
+        <v>10</v>
+      </c>
+      <c r="G41" t="s">
+        <v>148</v>
+      </c>
+      <c r="H41" t="s">
+        <v>11</v>
+      </c>
+      <c r="I41" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J41" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B42" t="s">
+        <v>77</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
         <v>17</v>
       </c>
-      <c r="F41" t="s">
-        <v>17</v>
-      </c>
-      <c r="G41" t="s">
-        <v>159</v>
-      </c>
-      <c r="H41" t="s">
+      <c r="F42" t="s">
+        <v>86</v>
+      </c>
+      <c r="G42" t="s">
+        <v>150</v>
+      </c>
+      <c r="H42" t="s">
         <v>16</v>
       </c>
-      <c r="I41" t="str">
+      <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
       </c>
-      <c r="J41" t="str">
+      <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A42" s="5">
-        <v>46092</v>
-      </c>
-      <c r="B42" t="s">
-        <v>30</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D42" t="s">
-        <v>13</v>
-      </c>
-      <c r="E42" t="s">
-        <v>18</v>
-      </c>
-      <c r="F42" t="s">
-        <v>18</v>
-      </c>
-      <c r="G42" t="s">
-        <v>91</v>
-      </c>
-      <c r="H42" t="s">
-        <v>26</v>
-      </c>
-      <c r="I42" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J42" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B43" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F43" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G43" t="s">
-        <v>70</v>
+        <v>152</v>
       </c>
       <c r="H43" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B44" t="s">
-        <v>30</v>
+        <v>77</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>162</v>
+        <v>153</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G44" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B45" t="s">
         <v>30</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>164</v>
+        <v>155</v>
       </c>
       <c r="D45" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E45" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="F45" t="s">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="G45" t="s">
-        <v>165</v>
+        <v>123</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2768,25 +2753,25 @@
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B46" t="s">
         <v>30</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="D46" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="F46" t="s">
-        <v>23</v>
+        <v>59</v>
       </c>
       <c r="G46" t="s">
-        <v>167</v>
+        <v>87</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
@@ -2802,28 +2787,28 @@
     </row>
     <row r="47" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B47" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="D47" t="s">
-        <v>83</v>
+        <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F47" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G47" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="H47" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2831,105 +2816,105 @@
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B48" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F48" t="s">
-        <v>89</v>
+        <v>25</v>
       </c>
       <c r="G48" t="s">
-        <v>170</v>
+        <v>83</v>
       </c>
       <c r="H48" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A49" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B49" t="s">
+        <v>30</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D49" t="s">
+        <v>161</v>
+      </c>
+      <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>14</v>
+      </c>
+      <c r="G49" t="s">
+        <v>95</v>
+      </c>
+      <c r="H49" t="s">
+        <v>11</v>
+      </c>
+      <c r="I49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A49" s="5">
-        <v>46092</v>
-      </c>
-      <c r="B49" t="s">
-        <v>81</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D49" t="s">
-        <v>13</v>
-      </c>
-      <c r="E49" t="s">
-        <v>25</v>
-      </c>
-      <c r="F49" t="s">
-        <v>25</v>
-      </c>
-      <c r="G49" t="s">
-        <v>148</v>
-      </c>
-      <c r="H49" t="s">
-        <v>26</v>
-      </c>
-      <c r="I49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B50" t="s">
-        <v>81</v>
+        <v>30</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="F50" t="s">
-        <v>89</v>
+        <v>38</v>
       </c>
       <c r="G50" t="s">
-        <v>173</v>
+        <v>84</v>
       </c>
       <c r="H50" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2938,127 +2923,127 @@
     </row>
     <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B51" t="s">
+        <v>30</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>19</v>
+      </c>
+      <c r="F51" t="s">
+        <v>19</v>
+      </c>
+      <c r="G51" t="s">
+        <v>120</v>
+      </c>
+      <c r="H51" t="s">
+        <v>11</v>
+      </c>
+      <c r="I51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A52" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B52" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="D52" t="s">
         <v>81</v>
       </c>
-      <c r="C51" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="D51" t="s">
-        <v>12</v>
-      </c>
-      <c r="E51" t="s">
+      <c r="E52" t="s">
         <v>23</v>
       </c>
-      <c r="F51" t="s">
-        <v>2</v>
-      </c>
-      <c r="G51" t="s">
-        <v>78</v>
-      </c>
-      <c r="H51" t="s">
-        <v>11</v>
-      </c>
-      <c r="I51" t="str">
+      <c r="F52" t="s">
+        <v>23</v>
+      </c>
+      <c r="G52" t="s">
+        <v>127</v>
+      </c>
+      <c r="H52" t="s">
+        <v>11</v>
+      </c>
+      <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J51" t="str">
+      <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A52" s="5">
-        <v>46092</v>
-      </c>
-      <c r="B52" t="s">
-        <v>81</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="D52" t="s">
-        <v>12</v>
-      </c>
-      <c r="E52" t="s">
-        <v>10</v>
-      </c>
-      <c r="F52" t="s">
-        <v>10</v>
-      </c>
-      <c r="G52" t="s">
-        <v>70</v>
-      </c>
-      <c r="H52" t="s">
-        <v>11</v>
-      </c>
-      <c r="I52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B53" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="D53" t="s">
         <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F53" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="G53" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B54" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="D54" t="s">
         <v>13</v>
       </c>
       <c r="E54" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F54" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G54" t="s">
-        <v>124</v>
+        <v>83</v>
       </c>
       <c r="H54" t="s">
         <v>26</v>
@@ -3069,169 +3054,169 @@
       </c>
       <c r="J54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B55" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="D55" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E55" t="s">
+        <v>33</v>
+      </c>
+      <c r="F55" t="s">
+        <v>2</v>
+      </c>
+      <c r="G55" t="s">
+        <v>83</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A56" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B56" t="s">
+        <v>79</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
         <v>10</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F56" t="s">
         <v>10</v>
       </c>
-      <c r="G55" t="s">
+      <c r="G56" t="s">
         <v>70</v>
       </c>
-      <c r="H55" t="s">
-        <v>11</v>
-      </c>
-      <c r="I55" t="str">
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J55" t="str">
+      <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A56" s="5">
-        <v>46092</v>
-      </c>
-      <c r="B56" t="s">
-        <v>29</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D56" t="s">
-        <v>12</v>
-      </c>
-      <c r="E56" t="s">
-        <v>25</v>
-      </c>
-      <c r="F56" t="s">
-        <v>25</v>
-      </c>
-      <c r="G56" t="s">
-        <v>148</v>
-      </c>
-      <c r="H56" t="s">
-        <v>26</v>
-      </c>
-      <c r="I56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B57" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F57" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G57" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B58" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>182</v>
+        <v>171</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F58" t="s">
-        <v>139</v>
+        <v>17</v>
       </c>
       <c r="G58" t="s">
-        <v>140</v>
+        <v>88</v>
       </c>
       <c r="H58" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B59" t="s">
         <v>29</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>183</v>
+        <v>172</v>
       </c>
       <c r="D59" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E59" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F59" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="G59" t="s">
-        <v>184</v>
+        <v>83</v>
       </c>
       <c r="H59" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3239,37 +3224,37 @@
       </c>
       <c r="J59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B60" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="D60" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F60" t="s">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="G60" t="s">
-        <v>186</v>
+        <v>70</v>
       </c>
       <c r="H60" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3278,47 +3263,47 @@
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B61" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>187</v>
+        <v>174</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="F61" t="s">
-        <v>38</v>
+        <v>59</v>
       </c>
       <c r="G61" t="s">
-        <v>115</v>
+        <v>87</v>
       </c>
       <c r="H61" t="s">
         <v>26</v>
       </c>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B62" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>188</v>
+        <v>175</v>
       </c>
       <c r="D62" t="s">
         <v>12</v>
@@ -3330,7 +3315,7 @@
         <v>23</v>
       </c>
       <c r="G62" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
@@ -3346,70 +3331,240 @@
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B63" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D63" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F63" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G63" t="s">
-        <v>148</v>
+        <v>70</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
       </c>
       <c r="I63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
-        <v>46092</v>
+        <v>46093</v>
       </c>
       <c r="B64" t="s">
-        <v>84</v>
+        <v>29</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>190</v>
+        <v>176</v>
       </c>
       <c r="D64" t="s">
         <v>12</v>
       </c>
       <c r="E64" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F64" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G64" t="s">
-        <v>124</v>
+        <v>85</v>
       </c>
       <c r="H64" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A65" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B65" t="s">
+        <v>82</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D65" t="s">
+        <v>13</v>
+      </c>
+      <c r="E65" t="s">
+        <v>23</v>
+      </c>
+      <c r="F65" t="s">
+        <v>23</v>
+      </c>
+      <c r="G65" t="s">
+        <v>127</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A66" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B66" t="s">
+        <v>82</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>10</v>
+      </c>
+      <c r="F66" t="s">
+        <v>10</v>
+      </c>
+      <c r="G66" t="s">
+        <v>95</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A67" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B67" t="s">
+        <v>82</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" t="s">
+        <v>10</v>
+      </c>
+      <c r="G67" t="s">
+        <v>85</v>
+      </c>
+      <c r="H67" t="s">
+        <v>11</v>
+      </c>
+      <c r="I67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A68" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B68" t="s">
+        <v>82</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" t="s">
+        <v>17</v>
+      </c>
+      <c r="F68" t="s">
+        <v>86</v>
+      </c>
+      <c r="G68" t="s">
+        <v>181</v>
+      </c>
+      <c r="H68" t="s">
+        <v>16</v>
+      </c>
+      <c r="I68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A69" s="5">
+        <v>46093</v>
+      </c>
+      <c r="B69" t="s">
+        <v>82</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" t="s">
+        <v>43</v>
+      </c>
+      <c r="F69" t="s">
+        <v>43</v>
+      </c>
+      <c r="G69" t="s">
+        <v>83</v>
+      </c>
+      <c r="H69" t="s">
+        <v>11</v>
+      </c>
+      <c r="I69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
       </c>
     </row>
   </sheetData>
@@ -3442,7 +3597,7 @@
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -3456,7 +3611,7 @@
         <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -3470,7 +3625,7 @@
         <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -3484,7 +3639,7 @@
         <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -3498,7 +3653,7 @@
         <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -3512,7 +3667,7 @@
         <v>40</v>
       </c>
       <c r="E6" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -3526,7 +3681,7 @@
         <v>41</v>
       </c>
       <c r="E7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -3540,7 +3695,7 @@
         <v>41</v>
       </c>
       <c r="E8" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -3554,7 +3709,7 @@
         <v>42</v>
       </c>
       <c r="E9" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -3582,7 +3737,7 @@
         <v>43</v>
       </c>
       <c r="E11" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -3596,7 +3751,7 @@
         <v>44</v>
       </c>
       <c r="E12" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -3610,7 +3765,7 @@
         <v>44</v>
       </c>
       <c r="E13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -3624,7 +3779,7 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -3638,7 +3793,7 @@
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -3652,7 +3807,7 @@
         <v>52</v>
       </c>
       <c r="E16" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -3666,7 +3821,7 @@
         <v>58</v>
       </c>
       <c r="E17" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -3680,7 +3835,7 @@
         <v>59</v>
       </c>
       <c r="E18" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -3694,7 +3849,7 @@
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -3708,7 +3863,7 @@
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -3722,7 +3877,7 @@
         <v>31</v>
       </c>
       <c r="E21" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -3736,7 +3891,7 @@
         <v>28</v>
       </c>
       <c r="E22" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -3750,7 +3905,7 @@
         <v>60</v>
       </c>
       <c r="E23" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -3764,7 +3919,7 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -3778,7 +3933,7 @@
         <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -3792,7 +3947,7 @@
         <v>61</v>
       </c>
       <c r="E26" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -3806,7 +3961,7 @@
         <v>33</v>
       </c>
       <c r="E27" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Reporte 13 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869E9C63-D6C3-433D-8114-6A50E7F7B5B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF76B69-5FAF-4177-91C4-4C547215B118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="197">
   <si>
     <t>Fecha</t>
   </si>
@@ -291,310 +291,343 @@
     <t>Mundial De Futbol</t>
   </si>
   <si>
-    <t>Mando Coordinado</t>
-  </si>
-  <si>
     <t>Deportes</t>
   </si>
   <si>
     <t>Alcalde</t>
   </si>
   <si>
-    <t>Índice De Actividad Industrial</t>
-  </si>
-  <si>
-    <t>Apoyo A La Mujer</t>
-  </si>
-  <si>
     <t>Combate a la delincuencia</t>
   </si>
   <si>
-    <t>La patineta ha salvado la vida de algunos skaters</t>
-  </si>
-  <si>
-    <t>Uso de pantallas debe regularse según la edad</t>
-  </si>
-  <si>
-    <t>Aseguran que aún hay trabas para las mujeres</t>
-  </si>
-  <si>
-    <t>Renovarán dirigencia del SNTE</t>
-  </si>
-  <si>
-    <t>Tiran en San Lázaro la reforma electoral</t>
-  </si>
-  <si>
     <t>Reforma Electoral</t>
   </si>
   <si>
-    <t>Visibilizan violencia en adultos mayores</t>
-  </si>
-  <si>
-    <t>IAAMEH</t>
-  </si>
-  <si>
-    <t>Violentómetro</t>
-  </si>
-  <si>
-    <t>Movimiento Ciudadano exige 52 mil pesos para su representante</t>
-  </si>
-  <si>
-    <t>Presupuesto IEEH</t>
-  </si>
-  <si>
-    <t>Aumentan enfermedades respiratorias</t>
-  </si>
-  <si>
-    <t>IRAS</t>
-  </si>
-  <si>
-    <t>Votan contra la reforma electoral</t>
-  </si>
-  <si>
-    <t>Nueva Alianza Hidalgo, en riesgo</t>
-  </si>
-  <si>
     <t>Fraude</t>
   </si>
   <si>
-    <t>Bienvenida Sudáfrica</t>
-  </si>
-  <si>
-    <t>La Reforma Electoral se podría analizar en tres planos: jurídico, político y electoral, y, por supuesto, rumbo al 2027. Jurídicamente, sí existe...</t>
-  </si>
-  <si>
-    <t>Pachuca.- La embajadora de Sudáfrica, Beryl Rose Sisulu, visitó Pachuca y recibió la bienvenida del gobernador Julio Menchaca. La diplomática hizo un recorrido por el estadio Hidalgo, donde la selección sudafricana entrenará durante el Mundial FIFA 2026.</t>
-  </si>
-  <si>
-    <t>REGRESAN TUZAS AL ESTADIO HIDALGO</t>
-  </si>
-  <si>
-    <t>LAS CASAS DEL MUNDIAL</t>
-  </si>
-  <si>
-    <t>SEIS EMPRESAS, CON CONTRATOS PESE A SANCIÓN</t>
-  </si>
-  <si>
-    <t>Inhabilitación de proveedores</t>
-  </si>
-  <si>
-    <t>FUERON PRIVADOS DE LA LIBERTAD 30 MENORES EN ENERO: SESNSP</t>
-  </si>
-  <si>
-    <t>Secuestros</t>
-  </si>
-  <si>
-    <t>Nuevo salón de Plenos será para mil asistentes</t>
-  </si>
-  <si>
-    <t>Junta de Gobierno</t>
-  </si>
-  <si>
-    <t>Salón De Plenos</t>
-  </si>
-  <si>
-    <t>SUDÁFRICA VE EN PACHUCA UN HOGAR</t>
-  </si>
-  <si>
-    <t>Coalición no está en riesgo por oposición: Rico Mercado</t>
-  </si>
-  <si>
-    <t>Alianzas Electorales</t>
-  </si>
-  <si>
-    <t>Sin cambio de placas 342 mil autos, a 2 años de iniciar programa</t>
-  </si>
-  <si>
-    <t>Reemplacamiento</t>
-  </si>
-  <si>
-    <t>Inauguración De Empresa</t>
-  </si>
-  <si>
-    <t>Por diversas irregularidades van 151 vehículos al corralón</t>
-  </si>
-  <si>
-    <t>Corralones</t>
-  </si>
-  <si>
-    <t>Confiscan autoridades celulares chips, droga...</t>
-  </si>
-  <si>
-    <t>Inspección Ceresos</t>
-  </si>
-  <si>
-    <t>Sí se avanza en seguridad, pero no se echan campanas al vuelo: Julio Menchaca</t>
-  </si>
-  <si>
-    <t>Morena activa el plan B, tras el timo del Verde y PT, sus aliados</t>
-  </si>
-  <si>
-    <t>Bienvenida. Sudáfrica resalta seguridad del país</t>
-  </si>
-  <si>
-    <t>Legisladores piden reforzar combate a la violencia de género</t>
-  </si>
-  <si>
-    <t>Erradicación Violencia De Género</t>
-  </si>
-  <si>
-    <t>PTAR acumula deuda de %100 millones por impuestos municipales</t>
-  </si>
-  <si>
-    <t>PTAR</t>
-  </si>
-  <si>
-    <t>Hidalgo y Sudáfrica se alistan para la Copa Mundial</t>
-  </si>
-  <si>
-    <t>Rechazan en San Lázaro reforma de Sheinbaum</t>
-  </si>
-  <si>
-    <t>La administración federal no perdió una reforma; compró estabilidad política y narrativa. En este tablero, el camino más corto hacia la consolidación requería, irónicamente, de una caída pública controlada”.</t>
-  </si>
-  <si>
-    <t>Lidera Hidalgo en crecimiento industrial</t>
-  </si>
-  <si>
-    <t>Se reúne Menchaca con embajadora de Sudáfrica rumbo al Mundial 2026</t>
-  </si>
-  <si>
-    <t>Podrían ampliar aforo del nuevo Salón de Plenos</t>
-  </si>
-  <si>
-    <t>Inaugura Grupo Indumil planta de blindaje en el Parque Industrial Platah</t>
-  </si>
-  <si>
-    <t>Xochiatipan se quedó sin energía eléctrica</t>
-  </si>
-  <si>
-    <t>CFE</t>
-  </si>
-  <si>
-    <t>Suministro eléctrico</t>
-  </si>
-  <si>
-    <t>Invierte gobierno 11 millones de pesos en campo huasteco</t>
-  </si>
-  <si>
-    <t>Entrega De Apoyos</t>
-  </si>
-  <si>
-    <t>Integra INE primer cabildo infantil Huejutla 2026</t>
-  </si>
-  <si>
-    <t>Cabildo Juvenil</t>
-  </si>
-  <si>
-    <t>Alcaldesa deja plantados a comités comunales</t>
-  </si>
-  <si>
-    <t>Mal desempeño de alcaldes</t>
-  </si>
-  <si>
-    <t>Adultos mayores enfrentan largas filas para cobrar pensiones</t>
-  </si>
-  <si>
-    <t>Pensión Del Bienestar</t>
-  </si>
-  <si>
-    <t>Sancionarán malas prácticas de quienes arrojen basura sobre el río de Colalambre</t>
-  </si>
-  <si>
-    <t>Sanciones por basura</t>
-  </si>
-  <si>
-    <t>Blindaje industrial en Hidalgo</t>
-  </si>
-  <si>
-    <t>Hidalgo lidera el crecimiento industrial del país</t>
-  </si>
-  <si>
-    <t>Comuneros del Mezquital ofrecen terrenos para nuevo Cereso</t>
-  </si>
-  <si>
-    <t>Construcción de Cereso</t>
-  </si>
-  <si>
-    <t>"Se puede caminar con el teléfono en la mano"</t>
-  </si>
-  <si>
-    <t>Una reforma enviada a morir</t>
-  </si>
-  <si>
     <t>Editorial</t>
   </si>
   <si>
-    <t>Presidente del Congreso pide mantener el Mando Coordinado en Pachuca</t>
-  </si>
-  <si>
-    <t>Morena prepara candidaturas y deja abierta la puerta a alianzas</t>
-  </si>
-  <si>
-    <t>SSPH combate al delito en Ceresos del estado con revisiones permanentes</t>
-  </si>
-  <si>
-    <t>Bomberos de Atitalaquia imparten capacitación en emergencias con materiales peligrosos</t>
-  </si>
-  <si>
-    <t>Prevención De Riesgos</t>
-  </si>
-  <si>
-    <t>Embajadora de Sudáfrica constata la riqueza cultural, histórica y gastronómica de Hidalgo</t>
-  </si>
-  <si>
-    <t>El deporte también une al magisterio</t>
-  </si>
-  <si>
-    <t>En Tlaxcoapan realizan reunión con delegados y comisariados para prevenir incendios</t>
-  </si>
-  <si>
-    <t>Prevención de incendios</t>
-  </si>
-  <si>
-    <t>Gobierno de Tlahuelilpan, DIF municipal y fundaciones realizan jornadas de salud femenina</t>
-  </si>
-  <si>
-    <t>Gobierno de Hidalgo fortalece cooperación con Sudáfrica rumbo al Mundial 2026</t>
-  </si>
-  <si>
-    <t>Ya se alista la lluvia de pétalos en Mineral del Chico</t>
-  </si>
-  <si>
-    <t>Hidalgo, estado con más crecimiento industrial de México</t>
-  </si>
-  <si>
-    <t>Aseguran a cuatro personas de Los Polos, banda delictiva en Pachuca</t>
-  </si>
-  <si>
-    <t>Tuzas reciben a Tijuana en el Huracán</t>
-  </si>
-  <si>
-    <t>Hallan celulares, marihuana y 96 puntas en penal de Pachuca</t>
-  </si>
-  <si>
-    <t>Diputados rechazan iniciativa de reforma electoral</t>
-  </si>
-  <si>
-    <t>Selección de Italia vence 9-1 a México</t>
-  </si>
-  <si>
-    <t>Toman violentamente el Relleno sanitario Regional de Apan</t>
-  </si>
-  <si>
-    <t>Toma violenta</t>
-  </si>
-  <si>
-    <t>Hidalgo coopera con Sudáfrica rumbo al Mundial 2026</t>
-  </si>
-  <si>
-    <t>Blindan a fuerzas de seguridad</t>
-  </si>
-  <si>
-    <t>Industria. Con un crecimiento superior a 30%, el estado supera la media nacional</t>
-  </si>
-  <si>
-    <t>Donan unidad del tren ligero al Tec de Pachuca</t>
+    <t>Crean reglas para peleas profesionales</t>
+  </si>
+  <si>
+    <t>Sheinbaum presenta su plan B electoral</t>
+  </si>
+  <si>
+    <t>Plan B</t>
+  </si>
+  <si>
+    <t>Pequeños comercios prefieren el efectivo</t>
+  </si>
+  <si>
+    <t>Irán reitera cierre de ruta clave del crudo</t>
+  </si>
+  <si>
+    <t>Temas internacionales</t>
+  </si>
+  <si>
+    <t>Acusa CNTE falta defensa sindical</t>
+  </si>
+  <si>
+    <t>Leyenda de Las Calderas del Progreso</t>
+  </si>
+  <si>
+    <t>Escamoles a precio alto por sobreexplotación</t>
+  </si>
+  <si>
+    <t>Línea de alta tensión detonará más inversiones</t>
+  </si>
+  <si>
+    <t>Atracción De Inversiones</t>
+  </si>
+  <si>
+    <t>HACEN SU LUCHITA</t>
+  </si>
+  <si>
+    <t>Iniciativa</t>
+  </si>
+  <si>
+    <t>Llegan las rutas a Almoloya</t>
+  </si>
+  <si>
+    <t>Ruta de la Transformación</t>
+  </si>
+  <si>
+    <t>Regidores de 5 municipios cuestan 42 mdp</t>
+  </si>
+  <si>
+    <t>Regidor</t>
+  </si>
+  <si>
+    <t>Salarios Regidores</t>
+  </si>
+  <si>
+    <t>Hay algo que conviene dejar claro desde el principio: la transparencia no pertenece a las instituciones, pertenece a la ciudadanía, los...</t>
+  </si>
+  <si>
+    <t>Combate a la corrupción</t>
+  </si>
+  <si>
+    <t>C4 en Mineral de la Reforma</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>DURA PRUEBA PARA LA ZAGA</t>
+  </si>
+  <si>
+    <t>SUEÑAN CON  EL MUNDIAL</t>
+  </si>
+  <si>
+    <t>LA CENTRAL DE ABASTOS, “UNA BOMBA DE TIEMPO”</t>
+  </si>
+  <si>
+    <t>Central De Abastos</t>
+  </si>
+  <si>
+    <t>PREPARAN LA EDICIÓN  2026 DEL VIACRUCIS  DEL BARRIO LAS LAJAS</t>
+  </si>
+  <si>
+    <t>Viacrucis</t>
+  </si>
+  <si>
+    <t>Impiden la salida de alumnos de la UAEH</t>
+  </si>
+  <si>
+    <t>Seguridad</t>
+  </si>
+  <si>
+    <t>TANIA MEZA NO  PODRÁ RETOMAR INICIATIVA SOBRE EL PERIODISMO</t>
+  </si>
+  <si>
+    <t>GLMorena</t>
+  </si>
+  <si>
+    <t>Ley de Protección a Periodistas</t>
+  </si>
+  <si>
+    <t>Denuncian violación a intimidad en 73% de municipios del estado</t>
+  </si>
+  <si>
+    <t>Violencia digital</t>
+  </si>
+  <si>
+    <t>Hacen frente en Pachuca a bandas y narcomenudistas</t>
+  </si>
+  <si>
+    <t>Destinan 100 mdp para la construcción de C4</t>
+  </si>
+  <si>
+    <t>Se imponen concesionados y Guardia disuade a Uber y Didi</t>
+  </si>
+  <si>
+    <t>En 6 cabildos ven un posible recorte a las regidurías</t>
+  </si>
+  <si>
+    <t>Operativos de movilidad detectan 43 taxis que dan servicios sin tener placas</t>
+  </si>
+  <si>
+    <t>Operativo de transporte</t>
+  </si>
+  <si>
+    <t>Gana chileno Radic el Nóbel de arquitectura</t>
+  </si>
+  <si>
+    <t>El Plan B es una iniciativa constitucional, no para leyes secundarias: Morena</t>
+  </si>
+  <si>
+    <t>El beisbol como una expresión de diversidad</t>
+  </si>
+  <si>
+    <t>Hidalgo destina  $11 millones para  sus 30 diputados</t>
+  </si>
+  <si>
+    <t>Sube a 20  el número de muertes  por influenza</t>
+  </si>
+  <si>
+    <t>Influenza</t>
+  </si>
+  <si>
+    <t>Avanzan trabajos para la reubicación de ambulantes</t>
+  </si>
+  <si>
+    <t>Ambulantaje</t>
+  </si>
+  <si>
+    <t>Presenta  Sheinbaum su  plan electoral B</t>
+  </si>
+  <si>
+    <t>Leyes hay, que las cumplan es otra cosa, y el comentario viene a cuento porque de nueva cuenta la Ley de  Protección a los Derechos de los Periodistas, impulsada por los legisladores, en este caso concreto por la  diputada morenista Tania Meza Escorza, fue frenada cuando apenas iba a entrar a discusión”.</t>
+  </si>
+  <si>
+    <t>Anuncia Menchaca nuevos proyectos de  infraestructura para Almoloya</t>
+  </si>
+  <si>
+    <t>Reconoce embajadora de Sudáfrica  la seguridad que priva en Hidalgo</t>
+  </si>
+  <si>
+    <t>Investiga Fiscalía de Delitos Electorales  presunto fraude cibernético contra Panalh</t>
+  </si>
+  <si>
+    <t>Fede</t>
+  </si>
+  <si>
+    <t>Lanzan alerta roja por fuertes rachas de  viento en Hidalgo</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>Alerta Meteorológica</t>
+  </si>
+  <si>
+    <t>CEAA advierte sobre la temporada de estiaje en Hidalgo</t>
+  </si>
+  <si>
+    <t>Sipdus</t>
+  </si>
+  <si>
+    <t>CEAA</t>
+  </si>
+  <si>
+    <t>Mitigación estiaje</t>
+  </si>
+  <si>
+    <t>El carnaval #Huejutla 2026 ya está aquí</t>
+  </si>
+  <si>
+    <t>Carnavales</t>
+  </si>
+  <si>
+    <t>Julio Menchaca destina más de 57 mdp para obras públicas en Almoloya</t>
+  </si>
+  <si>
+    <t>Solicitan a delegados evitar tiradero clandestinos de basura</t>
+  </si>
+  <si>
+    <t>Basurero Clandestino</t>
+  </si>
+  <si>
+    <t>Llama obispo de Huejutla a vivir la cuaresma con reflexón y conversión</t>
+  </si>
+  <si>
+    <t>Deteriorada e intransitable la carretera federal 102</t>
+  </si>
+  <si>
+    <t>SICT</t>
+  </si>
+  <si>
+    <t>Carretera En Mal Estado</t>
+  </si>
+  <si>
+    <t>Medécigo busca 100 millones para nuevo C4</t>
+  </si>
+  <si>
+    <t>Claudia Sheinbaum plantea reducir gastos en congresos</t>
+  </si>
+  <si>
+    <t>Irrumpen en Cabildo de Tepeji y agreden al oficial mayor</t>
+  </si>
+  <si>
+    <t>Agresión</t>
+  </si>
+  <si>
+    <t>Entre mareos y miedo</t>
+  </si>
+  <si>
+    <t>Pemex</t>
+  </si>
+  <si>
+    <t>Fuga de hidrocarburo</t>
+  </si>
+  <si>
+    <t>MC Hidalgo reclamando lo que votó recortar</t>
+  </si>
+  <si>
+    <t>De 45 millones en Tepeapulco, exalcaldesa debe solventar 25</t>
+  </si>
+  <si>
+    <t>Observaciones ASEH</t>
+  </si>
+  <si>
+    <t>Menchaca destina 57 millones en Almoloya</t>
+  </si>
+  <si>
+    <t>Diputados de Hidalgo se dividen en votación de Reforma Electoral</t>
+  </si>
+  <si>
+    <t>Prevén rachas de viento fuertes en Hidalgo; piden extremar precauciones</t>
+  </si>
+  <si>
+    <t>Claudia Sandoval camina y escucha al pueblo, ahora en Tezoquipa</t>
+  </si>
+  <si>
+    <t>Atención a la ciudadanía</t>
+  </si>
+  <si>
+    <t>Menchaca destina más de 57 mdp para obras públicas en Almoloya</t>
+  </si>
+  <si>
+    <t>Realizan Feria de Servicios municipales</t>
+  </si>
+  <si>
+    <t>Feria de servicios</t>
+  </si>
+  <si>
+    <t>Se fortalece el diálogo entre juventudes y autoridades en encuentro estatal</t>
+  </si>
+  <si>
+    <t>Atención a jóvenes</t>
+  </si>
+  <si>
+    <t>Xochitlán de las Flores se transforma mediante diálogo y el trabajo en conjunto</t>
+  </si>
+  <si>
+    <t>Diálogo institucional fortalece al magisterio hidalguense</t>
+  </si>
+  <si>
+    <t>Menchaca pide denunciar formalmente a funcionarios señalados en tendederos del 8M</t>
+  </si>
+  <si>
+    <t>Marcha 8M</t>
+  </si>
+  <si>
+    <t>Fuertes rachas de viento en HIdalgo</t>
+  </si>
+  <si>
+    <t>Lanzan convocatoria 2016 para apoyar a cuidadores de personas con discapacidad</t>
+  </si>
+  <si>
+    <t>Cuidadores De Adultos Mayores</t>
+  </si>
+  <si>
+    <t>¿Buscas trabajo? este viernes realizarán feria nacional de empleo para las mujeres</t>
+  </si>
+  <si>
+    <t>Feria De Empleo</t>
+  </si>
+  <si>
+    <t>Embajadora de Sudáfrica recorrió más puntos de la entidad de cara al mundial</t>
+  </si>
+  <si>
+    <t>Tuzas vencen 2-0 a Tijuana en liga MX femenil</t>
+  </si>
+  <si>
+    <t>Atraparon a 4 vinculados a la célula de ""Los Polos""</t>
+  </si>
+  <si>
+    <t>Emiten recomendaciones contra la extorsión sexual digital</t>
+  </si>
+  <si>
+    <t>Morena y la 4T tienen fisuras, como quedó demostrado con los votos en contra de legisladores morenistas en la fallida Reforma Electoral</t>
+  </si>
+  <si>
+    <t>Destinan más de 57 mdp para obras en Almoloya</t>
+  </si>
+  <si>
+    <t>Crean iniciativa para homologar investigación de feminicidios</t>
   </si>
 </sst>
 </file>
@@ -841,8 +874,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J69" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J71" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J71" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1208,7 +1241,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -1257,7 +1290,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B2" t="s">
         <v>71</v>
@@ -1269,20 +1302,20 @@
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G2" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1291,7 +1324,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B3" t="s">
         <v>71</v>
@@ -1303,20 +1336,20 @@
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1325,16 +1358,16 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B4" t="s">
         <v>71</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -1359,13 +1392,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B5" t="s">
         <v>71</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
@@ -1377,7 +1410,7 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
@@ -1393,32 +1426,32 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B6" t="s">
         <v>71</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1427,66 +1460,66 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B7" t="s">
         <v>71</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>97</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J7" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8" s="5">
+        <v>46094</v>
+      </c>
+      <c r="B8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="H7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J7" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A8" s="5">
-        <v>46093</v>
-      </c>
-      <c r="B8" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>99</v>
-      </c>
       <c r="D8" t="s">
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="H8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1495,28 +1528,28 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B9" t="s">
         <v>72</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="F9" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="H9" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1529,32 +1562,32 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B10" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1563,149 +1596,149 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B11" t="s">
         <v>72</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" t="s">
         <v>104</v>
       </c>
-      <c r="D11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" t="s">
-        <v>51</v>
-      </c>
-      <c r="F11" t="s">
-        <v>51</v>
-      </c>
-      <c r="G11" t="s">
-        <v>105</v>
-      </c>
       <c r="H11" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B12" t="s">
         <v>72</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
         <v>106</v>
       </c>
-      <c r="D12" t="s">
-        <v>9</v>
-      </c>
-      <c r="E12" t="s">
-        <v>33</v>
-      </c>
-      <c r="F12" t="s">
-        <v>33</v>
-      </c>
       <c r="G12" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="H12" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B13" t="s">
         <v>72</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="F13" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G13" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B14" t="s">
         <v>72</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="G14" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B15" t="s">
         <v>76</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -1717,7 +1750,7 @@
         <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
@@ -1733,13 +1766,13 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B16" t="s">
         <v>76</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -1751,7 +1784,7 @@
         <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
@@ -1767,25 +1800,25 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B17" t="s">
         <v>76</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D17" t="s">
         <v>13</v>
       </c>
       <c r="E17" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="F17" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="G17" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
@@ -1801,59 +1834,59 @@
     </row>
     <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B18" t="s">
         <v>76</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F18" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B19" t="s">
         <v>76</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>38</v>
+        <v>64</v>
       </c>
       <c r="F19" t="s">
-        <v>116</v>
+        <v>64</v>
       </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H19" t="s">
         <v>11</v>
@@ -1867,98 +1900,98 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B20" t="s">
         <v>76</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D20" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="F20" t="s">
-        <v>33</v>
+        <v>121</v>
       </c>
       <c r="G20" t="s">
-        <v>83</v>
+        <v>122</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J20" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A21" s="5">
+        <v>46094</v>
+      </c>
+      <c r="B21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+      <c r="E21" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" t="s">
+        <v>18</v>
+      </c>
+      <c r="G21" t="s">
+        <v>124</v>
+      </c>
+      <c r="H21" t="s">
+        <v>11</v>
+      </c>
+      <c r="I21" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J20" t="str">
+      <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A21" s="5">
-        <v>46093</v>
-      </c>
-      <c r="B21" t="s">
-        <v>76</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="D21" t="s">
-        <v>12</v>
-      </c>
-      <c r="E21" t="s">
-        <v>19</v>
-      </c>
-      <c r="F21" t="s">
-        <v>2</v>
-      </c>
-      <c r="G21" t="s">
-        <v>120</v>
-      </c>
-      <c r="H21" t="s">
-        <v>11</v>
-      </c>
-      <c r="I21" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J21" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B22" t="s">
         <v>73</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="F22" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="G22" t="s">
-        <v>122</v>
+        <v>86</v>
       </c>
       <c r="H22" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1971,66 +2004,66 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B23" t="s">
         <v>73</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>183</v>
+        <v>126</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="F23" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="G23" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B24" t="s">
         <v>73</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D24" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E24" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F24" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>125</v>
+        <v>83</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2039,59 +2072,59 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B25" t="s">
         <v>73</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F25" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G25" t="s">
-        <v>127</v>
+        <v>107</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B26" t="s">
         <v>73</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F26" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G26" t="s">
-        <v>89</v>
+        <v>130</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
@@ -2102,52 +2135,52 @@
       </c>
       <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B27" t="s">
         <v>73</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>184</v>
+        <v>131</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="F27" t="s">
-        <v>59</v>
+        <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
       <c r="H27" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B28" t="s">
         <v>73</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
@@ -2159,7 +2192,7 @@
         <v>19</v>
       </c>
       <c r="G28" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H28" t="s">
         <v>11</v>
@@ -2175,229 +2208,229 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B29" t="s">
         <v>73</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D29" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H29" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B30" t="s">
         <v>74</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D30" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E30" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="F30" t="s">
-        <v>38</v>
+        <v>106</v>
       </c>
       <c r="G30" t="s">
-        <v>132</v>
+        <v>107</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B31" t="s">
         <v>74</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F31" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G31" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B32" t="s">
         <v>74</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D32" t="s">
         <v>9</v>
       </c>
       <c r="E32" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F32" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G32" t="s">
-        <v>83</v>
+        <v>138</v>
       </c>
       <c r="H32" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B33" t="s">
         <v>74</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F33" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B34" t="s">
         <v>74</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="F34" t="s">
-        <v>14</v>
+        <v>121</v>
       </c>
       <c r="G34" t="s">
-        <v>95</v>
+        <v>122</v>
       </c>
       <c r="H34" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B35" t="s">
         <v>75</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D35" t="s">
         <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="F35" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="G35" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="H35" t="s">
         <v>26</v>
@@ -2408,33 +2441,33 @@
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B36" t="s">
         <v>75</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F36" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="G36" t="s">
         <v>83</v>
       </c>
       <c r="H36" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2442,64 +2475,64 @@
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B37" t="s">
         <v>75</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="F37" t="s">
-        <v>116</v>
+        <v>144</v>
       </c>
       <c r="G37" t="s">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B38" t="s">
         <v>75</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="F38" t="s">
-        <v>59</v>
+        <v>146</v>
       </c>
       <c r="G38" t="s">
-        <v>123</v>
+        <v>147</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -2515,115 +2548,115 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B39" t="s">
         <v>77</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="D39" t="s">
         <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="F39" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="G39" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H39" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B40" t="s">
         <v>77</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>58</v>
+        <v>17</v>
       </c>
       <c r="F40" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G40" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B41" t="s">
         <v>77</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F41" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G41" t="s">
-        <v>148</v>
+        <v>104</v>
       </c>
       <c r="H41" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B42" t="s">
         <v>77</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
@@ -2632,13 +2665,13 @@
         <v>17</v>
       </c>
       <c r="F42" t="s">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="G42" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="H42" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2649,68 +2682,68 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B43" t="s">
         <v>77</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G43" t="s">
-        <v>152</v>
+        <v>70</v>
       </c>
       <c r="H43" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B44" t="s">
         <v>77</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>159</v>
       </c>
       <c r="G44" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="H44" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2719,368 +2752,368 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B45" t="s">
         <v>30</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D45" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="F45" t="s">
-        <v>59</v>
+        <v>85</v>
       </c>
       <c r="G45" t="s">
-        <v>123</v>
+        <v>111</v>
       </c>
       <c r="H45" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B46" t="s">
         <v>30</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D46" t="s">
         <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="F46" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B47" t="s">
         <v>30</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="D47" t="s">
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G47" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B48" t="s">
         <v>30</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="D48" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E48" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F48" t="s">
-        <v>25</v>
+        <v>166</v>
       </c>
       <c r="G48" t="s">
-        <v>83</v>
+        <v>167</v>
       </c>
       <c r="H48" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B49" t="s">
         <v>30</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D49" t="s">
-        <v>161</v>
+        <v>89</v>
       </c>
       <c r="E49" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="F49" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G49" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="H49" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Partidos</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B50" t="s">
         <v>30</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>38</v>
+        <v>85</v>
       </c>
       <c r="G50" t="s">
-        <v>84</v>
+        <v>170</v>
       </c>
       <c r="H50" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B51" t="s">
         <v>30</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="F51" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G51" t="s">
-        <v>120</v>
+        <v>104</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D52" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>127</v>
+        <v>87</v>
       </c>
       <c r="H52" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B53" t="s">
         <v>79</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="D53" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="E53" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F53" t="s">
-        <v>17</v>
+        <v>146</v>
       </c>
       <c r="G53" t="s">
-        <v>166</v>
+        <v>147</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B54" t="s">
         <v>79</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F54" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="G54" t="s">
-        <v>83</v>
+        <v>175</v>
       </c>
       <c r="H54" t="s">
         <v>26</v>
       </c>
       <c r="I54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B55" t="s">
         <v>79</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="D55" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E55" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="F55" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G55" t="s">
-        <v>83</v>
+        <v>104</v>
       </c>
       <c r="H55" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3088,37 +3121,37 @@
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B56" t="s">
         <v>79</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F56" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G56" t="s">
-        <v>70</v>
+        <v>178</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3127,47 +3160,47 @@
     </row>
     <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A57" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B57" t="s">
         <v>79</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F57" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G57" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B58" t="s">
         <v>79</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
@@ -3176,10 +3209,10 @@
         <v>17</v>
       </c>
       <c r="F58" t="s">
-        <v>17</v>
+        <v>85</v>
       </c>
       <c r="G58" t="s">
-        <v>88</v>
+        <v>175</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
@@ -3193,95 +3226,95 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B59" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="D59" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E59" t="s">
+        <v>10</v>
+      </c>
+      <c r="F59" t="s">
+        <v>10</v>
+      </c>
+      <c r="G59" t="s">
+        <v>70</v>
+      </c>
+      <c r="H59" t="s">
+        <v>11</v>
+      </c>
+      <c r="I59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A60" s="5">
+        <v>46094</v>
+      </c>
+      <c r="B60" t="s">
+        <v>79</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+      <c r="E60" t="s">
         <v>25</v>
       </c>
-      <c r="F59" t="s">
+      <c r="F60" t="s">
         <v>25</v>
       </c>
-      <c r="G59" t="s">
-        <v>83</v>
-      </c>
-      <c r="H59" t="s">
-        <v>26</v>
-      </c>
-      <c r="I59" t="str">
+      <c r="G60" t="s">
+        <v>184</v>
+      </c>
+      <c r="H60" t="s">
+        <v>11</v>
+      </c>
+      <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J59" t="str">
+      <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A60" s="5">
-        <v>46093</v>
-      </c>
-      <c r="B60" t="s">
-        <v>29</v>
-      </c>
-      <c r="C60" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D60" t="s">
-        <v>12</v>
-      </c>
-      <c r="E60" t="s">
-        <v>10</v>
-      </c>
-      <c r="F60" t="s">
-        <v>10</v>
-      </c>
-      <c r="G60" t="s">
-        <v>70</v>
-      </c>
-      <c r="H60" t="s">
-        <v>11</v>
-      </c>
-      <c r="I60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B61" t="s">
         <v>29</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>174</v>
+        <v>154</v>
       </c>
       <c r="D61" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E61" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="F61" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="G61" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="H61" t="s">
         <v>26</v>
@@ -3292,30 +3325,30 @@
       </c>
       <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B62" t="s">
         <v>29</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="D62" t="s">
         <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F62" t="s">
-        <v>23</v>
+        <v>146</v>
       </c>
       <c r="G62" t="s">
-        <v>89</v>
+        <v>147</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
@@ -3329,95 +3362,95 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A63" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B63" t="s">
         <v>29</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F63" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G63" t="s">
-        <v>70</v>
+        <v>187</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
       </c>
       <c r="I63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B64" t="s">
         <v>29</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="D64" t="s">
         <v>12</v>
       </c>
       <c r="E64" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F64" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G64" t="s">
-        <v>85</v>
+        <v>189</v>
       </c>
       <c r="H64" t="s">
         <v>11</v>
       </c>
       <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B65" t="s">
-        <v>82</v>
+        <v>29</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>177</v>
+        <v>190</v>
       </c>
       <c r="D65" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E65" t="s">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="F65" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G65" t="s">
-        <v>127</v>
+        <v>83</v>
       </c>
       <c r="H65" t="s">
         <v>11</v>
@@ -3433,13 +3466,13 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A66" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B66" t="s">
-        <v>82</v>
+        <v>29</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>178</v>
+        <v>191</v>
       </c>
       <c r="D66" t="s">
         <v>12</v>
@@ -3451,7 +3484,7 @@
         <v>10</v>
       </c>
       <c r="G66" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="H66" t="s">
         <v>11</v>
@@ -3467,104 +3500,172 @@
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A67" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B67" t="s">
         <v>82</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>179</v>
+        <v>192</v>
       </c>
       <c r="D67" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E67" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F67" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G67" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H67" t="s">
         <v>11</v>
       </c>
       <c r="I67" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J67" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A68" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B68" t="s">
         <v>82</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>180</v>
+        <v>193</v>
       </c>
       <c r="D68" t="s">
         <v>12</v>
       </c>
       <c r="E68" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F68" t="s">
-        <v>86</v>
+        <v>23</v>
       </c>
       <c r="G68" t="s">
-        <v>181</v>
+        <v>124</v>
       </c>
       <c r="H68" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I68" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J68" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A69" s="5">
-        <v>46093</v>
+        <v>46094</v>
       </c>
       <c r="B69" t="s">
         <v>82</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="D69" t="s">
-        <v>12</v>
+        <v>89</v>
       </c>
       <c r="E69" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="F69" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="G69" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H69" t="s">
         <v>11</v>
       </c>
       <c r="I69" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A70" s="5">
+        <v>46094</v>
+      </c>
+      <c r="B70" t="s">
+        <v>82</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D70" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" t="s">
+        <v>25</v>
+      </c>
+      <c r="F70" t="s">
+        <v>25</v>
+      </c>
+      <c r="G70" t="s">
+        <v>104</v>
+      </c>
+      <c r="H70" t="s">
+        <v>11</v>
+      </c>
+      <c r="I70" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+      <c r="J70" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A71" s="5">
+        <v>46094</v>
+      </c>
+      <c r="B71" t="s">
+        <v>82</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D71" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71" t="s">
+        <v>38</v>
+      </c>
+      <c r="F71" t="s">
+        <v>38</v>
+      </c>
+      <c r="G71" t="s">
+        <v>102</v>
+      </c>
+      <c r="H71" t="s">
+        <v>11</v>
+      </c>
+      <c r="I71" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J71" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reporte 17 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF76B69-5FAF-4177-91C4-4C547215B118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5319CB0-CEE3-4F1D-A315-A90748902B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="192">
   <si>
     <t>Fecha</t>
   </si>
@@ -129,9 +129,6 @@
     <t>Pachuca Brilla</t>
   </si>
   <si>
-    <t>Effetá</t>
-  </si>
-  <si>
     <t>Semot</t>
   </si>
   <si>
@@ -288,18 +285,9 @@
     <t>Plaza Juárez</t>
   </si>
   <si>
-    <t>Mundial De Futbol</t>
-  </si>
-  <si>
     <t>Deportes</t>
   </si>
   <si>
-    <t>Alcalde</t>
-  </si>
-  <si>
-    <t>Combate a la delincuencia</t>
-  </si>
-  <si>
     <t>Reforma Electoral</t>
   </si>
   <si>
@@ -309,325 +297,322 @@
     <t>Editorial</t>
   </si>
   <si>
-    <t>Crean reglas para peleas profesionales</t>
-  </si>
-  <si>
-    <t>Sheinbaum presenta su plan B electoral</t>
-  </si>
-  <si>
-    <t>Plan B</t>
-  </si>
-  <si>
-    <t>Pequeños comercios prefieren el efectivo</t>
-  </si>
-  <si>
-    <t>Irán reitera cierre de ruta clave del crudo</t>
-  </si>
-  <si>
     <t>Temas internacionales</t>
   </si>
   <si>
-    <t>Acusa CNTE falta defensa sindical</t>
-  </si>
-  <si>
-    <t>Leyenda de Las Calderas del Progreso</t>
-  </si>
-  <si>
-    <t>Escamoles a precio alto por sobreexplotación</t>
-  </si>
-  <si>
-    <t>Línea de alta tensión detonará más inversiones</t>
-  </si>
-  <si>
-    <t>Atracción De Inversiones</t>
-  </si>
-  <si>
-    <t>HACEN SU LUCHITA</t>
-  </si>
-  <si>
-    <t>Iniciativa</t>
-  </si>
-  <si>
-    <t>Llegan las rutas a Almoloya</t>
-  </si>
-  <si>
-    <t>Ruta de la Transformación</t>
-  </si>
-  <si>
-    <t>Regidores de 5 municipios cuestan 42 mdp</t>
-  </si>
-  <si>
     <t>Regidor</t>
   </si>
   <si>
-    <t>Salarios Regidores</t>
-  </si>
-  <si>
-    <t>Hay algo que conviene dejar claro desde el principio: la transparencia no pertenece a las instituciones, pertenece a la ciudadanía, los...</t>
-  </si>
-  <si>
-    <t>Combate a la corrupción</t>
-  </si>
-  <si>
-    <t>C4 en Mineral de la Reforma</t>
-  </si>
-  <si>
-    <t>C4</t>
-  </si>
-  <si>
-    <t>DURA PRUEBA PARA LA ZAGA</t>
-  </si>
-  <si>
-    <t>SUEÑAN CON  EL MUNDIAL</t>
-  </si>
-  <si>
-    <t>LA CENTRAL DE ABASTOS, “UNA BOMBA DE TIEMPO”</t>
-  </si>
-  <si>
-    <t>Central De Abastos</t>
-  </si>
-  <si>
-    <t>PREPARAN LA EDICIÓN  2026 DEL VIACRUCIS  DEL BARRIO LAS LAJAS</t>
-  </si>
-  <si>
     <t>Viacrucis</t>
   </si>
   <si>
-    <t>Impiden la salida de alumnos de la UAEH</t>
-  </si>
-  <si>
-    <t>Seguridad</t>
-  </si>
-  <si>
-    <t>TANIA MEZA NO  PODRÁ RETOMAR INICIATIVA SOBRE EL PERIODISMO</t>
-  </si>
-  <si>
-    <t>GLMorena</t>
-  </si>
-  <si>
-    <t>Ley de Protección a Periodistas</t>
-  </si>
-  <si>
-    <t>Denuncian violación a intimidad en 73% de municipios del estado</t>
-  </si>
-  <si>
-    <t>Violencia digital</t>
-  </si>
-  <si>
-    <t>Hacen frente en Pachuca a bandas y narcomenudistas</t>
-  </si>
-  <si>
-    <t>Destinan 100 mdp para la construcción de C4</t>
-  </si>
-  <si>
-    <t>Se imponen concesionados y Guardia disuade a Uber y Didi</t>
-  </si>
-  <si>
-    <t>En 6 cabildos ven un posible recorte a las regidurías</t>
-  </si>
-  <si>
-    <t>Operativos de movilidad detectan 43 taxis que dan servicios sin tener placas</t>
-  </si>
-  <si>
-    <t>Operativo de transporte</t>
-  </si>
-  <si>
-    <t>Gana chileno Radic el Nóbel de arquitectura</t>
-  </si>
-  <si>
-    <t>El Plan B es una iniciativa constitucional, no para leyes secundarias: Morena</t>
-  </si>
-  <si>
-    <t>El beisbol como una expresión de diversidad</t>
-  </si>
-  <si>
-    <t>Hidalgo destina  $11 millones para  sus 30 diputados</t>
-  </si>
-  <si>
-    <t>Sube a 20  el número de muertes  por influenza</t>
-  </si>
-  <si>
-    <t>Influenza</t>
-  </si>
-  <si>
-    <t>Avanzan trabajos para la reubicación de ambulantes</t>
-  </si>
-  <si>
-    <t>Ambulantaje</t>
-  </si>
-  <si>
-    <t>Presenta  Sheinbaum su  plan electoral B</t>
-  </si>
-  <si>
-    <t>Leyes hay, que las cumplan es otra cosa, y el comentario viene a cuento porque de nueva cuenta la Ley de  Protección a los Derechos de los Periodistas, impulsada por los legisladores, en este caso concreto por la  diputada morenista Tania Meza Escorza, fue frenada cuando apenas iba a entrar a discusión”.</t>
-  </si>
-  <si>
-    <t>Anuncia Menchaca nuevos proyectos de  infraestructura para Almoloya</t>
-  </si>
-  <si>
-    <t>Reconoce embajadora de Sudáfrica  la seguridad que priva en Hidalgo</t>
-  </si>
-  <si>
-    <t>Investiga Fiscalía de Delitos Electorales  presunto fraude cibernético contra Panalh</t>
-  </si>
-  <si>
-    <t>Fede</t>
-  </si>
-  <si>
-    <t>Lanzan alerta roja por fuertes rachas de  viento en Hidalgo</t>
-  </si>
-  <si>
-    <t>PC</t>
-  </si>
-  <si>
-    <t>Alerta Meteorológica</t>
-  </si>
-  <si>
-    <t>CEAA advierte sobre la temporada de estiaje en Hidalgo</t>
-  </si>
-  <si>
     <t>Sipdus</t>
   </si>
   <si>
-    <t>CEAA</t>
-  </si>
-  <si>
-    <t>Mitigación estiaje</t>
-  </si>
-  <si>
-    <t>El carnaval #Huejutla 2026 ya está aquí</t>
-  </si>
-  <si>
-    <t>Carnavales</t>
-  </si>
-  <si>
-    <t>Julio Menchaca destina más de 57 mdp para obras públicas en Almoloya</t>
-  </si>
-  <si>
-    <t>Solicitan a delegados evitar tiradero clandestinos de basura</t>
-  </si>
-  <si>
-    <t>Basurero Clandestino</t>
-  </si>
-  <si>
-    <t>Llama obispo de Huejutla a vivir la cuaresma con reflexón y conversión</t>
-  </si>
-  <si>
-    <t>Deteriorada e intransitable la carretera federal 102</t>
-  </si>
-  <si>
     <t>SICT</t>
   </si>
   <si>
-    <t>Carretera En Mal Estado</t>
-  </si>
-  <si>
-    <t>Medécigo busca 100 millones para nuevo C4</t>
-  </si>
-  <si>
-    <t>Claudia Sheinbaum plantea reducir gastos en congresos</t>
-  </si>
-  <si>
-    <t>Irrumpen en Cabildo de Tepeji y agreden al oficial mayor</t>
-  </si>
-  <si>
-    <t>Agresión</t>
-  </si>
-  <si>
-    <t>Entre mareos y miedo</t>
-  </si>
-  <si>
     <t>Pemex</t>
   </si>
   <si>
-    <t>Fuga de hidrocarburo</t>
-  </si>
-  <si>
-    <t>MC Hidalgo reclamando lo que votó recortar</t>
-  </si>
-  <si>
-    <t>De 45 millones en Tepeapulco, exalcaldesa debe solventar 25</t>
-  </si>
-  <si>
-    <t>Observaciones ASEH</t>
-  </si>
-  <si>
-    <t>Menchaca destina 57 millones en Almoloya</t>
-  </si>
-  <si>
-    <t>Diputados de Hidalgo se dividen en votación de Reforma Electoral</t>
-  </si>
-  <si>
-    <t>Prevén rachas de viento fuertes en Hidalgo; piden extremar precauciones</t>
-  </si>
-  <si>
-    <t>Claudia Sandoval camina y escucha al pueblo, ahora en Tezoquipa</t>
-  </si>
-  <si>
     <t>Atención a la ciudadanía</t>
   </si>
   <si>
-    <t>Menchaca destina más de 57 mdp para obras públicas en Almoloya</t>
-  </si>
-  <si>
-    <t>Realizan Feria de Servicios municipales</t>
-  </si>
-  <si>
-    <t>Feria de servicios</t>
-  </si>
-  <si>
-    <t>Se fortalece el diálogo entre juventudes y autoridades en encuentro estatal</t>
-  </si>
-  <si>
-    <t>Atención a jóvenes</t>
-  </si>
-  <si>
-    <t>Xochitlán de las Flores se transforma mediante diálogo y el trabajo en conjunto</t>
-  </si>
-  <si>
-    <t>Diálogo institucional fortalece al magisterio hidalguense</t>
-  </si>
-  <si>
-    <t>Menchaca pide denunciar formalmente a funcionarios señalados en tendederos del 8M</t>
-  </si>
-  <si>
-    <t>Marcha 8M</t>
-  </si>
-  <si>
-    <t>Fuertes rachas de viento en HIdalgo</t>
-  </si>
-  <si>
-    <t>Lanzan convocatoria 2016 para apoyar a cuidadores de personas con discapacidad</t>
-  </si>
-  <si>
-    <t>Cuidadores De Adultos Mayores</t>
-  </si>
-  <si>
-    <t>¿Buscas trabajo? este viernes realizarán feria nacional de empleo para las mujeres</t>
-  </si>
-  <si>
-    <t>Feria De Empleo</t>
-  </si>
-  <si>
-    <t>Embajadora de Sudáfrica recorrió más puntos de la entidad de cara al mundial</t>
-  </si>
-  <si>
-    <t>Tuzas vencen 2-0 a Tijuana en liga MX femenil</t>
-  </si>
-  <si>
-    <t>Atraparon a 4 vinculados a la célula de ""Los Polos""</t>
-  </si>
-  <si>
-    <t>Emiten recomendaciones contra la extorsión sexual digital</t>
-  </si>
-  <si>
-    <t>Morena y la 4T tienen fisuras, como quedó demostrado con los votos en contra de legisladores morenistas en la fallida Reforma Electoral</t>
-  </si>
-  <si>
-    <t>Destinan más de 57 mdp para obras en Almoloya</t>
-  </si>
-  <si>
-    <t>Crean iniciativa para homologar investigación de feminicidios</t>
+    <t>Suman 55 casos de gusano barrenador en Hidalgo</t>
+  </si>
+  <si>
+    <t>Gusano barrenador</t>
+  </si>
+  <si>
+    <t>Biblioteca municipal de Huehuetal sin acervo</t>
+  </si>
+  <si>
+    <t>Huracán Priscilla</t>
+  </si>
+  <si>
+    <t>Preparan el viacrucis tras jornada laboral</t>
+  </si>
+  <si>
+    <t>Piden mejorar Cereso en lugar de hacer otro</t>
+  </si>
+  <si>
+    <t>Construcción de Cereso</t>
+  </si>
+  <si>
+    <t>En alerta por derrames de hidrocarburo en río</t>
+  </si>
+  <si>
+    <t>Contaminación de río</t>
+  </si>
+  <si>
+    <t>Siguen las largas filas en la farmacia del IMSS</t>
+  </si>
+  <si>
+    <t>IMSS</t>
+  </si>
+  <si>
+    <t>Abasto De Medicamentos</t>
+  </si>
+  <si>
+    <t>Guerra entre alcaldes y regidores afecta a 8 municipios</t>
+  </si>
+  <si>
+    <t>Opacidad</t>
+  </si>
+  <si>
+    <t>Trabajo de altura</t>
+  </si>
+  <si>
+    <t>Obras públicas</t>
+  </si>
+  <si>
+    <t>Imagen Urbana</t>
+  </si>
+  <si>
+    <t>Temen por gusano barrenador</t>
+  </si>
+  <si>
+    <t>Hay material para sustituciones</t>
+  </si>
+  <si>
+    <t>Simey</t>
+  </si>
+  <si>
+    <t>Afiliación Partidista</t>
+  </si>
+  <si>
+    <t>Canaco Servytur Pachuca se renueva</t>
+  </si>
+  <si>
+    <t>Nombramientos</t>
+  </si>
+  <si>
+    <t>Los recientes cambios en el BA JO RE SERVA calendario interno de Morena para designar a las personas que podrían opcupar un cargo de elección popular en el...</t>
+  </si>
+  <si>
+    <t>Sucesión alcaldía</t>
+  </si>
+  <si>
+    <t>EL REY IMPONE  LEY GOLEADORA</t>
+  </si>
+  <si>
+    <t>CHAMPIONS  AL ROJO VIVO</t>
+  </si>
+  <si>
+    <t>SIN SEÑALÉTICA NI LUZ, LA CARRETERA REAL-HUASCA</t>
+  </si>
+  <si>
+    <t>Carretera Huasca</t>
+  </si>
+  <si>
+    <t>Instalaron valla para seguridad de los peatones</t>
+  </si>
+  <si>
+    <t>Falta de puente</t>
+  </si>
+  <si>
+    <t>Van tres ataques armados y siete restos hallados durante marzo</t>
+  </si>
+  <si>
+    <t>Incidencia Delictiva</t>
+  </si>
+  <si>
+    <t>LA ALCALDÍA BUSCA  REGULARIZAR LOS FRACCIONAMIENTOS EN HUASCA: LUGO</t>
+  </si>
+  <si>
+    <t>Regularización De Tierras</t>
+  </si>
+  <si>
+    <t>Morena ""pepena"" alcaldes hasta a sus aliados: dice dirigente priista</t>
+  </si>
+  <si>
+    <t>PRI</t>
+  </si>
+  <si>
+    <t>Militancia Partidista</t>
+  </si>
+  <si>
+    <t>Circulan sin verificar, 2 mil 733 unidades de transporte público</t>
+  </si>
+  <si>
+    <t>verificación vehicular</t>
+  </si>
+  <si>
+    <t>Multas crecen 379%</t>
+  </si>
+  <si>
+    <t>Multas transporte público</t>
+  </si>
+  <si>
+    <t>Concluirán reparaición antes del periodo escolar</t>
+  </si>
+  <si>
+    <t>Denuncias por secuestro caen 72% en 5 años, revela la PGJEH</t>
+  </si>
+  <si>
+    <t>Combate Al Secuestro</t>
+  </si>
+  <si>
+    <t>Gubernatura para mujer: Inician mesas de análisis sobre iniciativa pendiente</t>
+  </si>
+  <si>
+    <t>Junta de Gobierno</t>
+  </si>
+  <si>
+    <t>Inversión hídrica alcanza los $4 mil 730 millones</t>
+  </si>
+  <si>
+    <t>Caasim</t>
+  </si>
+  <si>
+    <t>Infraestructura Hidráulica</t>
+  </si>
+  <si>
+    <t>Un Big Brother vigila el límite de la biología</t>
+  </si>
+  <si>
+    <t>Reconoce Felipe VI que sí hubo ""mucho abuso"" durante dla Conquista</t>
+  </si>
+  <si>
+    <t>La moedia, otro superpoder de Eiza</t>
+  </si>
+  <si>
+    <t>Avanzan trabajos de la  nueva estación de Bomberos</t>
+  </si>
+  <si>
+    <t>Nueva estación de Bomberos</t>
+  </si>
+  <si>
+    <t>En lo que va del año suman 25 homicidios violentos en región de Tula</t>
+  </si>
+  <si>
+    <t>Homicidios</t>
+  </si>
+  <si>
+    <t>Cuatro partidos suman multas por 46.7 mdp por auditorías del INE</t>
+  </si>
+  <si>
+    <t>Multas INE</t>
+  </si>
+  <si>
+    <t>García Harfuch descongela diálogo con  la DEA; acude  a Washington</t>
+  </si>
+  <si>
+    <t>La diferencia es crucial, una cosa es que el presidente dé una posición oficial de México, otra  muy distinta es que un ciudadano manifieste sus posturas ideológicas. Confundir ambas cosas es  deliberado”.</t>
+  </si>
+  <si>
+    <t>Hidalgo, libre de sequía: Conagua</t>
+  </si>
+  <si>
+    <t>Conagua</t>
+  </si>
+  <si>
+    <t>Disponibilidad de agua</t>
+  </si>
+  <si>
+    <t>Mejoran imagen de Pachuca con retiro de 80 espectaculares</t>
+  </si>
+  <si>
+    <t>Supera Hidalgo 5 mil 600 movilizaciones laborales dentro y fuera del país</t>
+  </si>
+  <si>
+    <t>Movilidad laboral</t>
+  </si>
+  <si>
+    <t>Abrirán registro del programa ""Viviendas del bienestar"" para derechohabientes</t>
+  </si>
+  <si>
+    <t>Infonavit</t>
+  </si>
+  <si>
+    <t>Plan Nacional De Vivienda</t>
+  </si>
+  <si>
+    <t>Sipdus transforma la infraestructura hídrica del estado de Hidalgo</t>
+  </si>
+  <si>
+    <t>Celebran X aniversario de la ordenación del obispo de la diósesis de Huejutla</t>
+  </si>
+  <si>
+    <t>Alistan la primera sesión del cabildo infantil 2025 en Huejutla</t>
+  </si>
+  <si>
+    <t>Cabildo Juvenil</t>
+  </si>
+  <si>
+    <t>Fresco amanecer en la Huasteca, por el frente frío 41</t>
+  </si>
+  <si>
+    <t>Hidalgo protege a su gente; movilidad laboral segura y trato digno</t>
+  </si>
+  <si>
+    <t>Mega feria Infornavit en Pachuca abrirá registrto de vivienda para el Bienestar</t>
+  </si>
+  <si>
+    <t>Con inversión histórica de 4 mil 730 mdp, Sipdus transforma la infraestructura hídrica de Hidalgo</t>
+  </si>
+  <si>
+    <t>Concluye con éxito la 4a edición de le Expo Acuícola Hidalgo 2026</t>
+  </si>
+  <si>
+    <t>Expo acuícola</t>
+  </si>
+  <si>
+    <t>Pachua impulsa acciones de imagen iurbana con retiro de estructuras puiblicitarias irregulares</t>
+  </si>
+  <si>
+    <t>Sebiso impulsa a sectores vulnerables con programa ""Apoyo para el Bienestar y Desarrollo""</t>
+  </si>
+  <si>
+    <t>Combate a la pobreza</t>
+  </si>
+  <si>
+    <t>Feria San José</t>
+  </si>
+  <si>
+    <t>Publicidad</t>
+  </si>
+  <si>
+    <t>Feria Patronal</t>
+  </si>
+  <si>
+    <t>Conoce la pirámide de movilidad</t>
+  </si>
+  <si>
+    <t>Publicidad gubernamental</t>
+  </si>
+  <si>
+    <t>Retiran estructuras publicitarias irregulares en Pachuca</t>
+  </si>
+  <si>
+    <t>Con inversión histórica de 4 mil 730 mdp, Sipdus transforma la infraestructura hídrica</t>
+  </si>
+  <si>
+    <t>Sorprenden policías de Pachuca a Niño en su cumpleaños</t>
+  </si>
+  <si>
+    <t>Policía municipal</t>
+  </si>
+  <si>
+    <t>Abrirán registro para programa apoyo para el Bienestar y Desarrollo en Hidalgo</t>
+  </si>
+  <si>
+    <t>Colocan rejas para evitar cruce de peatones sobre avenida madero</t>
+  </si>
+  <si>
+    <t>En 24 horas: un calcinado, un encobijado y dos ejecutados</t>
+  </si>
+  <si>
+    <t>Ejecuciones</t>
+  </si>
+  <si>
+    <t>Pro fraude y domentos falsos vincularon a regidora de Apan</t>
+  </si>
+  <si>
+    <t>Tan malo el pinto como el colorado. Por un lado, Trump garantiza sometimiento e Cuba disfrazado de libertad; y el régimen castrista en la isla garantiza la continuación de sometimiento y el empoderamiento que ha sufrido el  pueblo cubano por generaciones</t>
+  </si>
+  <si>
+    <t>García Harfuch habla con el director de la DEA</t>
   </si>
 </sst>
 </file>
@@ -874,8 +859,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J71" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J71" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J60" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J60" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1241,22 +1226,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J71"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J60"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.7265625" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1285,89 +1270,89 @@
         <v>8</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="G3" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
         <v>10</v>
@@ -1376,7 +1361,7 @@
         <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>70</v>
+        <v>88</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
@@ -1390,355 +1375,355 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G5" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="G6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H6" t="s">
+        <v>16</v>
+      </c>
+      <c r="I6" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J6" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
+        <v>46098</v>
+      </c>
+      <c r="B7" t="s">
         <v>70</v>
       </c>
-      <c r="H6" t="s">
-        <v>11</v>
-      </c>
-      <c r="I6" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J6" t="str">
+      <c r="C7" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>14</v>
+      </c>
+      <c r="F7" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7" t="s">
+        <v>104</v>
+      </c>
+      <c r="H7" t="s">
+        <v>16</v>
+      </c>
+      <c r="I7" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" t="s">
-        <v>10</v>
-      </c>
-      <c r="G7" t="s">
-        <v>70</v>
-      </c>
-      <c r="H7" t="s">
-        <v>11</v>
-      </c>
-      <c r="I7" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J7" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B8" t="s">
         <v>71</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" t="s">
+        <v>106</v>
+      </c>
+      <c r="H8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I8" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J8" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
+        <v>46098</v>
+      </c>
+      <c r="B9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D9" t="s">
+        <v>9</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" t="s">
+        <v>108</v>
+      </c>
+      <c r="G9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H9" t="s">
+        <v>11</v>
+      </c>
+      <c r="I9" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J9" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
+        <v>46098</v>
+      </c>
+      <c r="B10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="D10" t="s">
         <v>12</v>
       </c>
-      <c r="E8" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G8" t="s">
-        <v>70</v>
-      </c>
-      <c r="H8" t="s">
-        <v>11</v>
-      </c>
-      <c r="I8" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J8" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B9" t="s">
-        <v>72</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="D9" t="s">
-        <v>13</v>
-      </c>
-      <c r="E9" t="s">
-        <v>59</v>
-      </c>
-      <c r="F9" t="s">
-        <v>2</v>
-      </c>
-      <c r="G9" t="s">
-        <v>100</v>
-      </c>
-      <c r="H9" t="s">
-        <v>26</v>
-      </c>
-      <c r="I9" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J9" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B10" t="s">
-        <v>72</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="D10" t="s">
-        <v>9</v>
-      </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="F10" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="G10" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B11" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>112</v>
       </c>
       <c r="G11" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Sucesión gubernamental</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>106</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="H12" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B14" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>82</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
@@ -1750,7 +1735,7 @@
         <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
@@ -1764,61 +1749,61 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="D16" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F16" t="s">
-        <v>10</v>
+        <v>90</v>
       </c>
       <c r="G16" t="s">
-        <v>84</v>
+        <v>121</v>
       </c>
       <c r="H16" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="D17" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>22</v>
+        <v>89</v>
       </c>
       <c r="F17" t="s">
-        <v>22</v>
+        <v>89</v>
       </c>
       <c r="G17" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
@@ -1832,129 +1817,129 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="D18" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="F18" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G18" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="H18" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>64</v>
+        <v>17</v>
       </c>
       <c r="G19" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="H19" t="s">
         <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>38</v>
+        <v>129</v>
       </c>
       <c r="F20" t="s">
-        <v>121</v>
+        <v>2</v>
       </c>
       <c r="G20" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Partidos</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D21" t="s">
         <v>13</v>
       </c>
       <c r="E21" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="F21" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
@@ -1968,30 +1953,30 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F22" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="G22" t="s">
-        <v>86</v>
+        <v>134</v>
       </c>
       <c r="H22" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2002,132 +1987,132 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="F23" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="G23" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="D24" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F24" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="G24" t="s">
-        <v>83</v>
+        <v>137</v>
       </c>
       <c r="H24" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="F25" t="s">
-        <v>17</v>
+        <v>139</v>
       </c>
       <c r="G25" t="s">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>31</v>
+        <v>89</v>
       </c>
       <c r="F26" t="s">
-        <v>31</v>
+        <v>141</v>
       </c>
       <c r="G26" t="s">
-        <v>130</v>
+        <v>142</v>
       </c>
       <c r="H26" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2138,15 +2123,15 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>131</v>
+        <v>143</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -2158,7 +2143,7 @@
         <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
@@ -2172,49 +2157,49 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B28" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="G28" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="H28" t="s">
         <v>11</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B29" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
@@ -2226,7 +2211,7 @@
         <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
@@ -2240,64 +2225,64 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>134</v>
+        <v>146</v>
       </c>
       <c r="D30" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E30" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="F30" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="G30" t="s">
-        <v>107</v>
+        <v>147</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>135</v>
+        <v>148</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="F31" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G31" t="s">
-        <v>136</v>
+        <v>149</v>
       </c>
       <c r="H31" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2308,49 +2293,49 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>137</v>
+        <v>150</v>
       </c>
       <c r="D32" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E32" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F32" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G32" t="s">
-        <v>138</v>
+        <v>151</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>139</v>
+        <v>152</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
@@ -2362,7 +2347,7 @@
         <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
@@ -2376,30 +2361,30 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="87" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="F34" t="s">
-        <v>121</v>
+        <v>10</v>
       </c>
       <c r="G34" t="s">
-        <v>122</v>
+        <v>69</v>
       </c>
       <c r="H34" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2410,98 +2395,98 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="D35" t="s">
         <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F35" t="s">
-        <v>25</v>
+        <v>155</v>
       </c>
       <c r="G35" t="s">
-        <v>104</v>
+        <v>156</v>
       </c>
       <c r="H35" t="s">
         <v>26</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B36" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>2</v>
+        <v>108</v>
       </c>
       <c r="G36" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="H36" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="F37" t="s">
-        <v>144</v>
+        <v>60</v>
       </c>
       <c r="G37" t="s">
-        <v>88</v>
+        <v>159</v>
       </c>
       <c r="H37" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2512,64 +2497,64 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>145</v>
+        <v>160</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F38" t="s">
-        <v>146</v>
+        <v>161</v>
       </c>
       <c r="G38" t="s">
-        <v>147</v>
+        <v>162</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B39" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="D39" t="s">
         <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>149</v>
+        <v>89</v>
       </c>
       <c r="F39" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="G39" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="H39" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2580,166 +2565,166 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B40" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G40" t="s">
-        <v>153</v>
+        <v>69</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B41" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>104</v>
+        <v>166</v>
       </c>
       <c r="H41" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B42" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>156</v>
+        <v>69</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="F43" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="G43" t="s">
-        <v>70</v>
+        <v>159</v>
       </c>
       <c r="H43" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B44" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="D44" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="E44" t="s">
         <v>14</v>
       </c>
       <c r="F44" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G44" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H44" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2750,83 +2735,83 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B45" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>17</v>
+        <v>89</v>
       </c>
       <c r="F45" t="s">
-        <v>85</v>
+        <v>141</v>
       </c>
       <c r="G45" t="s">
-        <v>111</v>
+        <v>142</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B46" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="D46" t="s">
         <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="F46" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G46" t="s">
-        <v>92</v>
+        <v>172</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B47" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="D47" t="s">
         <v>12</v>
@@ -2835,10 +2820,10 @@
         <v>17</v>
       </c>
       <c r="F47" t="s">
-        <v>17</v>
+        <v>108</v>
       </c>
       <c r="G47" t="s">
-        <v>164</v>
+        <v>109</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
@@ -2852,98 +2837,98 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B48" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="D48" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="F48" t="s">
-        <v>166</v>
+        <v>20</v>
       </c>
       <c r="G48" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="H48" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="5">
+        <v>46098</v>
+      </c>
+      <c r="B49" t="s">
+        <v>78</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D49" t="s">
+        <v>177</v>
+      </c>
+      <c r="E49" t="s">
+        <v>17</v>
+      </c>
+      <c r="F49" t="s">
+        <v>17</v>
+      </c>
+      <c r="G49" t="s">
+        <v>178</v>
+      </c>
+      <c r="H49" t="s">
+        <v>11</v>
+      </c>
+      <c r="I49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A49" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B49" t="s">
-        <v>30</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="D49" t="s">
-        <v>89</v>
-      </c>
-      <c r="E49" t="s">
-        <v>48</v>
-      </c>
-      <c r="F49" t="s">
-        <v>48</v>
-      </c>
-      <c r="G49" t="s">
-        <v>87</v>
-      </c>
-      <c r="H49" t="s">
-        <v>16</v>
-      </c>
-      <c r="I49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B50" t="s">
-        <v>30</v>
+        <v>78</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="D50" t="s">
-        <v>12</v>
+        <v>177</v>
       </c>
       <c r="E50" t="s">
         <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>85</v>
+        <v>17</v>
       </c>
       <c r="G50" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="H50" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2954,166 +2939,166 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B51" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="D51" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E51" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F51" t="s">
-        <v>25</v>
+        <v>108</v>
       </c>
       <c r="G51" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B52" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>10</v>
+        <v>89</v>
       </c>
       <c r="F52" t="s">
-        <v>10</v>
+        <v>141</v>
       </c>
       <c r="G52" t="s">
-        <v>87</v>
+        <v>142</v>
       </c>
       <c r="H52" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="5">
+        <v>46098</v>
+      </c>
+      <c r="B53" t="s">
+        <v>29</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>17</v>
+      </c>
+      <c r="F53" t="s">
+        <v>184</v>
+      </c>
+      <c r="G53" t="s">
+        <v>92</v>
+      </c>
+      <c r="H53" t="s">
+        <v>26</v>
+      </c>
+      <c r="I53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A53" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B53" t="s">
-        <v>79</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D53" t="s">
-        <v>81</v>
-      </c>
-      <c r="E53" t="s">
-        <v>24</v>
-      </c>
-      <c r="F53" t="s">
-        <v>146</v>
-      </c>
-      <c r="G53" t="s">
-        <v>147</v>
-      </c>
-      <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B54" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F54" t="s">
-        <v>85</v>
+        <v>20</v>
       </c>
       <c r="G54" t="s">
         <v>175</v>
       </c>
       <c r="H54" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B55" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
       <c r="D55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>25</v>
+        <v>89</v>
       </c>
       <c r="F55" t="s">
-        <v>25</v>
+        <v>89</v>
       </c>
       <c r="G55" t="s">
-        <v>104</v>
+        <v>123</v>
       </c>
       <c r="H55" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3121,21 +3106,21 @@
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B56" t="s">
-        <v>79</v>
+        <v>29</v>
       </c>
       <c r="C56" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="D56" t="s">
         <v>177</v>
-      </c>
-      <c r="D56" t="s">
-        <v>12</v>
       </c>
       <c r="E56" t="s">
         <v>17</v>
@@ -3144,7 +3129,7 @@
         <v>17</v>
       </c>
       <c r="G56" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
@@ -3158,30 +3143,30 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B57" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D57" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E57" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F57" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="G57" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="H57" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3192,15 +3177,15 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B58" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
@@ -3209,35 +3194,35 @@
         <v>17</v>
       </c>
       <c r="F58" t="s">
+        <v>87</v>
+      </c>
+      <c r="G58" t="s">
+        <v>84</v>
+      </c>
+      <c r="H58" t="s">
+        <v>16</v>
+      </c>
+      <c r="I58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A59" s="5">
+        <v>46098</v>
+      </c>
+      <c r="B59" t="s">
+        <v>81</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D59" t="s">
         <v>85</v>
-      </c>
-      <c r="G58" t="s">
-        <v>175</v>
-      </c>
-      <c r="H58" t="s">
-        <v>11</v>
-      </c>
-      <c r="I58" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J58" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A59" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B59" t="s">
-        <v>79</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="D59" t="s">
-        <v>12</v>
       </c>
       <c r="E59" t="s">
         <v>10</v>
@@ -3246,10 +3231,10 @@
         <v>10</v>
       </c>
       <c r="G59" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="H59" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3260,410 +3245,36 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46094</v>
+        <v>46098</v>
       </c>
       <c r="B60" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="D60" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E60" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F60" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="G60" t="s">
-        <v>184</v>
+        <v>69</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A61" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B61" t="s">
-        <v>29</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="D61" t="s">
-        <v>13</v>
-      </c>
-      <c r="E61" t="s">
-        <v>25</v>
-      </c>
-      <c r="F61" t="s">
-        <v>25</v>
-      </c>
-      <c r="G61" t="s">
-        <v>104</v>
-      </c>
-      <c r="H61" t="s">
-        <v>26</v>
-      </c>
-      <c r="I61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A62" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B62" t="s">
-        <v>29</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>185</v>
-      </c>
-      <c r="D62" t="s">
-        <v>12</v>
-      </c>
-      <c r="E62" t="s">
-        <v>24</v>
-      </c>
-      <c r="F62" t="s">
-        <v>146</v>
-      </c>
-      <c r="G62" t="s">
-        <v>147</v>
-      </c>
-      <c r="H62" t="s">
-        <v>11</v>
-      </c>
-      <c r="I62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A63" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B63" t="s">
-        <v>29</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="D63" t="s">
-        <v>12</v>
-      </c>
-      <c r="E63" t="s">
-        <v>20</v>
-      </c>
-      <c r="F63" t="s">
-        <v>2</v>
-      </c>
-      <c r="G63" t="s">
-        <v>187</v>
-      </c>
-      <c r="H63" t="s">
-        <v>11</v>
-      </c>
-      <c r="I63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A64" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B64" t="s">
-        <v>29</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="D64" t="s">
-        <v>12</v>
-      </c>
-      <c r="E64" t="s">
-        <v>14</v>
-      </c>
-      <c r="F64" t="s">
-        <v>14</v>
-      </c>
-      <c r="G64" t="s">
-        <v>189</v>
-      </c>
-      <c r="H64" t="s">
-        <v>11</v>
-      </c>
-      <c r="I64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A65" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B65" t="s">
-        <v>29</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D65" t="s">
-        <v>12</v>
-      </c>
-      <c r="E65" t="s">
-        <v>33</v>
-      </c>
-      <c r="F65" t="s">
-        <v>2</v>
-      </c>
-      <c r="G65" t="s">
-        <v>83</v>
-      </c>
-      <c r="H65" t="s">
-        <v>11</v>
-      </c>
-      <c r="I65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A66" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B66" t="s">
-        <v>29</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="D66" t="s">
-        <v>12</v>
-      </c>
-      <c r="E66" t="s">
-        <v>10</v>
-      </c>
-      <c r="F66" t="s">
-        <v>10</v>
-      </c>
-      <c r="G66" t="s">
-        <v>84</v>
-      </c>
-      <c r="H66" t="s">
-        <v>11</v>
-      </c>
-      <c r="I66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B67" t="s">
-        <v>82</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="D67" t="s">
-        <v>13</v>
-      </c>
-      <c r="E67" t="s">
-        <v>23</v>
-      </c>
-      <c r="F67" t="s">
-        <v>23</v>
-      </c>
-      <c r="G67" t="s">
-        <v>86</v>
-      </c>
-      <c r="H67" t="s">
-        <v>11</v>
-      </c>
-      <c r="I67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A68" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B68" t="s">
-        <v>82</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D68" t="s">
-        <v>12</v>
-      </c>
-      <c r="E68" t="s">
-        <v>23</v>
-      </c>
-      <c r="F68" t="s">
-        <v>23</v>
-      </c>
-      <c r="G68" t="s">
-        <v>124</v>
-      </c>
-      <c r="H68" t="s">
-        <v>11</v>
-      </c>
-      <c r="I68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A69" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B69" t="s">
-        <v>82</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="D69" t="s">
-        <v>89</v>
-      </c>
-      <c r="E69" t="s">
-        <v>19</v>
-      </c>
-      <c r="F69" t="s">
-        <v>19</v>
-      </c>
-      <c r="G69" t="s">
-        <v>87</v>
-      </c>
-      <c r="H69" t="s">
-        <v>11</v>
-      </c>
-      <c r="I69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A70" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B70" t="s">
-        <v>82</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="D70" t="s">
-        <v>12</v>
-      </c>
-      <c r="E70" t="s">
-        <v>25</v>
-      </c>
-      <c r="F70" t="s">
-        <v>25</v>
-      </c>
-      <c r="G70" t="s">
-        <v>104</v>
-      </c>
-      <c r="H70" t="s">
-        <v>11</v>
-      </c>
-      <c r="I70" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J70" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A71" s="5">
-        <v>46094</v>
-      </c>
-      <c r="B71" t="s">
-        <v>82</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="D71" t="s">
-        <v>12</v>
-      </c>
-      <c r="E71" t="s">
-        <v>38</v>
-      </c>
-      <c r="F71" t="s">
-        <v>38</v>
-      </c>
-      <c r="G71" t="s">
-        <v>102</v>
-      </c>
-      <c r="H71" t="s">
-        <v>11</v>
-      </c>
-      <c r="I71" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J71" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
@@ -3680,140 +3291,140 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8151DEFD-FF29-4969-B1FC-DF47C7CD743C}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D1" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B2" t="s">
         <v>66</v>
-      </c>
-      <c r="B2" t="s">
-        <v>67</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>37</v>
-      </c>
-      <c r="B6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>38</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E7" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>42</v>
-      </c>
       <c r="E9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -3827,121 +3438,121 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>40</v>
       </c>
-      <c r="B11" t="s">
-        <v>36</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" t="s">
-        <v>36</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>44</v>
-      </c>
       <c r="E12" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E13" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E16" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="E17" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>43</v>
       </c>
-      <c r="B17" t="s">
-        <v>36</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+      <c r="D18" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E17" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="E18" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>44</v>
-      </c>
-      <c r="B18" t="s">
-        <v>36</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>59</v>
-      </c>
-      <c r="E18" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>45</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>
@@ -3950,66 +3561,66 @@
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" t="s">
         <v>46</v>
-      </c>
-      <c r="B20" t="s">
-        <v>47</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>47</v>
+      </c>
+      <c r="B21" t="s">
         <v>48</v>
       </c>
-      <c r="B21" t="s">
-        <v>49</v>
-      </c>
       <c r="D21" s="9" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E21" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
       <c r="B22" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>28</v>
       </c>
       <c r="E22" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E23" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -4020,214 +3631,214 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B27" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D27" s="11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E27" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>18</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>52</v>
       </c>
-      <c r="B29" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>53</v>
-      </c>
       <c r="B30" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
       <c r="B31" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+      <c r="B32" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>55</v>
       </c>
-      <c r="B32" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+      <c r="B33" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>56</v>
       </c>
-      <c r="B33" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>57</v>
       </c>
-      <c r="B34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="B35" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>58</v>
       </c>
-      <c r="B35" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>59</v>
-      </c>
       <c r="B36" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>24</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>21</v>
       </c>
       <c r="B38" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B39" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>28</v>
       </c>
       <c r="B40" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B41" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>23</v>
       </c>
       <c r="B43" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>60</v>
+      </c>
+      <c r="B44" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>61</v>
-      </c>
-      <c r="B44" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>62</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B47" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Reporte 19 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21B59D5C-73C1-4445-92F7-FFAEFAC5097D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E5091B-BC6E-4ECB-86A7-124BFB3ACEC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="210">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="199">
   <si>
     <t>Fecha</t>
   </si>
@@ -297,21 +297,6 @@
     <t>Pemex</t>
   </si>
   <si>
-    <t>Atención a la ciudadanía</t>
-  </si>
-  <si>
-    <t>Falta de puente</t>
-  </si>
-  <si>
-    <t>PRI</t>
-  </si>
-  <si>
-    <t>Militancia Partidista</t>
-  </si>
-  <si>
-    <t>Multas INE</t>
-  </si>
-  <si>
     <t>Plan Nacional De Vivienda</t>
   </si>
   <si>
@@ -327,346 +312,328 @@
     <t>Policía municipal</t>
   </si>
   <si>
-    <t>Ejecuciones</t>
-  </si>
-  <si>
-    <t>Sheinmabum, invitada a inaugurar oficinas</t>
-  </si>
-  <si>
-    <t>Visita Sheinbaum</t>
-  </si>
-  <si>
-    <t>Entregarán sólo 2,801 viviendas del Bienestar</t>
-  </si>
-  <si>
-    <t>Consideran innecesario el cercado</t>
-  </si>
-  <si>
-    <t>Sastrería resiste a la moda rápida: Solís</t>
-  </si>
-  <si>
-    <t>Controversia por la iniciativa del Plan B</t>
-  </si>
-  <si>
-    <t>Cierran tres días el mercado Barreteros</t>
-  </si>
-  <si>
-    <t>Parteras buscan ingresar a programa</t>
-  </si>
-  <si>
-    <t>Parteras Tradicionales</t>
-  </si>
-  <si>
-    <t>Respalda Menchaca el Plan B de la reforma electoral</t>
-  </si>
-  <si>
     <t>Plan B</t>
   </si>
   <si>
-    <t>En la ciudad de Pachuca existen pocos inmuebles tan simbólicos como el Reloj Monumental. Basta mencionarlo para que aparezca en...</t>
-  </si>
-  <si>
-    <t>Reloj De Pachuca</t>
-  </si>
-  <si>
-    <t>Se ponen guapos</t>
-  </si>
-  <si>
-    <t>Ruta de la Transformación</t>
-  </si>
-  <si>
-    <t>Reinician transmisiones</t>
-  </si>
-  <si>
-    <t>RTVH</t>
-  </si>
-  <si>
-    <t>Recuperación radiodifusoras</t>
-  </si>
-  <si>
-    <t>Alistan CEAR para inauguración</t>
-  </si>
-  <si>
-    <t>Centro de Alto Rendimiento</t>
-  </si>
-  <si>
-    <t>PRESENTAN SITIO WEB RUMBO A ELECCIONES 2027</t>
-  </si>
-  <si>
-    <t>Elecciones</t>
-  </si>
-  <si>
-    <t>PESH no tiene comités</t>
-  </si>
-  <si>
-    <t>pérdida de registro</t>
-  </si>
-  <si>
-    <t>REMODELACIÓN, ANTES DE 2028: GOBERNADOR</t>
-  </si>
-  <si>
-    <t>El PRI culpa a Julio Valera de multa de $5 millones</t>
-  </si>
-  <si>
-    <t>Multas Partidos</t>
-  </si>
-  <si>
-    <t>Iniciativa antitaurina, estancada en Hidalgo</t>
-  </si>
-  <si>
-    <t>Tauromaquia</t>
-  </si>
-  <si>
-    <t>Pachuca busca vencer maleficio</t>
-  </si>
-  <si>
-    <t>"Un hecho aislado", aparición de mantas</t>
-  </si>
-  <si>
-    <t>Narcomanta</t>
-  </si>
-  <si>
-    <t>Dirigente estatal niega la decadencia del PAN</t>
-  </si>
-  <si>
-    <t>Sube a 3 mil 200 el número de familias que deben reubicarse</t>
-  </si>
-  <si>
     <t>Reubicación de viviendas</t>
   </si>
   <si>
-    <t>Prometen autoridades su entrega para el mes de abril</t>
-  </si>
-  <si>
-    <t>Tendrá el estado 25 nuevos espacios previo al Mundial</t>
-  </si>
-  <si>
-    <t>Inhide</t>
-  </si>
-  <si>
-    <t>Mundial De Futbol</t>
-  </si>
-  <si>
-    <t>Alcalde dice que no le han notificado recomendación</t>
-  </si>
-  <si>
-    <t>Recomendaciones CDHEH</t>
-  </si>
-  <si>
-    <t>Exjefe contraterrorista exhibe a Trump: "Irán no era amenaza"</t>
-  </si>
-  <si>
-    <t>La Refinería cumple hoy medio siglo</t>
-  </si>
-  <si>
-    <t>Conmemoración Aniversario</t>
-  </si>
-  <si>
-    <t>Se encuentra en proceso de reconfiguración para disminuir impacto</t>
-  </si>
-  <si>
     <t>Refinería</t>
   </si>
   <si>
-    <t>Para operar en 2026, el IEEH requiere un alza presupuestal de 28 millones de pesos</t>
-  </si>
-  <si>
-    <t>Presupuesto IEEH</t>
-  </si>
-  <si>
-    <t>Derrama económica</t>
-  </si>
-  <si>
-    <t>Inversión de 25% del PIB es clave, dice en entrevista Eduardo Osuma</t>
-  </si>
-  <si>
-    <t>Un bombero cultiva el oficio de domeñar la lava en Islandia</t>
-  </si>
-  <si>
-    <t>IEEH analiza pedir 28 mdp extra de presupuesto tras recorte</t>
-  </si>
-  <si>
-    <t>Hidalgo recupera dos frecuencias de radio perdidas en 2022</t>
-  </si>
-  <si>
-    <t>Incendio en Dos Bocas deja cinco muertos: Pemex</t>
-  </si>
-  <si>
-    <t>Incendio refinería</t>
-  </si>
-  <si>
-    <t>Avanza control de fuga de petróleo en Santiago Talpacoya</t>
-  </si>
-  <si>
     <t>PC</t>
   </si>
   <si>
     <t>Fuga de hidrocarburo</t>
   </si>
   <si>
-    <t>¿Hay que separar la obra del artista? ¿Hay que dejar de cancelar completamente en todos los aspectos a les agresores? Son preguntas a las que le he dado vueltas una y otra vez. En mi librero y en mis listas de reproducción de música hay muchos artistas, políticxs, académicxs canceladxs. Seguro hay más de los que conozco públicamente, porque tengo claro que ninguna persona está exenta de haber discriminado o violentado a alguien, ni siquiera yo”.</t>
-  </si>
-  <si>
-    <t>Vuelven a encender su transmisión Radio Mezquital y Tlanchinol</t>
-  </si>
-  <si>
-    <t>Recibirá Hidalgo 50 mdp para construir canchas de fútbol en 22 municipios</t>
-  </si>
-  <si>
-    <t>Fortalece gobierno estatal infraestructura en Zempoala con 192 mdp</t>
-  </si>
-  <si>
-    <t>Aumentan a 17 los casos de sarampión en la entidad</t>
-  </si>
-  <si>
     <t>Sarampión</t>
   </si>
   <si>
-    <t>El objetivo del ejercicio del poder es servir a la gente: Julio Menchaca</t>
-  </si>
-  <si>
-    <t>La herencia musical de don Omegar Salazar es un "estilo de vida"</t>
-  </si>
-  <si>
-    <t>Pobladores dirimen sus diferencias a golpes y pedradas</t>
-  </si>
-  <si>
-    <t>Enfrentamiento</t>
-  </si>
-  <si>
-    <t>Acercan servicios estatales a la población de Yahualica</t>
-  </si>
-  <si>
-    <t>Unidades móviles</t>
-  </si>
-  <si>
-    <t>Capacita Salud a más de 5 mil personas para prevenir riesgos sanitarios</t>
-  </si>
-  <si>
     <t>Copriseh</t>
   </si>
   <si>
-    <t>Capacitación sanitaria</t>
-  </si>
-  <si>
     <t>Effetá</t>
   </si>
   <si>
-    <t>Golpeteo de regidores deja a Ajacuba sin inversiones locales y federales: alcaldesa</t>
-  </si>
-  <si>
     <t>Alcalde</t>
   </si>
   <si>
-    <t>Enfrentamiento Político</t>
-  </si>
-  <si>
-    <t>Menchaca revive dos estaciones tras años fuera del aire</t>
-  </si>
-  <si>
     <t>Recuperación de radiodifusoras</t>
   </si>
   <si>
-    <t>Gobernador lleva Rutas de la Transformación a Epazoyucan y Zempoala</t>
-  </si>
-  <si>
-    <t>INE castiga a partidos en Hidalgo con 21 millones</t>
-  </si>
-  <si>
-    <t>Aprueban 22 millones para Cuautepec</t>
-  </si>
-  <si>
-    <t>Deuda Pública</t>
-  </si>
-  <si>
-    <t>Cae presunta banda de robo de autos en Pachuca</t>
-  </si>
-  <si>
-    <t>Detención</t>
-  </si>
-  <si>
-    <t>Activan Comité de Emergencias ante fuertes lluvias</t>
-  </si>
-  <si>
-    <t>Reunión Gabinete De Seguridad</t>
-  </si>
-  <si>
-    <t>Policías de Pachuca asisten a mujer de la tercera edad que se encontraba desorientada</t>
-  </si>
-  <si>
-    <t>IEEH presenta la nueva imagen y funcionalidad de su página web</t>
-  </si>
-  <si>
-    <t>Plataforma tecnológica</t>
-  </si>
-  <si>
-    <t>Menchaca anuncia reinicio de trnasmisiones de Radio Mezquital y la Voz de la Sierra Hidalguense</t>
-  </si>
-  <si>
-    <t>Refinería de Tula cumple 50 años de legado, impacto y futuro</t>
-  </si>
-  <si>
-    <t>Copladem</t>
-  </si>
-  <si>
     <t>COPLADEM</t>
   </si>
   <si>
-    <t>Bomberos de Atitalaquia controlan incendio de llantas</t>
-  </si>
-  <si>
-    <t>Control de incendios</t>
-  </si>
-  <si>
-    <t>Más de 450 personas participan en la primera caminata de luna llena en el Cerro de Gómez</t>
-  </si>
-  <si>
-    <t>Evento turístico</t>
-  </si>
-  <si>
-    <t>Construirán 25 canchas por el Mundial Social en Hidalgo: Conejo Pérez</t>
-  </si>
-  <si>
-    <t>Reinician transmisiones de Radio Mezqutial y la Voz de la Sierra Hidalguense</t>
-  </si>
-  <si>
-    <t>Apoyo para madres trabajadoras en la entidad: conoce fecha</t>
-  </si>
-  <si>
-    <t>Programas del Pueblo</t>
-  </si>
-  <si>
-    <t>Inaugura Jorge Reyes los nuevos murales del Barrio del Arbolito</t>
-  </si>
-  <si>
-    <t>Exalcalde</t>
-  </si>
-  <si>
-    <t>Muralismo</t>
-  </si>
-  <si>
-    <t>Presenta CNDH acción de inconstitucionalidad contra Apan</t>
-  </si>
-  <si>
-    <t>Inconstitucionalidad</t>
-  </si>
-  <si>
-    <t>México impulsa plan b electoral con recorte de privilegios</t>
-  </si>
-  <si>
-    <t>Radio Mezquital y La Voz de la Sierra Hidalguense, al aire</t>
-  </si>
-  <si>
-    <t>La Secretaría de Turismo ha realizado más de mil giras</t>
-  </si>
-  <si>
-    <t>Promoción turística</t>
-  </si>
-  <si>
-    <t>Ejecutaron a balazos a hombre en su casa, frente a su novia</t>
-  </si>
-  <si>
-    <t>Tras el puente los turistas dejan en el estado 260 mdp</t>
+    <t>DJS impulsan la escena musical</t>
+  </si>
+  <si>
+    <t>En Hidalgo han localizado a 86 personas reportadas desaparecidas</t>
+  </si>
+  <si>
+    <t>Localización de persona</t>
+  </si>
+  <si>
+    <t>Identifican asentamiento preshipánico</t>
+  </si>
+  <si>
+    <t>INAH</t>
+  </si>
+  <si>
+    <t>Zona Arqueológica</t>
+  </si>
+  <si>
+    <t>Señalan riesgos en uso de IA</t>
+  </si>
+  <si>
+    <t>Dallece lomito por gusano barrenador</t>
+  </si>
+  <si>
+    <t>Gusano barrenador</t>
+  </si>
+  <si>
+    <t>Reprueban revisión unos 40 balnearios</t>
+  </si>
+  <si>
+    <t>Supervisión sanitaria</t>
+  </si>
+  <si>
+    <t>Casas del Bienestar aún en construcción</t>
+  </si>
+  <si>
+    <t>DESCTI</t>
+  </si>
+  <si>
+    <t>Celebran al teatro</t>
+  </si>
+  <si>
+    <t>Cecultah</t>
+  </si>
+  <si>
+    <t>Días Internacionales</t>
+  </si>
+  <si>
+    <t>Levantan bloqueo en San Salvador</t>
+  </si>
+  <si>
+    <t>Bloqueo Carretero</t>
+  </si>
+  <si>
+    <t>Congreso recortaría gastos por el Plan B del gobierno federal</t>
+  </si>
+  <si>
+    <t>Clúster de franquicias</t>
+  </si>
+  <si>
+    <t>Atracción De Inversiones</t>
+  </si>
+  <si>
+    <t>inician limpia de anuncios espectaculares</t>
+  </si>
+  <si>
+    <t>Imagen Urbana</t>
+  </si>
+  <si>
+    <t>Jóvenes, mayoría de las personas desaparecidas</t>
+  </si>
+  <si>
+    <t>CBPEH</t>
+  </si>
+  <si>
+    <t>Personas desaparecidas</t>
+  </si>
+  <si>
+    <t>Frenan dictamen en Congreso local sobre buscadores</t>
+  </si>
+  <si>
+    <t>GLMorena</t>
+  </si>
+  <si>
+    <t>Búsqueda de personas</t>
+  </si>
+  <si>
+    <t>LAS MEMORIAS  DE LA PANDEMIA  DE CORONAVIRUS  EN LA ENTIDAD</t>
+  </si>
+  <si>
+    <t>Covid 19</t>
+  </si>
+  <si>
+    <t>Mohamed, rival tuzo incómodo</t>
+  </si>
+  <si>
+    <t>Preparan la edición 57 del viacrucis en El Arbolito</t>
+  </si>
+  <si>
+    <t>Viacrucis</t>
+  </si>
+  <si>
+    <t>Van por sancionar violación a la intimidad mediante la IA</t>
+  </si>
+  <si>
+    <t>Violencia digital</t>
+  </si>
+  <si>
+    <t>Encuentran a 9 de cada diez desaparecidos en el trimestre</t>
+  </si>
+  <si>
+    <t>Operativo. Verifican posibles irregularidades en autos</t>
+  </si>
+  <si>
+    <t>Operativo de Seguridad</t>
+  </si>
+  <si>
+    <t>México y EU, "matrimonio con resultados reales"</t>
+  </si>
+  <si>
+    <t>Delcy destituye al ministro de Defensa en Venezuela</t>
+  </si>
+  <si>
+    <t>Detectan en ganado 89 casos de gusano barrenador</t>
+  </si>
+  <si>
+    <t>PUBLICIDAD</t>
+  </si>
+  <si>
+    <t>Atienden problemática en San Salvador tras retención de alcalde</t>
+  </si>
+  <si>
+    <t>Retención alcalde</t>
+  </si>
+  <si>
+    <t>Morena anticipa respaldo a iniciativa para reducir regidurías</t>
+  </si>
+  <si>
+    <t>Desaparecen tres hombres; salieron a vender camionetas</t>
+  </si>
+  <si>
+    <t>Sheinbaum invita a Felipe VI al Mundial</t>
+  </si>
+  <si>
+    <t>El choque entre Morena Hidalgo y el Congreso local contra la Presidencia también deja un mensaje  incómodo hacia dentro del propio movimiento. Si no hay acuerdo en cómo medir la austeridad, la  narrativa de disciplina pierde consistencia mientras la soberbia se impone”.</t>
+  </si>
+  <si>
+    <t>Supera Hidalgo el 90% de localización de personas desaparecidas</t>
+  </si>
+  <si>
+    <t>Avanza al 90% limpieza de crudo  maya en Tlapacoya</t>
+  </si>
+  <si>
+    <t>Invita Infonavit a obtener descuentos  sobre créditos hipotecarios</t>
+  </si>
+  <si>
+    <t>Infonavit</t>
+  </si>
+  <si>
+    <t>Crédito hipotecario</t>
+  </si>
+  <si>
+    <t>Aprueban modificación de Ley de  Ingresos en ayuntamiento de Pachuca</t>
+  </si>
+  <si>
+    <t>Ley De Ingresos</t>
+  </si>
+  <si>
+    <t>Se prevé que se repita la sequía como en el 2024</t>
+  </si>
+  <si>
+    <t>Conagua</t>
+  </si>
+  <si>
+    <t>Sequía</t>
+  </si>
+  <si>
+    <t>Gobierno refuerza compromiso con jornaleros</t>
+  </si>
+  <si>
+    <t>Vinculación Laboral</t>
+  </si>
+  <si>
+    <t>Comerciantes de la UCLA esperan convocatoria para renovar dirigencia</t>
+  </si>
+  <si>
+    <t>Hidalgo, ejemplo a seguir en capacitación para el trabajo</t>
+  </si>
+  <si>
+    <t>ICATHI</t>
+  </si>
+  <si>
+    <t>Capacitación Laboral</t>
+  </si>
+  <si>
+    <t>Conmemoran el 88 aniversario de la Expropiación Petrolera</t>
+  </si>
+  <si>
+    <t>Pide Morena frenar acusaciones sin sustento contra alcaldes de Hidalgo</t>
+  </si>
+  <si>
+    <t>Golpeteo político</t>
+  </si>
+  <si>
+    <t>Tecnología, drones y perros</t>
+  </si>
+  <si>
+    <t>Refuerzo De Seguridad</t>
+  </si>
+  <si>
+    <t>La radio que nunca debió perderse</t>
+  </si>
+  <si>
+    <t>Editorial</t>
+  </si>
+  <si>
+    <t>Alcalde de San Salvador no fue retenido""</t>
+  </si>
+  <si>
+    <t>Reportan 94 desaparecidos en hidalgo en 2026</t>
+  </si>
+  <si>
+    <t>Proponen impedir que deudores ocupen cargos en Hidalgo</t>
+  </si>
+  <si>
+    <t>Deudor Alimentario</t>
+  </si>
+  <si>
+    <t>Derrame de crudo en Tlapacoya fue provocado por vandalismo</t>
+  </si>
+  <si>
+    <t>Mediará Gobierno estatal en conflicto de San Salvador por distribución de recursos</t>
+  </si>
+  <si>
+    <t>Atención A Manifestantes</t>
+  </si>
+  <si>
+    <t>Claudia Sandoval presenta obras prioritarias para 2026 en Copladem</t>
+  </si>
+  <si>
+    <t>Petroleros conmemoran 50 años de la Refinería de Tulay 88 años de la Expropiación Petrolera</t>
+  </si>
+  <si>
+    <t>Respalda Menchaca reforma electoral, pero pide analizar impacto local</t>
+  </si>
+  <si>
+    <t>Impulsan iniciativa para incorporar control emocional y prevención de violencia vial en la movilidad de Hidalgo</t>
+  </si>
+  <si>
+    <t>Iniciativa</t>
+  </si>
+  <si>
+    <t>Refuerza Pachuca despliegue operativo con acciones coordinadas de seguridad</t>
+  </si>
+  <si>
+    <t>Tula, sede regional por el Día Mundial del Agua</t>
+  </si>
+  <si>
+    <t>Reinauguran sala de artes en Pachuca con programación especial</t>
+  </si>
+  <si>
+    <t>Evento Cultural</t>
+  </si>
+  <si>
+    <t>En Xochicoatlán, convocan a programa de relocalización de vivienda</t>
+  </si>
+  <si>
+    <t>SSPH frustra robo de 32 toneladas de mercancía en Tepeji</t>
+  </si>
+  <si>
+    <t>Combate a la delincuencia</t>
+  </si>
+  <si>
+    <t>Hidalgo, debajo de la media nacional en casos de sarampión</t>
+  </si>
+  <si>
+    <t>Buscan a tres hombres desaparecidos en Tulancingo</t>
+  </si>
+  <si>
+    <t>Retienen a edil por incumplir promesas de campaña</t>
+  </si>
+  <si>
+    <t>Quitarán patria potestad a padres que simulen ingresos</t>
+  </si>
+  <si>
+    <t>Indagan causas de incendio en refinería de Pemex</t>
+  </si>
+  <si>
+    <t>Los trabajadores de gobierno tienen derecho a ejercer la desconexión digital, pues muchas veces con estas herramientas se alarga su tiempo de labor. Interesante la propuesta de ley de los diputados locales</t>
   </si>
 </sst>
 </file>
@@ -913,8 +880,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J71" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J71" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J64" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J64" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1280,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1329,100 +1296,100 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B2" t="s">
         <v>70</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>98</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B3" t="s">
         <v>70</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="G3" t="s">
-        <v>91</v>
+        <v>104</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B4" t="s">
         <v>70</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
       </c>
       <c r="E4" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>106</v>
       </c>
       <c r="G4" t="s">
-        <v>87</v>
+        <v>107</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1431,13 +1398,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B5" t="s">
         <v>70</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
@@ -1465,32 +1432,32 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B6" t="s">
         <v>70</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>83</v>
+        <v>110</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1499,59 +1466,59 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B7" t="s">
         <v>70</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>10</v>
+        <v>97</v>
       </c>
       <c r="G7" t="s">
-        <v>69</v>
+        <v>112</v>
       </c>
       <c r="H7" t="s">
         <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B8" t="s">
         <v>70</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D8" t="s">
         <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>51</v>
       </c>
       <c r="F8" t="s">
-        <v>15</v>
+        <v>114</v>
       </c>
       <c r="G8" t="s">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
@@ -1567,25 +1534,25 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B9" t="s">
         <v>71</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>116</v>
       </c>
       <c r="G9" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
@@ -1596,237 +1563,237 @@
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B10" t="s">
         <v>71</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G10" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="H10" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B11" t="s">
         <v>71</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D11" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E11" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="G11" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="H11" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B12" t="s">
         <v>71</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>113</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="H12" t="s">
         <v>26</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B13" t="s">
         <v>71</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G13" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B14" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="F14" t="s">
-        <v>44</v>
+        <v>126</v>
       </c>
       <c r="G14" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="H14" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>68</v>
+        <v>129</v>
       </c>
       <c r="G15" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="H15" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B16" t="s">
         <v>75</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F16" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="G16" t="s">
-        <v>109</v>
+        <v>132</v>
       </c>
       <c r="H16" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1834,37 +1801,37 @@
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B17" t="s">
         <v>75</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>88</v>
+        <v>10</v>
       </c>
       <c r="F17" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G17" t="s">
-        <v>123</v>
+        <v>82</v>
       </c>
       <c r="H17" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1873,96 +1840,96 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B18" t="s">
         <v>75</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" t="s">
+        <v>135</v>
+      </c>
+      <c r="H18" t="s">
+        <v>11</v>
+      </c>
+      <c r="I18" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J18" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D19" t="s">
         <v>13</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E19" t="s">
         <v>37</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F19" t="s">
         <v>37</v>
       </c>
-      <c r="G18" t="s">
-        <v>125</v>
-      </c>
-      <c r="H18" t="s">
-        <v>16</v>
-      </c>
-      <c r="I18" t="str">
+      <c r="G19" t="s">
+        <v>137</v>
+      </c>
+      <c r="H19" t="s">
+        <v>11</v>
+      </c>
+      <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J18" t="str">
+      <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B19" t="s">
-        <v>75</v>
-      </c>
-      <c r="C19" s="6" t="s">
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" t="s">
         <v>126</v>
       </c>
-      <c r="D19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" t="s">
-        <v>10</v>
-      </c>
-      <c r="G19" t="s">
-        <v>82</v>
-      </c>
-      <c r="H19" t="s">
-        <v>11</v>
-      </c>
-      <c r="I19" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J19" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A20" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B20" t="s">
-        <v>75</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D20" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" t="s">
-        <v>25</v>
-      </c>
-      <c r="F20" t="s">
-        <v>25</v>
-      </c>
       <c r="G20" t="s">
-        <v>128</v>
+        <v>104</v>
       </c>
       <c r="H20" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1970,98 +1937,98 @@
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="D21" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E21" t="s">
-        <v>49</v>
+        <v>17</v>
       </c>
       <c r="F21" t="s">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="G21" t="s">
-        <v>89</v>
+        <v>140</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B22" t="s">
         <v>72</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="D22" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F22" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G22" t="s">
-        <v>131</v>
+        <v>69</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B23" t="s">
         <v>72</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="G23" t="s">
-        <v>91</v>
+        <v>69</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
@@ -2077,28 +2044,28 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B24" t="s">
         <v>72</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>28</v>
+        <v>57</v>
       </c>
       <c r="F24" t="s">
-        <v>134</v>
+        <v>57</v>
       </c>
       <c r="G24" t="s">
-        <v>135</v>
+        <v>110</v>
       </c>
       <c r="H24" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2111,32 +2078,32 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B25" t="s">
         <v>72</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="D25" t="s">
-        <v>12</v>
+        <v>87</v>
       </c>
       <c r="E25" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>137</v>
+        <v>87</v>
       </c>
       <c r="H25" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2145,66 +2112,66 @@
     </row>
     <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="D26" t="s">
         <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F26" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G26" t="s">
-        <v>84</v>
+        <v>146</v>
       </c>
       <c r="H26" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J26" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B27" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
+        <v>37</v>
+      </c>
+      <c r="F27" t="s">
+        <v>129</v>
+      </c>
+      <c r="G27" t="s">
+        <v>91</v>
+      </c>
+      <c r="H27" t="s">
+        <v>11</v>
+      </c>
+      <c r="I27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
-      </c>
-      <c r="J26" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A27" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B27" t="s">
-        <v>72</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="D27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" t="s">
-        <v>14</v>
-      </c>
-      <c r="F27" t="s">
-        <v>85</v>
-      </c>
-      <c r="G27" t="s">
-        <v>140</v>
-      </c>
-      <c r="H27" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2213,202 +2180,202 @@
     </row>
     <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
       </c>
       <c r="E28" t="s">
+        <v>23</v>
+      </c>
+      <c r="F28" t="s">
+        <v>23</v>
+      </c>
+      <c r="G28" t="s">
+        <v>127</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="I28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B29" t="s">
+        <v>73</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
         <v>14</v>
       </c>
-      <c r="F28" t="s">
-        <v>85</v>
-      </c>
-      <c r="G28" t="s">
-        <v>142</v>
-      </c>
-      <c r="H28" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" t="str">
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Presidencia de la República</v>
       </c>
-      <c r="J28" t="str">
+      <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B29" t="s">
-        <v>72</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F29" t="s">
-        <v>44</v>
-      </c>
-      <c r="G29" t="s">
-        <v>144</v>
-      </c>
-      <c r="H29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J29" t="str">
+    <row r="30" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B30" t="s">
+        <v>73</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>19</v>
+      </c>
+      <c r="F30" t="s">
+        <v>19</v>
+      </c>
+      <c r="G30" t="s">
+        <v>91</v>
+      </c>
+      <c r="H30" t="s">
+        <v>16</v>
+      </c>
+      <c r="I30" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A30" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B30" t="s">
-        <v>72</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D30" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" t="s">
-        <v>32</v>
-      </c>
-      <c r="F30" t="s">
-        <v>32</v>
-      </c>
-      <c r="G30" t="s">
-        <v>145</v>
-      </c>
-      <c r="H30" t="s">
-        <v>26</v>
-      </c>
-      <c r="I30" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J30" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F31" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G31" t="s">
-        <v>69</v>
+        <v>104</v>
       </c>
       <c r="H31" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F32" t="s">
-        <v>10</v>
+        <v>94</v>
       </c>
       <c r="G32" t="s">
-        <v>69</v>
+        <v>95</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="F33" t="s">
-        <v>44</v>
+        <v>154</v>
       </c>
       <c r="G33" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2417,59 +2384,59 @@
     </row>
     <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="D34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F34" t="s">
-        <v>113</v>
+        <v>37</v>
       </c>
       <c r="G34" t="s">
-        <v>114</v>
+        <v>157</v>
       </c>
       <c r="H34" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B35" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
         <v>14</v>
       </c>
       <c r="F35" t="s">
-        <v>85</v>
+        <v>159</v>
       </c>
       <c r="G35" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
@@ -2483,27 +2450,27 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B36" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="D36" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="F36" t="s">
-        <v>153</v>
+        <v>20</v>
       </c>
       <c r="G36" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
@@ -2517,15 +2484,15 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="135" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
@@ -2553,25 +2520,25 @@
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B38" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="D38" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="F38" t="s">
-        <v>25</v>
+        <v>165</v>
       </c>
       <c r="G38" t="s">
-        <v>114</v>
+        <v>166</v>
       </c>
       <c r="H38" t="s">
         <v>26</v>
@@ -2582,123 +2549,123 @@
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B39" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="F39" t="s">
-        <v>134</v>
+        <v>85</v>
       </c>
       <c r="G39" t="s">
-        <v>135</v>
+        <v>93</v>
       </c>
       <c r="H39" t="s">
         <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B40" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="F40" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="G40" t="s">
-        <v>111</v>
+        <v>169</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B41" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>159</v>
+        <v>170</v>
       </c>
       <c r="D41" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E41" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F41" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>160</v>
+        <v>171</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>161</v>
+        <v>172</v>
       </c>
       <c r="D42" t="s">
-        <v>9</v>
+        <v>173</v>
       </c>
       <c r="E42" t="s">
         <v>25</v>
@@ -2707,10 +2674,10 @@
         <v>25</v>
       </c>
       <c r="G42" t="s">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="H42" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2721,129 +2688,129 @@
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B43" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F43" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G43" t="s">
-        <v>69</v>
+        <v>146</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B44" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="D44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="G44" t="s">
-        <v>164</v>
+        <v>127</v>
       </c>
       <c r="H44" t="s">
         <v>16</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B45" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F45" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="G45" t="s">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B46" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="D46" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="E46" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F46" t="s">
-        <v>168</v>
+        <v>94</v>
       </c>
       <c r="G46" t="s">
-        <v>169</v>
+        <v>95</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
@@ -2859,251 +2826,251 @@
     </row>
     <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B47" t="s">
-        <v>170</v>
+        <v>78</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="D47" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F47" t="s">
-        <v>172</v>
+        <v>2</v>
       </c>
       <c r="G47" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B48" t="s">
-        <v>170</v>
+        <v>78</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>25</v>
+        <v>99</v>
       </c>
       <c r="G48" t="s">
-        <v>175</v>
+        <v>101</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B49" t="s">
-        <v>170</v>
+        <v>78</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E49" t="s">
+        <v>14</v>
+      </c>
+      <c r="F49" t="s">
+        <v>85</v>
+      </c>
+      <c r="G49" t="s">
+        <v>93</v>
+      </c>
+      <c r="H49" t="s">
+        <v>11</v>
+      </c>
+      <c r="I49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B50" t="s">
+        <v>78</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
         <v>25</v>
       </c>
-      <c r="F49" t="s">
+      <c r="F50" t="s">
         <v>25</v>
       </c>
-      <c r="G49" t="s">
-        <v>111</v>
-      </c>
-      <c r="H49" t="s">
-        <v>11</v>
-      </c>
-      <c r="I49" t="str">
+      <c r="G50" t="s">
+        <v>83</v>
+      </c>
+      <c r="H50" t="s">
+        <v>11</v>
+      </c>
+      <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J49" t="str">
+      <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B50" t="s">
-        <v>170</v>
-      </c>
-      <c r="C50" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="D50" t="s">
-        <v>12</v>
-      </c>
-      <c r="E50" t="s">
-        <v>88</v>
-      </c>
-      <c r="F50" t="s">
-        <v>88</v>
-      </c>
-      <c r="G50" t="s">
-        <v>90</v>
-      </c>
-      <c r="H50" t="s">
-        <v>16</v>
-      </c>
-      <c r="I50" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J50" t="str">
+    <row r="51" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B51" t="s">
+        <v>78</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>37</v>
+      </c>
+      <c r="F51" t="s">
+        <v>37</v>
+      </c>
+      <c r="G51" t="s">
+        <v>185</v>
+      </c>
+      <c r="H51" t="s">
+        <v>11</v>
+      </c>
+      <c r="I51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B51" t="s">
-        <v>170</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="D51" t="s">
-        <v>12</v>
-      </c>
-      <c r="E51" t="s">
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="5">
+        <v>46100</v>
+      </c>
+      <c r="B52" t="s">
+        <v>78</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
         <v>17</v>
       </c>
-      <c r="F51" t="s">
+      <c r="F52" t="s">
         <v>17</v>
       </c>
-      <c r="G51" t="s">
-        <v>179</v>
-      </c>
-      <c r="H51" t="s">
-        <v>11</v>
-      </c>
-      <c r="I51" t="str">
+      <c r="G52" t="s">
+        <v>171</v>
+      </c>
+      <c r="H52" t="s">
+        <v>11</v>
+      </c>
+      <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
       </c>
-      <c r="J51" t="str">
+      <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B52" t="s">
-        <v>170</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D52" t="s">
-        <v>12</v>
-      </c>
-      <c r="E52" t="s">
-        <v>23</v>
-      </c>
-      <c r="F52" t="s">
-        <v>23</v>
-      </c>
-      <c r="G52" t="s">
-        <v>181</v>
-      </c>
-      <c r="H52" t="s">
-        <v>11</v>
-      </c>
-      <c r="I52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B53" t="s">
         <v>78</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="D53" t="s">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F53" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G53" t="s">
-        <v>183</v>
+        <v>117</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B54" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
@@ -3112,10 +3079,10 @@
         <v>17</v>
       </c>
       <c r="F54" t="s">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="G54" t="s">
-        <v>86</v>
+        <v>189</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
@@ -3131,32 +3098,32 @@
     </row>
     <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B55" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D55" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E55" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="F55" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="G55" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="H55" t="s">
         <v>11</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3165,25 +3132,25 @@
     </row>
     <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B56" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D56" t="s">
-        <v>13</v>
+        <v>87</v>
       </c>
       <c r="E56" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="F56" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G56" t="s">
-        <v>175</v>
+        <v>92</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
@@ -3194,89 +3161,89 @@
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B57" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F57" t="s">
-        <v>85</v>
+        <v>23</v>
       </c>
       <c r="G57" t="s">
-        <v>142</v>
+        <v>192</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B58" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="D58" t="s">
-        <v>92</v>
+        <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F58" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="G58" t="s">
-        <v>190</v>
+        <v>96</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B59" t="s">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>191</v>
+        <v>88</v>
       </c>
       <c r="D59" t="s">
-        <v>12</v>
+        <v>87</v>
       </c>
       <c r="E59" t="s">
         <v>17</v>
@@ -3285,7 +3252,7 @@
         <v>17</v>
       </c>
       <c r="G59" t="s">
-        <v>192</v>
+        <v>89</v>
       </c>
       <c r="H59" t="s">
         <v>11</v>
@@ -3299,80 +3266,80 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B60" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D60" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E60" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F60" t="s">
-        <v>17</v>
+        <v>126</v>
       </c>
       <c r="G60" t="s">
-        <v>194</v>
+        <v>127</v>
       </c>
       <c r="H60" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B61" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="C61" s="6" t="s">
         <v>195</v>
       </c>
       <c r="D61" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="F61" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="G61" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="H61" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B62" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="C62" s="6" t="s">
         <v>196</v>
@@ -3381,330 +3348,92 @@
         <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="F62" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="G62" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
       </c>
       <c r="I62" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J62" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B63" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>161</v>
+        <v>197</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="F63" t="s">
-        <v>25</v>
+        <v>85</v>
       </c>
       <c r="G63" t="s">
-        <v>111</v>
+        <v>69</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
       </c>
       <c r="I63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
-        <v>46099</v>
+        <v>46100</v>
       </c>
       <c r="B64" t="s">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D64" t="s">
-        <v>12</v>
+        <v>173</v>
       </c>
       <c r="E64" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="F64" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="G64" t="s">
-        <v>198</v>
+        <v>185</v>
       </c>
       <c r="H64" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A65" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B65" t="s">
-        <v>29</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="D65" t="s">
-        <v>12</v>
-      </c>
-      <c r="E65" t="s">
-        <v>17</v>
-      </c>
-      <c r="F65" t="s">
-        <v>200</v>
-      </c>
-      <c r="G65" t="s">
-        <v>201</v>
-      </c>
-      <c r="H65" t="s">
-        <v>11</v>
-      </c>
-      <c r="I65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A66" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B66" t="s">
-        <v>29</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="D66" t="s">
-        <v>92</v>
-      </c>
-      <c r="E66" t="s">
-        <v>17</v>
-      </c>
-      <c r="F66" t="s">
-        <v>17</v>
-      </c>
-      <c r="G66" t="s">
-        <v>94</v>
-      </c>
-      <c r="H66" t="s">
-        <v>11</v>
-      </c>
-      <c r="I66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A67" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B67" t="s">
-        <v>81</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="D67" t="s">
-        <v>13</v>
-      </c>
-      <c r="E67" t="s">
-        <v>37</v>
-      </c>
-      <c r="F67" t="s">
-        <v>37</v>
-      </c>
-      <c r="G67" t="s">
-        <v>203</v>
-      </c>
-      <c r="H67" t="s">
-        <v>11</v>
-      </c>
-      <c r="I67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A68" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B68" t="s">
-        <v>81</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="D68" t="s">
-        <v>12</v>
-      </c>
-      <c r="E68" t="s">
-        <v>14</v>
-      </c>
-      <c r="F68" t="s">
-        <v>14</v>
-      </c>
-      <c r="G68" t="s">
-        <v>107</v>
-      </c>
-      <c r="H68" t="s">
-        <v>11</v>
-      </c>
-      <c r="I68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A69" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B69" t="s">
-        <v>81</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D69" t="s">
-        <v>12</v>
-      </c>
-      <c r="E69" t="s">
-        <v>25</v>
-      </c>
-      <c r="F69" t="s">
-        <v>25</v>
-      </c>
-      <c r="G69" t="s">
-        <v>175</v>
-      </c>
-      <c r="H69" t="s">
-        <v>11</v>
-      </c>
-      <c r="I69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A70" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B70" t="s">
-        <v>81</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="D70" t="s">
-        <v>12</v>
-      </c>
-      <c r="E70" t="s">
-        <v>32</v>
-      </c>
-      <c r="F70" t="s">
-        <v>2</v>
-      </c>
-      <c r="G70" t="s">
-        <v>207</v>
-      </c>
-      <c r="H70" t="s">
-        <v>11</v>
-      </c>
-      <c r="I70" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J70" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A71" s="5">
-        <v>46099</v>
-      </c>
-      <c r="B71" t="s">
-        <v>81</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="D71" t="s">
-        <v>12</v>
-      </c>
-      <c r="E71" t="s">
-        <v>23</v>
-      </c>
-      <c r="F71" t="s">
-        <v>23</v>
-      </c>
-      <c r="G71" t="s">
-        <v>96</v>
-      </c>
-      <c r="H71" t="s">
-        <v>16</v>
-      </c>
-      <c r="I71" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J71" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reporte 24 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45411589-3632-4C10-8284-BC8CB6196A7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2247F84-3C23-40D6-A3D7-02B22C45E09C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
+    <workbookView xWindow="360" yWindow="360" windowWidth="20460" windowHeight="10890" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="608" uniqueCount="189">
   <si>
     <t>Fecha</t>
   </si>
@@ -270,316 +270,340 @@
     <t>Nivel</t>
   </si>
   <si>
+    <t>Gabinete</t>
+  </si>
+  <si>
+    <t>Plaza Juárez</t>
+  </si>
+  <si>
+    <t>Deportes</t>
+  </si>
+  <si>
+    <t>Effetá</t>
+  </si>
+  <si>
+    <t>Huracán Priscilla</t>
+  </si>
+  <si>
+    <t>Semana Santa</t>
+  </si>
+  <si>
+    <t>Disposición de basura</t>
+  </si>
+  <si>
+    <t>Milenio Hidalgo</t>
+  </si>
+  <si>
+    <t>Conmemoración Aniversario</t>
+  </si>
+  <si>
+    <t>Publicidad</t>
+  </si>
+  <si>
+    <t>Editorial</t>
+  </si>
+  <si>
+    <t>PRI</t>
+  </si>
+  <si>
+    <t>Impacta gusano barrenador al sector cárnico</t>
+  </si>
+  <si>
+    <t>Gusano barrenador</t>
+  </si>
+  <si>
+    <t>Entregan apoyos a 24 cooperativas en Hidalgo</t>
+  </si>
+  <si>
+    <t>Economía social</t>
+  </si>
+  <si>
+    <t>Afecta el aumento de diésel en servicios agrícolas</t>
+  </si>
+  <si>
+    <t>Prohíben caza de venados</t>
+  </si>
+  <si>
+    <t>Protección Biodiversidad</t>
+  </si>
+  <si>
+    <t>Exponen violencia política de género en El Boxtha</t>
+  </si>
+  <si>
+    <t>Violencia Política De Género</t>
+  </si>
+  <si>
+    <t>Proyectan otra ruta troncal del Tuzobús</t>
+  </si>
+  <si>
+    <t>Modernización Tuzobús</t>
+  </si>
+  <si>
+    <t>Inmueble recuperado será sede del Tribunal de Justicia Administrativa</t>
+  </si>
+  <si>
+    <t>Recuperación De Espacios Públicos</t>
+  </si>
+  <si>
+    <t>Para salvar vidas</t>
+  </si>
+  <si>
+    <t>Hospital del Niño</t>
+  </si>
+  <si>
+    <t>Entrenamiento médico</t>
+  </si>
+  <si>
+    <t>Gabinete desplegará policías</t>
+  </si>
+  <si>
+    <t>Reunión Gabinete De Seguridad</t>
+  </si>
+  <si>
+    <t>Mandarán basura a Querétaro</t>
+  </si>
+  <si>
+    <t>Detectan 20% de niños con obesidad</t>
+  </si>
+  <si>
+    <t>Vida Saludable</t>
+  </si>
+  <si>
+    <t>INAMOVIBLE,  EN PACHUCA</t>
+  </si>
+  <si>
+    <t>Mbappé apunta al Mundial 2026</t>
+  </si>
+  <si>
+    <t>PLANTEAN NUEVA RUTA TRONCAL DEL SISTEMA TUZOBÚS</t>
+  </si>
+  <si>
+    <t>POR ACOSO SEXUAL, RETIRAN CONCESIÓN A CAFETERÍA ESCOLAR,  INFORMÓ CASTREJÓN</t>
+  </si>
+  <si>
+    <t>Acoso Sexual</t>
+  </si>
+  <si>
+    <t>El Hospital del Niño DIF cumplió años</t>
+  </si>
+  <si>
+    <t>PRI Hidalgo alista una denuncia tras freno a iniciativa</t>
+  </si>
+  <si>
+    <t>Concluye Pachuca pavimentaciones</t>
+  </si>
+  <si>
+    <t>Rehabilitación Vial</t>
+  </si>
+  <si>
+    <t>Tragedia en la sierra: viven entre ruinas, riesgos, incertidumbre...</t>
+  </si>
+  <si>
+    <t>Invierten apenas 15 mdp en obras de rehabilitación</t>
+  </si>
+  <si>
+    <t>Relleno sanitario de Tula rebasado e irregular</t>
+  </si>
+  <si>
+    <t>Relleno Sanitario</t>
+  </si>
+  <si>
+    <t>Moverse en Pachuca es aun más lento</t>
+  </si>
+  <si>
+    <t>Movilidad urbana</t>
+  </si>
+  <si>
+    <t>Registró PJE 126 quejas contra jueces durante 2025</t>
+  </si>
+  <si>
+    <t>Quejas contra jueces</t>
+  </si>
+  <si>
+    <t>Obesidad, caries y mala visión afectan a alumnos</t>
+  </si>
+  <si>
+    <t>Escribo con rima en imágenes en forma coloquial""</t>
+  </si>
+  <si>
+    <t>Más cocineros estadounidenses que mexicanos en sentencias</t>
+  </si>
+  <si>
+    <t>Incumplen 60% de balnearios con las normas de sanidad</t>
+  </si>
+  <si>
+    <t>Copriseh</t>
+  </si>
+  <si>
+    <t>Certificación sanitaria</t>
+  </si>
+  <si>
+    <t>Olivares se reúne con mujeres destacadas en la política</t>
+  </si>
+  <si>
+    <t>Reunión con actores</t>
+  </si>
+  <si>
+    <t>JMS admite  inquietud por  adjudicaciones  directas en ayuntamientos</t>
+  </si>
+  <si>
+    <t>Transparencia para el Pueblo</t>
+  </si>
+  <si>
+    <t>En ciernes, nueva  troncal para ampliar el sistema Tuzobús</t>
+  </si>
+  <si>
+    <t>Defiende edila cobro en playa  con cuchillo  en mano</t>
+  </si>
+  <si>
+    <t>Morena tiene que entender que gobernar con aliados transaccionales es gobernar con freno de mano.  Cada iniciativa importante tendrá que pasar por el filtro de los intereses del PT y el Verde. Cada reforma  estructural será objeto de negociación, de concesiones, de desgaste”.</t>
+  </si>
+  <si>
+    <t>Plan B</t>
+  </si>
+  <si>
+    <t>Otorga Menchaca 4.8 mdp en apoyos a 24 cooperativas hidalguenses</t>
+  </si>
+  <si>
+    <t>Alistan operativo de seguridad para Semana Santa en Hidalgo</t>
+  </si>
+  <si>
+    <t>Entrega Jorge Reyes pavimentaciones en Valle y Ampliación El Palmar</t>
+  </si>
+  <si>
+    <t>Alcalde</t>
+  </si>
+  <si>
+    <t>Hallan a menor de San Agustín Tlaxiaca en Morelos</t>
+  </si>
+  <si>
+    <t>Localización de persona</t>
+  </si>
+  <si>
+    <t>Con premios y baile cierran las fiestas de Tlanchinol</t>
+  </si>
+  <si>
+    <t>Juventud, cultura y deporte marcan el rumbo de una nueva etapa en Huejutla</t>
+  </si>
+  <si>
+    <t>Visita a escuela</t>
+  </si>
+  <si>
+    <t>Inauguraron encuentro cultural y deportivo de instituciones de educación superior</t>
+  </si>
+  <si>
+    <t>Universidades</t>
+  </si>
+  <si>
+    <t>Encuentro académico</t>
+  </si>
+  <si>
+    <t>Clínica comunitaria ofrece servicios accesibles</t>
+  </si>
+  <si>
+    <t>Clínica comunitaria</t>
+  </si>
+  <si>
+    <t>Denuncian doble venta y acuerdos tras disputa legal en predios de la Tres Huastecas</t>
+  </si>
+  <si>
+    <t>Obras atienden demanda pertinente: Jorge Reyes</t>
+  </si>
+  <si>
+    <t>alcalde</t>
+  </si>
+  <si>
+    <t>Ejecución de obras</t>
+  </si>
+  <si>
+    <t>¿Se busca sucesora?</t>
+  </si>
+  <si>
+    <t>Sucesión Gubernamental</t>
+  </si>
+  <si>
+    <t>Proyectan segunda troncal del Tuzobús</t>
+  </si>
+  <si>
+    <t>No a adjudicaciones directas</t>
+  </si>
+  <si>
+    <t>PRI afirma que le alcanzará para recuperar Hidalgo en 2028</t>
+  </si>
+  <si>
     <t>Marfeca</t>
   </si>
   <si>
-    <t>Gabinete</t>
-  </si>
-  <si>
-    <t>Plaza Juárez</t>
-  </si>
-  <si>
-    <t>Deportes</t>
-  </si>
-  <si>
-    <t>Policía municipal</t>
-  </si>
-  <si>
-    <t>Plan B</t>
-  </si>
-  <si>
-    <t>Effetá</t>
-  </si>
-  <si>
-    <t>Alcalde</t>
-  </si>
-  <si>
-    <t>Días Internacionales</t>
-  </si>
-  <si>
-    <t>CBPEH</t>
-  </si>
-  <si>
-    <t>Búsqueda de personas</t>
-  </si>
-  <si>
-    <t>Viacrucis</t>
-  </si>
-  <si>
-    <t>Iniciativa</t>
-  </si>
-  <si>
-    <t>Combate a la delincuencia</t>
-  </si>
-  <si>
-    <t>Fortalece la inversión privada al sector textil</t>
-  </si>
-  <si>
-    <t>Reunión Con Empresarios</t>
-  </si>
-  <si>
-    <t>Tensión en Ixmiquilpan por revuelta social</t>
-  </si>
-  <si>
-    <t>Leyenda del crimen en La Pasadita</t>
-  </si>
-  <si>
-    <t>Festejan con mañanitas a San José</t>
-  </si>
-  <si>
-    <t>Pese a no cumplir, balnearios abrirán</t>
-  </si>
-  <si>
-    <t>Balnearios</t>
-  </si>
-  <si>
-    <t>Alistan la edición 45 de la Muestra Gastronómica</t>
-  </si>
-  <si>
-    <t>Festival Gastronómico</t>
-  </si>
-  <si>
-    <t>Dirigentes del PRDH se aumentan salario hasta en w w w.e l u n i ve r s a l h i d a l g o.c o m . m x LUIS SORIANO 100 por ciento</t>
-  </si>
-  <si>
-    <t>Tabulador salarial</t>
-  </si>
-  <si>
-    <t>Sabores con magia</t>
-  </si>
-  <si>
-    <t>“El 20 de marzo, el mundo celebra el Día Internacional de la Felicidad; este año la fecha tiene un simbolismo especial, coincide con el equinoccio que marca el...”</t>
-  </si>
-  <si>
-    <t>Partidos aliados respaldan Plan B del gobierno</t>
-  </si>
-  <si>
-    <t>La Sinfónica en la Lotería</t>
-  </si>
-  <si>
-    <t>Billete de lotería</t>
-  </si>
-  <si>
-    <t>Tengo 11 leones sin miedo: Tano</t>
-  </si>
-  <si>
-    <t>AGUIRRE REVELA  CONVOCATORIA</t>
-  </si>
-  <si>
-    <t>Razers tienen un mes para regularizarse</t>
-  </si>
-  <si>
-    <t>Regularización De Vehículos Turísticos</t>
-  </si>
-  <si>
-    <t>AVANZA ADECUACIÓN  DE GLORIETA MIGUEL  HIDALGO, EN PACHUCA</t>
-  </si>
-  <si>
-    <t>Sipdus</t>
-  </si>
-  <si>
-    <t>Glorieta 24 Horas</t>
-  </si>
-  <si>
-    <t>Entre el sudor y devoción: El Lobo prepara el Viacrucis</t>
-  </si>
-  <si>
-    <t>PLANTEAN BORRAR CAPÍTULO SOBRE RECLUTAMIENTO  DE LOS MENORES</t>
-  </si>
-  <si>
-    <t>ANALIZAN DAR APOYOS A LOS  DEUDOS DE TRES ASESINADOS</t>
-  </si>
-  <si>
-    <t>Homicidios</t>
-  </si>
-  <si>
-    <t>Banca ve "blindado" a México; en el Mundial, estancia feliz</t>
-  </si>
-  <si>
-    <t>Mundial De Futbol</t>
-  </si>
-  <si>
-    <t>La migra deja campos sin mano de obra</t>
-  </si>
-  <si>
-    <t>Este año ""hay condiciones"" Altagracia pide que se deje de prestar a los de siempre</t>
-  </si>
-  <si>
-    <t>Textileros: la revisión del T-MEC debe consolidarnos</t>
-  </si>
-  <si>
-    <t>Defensa de soberanías"". China cooperará en AL ""sin importar el bando político""</t>
-  </si>
-  <si>
-    <t>Turismo. Anuncia el estado la muestra gastronómica de Santiago de Anaya</t>
-  </si>
-  <si>
-    <t>Congreso Nacional del Vestido en Pachuca</t>
-  </si>
-  <si>
-    <t>Continúan con la búsqueda de ocho personas, a 5 meses de la vaguada monzónica</t>
-  </si>
-  <si>
-    <t>Huracán Priscilla</t>
-  </si>
-  <si>
-    <t>Encuentran sin vida a tres personas en Tulancingo</t>
-  </si>
-  <si>
-    <t>Alcaldes, a favor de la reducción de regidores como parte del Plan B</t>
-  </si>
-  <si>
-    <t>Emiten billete conmemorativo de la Sinfónica del Estado</t>
-  </si>
-  <si>
-    <t>Plan B recortaría exceso de regidores en seis municipios</t>
-  </si>
-  <si>
-    <t>Detienen a  cinco presuntos  implicados en  triple homicidio</t>
-  </si>
-  <si>
-    <t>Tlaxcala será el estado invitado en Muestra Gastronómica</t>
-  </si>
-  <si>
-    <t>Joven mexicano  muere bajo  custodia de ICE  en Florida</t>
-  </si>
-  <si>
-    <t>En una democracia, la obra pública no lo es todo. Tener un Congreso plural, en el que se escuchen  las distintas fuerzas políticas, también representa un beneficio para la población. Y el mismo  razonamiento aplica para la intención de reducir los espacios en los cabildos”.</t>
-  </si>
-  <si>
-    <t>Menchaca destaca papel de Hidalgo  en encuentro de industria textil nacional</t>
-  </si>
-  <si>
-    <t>Caen cinco tras desaparición y  homicidio de tres personas en  Tulancingo</t>
-  </si>
-  <si>
-    <t>Detención</t>
-  </si>
-  <si>
-    <t>Obtiene Secretaría de Gobierno del  estado certificación ISO 9001:2015</t>
-  </si>
-  <si>
-    <t>Certificación</t>
-  </si>
-  <si>
-    <t>Propone Ricardo Crespo plataforma para aumentar tranasplantes exitosos</t>
-  </si>
-  <si>
-    <t>Delegado de Parque de Poblamiento rechaza acusaciones</t>
-  </si>
-  <si>
-    <t>Inauguran bazar artesanal</t>
-  </si>
-  <si>
-    <t>Julio Menchaca cobija a la cadena Fibra-Textil-Vestido-Calzado</t>
-  </si>
-  <si>
-    <t>En aumento los casos de sarna en callejeros</t>
-  </si>
-  <si>
-    <t>Presidencia y DIF entregan ayudas técnicas y funcionales</t>
-  </si>
-  <si>
-    <t>Ayudas funcionales</t>
-  </si>
-  <si>
-    <t>Detienen a cinco por asesinato de Ángel, Enrique y Miguel</t>
-  </si>
-  <si>
-    <t>Hidalgo, primer lugar en denuncias contra servidores públicos</t>
-  </si>
-  <si>
-    <t>Delitos servidores públicos</t>
-  </si>
-  <si>
-    <t>Víctimas eran familiares de regidora del PT</t>
-  </si>
-  <si>
-    <t>detenci</t>
-  </si>
-  <si>
-    <t>Golpes certeros buscan frenar la impunidad; Olivares""</t>
-  </si>
-  <si>
-    <t>menchaca respalda a la industria textil</t>
-  </si>
-  <si>
-    <t>Ana María Rivera inaugura drenaje en sanitaros en Hutitel</t>
-  </si>
-  <si>
-    <t>Drenaje</t>
-  </si>
-  <si>
-    <t>Menchaca cobija a la cadena Fibra-Textil-Vestido-Calzado</t>
-  </si>
-  <si>
-    <t>Segobh obtiene certicación ISO 9001:2015</t>
-  </si>
-  <si>
-    <t>Claudia Sandoval condintúa con la atención del pueblo, ahora en Tablón</t>
-  </si>
-  <si>
-    <t>Atención a la ciudadanía</t>
-  </si>
-  <si>
-    <t>El Gabienete de Seguridad da seguimiento a 3 personas desapareidas en Tulancingo de Bravo</t>
-  </si>
-  <si>
-    <t>PGJEH y FGJEM investigan desaparición y homicidio de tres personas, ocurridos en Hidalgo y Estado de México, respectivamente</t>
-  </si>
-  <si>
-    <t>Activan Mega Operativo de seguridad para la Feria San José</t>
+    <t>Se restablecerá al 100% la recolección de basura en Tula esta semana: alcalde</t>
+  </si>
+  <si>
+    <t>Recolección De Basura</t>
+  </si>
+  <si>
+    <t>Menchaca detona desarrollo productivo de Hidalgo con economía social y cooperativismo</t>
+  </si>
+  <si>
+    <t>Atotonilco de Tula abre nueva campaña de escrituración a bajo costo</t>
+  </si>
+  <si>
+    <t>Entrega De Escrituras</t>
+  </si>
+  <si>
+    <t>Gabinete de seguridad de Hidalgo desplegará 5 mil 500 elementos en operativo de Semana Santa</t>
+  </si>
+  <si>
+    <t>Hidalgo fortalece la economía social con firma de convenio entre el Gobierno del Estado e Inaes</t>
+  </si>
+  <si>
+    <t>Notariado hidalguense fortalece la certeza jurídica y la modenrización con el curso de actualización anual</t>
+  </si>
+  <si>
+    <t>Concluye feria San José Tula</t>
   </si>
   <si>
     <t>Feria Patronal</t>
   </si>
   <si>
-    <t>Servicios y atención directa en El Depósito, Tlahuelilpan</t>
-  </si>
-  <si>
-    <t>Promete Muestra Gastrnómica cultivar paladares de Santiago de Anaya</t>
-  </si>
-  <si>
-    <t>Segobh obtiene certificación ISO 9001:2015 en procesos de atención ciudadana</t>
-  </si>
-  <si>
-    <t>Cinco detenidos y camionetas recuperadas, en Tulantepec y Tulancingo</t>
-  </si>
-  <si>
-    <t>Julio Menchaca conija a la cadena fibra-textil-vesttido</t>
-  </si>
-  <si>
-    <t>Dejaron volcanes Popo e Izta blanca postal desde Hidalgo</t>
-  </si>
-  <si>
-    <t>Iban a vender autos, los encontraron sin vida</t>
-  </si>
-  <si>
-    <t>Arrestan a la hija del ""Mayo"" Zambada y después la liberan</t>
-  </si>
-  <si>
-    <t>Liberación de detenido</t>
-  </si>
-  <si>
-    <t>Crece el número de delitos en Hidalgo,lo cual no es novedad, porque sucede en todo el país; pero no debemos normalizar esta situación, aún es tiempo de desterrar el flagelo de la violencia con medidas más radicales y profesionales</t>
-  </si>
-  <si>
-    <t>Inseguridad</t>
-  </si>
-  <si>
-    <t>Piden agilizar las investigaciones de abuso sexual</t>
-  </si>
-  <si>
-    <t>Media superior</t>
-  </si>
-  <si>
-    <t>Abuso Sexual</t>
-  </si>
-  <si>
-    <t>Buscan combatir la violencia cometida por choferes</t>
-  </si>
-  <si>
-    <t>Capacitación a transportistas</t>
+    <t>Tania Valdez sufre fractura de fémur tras accidente</t>
+  </si>
+  <si>
+    <t>Proyectan segunda línea de Tuzobús; iría hacia Mineral de la Reforma</t>
+  </si>
+  <si>
+    <t>Obras en valle y ampliación El Palmar atienden una demanda pendiente con familias: Jorge Reyes</t>
+  </si>
+  <si>
+    <t>Localizan a adolescente extraviada en Talxiaca; estaba en Morelos</t>
+  </si>
+  <si>
+    <t>Julio Menchaca detona desarrollo productivo con economía social y cooperativismo</t>
+  </si>
+  <si>
+    <t>Hidalgo ampliará cobertura en media superior con nuevos bachilleratos</t>
+  </si>
+  <si>
+    <t>Bachillerato Nacional</t>
+  </si>
+  <si>
+    <t>Conoce la pirámide de Movilidad</t>
+  </si>
+  <si>
+    <t>publicidad gubernamental</t>
+  </si>
+  <si>
+    <t>Trabaja gobierno estatal en la movilidad: JMS</t>
+  </si>
+  <si>
+    <t>Sheinbaum defiende revocación de mandato</t>
+  </si>
+  <si>
+    <t>Revocación De Mandato</t>
+  </si>
+  <si>
+    <t>Desplegarán 5 mil 500 elementos en operativo de Semana Santa</t>
+  </si>
+  <si>
+    <t>Si el PIMUS se cumple en tiempo y forma, Tello llegará sin problemas a la estación San Lázaro</t>
   </si>
 </sst>
 </file>
@@ -826,8 +850,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J67" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J67" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J65" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J65" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1193,22 +1217,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J67"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J65"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.7265625" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1240,27 +1264,27 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B2" t="s">
         <v>70</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="F2" t="s">
-        <v>25</v>
+        <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
@@ -1271,52 +1295,52 @@
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B3" t="s">
         <v>70</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>69</v>
+        <v>92</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B4" t="s">
         <v>70</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
@@ -1342,43 +1366,43 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B5" t="s">
         <v>70</v>
       </c>
       <c r="C5" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F5" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" t="s">
         <v>95</v>
       </c>
-      <c r="D5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F5" t="s">
-        <v>10</v>
-      </c>
-      <c r="G5" t="s">
-        <v>69</v>
-      </c>
       <c r="H5" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B6" t="s">
         <v>70</v>
@@ -1387,13 +1411,13 @@
         <v>96</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>2</v>
+        <v>44</v>
       </c>
       <c r="G6" t="s">
         <v>97</v>
@@ -1403,16 +1427,16 @@
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B7" t="s">
         <v>70</v>
@@ -1424,10 +1448,10 @@
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F7" t="s">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="G7" t="s">
         <v>99</v>
@@ -1444,9 +1468,9 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B8" t="s">
         <v>71</v>
@@ -1458,10 +1482,10 @@
         <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
         <v>101</v>
@@ -1471,16 +1495,16 @@
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B9" t="s">
         <v>71</v>
@@ -1492,13 +1516,13 @@
         <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>32</v>
+        <v>103</v>
       </c>
       <c r="G9" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
@@ -1512,27 +1536,27 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B10" t="s">
         <v>71</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>85</v>
+        <v>106</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
@@ -1543,64 +1567,64 @@
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B11" t="s">
         <v>71</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B12" t="s">
         <v>71</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F12" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G12" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
@@ -1614,15 +1638,15 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B13" t="s">
         <v>74</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1634,7 +1658,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -1648,15 +1672,15 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B14" t="s">
         <v>74</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -1668,7 +1692,7 @@
         <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
@@ -1682,27 +1706,27 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
         <v>13</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
       <c r="F15" t="s">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="G15" t="s">
-        <v>110</v>
+        <v>99</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
@@ -1716,27 +1740,27 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B16" t="s">
         <v>74</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="F16" t="s">
-        <v>112</v>
+        <v>2</v>
       </c>
       <c r="G16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
@@ -1750,49 +1774,49 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B17" t="s">
         <v>74</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D17" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F17" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G17" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B18" t="s">
         <v>74</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
@@ -1804,10 +1828,10 @@
         <v>37</v>
       </c>
       <c r="G18" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H18" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1818,80 +1842,80 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B19" t="s">
         <v>74</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F19" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H19" t="s">
         <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D20" t="s">
         <v>13</v>
       </c>
       <c r="E20" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="F20" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="G20" t="s">
-        <v>119</v>
+        <v>81</v>
       </c>
       <c r="H20" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B21" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>120</v>
@@ -1900,32 +1924,32 @@
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="F21" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="G21" t="s">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="H21" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B22" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>121</v>
@@ -1934,526 +1958,526 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
+        <v>17</v>
+      </c>
+      <c r="F22" t="s">
+        <v>17</v>
+      </c>
+      <c r="G22" t="s">
+        <v>122</v>
+      </c>
+      <c r="H22" t="s">
+        <v>16</v>
+      </c>
+      <c r="I22" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J22" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B23" t="s">
+        <v>84</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>30</v>
+      </c>
+      <c r="F23" t="s">
+        <v>30</v>
+      </c>
+      <c r="G23" t="s">
+        <v>124</v>
+      </c>
+      <c r="H23" t="s">
+        <v>16</v>
+      </c>
+      <c r="I23" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J23" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B24" t="s">
+        <v>84</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" t="s">
+        <v>18</v>
+      </c>
+      <c r="G24" t="s">
+        <v>126</v>
+      </c>
+      <c r="H24" t="s">
+        <v>11</v>
+      </c>
+      <c r="I24" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J24" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B25" t="s">
+        <v>84</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" t="s">
+        <v>28</v>
+      </c>
+      <c r="G25" t="s">
+        <v>109</v>
+      </c>
+      <c r="H25" t="s">
+        <v>11</v>
+      </c>
+      <c r="I25" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J25" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B26" t="s">
+        <v>84</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
         <v>10</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F26" t="s">
         <v>10</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G26" t="s">
         <v>69</v>
       </c>
-      <c r="H22" t="s">
-        <v>11</v>
-      </c>
-      <c r="I22" t="str">
+      <c r="H26" t="s">
+        <v>11</v>
+      </c>
+      <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J22" t="str">
+      <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A23" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B23" t="s">
-        <v>74</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="D23" t="s">
-        <v>12</v>
-      </c>
-      <c r="E23" t="s">
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B27" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
         <v>10</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F27" t="s">
         <v>10</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G27" t="s">
         <v>69</v>
       </c>
-      <c r="H23" t="s">
-        <v>11</v>
-      </c>
-      <c r="I23" t="str">
+      <c r="H27" t="s">
+        <v>11</v>
+      </c>
+      <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J23" t="str">
+      <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A24" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B24" t="s">
-        <v>74</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="D24" t="s">
-        <v>12</v>
-      </c>
-      <c r="E24" t="s">
-        <v>10</v>
-      </c>
-      <c r="F24" t="s">
-        <v>10</v>
-      </c>
-      <c r="G24" t="s">
-        <v>69</v>
-      </c>
-      <c r="H24" t="s">
-        <v>11</v>
-      </c>
-      <c r="I24" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J24" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A25" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B25" t="s">
-        <v>74</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="D25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" t="s">
-        <v>32</v>
-      </c>
-      <c r="F25" t="s">
-        <v>32</v>
-      </c>
-      <c r="G25" t="s">
-        <v>99</v>
-      </c>
-      <c r="H25" t="s">
-        <v>11</v>
-      </c>
-      <c r="I25" t="str">
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B28" t="s">
+        <v>84</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" t="s">
+        <v>131</v>
+      </c>
+      <c r="G28" t="s">
+        <v>132</v>
+      </c>
+      <c r="H28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J25" t="str">
+      <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B26" t="s">
-        <v>74</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" t="s">
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B29" t="s">
+        <v>72</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D29" t="s">
         <v>9</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29" t="s">
+        <v>2</v>
+      </c>
+      <c r="G29" t="s">
+        <v>134</v>
+      </c>
+      <c r="H29" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J29" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B30" t="s">
+        <v>72</v>
+      </c>
+      <c r="C30" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
         <v>25</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F30" t="s">
         <v>25</v>
       </c>
-      <c r="G26" t="s">
-        <v>92</v>
-      </c>
-      <c r="H26" t="s">
-        <v>26</v>
-      </c>
-      <c r="I26" t="str">
+      <c r="G30" t="s">
+        <v>136</v>
+      </c>
+      <c r="H30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J26" t="str">
+      <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A27" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B27" t="s">
-        <v>74</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" t="s">
-        <v>24</v>
-      </c>
-      <c r="F27" t="s">
-        <v>86</v>
-      </c>
-      <c r="G27" t="s">
-        <v>127</v>
-      </c>
-      <c r="H27" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A28" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B28" t="s">
-        <v>74</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D28" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" t="s">
-        <v>18</v>
-      </c>
-      <c r="F28" t="s">
-        <v>18</v>
-      </c>
-      <c r="G28" t="s">
-        <v>117</v>
-      </c>
-      <c r="H28" t="s">
-        <v>16</v>
-      </c>
-      <c r="I28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A29" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B29" t="s">
-        <v>74</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
-        <v>17</v>
-      </c>
-      <c r="F29" t="s">
-        <v>84</v>
-      </c>
-      <c r="G29" t="s">
-        <v>82</v>
-      </c>
-      <c r="H29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B30" t="s">
-        <v>74</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="D30" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" t="s">
-        <v>31</v>
-      </c>
-      <c r="F30" t="s">
-        <v>31</v>
-      </c>
-      <c r="G30" t="s">
-        <v>106</v>
-      </c>
-      <c r="H30" t="s">
-        <v>11</v>
-      </c>
-      <c r="I30" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J30" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B31" t="s">
         <v>72</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D31" t="s">
         <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="F31" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G31" t="s">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B32" t="s">
         <v>72</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F32" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G32" t="s">
-        <v>117</v>
+        <v>69</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B33" t="s">
         <v>72</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D33" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="F33" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="G33" t="s">
-        <v>99</v>
+        <v>140</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J33" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B34" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" t="s">
+        <v>25</v>
+      </c>
+      <c r="F34" t="s">
+        <v>25</v>
+      </c>
+      <c r="G34" t="s">
+        <v>92</v>
+      </c>
+      <c r="H34" t="s">
+        <v>11</v>
+      </c>
+      <c r="I34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J33" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B34" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="D34" t="s">
-        <v>12</v>
-      </c>
-      <c r="E34" t="s">
-        <v>10</v>
-      </c>
-      <c r="F34" t="s">
-        <v>10</v>
-      </c>
-      <c r="G34" t="s">
-        <v>69</v>
-      </c>
-      <c r="H34" t="s">
-        <v>11</v>
-      </c>
-      <c r="I34" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F35" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G35" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B36" t="s">
         <v>73</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="D36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>25</v>
+        <v>144</v>
       </c>
       <c r="G36" t="s">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B37" t="s">
         <v>73</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="F37" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="G37" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="H37" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2464,117 +2488,117 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B38" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="D38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E38" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F38" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G38" t="s">
-        <v>140</v>
+        <v>69</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="D39" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E39" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F39" t="s">
-        <v>10</v>
+        <v>144</v>
       </c>
       <c r="G39" t="s">
-        <v>89</v>
+        <v>149</v>
       </c>
       <c r="H39" t="s">
         <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B40" t="s">
         <v>75</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="D40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>10</v>
+        <v>151</v>
       </c>
       <c r="G40" t="s">
-        <v>69</v>
+        <v>152</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B41" t="s">
         <v>75</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
@@ -2586,7 +2610,7 @@
         <v>17</v>
       </c>
       <c r="G41" t="s">
-        <v>69</v>
+        <v>154</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
@@ -2600,129 +2624,129 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B42" t="s">
         <v>75</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J42" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A43" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B43" t="s">
+        <v>80</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>17</v>
+      </c>
+      <c r="F43" t="s">
+        <v>157</v>
+      </c>
+      <c r="G43" t="s">
+        <v>158</v>
+      </c>
+      <c r="H43" t="s">
+        <v>11</v>
+      </c>
+      <c r="I43" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J43" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B44" t="s">
+        <v>80</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D44" t="s">
+        <v>9</v>
+      </c>
+      <c r="E44" t="s">
+        <v>24</v>
+      </c>
+      <c r="F44" t="s">
+        <v>2</v>
+      </c>
+      <c r="G44" t="s">
+        <v>160</v>
+      </c>
+      <c r="H44" t="s">
+        <v>11</v>
+      </c>
+      <c r="I44" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J42" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A43" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B43" t="s">
-        <v>75</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="D43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" t="s">
-        <v>10</v>
-      </c>
-      <c r="F43" t="s">
-        <v>10</v>
-      </c>
-      <c r="G43" t="s">
-        <v>69</v>
-      </c>
-      <c r="H43" t="s">
-        <v>11</v>
-      </c>
-      <c r="I43" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J43" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A44" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B44" t="s">
-        <v>75</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="D44" t="s">
-        <v>12</v>
-      </c>
-      <c r="E44" t="s">
-        <v>17</v>
-      </c>
-      <c r="F44" t="s">
-        <v>17</v>
-      </c>
-      <c r="G44" t="s">
-        <v>147</v>
-      </c>
-      <c r="H44" t="s">
-        <v>11</v>
-      </c>
-      <c r="I44" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B45" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>148</v>
+        <v>161</v>
       </c>
       <c r="D45" t="s">
         <v>13</v>
       </c>
       <c r="E45" t="s">
-        <v>23</v>
+        <v>51</v>
       </c>
       <c r="F45" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G45" t="s">
-        <v>138</v>
+        <v>99</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
@@ -2736,120 +2760,120 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B46" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F46" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G46" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="H46" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A47" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B47" t="s">
+        <v>80</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" t="s">
+        <v>88</v>
+      </c>
+      <c r="F47" t="s">
+        <v>88</v>
+      </c>
+      <c r="G47" t="s">
+        <v>160</v>
+      </c>
+      <c r="H47" t="s">
+        <v>11</v>
+      </c>
+      <c r="I47" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J47" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A47" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B47" t="s">
-        <v>83</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="D47" t="s">
-        <v>12</v>
-      </c>
-      <c r="E47" t="s">
-        <v>23</v>
-      </c>
-      <c r="F47" t="s">
-        <v>23</v>
-      </c>
-      <c r="G47" t="s">
-        <v>152</v>
-      </c>
-      <c r="H47" t="s">
-        <v>11</v>
-      </c>
-      <c r="I47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B48" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>2</v>
+        <v>144</v>
       </c>
       <c r="G48" t="s">
-        <v>90</v>
+        <v>166</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B49" t="s">
-        <v>83</v>
+        <v>164</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E49" t="s">
         <v>25</v>
@@ -2861,7 +2885,7 @@
         <v>92</v>
       </c>
       <c r="H49" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2872,15 +2896,15 @@
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>164</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>155</v>
+        <v>168</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -2892,7 +2916,7 @@
         <v>17</v>
       </c>
       <c r="G50" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
@@ -2906,18 +2930,18 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B51" t="s">
-        <v>77</v>
+        <v>164</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="D51" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E51" t="s">
         <v>25</v>
@@ -2926,199 +2950,199 @@
         <v>25</v>
       </c>
       <c r="G51" t="s">
+        <v>106</v>
+      </c>
+      <c r="H51" t="s">
+        <v>11</v>
+      </c>
+      <c r="I51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A52" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B52" t="s">
+        <v>164</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>25</v>
+      </c>
+      <c r="F52" t="s">
+        <v>25</v>
+      </c>
+      <c r="G52" t="s">
         <v>92</v>
       </c>
-      <c r="H51" t="s">
-        <v>11</v>
-      </c>
-      <c r="I51" t="str">
+      <c r="H52" t="s">
+        <v>11</v>
+      </c>
+      <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J51" t="str">
+      <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A52" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B52" t="s">
-        <v>77</v>
-      </c>
-      <c r="C52" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="D52" t="s">
-        <v>12</v>
-      </c>
-      <c r="E52" t="s">
-        <v>24</v>
-      </c>
-      <c r="F52" t="s">
+    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A53" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B53" t="s">
+        <v>164</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53" t="s">
+        <v>69</v>
+      </c>
+      <c r="H53" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B54" t="s">
+        <v>164</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>17</v>
+      </c>
+      <c r="F54" t="s">
+        <v>17</v>
+      </c>
+      <c r="G54" t="s">
+        <v>174</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+      <c r="I54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B55" t="s">
+        <v>164</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>10</v>
+      </c>
+      <c r="F55" t="s">
+        <v>10</v>
+      </c>
+      <c r="G55" t="s">
+        <v>69</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A56" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B56" t="s">
+        <v>29</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="D56" t="s">
+        <v>13</v>
+      </c>
+      <c r="E56" t="s">
+        <v>51</v>
+      </c>
+      <c r="F56" t="s">
         <v>2</v>
       </c>
-      <c r="G52" t="s">
-        <v>140</v>
-      </c>
-      <c r="H52" t="s">
-        <v>11</v>
-      </c>
-      <c r="I52" t="str">
+      <c r="G56" t="s">
+        <v>99</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J52" t="str">
+      <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A53" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B53" t="s">
-        <v>77</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="D53" t="s">
-        <v>12</v>
-      </c>
-      <c r="E53" t="s">
-        <v>17</v>
-      </c>
-      <c r="F53" t="s">
-        <v>84</v>
-      </c>
-      <c r="G53" t="s">
-        <v>160</v>
-      </c>
-      <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A54" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B54" t="s">
-        <v>77</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D54" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" t="s">
-        <v>41</v>
-      </c>
-      <c r="F54" t="s">
-        <v>41</v>
-      </c>
-      <c r="G54" t="s">
-        <v>87</v>
-      </c>
-      <c r="H54" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A55" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B55" t="s">
-        <v>77</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>18</v>
-      </c>
-      <c r="F55" t="s">
-        <v>18</v>
-      </c>
-      <c r="G55" t="s">
-        <v>117</v>
-      </c>
-      <c r="H55" t="s">
-        <v>11</v>
-      </c>
-      <c r="I55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A56" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B56" t="s">
-        <v>77</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D56" t="s">
-        <v>12</v>
-      </c>
-      <c r="E56" t="s">
-        <v>17</v>
-      </c>
-      <c r="F56" t="s">
-        <v>81</v>
-      </c>
-      <c r="G56" t="s">
-        <v>164</v>
-      </c>
-      <c r="H56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B57" t="s">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
@@ -3127,10 +3151,10 @@
         <v>17</v>
       </c>
       <c r="F57" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="G57" t="s">
-        <v>69</v>
+        <v>158</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
@@ -3144,30 +3168,30 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B58" t="s">
         <v>29</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="D58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="F58" t="s">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="G58" t="s">
-        <v>99</v>
+        <v>146</v>
       </c>
       <c r="H58" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3178,27 +3202,27 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B59" t="s">
         <v>29</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="D59" t="s">
         <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F59" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G59" t="s">
-        <v>140</v>
+        <v>92</v>
       </c>
       <c r="H59" t="s">
         <v>11</v>
@@ -3209,30 +3233,30 @@
       </c>
       <c r="J59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B60" t="s">
         <v>29</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="D60" t="s">
         <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="F60" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G60" t="s">
-        <v>138</v>
+        <v>181</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
@@ -3246,242 +3270,174 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B61" t="s">
         <v>29</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D61" t="s">
-        <v>12</v>
+        <v>86</v>
       </c>
       <c r="E61" t="s">
+        <v>17</v>
+      </c>
+      <c r="F61" t="s">
+        <v>17</v>
+      </c>
+      <c r="G61" t="s">
+        <v>183</v>
+      </c>
+      <c r="H61" t="s">
+        <v>11</v>
+      </c>
+      <c r="I61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B62" t="s">
+        <v>78</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D62" t="s">
+        <v>13</v>
+      </c>
+      <c r="E62" t="s">
         <v>25</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F62" t="s">
         <v>25</v>
       </c>
-      <c r="G61" t="s">
-        <v>92</v>
-      </c>
-      <c r="H61" t="s">
-        <v>11</v>
-      </c>
-      <c r="I61" t="str">
+      <c r="G62" t="s">
+        <v>124</v>
+      </c>
+      <c r="H62" t="s">
+        <v>26</v>
+      </c>
+      <c r="I62" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J61" t="str">
+      <c r="J62" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A62" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B62" t="s">
-        <v>29</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="D62" t="s">
-        <v>12</v>
-      </c>
-      <c r="E62" t="s">
-        <v>10</v>
-      </c>
-      <c r="F62" t="s">
-        <v>10</v>
-      </c>
-      <c r="G62" t="s">
-        <v>69</v>
-      </c>
-      <c r="H62" t="s">
-        <v>11</v>
-      </c>
-      <c r="I62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J62" t="str">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B63" t="s">
+        <v>78</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>14</v>
+      </c>
+      <c r="F63" t="s">
+        <v>14</v>
+      </c>
+      <c r="G63" t="s">
+        <v>186</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+      <c r="I63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A63" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B63" t="s">
-        <v>79</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="D63" t="s">
-        <v>13</v>
-      </c>
-      <c r="E63" t="s">
-        <v>18</v>
-      </c>
-      <c r="F63" t="s">
-        <v>18</v>
-      </c>
-      <c r="G63" t="s">
-        <v>117</v>
-      </c>
-      <c r="H63" t="s">
-        <v>16</v>
-      </c>
-      <c r="I63" t="str">
+    <row r="64" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A64" s="5">
+        <v>46105</v>
+      </c>
+      <c r="B64" t="s">
+        <v>78</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D64" t="s">
+        <v>9</v>
+      </c>
+      <c r="E64" t="s">
+        <v>41</v>
+      </c>
+      <c r="F64" t="s">
+        <v>41</v>
+      </c>
+      <c r="G64" t="s">
+        <v>82</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J63" t="str">
+      <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B64" t="s">
-        <v>79</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D64" t="s">
-        <v>12</v>
-      </c>
-      <c r="E64" t="s">
-        <v>14</v>
-      </c>
-      <c r="F64" t="s">
-        <v>14</v>
-      </c>
-      <c r="G64" t="s">
-        <v>173</v>
-      </c>
-      <c r="H64" t="s">
-        <v>11</v>
-      </c>
-      <c r="I64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
-        <v>46101</v>
+        <v>46105</v>
       </c>
       <c r="B65" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>174</v>
+        <v>188</v>
       </c>
       <c r="D65" t="s">
-        <v>12</v>
+        <v>87</v>
       </c>
       <c r="E65" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="F65" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G65" t="s">
-        <v>175</v>
+        <v>124</v>
       </c>
       <c r="H65" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A66" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B66" t="s">
-        <v>79</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D66" t="s">
-        <v>12</v>
-      </c>
-      <c r="E66" t="s">
-        <v>28</v>
-      </c>
-      <c r="F66" t="s">
-        <v>177</v>
-      </c>
-      <c r="G66" t="s">
-        <v>178</v>
-      </c>
-      <c r="H66" t="s">
-        <v>16</v>
-      </c>
-      <c r="I66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67" s="5">
-        <v>46101</v>
-      </c>
-      <c r="B67" t="s">
-        <v>79</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D67" t="s">
-        <v>12</v>
-      </c>
-      <c r="E67" t="s">
-        <v>37</v>
-      </c>
-      <c r="F67" t="s">
-        <v>37</v>
-      </c>
-      <c r="G67" t="s">
-        <v>180</v>
-      </c>
-      <c r="H67" t="s">
-        <v>11</v>
-      </c>
-      <c r="I67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
   </sheetData>
@@ -3496,14 +3452,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8151DEFD-FF29-4969-B1FC-DF47C7CD743C}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -3517,7 +3473,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -3528,10 +3484,10 @@
         <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -3542,10 +3498,10 @@
         <v>36</v>
       </c>
       <c r="E3" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -3556,10 +3512,10 @@
         <v>38</v>
       </c>
       <c r="E4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>64</v>
       </c>
@@ -3570,10 +3526,10 @@
         <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>36</v>
       </c>
@@ -3584,10 +3540,10 @@
         <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -3598,10 +3554,10 @@
         <v>40</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>38</v>
       </c>
@@ -3612,10 +3568,10 @@
         <v>40</v>
       </c>
       <c r="E8" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -3626,10 +3582,10 @@
         <v>41</v>
       </c>
       <c r="E9" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -3643,7 +3599,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -3654,10 +3610,10 @@
         <v>42</v>
       </c>
       <c r="E11" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>40</v>
       </c>
@@ -3668,10 +3624,10 @@
         <v>43</v>
       </c>
       <c r="E12" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>40</v>
       </c>
@@ -3682,10 +3638,10 @@
         <v>43</v>
       </c>
       <c r="E13" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>67</v>
       </c>
@@ -3696,10 +3652,10 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>41</v>
       </c>
@@ -3710,10 +3666,10 @@
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -3724,10 +3680,10 @@
         <v>51</v>
       </c>
       <c r="E16" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>42</v>
       </c>
@@ -3738,10 +3694,10 @@
         <v>57</v>
       </c>
       <c r="E17" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>43</v>
       </c>
@@ -3752,10 +3708,10 @@
         <v>58</v>
       </c>
       <c r="E18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>44</v>
       </c>
@@ -3766,10 +3722,10 @@
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -3780,10 +3736,10 @@
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -3794,10 +3750,10 @@
         <v>30</v>
       </c>
       <c r="E21" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -3808,10 +3764,10 @@
         <v>28</v>
       </c>
       <c r="E22" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -3822,10 +3778,10 @@
         <v>59</v>
       </c>
       <c r="E23" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -3836,10 +3792,10 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>49</v>
       </c>
@@ -3850,10 +3806,10 @@
         <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>50</v>
       </c>
@@ -3864,10 +3820,10 @@
         <v>60</v>
       </c>
       <c r="E26" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -3878,10 +3834,10 @@
         <v>32</v>
       </c>
       <c r="E27" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -3889,7 +3845,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>51</v>
       </c>
@@ -3897,7 +3853,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>52</v>
       </c>
@@ -3905,7 +3861,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
@@ -3913,7 +3869,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>54</v>
       </c>
@@ -3921,7 +3877,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>55</v>
       </c>
@@ -3929,7 +3885,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>56</v>
       </c>
@@ -3937,7 +3893,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>57</v>
       </c>
@@ -3945,7 +3901,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>58</v>
       </c>
@@ -3953,7 +3909,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>24</v>
       </c>
@@ -3961,7 +3917,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>21</v>
       </c>
@@ -3969,7 +3925,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>30</v>
       </c>
@@ -3977,7 +3933,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -3985,7 +3941,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>59</v>
       </c>
@@ -3993,7 +3949,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -4001,7 +3957,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>23</v>
       </c>
@@ -4009,7 +3965,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>60</v>
       </c>
@@ -4017,7 +3973,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>61</v>
       </c>
@@ -4025,7 +3981,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>62</v>
       </c>
@@ -4033,7 +3989,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>32</v>
       </c>
@@ -4041,7 +3997,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>63</v>
       </c>

</xml_diff>

<commit_message>
Reporte 26 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D875261-7437-4C95-994C-1B6481790ADD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD2B5C94-5934-4702-BA6C-9E9E42C270CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="196">
   <si>
     <t>Fecha</t>
   </si>
@@ -294,274 +294,337 @@
     <t>Alcalde</t>
   </si>
   <si>
-    <t>Reunión con actores políticos</t>
-  </si>
-  <si>
-    <t>Logran mejora salarial de 7%</t>
-  </si>
-  <si>
-    <t>Aumento salarial</t>
-  </si>
-  <si>
-    <t>Jorge Reyes entrega 5 nuevas patrullas</t>
-  </si>
-  <si>
-    <t>alc</t>
-  </si>
-  <si>
-    <t>Entrega de patrullas</t>
-  </si>
-  <si>
-    <t>Personas buscadoras, defensoras de los DH</t>
-  </si>
-  <si>
     <t>Reforma De Ley</t>
   </si>
   <si>
-    <t>Luego de días santos dirán si suben precios</t>
-  </si>
-  <si>
-    <t>Viviendas sin agua por falla eléctrica</t>
-  </si>
-  <si>
-    <t>Agua</t>
-  </si>
-  <si>
-    <t>Fallas CFE</t>
-  </si>
-  <si>
-    <t>Impulsan desarrollo en la región de Zapotlán</t>
-  </si>
-  <si>
-    <t>Ruta de la Transformación</t>
-  </si>
-  <si>
-    <t>Estiman aumento en población adulta mayor</t>
-  </si>
-  <si>
-    <t>Coespo</t>
-  </si>
-  <si>
-    <t>Aumento poblacional</t>
-  </si>
-  <si>
-    <t>Alistan Zapotlán para la llegada de un Polo del Bienestar</t>
-  </si>
-  <si>
-    <t>Polos del Bienestar</t>
-  </si>
-  <si>
-    <t>Fiebre futbolera</t>
-  </si>
-  <si>
     <t>Mundial De Futbol</t>
   </si>
   <si>
-    <t>Entregan patrullas en Pachuca</t>
-  </si>
-  <si>
-    <t>Aprueban cobrar multa a partidos</t>
-  </si>
-  <si>
-    <t>Multas IEEH</t>
-  </si>
-  <si>
-    <t>Iniciativa contra el feminicidio</t>
-  </si>
-  <si>
     <t>Iniciativa</t>
   </si>
   <si>
-    <t>Baños cumplió con reparación del daño""</t>
-  </si>
-  <si>
-    <t>Discriminación</t>
-  </si>
-  <si>
-    <t>Suman cinco patrullas a la flotilla de SSP de Pachuca</t>
-  </si>
-  <si>
-    <t>Aprueban dictamen de personas buscadoras</t>
-  </si>
-  <si>
-    <t>MONUMENTO  ECUMÉNICO, CON SIGNOS   DE DETERIORO</t>
-  </si>
-  <si>
     <t>Sipdus</t>
   </si>
   <si>
-    <t>Abandono de obra</t>
-  </si>
-  <si>
-    <t>Dos Tuzos, en la fecha FIFA</t>
-  </si>
-  <si>
-    <t>ARRANCA EL  REPECHAJE  A LA COPA  DEL MUNDO</t>
-  </si>
-  <si>
-    <t>TUZOBÚS: PIDEN PLANEAR  BIEN LA NUEVA TRONCAL</t>
-  </si>
-  <si>
     <t>Sitmah</t>
   </si>
   <si>
     <t>Ampliación Tuzobús</t>
   </si>
   <si>
-    <t>La reconstrucción en zonas afectadas avanza pese a retos: Menchaca</t>
-  </si>
-  <si>
-    <t>Habitantes de Tlaolula manifiestan desconfianza</t>
-  </si>
-  <si>
     <t>Reubicación de viviendas</t>
   </si>
   <si>
-    <t>Descubren altar tolteca en Tula</t>
-  </si>
-  <si>
-    <t>INAH</t>
-  </si>
-  <si>
-    <t>Vestigios Arqueológicos</t>
-  </si>
-  <si>
-    <t>Reciben nuevas unidades para reforzar la vigilancia</t>
-  </si>
-  <si>
-    <t>Coordinación contra el delito</t>
-  </si>
-  <si>
-    <t>Coordinación interestatal</t>
-  </si>
-  <si>
-    <t>Se rebela el PT contra el plan de Claudia Sheinbaum que avanza en comisiones</t>
-  </si>
-  <si>
-    <t>Multas que deben cubrir ascienden a 56 millones</t>
-  </si>
-  <si>
-    <t>Sabines, el poeta universal: en camino, versos inéditos en un libro</t>
-  </si>
-  <si>
-    <t>Van 313 mdp para activación de polo económico en zona de Zapotlán</t>
-  </si>
-  <si>
-    <t>Apuntalan polo en Zapotlán con 313 mdp</t>
-  </si>
-  <si>
-    <t>Estalla inconformidad en la UAEH luego de revisión contractual</t>
-  </si>
-  <si>
-    <t>Paro laboral</t>
-  </si>
-  <si>
-    <t>CSP impulsa ley para sancionar el feminicidio</t>
-  </si>
-  <si>
-    <t>Alumno mata a dos maestras en Michoacán</t>
-  </si>
-  <si>
-    <t>Ataque Armado</t>
-  </si>
-  <si>
-    <t>Pachuca consolida estrategia de seguridad con nuevas patrullas</t>
-  </si>
-  <si>
-    <t>El bastión y estructura que presumían tener en la Universidad  Autónoma del estado (UAEH), la que han controlado desde hace cuatro  décadas, comienza a desgastarse y mostrar signos de rebeldía, por las  decisiones equivocadas de Agustín Sosa”.</t>
-  </si>
-  <si>
     <t>Grupo Universidad</t>
   </si>
   <si>
-    <t>Incrementa Pachuca seguridad con 5 patrullas nuevas</t>
-  </si>
-  <si>
-    <t>Prepara gobierno estatal a Zapotlán para la llegada del Polo del Bienestar</t>
-  </si>
-  <si>
-    <t>Hay bastantes indicios"" contra 5 detenidos por desaparecidos en Tulancingo: PGJEH</t>
-  </si>
-  <si>
-    <t>Vinculación A Proceso</t>
-  </si>
-  <si>
-    <t>Respaldan labor de Julio Menchaca al frente del Poder Ejecutivo estatal</t>
-  </si>
-  <si>
-    <t>Labor destacada</t>
-  </si>
-  <si>
-    <t>IEEH cobrará más de 56 millones en multas a partidos de Hidalgo</t>
-  </si>
-  <si>
-    <t>Jorge Reyes refuerza seguridad con nuevas patrullas</t>
-  </si>
-  <si>
-    <t>Menchaca respalda actuación de la policía durante bloqueo</t>
-  </si>
-  <si>
-    <t>Exigen localización de persona</t>
-  </si>
-  <si>
-    <t>Luego de confrontación, Congreso alcanza acuerdo</t>
-  </si>
-  <si>
-    <t>TEEH reparte más de 2.5 millones en aguinaldos</t>
-  </si>
-  <si>
-    <t>Aguinaldos</t>
-  </si>
-  <si>
-    <t>Hidalgo inyecta 130 millones a caminos rurales</t>
-  </si>
-  <si>
-    <t>Carretera artesanal</t>
-  </si>
-  <si>
-    <t>Entrega Jorge Reyes nuevas patrullas y consolida estrategia integral de seguridad en Pachuca</t>
-  </si>
-  <si>
-    <t>Abren venta de boletos para finales de Concacaf W en el Hidalgo</t>
-  </si>
-  <si>
-    <t>Gobierno de Julio Menchaca prepara a Zapotlán para la llegada del Polo del Bienestar</t>
-  </si>
-  <si>
-    <t>Participa en la semana nacional de vacunación antirrábica</t>
-  </si>
-  <si>
-    <t>Vacunación Antirrábica</t>
-  </si>
-  <si>
-    <t>Hidalgo refuerza la coordinación interestatal en la mesa de paz</t>
-  </si>
-  <si>
     <t>Conoce la pirámide de MOVILIDAD</t>
   </si>
   <si>
     <t>Publicidad gubernamental</t>
   </si>
   <si>
-    <t>Protesta el PRI por una presunta venganza de Morena</t>
-  </si>
-  <si>
-    <t>GLMorena</t>
-  </si>
-  <si>
-    <t>Entregan nuevas patrullas en Pachuca</t>
-  </si>
-  <si>
-    <t>Luego entonces, en la ya famosa foto: ¿ni son todas las que están, ni están todas las que son?</t>
-  </si>
-  <si>
-    <t>Presentan iniciativa para elevar sanciones contra el feminicidio</t>
-  </si>
-  <si>
-    <t>Luego de persecución, detienen a una pareja con huachicol</t>
-  </si>
-  <si>
-    <t>Combate Al Huachicol</t>
+    <t>El nuevo estadio Banorte está listo para el Mundial 2026</t>
+  </si>
+  <si>
+    <t>Arranca Operativo Semana Santa 2026</t>
+  </si>
+  <si>
+    <t>Semana Santa</t>
+  </si>
+  <si>
+    <t>Semáforos mejoran tránsito en Madero</t>
+  </si>
+  <si>
+    <t>Mantenimiento de semáforos</t>
+  </si>
+  <si>
+    <t>Vecinos se pronuncian ante proyecto Tuzobús</t>
+  </si>
+  <si>
+    <t>Esperan alta demanda de turistas en Tula</t>
+  </si>
+  <si>
+    <t>Analizan revocación a concesionaria de basurero</t>
+  </si>
+  <si>
+    <t>Relleno Sanitario</t>
+  </si>
+  <si>
+    <t>Vacaciones seguras</t>
+  </si>
+  <si>
+    <t>Más vigilancia en balnearios</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>MC votaría en contra del Plan B de reforma</t>
+  </si>
+  <si>
+    <t>Diálogo en Palacio Nacional</t>
+  </si>
+  <si>
+    <t>Reunión con funcionario federal</t>
+  </si>
+  <si>
+    <t>Habrá padrón digital para migrantes</t>
+  </si>
+  <si>
+    <t>“El objetivo es erradicar el feminicidio en México: que ninguna mujer muera en manos de alguien por el solo hecho de ser mujer y que nunca... |</t>
+  </si>
+  <si>
+    <t>Feminicidio</t>
+  </si>
+  <si>
+    <t>RECONSTRUYEN LOS TUZOS SU CANTERA</t>
+  </si>
+  <si>
+    <t>ITALIA SE JUEGA  TODO  POR EL  MUNDIAL 2026</t>
+  </si>
+  <si>
+    <t>VIVEN EN SITUACIÓN DE CALLE 1,800 PERSONAS</t>
+  </si>
+  <si>
+    <t>Personas en situación de calle</t>
+  </si>
+  <si>
+    <t>LA BARBACOA  QUE CONQUISTÓ  AL PONTÍFICE  JUAN PABLO II</t>
+  </si>
+  <si>
+    <t>COLABORADORA DE  CRITERIO, VÍCTIMA DE HOSTIGAMIENTO  SEXUAL EN PACHUCA</t>
+  </si>
+  <si>
+    <t>Acoso Sexual</t>
+  </si>
+  <si>
+    <t>Plantean crear padrón de agresores digitales</t>
+  </si>
+  <si>
+    <t>Proyecto de la economía circular sería retomado: JMS</t>
+  </si>
+  <si>
+    <t>Economía Circular</t>
+  </si>
+  <si>
+    <t>Damnificados: ""Ni con la Guardia nos van a sacar""</t>
+  </si>
+  <si>
+    <t>Prevén que el padrón de inmuebles puede amumentar</t>
+  </si>
+  <si>
+    <t>CEVI</t>
+  </si>
+  <si>
+    <t>Organizan corrida de toros para apoyar a afectados</t>
+  </si>
+  <si>
+    <t>Junta de Gobierno</t>
+  </si>
+  <si>
+    <t>Se triplican los incendios, entres meses se registran 260</t>
+  </si>
+  <si>
+    <t>Incendios forestales</t>
+  </si>
+  <si>
+    <t>Invitan a visitar el estado, despliegan a 5 mil 700 elementos</t>
+  </si>
+  <si>
+    <t>Alcalde de San Salvador acusa laudos por 13 mdp</t>
+  </si>
+  <si>
+    <t>Laudos Municipios</t>
+  </si>
+  <si>
+    <t>Notificarán a alcalde fallo de Derechos Humanos</t>
+  </si>
+  <si>
+    <t>Recomendaciones CDHEH</t>
+  </si>
+  <si>
+    <t>Fallan cntra Meta y Google por adicciones</t>
+  </si>
+  <si>
+    <t>Se sale con la suya el PT y queda fuera del Plan B la revocación de mandato</t>
+  </si>
+  <si>
+    <t>Próxima década, clave</t>
+  </si>
+  <si>
+    <t>Gobernador advierte sanciones tras fallas en basurero de Tula</t>
+  </si>
+  <si>
+    <t>Congreso aprueba crear el padrón de migrantes</t>
+  </si>
+  <si>
+    <t>Claudia Sheinbaum  destaca respaldo  de 70% a su gestión</t>
+  </si>
+  <si>
+    <t>Aprobación Sheinbaum</t>
+  </si>
+  <si>
+    <t>Cautivos del ICE ,  más de 13 mil  mexicanos</t>
+  </si>
+  <si>
+    <t>Inicia operativo para reforzar seguridad en Semana Santa</t>
+  </si>
+  <si>
+    <t>La afectación a derechos y logros laborales, desde que los sindicatos  universitarios se crearon en 1979, es la gota que derramó el vaso,  porque Agustín Sosa mantiene una actitud despótica, ‘se sigue  sintiendo presidente de la FEUH’, acusan”.</t>
+  </si>
+  <si>
+    <t>Activa Hidalgo Operativo Semana Santa con 5 mil 700 elementos</t>
+  </si>
+  <si>
+    <t>Alistan rehabilitación de fachada del  panteón municipal de Pachuca</t>
+  </si>
+  <si>
+    <t>Panteón Municipal</t>
+  </si>
+  <si>
+    <t>No descarta Menchaca retomar  parque de economía circular por  saturación del relleno en Tula</t>
+  </si>
+  <si>
+    <t>Entra en operación pozo  10 Laguna en Pachuca</t>
+  </si>
+  <si>
+    <t>Caasim</t>
+  </si>
+  <si>
+    <t>Rehabilitación de pozo</t>
+  </si>
+  <si>
+    <t>Gasolina se dispara en Pachuca: precios rozan los 29 pesos por litro</t>
+  </si>
+  <si>
+    <t>Sancionan a 36 por invadir carril del Tuzobús</t>
+  </si>
+  <si>
+    <t>Carril confinado</t>
+  </si>
+  <si>
+    <t>Cazan desde el aire</t>
+  </si>
+  <si>
+    <t>Policía municipal</t>
+  </si>
+  <si>
+    <t>Videovigilancia</t>
+  </si>
+  <si>
+    <t>Crisis de basura en Tula: gobierno evalúa dos proyectos</t>
+  </si>
+  <si>
+    <t>Congreso batea pagos del IEEH a representantes partidistas</t>
+  </si>
+  <si>
+    <t>Presupuesto IEEH</t>
+  </si>
+  <si>
+    <t>7 millones por transimisión ponenn en duda Fan Fest en Pachuca</t>
+  </si>
+  <si>
+    <t>OEEH</t>
+  </si>
+  <si>
+    <t>Municipios sin licitaciones. ¿La nueva práctica?</t>
+  </si>
+  <si>
+    <t>Licitaciones</t>
+  </si>
+  <si>
+    <t>Marfeca</t>
+  </si>
+  <si>
+    <t>Analizan dos opciones ante colapso del basurero de Tula</t>
+  </si>
+  <si>
+    <t>Cintillo</t>
+  </si>
+  <si>
+    <t>Inicia construcción de cancha de futbol 5 en Doxey de cara al mundial</t>
+  </si>
+  <si>
+    <t>Hidalgo enfrenta una crisis en la disposición de residuos: urge replantear el modelo</t>
+  </si>
+  <si>
+    <t>Disposición de basura</t>
+  </si>
+  <si>
+    <t>Menchaca da inicio al Operativo Semana Santa 2026 en Hidalgo</t>
+  </si>
+  <si>
+    <t>Arranca operativo ""Semana Santa Segura"" en Tezontepec</t>
+  </si>
+  <si>
+    <t>Refuerzan seguridad en Tlahuelilpan con operativo ""Semana Santa""</t>
+  </si>
+  <si>
+    <t>Ajacuba recibe distintivo sanitario</t>
+  </si>
+  <si>
+    <t>titular</t>
+  </si>
+  <si>
+    <t>Certificación sanitaria</t>
+  </si>
+  <si>
+    <t>Hombre de la tercera edad cae de un peñasco de 6 metros en Tula</t>
+  </si>
+  <si>
+    <t>Localizan en Pachuca a menor con reporte de desaparición</t>
+  </si>
+  <si>
+    <t>CBPEH</t>
+  </si>
+  <si>
+    <t>Localización de persona</t>
+  </si>
+  <si>
+    <t>En efectivo operativo, policías de Pachuca detienen a 3 en intento de robo</t>
+  </si>
+  <si>
+    <t>Detención</t>
+  </si>
+  <si>
+    <t>Julio Menchaca da inicio a Operativo Semana Santa 2026</t>
+  </si>
+  <si>
+    <t>¡Llegamos a 300 mil seguidores en Facebook!</t>
+  </si>
+  <si>
+    <t>SSPH asegura en El Arenal a presunto implicado en robo de patrulla</t>
+  </si>
+  <si>
+    <t>Robo de patrulla</t>
+  </si>
+  <si>
+    <t>Entra en operación pozo 10 Laguna:. beneficiará a oriente de Pachuca</t>
+  </si>
+  <si>
+    <t>Anuncian corrida de toros a beneficio de afectados por vaguada monzónica</t>
+  </si>
+  <si>
+    <t>Plaza Juárez</t>
+  </si>
+  <si>
+    <t>Respaldan corrida de toros en apoyo a damnificados</t>
+  </si>
+  <si>
+    <t>Entablan mesa de diálogo con habitantes de Villas de Sahagún</t>
+  </si>
+  <si>
+    <t>Atención a la ciudadanía</t>
+  </si>
+  <si>
+    <t>13 mexicanos fallecieron bajo custodia del ICE el año pasado</t>
+  </si>
+  <si>
+    <t>Inicia operativo Semana Santa 2026</t>
+  </si>
+  <si>
+    <t>Colapsa el servicio de recolección de basura en Tula</t>
   </si>
 </sst>
 </file>
@@ -715,43 +778,6 @@
   </cellStyles>
   <dxfs count="6">
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="d/m/yy;@"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="1"/>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -794,6 +820,43 @@
         </left>
       </border>
     </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="d/m/yy;@"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="1"/>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -808,12 +871,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J56" totalsRowShown="0" headerRowDxfId="3" headerRowBorderDxfId="2">
-  <autoFilter ref="A1:J56" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J69" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
-    <tableColumn id="3" xr3:uid="{4CA37DD5-010E-43EE-907D-87C1845DB2AB}" name="Titular" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{4CA37DD5-010E-43EE-907D-87C1845DB2AB}" name="Titular" dataDxfId="2"/>
     <tableColumn id="4" xr3:uid="{1E763E28-25D7-4FE7-AD1A-91C7A0FE0E7A}" name="Recurso editorial"/>
     <tableColumn id="5" xr3:uid="{F8C19AF2-6D19-449B-9F8B-6424964B1BCF}" name="Dependencia"/>
     <tableColumn id="6" xr3:uid="{46DF0510-7A9A-4625-979E-4EBC30CC7AA3}" name="Organismo"/>
@@ -845,13 +908,13 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{80AFAA35-C663-4971-9820-992B55167F9C}" name="Tabla3" displayName="Tabla3" ref="D1:E27" totalsRowShown="0" tableBorderDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{80AFAA35-C663-4971-9820-992B55167F9C}" name="Tabla3" displayName="Tabla3" ref="D1:E27" totalsRowShown="0" tableBorderDxfId="1">
   <autoFilter ref="D1:E27" xr:uid="{80AFAA35-C663-4971-9820-992B55167F9C}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D2:E27">
     <sortCondition ref="D1:D27"/>
   </sortState>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{A040A308-8C62-4D4B-B3BE-EC124A9B961C}" name="Dependencia" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{A040A308-8C62-4D4B-B3BE-EC124A9B961C}" name="Dependencia" dataDxfId="0"/>
     <tableColumn id="2" xr3:uid="{2B2FFCF1-496A-4D37-8C8B-790A66FD9968}" name="Nivel"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1175,7 +1238,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1224,25 +1287,25 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B2" t="s">
         <v>70</v>
       </c>
       <c r="C2" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
         <v>86</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>63</v>
-      </c>
-      <c r="F2" t="s">
-        <v>63</v>
-      </c>
-      <c r="G2" t="s">
-        <v>87</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
@@ -1258,66 +1321,66 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B3" t="s">
         <v>70</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F3" t="s">
-        <v>89</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B4" t="s">
         <v>70</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="H4" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1326,32 +1389,32 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B5" t="s">
         <v>70</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="H5" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1360,93 +1423,93 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B6" t="s">
         <v>70</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="F6" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G6" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B7" t="s">
         <v>70</v>
       </c>
       <c r="C7" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" t="s">
         <v>97</v>
       </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" t="s">
-        <v>25</v>
-      </c>
-      <c r="G7" t="s">
-        <v>98</v>
-      </c>
       <c r="H7" t="s">
         <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
@@ -1457,33 +1520,33 @@
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B9" t="s">
         <v>71</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G9" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="H9" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1491,71 +1554,71 @@
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B10" t="s">
         <v>71</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>106</v>
       </c>
       <c r="G10" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B11" t="s">
         <v>71</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="F11" t="s">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Partidos</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1564,25 +1627,25 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B12" t="s">
         <v>71</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
@@ -1598,44 +1661,44 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B13" t="s">
         <v>71</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="F13" t="s">
-        <v>14</v>
+        <v>37</v>
       </c>
       <c r="G13" t="s">
-        <v>110</v>
+        <v>85</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>111</v>
@@ -1644,10 +1707,10 @@
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F14" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G14" t="s">
         <v>112</v>
@@ -1657,7 +1720,7 @@
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1666,7 +1729,7 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
@@ -1678,20 +1741,20 @@
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1700,7 +1763,7 @@
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B16" t="s">
         <v>74</v>
@@ -1712,13 +1775,13 @@
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="F16" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="G16" t="s">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
@@ -1732,9 +1795,9 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B17" t="s">
         <v>74</v>
@@ -1743,19 +1806,19 @@
         <v>115</v>
       </c>
       <c r="D17" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E17" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" t="s">
+        <v>42</v>
+      </c>
+      <c r="G17" t="s">
         <v>116</v>
       </c>
-      <c r="F17" t="s">
-        <v>116</v>
-      </c>
-      <c r="G17" t="s">
-        <v>117</v>
-      </c>
       <c r="H17" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1766,18 +1829,18 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B18" t="s">
         <v>74</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D18" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E18" t="s">
         <v>10</v>
@@ -1786,7 +1849,7 @@
         <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
@@ -1800,15 +1863,15 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B19" t="s">
         <v>74</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
@@ -1820,7 +1883,7 @@
         <v>10</v>
       </c>
       <c r="G19" t="s">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="H19" t="s">
         <v>11</v>
@@ -1836,7 +1899,7 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B20" t="s">
         <v>74</v>
@@ -1848,38 +1911,38 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="F20" t="s">
+        <v>37</v>
+      </c>
+      <c r="G20" t="s">
+        <v>87</v>
+      </c>
+      <c r="H20" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J20" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A21" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B21" t="s">
+        <v>74</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G20" t="s">
-        <v>122</v>
-      </c>
-      <c r="H20" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J20" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="5">
-        <v>46106</v>
-      </c>
-      <c r="B21" t="s">
-        <v>80</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>123</v>
-      </c>
       <c r="D21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E21" t="s">
         <v>25</v>
@@ -1888,7 +1951,7 @@
         <v>25</v>
       </c>
       <c r="G21" t="s">
-        <v>79</v>
+        <v>122</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
@@ -1904,16 +1967,16 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B22" t="s">
         <v>80</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D22" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E22" t="s">
         <v>42</v>
@@ -1922,7 +1985,7 @@
         <v>42</v>
       </c>
       <c r="G22" t="s">
-        <v>125</v>
+        <v>91</v>
       </c>
       <c r="H22" t="s">
         <v>16</v>
@@ -1938,93 +2001,93 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B23" t="s">
         <v>80</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="F23" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="G23" t="s">
-        <v>128</v>
+        <v>79</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B24" t="s">
         <v>80</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D24" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="F24" t="s">
-        <v>17</v>
+        <v>127</v>
       </c>
       <c r="G24" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B25" t="s">
         <v>80</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="F25" t="s">
-        <v>41</v>
+        <v>106</v>
       </c>
       <c r="G25" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
@@ -2040,94 +2103,94 @@
     </row>
     <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B26" t="s">
         <v>80</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="F26" t="s">
-        <v>55</v>
+        <v>106</v>
       </c>
       <c r="G26" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
       <c r="H26" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B27" t="s">
         <v>80</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="F27" t="s">
-        <v>44</v>
+        <v>84</v>
       </c>
       <c r="G27" t="s">
-        <v>108</v>
+        <v>132</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B28" t="s">
         <v>80</v>
       </c>
       <c r="C28" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" t="s">
+        <v>127</v>
+      </c>
+      <c r="G28" t="s">
         <v>134</v>
       </c>
-      <c r="D28" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" t="s">
-        <v>10</v>
-      </c>
-      <c r="F28" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" t="s">
-        <v>69</v>
-      </c>
       <c r="H28" t="s">
         <v>11</v>
       </c>
@@ -2140,9 +2203,9 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B29" t="s">
         <v>80</v>
@@ -2154,32 +2217,32 @@
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>136</v>
@@ -2188,47 +2251,47 @@
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G30" t="s">
-        <v>103</v>
+        <v>83</v>
       </c>
       <c r="H30" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>137</v>
       </c>
       <c r="D31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="F31" t="s">
-        <v>63</v>
+        <v>10</v>
       </c>
       <c r="G31" t="s">
-        <v>138</v>
+        <v>69</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
@@ -2242,64 +2305,64 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B32" t="s">
         <v>72</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E32" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F32" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G32" t="s">
-        <v>110</v>
+        <v>122</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B33" t="s">
         <v>72</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F33" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="G33" t="s">
-        <v>141</v>
+        <v>85</v>
       </c>
       <c r="H33" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2312,161 +2375,161 @@
     </row>
     <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B34" t="s">
         <v>72</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F34" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>90</v>
+        <v>141</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B35" t="s">
         <v>72</v>
       </c>
       <c r="C35" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35" t="s">
+        <v>69</v>
+      </c>
+      <c r="H35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J35" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B36" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="D35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" t="s">
+      <c r="D36" t="s">
+        <v>9</v>
+      </c>
+      <c r="E36" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" t="s">
+        <v>106</v>
+      </c>
+      <c r="G36" t="s">
+        <v>97</v>
+      </c>
+      <c r="H36" t="s">
+        <v>11</v>
+      </c>
+      <c r="I36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B37" t="s">
+        <v>72</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D37" t="s">
+        <v>12</v>
+      </c>
+      <c r="E37" t="s">
         <v>63</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F37" t="s">
         <v>63</v>
       </c>
-      <c r="G35" t="s">
-        <v>144</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="G37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H37" t="s">
         <v>16</v>
       </c>
-      <c r="I35" t="str">
+      <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J35" t="str">
+      <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36" s="5">
-        <v>46106</v>
-      </c>
-      <c r="B36" t="s">
-        <v>73</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="D36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s">
-        <v>17</v>
-      </c>
-      <c r="F36" t="s">
-        <v>17</v>
-      </c>
-      <c r="G36" t="s">
-        <v>90</v>
-      </c>
-      <c r="H36" t="s">
-        <v>11</v>
-      </c>
-      <c r="I36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" s="5">
-        <v>46106</v>
-      </c>
-      <c r="B37" t="s">
-        <v>73</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="D37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E37" t="s">
-        <v>25</v>
-      </c>
-      <c r="F37" t="s">
-        <v>25</v>
-      </c>
-      <c r="G37" t="s">
-        <v>103</v>
-      </c>
-      <c r="H37" t="s">
-        <v>11</v>
-      </c>
-      <c r="I37" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J37" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B38" t="s">
         <v>73</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E38" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F38" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G38" t="s">
-        <v>148</v>
+        <v>97</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -2477,216 +2540,216 @@
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B39" t="s">
         <v>73</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F39" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G39" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H39" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B40" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="D40" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="F40" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="G40" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B41" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D41" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>17</v>
+        <v>88</v>
       </c>
       <c r="F41" t="s">
-        <v>84</v>
+        <v>150</v>
       </c>
       <c r="G41" t="s">
-        <v>90</v>
+        <v>151</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B42" t="s">
         <v>78</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>154</v>
+        <v>69</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B43" t="s">
         <v>78</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D43" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E43" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F43" t="s">
-        <v>37</v>
+        <v>89</v>
       </c>
       <c r="G43" t="s">
-        <v>110</v>
+        <v>154</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B44" t="s">
         <v>78</v>
       </c>
       <c r="C44" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="D44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>17</v>
+      </c>
+      <c r="F44" t="s">
         <v>156</v>
-      </c>
-      <c r="D44" t="s">
-        <v>12</v>
-      </c>
-      <c r="E44" t="s">
-        <v>61</v>
-      </c>
-      <c r="F44" t="s">
-        <v>61</v>
       </c>
       <c r="G44" t="s">
         <v>157</v>
       </c>
       <c r="H44" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B45" t="s">
         <v>78</v>
@@ -2698,13 +2761,13 @@
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="F45" t="s">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="G45" t="s">
-        <v>159</v>
+        <v>122</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
@@ -2715,37 +2778,37 @@
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B46" t="s">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="C46" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>37</v>
+      </c>
+      <c r="F46" t="s">
+        <v>37</v>
+      </c>
+      <c r="G46" t="s">
         <v>160</v>
       </c>
-      <c r="D46" t="s">
-        <v>13</v>
-      </c>
-      <c r="E46" t="s">
-        <v>17</v>
-      </c>
-      <c r="F46" t="s">
-        <v>84</v>
-      </c>
-      <c r="G46" t="s">
-        <v>90</v>
-      </c>
       <c r="H46" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2754,10 +2817,10 @@
     </row>
     <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B47" t="s">
-        <v>29</v>
+        <v>78</v>
       </c>
       <c r="C47" s="6" t="s">
         <v>161</v>
@@ -2766,81 +2829,81 @@
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F47" t="s">
-        <v>10</v>
+        <v>162</v>
       </c>
       <c r="G47" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B48" t="s">
+        <v>78</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D48" t="s">
+        <v>82</v>
+      </c>
+      <c r="E48" t="s">
+        <v>17</v>
+      </c>
+      <c r="F48" t="s">
+        <v>17</v>
+      </c>
+      <c r="G48" t="s">
+        <v>164</v>
+      </c>
+      <c r="H48" t="s">
+        <v>16</v>
+      </c>
+      <c r="I48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="5">
-        <v>46106</v>
-      </c>
-      <c r="B48" t="s">
-        <v>29</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="D48" t="s">
-        <v>12</v>
-      </c>
-      <c r="E48" t="s">
-        <v>25</v>
-      </c>
-      <c r="F48" t="s">
-        <v>25</v>
-      </c>
-      <c r="G48" t="s">
-        <v>103</v>
-      </c>
-      <c r="H48" t="s">
-        <v>11</v>
-      </c>
-      <c r="I48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B49" t="s">
-        <v>29</v>
+        <v>165</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>167</v>
       </c>
       <c r="E49" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="F49" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G49" t="s">
-        <v>164</v>
+        <v>122</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
@@ -2851,120 +2914,120 @@
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B50" t="s">
-        <v>29</v>
+        <v>165</v>
       </c>
       <c r="C50" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>17</v>
+      </c>
+      <c r="F50" t="s">
+        <v>17</v>
+      </c>
+      <c r="G50" t="s">
+        <v>86</v>
+      </c>
+      <c r="H50" t="s">
+        <v>11</v>
+      </c>
+      <c r="I50" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J50" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B51" t="s">
         <v>165</v>
       </c>
-      <c r="D50" t="s">
-        <v>12</v>
-      </c>
-      <c r="E50" t="s">
-        <v>41</v>
-      </c>
-      <c r="F50" t="s">
-        <v>41</v>
-      </c>
-      <c r="G50" t="s">
-        <v>131</v>
-      </c>
-      <c r="H50" t="s">
-        <v>11</v>
-      </c>
-      <c r="I50" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J50" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" s="5">
-        <v>46106</v>
-      </c>
-      <c r="B51" t="s">
-        <v>29</v>
-      </c>
       <c r="C51" s="6" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D51" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="F51" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="G51" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>165</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="D52" t="s">
         <v>13</v>
       </c>
       <c r="E52" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="F52" t="s">
-        <v>169</v>
+        <v>25</v>
       </c>
       <c r="G52" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="H52" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B53" t="s">
-        <v>29</v>
+        <v>165</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D53" t="s">
         <v>12</v>
@@ -2973,10 +3036,10 @@
         <v>17</v>
       </c>
       <c r="F53" t="s">
-        <v>17</v>
+        <v>84</v>
       </c>
       <c r="G53" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
@@ -2992,104 +3055,546 @@
     </row>
     <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B54" t="s">
-        <v>29</v>
+        <v>165</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D54" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F54" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="G54" t="s">
-        <v>85</v>
+        <v>97</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
       </c>
       <c r="I54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B55" t="s">
+        <v>165</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>15</v>
+      </c>
+      <c r="F55" t="s">
+        <v>175</v>
+      </c>
+      <c r="G55" t="s">
+        <v>176</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J54" t="str">
+      <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55" s="5">
-        <v>46106</v>
-      </c>
-      <c r="B55" t="s">
-        <v>29</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>14</v>
-      </c>
-      <c r="F55" t="s">
-        <v>14</v>
-      </c>
-      <c r="G55" t="s">
-        <v>110</v>
-      </c>
-      <c r="H55" t="s">
-        <v>11</v>
-      </c>
-      <c r="I55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46106</v>
+        <v>46107</v>
       </c>
       <c r="B56" t="s">
+        <v>165</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>10</v>
+      </c>
+      <c r="G56" t="s">
+        <v>69</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B57" t="s">
+        <v>165</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>24</v>
+      </c>
+      <c r="F57" t="s">
+        <v>179</v>
+      </c>
+      <c r="G57" t="s">
+        <v>180</v>
+      </c>
+      <c r="H57" t="s">
+        <v>26</v>
+      </c>
+      <c r="I57" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J57" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A58" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B58" t="s">
+        <v>165</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>17</v>
+      </c>
+      <c r="F58" t="s">
+        <v>156</v>
+      </c>
+      <c r="G58" t="s">
+        <v>182</v>
+      </c>
+      <c r="H58" t="s">
+        <v>26</v>
+      </c>
+      <c r="I58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A59" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B59" t="s">
         <v>29</v>
       </c>
-      <c r="C56" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D56" t="s">
-        <v>12</v>
-      </c>
-      <c r="E56" t="s">
+      <c r="C59" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D59" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" t="s">
+        <v>25</v>
+      </c>
+      <c r="F59" t="s">
+        <v>25</v>
+      </c>
+      <c r="G59" t="s">
+        <v>97</v>
+      </c>
+      <c r="H59" t="s">
+        <v>11</v>
+      </c>
+      <c r="I59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A60" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B60" t="s">
+        <v>29</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D60" t="s">
+        <v>81</v>
+      </c>
+      <c r="E60" t="s">
+        <v>10</v>
+      </c>
+      <c r="F60" t="s">
+        <v>10</v>
+      </c>
+      <c r="G60" t="s">
+        <v>69</v>
+      </c>
+      <c r="H60" t="s">
+        <v>11</v>
+      </c>
+      <c r="I60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B61" t="s">
+        <v>29</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" t="s">
         <v>23</v>
       </c>
-      <c r="F56" t="s">
+      <c r="F61" t="s">
         <v>23</v>
       </c>
-      <c r="G56" t="s">
-        <v>174</v>
-      </c>
-      <c r="H56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I56" t="str">
+      <c r="G61" t="s">
+        <v>186</v>
+      </c>
+      <c r="H61" t="s">
+        <v>26</v>
+      </c>
+      <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J56" t="str">
+      <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A62" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B62" t="s">
+        <v>29</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>88</v>
+      </c>
+      <c r="F62" t="s">
+        <v>150</v>
+      </c>
+      <c r="G62" t="s">
+        <v>151</v>
+      </c>
+      <c r="H62" t="s">
+        <v>26</v>
+      </c>
+      <c r="I62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B63" t="s">
+        <v>29</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>37</v>
+      </c>
+      <c r="F63" t="s">
+        <v>127</v>
+      </c>
+      <c r="G63" t="s">
+        <v>79</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+      <c r="I63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B64" t="s">
+        <v>29</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D64" t="s">
+        <v>81</v>
+      </c>
+      <c r="E64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F64" t="s">
+        <v>17</v>
+      </c>
+      <c r="G64" t="s">
+        <v>94</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B65" t="s">
+        <v>189</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D65" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65" t="s">
+        <v>37</v>
+      </c>
+      <c r="F65" t="s">
+        <v>127</v>
+      </c>
+      <c r="G65" t="s">
+        <v>79</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A66" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B66" t="s">
+        <v>189</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>24</v>
+      </c>
+      <c r="F66" t="s">
+        <v>2</v>
+      </c>
+      <c r="G66" t="s">
+        <v>192</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B67" t="s">
+        <v>189</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>10</v>
+      </c>
+      <c r="F67" t="s">
+        <v>10</v>
+      </c>
+      <c r="G67" t="s">
+        <v>69</v>
+      </c>
+      <c r="H67" t="s">
+        <v>11</v>
+      </c>
+      <c r="I67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A68" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B68" t="s">
+        <v>189</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" t="s">
+        <v>24</v>
+      </c>
+      <c r="F68" t="s">
+        <v>106</v>
+      </c>
+      <c r="G68" t="s">
+        <v>97</v>
+      </c>
+      <c r="H68" t="s">
+        <v>11</v>
+      </c>
+      <c r="I68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" s="5">
+        <v>46107</v>
+      </c>
+      <c r="B69" t="s">
+        <v>189</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" t="s">
+        <v>25</v>
+      </c>
+      <c r="F69" t="s">
+        <v>25</v>
+      </c>
+      <c r="G69" t="s">
+        <v>122</v>
+      </c>
+      <c r="H69" t="s">
+        <v>11</v>
+      </c>
+      <c r="I69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Reporte 31 de marzo
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{752C8D3E-40EA-48B0-AFA3-396176307FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE1FCAE8-DE8F-4C3D-81FF-FD7607F6097F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="194">
   <si>
     <t>Fecha</t>
   </si>
@@ -288,12 +288,6 @@
     <t>Alcalde</t>
   </si>
   <si>
-    <t>Sipdus</t>
-  </si>
-  <si>
-    <t>Sitmah</t>
-  </si>
-  <si>
     <t>Publicidad gubernamental</t>
   </si>
   <si>
@@ -312,301 +306,319 @@
     <t>Plaza Juárez</t>
   </si>
   <si>
-    <t>Fuga de hidrocarburo</t>
-  </si>
-  <si>
-    <t>Tecnificación De Riego</t>
-  </si>
-  <si>
     <t>Zunoticia</t>
   </si>
   <si>
-    <t>Israel Félix</t>
-  </si>
-  <si>
-    <t>alcalde</t>
-  </si>
-  <si>
-    <t>Reabre El Chico por temporada vacacional</t>
-  </si>
-  <si>
-    <t>Saneamiento forestal</t>
-  </si>
-  <si>
-    <t>Pachuca inicia con poco movimiento turístico</t>
-  </si>
-  <si>
-    <t>Certifican al Hospital del Niño</t>
-  </si>
-  <si>
     <t>Certificación</t>
   </si>
   <si>
-    <t>Difícil respoetar el carril del Tuzobús</t>
-  </si>
-  <si>
-    <t>Carril confinado</t>
-  </si>
-  <si>
-    <t>Avanza remodelación en mercado Barreteros</t>
-  </si>
-  <si>
-    <t>Rehabilitación De Mercados</t>
-  </si>
-  <si>
-    <t>Inicia Semana Santa con llamado a la fe y humildad</t>
-  </si>
-  <si>
-    <t>Avanza 40% el Parque Industrial en Cd. Sahagún</t>
-  </si>
-  <si>
-    <t>Parque industrial</t>
-  </si>
-  <si>
-    <t>Santas vacaciones</t>
-  </si>
-  <si>
-    <t>Hospital del Niño</t>
-  </si>
-  <si>
-    <t>INE desginará 2 consejerías del IEEH en noviembre</t>
-  </si>
-  <si>
-    <t>Consejeros Electorales</t>
-  </si>
-  <si>
-    <t>MANTIENEN LA  CARLOS  MORENO  AMBICIÓN VIVA</t>
-  </si>
-  <si>
-    <t>EL AZTECA SE DECLARA LISTO P113</t>
-  </si>
-  <si>
-    <t>SIGUE LA BÚSQUEDA DE DORIAN Y CARLA DONAJÍ</t>
-  </si>
-  <si>
-    <t>Personas desaparecidas</t>
-  </si>
-  <si>
-    <t>LAS LAJAS CELEBRA EL DOMINGO DE RAMOS;  INICIA SEMANA SANTA</t>
-  </si>
-  <si>
-    <t>EN HIDALGO SE  CONCENTRA CASI  30 POR CIENTO  DEL HUACHICOLEO</t>
-  </si>
-  <si>
-    <t>Huachicol</t>
-  </si>
-  <si>
-    <t>LANZA MORENA  ADVERTENCIA DE  RESTRICCIONES  A CANDIDATOS</t>
-  </si>
-  <si>
-    <t>Sucesión alcaldía</t>
-  </si>
-  <si>
-    <t>VENDEN PALMAS Y DIFUNDEN LAS  ESCRITURAS ENTRE LOS NIÑOS</t>
-  </si>
-  <si>
-    <t>Señalan hacinamiento y 33 incidencias dentro de los penales estatales</t>
-  </si>
-  <si>
-    <t>Deficiencias Ceresos</t>
-  </si>
-  <si>
-    <t>Sumaron cárceles 2025 158 quejas ante el organismo</t>
-  </si>
-  <si>
-    <t>Queja CDHEH</t>
-  </si>
-  <si>
-    <t>La policía arresta a 25 por quemar basura en la capital</t>
-  </si>
-  <si>
-    <t>Sanciones por basura</t>
-  </si>
-  <si>
-    <t>En Apan caen con camiones y toneladas de carga robada</t>
-  </si>
-  <si>
-    <t>Combate a la delincuencia</t>
-  </si>
-  <si>
-    <t>Llevan vecinos a escena la entrada de Jesús a Jerusalén</t>
-  </si>
-  <si>
-    <t>Revelan que los humanos tuvieron perros antes que agricultura</t>
-  </si>
-  <si>
-    <t>Trump expulsó menos mexicanos que Biden</t>
-  </si>
-  <si>
-    <t>Irán destruye un avión de EU en una base de Arabia Saudí</t>
-  </si>
-  <si>
-    <t>Colección Gelman sigue siendo mexicana por convenio tripartita</t>
-  </si>
-  <si>
-    <t>Aumentaron en febrero delitos contra la familia</t>
-  </si>
-  <si>
-    <t>Violencia familiar</t>
-  </si>
-  <si>
-    <t>Sheinbaum entrega títulos agrarios a mujeres: fija meta sexenal de 150 mil</t>
-  </si>
-  <si>
-    <t>Apoyo A La Mujer</t>
-  </si>
-  <si>
-    <t>Gobierno prevé ahorrar 15 mil litros de agua por segundo vía tecnificación</t>
-  </si>
-  <si>
-    <t>Hallan 16 restos  humanos en  Guaymas</t>
-  </si>
-  <si>
-    <t>FGR</t>
-  </si>
-  <si>
-    <t>Localización De Restos</t>
-  </si>
-  <si>
-    <t>Domingo de Ramos en Pachuca</t>
-  </si>
-  <si>
-    <t>Guerras, rupturas del orden internacional, resquebrajamiento  democrático, conflictos migratorios y crisis económicas  aparte, la IA ha marcado ya el siglo XXI”.</t>
-  </si>
-  <si>
-    <t>Convocan a reflexionar y renovar la fe tras inicio de Semana Santa</t>
-  </si>
-  <si>
-    <t>Se movilizan cuerpos de  emergencia por derrame de  gasolina en Tlaxiaca</t>
-  </si>
-  <si>
-    <t>Certifica organismo internacional a Hospital del Niño DIF por bienestar organizacional</t>
-  </si>
-  <si>
-    <t>Refuerzan seguridad  en Pachuca con  presencia operativa y  módulos informativos</t>
-  </si>
-  <si>
-    <t>Refuerzo De Seguridad</t>
-  </si>
-  <si>
-    <t>Frustra chofer intento de asalto sobre la México-Pachuca; hubo cuatro lesionados</t>
-  </si>
-  <si>
-    <t>Asalto a transporte público</t>
-  </si>
-  <si>
-    <t>SSH llaman a reforzar prevención ante casos de Coxackie en la región</t>
-  </si>
-  <si>
-    <t>titul</t>
-  </si>
-  <si>
-    <t>Prevención De Enfermedades</t>
-  </si>
-  <si>
-    <t>Logra Hospital del Niño DIF Hidalgo certificación internacional</t>
-  </si>
-  <si>
-    <t>Se cumplen 49 años de la aparición de la virgen de Tahuizán</t>
-  </si>
-  <si>
-    <t>Palmas, tradición de Domingo de Ramos</t>
-  </si>
-  <si>
-    <t>Ordenar, dignificar y participar: así transforma Hidalgo su imagen urbana</t>
-  </si>
-  <si>
-    <t>Imagen Urbana</t>
-  </si>
-  <si>
-    <t>Mi futuro político está en la sección 15 del SNTE: Said Vargas</t>
-  </si>
-  <si>
-    <t>Israel Félix, el reciclaje incómodo y la prueba de Morena</t>
-  </si>
-  <si>
-    <t>Gobers"" combaten al crimen</t>
-  </si>
-  <si>
-    <t>Propone Reyes tarifa única de estacionamientos en Hidalgo</t>
-  </si>
-  <si>
-    <t>Estacionamientos</t>
-  </si>
-  <si>
-    <t>Invadir carril pone en riesgo a 70 mil usuarios</t>
-  </si>
-  <si>
-    <t>Evacuán gasolinera en San Agustín Tlaxiaca por fuga de gasolina</t>
-  </si>
-  <si>
-    <t>Pachuca reasigna casi 190 mdp a infraestructura en primera modificación presupuestal</t>
-  </si>
-  <si>
-    <t>Obras De Infraestructura</t>
-  </si>
-  <si>
-    <t>Juegos magisteriales</t>
-  </si>
-  <si>
-    <t>Realizan jornada masiva integral de recuperación en Quma</t>
-  </si>
-  <si>
-    <t>Recuperación De Espacios Públicos</t>
-  </si>
-  <si>
-    <t>Policía de Pachuca mantiene activos módulos de atención</t>
-  </si>
-  <si>
-    <t>Policía municipal</t>
-  </si>
-  <si>
-    <t>Fundación ""Nadie se queda atrás"" dona 250 kilos de alimento a Todo por Ellos</t>
-  </si>
-  <si>
-    <t>Supervisarán razers en Mineral del Chico tras accidente; inspecciones iniciarán en abril</t>
-  </si>
-  <si>
-    <t>Regularización De Vehículos Turísticos</t>
-  </si>
-  <si>
-    <t>Profeco desplegará operativo en Hidalgo para evitar alza de precios en Semana Santa</t>
-  </si>
-  <si>
-    <t>Conoce la pirámide de Movilidad</t>
-  </si>
-  <si>
-    <t>Despliegan estrategia territorial por ley de imagen urbana en Hidalgo</t>
-  </si>
-  <si>
-    <t>Activa seguridad pública de Pachuca módulos de atención en los principales accesos</t>
-  </si>
-  <si>
-    <t>Atienden fuga de combustible en una estación de la Pachuca-Actopan</t>
-  </si>
-  <si>
-    <t>Recuperan 15 tractocamiones y 24 toneladas de mercancía en Apan</t>
-  </si>
-  <si>
-    <t>Logra Hospital del Niño DIF certificación internacional</t>
-  </si>
-  <si>
-    <t>Anúnciate con nosotros</t>
-  </si>
-  <si>
-    <t>Se vivió el Domingo de Ramos en el Arbolito</t>
-  </si>
-  <si>
-    <t>Más de 300 elementos buscan a mineros atrapados en Sinaloa</t>
-  </si>
-  <si>
-    <t>Encuentran a hombre sin vida, se habría suicidado</t>
-  </si>
-  <si>
-    <t>Realizan diagnósticos en 70 municipios</t>
-  </si>
-  <si>
-    <t>Es preciso, urgente, entender que la vida va más allá de la grilla barata, la diversión con el dolor ajeno. Es preciso entender, que de alguna forma, todos, absolutamente todos, vamos en la misma embarcación, que es la existencia</t>
+    <t>Apan, verifican en unidad móvil</t>
+  </si>
+  <si>
+    <t>Verificación vehicular</t>
+  </si>
+  <si>
+    <t>Votan por eliminar pensión dorada</t>
+  </si>
+  <si>
+    <t>Reforma De Ley</t>
+  </si>
+  <si>
+    <t>Viento mejora calidad del aire en Pachuca</t>
+  </si>
+  <si>
+    <t>Calidad del aire</t>
+  </si>
+  <si>
+    <t>Registran primer caso de barrenador en Alfajayucan</t>
+  </si>
+  <si>
+    <t>Gusano barrenador</t>
+  </si>
+  <si>
+    <t>Fallece otro mexicano en EU</t>
+  </si>
+  <si>
+    <t>Por participación política de mujeres, 10 partidos destinarán 12.7 mdp</t>
+  </si>
+  <si>
+    <t>Financiamiento a Partidos</t>
+  </si>
+  <si>
+    <t>Misticismo y arte</t>
+  </si>
+  <si>
+    <t>Muralismo</t>
+  </si>
+  <si>
+    <t>En estos días, miles de personas tienen la posibilidad de tomar un periodo de vacaciones. Muchos de ellos eligen destinos tradicionales...</t>
+  </si>
+  <si>
+    <t>Ponen freno a delitos en Hidalgo</t>
+  </si>
+  <si>
+    <t>Reunión Gabinete De Seguridad</t>
+  </si>
+  <si>
+    <t>Conagua extiende demora de obra</t>
+  </si>
+  <si>
+    <t>Conagua</t>
+  </si>
+  <si>
+    <t>Obra inconclusa</t>
+  </si>
+  <si>
+    <t>BASURERO DE TULA OPERA SIN MIA</t>
+  </si>
+  <si>
+    <t>Disposición de residuos</t>
+  </si>
+  <si>
+    <t>LOS TUZOS BUSCAN  SALTO COMPETITIVO</t>
+  </si>
+  <si>
+    <t>ENSAYO  DE FUEGO  PARA EL  TRICOLOR</t>
+  </si>
+  <si>
+    <t>BASURERO COLAPSÓ  PORQUE LA CELDA “SE  PARTIÓ”: SEMARNATH</t>
+  </si>
+  <si>
+    <t>Disposición de basura</t>
+  </si>
+  <si>
+    <t>DETECTA LA SSH PLAGA DE GUSANO BARRENADOR EN  PERROS Y GATOS</t>
+  </si>
+  <si>
+    <t>Hidalgo tiene 5 casos activos de sarampión</t>
+  </si>
+  <si>
+    <t>Sarampión</t>
+  </si>
+  <si>
+    <t>Hidlago, con 4 nominaciones en lo Mejor de México 2026</t>
+  </si>
+  <si>
+    <t>Premio turístico</t>
+  </si>
+  <si>
+    <t>AVALAN LÍMITE  A SALARIOS Y  PENSIONES DE  LOS SERVIDORES</t>
+  </si>
+  <si>
+    <t>Crisis en Tula: relleno sanitario pone en jaque a 14 municipios</t>
+  </si>
+  <si>
+    <t>Vehículos e incendios afectan la calidad del aire</t>
+  </si>
+  <si>
+    <t>Gusano barrenador. Advierten daño a mascotas; detectan 67 casos en ganado</t>
+  </si>
+  <si>
+    <t>Suman 459 internos del fuero federal en el estado</t>
+  </si>
+  <si>
+    <t>Anomalías Ceresos</t>
+  </si>
+  <si>
+    <t>Accidente. Tráiler provoca cierre de la México Pachuca</t>
+  </si>
+  <si>
+    <t>Accidente Carretero</t>
+  </si>
+  <si>
+    <t>Decomisan casi 100 mil litros de gas LP en operativo</t>
+  </si>
+  <si>
+    <t>Combate Al Gaschicol</t>
+  </si>
+  <si>
+    <t>Por presuntas omisiones e irregularidades los indagan</t>
+  </si>
+  <si>
+    <t>Omisión</t>
+  </si>
+  <si>
+    <t>México llevará ante la CIDH la muerte de 14 paisanos en custodia de Inmigración</t>
+  </si>
+  <si>
+    <t>El cáncer más subestimado y tratable</t>
+  </si>
+  <si>
+    <t>Analizan  traer barcos contra culex</t>
+  </si>
+  <si>
+    <t>Mosco Culex</t>
+  </si>
+  <si>
+    <t>Alcaldías de la región Tula presionan para  reactivar basurero</t>
+  </si>
+  <si>
+    <t>Inauguración  del Mundial será “histórica”</t>
+  </si>
+  <si>
+    <t>Mundial De Futbol</t>
+  </si>
+  <si>
+    <t>El “solárium”   de Palacio  Nacional</t>
+  </si>
+  <si>
+    <t>Pobladores de la comunidad de Doxey acusaron que, ante la falta de alternativas para depositar los desechos urbanos de  Tlaxcoapan, la alcaldía habilitó un tiradero clandestino en terrenos cercanos a la autopista Arco Norte.</t>
+  </si>
+  <si>
+    <t>Basurero Clandestino</t>
+  </si>
+  <si>
+    <t>Ricardo Salinas Pliego propuso que las personas que reciben programas sociales no deberían poder votar.  La declaración no fue un desliz, sino una confesión. Porque detrás de esa idea hay una ideología muy  peligrosa: el populismo de derechas”.</t>
+  </si>
+  <si>
+    <t>Hay 67 casos activos de gusano barrenador; cinco se detectaron en caminos</t>
+  </si>
+  <si>
+    <t>Avala Congreso estatal reforma para  eliminar “pensiones doradas”</t>
+  </si>
+  <si>
+    <t>Promueven justicia agraria para  mujeres mediante caravana  federal en Huejutla</t>
+  </si>
+  <si>
+    <t>Caravana para mujeres</t>
+  </si>
+  <si>
+    <t>Hidalgo, segundo lugar nacional en  hectáreas afectadas por incendios  forestales</t>
+  </si>
+  <si>
+    <t>Incendios forestales</t>
+  </si>
+  <si>
+    <t>¿Y el agua para cuándo...?</t>
+  </si>
+  <si>
+    <t>Agua</t>
+  </si>
+  <si>
+    <t>Abasto De Agua</t>
+  </si>
+  <si>
+    <t>Nuevas experiencias posicionan a Hidalgo entre los destinos preferidos de México</t>
+  </si>
+  <si>
+    <t>Promoción turística</t>
+  </si>
+  <si>
+    <t>Banderazo del operativo de Semana Santa 2026 en Huejutla</t>
+  </si>
+  <si>
+    <t>Fortalece Hidalgo estrategia para control y erradicación del gusano barrenador</t>
+  </si>
+  <si>
+    <t>Comerciantes instalan puestos de venta en la ribera del Río Atlapexco</t>
+  </si>
+  <si>
+    <t>Ambulantaje</t>
+  </si>
+  <si>
+    <t>Autoridades refuerzan seguridad y servicios durante Semana Santa 2026</t>
+  </si>
+  <si>
+    <t>Plaga avanza: detectan gusano barrenador en perros de Hidalgo</t>
+  </si>
+  <si>
+    <t>gusano</t>
+  </si>
+  <si>
+    <t>Colapso de relleno sanitario exhibe omisión de municipios</t>
+  </si>
+  <si>
+    <t>Rescate arqueológico</t>
+  </si>
+  <si>
+    <t>INAH</t>
+  </si>
+  <si>
+    <t>Zona Arqueológica</t>
+  </si>
+  <si>
+    <t>Colapsa auditorio en Zimapán tras granizada</t>
+  </si>
+  <si>
+    <t>Afectaciones Por Lluvias</t>
+  </si>
+  <si>
+    <t>Hidalgo vs pensiones doradas</t>
+  </si>
+  <si>
+    <t>Partido Verde arma estructura en Zimapán</t>
+  </si>
+  <si>
+    <t>Trabajo partidista</t>
+  </si>
+  <si>
+    <t>El pase turístico que es todo menos turístico</t>
+  </si>
+  <si>
+    <t>Pase turístico</t>
+  </si>
+  <si>
+    <t>Más de 100 sabores en la 2a feria del helado</t>
+  </si>
+  <si>
+    <t>Festival Gastronómico</t>
+  </si>
+  <si>
+    <t>Sección 15 se fortalece: avances históricos y unidad marcan el liderazgo de Said Vargas</t>
+  </si>
+  <si>
+    <t>Gabinete de Seguridad detiene a 40 personas durante operativos permanentes</t>
+  </si>
+  <si>
+    <t>Atitalaquia estrena nuevo camión recolector de basura</t>
+  </si>
+  <si>
+    <t>Recolección De Basura</t>
+  </si>
+  <si>
+    <t>Atitalaquia y Atotonilco dan banderazo de arranque al Operativo Semana Santa</t>
+  </si>
+  <si>
+    <t>Claudia Sandoval recibe nueva patrulla</t>
+  </si>
+  <si>
+    <t>Entrega de patrullas</t>
+  </si>
+  <si>
+    <t>Refuerzan seguridad en Ajacuba</t>
+  </si>
+  <si>
+    <t>Tlahuelilpan foralece seguridad</t>
+  </si>
+  <si>
+    <t>Este martes, último día para pagar predial con descuento</t>
+  </si>
+  <si>
+    <t>Predial</t>
+  </si>
+  <si>
+    <t>Gabinete de seguridad detiene a 40 personas durante operativos permanentes</t>
+  </si>
+  <si>
+    <t>Instalarán unidad móvil para verificación vehicular en Pachuca</t>
+  </si>
+  <si>
+    <t>Pirámide de Movilidad</t>
+  </si>
+  <si>
+    <t>En una semana, detuvieron a 40 presuntos delincuentes</t>
+  </si>
+  <si>
+    <t>México trabaja para reactivar el envío de petróleo a Cuba</t>
+  </si>
+  <si>
+    <t>Tan lejos de Dios y tan cerca del Edomex</t>
+  </si>
+  <si>
+    <t>Diputados se pronuncian ante caso de violencia</t>
+  </si>
+  <si>
+    <t>Exhorto</t>
   </si>
 </sst>
 </file>
@@ -853,8 +865,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J70" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J70" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J69" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J69" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1220,7 +1232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1269,16 +1281,16 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B2" t="s">
         <v>70</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
         <v>21</v>
@@ -1287,7 +1299,7 @@
         <v>21</v>
       </c>
       <c r="G2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
@@ -1303,25 +1315,25 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B3" t="s">
         <v>70</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="G3" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
@@ -1337,59 +1349,59 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B4" t="s">
         <v>70</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B5" t="s">
         <v>70</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
       <c r="F5" t="s">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="G5" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
@@ -1405,50 +1417,50 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B6" t="s">
         <v>70</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
         <v>10</v>
@@ -1457,7 +1469,7 @@
         <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>86</v>
+        <v>101</v>
       </c>
       <c r="H7" t="s">
         <v>11</v>
@@ -1473,66 +1485,66 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B8" t="s">
         <v>71</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H8" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B9" t="s">
         <v>71</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1541,28 +1553,28 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B10" t="s">
         <v>71</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>109</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H10" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1570,37 +1582,37 @@
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B11" t="s">
         <v>71</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F11" t="s">
-        <v>10</v>
+        <v>108</v>
       </c>
       <c r="G11" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H11" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1609,32 +1621,32 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F12" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G12" t="s">
-        <v>77</v>
+        <v>111</v>
       </c>
       <c r="H12" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1643,13 +1655,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B13" t="s">
         <v>74</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1677,96 +1689,96 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B14" t="s">
         <v>74</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>115</v>
+        <v>77</v>
       </c>
       <c r="H14" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E15" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F15" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G15" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B16" t="s">
         <v>74</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="F16" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="G16" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="H16" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1777,197 +1789,197 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B17" t="s">
         <v>74</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F17" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="G17" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B18" t="s">
         <v>74</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="D18" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F18" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G18" t="s">
-        <v>69</v>
+        <v>120</v>
       </c>
       <c r="H18" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B19" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="F19" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="G19" t="s">
-        <v>123</v>
+        <v>94</v>
       </c>
       <c r="H19" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B20" t="s">
         <v>79</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E20" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F20" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G20" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="H20" t="s">
         <v>16</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B21" t="s">
         <v>79</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F21" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G21" t="s">
-        <v>127</v>
+        <v>96</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B22" t="s">
         <v>79</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="F22" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="G22" t="s">
-        <v>129</v>
+        <v>98</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
@@ -1983,50 +1995,50 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B23" t="s">
         <v>79</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D23" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F23" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G23" t="s">
-        <v>86</v>
+        <v>126</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B24" t="s">
         <v>79</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="D24" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E24" t="s">
         <v>10</v>
@@ -2035,7 +2047,7 @@
         <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>69</v>
+        <v>128</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
@@ -2051,47 +2063,47 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B25" t="s">
         <v>79</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F25" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G25" t="s">
-        <v>69</v>
+        <v>130</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B26" t="s">
         <v>79</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
@@ -2103,10 +2115,10 @@
         <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>69</v>
+        <v>132</v>
       </c>
       <c r="H26" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2119,13 +2131,13 @@
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B27" t="s">
         <v>79</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -2153,93 +2165,93 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B28" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G28" t="s">
-        <v>136</v>
+        <v>69</v>
       </c>
       <c r="H28" t="s">
         <v>11</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B29" t="s">
         <v>72</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F29" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G29" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B30" t="s">
         <v>72</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D30" t="s">
         <v>13</v>
       </c>
       <c r="E30" t="s">
-        <v>83</v>
+        <v>21</v>
       </c>
       <c r="F30" t="s">
-        <v>83</v>
+        <v>2</v>
       </c>
       <c r="G30" t="s">
-        <v>92</v>
+        <v>115</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
@@ -2255,13 +2267,13 @@
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B31" t="s">
         <v>72</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
@@ -2270,13 +2282,13 @@
         <v>14</v>
       </c>
       <c r="F31" t="s">
-        <v>141</v>
+        <v>14</v>
       </c>
       <c r="G31" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="H31" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2289,84 +2301,84 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B32" t="s">
         <v>72</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D32" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F32" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B33" t="s">
         <v>72</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E33" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F33" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G33" t="s">
-        <v>69</v>
+        <v>142</v>
       </c>
       <c r="H33" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
         <v>10</v>
@@ -2391,25 +2403,25 @@
     </row>
     <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B35" t="s">
         <v>73</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="F35" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="G35" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
@@ -2425,66 +2437,66 @@
     </row>
     <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B36" t="s">
         <v>73</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F36" t="s">
-        <v>109</v>
+        <v>37</v>
       </c>
       <c r="G36" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B37" t="s">
         <v>73</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F37" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G37" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2493,96 +2505,96 @@
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B38" t="s">
         <v>73</v>
       </c>
       <c r="C38" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>21</v>
+      </c>
+      <c r="F38" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" t="s">
+        <v>149</v>
+      </c>
+      <c r="H38" t="s">
+        <v>16</v>
+      </c>
+      <c r="I38" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J38" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="5">
+        <v>46112</v>
+      </c>
+      <c r="B39" t="s">
+        <v>89</v>
+      </c>
+      <c r="C39" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="D38" t="s">
-        <v>12</v>
-      </c>
-      <c r="E38" t="s">
-        <v>10</v>
-      </c>
-      <c r="F38" t="s">
-        <v>10</v>
-      </c>
-      <c r="G38" t="s">
-        <v>151</v>
-      </c>
-      <c r="H38" t="s">
-        <v>11</v>
-      </c>
-      <c r="I38" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J38" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" s="5">
-        <v>46111</v>
-      </c>
-      <c r="B39" t="s">
-        <v>93</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>152</v>
       </c>
       <c r="D39" t="s">
         <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F39" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G39" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H39" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B40" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="F40" t="s">
-        <v>109</v>
+        <v>32</v>
       </c>
       <c r="G40" t="s">
-        <v>100</v>
+        <v>154</v>
       </c>
       <c r="H40" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2595,134 +2607,134 @@
     </row>
     <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B41" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C41" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
+        <v>17</v>
+      </c>
+      <c r="F41" t="s">
+        <v>17</v>
+      </c>
+      <c r="G41" t="s">
+        <v>84</v>
+      </c>
+      <c r="H41" t="s">
+        <v>11</v>
+      </c>
+      <c r="I41" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J41" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="5">
+        <v>46112</v>
+      </c>
+      <c r="B42" t="s">
+        <v>89</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="D41" t="s">
-        <v>12</v>
-      </c>
-      <c r="E41" t="s">
-        <v>10</v>
-      </c>
-      <c r="F41" t="s">
-        <v>10</v>
-      </c>
-      <c r="G41" t="s">
-        <v>69</v>
-      </c>
-      <c r="H41" t="s">
-        <v>11</v>
-      </c>
-      <c r="I41" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J41" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42" s="5">
-        <v>46111</v>
-      </c>
-      <c r="B42" t="s">
-        <v>93</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>157</v>
-      </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="F42" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="G42" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B43" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="C43" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" t="s">
+        <v>10</v>
+      </c>
+      <c r="G43" t="s">
         <v>158</v>
       </c>
-      <c r="D43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" t="s">
-        <v>36</v>
-      </c>
-      <c r="F43" t="s">
-        <v>36</v>
-      </c>
-      <c r="G43" t="s">
-        <v>159</v>
-      </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B44" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D44" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G44" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2731,41 +2743,41 @@
     </row>
     <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B45" t="s">
         <v>78</v>
       </c>
       <c r="C45" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="D45" t="s">
+        <v>13</v>
+      </c>
+      <c r="E45" t="s">
+        <v>57</v>
+      </c>
+      <c r="F45" t="s">
+        <v>57</v>
+      </c>
+      <c r="G45" t="s">
         <v>161</v>
       </c>
-      <c r="D45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E45" t="s">
-        <v>19</v>
-      </c>
-      <c r="F45" t="s">
-        <v>19</v>
-      </c>
-      <c r="G45" t="s">
-        <v>94</v>
-      </c>
       <c r="H45" t="s">
         <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B46" t="s">
         <v>78</v>
@@ -2777,13 +2789,13 @@
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="F46" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="G46" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
@@ -2794,12 +2806,12 @@
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B47" t="s">
         <v>78</v>
@@ -2808,23 +2820,23 @@
         <v>163</v>
       </c>
       <c r="D47" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E47" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F47" t="s">
-        <v>82</v>
+        <v>164</v>
       </c>
       <c r="G47" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2833,25 +2845,25 @@
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B48" t="s">
         <v>78</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="F48" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="G48" t="s">
-        <v>102</v>
+        <v>167</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
@@ -2865,68 +2877,68 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B49" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D49" t="s">
-        <v>89</v>
+        <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="F49" t="s">
-        <v>87</v>
+        <v>37</v>
       </c>
       <c r="G49" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B50" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="F50" t="s">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="G50" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Partidos</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2935,50 +2947,50 @@
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B51" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="F51" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="G51" t="s">
-        <v>69</v>
+        <v>172</v>
       </c>
       <c r="H51" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B52" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D52" t="s">
-        <v>13</v>
+        <v>87</v>
       </c>
       <c r="E52" t="s">
         <v>17</v>
@@ -2987,7 +2999,7 @@
         <v>17</v>
       </c>
       <c r="G52" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
@@ -3003,16 +3015,16 @@
     </row>
     <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B53" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E53" t="s">
         <v>10</v>
@@ -3037,66 +3049,66 @@
     </row>
     <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B54" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D54" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E54" t="s">
+        <v>25</v>
+      </c>
+      <c r="F54" t="s">
+        <v>25</v>
+      </c>
+      <c r="G54" t="s">
+        <v>106</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+      <c r="I54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>46112</v>
+      </c>
+      <c r="B55" t="s">
+        <v>86</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
         <v>17</v>
       </c>
-      <c r="F54" t="s">
-        <v>173</v>
-      </c>
-      <c r="G54" t="s">
-        <v>86</v>
-      </c>
-      <c r="H54" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" t="str">
+      <c r="F55" t="s">
+        <v>17</v>
+      </c>
+      <c r="G55" t="s">
+        <v>178</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
-      </c>
-      <c r="J54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A55" s="5">
-        <v>46111</v>
-      </c>
-      <c r="B55" t="s">
-        <v>88</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>10</v>
-      </c>
-      <c r="F55" t="s">
-        <v>10</v>
-      </c>
-      <c r="G55" t="s">
-        <v>69</v>
-      </c>
-      <c r="H55" t="s">
-        <v>11</v>
-      </c>
-      <c r="I55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3105,66 +3117,66 @@
     </row>
     <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B56" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="F56" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="G56" t="s">
-        <v>176</v>
+        <v>84</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B57" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="D57" t="s">
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F57" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G57" t="s">
-        <v>86</v>
+        <v>181</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3173,161 +3185,161 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B58" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="D58" t="s">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="E58" t="s">
         <v>17</v>
       </c>
       <c r="F58" t="s">
+        <v>82</v>
+      </c>
+      <c r="G58" t="s">
+        <v>181</v>
+      </c>
+      <c r="H58" t="s">
+        <v>11</v>
+      </c>
+      <c r="I58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A59" s="5">
+        <v>46112</v>
+      </c>
+      <c r="B59" t="s">
+        <v>86</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D59" t="s">
+        <v>12</v>
+      </c>
+      <c r="E59" t="s">
         <v>17</v>
       </c>
-      <c r="G58" t="s">
-        <v>85</v>
-      </c>
-      <c r="H58" t="s">
-        <v>11</v>
-      </c>
-      <c r="I58" t="str">
+      <c r="F59" t="s">
+        <v>17</v>
+      </c>
+      <c r="G59" t="s">
+        <v>90</v>
+      </c>
+      <c r="H59" t="s">
+        <v>11</v>
+      </c>
+      <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
       </c>
-      <c r="J58" t="str">
+      <c r="J59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A59" s="5">
-        <v>46111</v>
-      </c>
-      <c r="B59" t="s">
-        <v>29</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="D59" t="s">
-        <v>13</v>
-      </c>
-      <c r="E59" t="s">
-        <v>36</v>
-      </c>
-      <c r="F59" t="s">
-        <v>36</v>
-      </c>
-      <c r="G59" t="s">
-        <v>159</v>
-      </c>
-      <c r="H59" t="s">
-        <v>11</v>
-      </c>
-      <c r="I59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B60" t="s">
         <v>29</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>180</v>
+        <v>153</v>
       </c>
       <c r="D60" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E60" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="F60" t="s">
-        <v>173</v>
+        <v>32</v>
       </c>
       <c r="G60" t="s">
-        <v>86</v>
+        <v>154</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B61" t="s">
         <v>29</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F61" t="s">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="G61" t="s">
-        <v>91</v>
+        <v>185</v>
       </c>
       <c r="H61" t="s">
         <v>11</v>
       </c>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A62" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B62" t="s">
         <v>29</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="D62" t="s">
         <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F62" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G62" t="s">
-        <v>129</v>
+        <v>106</v>
       </c>
       <c r="H62" t="s">
         <v>11</v>
@@ -3338,30 +3350,30 @@
       </c>
       <c r="J62" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A63" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B63" t="s">
         <v>29</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>183</v>
+        <v>156</v>
       </c>
       <c r="D63" t="s">
         <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>40</v>
+        <v>57</v>
       </c>
       <c r="F63" t="s">
-        <v>109</v>
+        <v>57</v>
       </c>
       <c r="G63" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H63" t="s">
         <v>11</v>
@@ -3375,126 +3387,126 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B64" t="s">
         <v>29</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="D64" t="s">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="E64" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="F64" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G64" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="H64" t="s">
         <v>11</v>
       </c>
       <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B65" t="s">
         <v>29</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="D65" t="s">
         <v>80</v>
       </c>
       <c r="E65" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F65" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G65" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="H65" t="s">
         <v>11</v>
       </c>
       <c r="I65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A66" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B66" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="D66" t="s">
         <v>13</v>
       </c>
       <c r="E66" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F66" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G66" t="s">
-        <v>69</v>
+        <v>106</v>
       </c>
       <c r="H66" t="s">
         <v>11</v>
       </c>
       <c r="I66" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J66" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B67" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="D67" t="s">
         <v>12</v>
       </c>
       <c r="E67" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F67" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G67" t="s">
         <v>69</v>
@@ -3504,7 +3516,7 @@
       </c>
       <c r="I67" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J67" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3513,16 +3525,16 @@
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B68" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="D68" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="E68" t="s">
         <v>10</v>
@@ -3547,68 +3559,34 @@
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" s="5">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B69" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="D69" t="s">
         <v>12</v>
       </c>
       <c r="E69" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F69" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G69" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="H69" t="s">
         <v>11</v>
       </c>
       <c r="I69" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" ht="75" x14ac:dyDescent="0.25">
-      <c r="A70" s="5">
-        <v>46111</v>
-      </c>
-      <c r="B70" t="s">
-        <v>90</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D70" t="s">
-        <v>81</v>
-      </c>
-      <c r="E70" t="s">
-        <v>10</v>
-      </c>
-      <c r="F70" t="s">
-        <v>10</v>
-      </c>
-      <c r="G70" t="s">
-        <v>69</v>
-      </c>
-      <c r="H70" t="s">
-        <v>11</v>
-      </c>
-      <c r="I70" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J70" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>

</xml_diff>

<commit_message>
Actualización de portadas al 7 de abril de 2026
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E49C8A-4C8F-4A3E-8428-B291305230CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAC76A32-E250-4E9A-9715-E4C938BAC0BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="201">
   <si>
     <t>Fecha</t>
   </si>
@@ -297,268 +297,349 @@
     <t>Reforma De Ley</t>
   </si>
   <si>
-    <t>Mundial De Futbol</t>
-  </si>
-  <si>
     <t>Policía municipal</t>
   </si>
   <si>
-    <t>Entrega De Apoyos</t>
-  </si>
-  <si>
     <t>Sipdus</t>
   </si>
   <si>
     <t>El Sol de Hidalgo</t>
   </si>
   <si>
-    <t>Deja alta movilidad, segundo fin de semana vacacional</t>
-  </si>
-  <si>
-    <t>La CURP biométrica no desplaza a la credencial para votar: INE</t>
-  </si>
-  <si>
-    <t>CURP Biométrica</t>
-  </si>
-  <si>
-    <t>Hidalgo registra 286 robos de vehículos</t>
-  </si>
-  <si>
-    <t>Incidencia Delictiva</t>
-  </si>
-  <si>
-    <t>Reduce el paso de migrantes</t>
-  </si>
-  <si>
-    <t>Migrantes</t>
-  </si>
-  <si>
-    <t>Laura y Rubén son ganadores de Santiago</t>
-  </si>
-  <si>
-    <t>Festival Gastronómico</t>
-  </si>
-  <si>
-    <t>Instalan iluminación en El Salitre, Tula</t>
-  </si>
-  <si>
-    <t>Luminarias</t>
-  </si>
-  <si>
-    <t>Gastará el IEEH más de 6 mdp en salarios de consejeros</t>
-  </si>
-  <si>
     <t>Presupuesto IEEH</t>
   </si>
   <si>
-    <t>Manjares y Pulque</t>
-  </si>
-  <si>
-    <t>Comercio local se alista para el mundial</t>
-  </si>
-  <si>
-    <t>Mayelli Rosquero pierde su título</t>
-  </si>
-  <si>
-    <t>Llueven pétalos en plena misa</t>
-  </si>
-  <si>
-    <t>Deria de goles en el Hidalgo</t>
-  </si>
-  <si>
-    <t>ROSQUERO CAYÓ ENTRE POLÉMICA</t>
-  </si>
-  <si>
-    <t>SE REGISTRARON 33 HOMICIDIOS EN TRES MESES</t>
-  </si>
-  <si>
-    <t>Homicidios</t>
-  </si>
-  <si>
-    <t>Reviven la pasión de Cristo en los barrios</t>
-  </si>
-  <si>
-    <t>PIDEN AL CONGRESO  PROBAR REPOSICIÓN DE CONSULTA A LOS PUEBLOS INDÍGENAS</t>
-  </si>
-  <si>
-    <t>Consulta Indígena</t>
-  </si>
-  <si>
-    <t>PLANTEAN ACTUALIZAR  LA CONSTITUCIÓN  POLÍTICA ESTATAL EN  LENGUAS ORIGINARIAS</t>
-  </si>
-  <si>
-    <t>GLMorena</t>
-  </si>
-  <si>
     <t>Iniciativa</t>
   </si>
   <si>
-    <t>Domingo de resurrección da fin a la Semana Santa</t>
-  </si>
-  <si>
-    <t>Golpea estado al narcomenudeo meidante extinción de dominio</t>
-  </si>
-  <si>
-    <t>Extinción de dominio</t>
-  </si>
-  <si>
-    <t>Violencia escolar. La Secretaría de Educación activa el registro de casos</t>
-  </si>
-  <si>
-    <t>Violencia Escolar</t>
-  </si>
-  <si>
-    <t>Detienen a tres por robo, violencia y drogas</t>
-  </si>
-  <si>
-    <t>Combate a la delincuencia</t>
-  </si>
-  <si>
-    <t>Celebración. Tradicional lluvia de pétalos en Mineral del Chico</t>
-  </si>
-  <si>
-    <t>Reconocen un atraso en 20 obras de restauración</t>
-  </si>
-  <si>
-    <t>Obra inconclusa</t>
-  </si>
-  <si>
-    <t>Registran afluencia moderada en los días santos</t>
-  </si>
-  <si>
-    <t>Prevén cierres carreteros por protesta de transportistas</t>
-  </si>
-  <si>
     <t>Cierre Carretero</t>
   </si>
   <si>
-    <t>Sheinbaum supera a Fox, Calderón, Peña y AMLO</t>
-  </si>
-  <si>
-    <t>Dilema de la IA: más crecimiento, menos empleos</t>
-  </si>
-  <si>
-    <t>Coparmex prevé alza de costos por conflictos políticos</t>
-  </si>
-  <si>
-    <t>Proyectan parque solar fotovoltaico para Huichapan</t>
-  </si>
-  <si>
     <t>Parque Fotovoltaico</t>
   </si>
   <si>
-    <t>Inclumplimientos del gobierno dan pie a bloqueo carretero hoy</t>
-  </si>
-  <si>
     <t>Bloqueo Carretero</t>
   </si>
   <si>
-    <t>Lluvia de pétalos reúne a miles de visitantes en El Chico</t>
-  </si>
-  <si>
-    <t>Hablar del active shooter no es importar miedos ajenos ni copiar debates  extranjeros, es reconocer, con serenidad y firmeza, que las amenazas  cambian, que los entornos escolares no son inmunes y que la seguridad  contemporánea exige anticipación, no solo reacción”.</t>
-  </si>
-  <si>
-    <t>Brindan apoyo vial a turistas que visitaron al estado</t>
-  </si>
-  <si>
-    <t>Asesinan a mano armada a un hombre en tianguis de Cuautepec</t>
-  </si>
-  <si>
-    <t>Ejecuciones</t>
-  </si>
-  <si>
-    <t>Va por Hidalgo alumna huejutlense en concurso nacional de fotografía</t>
-  </si>
-  <si>
-    <t>Concurso Nacional</t>
-  </si>
-  <si>
-    <t>Mediante viacrucis piden por la paz</t>
-  </si>
-  <si>
-    <t>Santiago de Anaya celebra su riqueza culinaria con la XLV muestra Gastronómica</t>
-  </si>
-  <si>
-    <t>cul</t>
-  </si>
-  <si>
-    <t>Entregan apoyos económicos y agrícolas en Tlanchinol</t>
-  </si>
-  <si>
-    <t>Turistas y familias de la región disfrutaron la mega alberca</t>
-  </si>
-  <si>
-    <t>5 lesionnados tras volcar camioneta en el Arco Norte</t>
-  </si>
-  <si>
     <t>Cintillo</t>
   </si>
   <si>
-    <t>Accidente Carretero</t>
-  </si>
-  <si>
-    <t>Policías de Pachuca mantienen operativo de Semana Santa</t>
-  </si>
-  <si>
-    <t>Concluye con éxito la fiesta de Semana Santa en Ajacuba</t>
-  </si>
-  <si>
-    <t>Voluntarios y autoridades atienen incendio forestal en Jacala</t>
-  </si>
-  <si>
-    <t>Control de incendios</t>
-  </si>
-  <si>
-    <t>Todo un éxito la 2a Feria del Helado Artesanal</t>
-  </si>
-  <si>
-    <t>5 lesionados tras volcar camioneta en el Arco Norte</t>
-  </si>
-  <si>
-    <t>Lluvias, viento y bajas temperaturas, pronóstico para las próximas horas</t>
-  </si>
-  <si>
-    <t>PC</t>
-  </si>
-  <si>
     <t>Alerta Meteorológica</t>
   </si>
   <si>
     <t>Usa el puente peatonal</t>
   </si>
   <si>
-    <t>Se hacían pasar por funcionarios para vender viajes VIP en Hidalgo: 4 detenidos</t>
-  </si>
-  <si>
-    <t>Combate a la extorsión</t>
-  </si>
-  <si>
-    <t>Develan Tuzas palco en homenaje a Karla Nieto</t>
-  </si>
-  <si>
-    <t>Pachuca mantiene atención en la capital y apoya monitoreo en puntos turísticos</t>
-  </si>
-  <si>
-    <t>Amagan transportistas con bloqueos en México-Pachuca y otras vías este lunes</t>
-  </si>
-  <si>
-    <t>Concluyó la Muestra Gastronómica de Santiago de Anaya</t>
-  </si>
-  <si>
-    <t>¡Cristo vive!</t>
-  </si>
-  <si>
-    <t>De cinco balazos, ejecutaron al "Comandante" en su casa</t>
-  </si>
-  <si>
-    <t>¿Qué diría el maestro, si al regresar encontrara lo que hemos hecho con el mundo?</t>
-  </si>
-  <si>
-    <t>Transportistas y campesinos alistan bloqueos en carreteras</t>
-  </si>
-  <si>
-    <t>Publican primera foto de cara oculta de la luna</t>
+    <t>Mascotas, en riesgo de sufrir golpe de calor</t>
+  </si>
+  <si>
+    <t>Barrenador, en 36 de 84 municipios</t>
+  </si>
+  <si>
+    <t>Gusano barrenador</t>
+  </si>
+  <si>
+    <t>Buscan reconocimiento a Procesión del silencio</t>
+  </si>
+  <si>
+    <t>llamao</t>
+  </si>
+  <si>
+    <t>Hidalgo, con mil 686 personas sin localizar</t>
+  </si>
+  <si>
+    <t>CBPEH</t>
+  </si>
+  <si>
+    <t>Personas desaparecidas</t>
+  </si>
+  <si>
+    <t>No hubo megaparo en vías estatales</t>
+  </si>
+  <si>
+    <t>Son los humanos más lejos han llegado</t>
+  </si>
+  <si>
+    <t>Crearán comité para atender casos de gusano barrenador</t>
+  </si>
+  <si>
+    <t>Planean proyecto solar en Huichapan</t>
+  </si>
+  <si>
+    <t>Casa de la Mujer Indígena</t>
+  </si>
+  <si>
+    <t>Cedspi</t>
+  </si>
+  <si>
+    <t>Simey Olvera visita a Mario Delgado</t>
+  </si>
+  <si>
+    <t>Simey</t>
+  </si>
+  <si>
+    <t>Reunión con funcionario federal</t>
+  </si>
+  <si>
+    <t>Más de 4 mil apoyos en vacaciones</t>
+  </si>
+  <si>
+    <t>Reunión Gabinete De Seguridad</t>
+  </si>
+  <si>
+    <t>UN ARRANQUE  LA EFECTIVIDAD  PROMETEDOR</t>
+  </si>
+  <si>
+    <t>CHOQUE DE  GIGANTES</t>
+  </si>
+  <si>
+    <t>Alcalde gana $48 mil con la prepa trunca</t>
+  </si>
+  <si>
+    <t>Alcalde</t>
+  </si>
+  <si>
+    <t>Perfil académico</t>
+  </si>
+  <si>
+    <t>ESTRENARÁ EL  TUZOBÚS 140  UNIDADES EN MAYO: SEMOT</t>
+  </si>
+  <si>
+    <t>Sitmah</t>
+  </si>
+  <si>
+    <t>Modernización Tuzobús</t>
+  </si>
+  <si>
+    <t>Avanza obra para reubicar ambulantes</t>
+  </si>
+  <si>
+    <t>Ambulantaje</t>
+  </si>
+  <si>
+    <t>Municipios deben vigilar los rellenos sanitarios</t>
+  </si>
+  <si>
+    <t>Relleno Sanitario</t>
+  </si>
+  <si>
+    <t>Hidalgo, con 203 casos de barrenador, señala Sader</t>
+  </si>
+  <si>
+    <t>Presentan denuncias por fraude en ofertas de empleo para EU</t>
+  </si>
+  <si>
+    <t>Fraude</t>
+  </si>
+  <si>
+    <t>Autoridades reconocen que falta mano de obra calificada</t>
+  </si>
+  <si>
+    <t>Mano de obra calificada</t>
+  </si>
+  <si>
+    <t>Más de 30 mil personas tienen acceso a apoyos</t>
+  </si>
+  <si>
+    <t>Huracán Priscilla</t>
+  </si>
+  <si>
+    <t>Café de la sierra, fruto de calidad</t>
+  </si>
+  <si>
+    <t>Caficultura</t>
+  </si>
+  <si>
+    <t>Sheinbaum: desdeñó la ONU todo avance sobre desaparecidos</t>
+  </si>
+  <si>
+    <t>Artemis II. Comienza el retorno luego de la caminata más larga por el espacio</t>
+  </si>
+  <si>
+    <t>Temas internacionales</t>
+  </si>
+  <si>
+    <t>Irán puede desaparecer esta noche"": Trump</t>
+  </si>
+  <si>
+    <t>UIF congelará cuentas sin contar con orden judicial</t>
+  </si>
+  <si>
+    <t>Niegan en IEEH alza en salarios: ""son los mismos desde 2019""</t>
+  </si>
+  <si>
+    <t>Sube a 229 el número de casos de gusano barrenador</t>
+  </si>
+  <si>
+    <t>Construirán 50 ollas de captación contra la sequía</t>
+  </si>
+  <si>
+    <t>Captación De Agua</t>
+  </si>
+  <si>
+    <t>Gusano barrenador del ganado afecta a 36 municipios</t>
+  </si>
+  <si>
+    <t>Se desinfla paro de transportistas</t>
+  </si>
+  <si>
+    <t>Invierten 64 millones de pesos en dos casas de la Mujer Indígena</t>
+  </si>
+  <si>
+    <t>El gusano barrenador no solo afecta al ganado. Expone debilidades en la  cadena de control, en la prevención y en la respuesta. La falta de supervisión  en la movilidad, el abandono animal y la atención tardía de lesiones generan  condiciones que facilitan su permanencia”.</t>
+  </si>
+  <si>
+    <t>Instruye Menchaca reforzar seguridad para concluir periodo vacacional</t>
+  </si>
+  <si>
+    <t>Presenta Secretaría del trabajo cinco denuncias por ofertas laborales fraudulentas</t>
+  </si>
+  <si>
+    <t>Buscan incluir participación de expertos en la construcción de dictámenes</t>
+  </si>
+  <si>
+    <t>Defiende Crespo acciones del gobierno estatal y destaca avances contra la pobreza</t>
+  </si>
+  <si>
+    <t>Bloquearon la carretera Huejutla-Orizatlán</t>
+  </si>
+  <si>
+    <t>Frente frío 43 afecta a la Huasteca</t>
+  </si>
+  <si>
+    <t>Hidalgo fortalece desarrollo económico, empleo y sanidad agropecuaria</t>
+  </si>
+  <si>
+    <t>Mañanera de Hidalgo</t>
+  </si>
+  <si>
+    <t>Refuerzan coordinación en seguridad</t>
+  </si>
+  <si>
+    <t>Coordinación Interinstitucional</t>
+  </si>
+  <si>
+    <t>Lluvias ocasionron deslaves en Coatzonco y Acatépec</t>
+  </si>
+  <si>
+    <t>Afectaciones Por Lluvias</t>
+  </si>
+  <si>
+    <t>Cercanía y diálogos fortalecen el bienestar en comunidades: San Román</t>
+  </si>
+  <si>
+    <t>Effetá</t>
+  </si>
+  <si>
+    <t>Preparan megaproyecto solar en Huichapan</t>
+  </si>
+  <si>
+    <t>Semana Santa: Mueren 9 en carreteras</t>
+  </si>
+  <si>
+    <t>Exalcalde de San Salvador tramita amparo ante posible orden de aprehensión</t>
+  </si>
+  <si>
+    <t>Exalcalde</t>
+  </si>
+  <si>
+    <t>Amparo</t>
+  </si>
+  <si>
+    <t>Aclara Ixmiquilpan: no hay tres desaparecidos, solo un no localizado</t>
+  </si>
+  <si>
+    <t>Suman 229 casos de gusano barrenador</t>
+  </si>
+  <si>
+    <t>Te prometen 30 dólares por hora... ¡Pero es estafa!</t>
+  </si>
+  <si>
+    <t>Alerta De Fraude</t>
+  </si>
+  <si>
+    <t>El toreo legislativo</t>
+  </si>
+  <si>
+    <t>GLPVEM</t>
+  </si>
+  <si>
+    <t>Tauromaquia</t>
+  </si>
+  <si>
+    <t>Los retos de Moronatti en Pachuca</t>
+  </si>
+  <si>
+    <t>Mando Coordinado</t>
+  </si>
+  <si>
+    <t>IMSS emite recomendaciones para prevenir deshidratación en menores</t>
+  </si>
+  <si>
+    <t>IMSS</t>
+  </si>
+  <si>
+    <t>Prevención De Enfermedades</t>
+  </si>
+  <si>
+    <t>Gabinete de Seguridad refuerza operativo para concluir periodo vacacional</t>
+  </si>
+  <si>
+    <t>Hidalgo fortalece acciones integrales para el bienestar, desarrollo ecoómico, empleo y sanidad agropecuaria</t>
+  </si>
+  <si>
+    <t>Convierte Sipdus terracería en camino digno en Omitlán de Juárez</t>
+  </si>
+  <si>
+    <t>Carretera artesanal</t>
+  </si>
+  <si>
+    <t>El Inhide invierte todos sus recursos para que más personas practiquen deporte en mejores condiciones</t>
+  </si>
+  <si>
+    <t>Inhide</t>
+  </si>
+  <si>
+    <t>Impulso al deporte</t>
+  </si>
+  <si>
+    <t>publicidad gubernamental</t>
+  </si>
+  <si>
+    <t>Para mayo, las nuevas unidades del Tuzobús</t>
+  </si>
+  <si>
+    <t>Gabinete de seguridad refuerza operativo para concluir periodo vacacional</t>
+  </si>
+  <si>
+    <t>Detectan en Hidalgo vacantes fraudulentas para laborar en EU</t>
+  </si>
+  <si>
+    <t>Glorieta 24 Horas, con nuevas adecuaciones para movilidad</t>
+  </si>
+  <si>
+    <t>Glorieta 24 Horas</t>
+  </si>
+  <si>
+    <t>Hidalgo fortalece acciones integrales para el Bienestar, Desarrollo Económico, empleo y sanidad agropecuaria</t>
+  </si>
+  <si>
+    <t>Afecta gusano barrenador a 36 municipios</t>
+  </si>
+  <si>
+    <t>Identifican a nueve mineros secuestrados en Sinaloa</t>
+  </si>
+  <si>
+    <t>Un incendio consume centro de reciclaje en Emiliano Zapata</t>
+  </si>
+  <si>
+    <t>Incendio de basurero</t>
+  </si>
+  <si>
+    <t>Pasada la Semana Santa, resulta que en asuntos más terrenales, la pelea por candidaturas de Morena ya está en su apogeo y no dude usted que un Barrabás, con todo y cadenas, es decir, brazalete en pierna, andará de campaña</t>
+  </si>
+  <si>
+    <t>Candidaturas</t>
   </si>
 </sst>
 </file>
@@ -805,8 +886,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J59" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J59" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J68" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J68" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1172,7 +1253,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J59"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1221,13 +1302,13 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
@@ -1239,7 +1320,7 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
@@ -1253,170 +1334,170 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>101</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>103</v>
       </c>
       <c r="G5" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="H5" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="D6" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>99</v>
+        <v>91</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>101</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
         <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1425,62 +1506,62 @@
     </row>
     <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B8" t="s">
         <v>70</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D8" t="s">
         <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="F8" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H8" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B9" t="s">
         <v>70</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D9" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>31</v>
+        <v>58</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
+        <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="H9" t="s">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1493,66 +1574,66 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B10" t="s">
         <v>70</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="G10" t="s">
-        <v>86</v>
+        <v>109</v>
       </c>
       <c r="H10" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B11" t="s">
         <v>70</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>10</v>
+        <v>65</v>
       </c>
       <c r="F11" t="s">
-        <v>10</v>
+        <v>112</v>
       </c>
       <c r="G11" t="s">
-        <v>76</v>
+        <v>113</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Sucesión gubernamental</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1561,47 +1642,47 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B12" t="s">
         <v>70</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G12" t="s">
-        <v>81</v>
+        <v>115</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B13" t="s">
         <v>73</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1629,13 +1710,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B14" t="s">
         <v>73</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -1663,195 +1744,195 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B15" t="s">
         <v>73</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="D15" t="s">
         <v>13</v>
       </c>
       <c r="E15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>119</v>
       </c>
       <c r="G15" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="H15" t="s">
         <v>16</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B16" t="s">
         <v>73</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="F16" t="s">
-        <v>10</v>
+        <v>122</v>
       </c>
       <c r="G16" t="s">
-        <v>81</v>
+        <v>123</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B17" t="s">
         <v>73</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="D17" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E17" t="s">
-        <v>10</v>
+        <v>87</v>
       </c>
       <c r="F17" t="s">
-        <v>10</v>
+        <v>87</v>
       </c>
       <c r="G17" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B18" t="s">
         <v>73</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="F18" t="s">
-        <v>116</v>
+        <v>2</v>
       </c>
       <c r="G18" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B19" t="s">
         <v>73</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="F19" t="s">
-        <v>10</v>
+        <v>57</v>
       </c>
       <c r="G19" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H19" t="s">
         <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B20" t="s">
         <v>77</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="D20" t="s">
         <v>13</v>
       </c>
       <c r="E20" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="F20" t="s">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="G20" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="H20" t="s">
         <v>26</v>
@@ -1867,28 +1948,28 @@
     </row>
     <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B21" t="s">
         <v>77</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="F21" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="G21" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="H21" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1901,28 +1982,28 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B22" t="s">
         <v>77</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="F22" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G22" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="H22" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1933,120 +2014,120 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B23" t="s">
         <v>77</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="D23" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="F23" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="G23" t="s">
-        <v>81</v>
+        <v>136</v>
       </c>
       <c r="H23" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B24" t="s">
         <v>77</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>89</v>
+        <v>14</v>
       </c>
       <c r="F24" t="s">
-        <v>89</v>
+        <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="H24" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B25" t="s">
         <v>77</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>81</v>
+        <v>139</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B26" t="s">
         <v>77</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -2055,10 +2136,10 @@
         <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="H26" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2071,13 +2152,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B27" t="s">
         <v>77</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -2103,30 +2184,30 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B28" t="s">
         <v>77</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="F28" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="G28" t="s">
-        <v>69</v>
+        <v>89</v>
       </c>
       <c r="H28" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2139,59 +2220,59 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B29" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F29" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G29" t="s">
-        <v>69</v>
+        <v>99</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B30" t="s">
         <v>71</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="D30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G30" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
@@ -2205,166 +2286,166 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B31" t="s">
         <v>71</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="D31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="F31" t="s">
-        <v>14</v>
+        <v>57</v>
       </c>
       <c r="G31" t="s">
-        <v>137</v>
+        <v>99</v>
       </c>
       <c r="H31" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B32" t="s">
         <v>71</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="D32" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F32" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B33" t="s">
         <v>71</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="D33" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E33" t="s">
-        <v>10</v>
+        <v>51</v>
       </c>
       <c r="F33" t="s">
-        <v>10</v>
+        <v>110</v>
       </c>
       <c r="G33" t="s">
-        <v>69</v>
+        <v>109</v>
       </c>
       <c r="H33" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="90" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="D34" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>17</v>
+        <v>57</v>
       </c>
       <c r="F34" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="G34" t="s">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="H34" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B35" t="s">
         <v>72</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F35" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="G35" t="s">
-        <v>142</v>
+        <v>115</v>
       </c>
       <c r="H35" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2372,30 +2453,30 @@
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B36" t="s">
         <v>72</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>28</v>
+        <v>60</v>
       </c>
       <c r="F36" t="s">
-        <v>28</v>
+        <v>2</v>
       </c>
       <c r="G36" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
@@ -2409,27 +2490,27 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B37" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="D37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F37" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="G37" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
@@ -2445,183 +2526,183 @@
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B38" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F38" t="s">
-        <v>147</v>
+        <v>10</v>
       </c>
       <c r="G38" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B39" t="s">
         <v>84</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="D39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="F39" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G39" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H39" t="s">
         <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B40" t="s">
         <v>84</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G40" t="s">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B41" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="D41" t="s">
-        <v>151</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="F41" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="G41" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H41" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="F42" t="s">
-        <v>87</v>
+        <v>23</v>
       </c>
       <c r="G42" t="s">
-        <v>81</v>
+        <v>159</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B43" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
@@ -2633,7 +2714,7 @@
         <v>17</v>
       </c>
       <c r="G43" t="s">
-        <v>81</v>
+        <v>161</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
@@ -2649,152 +2730,152 @@
     </row>
     <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B44" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="G44" t="s">
-        <v>156</v>
+        <v>69</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B45" t="s">
-        <v>82</v>
+        <v>163</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>17</v>
+        <v>58</v>
       </c>
       <c r="F45" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G45" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B46" t="s">
-        <v>82</v>
+        <v>163</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F46" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="G46" t="s">
-        <v>152</v>
+        <v>81</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B47" t="s">
-        <v>82</v>
+        <v>163</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D47" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E47" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="G47" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="H47" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B48" t="s">
-        <v>82</v>
+        <v>163</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D48" t="s">
-        <v>78</v>
+        <v>12</v>
       </c>
       <c r="E48" t="s">
         <v>17</v>
@@ -2803,7 +2884,7 @@
         <v>17</v>
       </c>
       <c r="G48" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
@@ -2817,27 +2898,27 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B49" t="s">
-        <v>29</v>
+        <v>163</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="D49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="F49" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
       <c r="G49" t="s">
-        <v>164</v>
+        <v>99</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
@@ -2853,100 +2934,100 @@
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B50" t="s">
-        <v>29</v>
+        <v>163</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="F50" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G50" t="s">
-        <v>76</v>
+        <v>172</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J50" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A51" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B51" t="s">
+        <v>163</v>
+      </c>
+      <c r="C51" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>37</v>
+      </c>
+      <c r="F51" t="s">
+        <v>174</v>
+      </c>
+      <c r="G51" t="s">
+        <v>175</v>
+      </c>
+      <c r="H51" t="s">
+        <v>16</v>
+      </c>
+      <c r="I51" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J50" t="str">
+      <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A51" s="5">
-        <v>46118</v>
-      </c>
-      <c r="B51" t="s">
-        <v>29</v>
-      </c>
-      <c r="C51" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="D51" t="s">
-        <v>12</v>
-      </c>
-      <c r="E51" t="s">
-        <v>23</v>
-      </c>
-      <c r="F51" t="s">
-        <v>23</v>
-      </c>
-      <c r="G51" t="s">
-        <v>81</v>
-      </c>
-      <c r="H51" t="s">
-        <v>11</v>
-      </c>
-      <c r="I51" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J51" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B52" t="s">
-        <v>29</v>
+        <v>163</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F52" t="s">
-        <v>14</v>
+        <v>86</v>
       </c>
       <c r="G52" t="s">
-        <v>137</v>
+        <v>177</v>
       </c>
       <c r="H52" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2955,130 +3036,130 @@
     </row>
     <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B53" t="s">
-        <v>29</v>
+        <v>82</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="D53" t="s">
-        <v>12</v>
+        <v>94</v>
       </c>
       <c r="E53" t="s">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="F53" t="s">
-        <v>31</v>
+        <v>179</v>
       </c>
       <c r="G53" t="s">
-        <v>99</v>
+        <v>180</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B54" t="s">
+        <v>82</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D54" t="s">
+        <v>13</v>
+      </c>
+      <c r="E54" t="s">
+        <v>25</v>
+      </c>
+      <c r="F54" t="s">
+        <v>25</v>
+      </c>
+      <c r="G54" t="s">
+        <v>115</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+      <c r="I54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J53" t="str">
+      <c r="J54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A55" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B55" t="s">
+        <v>82</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>36</v>
+      </c>
+      <c r="F55" t="s">
+        <v>36</v>
+      </c>
+      <c r="G55" t="s">
+        <v>157</v>
+      </c>
+      <c r="H55" t="s">
+        <v>26</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A54" s="5">
-        <v>46118</v>
-      </c>
-      <c r="B54" t="s">
-        <v>29</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="D54" t="s">
-        <v>78</v>
-      </c>
-      <c r="E54" t="s">
-        <v>17</v>
-      </c>
-      <c r="F54" t="s">
-        <v>17</v>
-      </c>
-      <c r="G54" t="s">
-        <v>80</v>
-      </c>
-      <c r="H54" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" s="5">
-        <v>46118</v>
-      </c>
-      <c r="B55" t="s">
-        <v>83</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="D55" t="s">
-        <v>13</v>
-      </c>
-      <c r="E55" t="s">
-        <v>10</v>
-      </c>
-      <c r="F55" t="s">
-        <v>10</v>
-      </c>
-      <c r="G55" t="s">
-        <v>81</v>
-      </c>
-      <c r="H55" t="s">
-        <v>11</v>
-      </c>
-      <c r="I55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B56" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="F56" t="s">
-        <v>23</v>
+        <v>87</v>
       </c>
       <c r="G56" t="s">
-        <v>142</v>
+        <v>184</v>
       </c>
       <c r="H56" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3091,66 +3172,66 @@
     </row>
     <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B57" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>171</v>
+        <v>185</v>
       </c>
       <c r="D57" t="s">
-        <v>79</v>
+        <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="F57" t="s">
-        <v>10</v>
+        <v>186</v>
       </c>
       <c r="G57" t="s">
-        <v>69</v>
+        <v>187</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B58" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>172</v>
+        <v>96</v>
       </c>
       <c r="D58" t="s">
-        <v>12</v>
+        <v>78</v>
       </c>
       <c r="E58" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F58" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G58" t="s">
-        <v>137</v>
+        <v>188</v>
       </c>
       <c r="H58" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3159,34 +3240,340 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
-        <v>46118</v>
+        <v>46119</v>
       </c>
       <c r="B59" t="s">
+        <v>29</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D59" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" t="s">
+        <v>30</v>
+      </c>
+      <c r="F59" t="s">
+        <v>122</v>
+      </c>
+      <c r="G59" t="s">
+        <v>123</v>
+      </c>
+      <c r="H59" t="s">
+        <v>11</v>
+      </c>
+      <c r="I59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A60" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B60" t="s">
+        <v>29</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+      <c r="E60" t="s">
+        <v>25</v>
+      </c>
+      <c r="F60" t="s">
+        <v>25</v>
+      </c>
+      <c r="G60" t="s">
+        <v>115</v>
+      </c>
+      <c r="H60" t="s">
+        <v>11</v>
+      </c>
+      <c r="I60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A61" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B61" t="s">
+        <v>29</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" t="s">
+        <v>60</v>
+      </c>
+      <c r="F61" t="s">
+        <v>2</v>
+      </c>
+      <c r="G61" t="s">
+        <v>172</v>
+      </c>
+      <c r="H61" t="s">
+        <v>11</v>
+      </c>
+      <c r="I61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A62" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B62" t="s">
+        <v>29</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>87</v>
+      </c>
+      <c r="F62" t="s">
+        <v>87</v>
+      </c>
+      <c r="G62" t="s">
+        <v>193</v>
+      </c>
+      <c r="H62" t="s">
+        <v>11</v>
+      </c>
+      <c r="I62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B63" t="s">
+        <v>29</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>36</v>
+      </c>
+      <c r="F63" t="s">
+        <v>36</v>
+      </c>
+      <c r="G63" t="s">
+        <v>157</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+      <c r="I63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B64" t="s">
+        <v>29</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D64" t="s">
+        <v>78</v>
+      </c>
+      <c r="E64" t="s">
+        <v>17</v>
+      </c>
+      <c r="F64" t="s">
+        <v>17</v>
+      </c>
+      <c r="G64" t="s">
+        <v>80</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B65" t="s">
         <v>83</v>
       </c>
-      <c r="C59" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D59" t="s">
-        <v>12</v>
-      </c>
-      <c r="E59" t="s">
-        <v>10</v>
-      </c>
-      <c r="F59" t="s">
-        <v>10</v>
-      </c>
-      <c r="G59" t="s">
-        <v>69</v>
-      </c>
-      <c r="H59" t="s">
-        <v>11</v>
-      </c>
-      <c r="I59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J59" t="str">
+      <c r="C65" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D65" t="s">
+        <v>13</v>
+      </c>
+      <c r="E65" t="s">
+        <v>57</v>
+      </c>
+      <c r="F65" t="s">
+        <v>57</v>
+      </c>
+      <c r="G65" t="s">
+        <v>99</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A66" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B66" t="s">
+        <v>83</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>14</v>
+      </c>
+      <c r="F66" t="s">
+        <v>14</v>
+      </c>
+      <c r="G66" t="s">
+        <v>104</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A67" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B67" t="s">
+        <v>83</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>17</v>
+      </c>
+      <c r="F67" t="s">
+        <v>17</v>
+      </c>
+      <c r="G67" t="s">
+        <v>198</v>
+      </c>
+      <c r="H67" t="s">
+        <v>16</v>
+      </c>
+      <c r="I67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A68" s="5">
+        <v>46119</v>
+      </c>
+      <c r="B68" t="s">
+        <v>83</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="D68" t="s">
+        <v>79</v>
+      </c>
+      <c r="E68" t="s">
+        <v>19</v>
+      </c>
+      <c r="F68" t="s">
+        <v>19</v>
+      </c>
+      <c r="G68" t="s">
+        <v>200</v>
+      </c>
+      <c r="H68" t="s">
+        <v>16</v>
+      </c>
+      <c r="I68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J68" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>

</xml_diff>

<commit_message>
Reporte 15 de abril
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8A07F4-2FF5-4E6D-8CC8-25E35773521E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{262BA2E7-F8F8-4A83-8875-527A909B9A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="194">
   <si>
     <t>Fecha</t>
   </si>
@@ -252,9 +252,6 @@
     <t>Síntesis</t>
   </si>
   <si>
-    <t>Criterio</t>
-  </si>
-  <si>
     <t>Nivel</t>
   </si>
   <si>
@@ -288,9 +285,6 @@
     <t>Effetá</t>
   </si>
   <si>
-    <t>Tauromaquia</t>
-  </si>
-  <si>
     <t>Semana Santa</t>
   </si>
   <si>
@@ -300,277 +294,331 @@
     <t>Temas internacionales</t>
   </si>
   <si>
-    <t>Regreso A Clases</t>
-  </si>
-  <si>
-    <t>Denuncian anomalías en Casa del Adulto Mayor</t>
-  </si>
-  <si>
-    <t>Atención a adultos mayores</t>
-  </si>
-  <si>
-    <t>El tren Aifa avanza lento hacia su apertura</t>
-  </si>
-  <si>
-    <t>llanado</t>
-  </si>
-  <si>
     <t>SICT</t>
   </si>
   <si>
-    <t>Tren AIFA</t>
-  </si>
-  <si>
-    <t>Molestos por el uso de afores en obras</t>
-  </si>
-  <si>
-    <t>Inconformidad por obra</t>
-  </si>
-  <si>
-    <t>Registran más de diez deslaves tras lluvias</t>
-  </si>
-  <si>
-    <t>Afectaciones Por Lluvias</t>
-  </si>
-  <si>
-    <t>Alertan sobre zonas de alto riesgo en Tianguistengo</t>
-  </si>
-  <si>
     <t>PC</t>
   </si>
   <si>
     <t>Prevención De Riesgos</t>
   </si>
   <si>
-    <t>Desaparecen ambulancias en 7 municipios</t>
-  </si>
-  <si>
-    <t>Ambulancia dañada</t>
-  </si>
-  <si>
-    <t>CONCURSO DE HUAPANGO</t>
-  </si>
-  <si>
-    <t>Concurso De Huapango</t>
-  </si>
-  <si>
-    <t>Monitorean zonas de riesgo</t>
-  </si>
-  <si>
-    <t>Reunión Gabinete De Seguridad</t>
-  </si>
-  <si>
-    <t>En la vorágine internacional marcada por el conflicto bélico de Estados Unidos contra Irán, un caso se ha quedado perdido en una especie de limbo; se trata...</t>
-  </si>
-  <si>
-    <t>Abrirán nuevos bachilleratos</t>
-  </si>
-  <si>
-    <t>Bachillerato Nacional</t>
-  </si>
-  <si>
-    <t>TUZOS VS SU BESTIA</t>
-  </si>
-  <si>
-    <t>MADRID Y BARCELONA VAN POR LA REMONTADA</t>
-  </si>
-  <si>
-    <t>REPORTA SEPH SALDO BLANCO TRAS EL ASUETO</t>
-  </si>
-  <si>
-    <t>Busca el PAN retirar los bolardos del Tuzobús</t>
-  </si>
-  <si>
     <t>Carril confinado</t>
   </si>
   <si>
-    <t>COLAPSA PUENTE PROVISIONAL EN TIANGUISTENGO</t>
-  </si>
-  <si>
-    <t>Colapso de puente</t>
-  </si>
-  <si>
-    <t>Tienen siete municipios ambulancias sin ser usadas</t>
-  </si>
-  <si>
-    <t>Canasta básica alcanzó $1,062 en zona de Pachuca</t>
-  </si>
-  <si>
-    <t>Regularán las motos y scooters; habrá multas para incumplidos</t>
-  </si>
-  <si>
-    <t>Actualización de reglamentos</t>
-  </si>
-  <si>
-    <t>Detectan irregularidades en unidades municipales</t>
-  </si>
-  <si>
-    <t>EL robo de combustibles se registra en 41 localidades</t>
-  </si>
-  <si>
-    <t>Huachicol</t>
-  </si>
-  <si>
-    <t>Los restaurantes captan 260 mdp en Semana Santa</t>
-  </si>
-  <si>
-    <t>La industria eléctrica china, gran beneficiada por el conflicto</t>
-  </si>
-  <si>
-    <t>Vance ve avances para nuevo diálogo</t>
-  </si>
-  <si>
-    <t>José Revueltas: de los libros a la acción directa</t>
-  </si>
-  <si>
-    <t>Viene recorte franciscano para sostener gasolinas y los programas sociales</t>
-  </si>
-  <si>
-    <t>Austeridad</t>
-  </si>
-  <si>
-    <t>Claudia pedirá a Sánchez conocer la visión indígena</t>
-  </si>
-  <si>
-    <t>Jugará Gabriela Jáquez con Chicago en la WNBA</t>
-  </si>
-  <si>
-    <t>Construirán 26 bachilleratos con una inversión de más de 491 mdp</t>
-  </si>
-  <si>
-    <t>Mantiene activo gobierno estatal Comité de Emergencias por lluvias</t>
-  </si>
-  <si>
-    <t>Saldo blanco en escuelas durante vacaciones; sin robos y regreso normal: SEPH</t>
-  </si>
-  <si>
-    <t>Fallece motociclista en bulevar Las Torres; lo impactó un camión</t>
-  </si>
-  <si>
-    <t>Accidente Vial</t>
-  </si>
-  <si>
-    <t>Supervisan instalaciones del IMSS Bienestar en Atlapexco</t>
-  </si>
-  <si>
-    <t>Recorrido por instalaciones</t>
-  </si>
-  <si>
-    <t>Vacunación , principal herramienta preventiva contra el sarampión</t>
-  </si>
-  <si>
     <t>titular</t>
   </si>
   <si>
-    <t>Sarampión</t>
-  </si>
-  <si>
-    <t>Semarnat evalurrá sanitización de basurero Atlapexco</t>
-  </si>
-  <si>
-    <t>Medio ambiente</t>
-  </si>
-  <si>
-    <t>Supervisión sanitaria</t>
-  </si>
-  <si>
-    <t>Regresan a clases estudiantes, tras concluir periodo vacacional de semana santa</t>
-  </si>
-  <si>
-    <t>Regreso a clases en preescolar fortalece valores y compromiso educativo</t>
-  </si>
-  <si>
-    <t>La UCLA no tiene razón de ser</t>
-  </si>
-  <si>
-    <t>PAN pide regresar carril compartido del Tuzobús</t>
-  </si>
-  <si>
-    <t>Tren, el boom de Mineral de la Reforma</t>
-  </si>
-  <si>
-    <t>Tesoro ancestral, hallan arte rupestre de más de 4 mil años en zona del tren México Querétaro</t>
-  </si>
-  <si>
     <t>Tren México Querétaro</t>
   </si>
   <si>
-    <t>"No es pedir por pedir"</t>
-  </si>
-  <si>
-    <t>Presupuesto IEEH</t>
-  </si>
-  <si>
-    <t>Piden consulta por toros</t>
-  </si>
-  <si>
-    <t>Gobierno de Hidalgo previene e informa a familias ubicadas en zonas de riesgo</t>
-  </si>
-  <si>
-    <t>Hidalgo impulsa 115 becas para formar talento altamente especializado en 2026</t>
-  </si>
-  <si>
-    <t>Citnova</t>
-  </si>
-  <si>
-    <t>Impulso A La Ciencia</t>
-  </si>
-  <si>
-    <t>Comité de Emergencias está activo, monitorea Tianguistengo y Huehuetla ante precipitaciones</t>
-  </si>
-  <si>
-    <t>Construirán 26 bachilleratos para ampliar cobertura educativa en Hidalgo</t>
-  </si>
-  <si>
-    <t>Pachuca avanza en el ordenamiento urbano con participación ciudadana</t>
-  </si>
-  <si>
-    <t>Ordenamiento Territorial</t>
-  </si>
-  <si>
-    <t>Preside Cepeda Salas histórica toma de protesta a 4 mil 700 representantes sindicales en la Sección 15 del SNTE</t>
-  </si>
-  <si>
-    <t>Construirán 26 planteles de educación media superior en Hidalgo</t>
-  </si>
-  <si>
-    <t>Suben peaje de las autopistas del país; tres pesos la México-Pachuca</t>
-  </si>
-  <si>
-    <t>Aumento de peaje</t>
-  </si>
-  <si>
-    <t>Con 115 becas, impulsan formación de talento altamente especializado</t>
-  </si>
-  <si>
-    <t>Mantienen combate a saramipón mediante vacunación</t>
-  </si>
-  <si>
-    <t>Huehuetla, zona de riesgo por crecida de río</t>
-  </si>
-  <si>
-    <t>Desbordamiento de río</t>
-  </si>
-  <si>
-    <t>"No se cumplió con la meta de ingressos a restauranteros"</t>
-  </si>
-  <si>
-    <t>Primero el sarampión regresó como enfermedad masiva de alta peligrosidad, ahora también la tos ferina, todo por descuidar la vacunación</t>
-  </si>
-  <si>
     <t>Editorial</t>
   </si>
   <si>
-    <t>Vacunación</t>
-  </si>
-  <si>
-    <t>"Está bajo control el derrame en refinería Deer Park"</t>
-  </si>
-  <si>
     <t>Fuga de hidrocarburo</t>
   </si>
   <si>
-    <t>Construirán 26 nuevos planteles para educación media superior</t>
+    <t>Menos homicidios dolosos en Hidalgo</t>
+  </si>
+  <si>
+    <t>Incidencia Delictiva</t>
+  </si>
+  <si>
+    <t>Positiva</t>
+  </si>
+  <si>
+    <t>Limitan interacción por miedo a ser funados</t>
+  </si>
+  <si>
+    <t>Clausuran barranca de Metztitlán por explotación</t>
+  </si>
+  <si>
+    <t>Clausura de empresa contaminante</t>
+  </si>
+  <si>
+    <t>Ley de devolución excluye al Códice Borbónico</t>
+  </si>
+  <si>
+    <t>Códice borbónico</t>
+  </si>
+  <si>
+    <t>Aumento de pasaje no afectará economía</t>
+  </si>
+  <si>
+    <t>Aumento Tarifa De Transporte</t>
+  </si>
+  <si>
+    <t>Dan espacio al arte</t>
+  </si>
+  <si>
+    <t>Intervención Gráfica</t>
+  </si>
+  <si>
+    <t>Bajan homicidios dolosos: CSP</t>
+  </si>
+  <si>
+    <t>Planean regular salarios de alcaldes sin violar autonomía</t>
+  </si>
+  <si>
+    <t>GLMorena</t>
+  </si>
+  <si>
+    <t>Iniciativa</t>
+  </si>
+  <si>
+    <t>Avisan vía notario de riesgo a afectados</t>
+  </si>
+  <si>
+    <t>Reubicación de viviendas</t>
+  </si>
+  <si>
+    <t>Pensar la historia como una disciplina fundamental implica reconocer que el pasado no es un conjunto de fechas y nombres, sino un campo vivo de...</t>
+  </si>
+  <si>
+    <t>TUZOS BUSCARÁN LACOPA LA INMORTALIDAD</t>
+  </si>
+  <si>
+    <t>PSG Y EL ATLÉTICO  AVANZAN A SEMIS</t>
+  </si>
+  <si>
+    <t>NO ACEPTARÁN “CHANTAJE” POR EL NUEVO PASAJE</t>
+  </si>
+  <si>
+    <t>PROPONEN ELIMINAR  LAS SINDICATURAS DE  MINORÍA EN CABILDOS</t>
+  </si>
+  <si>
+    <t>ALCALDÍA Y  TIENDAS OXXO  REHABILITAN EL  JARDÍN DEL ARTE</t>
+  </si>
+  <si>
+    <t>Alcalde</t>
+  </si>
+  <si>
+    <t>Rehabilitación de espacios públicos</t>
+  </si>
+  <si>
+    <t>Hidalgo ingresó 1,235 millones de pesos en la Semana Santa</t>
+  </si>
+  <si>
+    <t>Esperan que Hospital General de Actopan funcione este año</t>
+  </si>
+  <si>
+    <t>Nuevo Hospital General</t>
+  </si>
+  <si>
+    <t>Crece el presupuesto de Pachuca; priorizan inversión en seguridad</t>
+  </si>
+  <si>
+    <t>Modificación Presupuestal</t>
+  </si>
+  <si>
+    <t>Preparan actividades para recibir  a los turistas</t>
+  </si>
+  <si>
+    <t>Mundial De Futbol</t>
+  </si>
+  <si>
+    <t>En Semana Santa estado recibe más de 1,235 mdp</t>
+  </si>
+  <si>
+    <t>Tuzobús no logra metas de viajes... ni de ingresos</t>
+  </si>
+  <si>
+    <t>Sitmah</t>
+  </si>
+  <si>
+    <t>Deficiencias Tuzobús</t>
+  </si>
+  <si>
+    <t>Hallan vestigios de más de 4 mil años; cambian trazo del tren</t>
+  </si>
+  <si>
+    <t>Julio Menchaca: habrá aumento en la tarifa, pero sin chantajes</t>
+  </si>
+  <si>
+    <t>Originario de Zimapán, el minero que sigue atrapado</t>
+  </si>
+  <si>
+    <t>Tratamientos para vivir más sin certificado científico</t>
+  </si>
+  <si>
+    <t>Magnicharters adeuda $150 millones a agencias y dueños se esfuman</t>
+  </si>
+  <si>
+    <t>Una fuente de electricidad al menos por familia en 2030</t>
+  </si>
+  <si>
+    <t>Energías renovables</t>
+  </si>
+  <si>
+    <t>Shock chino 2.0 con productos de alta tecnología</t>
+  </si>
+  <si>
+    <t>La Jornada Hidalgo</t>
+  </si>
+  <si>
+    <t>Nuevas tarifas del transporte estarán listas este mes: JMS</t>
+  </si>
+  <si>
+    <t>Municipios buscan contratar deuda tras daños por vaguada</t>
+  </si>
+  <si>
+    <t>Huracán Priscilla</t>
+  </si>
+  <si>
+    <t>Sheinbaum destaca caída de 45% en homicidios y escuela de Mandos</t>
+  </si>
+  <si>
+    <t>Lluvias arrastran hidrocarburo a Poza Rica y Coatzintla: Pemex</t>
+  </si>
+  <si>
+    <t>Pemex</t>
+  </si>
+  <si>
+    <t>Colaplsa barda de INFRA y destroza camioneta</t>
+  </si>
+  <si>
+    <t>La diferencia es que en San Luis Potosí el gobierno es ecologista y aquí  morenista y, por lo que se ha visto, el grupo en el poder no está dispuesto  a perder en las primeras elecciones los que les llevó tanto tiempo ganar”.</t>
+  </si>
+  <si>
+    <t>Alianzas Electorales</t>
+  </si>
+  <si>
+    <t>Exponen 15 hidalguenses su arte en Palacio de  Gobierno con “Hióki”</t>
+  </si>
+  <si>
+    <t>Pachuca rehabilita el Jardín del Arte con apoyo de la iniciativa privada</t>
+  </si>
+  <si>
+    <t>alcalde</t>
+  </si>
+  <si>
+    <t>Supera Hidalgo los 2.4 millones de visitantes en Semana Santa 2026</t>
+  </si>
+  <si>
+    <t>Aumento de tarifa del transporte  será “razonable” y podría definirse  este mes: Menchaca</t>
+  </si>
+  <si>
+    <t>Pide Napeoleón a productores no caer en pánico por gusano barrenador</t>
+  </si>
+  <si>
+    <t>Gusano barrenador</t>
+  </si>
+  <si>
+    <t>JULIO MENCHACA INAUGURA INTERVENCIÓN GRÁFICA 4.1 HlóKi</t>
+  </si>
+  <si>
+    <t>Productores apícolas piden certificación</t>
+  </si>
+  <si>
+    <t>Certificación</t>
+  </si>
+  <si>
+    <t>La reconstrucción de los puentes es con recurso federal: SICT</t>
+  </si>
+  <si>
+    <t>Reactivan ícono de Pachuca</t>
+  </si>
+  <si>
+    <t>El oficio político en tiempos de protagonismo</t>
+  </si>
+  <si>
+    <t>Labor destacada</t>
+  </si>
+  <si>
+    <t>Carril exclusivo del Tuzobús, decisión en beneficio de la mayoría: Menchaca</t>
+  </si>
+  <si>
+    <t>PAN acusa ""robo"" de militantes</t>
+  </si>
+  <si>
+    <t>Militancia Partidista</t>
+  </si>
+  <si>
+    <t>En abril, aumento al pasaje</t>
+  </si>
+  <si>
+    <t>¡Solo dos sanciones en 10 años!</t>
+  </si>
+  <si>
+    <t>Proespa</t>
+  </si>
+  <si>
+    <t>Maltrato animal</t>
+  </si>
+  <si>
+    <t>Hidalgo fortalece acciones para prevenir el embarazo en niñas y adolescentes</t>
+  </si>
+  <si>
+    <t>Coespo</t>
+  </si>
+  <si>
+    <t>Prevención De Embarazo Adolescente</t>
+  </si>
+  <si>
+    <t>Entregan en Tula calentadores del programa ""Energía para el Bienestar""</t>
+  </si>
+  <si>
+    <t>AEEH</t>
+  </si>
+  <si>
+    <t>Energía para el Bienestar</t>
+  </si>
+  <si>
+    <t>Iniciaron los trabajos de pavimentación asfáltica en Ignacio Zaragoza</t>
+  </si>
+  <si>
+    <t>Pavimentación</t>
+  </si>
+  <si>
+    <t>Como un "acto de reconstrucción", Julio Menchaca inaugura intervención gráfica 4.1</t>
+  </si>
+  <si>
+    <t>Jorge Reyes y Oxxo intervienen el Jardín del Arte para reactivar un espacio emblemático</t>
+  </si>
+  <si>
+    <t>Apropiación de espacios públicos</t>
+  </si>
+  <si>
+    <t>Rehabilitación de la calle Vía de los Reyes fortalece la conectividad en EI Daxthá, Actopan</t>
+  </si>
+  <si>
+    <t>Rehabilitación Vial</t>
+  </si>
+  <si>
+    <t>Natividad Castrejón abandera delegación hidalguense rumbo a la Olimpiada Nacional Conade</t>
+  </si>
+  <si>
+    <t>Justa Deportiva</t>
+  </si>
+  <si>
+    <t>Nueva tarifa de transporte, para este mes: Julio Menchaca</t>
+  </si>
+  <si>
+    <t>Abanderan delegación hidalguense rumbo a la Olimpiada Nacional</t>
+  </si>
+  <si>
+    <t>Participan 15 artistas en intervención gráfica 4.1 Hióki, en edificio de gobierno</t>
+  </si>
+  <si>
+    <t>Máquina del tiempo</t>
+  </si>
+  <si>
+    <t>Confirman incremento al pasaje del transporte público</t>
+  </si>
+  <si>
+    <t>Refuerzan atención y control del gusano barrenador</t>
+  </si>
+  <si>
+    <t>Denuncian entrega de bonos a regidores mediante apoyos</t>
+  </si>
+  <si>
+    <t>Entrega De Apoyos</t>
+  </si>
+  <si>
+    <t>Los homicidios cayeron un 41% en 18 meses con Sheinbaum</t>
+  </si>
+  <si>
+    <t>A pesar de que no han subido de precio las gasolinas, los demás productos básico se han elevado como cohetes, lo que obliga a la gente a comprar por medios kilos o medios litros</t>
   </si>
 </sst>
 </file>
@@ -817,8 +865,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J61" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J61" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J68" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J68" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1184,7 +1232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J61"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -1228,71 +1276,71 @@
         <v>8</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G2" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
-        <v>91</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>92</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>93</v>
+        <v>68</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1301,16 +1349,16 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E4" t="s">
         <v>14</v>
@@ -1319,10 +1367,10 @@
         <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="H4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1335,32 +1383,32 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1369,28 +1417,28 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>99</v>
+        <v>25</v>
       </c>
       <c r="G6" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H6" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1398,33 +1446,33 @@
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B7" t="s">
         <v>69</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="F7" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H7" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1437,149 +1485,149 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B8" t="s">
         <v>69</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="G8" t="s">
-        <v>104</v>
+        <v>94</v>
       </c>
       <c r="H8" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B9" t="s">
         <v>69</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>25</v>
+        <v>107</v>
       </c>
       <c r="G9" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="H9" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B10" t="s">
         <v>69</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>68</v>
+        <v>110</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B11" t="s">
         <v>69</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>109</v>
+        <v>68</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B12" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -1591,7 +1639,7 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
@@ -1607,13 +1655,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B13" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1625,7 +1673,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -1641,28 +1689,28 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B14" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="D14" t="s">
         <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="H14" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1670,52 +1718,52 @@
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="F15" t="s">
-        <v>48</v>
+        <v>107</v>
       </c>
       <c r="G15" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B16" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="D16" t="s">
         <v>9</v>
@@ -1724,13 +1772,13 @@
         <v>17</v>
       </c>
       <c r="F16" t="s">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="G16" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H16" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1743,28 +1791,28 @@
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="F17" t="s">
-        <v>15</v>
+        <v>31</v>
       </c>
       <c r="G17" t="s">
-        <v>102</v>
+        <v>82</v>
       </c>
       <c r="H17" t="s">
-        <v>16</v>
+        <v>95</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1777,47 +1825,47 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F18" t="s">
-        <v>10</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s">
-        <v>68</v>
+        <v>121</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B19" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D19" t="s">
         <v>13</v>
@@ -1829,10 +1877,10 @@
         <v>17</v>
       </c>
       <c r="G19" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H19" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1845,62 +1893,62 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F20" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G20" t="s">
-        <v>102</v>
+        <v>125</v>
       </c>
       <c r="H20" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="F21" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="G21" t="s">
-        <v>123</v>
+        <v>82</v>
       </c>
       <c r="H21" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1913,124 +1961,124 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F22" t="s">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="G22" t="s">
-        <v>84</v>
+        <v>129</v>
       </c>
       <c r="H22" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D23" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F23" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G23" t="s">
-        <v>68</v>
+        <v>90</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F24" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G24" t="s">
-        <v>68</v>
+        <v>102</v>
       </c>
       <c r="H24" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B25" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F25" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G25" t="s">
         <v>68</v>
@@ -2040,56 +2088,56 @@
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J25" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A26" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B26" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>10</v>
+      </c>
+      <c r="F26" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" t="s">
+        <v>68</v>
+      </c>
+      <c r="H26" t="s">
+        <v>11</v>
+      </c>
+      <c r="I26" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J25" t="str">
+      <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A26" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B26" t="s">
-        <v>75</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D26" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" t="s">
-        <v>14</v>
-      </c>
-      <c r="F26" t="s">
-        <v>14</v>
-      </c>
-      <c r="G26" t="s">
-        <v>129</v>
-      </c>
-      <c r="H26" t="s">
-        <v>11</v>
-      </c>
-      <c r="I26" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J26" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B27" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
@@ -2101,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="G27" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
@@ -2117,81 +2165,81 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B28" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
       </c>
       <c r="E28" t="s">
+        <v>14</v>
+      </c>
+      <c r="F28" t="s">
+        <v>14</v>
+      </c>
+      <c r="G28" t="s">
+        <v>136</v>
+      </c>
+      <c r="H28" t="s">
+        <v>95</v>
+      </c>
+      <c r="I28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A29" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B29" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
         <v>10</v>
       </c>
-      <c r="F28" t="s">
+      <c r="F29" t="s">
         <v>10</v>
       </c>
-      <c r="G28" t="s">
-        <v>74</v>
-      </c>
-      <c r="H28" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" t="str">
+      <c r="G29" t="s">
+        <v>84</v>
+      </c>
+      <c r="H29" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J28" t="str">
+      <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A29" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B29" t="s">
-        <v>70</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="D29" t="s">
-        <v>13</v>
-      </c>
-      <c r="E29" t="s">
-        <v>27</v>
-      </c>
-      <c r="F29" t="s">
-        <v>2</v>
-      </c>
-      <c r="G29" t="s">
-        <v>109</v>
-      </c>
-      <c r="H29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B30" t="s">
-        <v>70</v>
+        <v>138</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
@@ -2203,7 +2251,7 @@
         <v>25</v>
       </c>
       <c r="G30" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
@@ -2217,129 +2265,129 @@
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>138</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="D31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F31" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="G31" t="s">
-        <v>87</v>
+        <v>141</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B32" t="s">
-        <v>70</v>
+        <v>138</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F32" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>136</v>
+        <v>94</v>
       </c>
       <c r="H32" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B33" t="s">
-        <v>80</v>
+        <v>138</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
         <v>14</v>
       </c>
       <c r="F33" t="s">
-        <v>14</v>
+        <v>144</v>
       </c>
       <c r="G33" t="s">
+        <v>92</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J33" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B34" t="s">
         <v>138</v>
       </c>
-      <c r="H33" t="s">
-        <v>11</v>
-      </c>
-      <c r="I33" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J33" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B34" t="s">
-        <v>80</v>
-      </c>
       <c r="C34" s="6" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D34" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E34" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="F34" t="s">
-        <v>140</v>
+        <v>86</v>
       </c>
       <c r="G34" t="s">
-        <v>141</v>
+        <v>87</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
@@ -2353,34 +2401,34 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B35" t="s">
-        <v>80</v>
+        <v>138</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="F35" t="s">
-        <v>143</v>
+        <v>19</v>
       </c>
       <c r="G35" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Partidos</v>
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2389,47 +2437,47 @@
     </row>
     <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B36" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D36" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E36" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F36" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="G36" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B37" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
@@ -2438,10 +2486,10 @@
         <v>17</v>
       </c>
       <c r="F37" t="s">
-        <v>17</v>
+        <v>150</v>
       </c>
       <c r="G37" t="s">
-        <v>87</v>
+        <v>118</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
@@ -2455,163 +2503,163 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B38" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="F38" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G38" t="s">
-        <v>68</v>
+        <v>82</v>
       </c>
       <c r="H38" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B39" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
+        <v>25</v>
+      </c>
+      <c r="F39" t="s">
+        <v>25</v>
+      </c>
+      <c r="G39" t="s">
+        <v>102</v>
+      </c>
+      <c r="H39" t="s">
+        <v>11</v>
+      </c>
+      <c r="I39" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J39" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A40" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B40" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D40" t="s">
         <v>13</v>
       </c>
-      <c r="E39" t="s">
-        <v>48</v>
-      </c>
-      <c r="F39" t="s">
-        <v>48</v>
-      </c>
-      <c r="G39" t="s">
-        <v>114</v>
-      </c>
-      <c r="H39" t="s">
-        <v>11</v>
-      </c>
-      <c r="I39" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J39" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A40" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B40" t="s">
-        <v>82</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D40" t="s">
-        <v>12</v>
-      </c>
       <c r="E40" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="F40" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G40" t="s">
-        <v>93</v>
+        <v>154</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="41" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B41" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D41" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="F41" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="G41" t="s">
-        <v>151</v>
+        <v>104</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B42" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="F42" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
@@ -2627,32 +2675,32 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B43" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="F43" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="G43" t="s">
-        <v>83</v>
+        <v>141</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2661,28 +2709,28 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B44" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>85</v>
+        <v>159</v>
       </c>
       <c r="D44" t="s">
-        <v>76</v>
+        <v>9</v>
       </c>
       <c r="E44" t="s">
         <v>17</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>117</v>
       </c>
       <c r="G44" t="s">
-        <v>77</v>
+        <v>118</v>
       </c>
       <c r="H44" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2693,30 +2741,30 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B45" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D45" t="s">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="E45" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="F45" t="s">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="G45" t="s">
-        <v>106</v>
+        <v>161</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
+        <v>95</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2724,30 +2772,30 @@
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B46" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="D46" t="s">
         <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F46" t="s">
-        <v>157</v>
+        <v>25</v>
       </c>
       <c r="G46" t="s">
-        <v>158</v>
+        <v>88</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
@@ -2758,166 +2806,166 @@
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A47" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B47" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" t="s">
+        <v>48</v>
+      </c>
+      <c r="F47" t="s">
+        <v>48</v>
+      </c>
+      <c r="G47" t="s">
+        <v>164</v>
+      </c>
+      <c r="H47" t="s">
+        <v>11</v>
+      </c>
+      <c r="I47" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J47" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A48" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B48" t="s">
+        <v>81</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" t="s">
+        <v>25</v>
+      </c>
+      <c r="F48" t="s">
+        <v>25</v>
+      </c>
+      <c r="G48" t="s">
+        <v>102</v>
+      </c>
+      <c r="H48" t="s">
+        <v>11</v>
+      </c>
+      <c r="I48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A49" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B49" t="s">
+        <v>81</v>
+      </c>
+      <c r="C49" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="D49" t="s">
+        <v>12</v>
+      </c>
+      <c r="E49" t="s">
+        <v>21</v>
+      </c>
+      <c r="F49" t="s">
+        <v>167</v>
+      </c>
+      <c r="G49" t="s">
+        <v>168</v>
+      </c>
+      <c r="H49" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A47" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B47" t="s">
-        <v>78</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="D47" t="s">
-        <v>12</v>
-      </c>
-      <c r="E47" t="s">
-        <v>25</v>
-      </c>
-      <c r="F47" t="s">
-        <v>25</v>
-      </c>
-      <c r="G47" t="s">
-        <v>106</v>
-      </c>
-      <c r="H47" t="s">
-        <v>11</v>
-      </c>
-      <c r="I47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A48" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B48" t="s">
-        <v>78</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D48" t="s">
-        <v>12</v>
-      </c>
-      <c r="E48" t="s">
-        <v>27</v>
-      </c>
-      <c r="F48" t="s">
-        <v>2</v>
-      </c>
-      <c r="G48" t="s">
-        <v>109</v>
-      </c>
-      <c r="H48" t="s">
-        <v>11</v>
-      </c>
-      <c r="I48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A49" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B49" t="s">
-        <v>78</v>
-      </c>
-      <c r="C49" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D49" t="s">
-        <v>12</v>
-      </c>
-      <c r="E49" t="s">
-        <v>17</v>
-      </c>
-      <c r="F49" t="s">
-        <v>17</v>
-      </c>
-      <c r="G49" t="s">
-        <v>162</v>
-      </c>
-      <c r="H49" t="s">
-        <v>11</v>
-      </c>
-      <c r="I49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F50" t="s">
-        <v>10</v>
+        <v>170</v>
       </c>
       <c r="G50" t="s">
-        <v>68</v>
+        <v>171</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B51" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="D51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>27</v>
+        <v>57</v>
       </c>
       <c r="F51" t="s">
-        <v>2</v>
+        <v>173</v>
       </c>
       <c r="G51" t="s">
-        <v>109</v>
+        <v>174</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
@@ -2933,32 +2981,32 @@
     </row>
     <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B52" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F52" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G52" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2967,25 +3015,25 @@
     </row>
     <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A53" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B53" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="D53" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E53" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="F53" t="s">
-        <v>157</v>
+        <v>25</v>
       </c>
       <c r="G53" t="s">
-        <v>158</v>
+        <v>104</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
@@ -2996,18 +3044,18 @@
       </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B54" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
@@ -3016,10 +3064,10 @@
         <v>17</v>
       </c>
       <c r="F54" t="s">
-        <v>17</v>
+        <v>150</v>
       </c>
       <c r="G54" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
@@ -3035,50 +3083,50 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B55" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>168</v>
+        <v>83</v>
       </c>
       <c r="D55" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="E55" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F55" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G55" t="s">
-        <v>141</v>
+        <v>76</v>
       </c>
       <c r="H55" t="s">
         <v>11</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A56" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B56" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>85</v>
+        <v>180</v>
       </c>
       <c r="D56" t="s">
-        <v>76</v>
+        <v>12</v>
       </c>
       <c r="E56" t="s">
         <v>17</v>
@@ -3087,41 +3135,41 @@
         <v>17</v>
       </c>
       <c r="G56" t="s">
+        <v>181</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B57" t="s">
         <v>77</v>
       </c>
-      <c r="H56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A57" s="5">
-        <v>46126</v>
-      </c>
-      <c r="B57" t="s">
-        <v>79</v>
-      </c>
       <c r="C57" s="6" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="D57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F57" t="s">
-        <v>99</v>
+        <v>2</v>
       </c>
       <c r="G57" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
@@ -3137,100 +3185,100 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B58" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="D58" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E58" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F58" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G58" t="s">
-        <v>68</v>
+        <v>102</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B59" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>172</v>
+        <v>185</v>
       </c>
       <c r="D59" t="s">
-        <v>173</v>
+        <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F59" t="s">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="G59" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="H59" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B60" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D60" t="s">
         <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F60" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G60" t="s">
-        <v>176</v>
+        <v>118</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3239,25 +3287,25 @@
     </row>
     <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
-        <v>46126</v>
+        <v>46127</v>
       </c>
       <c r="B61" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="F61" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="G61" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="H61" t="s">
         <v>11</v>
@@ -3269,6 +3317,244 @@
       <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A62" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B62" t="s">
+        <v>28</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D62" t="s">
+        <v>75</v>
+      </c>
+      <c r="E62" t="s">
+        <v>10</v>
+      </c>
+      <c r="F62" t="s">
+        <v>10</v>
+      </c>
+      <c r="G62" t="s">
+        <v>68</v>
+      </c>
+      <c r="H62" t="s">
+        <v>11</v>
+      </c>
+      <c r="I62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A63" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B63" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="D63" t="s">
+        <v>75</v>
+      </c>
+      <c r="E63" t="s">
+        <v>17</v>
+      </c>
+      <c r="F63" t="s">
+        <v>17</v>
+      </c>
+      <c r="G63" t="s">
+        <v>76</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+      <c r="I63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A64" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B64" t="s">
+        <v>78</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="D64" t="s">
+        <v>13</v>
+      </c>
+      <c r="E64" t="s">
+        <v>25</v>
+      </c>
+      <c r="F64" t="s">
+        <v>25</v>
+      </c>
+      <c r="G64" t="s">
+        <v>102</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A65" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B65" t="s">
+        <v>78</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D65" t="s">
+        <v>12</v>
+      </c>
+      <c r="E65" t="s">
+        <v>56</v>
+      </c>
+      <c r="F65" t="s">
+        <v>56</v>
+      </c>
+      <c r="G65" t="s">
+        <v>154</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A66" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B66" t="s">
+        <v>78</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D66" t="s">
+        <v>12</v>
+      </c>
+      <c r="E66" t="s">
+        <v>17</v>
+      </c>
+      <c r="F66" t="s">
+        <v>17</v>
+      </c>
+      <c r="G66" t="s">
+        <v>191</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A67" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B67" t="s">
+        <v>78</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="D67" t="s">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s">
+        <v>14</v>
+      </c>
+      <c r="F67" t="s">
+        <v>14</v>
+      </c>
+      <c r="G67" t="s">
+        <v>94</v>
+      </c>
+      <c r="H67" t="s">
+        <v>95</v>
+      </c>
+      <c r="I67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+      <c r="A68" s="5">
+        <v>46127</v>
+      </c>
+      <c r="B68" t="s">
+        <v>78</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" t="s">
+        <v>10</v>
+      </c>
+      <c r="F68" t="s">
+        <v>10</v>
+      </c>
+      <c r="G68" t="s">
+        <v>68</v>
+      </c>
+      <c r="H68" t="s">
+        <v>11</v>
+      </c>
+      <c r="I68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
       </c>
     </row>
   </sheetData>
@@ -3301,7 +3587,7 @@
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
@@ -3315,7 +3601,7 @@
         <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
@@ -3329,7 +3615,7 @@
         <v>35</v>
       </c>
       <c r="E3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -3343,7 +3629,7 @@
         <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
@@ -3357,7 +3643,7 @@
         <v>30</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
@@ -3371,7 +3657,7 @@
         <v>38</v>
       </c>
       <c r="E6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
@@ -3385,7 +3671,7 @@
         <v>39</v>
       </c>
       <c r="E7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
@@ -3399,7 +3685,7 @@
         <v>39</v>
       </c>
       <c r="E8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
@@ -3413,7 +3699,7 @@
         <v>40</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
@@ -3441,7 +3727,7 @@
         <v>41</v>
       </c>
       <c r="E11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
@@ -3455,7 +3741,7 @@
         <v>42</v>
       </c>
       <c r="E12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
@@ -3469,7 +3755,7 @@
         <v>42</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
@@ -3483,7 +3769,7 @@
         <v>22</v>
       </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
@@ -3497,7 +3783,7 @@
         <v>18</v>
       </c>
       <c r="E15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
@@ -3511,7 +3797,7 @@
         <v>50</v>
       </c>
       <c r="E16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
@@ -3525,7 +3811,7 @@
         <v>56</v>
       </c>
       <c r="E17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
@@ -3539,7 +3825,7 @@
         <v>57</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
@@ -3553,7 +3839,7 @@
         <v>24</v>
       </c>
       <c r="E19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
@@ -3567,7 +3853,7 @@
         <v>21</v>
       </c>
       <c r="E20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
@@ -3581,7 +3867,7 @@
         <v>29</v>
       </c>
       <c r="E21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
@@ -3595,7 +3881,7 @@
         <v>27</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
@@ -3609,7 +3895,7 @@
         <v>58</v>
       </c>
       <c r="E23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
@@ -3623,7 +3909,7 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
@@ -3637,7 +3923,7 @@
         <v>23</v>
       </c>
       <c r="E25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
@@ -3651,7 +3937,7 @@
         <v>59</v>
       </c>
       <c r="E26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
@@ -3665,7 +3951,7 @@
         <v>31</v>
       </c>
       <c r="E27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Reporte 16 de abril
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{262BA2E7-F8F8-4A83-8875-527A909B9A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2C9122A-58C2-4552-B872-40B809FED4F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="580" uniqueCount="184">
   <si>
     <t>Fecha</t>
   </si>
@@ -285,340 +285,310 @@
     <t>Effetá</t>
   </si>
   <si>
-    <t>Semana Santa</t>
-  </si>
-  <si>
     <t>Usa el puente peatonal</t>
   </si>
   <si>
-    <t>Temas internacionales</t>
-  </si>
-  <si>
-    <t>SICT</t>
-  </si>
-  <si>
-    <t>PC</t>
-  </si>
-  <si>
-    <t>Prevención De Riesgos</t>
-  </si>
-  <si>
-    <t>Carril confinado</t>
-  </si>
-  <si>
-    <t>titular</t>
-  </si>
-  <si>
-    <t>Tren México Querétaro</t>
-  </si>
-  <si>
     <t>Editorial</t>
   </si>
   <si>
-    <t>Fuga de hidrocarburo</t>
-  </si>
-  <si>
-    <t>Menos homicidios dolosos en Hidalgo</t>
-  </si>
-  <si>
-    <t>Incidencia Delictiva</t>
-  </si>
-  <si>
     <t>Positiva</t>
   </si>
   <si>
-    <t>Limitan interacción por miedo a ser funados</t>
-  </si>
-  <si>
-    <t>Clausuran barranca de Metztitlán por explotación</t>
-  </si>
-  <si>
-    <t>Clausura de empresa contaminante</t>
-  </si>
-  <si>
-    <t>Ley de devolución excluye al Códice Borbónico</t>
-  </si>
-  <si>
-    <t>Códice borbónico</t>
-  </si>
-  <si>
-    <t>Aumento de pasaje no afectará economía</t>
-  </si>
-  <si>
     <t>Aumento Tarifa De Transporte</t>
   </si>
   <si>
-    <t>Dan espacio al arte</t>
-  </si>
-  <si>
-    <t>Intervención Gráfica</t>
-  </si>
-  <si>
-    <t>Bajan homicidios dolosos: CSP</t>
-  </si>
-  <si>
-    <t>Planean regular salarios de alcaldes sin violar autonomía</t>
-  </si>
-  <si>
-    <t>GLMorena</t>
-  </si>
-  <si>
     <t>Iniciativa</t>
   </si>
   <si>
-    <t>Avisan vía notario de riesgo a afectados</t>
-  </si>
-  <si>
-    <t>Reubicación de viviendas</t>
-  </si>
-  <si>
-    <t>Pensar la historia como una disciplina fundamental implica reconocer que el pasado no es un conjunto de fechas y nombres, sino un campo vivo de...</t>
-  </si>
-  <si>
-    <t>TUZOS BUSCARÁN LACOPA LA INMORTALIDAD</t>
-  </si>
-  <si>
-    <t>PSG Y EL ATLÉTICO  AVANZAN A SEMIS</t>
-  </si>
-  <si>
-    <t>NO ACEPTARÁN “CHANTAJE” POR EL NUEVO PASAJE</t>
-  </si>
-  <si>
-    <t>PROPONEN ELIMINAR  LAS SINDICATURAS DE  MINORÍA EN CABILDOS</t>
-  </si>
-  <si>
-    <t>ALCALDÍA Y  TIENDAS OXXO  REHABILITAN EL  JARDÍN DEL ARTE</t>
-  </si>
-  <si>
-    <t>Alcalde</t>
-  </si>
-  <si>
-    <t>Rehabilitación de espacios públicos</t>
-  </si>
-  <si>
-    <t>Hidalgo ingresó 1,235 millones de pesos en la Semana Santa</t>
-  </si>
-  <si>
-    <t>Esperan que Hospital General de Actopan funcione este año</t>
-  </si>
-  <si>
-    <t>Nuevo Hospital General</t>
-  </si>
-  <si>
-    <t>Crece el presupuesto de Pachuca; priorizan inversión en seguridad</t>
-  </si>
-  <si>
-    <t>Modificación Presupuestal</t>
-  </si>
-  <si>
-    <t>Preparan actividades para recibir  a los turistas</t>
-  </si>
-  <si>
     <t>Mundial De Futbol</t>
   </si>
   <si>
-    <t>En Semana Santa estado recibe más de 1,235 mdp</t>
-  </si>
-  <si>
-    <t>Tuzobús no logra metas de viajes... ni de ingresos</t>
-  </si>
-  <si>
     <t>Sitmah</t>
   </si>
   <si>
-    <t>Deficiencias Tuzobús</t>
-  </si>
-  <si>
-    <t>Hallan vestigios de más de 4 mil años; cambian trazo del tren</t>
-  </si>
-  <si>
-    <t>Julio Menchaca: habrá aumento en la tarifa, pero sin chantajes</t>
-  </si>
-  <si>
-    <t>Originario de Zimapán, el minero que sigue atrapado</t>
-  </si>
-  <si>
-    <t>Tratamientos para vivir más sin certificado científico</t>
-  </si>
-  <si>
-    <t>Magnicharters adeuda $150 millones a agencias y dueños se esfuman</t>
-  </si>
-  <si>
-    <t>Una fuente de electricidad al menos por familia en 2030</t>
-  </si>
-  <si>
-    <t>Energías renovables</t>
-  </si>
-  <si>
-    <t>Shock chino 2.0 con productos de alta tecnología</t>
-  </si>
-  <si>
     <t>La Jornada Hidalgo</t>
   </si>
   <si>
-    <t>Nuevas tarifas del transporte estarán listas este mes: JMS</t>
-  </si>
-  <si>
-    <t>Municipios buscan contratar deuda tras daños por vaguada</t>
-  </si>
-  <si>
     <t>Huracán Priscilla</t>
   </si>
   <si>
-    <t>Sheinbaum destaca caída de 45% en homicidios y escuela de Mandos</t>
-  </si>
-  <si>
-    <t>Lluvias arrastran hidrocarburo a Poza Rica y Coatzintla: Pemex</t>
-  </si>
-  <si>
-    <t>Pemex</t>
-  </si>
-  <si>
-    <t>Colaplsa barda de INFRA y destroza camioneta</t>
-  </si>
-  <si>
-    <t>La diferencia es que en San Luis Potosí el gobierno es ecologista y aquí  morenista y, por lo que se ha visto, el grupo en el poder no está dispuesto  a perder en las primeras elecciones los que les llevó tanto tiempo ganar”.</t>
-  </si>
-  <si>
     <t>Alianzas Electorales</t>
   </si>
   <si>
-    <t>Exponen 15 hidalguenses su arte en Palacio de  Gobierno con “Hióki”</t>
-  </si>
-  <si>
-    <t>Pachuca rehabilita el Jardín del Arte con apoyo de la iniciativa privada</t>
-  </si>
-  <si>
     <t>alcalde</t>
   </si>
   <si>
-    <t>Supera Hidalgo los 2.4 millones de visitantes en Semana Santa 2026</t>
-  </si>
-  <si>
-    <t>Aumento de tarifa del transporte  será “razonable” y podría definirse  este mes: Menchaca</t>
-  </si>
-  <si>
-    <t>Pide Napeoleón a productores no caer en pánico por gusano barrenador</t>
-  </si>
-  <si>
     <t>Gusano barrenador</t>
   </si>
   <si>
-    <t>JULIO MENCHACA INAUGURA INTERVENCIÓN GRÁFICA 4.1 HlóKi</t>
-  </si>
-  <si>
-    <t>Productores apícolas piden certificación</t>
-  </si>
-  <si>
-    <t>Certificación</t>
-  </si>
-  <si>
-    <t>La reconstrucción de los puentes es con recurso federal: SICT</t>
-  </si>
-  <si>
-    <t>Reactivan ícono de Pachuca</t>
-  </si>
-  <si>
-    <t>El oficio político en tiempos de protagonismo</t>
-  </si>
-  <si>
-    <t>Labor destacada</t>
-  </si>
-  <si>
-    <t>Carril exclusivo del Tuzobús, decisión en beneficio de la mayoría: Menchaca</t>
-  </si>
-  <si>
-    <t>PAN acusa ""robo"" de militantes</t>
-  </si>
-  <si>
-    <t>Militancia Partidista</t>
-  </si>
-  <si>
-    <t>En abril, aumento al pasaje</t>
-  </si>
-  <si>
-    <t>¡Solo dos sanciones en 10 años!</t>
-  </si>
-  <si>
-    <t>Proespa</t>
-  </si>
-  <si>
-    <t>Maltrato animal</t>
-  </si>
-  <si>
-    <t>Hidalgo fortalece acciones para prevenir el embarazo en niñas y adolescentes</t>
-  </si>
-  <si>
     <t>Coespo</t>
   </si>
   <si>
     <t>Prevención De Embarazo Adolescente</t>
   </si>
   <si>
-    <t>Entregan en Tula calentadores del programa ""Energía para el Bienestar""</t>
-  </si>
-  <si>
-    <t>AEEH</t>
-  </si>
-  <si>
-    <t>Energía para el Bienestar</t>
-  </si>
-  <si>
-    <t>Iniciaron los trabajos de pavimentación asfáltica en Ignacio Zaragoza</t>
-  </si>
-  <si>
-    <t>Pavimentación</t>
-  </si>
-  <si>
-    <t>Como un "acto de reconstrucción", Julio Menchaca inaugura intervención gráfica 4.1</t>
-  </si>
-  <si>
-    <t>Jorge Reyes y Oxxo intervienen el Jardín del Arte para reactivar un espacio emblemático</t>
-  </si>
-  <si>
-    <t>Apropiación de espacios públicos</t>
-  </si>
-  <si>
-    <t>Rehabilitación de la calle Vía de los Reyes fortalece la conectividad en EI Daxthá, Actopan</t>
-  </si>
-  <si>
-    <t>Rehabilitación Vial</t>
-  </si>
-  <si>
-    <t>Natividad Castrejón abandera delegación hidalguense rumbo a la Olimpiada Nacional Conade</t>
-  </si>
-  <si>
-    <t>Justa Deportiva</t>
-  </si>
-  <si>
-    <t>Nueva tarifa de transporte, para este mes: Julio Menchaca</t>
-  </si>
-  <si>
-    <t>Abanderan delegación hidalguense rumbo a la Olimpiada Nacional</t>
-  </si>
-  <si>
-    <t>Participan 15 artistas en intervención gráfica 4.1 Hióki, en edificio de gobierno</t>
-  </si>
-  <si>
     <t>Máquina del tiempo</t>
   </si>
   <si>
-    <t>Confirman incremento al pasaje del transporte público</t>
-  </si>
-  <si>
-    <t>Refuerzan atención y control del gusano barrenador</t>
-  </si>
-  <si>
-    <t>Denuncian entrega de bonos a regidores mediante apoyos</t>
-  </si>
-  <si>
     <t>Entrega De Apoyos</t>
   </si>
   <si>
-    <t>Los homicidios cayeron un 41% en 18 meses con Sheinbaum</t>
-  </si>
-  <si>
-    <t>A pesar de que no han subido de precio las gasolinas, los demás productos básico se han elevado como cohetes, lo que obliga a la gente a comprar por medios kilos o medios litros</t>
+    <t>Aumenta el precio del jitomate en 126%: Inegi</t>
+  </si>
+  <si>
+    <t>Señalan comerciantes nuevo deterioro en piso</t>
+  </si>
+  <si>
+    <t>Rehabilitación De Mercados</t>
+  </si>
+  <si>
+    <t>Dicen no a la veda taurina</t>
+  </si>
+  <si>
+    <t>Tauromaquia</t>
+  </si>
+  <si>
+    <t>Crece la presencia de mariposa monarca</t>
+  </si>
+  <si>
+    <t>Coesbioh</t>
+  </si>
+  <si>
+    <t>Conservación Biodiversidad</t>
+  </si>
+  <si>
+    <t>Desalojan a comerciantes de Plaza Constitución</t>
+  </si>
+  <si>
+    <t>Ambulantaje</t>
+  </si>
+  <si>
+    <t>Hidalgo obtiene alta calificación con HR Ratings</t>
+  </si>
+  <si>
+    <t>Calificación crediticia</t>
+  </si>
+  <si>
+    <t>Retiran a comerciantes</t>
+  </si>
+  <si>
+    <t>Inclusión mediante la música</t>
+  </si>
+  <si>
+    <t>Morena descarta ruptura con PVEM</t>
+  </si>
+  <si>
+    <t>Buscan resolver violencia escolar</t>
+  </si>
+  <si>
+    <t>Violencia Escolar</t>
+  </si>
+  <si>
+    <t>Criterio</t>
+  </si>
+  <si>
+    <t>Pachuca factura con los Rayados</t>
+  </si>
+  <si>
+    <t>NOCHE DE LUCHA  IMPERDIBLE P13 3</t>
+  </si>
+  <si>
+    <t>GANAN DOS ALCALDES MÁS QUE MENCHACA</t>
+  </si>
+  <si>
+    <t>Tabulador salarial</t>
+  </si>
+  <si>
+    <t>Protestan para exigir consulta indígena sobre la tauromaquia</t>
+  </si>
+  <si>
+    <t>Retiran puestos ambulantes de plaza constitución</t>
+  </si>
+  <si>
+    <t>Concesionarios esperan alza en el pasaje entre 12 y 12.50 pesos</t>
+  </si>
+  <si>
+    <t>Exigen justicia para Iván; dicen que el caso no tiene avances</t>
+  </si>
+  <si>
+    <t>Exigen esclarecer homicidio</t>
+  </si>
+  <si>
+    <t>Adiós concesionarios; estado tomará control del sistema Tuzobús</t>
+  </si>
+  <si>
+    <t>Modernización Tuzobús</t>
+  </si>
+  <si>
+    <t>Proponen eliminar una sindicatura y regidores</t>
+  </si>
+  <si>
+    <t>Plan B</t>
+  </si>
+  <si>
+    <t>Cmabio en la SSPP era parte de un plan: Reyes</t>
+  </si>
+  <si>
+    <t>Nombramientos</t>
+  </si>
+  <si>
+    <t>Ponga fin a la ansiedad financiera</t>
+  </si>
+  <si>
+    <t>El estado se ubica entre los que más disminuyen el embarazo infantil</t>
+  </si>
+  <si>
+    <t>Piden no cancelar corridas; va nueva ley</t>
+  </si>
+  <si>
+    <t>El Verde mete presión a Morena y exige ""respeto"" a las encuestas</t>
+  </si>
+  <si>
+    <t>González Iñárritu y Tom Cruise agitan Las Vegas con Digger</t>
+  </si>
+  <si>
+    <t>Congreso propondrá endurecer penas a choferes homicidas</t>
+  </si>
+  <si>
+    <t>Ratifican positiva calificación crediticia</t>
+  </si>
+  <si>
+    <t>Fracking, hasta tener evaluación soberana</t>
+  </si>
+  <si>
+    <t>Fracking</t>
+  </si>
+  <si>
+    <t>Comunidad sale a las calles contra iniciativa antitaurina</t>
+  </si>
+  <si>
+    <t>El Clima ha dejado de ser una variable predecible para convertirse en un adversario</t>
+  </si>
+  <si>
+    <t>HR Ratings reonoce a Hidalgo por su disciplina financiera y eleva su perspectiva de estable a positiva</t>
+  </si>
+  <si>
+    <t>Plaza Constitución será liberada de vendedores ambulantes este jueves: Jorge Reyes</t>
+  </si>
+  <si>
+    <t>Amaga chofer de transporte público con agredir con machete a automovilista</t>
+  </si>
+  <si>
+    <t>Pelea transportistas</t>
+  </si>
+  <si>
+    <t>Taurinos marchan en contra de prohibir la fiesta brava en Hidalgo</t>
+  </si>
+  <si>
+    <t>Atiende gobierno derrumbe en carretera tianguistengo-Yatipán</t>
+  </si>
+  <si>
+    <t>Sipdus</t>
+  </si>
+  <si>
+    <t>Derrumbe Carretero</t>
+  </si>
+  <si>
+    <t>EXHORTA REGLAMENTOS DE HUEJUTLAA COMERCIOS A REGULARIZAR ADEUDOS.</t>
+  </si>
+  <si>
+    <t>Actualización de reglamentos</t>
+  </si>
+  <si>
+    <t>Sin respuesta de rebombeo en Tepeco</t>
+  </si>
+  <si>
+    <t>Agua</t>
+  </si>
+  <si>
+    <t>Abasto De Agua</t>
+  </si>
+  <si>
+    <t>Huejutla se suma al Mundial Social</t>
+  </si>
+  <si>
+    <t>HR Ratings ratifica a Hidalgo con alta calificación</t>
+  </si>
+  <si>
+    <t>Desalojo nocturno en Plaza Constitución</t>
+  </si>
+  <si>
+    <t>Hidalgo frena el embarazo infantil</t>
+  </si>
+  <si>
+    <t>Penas más duras contra choferes</t>
+  </si>
+  <si>
+    <t>Corridas sin muerte</t>
+  </si>
+  <si>
+    <t>ALerta ganadera</t>
+  </si>
+  <si>
+    <t>Taurinos exigen consulta indígena antes de prohibir corridas de toros en Hidalgo</t>
+  </si>
+  <si>
+    <t>Cintillo</t>
+  </si>
+  <si>
+    <t>DIF Tula busca ampliar hasta 40% su cobertura y recaudación sin aumentar costos</t>
+  </si>
+  <si>
+    <t>Más de 100 familias beneficiadas en Programa Hogares en Transformación</t>
+  </si>
+  <si>
+    <t>HR Ratings ratifica a Hidalgo con alta calificación y eleva su perspectiva de estable a positiva</t>
+  </si>
+  <si>
+    <t>Tezontepec, Pachuca, Tlahuelilpan, Tlaxcoapan, Ajacuba y Tula, entre los municipios que estrenarán cancha de Futbol 5</t>
+  </si>
+  <si>
+    <t>Cristhian Martínez impulsa la mejora de infraestructura con presupuesto participativo en la colonia Iturbe</t>
+  </si>
+  <si>
+    <t>¡Última oportunidad Tula-Tepeji!</t>
+  </si>
+  <si>
+    <t>Infonavit</t>
+  </si>
+  <si>
+    <t>Plan Nacional De Vivienda</t>
+  </si>
+  <si>
+    <t>ochoHR Ratings ratifica a Hidalgo con su alta calificación y eleva su perspectiva de estable a positiva</t>
+  </si>
+  <si>
+    <t>Este jueves vacunación contra sarampión en Parque Hidalgo</t>
+  </si>
+  <si>
+    <t>Sarampión</t>
+  </si>
+  <si>
+    <t>Refuerzan acciones de salud pública ante el Mundial Fifa 2026</t>
+  </si>
+  <si>
+    <t>Firman convenio para proyectos deportivos comunitarios</t>
+  </si>
+  <si>
+    <t>Firma De Convenio</t>
+  </si>
+  <si>
+    <t>Elevan la perspectiva de Hidalgo de ""Estable"" a ""Positiva""</t>
+  </si>
+  <si>
+    <t>La Fiesta Brava es un acto de crueldad animal: Avelino Tovar</t>
+  </si>
+  <si>
+    <t>GLPVEM</t>
+  </si>
+  <si>
+    <t>En momentos que padecemos asesinatos y desapariciones de miles de mexicanos, el diputado Avelino del partido Verde, se preocupa más por el sufrimiento de los toros</t>
+  </si>
+  <si>
+    <t>Trabajador atrapado en mina de Sinaloa sería hidalguense</t>
+  </si>
+  <si>
+    <t>Rescate de persona</t>
   </si>
 </sst>
 </file>
@@ -865,8 +835,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J68" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J68" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J61" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J61" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1232,7 +1202,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -1281,66 +1251,66 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B2" t="s">
         <v>80</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="H2" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B3" t="s">
         <v>80</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1349,32 +1319,32 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B4" t="s">
         <v>80</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="G4" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1383,96 +1353,96 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B5" t="s">
         <v>80</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>104</v>
       </c>
       <c r="G5" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B6" t="s">
         <v>80</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D6" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H6" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B7" t="s">
         <v>69</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="D7" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="F7" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G7" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H7" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1485,32 +1455,32 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B8" t="s">
         <v>69</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F8" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G8" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="H8" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1519,32 +1489,32 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B9" t="s">
         <v>69</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>112</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="F9" t="s">
-        <v>107</v>
+        <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="H9" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Partidos</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1553,47 +1523,47 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B10" t="s">
         <v>69</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="F10" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="G10" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
@@ -1605,7 +1575,7 @@
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
@@ -1621,13 +1591,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B12" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -1655,32 +1625,32 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B13" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F13" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>119</v>
       </c>
       <c r="H13" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1689,66 +1659,66 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="D14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
         <v>102</v>
       </c>
       <c r="H14" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="D15" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E15" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="F15" t="s">
+        <v>17</v>
+      </c>
+      <c r="G15" t="s">
         <v>107</v>
       </c>
-      <c r="G15" t="s">
-        <v>108</v>
-      </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1757,62 +1727,62 @@
     </row>
     <row r="16" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A16" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D16" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E16" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>117</v>
+        <v>29</v>
       </c>
       <c r="G16" t="s">
-        <v>118</v>
+        <v>85</v>
       </c>
       <c r="H16" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>115</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="F17" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="G17" t="s">
-        <v>82</v>
+        <v>124</v>
       </c>
       <c r="H17" t="s">
-        <v>95</v>
+        <v>16</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1823,30 +1793,30 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B18" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D18" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E18" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="F18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G18" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H18" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1857,34 +1827,34 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B19" t="s">
         <v>74</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="D19" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="F19" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="G19" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="H19" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1893,13 +1863,13 @@
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B20" t="s">
         <v>74</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
@@ -1908,10 +1878,10 @@
         <v>17</v>
       </c>
       <c r="F20" t="s">
-        <v>17</v>
+        <v>92</v>
       </c>
       <c r="G20" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
@@ -1927,62 +1897,62 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B21" t="s">
         <v>74</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="G21" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="H21" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B22" t="s">
         <v>74</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="F22" t="s">
-        <v>128</v>
+        <v>94</v>
       </c>
       <c r="G22" t="s">
-        <v>129</v>
+        <v>95</v>
       </c>
       <c r="H22" t="s">
-        <v>16</v>
+        <v>84</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1995,32 +1965,32 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B23" t="s">
         <v>74</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
         <v>9</v>
       </c>
       <c r="E23" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F23" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G23" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2029,56 +1999,56 @@
     </row>
     <row r="24" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B24" t="s">
         <v>74</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
       <c r="H24" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B25" t="s">
         <v>74</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
         <v>68</v>
@@ -2088,7 +2058,7 @@
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2097,25 +2067,25 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="F26" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="G26" t="s">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
@@ -2129,49 +2099,49 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="F27" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="G27" t="s">
-        <v>68</v>
+        <v>109</v>
       </c>
       <c r="H27" t="s">
         <v>11</v>
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
@@ -2183,10 +2153,10 @@
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H28" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2199,25 +2169,25 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D29" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E29" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="F29" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="G29" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
@@ -2231,27 +2201,27 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B30" t="s">
-        <v>138</v>
+        <v>89</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="F30" t="s">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="G30" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
@@ -2262,71 +2232,71 @@
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B31" t="s">
-        <v>138</v>
+        <v>70</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D31" t="s">
         <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="F31" t="s">
-        <v>17</v>
+        <v>42</v>
       </c>
       <c r="G31" t="s">
-        <v>141</v>
+        <v>109</v>
       </c>
       <c r="H31" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B32" t="s">
-        <v>138</v>
+        <v>70</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F32" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G32" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="H32" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2335,149 +2305,149 @@
     </row>
     <row r="33" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B33" t="s">
-        <v>138</v>
+        <v>70</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="F33" t="s">
-        <v>144</v>
+        <v>29</v>
       </c>
       <c r="G33" t="s">
-        <v>92</v>
+        <v>145</v>
       </c>
       <c r="H33" t="s">
         <v>16</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B34" t="s">
-        <v>138</v>
+        <v>70</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="F34" t="s">
-        <v>86</v>
+        <v>36</v>
       </c>
       <c r="G34" t="s">
-        <v>87</v>
+        <v>102</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A35" s="5">
+        <v>46128</v>
+      </c>
+      <c r="B35" t="s">
+        <v>79</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D35" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35" t="s">
+        <v>148</v>
+      </c>
+      <c r="F35" t="s">
+        <v>148</v>
+      </c>
+      <c r="G35" t="s">
+        <v>149</v>
+      </c>
+      <c r="H35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J34" t="str">
+      <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A35" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B35" t="s">
-        <v>138</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="D35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" t="s">
-        <v>19</v>
-      </c>
-      <c r="F35" t="s">
-        <v>19</v>
-      </c>
-      <c r="G35" t="s">
-        <v>147</v>
-      </c>
-      <c r="H35" t="s">
-        <v>11</v>
-      </c>
-      <c r="I35" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J35" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F36" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G36" t="s">
-        <v>104</v>
+        <v>151</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B37" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
@@ -2486,13 +2456,13 @@
         <v>17</v>
       </c>
       <c r="F37" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G37" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="H37" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2503,64 +2473,64 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B38" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="F38" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G38" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="H38" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B39" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="F39" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G39" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="H39" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2568,67 +2538,67 @@
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="D40" t="s">
         <v>13</v>
       </c>
       <c r="E40" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
       <c r="F40" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G40" t="s">
-        <v>154</v>
+        <v>107</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F41" t="s">
-        <v>25</v>
+        <v>94</v>
       </c>
       <c r="G41" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="H41" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2636,30 +2606,30 @@
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="F42" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="G42" t="s">
-        <v>157</v>
+        <v>86</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
@@ -2675,32 +2645,32 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B43" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D43" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E43" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F43" t="s">
-        <v>85</v>
+        <v>10</v>
       </c>
       <c r="G43" t="s">
-        <v>141</v>
+        <v>102</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2709,164 +2679,164 @@
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B44" t="s">
         <v>81</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D44" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="F44" t="s">
-        <v>117</v>
+        <v>56</v>
       </c>
       <c r="G44" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="H44" t="s">
-        <v>95</v>
+        <v>16</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B45" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D45" t="s">
-        <v>91</v>
+        <v>163</v>
       </c>
       <c r="E45" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="F45" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G45" t="s">
-        <v>161</v>
+        <v>102</v>
       </c>
       <c r="H45" t="s">
-        <v>95</v>
+        <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="46" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B46" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="F46" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="G46" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A47" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B47" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D47" t="s">
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="F47" t="s">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="G47" t="s">
-        <v>164</v>
+        <v>97</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B48" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D48" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E48" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="F48" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G48" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="H48" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2874,188 +2844,188 @@
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B49" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D49" t="s">
         <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="F49" t="s">
-        <v>167</v>
+        <v>17</v>
       </c>
       <c r="G49" t="s">
-        <v>168</v>
+        <v>87</v>
       </c>
       <c r="H49" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B50" t="s">
         <v>77</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F50" t="s">
-        <v>170</v>
+        <v>17</v>
       </c>
       <c r="G50" t="s">
-        <v>171</v>
+        <v>68</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B51" t="s">
         <v>77</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>57</v>
+        <v>14</v>
       </c>
       <c r="F51" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="G51" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B52" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="D52" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E52" t="s">
+        <v>42</v>
+      </c>
+      <c r="F52" t="s">
+        <v>42</v>
+      </c>
+      <c r="G52" t="s">
+        <v>109</v>
+      </c>
+      <c r="H52" t="s">
+        <v>84</v>
+      </c>
+      <c r="I52" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J52" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A53" s="5">
+        <v>46128</v>
+      </c>
+      <c r="B53" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D53" t="s">
+        <v>75</v>
+      </c>
+      <c r="E53" t="s">
         <v>17</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F53" t="s">
         <v>17</v>
       </c>
-      <c r="G52" t="s">
-        <v>176</v>
-      </c>
-      <c r="H52" t="s">
-        <v>11</v>
-      </c>
-      <c r="I52" t="str">
+      <c r="G53" t="s">
+        <v>174</v>
+      </c>
+      <c r="H53" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
       </c>
-      <c r="J52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A53" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B53" t="s">
-        <v>77</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="D53" t="s">
-        <v>13</v>
-      </c>
-      <c r="E53" t="s">
-        <v>25</v>
-      </c>
-      <c r="F53" t="s">
-        <v>25</v>
-      </c>
-      <c r="G53" t="s">
-        <v>104</v>
-      </c>
-      <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A54" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B54" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
@@ -3064,10 +3034,10 @@
         <v>17</v>
       </c>
       <c r="F54" t="s">
-        <v>150</v>
+        <v>17</v>
       </c>
       <c r="G54" t="s">
-        <v>179</v>
+        <v>87</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
@@ -3083,130 +3053,130 @@
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B55" t="s">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>83</v>
+        <v>176</v>
       </c>
       <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>27</v>
+      </c>
+      <c r="F55" t="s">
+        <v>2</v>
+      </c>
+      <c r="G55" t="s">
+        <v>177</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A56" s="5">
+        <v>46128</v>
+      </c>
+      <c r="B56" t="s">
+        <v>28</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D56" t="s">
         <v>75</v>
       </c>
-      <c r="E55" t="s">
+      <c r="E56" t="s">
+        <v>10</v>
+      </c>
+      <c r="F56" t="s">
+        <v>10</v>
+      </c>
+      <c r="G56" t="s">
+        <v>75</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A57" s="5">
+        <v>46128</v>
+      </c>
+      <c r="B57" t="s">
+        <v>28</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D57" t="s">
+        <v>75</v>
+      </c>
+      <c r="E57" t="s">
         <v>17</v>
       </c>
-      <c r="F55" t="s">
+      <c r="F57" t="s">
         <v>17</v>
       </c>
-      <c r="G55" t="s">
+      <c r="G57" t="s">
         <v>76</v>
       </c>
-      <c r="H55" t="s">
-        <v>11</v>
-      </c>
-      <c r="I55" t="str">
+      <c r="H57" t="s">
+        <v>11</v>
+      </c>
+      <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
       </c>
-      <c r="J55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A56" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B56" t="s">
-        <v>77</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="D56" t="s">
-        <v>12</v>
-      </c>
-      <c r="E56" t="s">
-        <v>17</v>
-      </c>
-      <c r="F56" t="s">
-        <v>17</v>
-      </c>
-      <c r="G56" t="s">
-        <v>181</v>
-      </c>
-      <c r="H56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A57" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B57" t="s">
-        <v>77</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="D57" t="s">
-        <v>12</v>
-      </c>
-      <c r="E57" t="s">
-        <v>27</v>
-      </c>
-      <c r="F57" t="s">
-        <v>2</v>
-      </c>
-      <c r="G57" t="s">
-        <v>183</v>
-      </c>
-      <c r="H57" t="s">
-        <v>11</v>
-      </c>
-      <c r="I57" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B58" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D58" t="s">
         <v>13</v>
       </c>
       <c r="E58" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="F58" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="G58" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="H58" t="s">
-        <v>11</v>
+        <v>84</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3214,345 +3184,107 @@
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B59" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="D59" t="s">
         <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="F59" t="s">
-        <v>2</v>
+        <v>180</v>
       </c>
       <c r="G59" t="s">
-        <v>183</v>
+        <v>102</v>
       </c>
       <c r="H59" t="s">
         <v>11</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A60" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B60" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D60" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="E60" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
       <c r="F60" t="s">
-        <v>17</v>
+        <v>180</v>
       </c>
       <c r="G60" t="s">
-        <v>118</v>
+        <v>102</v>
       </c>
       <c r="H60" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61" s="5">
-        <v>46127</v>
+        <v>46128</v>
       </c>
       <c r="B61" t="s">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="F61" t="s">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="G61" t="s">
-        <v>104</v>
+        <v>183</v>
       </c>
       <c r="H61" t="s">
         <v>11</v>
       </c>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A62" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B62" t="s">
-        <v>28</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D62" t="s">
-        <v>75</v>
-      </c>
-      <c r="E62" t="s">
-        <v>10</v>
-      </c>
-      <c r="F62" t="s">
-        <v>10</v>
-      </c>
-      <c r="G62" t="s">
-        <v>68</v>
-      </c>
-      <c r="H62" t="s">
-        <v>11</v>
-      </c>
-      <c r="I62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A63" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B63" t="s">
-        <v>28</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="D63" t="s">
-        <v>75</v>
-      </c>
-      <c r="E63" t="s">
-        <v>17</v>
-      </c>
-      <c r="F63" t="s">
-        <v>17</v>
-      </c>
-      <c r="G63" t="s">
-        <v>76</v>
-      </c>
-      <c r="H63" t="s">
-        <v>11</v>
-      </c>
-      <c r="I63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B64" t="s">
-        <v>78</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="D64" t="s">
-        <v>13</v>
-      </c>
-      <c r="E64" t="s">
-        <v>25</v>
-      </c>
-      <c r="F64" t="s">
-        <v>25</v>
-      </c>
-      <c r="G64" t="s">
-        <v>102</v>
-      </c>
-      <c r="H64" t="s">
-        <v>11</v>
-      </c>
-      <c r="I64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A65" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B65" t="s">
-        <v>78</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D65" t="s">
-        <v>12</v>
-      </c>
-      <c r="E65" t="s">
-        <v>56</v>
-      </c>
-      <c r="F65" t="s">
-        <v>56</v>
-      </c>
-      <c r="G65" t="s">
-        <v>154</v>
-      </c>
-      <c r="H65" t="s">
-        <v>11</v>
-      </c>
-      <c r="I65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A66" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B66" t="s">
-        <v>78</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D66" t="s">
-        <v>12</v>
-      </c>
-      <c r="E66" t="s">
-        <v>17</v>
-      </c>
-      <c r="F66" t="s">
-        <v>17</v>
-      </c>
-      <c r="G66" t="s">
-        <v>191</v>
-      </c>
-      <c r="H66" t="s">
-        <v>11</v>
-      </c>
-      <c r="I66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B67" t="s">
-        <v>78</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="D67" t="s">
-        <v>12</v>
-      </c>
-      <c r="E67" t="s">
-        <v>14</v>
-      </c>
-      <c r="F67" t="s">
-        <v>14</v>
-      </c>
-      <c r="G67" t="s">
-        <v>94</v>
-      </c>
-      <c r="H67" t="s">
-        <v>95</v>
-      </c>
-      <c r="I67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A68" s="5">
-        <v>46127</v>
-      </c>
-      <c r="B68" t="s">
-        <v>78</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D68" t="s">
-        <v>12</v>
-      </c>
-      <c r="E68" t="s">
-        <v>10</v>
-      </c>
-      <c r="F68" t="s">
-        <v>10</v>
-      </c>
-      <c r="G68" t="s">
-        <v>68</v>
-      </c>
-      <c r="H68" t="s">
-        <v>11</v>
-      </c>
-      <c r="I68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J68" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>

</xml_diff>

<commit_message>
Reporte 21 de abril
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66005485-087A-4EEF-9783-51B82615E70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E93A6EE-0F2B-4F9E-BA2F-5AC885091CAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="198">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="189">
   <si>
     <t>Fecha</t>
   </si>
@@ -288,349 +288,322 @@
     <t>Positiva</t>
   </si>
   <si>
-    <t>Mundial De Futbol</t>
-  </si>
-  <si>
     <t>La Jornada Hidalgo</t>
   </si>
   <si>
-    <t>Alianzas Electorales</t>
-  </si>
-  <si>
     <t>Tauromaquia</t>
   </si>
   <si>
     <t>Sipdus</t>
   </si>
   <si>
-    <t>Tren México Querétaro</t>
-  </si>
-  <si>
-    <t>Sucesión alcaldía</t>
-  </si>
-  <si>
-    <t>Regidor</t>
-  </si>
-  <si>
     <t>Alerta Meteorológica</t>
   </si>
   <si>
-    <t>Inhide</t>
-  </si>
-  <si>
     <t>Día del Niño</t>
   </si>
   <si>
     <t>Alcalde</t>
   </si>
   <si>
-    <t>OEEH</t>
-  </si>
-  <si>
-    <t>Expo feria</t>
-  </si>
-  <si>
     <t>Rehabilitación Vial</t>
   </si>
   <si>
     <t>Temas internacionales</t>
   </si>
   <si>
-    <t>Siguen hallando restos históricos</t>
-  </si>
-  <si>
-    <t>Festival de danza reúne a más de 400 bailarines</t>
-  </si>
-  <si>
-    <t>Festival Cultural</t>
-  </si>
-  <si>
-    <t>Registra Hidalgo alto riesgo de inundación</t>
-  </si>
-  <si>
-    <t>Prevención De Riesgos</t>
-  </si>
-  <si>
-    <t>Señalan inseguridad en paraderos públicos</t>
-  </si>
-  <si>
-    <t>Movilidad urbana</t>
-  </si>
-  <si>
-    <t>Limpia y restaurada luce plaza recuperada</t>
-  </si>
-  <si>
     <t>Recuperación De Espacios Públicos</t>
   </si>
   <si>
-    <t>Inician preparativos para el Día del Niño</t>
-  </si>
-  <si>
-    <t>Vuelve a brillar</t>
-  </si>
-  <si>
-    <t>Colonias en MR en riesgo por deslaves e inundaciones</t>
-  </si>
-  <si>
-    <t>Participación ciudadana, reto del INE</t>
-  </si>
-  <si>
-    <t>Elecciones</t>
-  </si>
-  <si>
-    <t>Baja la incidencia delictiva en 2026</t>
-  </si>
-  <si>
-    <t>Incidencia Delictiva</t>
-  </si>
-  <si>
-    <t>Van cuatro suicidios de estudiantes</t>
-  </si>
-  <si>
-    <t>Suicidio Estudiante</t>
-  </si>
-  <si>
-    <t>Operativo en Cuautepec deja a dos detenidos</t>
-  </si>
-  <si>
-    <t>Combate a la delincuencia</t>
-  </si>
-  <si>
-    <t>Sigue Hidalgo en primer lugar en Huachicoleo</t>
-  </si>
-  <si>
-    <t>Huachicol</t>
-  </si>
-  <si>
-    <t>El dirigente del PRI niega precandidatos para Pachuca</t>
-  </si>
-  <si>
-    <t>PRI</t>
-  </si>
-  <si>
-    <t>Sin sentencia, 29% de los feminicidios</t>
-  </si>
-  <si>
-    <t>Feminicidio</t>
-  </si>
-  <si>
-    <t>Reescriben su pasado</t>
-  </si>
-  <si>
     <t>Deportes</t>
   </si>
   <si>
-    <t>CLAUSURARON ESPECTACULARES EN LA REFORMA</t>
-  </si>
-  <si>
-    <t>Imagen Urbana</t>
-  </si>
-  <si>
-    <t>Meten emoción a la Premiere</t>
-  </si>
-  <si>
-    <t>ELIGIERON AL NUEVO América P10 3 P12 3 LÍDER DEL SUTSPEEH</t>
-  </si>
-  <si>
-    <t>Dirigencia SUTSPEEH</t>
-  </si>
-  <si>
-    <t>Buscan a 33 hidalguenses con ficha roja vigente de Interpol</t>
-  </si>
-  <si>
-    <t>Ficha De Búsqueda</t>
-  </si>
-  <si>
-    <t>Reportan baja en número de carpetas de investigación</t>
-  </si>
-  <si>
-    <t>La SSPH desmantela bodega de autopartes</t>
-  </si>
-  <si>
-    <t>Invertirá estado 28 mmdp en 2026, anuncia Menchaca</t>
-  </si>
-  <si>
-    <t>Disfrutan turistas de paseo por el Corredor de la Sierra</t>
-  </si>
-  <si>
-    <t>ASEH realiza observaciones a exalcaldesa de Tizayuca</t>
-  </si>
-  <si>
-    <t>ASEH</t>
-  </si>
-  <si>
-    <t>Observaciones ASEH</t>
-  </si>
-  <si>
-    <t>El estado se declara listo para albergar torneos</t>
-  </si>
-  <si>
-    <t>Revelan hoy avance en 48 de 54 temas del T-MEC que fueron cuestionados por EU</t>
-  </si>
-  <si>
-    <t>Resguardan especies protegidas tras aseguramiento</t>
-  </si>
-  <si>
-    <t>Rescate de especies</t>
-  </si>
-  <si>
-    <t>Salud mental: ellos se resisten a buscar ayuda</t>
-  </si>
-  <si>
-    <t>Atención Socioemocional</t>
-  </si>
-  <si>
-    <t>Crecen delitos contra la vida y lesiones en marzo</t>
-  </si>
-  <si>
-    <t>Reyes anticipa nueva intervención en Jardín del Arte</t>
-  </si>
-  <si>
-    <t>CSP refrenda cooperación para Coatlicue</t>
-  </si>
-  <si>
-    <t>Concluye la Feria Ganadera</t>
-  </si>
-  <si>
-    <t>Ahora, cuando parece moda hablar de soberanía, sumemos al tema  el uso cotidiano de nuestra lengua para privilegiarlo, y la asimilación  de otras imprescindibles a las actividades económicas, profesionales y  culturales: vivamos el español”.</t>
-  </si>
-  <si>
-    <t>Hidalgo entre los estados más seguros del país,  según organismo federal</t>
-  </si>
-  <si>
-    <t>Detienen en Tizayuca a presunto feminicida de Veracruz</t>
-  </si>
-  <si>
-    <t>Detención Feminicida</t>
-  </si>
-  <si>
-    <t>Buscarán triunfar estudiantes hidalguenses en concurso internacional</t>
-  </si>
-  <si>
-    <t>Campeonato de robótica</t>
-  </si>
-  <si>
-    <t>Pronostican lluvias fuertes en Hidalgo ante paso de frente frío 45</t>
-  </si>
-  <si>
-    <t>Conagua</t>
-  </si>
-  <si>
-    <t>No habrá alianzas a nivel nacional: Samperio</t>
-  </si>
-  <si>
-    <t>SSPH desarticula bodega con autopartes y droga: dos detenidos</t>
-  </si>
-  <si>
-    <t>Locatarios del laminado denuncias faltas a la moral en el sector</t>
-  </si>
-  <si>
-    <t>Abanderan a estudiantes de Hidalgo rumbo al mundial de robótica VEX</t>
-  </si>
-  <si>
-    <t>PILARES significan un punto de innovación y de encuentro: Anabel Mateos</t>
-  </si>
-  <si>
-    <t>Pilares</t>
-  </si>
-  <si>
-    <t>Gobierno constructores van juntos</t>
-  </si>
-  <si>
-    <t>Reunión Con Empresarios</t>
-  </si>
-  <si>
-    <t>Estamos rescatando y ordenando nuestros espacios públicos"": Jorge Reyes</t>
-  </si>
-  <si>
-    <t>Capturan a ""El Bukanas""</t>
-  </si>
-  <si>
-    <t>Procuraduría Agraria</t>
-  </si>
-  <si>
-    <t>Detención</t>
-  </si>
-  <si>
-    <t>Taurinos acusan intereses políticos y económicos</t>
-  </si>
-  <si>
-    <t>GLPVEM</t>
-  </si>
-  <si>
-    <t>Incautan red de inmuebles de desmantelamiento</t>
-  </si>
-  <si>
-    <t>Bomberos de Tula atienden parto en terminal de microbuses</t>
-  </si>
-  <si>
-    <t>Atención a la ciudadanía</t>
-  </si>
-  <si>
-    <t>El talento de la niñez transforma Atitalaquia con respaldo de Claudia Sandoval</t>
-  </si>
-  <si>
-    <t>Junto a la CMIC, Menchaca fortalece infraestructura de Hidalgo</t>
-  </si>
-  <si>
-    <t>Policía de Hidalgo desarticula bodega utilizada para almacenar autopartes y desmantelar vehículos robados en Cuautepec</t>
-  </si>
-  <si>
-    <t>Tras 25 años de abandono, el rastro municipal de Tula se transforma en el gobierno de Cristhian Martínez</t>
-  </si>
-  <si>
-    <t>Rastro municipal</t>
-  </si>
-  <si>
-    <t>Policías de Pachuca detienen a ""Spiderman""</t>
-  </si>
-  <si>
-    <t>Policía municipal</t>
-  </si>
-  <si>
-    <t>Diputado Alejandro Alcántara recibe a cooperativas en el Primer Encuentro por la Economía Social y el Cooperativismo</t>
-  </si>
-  <si>
-    <t>Economía social</t>
-  </si>
-  <si>
-    <t>Juntos llenaron de ritmo la Ganadera 2026</t>
-  </si>
-  <si>
-    <t>Aseguran a sujeto por pintar bancas recién rehabilitadas en plaza</t>
-  </si>
-  <si>
-    <t>Pancho Barraza dio cerrojazo de nuevo festejo en Hidalgo</t>
-  </si>
-  <si>
-    <t>Detienen en Hidalgo a presunto feminicida de Veracruz</t>
-  </si>
-  <si>
-    <t>SSPH desarticula bodega utilizada para almacenar autopartes y desmantelar vehículos robados</t>
-  </si>
-  <si>
-    <t>GREGJOSH salón de eventos</t>
-  </si>
-  <si>
-    <t>Aseguran predios; almacenaban autopartes y desarmaban autos</t>
-  </si>
-  <si>
-    <t>Presenta pachuqueña degustación gastronómica en París</t>
-  </si>
-  <si>
-    <t>Festival Gastronómico</t>
-  </si>
-  <si>
-    <t>¿Por qué reparan calles en Pachuca sólo a la mitad, mientras las otras partes en pésimas condiciones? Hay gato encerrado en esto, no cabe duda...</t>
-  </si>
-  <si>
     <t>Editorial</t>
   </si>
   <si>
-    <t>Exigen regidores de Cuautepec rendición de cuentas</t>
-  </si>
-  <si>
-    <t>Transparencia</t>
+    <t>Concentra Tula la mitad del PIB industrial</t>
+  </si>
+  <si>
+    <t>Rehabilitan circulación vial en calles</t>
+  </si>
+  <si>
+    <t>Streaming impacta economía de usuarios</t>
+  </si>
+  <si>
+    <t>Caxuxi seguirá con las corridas de toros</t>
+  </si>
+  <si>
+    <t>Aumentan fraudes financieros digitales</t>
+  </si>
+  <si>
+    <t>Alerta De Fraude</t>
+  </si>
+  <si>
+    <t>Celebrarán la niñez con futbol y diversión</t>
+  </si>
+  <si>
+    <t>Recuperan 385 inmuebles de 2022 a 2026 en Hidalgo</t>
+  </si>
+  <si>
+    <t>Gobierno estatal recuera más de 385 inmuebles y va por otros 51</t>
+  </si>
+  <si>
+    <t>Regresa la vida</t>
+  </si>
+  <si>
+    <t>Reloj De Pachuca</t>
+  </si>
+  <si>
+    <t>Anuncian nuevo museo en Pachuca</t>
+  </si>
+  <si>
+    <t>titular</t>
+  </si>
+  <si>
+    <t>Museo de la Ciudad</t>
+  </si>
+  <si>
+    <t>INE abre vacantes en el Consejo local</t>
+  </si>
+  <si>
+    <t>oitros</t>
+  </si>
+  <si>
+    <t>Consejeros Electorales</t>
+  </si>
+  <si>
+    <t>Para nadie fue una sorpresa que desde Palacio Nacional se anunciara la salida de Citlalli Hernández Mora de la Secretaría de Mujeres para i n co rp o ra rse. . . ”</t>
+  </si>
+  <si>
+    <t>Nombramientos</t>
+  </si>
+  <si>
+    <t>Criterio</t>
+  </si>
+  <si>
+    <t>La cifra mágica</t>
+  </si>
+  <si>
+    <t>LOS REYES DEL DEPORTE  BRILLAN EN LOS LAUREUS</t>
+  </si>
+  <si>
+    <t>RENTARÁN 60 UNIDADES MÁS PARA EL TUZOBÚS</t>
+  </si>
+  <si>
+    <t>Ampliación Tuzobús</t>
+  </si>
+  <si>
+    <t>Por cafetería sin permisos FACH perdió el comodato</t>
+  </si>
+  <si>
+    <t>Fundación Arturo Herrera</t>
+  </si>
+  <si>
+    <t>SE INVERTIRÁN 20 MDP PARA REHABILITACIÓN DE PARQUES</t>
+  </si>
+  <si>
+    <t>OCSAD</t>
+  </si>
+  <si>
+    <t>Mañanera de Hidalgo</t>
+  </si>
+  <si>
+    <t>Implementarán sistema digital de multas: Reyes</t>
+  </si>
+  <si>
+    <t>Multas</t>
+  </si>
+  <si>
+    <t>Recupera el estado patrimonio; 385 inmuebles por 1,230 mdp</t>
+  </si>
+  <si>
+    <t>Del gueto de Varsovia a Auschwitz</t>
+  </si>
+  <si>
+    <t>Aseguran más de 10 mil dosis de drogas y detienen a 32</t>
+  </si>
+  <si>
+    <t>Reunión Gabinete De Seguridad</t>
+  </si>
+  <si>
+    <t>Claudia quiere acuerdo en aluminio, acero y vehículos antes de revisión del T-Mec</t>
+  </si>
+  <si>
+    <t>Un viaje por el laberinto mágico y onírico de Leonora Carrington</t>
+  </si>
+  <si>
+    <t>El Niño puede prolongar periodo sin lluvias: PC</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>Abren céntrica calle de Morelos tras rehabilitación</t>
+  </si>
+  <si>
+    <t>Hidalgo recupera 385 inmuebles y suma a su patrimonio 1,230 mdp</t>
+  </si>
+  <si>
+    <t>Unidades del Tuzobús comenzarán en mayo</t>
+  </si>
+  <si>
+    <t>Desconocen  quehacer de  personal de  la embajada  de EU en México</t>
+  </si>
+  <si>
+    <t>No creo que alguien piense que gobernar es fácil, hay muchas cuestiones administrativas y  presupuestales que ralentizan esta tarea; sin embargo, creo que cuando se hace con convicción y  realmente con el pueblo (…), las cosas podrían salir mejor”.</t>
+  </si>
+  <si>
+    <t>Urge revisión de Gestión de Riesgos en inmueble ocupado por la FAHC: PC</t>
+  </si>
+  <si>
+    <t>Reincorpora Hidalgo a su patrimonio 85 inmuebles valuados por mil 230 mdp</t>
+  </si>
+  <si>
+    <t>Van por la renta de 60 unidades  más para Tuzobús; alcanzarán las 140</t>
+  </si>
+  <si>
+    <t>Regresarán murales al Jardín del Arte de Pachuca; participarán ocho artistas</t>
+  </si>
+  <si>
+    <t>Muralismo</t>
+  </si>
+  <si>
+    <t>INMUEBLE DE LA CALLE DE ALLENDE EN PACHUCA, REQUIERE INSPECCION MULTIDISCIPLINARIA</t>
+  </si>
+  <si>
+    <t>Flores Especiales"" buscan la inclusión en Atlapexco</t>
+  </si>
+  <si>
+    <t>Inclusión</t>
+  </si>
+  <si>
+    <t>Habitantes del Parque de Poblamiento se pronuncian contra delegado</t>
+  </si>
+  <si>
+    <t>Club de Leones entrega despensa</t>
+  </si>
+  <si>
+    <t>Reglamentos reordena a vendedores ambulantes</t>
+  </si>
+  <si>
+    <t>Ambulantaje</t>
+  </si>
+  <si>
+    <t>Combaten la violencia de género durante la Jornada por la Paz y Bienestar del Pueblo</t>
+  </si>
+  <si>
+    <t>Jornada por la paz</t>
+  </si>
+  <si>
+    <t>Gobernar implica ordenar"": Oficial Mayor</t>
+  </si>
+  <si>
+    <t>La Fundación: entre la cultura y la ley</t>
+  </si>
+  <si>
+    <t>Combaten al crimen</t>
+  </si>
+  <si>
+    <t>Pachuca destinará 20 millones para parques en 2026</t>
+  </si>
+  <si>
+    <t>Solo representan 28 hoteles""</t>
+  </si>
+  <si>
+    <t>Ocupación Hotelera</t>
+  </si>
+  <si>
+    <t>Juez frena multa de la Auditoría contra rector de la UAEH</t>
+  </si>
+  <si>
+    <t>2 personas sin vida y 15 lesionados en Balacera en Teotihuacán</t>
+  </si>
+  <si>
+    <t>Cintillo</t>
+  </si>
+  <si>
+    <t>Ataque Armado</t>
+  </si>
+  <si>
+    <t>Instalan Consejo Municipal de Participación</t>
+  </si>
+  <si>
+    <t>Espacios recuperados, para uso de todos, apuesta de Gobierno de Hidalgo y Pachuca</t>
+  </si>
+  <si>
+    <t>Entregan apoyos productivos para fortalecer el campo en Ajacuba</t>
+  </si>
+  <si>
+    <t>Apoyo Al Agro</t>
+  </si>
+  <si>
+    <t>Gobierno de Atotonilco invertirá 32 mdp en 2a etapa de modernización de la carretera Progreso</t>
+  </si>
+  <si>
+    <t>Rehabilitación carretera</t>
+  </si>
+  <si>
+    <t>La máquina volvió a Cruz Azul</t>
+  </si>
+  <si>
+    <t>Fortalecen el deporte en Tlahuelilpan con encuentro entre autoridades y atletas</t>
+  </si>
+  <si>
+    <t>Fomento Al Deporte</t>
+  </si>
+  <si>
+    <t>Said Vargas apuesta por consolidar la unión sindical bajo la responsabilidad institucional</t>
+  </si>
+  <si>
+    <t>Gobiernos de Hidalgo y Pachuca recuperan espacios públicos</t>
+  </si>
+  <si>
+    <t>Estudiantes de la UPP crean sistema inteligente para reducir consumo eléctrico en Hogares</t>
+  </si>
+  <si>
+    <t>Universidades</t>
+  </si>
+  <si>
+    <t>Innovación</t>
+  </si>
+  <si>
+    <t>OSEH y banda sinfónica presentan doble jornada musical esta semana</t>
+  </si>
+  <si>
+    <t>Orquesta Sinfónica</t>
+  </si>
+  <si>
+    <t>Gabinete de Seguridad asegura más de 10 mil estupefacientes y detiene a 32 personas</t>
+  </si>
+  <si>
+    <t>UAEH abre convocatoria para profesores investigadores de tiempo completo</t>
+  </si>
+  <si>
+    <t>Convocatoria</t>
+  </si>
+  <si>
+    <t>Gregjosh salón de eventos</t>
+  </si>
+  <si>
+    <t>Publicidad comercial</t>
+  </si>
+  <si>
+    <t>Tiroteo en Teotihuacán deja dos muertos</t>
+  </si>
+  <si>
+    <t>Fundación Arturo Herrera cabe en el nuevo Museo""</t>
+  </si>
+  <si>
+    <t>Una gran desgracia para México el ataque terrorista en Teotihuacán, que deja mal parado a nuestro país en el mundo, donde se comenta la criminalidad a gran escala que se vive aquí diariamente...</t>
+  </si>
+  <si>
+    <t>Aseguraron a 32 delincuentes en una semana</t>
+  </si>
+  <si>
+    <t>Surge desacuerdo entre regidor de Tula y Miguel Tello</t>
+  </si>
+  <si>
+    <t>Desavenencias</t>
   </si>
 </sst>
 </file>
@@ -877,8 +850,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J67" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J67" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J66" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J66" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1244,22 +1217,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J67"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J66"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.7265625" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1291,61 +1264,61 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B2" t="s">
         <v>79</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B3" t="s">
         <v>79</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>30</v>
+        <v>85</v>
       </c>
       <c r="G3" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
@@ -1359,268 +1332,268 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B4" t="s">
         <v>79</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B5" t="s">
         <v>79</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B6" t="s">
         <v>79</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F6" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="H6" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B7" t="s">
         <v>79</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="F7" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="H7" t="s">
         <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="G8" t="s">
-        <v>107</v>
+        <v>91</v>
       </c>
       <c r="H8" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B9" t="s">
         <v>69</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
       </c>
       <c r="E9" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="F9" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B10" t="s">
         <v>69</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B11" t="s">
         <v>69</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
-        <v>18</v>
+        <v>106</v>
       </c>
       <c r="G11" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="H11" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1631,367 +1604,367 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B12" t="s">
         <v>69</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F12" t="s">
-        <v>27</v>
+        <v>109</v>
       </c>
       <c r="G12" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="H12" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B13" t="s">
         <v>69</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="G13" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B14" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
       </c>
       <c r="E14" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F14" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G14" t="s">
-        <v>120</v>
+        <v>92</v>
       </c>
       <c r="H14" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>122</v>
+        <v>10</v>
       </c>
       <c r="F15" t="s">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="G15" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Otros</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B16" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="D16" t="s">
         <v>13</v>
       </c>
       <c r="E16" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F16" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="G16" t="s">
+        <v>117</v>
+      </c>
+      <c r="H16" t="s">
+        <v>11</v>
+      </c>
+      <c r="I16" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J16" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B17" t="s">
+        <v>113</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" t="s">
+        <v>24</v>
+      </c>
+      <c r="G17" t="s">
+        <v>119</v>
+      </c>
+      <c r="H17" t="s">
+        <v>11</v>
+      </c>
+      <c r="I17" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J17" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B18" t="s">
+        <v>113</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>121</v>
+      </c>
+      <c r="F18" t="s">
+        <v>121</v>
+      </c>
+      <c r="G18" t="s">
+        <v>122</v>
+      </c>
+      <c r="H18" t="s">
+        <v>11</v>
+      </c>
+      <c r="I18" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>No indexado</v>
+      </c>
+      <c r="J18" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B19" t="s">
+        <v>113</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" t="s">
+        <v>88</v>
+      </c>
+      <c r="G19" t="s">
         <v>124</v>
       </c>
-      <c r="H16" t="s">
-        <v>16</v>
-      </c>
-      <c r="I16" t="str">
+      <c r="H19" t="s">
+        <v>11</v>
+      </c>
+      <c r="I19" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J19" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B20" t="s">
+        <v>73</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20" t="s">
+        <v>22</v>
+      </c>
+      <c r="G20" t="s">
+        <v>91</v>
+      </c>
+      <c r="H20" t="s">
+        <v>11</v>
+      </c>
+      <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J16" t="str">
+      <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A17" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B17" t="s">
-        <v>69</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" t="s">
-        <v>10</v>
-      </c>
-      <c r="G17" t="s">
-        <v>126</v>
-      </c>
-      <c r="H17" t="s">
-        <v>11</v>
-      </c>
-      <c r="I17" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J17" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B18" t="s">
-        <v>69</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D18" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" t="s">
-        <v>17</v>
-      </c>
-      <c r="F18" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18" t="s">
-        <v>128</v>
-      </c>
-      <c r="H18" t="s">
-        <v>11</v>
-      </c>
-      <c r="I18" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J18" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A19" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B19" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="D19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" t="s">
-        <v>10</v>
-      </c>
-      <c r="F19" t="s">
-        <v>10</v>
-      </c>
-      <c r="G19" t="s">
-        <v>126</v>
-      </c>
-      <c r="H19" t="s">
-        <v>11</v>
-      </c>
-      <c r="I19" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J19" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A20" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B20" t="s">
-        <v>69</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="D20" t="s">
-        <v>12</v>
-      </c>
-      <c r="E20" t="s">
-        <v>41</v>
-      </c>
-      <c r="F20" t="s">
-        <v>41</v>
-      </c>
-      <c r="G20" t="s">
-        <v>131</v>
-      </c>
-      <c r="H20" t="s">
-        <v>11</v>
-      </c>
-      <c r="I20" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J20" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B21" t="s">
         <v>73</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G21" t="s">
-        <v>133</v>
+        <v>68</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B22" t="s">
         <v>73</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="F22" t="s">
-        <v>18</v>
+        <v>25</v>
       </c>
       <c r="G22" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
@@ -2002,645 +1975,645 @@
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B23" t="s">
         <v>73</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F23" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G23" t="s">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B24" t="s">
         <v>73</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F24" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B25" t="s">
         <v>73</v>
       </c>
       <c r="C25" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>24</v>
+      </c>
+      <c r="F25" t="s">
+        <v>132</v>
+      </c>
+      <c r="G25" t="s">
+        <v>86</v>
+      </c>
+      <c r="H25" t="s">
+        <v>11</v>
+      </c>
+      <c r="I25" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J25" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B26" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D26" t="s">
+        <v>9</v>
+      </c>
+      <c r="E26" t="s">
+        <v>85</v>
+      </c>
+      <c r="F26" t="s">
+        <v>85</v>
+      </c>
+      <c r="G26" t="s">
+        <v>89</v>
+      </c>
+      <c r="H26" t="s">
+        <v>11</v>
+      </c>
+      <c r="I26" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J26" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B27" t="s">
+        <v>83</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
+        <v>22</v>
+      </c>
+      <c r="F27" t="s">
+        <v>22</v>
+      </c>
+      <c r="G27" t="s">
+        <v>91</v>
+      </c>
+      <c r="H27" t="s">
+        <v>11</v>
+      </c>
+      <c r="I27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B28" t="s">
+        <v>83</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>22</v>
+      </c>
+      <c r="F28" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28" t="s">
+        <v>117</v>
+      </c>
+      <c r="H28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B29" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D29" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" t="s">
+        <v>14</v>
+      </c>
+      <c r="F29" t="s">
+        <v>14</v>
+      </c>
+      <c r="G29" t="s">
+        <v>90</v>
+      </c>
+      <c r="H29" t="s">
+        <v>11</v>
+      </c>
+      <c r="I29" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J29" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B30" t="s">
+        <v>83</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="D25" t="s">
-        <v>9</v>
-      </c>
-      <c r="E25" t="s">
+      <c r="D30" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" t="s">
+        <v>41</v>
+      </c>
+      <c r="F30" t="s">
+        <v>41</v>
+      </c>
+      <c r="G30" t="s">
+        <v>107</v>
+      </c>
+      <c r="H30" t="s">
+        <v>11</v>
+      </c>
+      <c r="I30" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J30" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31" t="s">
+        <v>132</v>
+      </c>
+      <c r="G31" t="s">
+        <v>119</v>
+      </c>
+      <c r="H31" t="s">
+        <v>11</v>
+      </c>
+      <c r="I31" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J31" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A32" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B32" t="s">
+        <v>70</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="D32" t="s">
+        <v>12</v>
+      </c>
+      <c r="E32" t="s">
+        <v>22</v>
+      </c>
+      <c r="F32" t="s">
+        <v>22</v>
+      </c>
+      <c r="G32" t="s">
+        <v>91</v>
+      </c>
+      <c r="H32" t="s">
+        <v>11</v>
+      </c>
+      <c r="I32" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J32" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B33" t="s">
+        <v>70</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D33" t="s">
+        <v>12</v>
+      </c>
+      <c r="E33" t="s">
+        <v>22</v>
+      </c>
+      <c r="F33" t="s">
+        <v>22</v>
+      </c>
+      <c r="G33" t="s">
+        <v>117</v>
+      </c>
+      <c r="H33" t="s">
+        <v>11</v>
+      </c>
+      <c r="I33" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J33" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D34" t="s">
+        <v>12</v>
+      </c>
+      <c r="E34" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" t="s">
+        <v>17</v>
+      </c>
+      <c r="G34" t="s">
+        <v>142</v>
+      </c>
+      <c r="H34" t="s">
+        <v>11</v>
+      </c>
+      <c r="I34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A35" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B35" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D35" t="s">
+        <v>12</v>
+      </c>
+      <c r="E35" t="s">
+        <v>24</v>
+      </c>
+      <c r="F35" t="s">
+        <v>132</v>
+      </c>
+      <c r="G35" t="s">
+        <v>119</v>
+      </c>
+      <c r="H35" t="s">
+        <v>11</v>
+      </c>
+      <c r="I35" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J35" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A36" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B36" t="s">
+        <v>78</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="D36" t="s">
+        <v>12</v>
+      </c>
+      <c r="E36" t="s">
         <v>10</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F36" t="s">
         <v>10</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G36" t="s">
+        <v>145</v>
+      </c>
+      <c r="H36" t="s">
+        <v>11</v>
+      </c>
+      <c r="I36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J36" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B37" t="s">
+        <v>78</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>146</v>
+      </c>
+      <c r="D37" t="s">
+        <v>13</v>
+      </c>
+      <c r="E37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" t="s">
+        <v>17</v>
+      </c>
+      <c r="G37" t="s">
         <v>68</v>
       </c>
-      <c r="H25" t="s">
-        <v>11</v>
-      </c>
-      <c r="I25" t="str">
+      <c r="H37" t="s">
+        <v>11</v>
+      </c>
+      <c r="I37" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J37" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A38" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B38" t="s">
+        <v>78</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D38" t="s">
+        <v>12</v>
+      </c>
+      <c r="E38" t="s">
+        <v>10</v>
+      </c>
+      <c r="F38" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" t="s">
+        <v>68</v>
+      </c>
+      <c r="H38" t="s">
+        <v>11</v>
+      </c>
+      <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J25" t="str">
+      <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A26" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B26" t="s">
-        <v>73</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="D26" t="s">
-        <v>12</v>
-      </c>
-      <c r="E26" t="s">
-        <v>36</v>
-      </c>
-      <c r="F26" t="s">
-        <v>139</v>
-      </c>
-      <c r="G26" t="s">
-        <v>140</v>
-      </c>
-      <c r="H26" t="s">
-        <v>11</v>
-      </c>
-      <c r="I26" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J26" t="str">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B39" t="s">
+        <v>78</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D39" t="s">
+        <v>12</v>
+      </c>
+      <c r="E39" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" t="s">
+        <v>149</v>
+      </c>
+      <c r="H39" t="s">
+        <v>11</v>
+      </c>
+      <c r="I39" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A27" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B27" t="s">
-        <v>73</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="D27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" t="s">
-        <v>27</v>
-      </c>
-      <c r="F27" t="s">
-        <v>92</v>
-      </c>
-      <c r="G27" t="s">
-        <v>83</v>
-      </c>
-      <c r="H27" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A28" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B28" t="s">
-        <v>73</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="D28" t="s">
-        <v>12</v>
-      </c>
-      <c r="E28" t="s">
-        <v>14</v>
-      </c>
-      <c r="F28" t="s">
-        <v>14</v>
-      </c>
-      <c r="G28" t="s">
-        <v>98</v>
-      </c>
-      <c r="H28" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A29" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B29" t="s">
-        <v>73</v>
-      </c>
-      <c r="C29" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="D29" t="s">
-        <v>12</v>
-      </c>
-      <c r="E29" t="s">
-        <v>21</v>
-      </c>
-      <c r="F29" t="s">
-        <v>21</v>
-      </c>
-      <c r="G29" t="s">
-        <v>144</v>
-      </c>
-      <c r="H29" t="s">
-        <v>11</v>
-      </c>
-      <c r="I29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J29" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A30" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B30" t="s">
-        <v>73</v>
-      </c>
-      <c r="C30" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="D30" t="s">
-        <v>12</v>
-      </c>
-      <c r="E30" t="s">
-        <v>10</v>
-      </c>
-      <c r="F30" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" t="s">
-        <v>146</v>
-      </c>
-      <c r="H30" t="s">
-        <v>11</v>
-      </c>
-      <c r="I30" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J30" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A31" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B31" t="s">
-        <v>84</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="D31" t="s">
-        <v>12</v>
-      </c>
-      <c r="E31" t="s">
-        <v>18</v>
-      </c>
-      <c r="F31" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" t="s">
-        <v>114</v>
-      </c>
-      <c r="H31" t="s">
-        <v>11</v>
-      </c>
-      <c r="I31" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J31" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A32" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B32" t="s">
-        <v>84</v>
-      </c>
-      <c r="C32" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="D32" t="s">
-        <v>13</v>
-      </c>
-      <c r="E32" t="s">
-        <v>17</v>
-      </c>
-      <c r="F32" t="s">
-        <v>94</v>
-      </c>
-      <c r="G32" t="s">
-        <v>107</v>
-      </c>
-      <c r="H32" t="s">
-        <v>11</v>
-      </c>
-      <c r="I32" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J32" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A33" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B33" t="s">
-        <v>84</v>
-      </c>
-      <c r="C33" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D33" t="s">
-        <v>12</v>
-      </c>
-      <c r="E33" t="s">
-        <v>14</v>
-      </c>
-      <c r="F33" t="s">
-        <v>14</v>
-      </c>
-      <c r="G33" t="s">
-        <v>98</v>
-      </c>
-      <c r="H33" t="s">
-        <v>11</v>
-      </c>
-      <c r="I33" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J33" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A34" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B34" t="s">
-        <v>84</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>150</v>
-      </c>
-      <c r="D34" t="s">
-        <v>9</v>
-      </c>
-      <c r="E34" t="s">
-        <v>31</v>
-      </c>
-      <c r="F34" t="s">
-        <v>95</v>
-      </c>
-      <c r="G34" t="s">
-        <v>96</v>
-      </c>
-      <c r="H34" t="s">
-        <v>11</v>
-      </c>
-      <c r="I34" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J34" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="58" x14ac:dyDescent="0.35">
-      <c r="A35" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B35" t="s">
-        <v>84</v>
-      </c>
-      <c r="C35" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="D35" t="s">
-        <v>12</v>
-      </c>
-      <c r="E35" t="s">
-        <v>10</v>
-      </c>
-      <c r="F35" t="s">
-        <v>10</v>
-      </c>
-      <c r="G35" t="s">
-        <v>68</v>
-      </c>
-      <c r="H35" t="s">
-        <v>11</v>
-      </c>
-      <c r="I35" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J35" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A36" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B36" t="s">
-        <v>70</v>
-      </c>
-      <c r="C36" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="D36" t="s">
-        <v>13</v>
-      </c>
-      <c r="E36" t="s">
-        <v>18</v>
-      </c>
-      <c r="F36" t="s">
-        <v>18</v>
-      </c>
-      <c r="G36" t="s">
-        <v>114</v>
-      </c>
-      <c r="H36" t="s">
-        <v>82</v>
-      </c>
-      <c r="I36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J36" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A37" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B37" t="s">
-        <v>70</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="D37" t="s">
-        <v>12</v>
-      </c>
-      <c r="E37" t="s">
-        <v>23</v>
-      </c>
-      <c r="F37" t="s">
-        <v>23</v>
-      </c>
-      <c r="G37" t="s">
-        <v>154</v>
-      </c>
-      <c r="H37" t="s">
-        <v>11</v>
-      </c>
-      <c r="I37" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J37" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A38" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B38" t="s">
-        <v>70</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="D38" t="s">
-        <v>12</v>
-      </c>
-      <c r="E38" t="s">
-        <v>27</v>
-      </c>
-      <c r="F38" t="s">
-        <v>2</v>
-      </c>
-      <c r="G38" t="s">
-        <v>156</v>
-      </c>
-      <c r="H38" t="s">
-        <v>11</v>
-      </c>
-      <c r="I38" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J38" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A39" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B39" t="s">
-        <v>70</v>
-      </c>
-      <c r="C39" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="D39" t="s">
-        <v>12</v>
-      </c>
-      <c r="E39" t="s">
-        <v>14</v>
-      </c>
-      <c r="F39" t="s">
-        <v>158</v>
-      </c>
-      <c r="G39" t="s">
-        <v>91</v>
-      </c>
-      <c r="H39" t="s">
-        <v>11</v>
-      </c>
-      <c r="I39" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J39" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B40" t="s">
         <v>78</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>159</v>
+        <v>150</v>
       </c>
       <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
+        <v>24</v>
+      </c>
+      <c r="F40" t="s">
+        <v>24</v>
+      </c>
+      <c r="G40" t="s">
+        <v>151</v>
+      </c>
+      <c r="H40" t="s">
+        <v>11</v>
+      </c>
+      <c r="I40" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J40" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A41" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B41" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="D41" t="s">
         <v>13</v>
       </c>
-      <c r="E40" t="s">
-        <v>46</v>
-      </c>
-      <c r="F40" t="s">
-        <v>46</v>
-      </c>
-      <c r="G40" t="s">
-        <v>85</v>
-      </c>
-      <c r="H40" t="s">
-        <v>11</v>
-      </c>
-      <c r="I40" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J40" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A41" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B41" t="s">
-        <v>78</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D41" t="s">
-        <v>12</v>
-      </c>
       <c r="E41" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F41" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="G41" t="s">
-        <v>118</v>
+        <v>91</v>
       </c>
       <c r="H41" t="s">
-        <v>11</v>
+        <v>82</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2651,61 +2624,61 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B42" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="F42" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="G42" t="s">
-        <v>68</v>
+        <v>119</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B43" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F43" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G43" t="s">
-        <v>156</v>
+        <v>128</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
@@ -2716,18 +2689,18 @@
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B44" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D44" t="s">
         <v>12</v>
@@ -2739,7 +2712,7 @@
         <v>17</v>
       </c>
       <c r="G44" t="s">
-        <v>164</v>
+        <v>122</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
@@ -2753,30 +2726,30 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B45" t="s">
         <v>80</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F45" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="G45" t="s">
-        <v>166</v>
+        <v>157</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2784,67 +2757,67 @@
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B46" t="s">
         <v>80</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>167</v>
+        <v>158</v>
       </c>
       <c r="D46" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>17</v>
+        <v>62</v>
       </c>
       <c r="F46" t="s">
-        <v>94</v>
+        <v>62</v>
       </c>
       <c r="G46" t="s">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="H46" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B47" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>168</v>
+        <v>159</v>
       </c>
       <c r="D47" t="s">
-        <v>12</v>
+        <v>160</v>
       </c>
       <c r="E47" t="s">
         <v>14</v>
       </c>
       <c r="F47" t="s">
-        <v>169</v>
+        <v>14</v>
       </c>
       <c r="G47" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="H47" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2855,117 +2828,117 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B48" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="D48" t="s">
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="F48" t="s">
-        <v>172</v>
+        <v>17</v>
       </c>
       <c r="G48" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="H48" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B49" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="D49" t="s">
         <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>23</v>
+        <v>121</v>
       </c>
       <c r="F49" t="s">
-        <v>23</v>
+        <v>121</v>
       </c>
       <c r="G49" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>No indexado</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B50" t="s">
         <v>76</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>17</v>
+        <v>56</v>
       </c>
       <c r="F50" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G50" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B51" t="s">
         <v>76</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
@@ -2974,10 +2947,10 @@
         <v>17</v>
       </c>
       <c r="F51" t="s">
-        <v>94</v>
+        <v>17</v>
       </c>
       <c r="G51" t="s">
-        <v>93</v>
+        <v>167</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
@@ -2991,200 +2964,200 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B52" t="s">
         <v>76</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>177</v>
+        <v>168</v>
       </c>
       <c r="D52" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>166</v>
+        <v>92</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B53" t="s">
         <v>76</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="D53" t="s">
         <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F53" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="G53" t="s">
-        <v>118</v>
+        <v>170</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B54" t="s">
         <v>76</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F54" t="s">
-        <v>94</v>
+        <v>10</v>
       </c>
       <c r="G54" t="s">
-        <v>180</v>
+        <v>68</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
       </c>
       <c r="I54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B55" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="D55" t="s">
         <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>17</v>
+        <v>121</v>
       </c>
       <c r="F55" t="s">
-        <v>182</v>
+        <v>121</v>
       </c>
       <c r="G55" t="s">
-        <v>170</v>
+        <v>122</v>
       </c>
       <c r="H55" t="s">
         <v>11</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>No indexado</v>
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B56" t="s">
-        <v>76</v>
+        <v>28</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="F56" t="s">
-        <v>36</v>
+        <v>174</v>
       </c>
       <c r="G56" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B57" t="s">
         <v>28</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="D57" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F57" t="s">
-        <v>95</v>
+        <v>30</v>
       </c>
       <c r="G57" t="s">
-        <v>96</v>
+        <v>177</v>
       </c>
       <c r="H57" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3195,61 +3168,61 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B58" t="s">
         <v>28</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D58" t="s">
         <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="F58" t="s">
-        <v>182</v>
+        <v>25</v>
       </c>
       <c r="G58" t="s">
-        <v>170</v>
+        <v>128</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B59" t="s">
         <v>28</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="D59" t="s">
         <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="F59" t="s">
-        <v>10</v>
+        <v>62</v>
       </c>
       <c r="G59" t="s">
-        <v>68</v>
+        <v>180</v>
       </c>
       <c r="H59" t="s">
         <v>11</v>
@@ -3263,234 +3236,234 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B60" t="s">
         <v>28</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>188</v>
+        <v>81</v>
       </c>
       <c r="D60" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="E60" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F60" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G60" t="s">
-        <v>154</v>
+        <v>75</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B61" t="s">
         <v>28</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="D61" t="s">
-        <v>12</v>
+        <v>74</v>
       </c>
       <c r="E61" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F61" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G61" t="s">
-        <v>118</v>
+        <v>182</v>
       </c>
       <c r="H61" t="s">
         <v>11</v>
       </c>
       <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A62" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B62" t="s">
+        <v>77</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D62" t="s">
+        <v>13</v>
+      </c>
+      <c r="E62" t="s">
+        <v>14</v>
+      </c>
+      <c r="F62" t="s">
+        <v>14</v>
+      </c>
+      <c r="G62" t="s">
+        <v>161</v>
+      </c>
+      <c r="H62" t="s">
+        <v>16</v>
+      </c>
+      <c r="I62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A63" s="5">
+        <v>46133</v>
+      </c>
+      <c r="B63" t="s">
+        <v>77</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>30</v>
+      </c>
+      <c r="F63" t="s">
+        <v>2</v>
+      </c>
+      <c r="G63" t="s">
+        <v>107</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+      <c r="I63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J61" t="str">
+      <c r="J63" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A62" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B62" t="s">
-        <v>28</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="D62" t="s">
-        <v>74</v>
-      </c>
-      <c r="E62" t="s">
-        <v>17</v>
-      </c>
-      <c r="F62" t="s">
-        <v>17</v>
-      </c>
-      <c r="G62" t="s">
-        <v>75</v>
-      </c>
-      <c r="H62" t="s">
-        <v>11</v>
-      </c>
-      <c r="I62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A63" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B63" t="s">
-        <v>28</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D63" t="s">
-        <v>74</v>
-      </c>
-      <c r="E63" t="s">
-        <v>10</v>
-      </c>
-      <c r="F63" t="s">
-        <v>10</v>
-      </c>
-      <c r="G63" t="s">
-        <v>68</v>
-      </c>
-      <c r="H63" t="s">
-        <v>11</v>
-      </c>
-      <c r="I63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A64" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B64" t="s">
         <v>77</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D64" t="s">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E64" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="F64" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G64" t="s">
-        <v>118</v>
+        <v>161</v>
       </c>
       <c r="H64" t="s">
         <v>11</v>
       </c>
       <c r="I64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J64" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B65" t="s">
         <v>77</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="D65" t="s">
         <v>12</v>
       </c>
       <c r="E65" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="F65" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="G65" t="s">
-        <v>193</v>
+        <v>128</v>
       </c>
       <c r="H65" t="s">
         <v>11</v>
       </c>
       <c r="I65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="5">
-        <v>46132</v>
+        <v>46133</v>
       </c>
       <c r="B66" t="s">
         <v>77</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="D66" t="s">
-        <v>195</v>
+        <v>12</v>
       </c>
       <c r="E66" t="s">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="F66" t="s">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="G66" t="s">
-        <v>97</v>
+        <v>188</v>
       </c>
       <c r="H66" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I66" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3499,40 +3472,6 @@
       <c r="J66" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67" s="5">
-        <v>46132</v>
-      </c>
-      <c r="B67" t="s">
-        <v>77</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>196</v>
-      </c>
-      <c r="D67" t="s">
-        <v>9</v>
-      </c>
-      <c r="E67" t="s">
-        <v>17</v>
-      </c>
-      <c r="F67" t="s">
-        <v>90</v>
-      </c>
-      <c r="G67" t="s">
-        <v>197</v>
-      </c>
-      <c r="H67" t="s">
-        <v>11</v>
-      </c>
-      <c r="I67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
   </sheetData>
@@ -3547,14 +3486,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8151DEFD-FF29-4969-B1FC-DF47C7CD743C}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -3568,7 +3507,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>64</v>
       </c>
@@ -3582,7 +3521,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -3596,7 +3535,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>20</v>
       </c>
@@ -3610,7 +3549,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>63</v>
       </c>
@@ -3624,7 +3563,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>35</v>
       </c>
@@ -3638,7 +3577,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -3652,7 +3591,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -3666,7 +3605,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -3680,7 +3619,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>26</v>
       </c>
@@ -3694,7 +3633,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>38</v>
       </c>
@@ -3708,7 +3647,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>39</v>
       </c>
@@ -3722,7 +3661,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>39</v>
       </c>
@@ -3736,7 +3675,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>66</v>
       </c>
@@ -3750,7 +3689,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>40</v>
       </c>
@@ -3764,7 +3703,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>25</v>
       </c>
@@ -3778,7 +3717,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>41</v>
       </c>
@@ -3792,7 +3731,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>42</v>
       </c>
@@ -3806,7 +3745,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -3820,7 +3759,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -3834,7 +3773,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -3848,7 +3787,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -3862,7 +3801,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -3876,7 +3815,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -3890,7 +3829,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>48</v>
       </c>
@@ -3904,7 +3843,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>49</v>
       </c>
@@ -3918,7 +3857,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>67</v>
       </c>
@@ -3932,7 +3871,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>18</v>
       </c>
@@ -3940,7 +3879,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>50</v>
       </c>
@@ -3948,7 +3887,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>51</v>
       </c>
@@ -3956,7 +3895,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
@@ -3964,7 +3903,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>53</v>
       </c>
@@ -3972,7 +3911,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>54</v>
       </c>
@@ -3980,7 +3919,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>55</v>
       </c>
@@ -3988,7 +3927,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>56</v>
       </c>
@@ -3996,7 +3935,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>57</v>
       </c>
@@ -4004,7 +3943,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>24</v>
       </c>
@@ -4012,7 +3951,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>21</v>
       </c>
@@ -4020,7 +3959,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>29</v>
       </c>
@@ -4028,7 +3967,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -4036,7 +3975,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>58</v>
       </c>
@@ -4044,7 +3983,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -4052,7 +3991,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>23</v>
       </c>
@@ -4060,7 +3999,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>59</v>
       </c>
@@ -4068,7 +4007,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>60</v>
       </c>
@@ -4076,7 +4015,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>61</v>
       </c>
@@ -4084,7 +4023,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>31</v>
       </c>
@@ -4092,7 +4031,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>62</v>
       </c>

</xml_diff>

<commit_message>
Reporte en PPTX 260526
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B384CC73-5C6D-47B8-9538-E950CFCC18B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A15627E-A172-4A45-8C6F-0692A37CCA04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="176">
   <si>
     <t>Fecha</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>Gobierno del estado</t>
-  </si>
-  <si>
-    <t>CGCG</t>
   </si>
   <si>
     <t>Congreso</t>
@@ -1225,7 +1222,7 @@
         <v>8</v>
       </c>
       <c r="J1" s="7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1233,10 +1230,10 @@
         <v>46168</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
@@ -1245,10 +1242,10 @@
         <v>14</v>
       </c>
       <c r="F2" t="s">
+        <v>85</v>
+      </c>
+      <c r="G2" t="s">
         <v>86</v>
-      </c>
-      <c r="G2" t="s">
-        <v>87</v>
       </c>
       <c r="H2" t="s">
         <v>11</v>
@@ -1267,10 +1264,10 @@
         <v>46168</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D3" t="s">
         <v>9</v>
@@ -1282,7 +1279,7 @@
         <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
@@ -1301,10 +1298,10 @@
         <v>46168</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
@@ -1313,10 +1310,10 @@
         <v>14</v>
       </c>
       <c r="F4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" t="s">
         <v>91</v>
-      </c>
-      <c r="G4" t="s">
-        <v>92</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
@@ -1335,10 +1332,10 @@
         <v>46168</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
@@ -1350,7 +1347,7 @@
         <v>18</v>
       </c>
       <c r="G5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
@@ -1369,10 +1366,10 @@
         <v>46168</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
@@ -1384,7 +1381,7 @@
         <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
@@ -1403,10 +1400,10 @@
         <v>46168</v>
       </c>
       <c r="B7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D7" t="s">
         <v>13</v>
@@ -1415,13 +1412,13 @@
         <v>16</v>
       </c>
       <c r="F7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G7" t="s">
         <v>97</v>
       </c>
-      <c r="G7" t="s">
-        <v>98</v>
-      </c>
       <c r="H7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1437,10 +1434,10 @@
         <v>46168</v>
       </c>
       <c r="B8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D8" t="s">
         <v>9</v>
@@ -1449,10 +1446,10 @@
         <v>27</v>
       </c>
       <c r="F8" t="s">
+        <v>99</v>
+      </c>
+      <c r="G8" t="s">
         <v>100</v>
-      </c>
-      <c r="G8" t="s">
-        <v>101</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
@@ -1471,10 +1468,10 @@
         <v>46168</v>
       </c>
       <c r="B9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
@@ -1486,7 +1483,7 @@
         <v>24</v>
       </c>
       <c r="G9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
@@ -1505,33 +1502,33 @@
         <v>46168</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G10" t="s">
         <v>105</v>
       </c>
-      <c r="F10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G10" t="s">
-        <v>106</v>
-      </c>
       <c r="H10" t="s">
         <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>No indexado</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -1539,33 +1536,33 @@
         <v>46168</v>
       </c>
       <c r="B11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F11" t="s">
+        <v>104</v>
+      </c>
+      <c r="G11" t="s">
         <v>105</v>
       </c>
-      <c r="F11" t="s">
-        <v>105</v>
-      </c>
-      <c r="G11" t="s">
-        <v>106</v>
-      </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>No indexado</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -1573,10 +1570,10 @@
         <v>46168</v>
       </c>
       <c r="B12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -1588,7 +1585,7 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
@@ -1607,10 +1604,10 @@
         <v>46168</v>
       </c>
       <c r="B13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1622,7 +1619,7 @@
         <v>10</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -1641,10 +1638,10 @@
         <v>46168</v>
       </c>
       <c r="B14" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D14" t="s">
         <v>13</v>
@@ -1656,7 +1653,7 @@
         <v>17</v>
       </c>
       <c r="G14" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
@@ -1675,10 +1672,10 @@
         <v>46168</v>
       </c>
       <c r="B15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D15" t="s">
         <v>9</v>
@@ -1687,10 +1684,10 @@
         <v>27</v>
       </c>
       <c r="F15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H15" t="s">
         <v>11</v>
@@ -1709,10 +1706,10 @@
         <v>46168</v>
       </c>
       <c r="B16" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -1721,10 +1718,10 @@
         <v>23</v>
       </c>
       <c r="F16" t="s">
+        <v>114</v>
+      </c>
+      <c r="G16" t="s">
         <v>115</v>
-      </c>
-      <c r="G16" t="s">
-        <v>116</v>
       </c>
       <c r="H16" t="s">
         <v>11</v>
@@ -1743,10 +1740,10 @@
         <v>46168</v>
       </c>
       <c r="B17" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
@@ -1758,7 +1755,7 @@
         <v>16</v>
       </c>
       <c r="G17" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
@@ -1777,10 +1774,10 @@
         <v>46168</v>
       </c>
       <c r="B18" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
@@ -1789,13 +1786,13 @@
         <v>27</v>
       </c>
       <c r="F18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1811,25 +1808,25 @@
         <v>46168</v>
       </c>
       <c r="B19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D19" t="s">
         <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H19" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1845,10 +1842,10 @@
         <v>46168</v>
       </c>
       <c r="B20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
@@ -1860,7 +1857,7 @@
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
@@ -1879,33 +1876,33 @@
         <v>46168</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
+        <v>104</v>
+      </c>
+      <c r="F21" t="s">
+        <v>104</v>
+      </c>
+      <c r="G21" t="s">
         <v>105</v>
       </c>
-      <c r="F21" t="s">
-        <v>105</v>
-      </c>
-      <c r="G21" t="s">
-        <v>106</v>
-      </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>No indexado</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -1913,33 +1910,33 @@
         <v>46168</v>
       </c>
       <c r="B22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
+        <v>104</v>
+      </c>
+      <c r="F22" t="s">
+        <v>104</v>
+      </c>
+      <c r="G22" t="s">
         <v>105</v>
       </c>
-      <c r="F22" t="s">
-        <v>105</v>
-      </c>
-      <c r="G22" t="s">
-        <v>106</v>
-      </c>
       <c r="H22" t="s">
         <v>11</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>No indexado</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -1947,10 +1944,10 @@
         <v>46168</v>
       </c>
       <c r="B23" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D23" t="s">
         <v>9</v>
@@ -1962,10 +1959,10 @@
         <v>14</v>
       </c>
       <c r="G23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1981,10 +1978,10 @@
         <v>46168</v>
       </c>
       <c r="B24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
@@ -1996,7 +1993,7 @@
         <v>10</v>
       </c>
       <c r="G24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
@@ -2015,10 +2012,10 @@
         <v>46168</v>
       </c>
       <c r="B25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
@@ -2030,7 +2027,7 @@
         <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
@@ -2049,10 +2046,10 @@
         <v>46168</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
@@ -2064,7 +2061,7 @@
         <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
@@ -2083,33 +2080,33 @@
         <v>46168</v>
       </c>
       <c r="B27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
       </c>
       <c r="E27" t="s">
+        <v>104</v>
+      </c>
+      <c r="F27" t="s">
+        <v>104</v>
+      </c>
+      <c r="G27" t="s">
         <v>105</v>
       </c>
-      <c r="F27" t="s">
-        <v>105</v>
-      </c>
-      <c r="G27" t="s">
-        <v>106</v>
-      </c>
       <c r="H27" t="s">
         <v>11</v>
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>No indexado</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2117,10 +2114,10 @@
         <v>46168</v>
       </c>
       <c r="B28" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D28" t="s">
         <v>13</v>
@@ -2129,10 +2126,10 @@
         <v>23</v>
       </c>
       <c r="F28" t="s">
+        <v>114</v>
+      </c>
+      <c r="G28" t="s">
         <v>115</v>
-      </c>
-      <c r="G28" t="s">
-        <v>116</v>
       </c>
       <c r="H28" t="s">
         <v>11</v>
@@ -2151,10 +2148,10 @@
         <v>46168</v>
       </c>
       <c r="B29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
@@ -2166,7 +2163,7 @@
         <v>18</v>
       </c>
       <c r="G29" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H29" t="s">
         <v>11</v>
@@ -2185,10 +2182,10 @@
         <v>46168</v>
       </c>
       <c r="B30" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D30" t="s">
         <v>9</v>
@@ -2197,10 +2194,10 @@
         <v>27</v>
       </c>
       <c r="F30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G30" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
@@ -2219,10 +2216,10 @@
         <v>46168</v>
       </c>
       <c r="B31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D31" t="s">
         <v>12</v>
@@ -2234,7 +2231,7 @@
         <v>10</v>
       </c>
       <c r="G31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
@@ -2253,25 +2250,25 @@
         <v>46168</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D32" t="s">
         <v>13</v>
       </c>
       <c r="E32" t="s">
+        <v>141</v>
+      </c>
+      <c r="F32" t="s">
+        <v>141</v>
+      </c>
+      <c r="G32" t="s">
         <v>142</v>
       </c>
-      <c r="F32" t="s">
-        <v>142</v>
-      </c>
-      <c r="G32" t="s">
-        <v>143</v>
-      </c>
       <c r="H32" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2287,10 +2284,10 @@
         <v>46168</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
@@ -2302,7 +2299,7 @@
         <v>29</v>
       </c>
       <c r="G33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
@@ -2321,10 +2318,10 @@
         <v>46168</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
@@ -2336,7 +2333,7 @@
         <v>17</v>
       </c>
       <c r="G34" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
@@ -2355,22 +2352,22 @@
         <v>46168</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G35" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
@@ -2389,10 +2386,10 @@
         <v>46168</v>
       </c>
       <c r="B36" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
@@ -2404,7 +2401,7 @@
         <v>10</v>
       </c>
       <c r="G36" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
@@ -2423,10 +2420,10 @@
         <v>46168</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D37" t="s">
         <v>9</v>
@@ -2438,7 +2435,7 @@
         <v>29</v>
       </c>
       <c r="G37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
@@ -2457,10 +2454,10 @@
         <v>46168</v>
       </c>
       <c r="B38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
@@ -2469,13 +2466,13 @@
         <v>14</v>
       </c>
       <c r="F38" t="s">
+        <v>151</v>
+      </c>
+      <c r="G38" t="s">
         <v>152</v>
       </c>
-      <c r="G38" t="s">
-        <v>153</v>
-      </c>
       <c r="H38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2491,10 +2488,10 @@
         <v>46168</v>
       </c>
       <c r="B39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
@@ -2503,10 +2500,10 @@
         <v>23</v>
       </c>
       <c r="F39" t="s">
+        <v>114</v>
+      </c>
+      <c r="G39" t="s">
         <v>115</v>
-      </c>
-      <c r="G39" t="s">
-        <v>116</v>
       </c>
       <c r="H39" t="s">
         <v>11</v>
@@ -2525,10 +2522,10 @@
         <v>46168</v>
       </c>
       <c r="B40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D40" t="s">
         <v>13</v>
@@ -2537,10 +2534,10 @@
         <v>14</v>
       </c>
       <c r="F40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G40" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
@@ -2559,10 +2556,10 @@
         <v>46168</v>
       </c>
       <c r="B41" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D41" t="s">
         <v>12</v>
@@ -2574,7 +2571,7 @@
         <v>10</v>
       </c>
       <c r="G41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
@@ -2593,22 +2590,22 @@
         <v>46168</v>
       </c>
       <c r="B42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F42" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G42" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
@@ -2627,22 +2624,22 @@
         <v>46168</v>
       </c>
       <c r="B43" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D43" t="s">
         <v>13</v>
       </c>
       <c r="E43" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F43" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G43" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
@@ -2661,22 +2658,22 @@
         <v>46168</v>
       </c>
       <c r="B44" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D44" t="s">
         <v>9</v>
       </c>
       <c r="E44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G44" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
@@ -2695,10 +2692,10 @@
         <v>46168</v>
       </c>
       <c r="B45" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
@@ -2710,10 +2707,10 @@
         <v>16</v>
       </c>
       <c r="G45" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="H45" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2729,10 +2726,10 @@
         <v>46168</v>
       </c>
       <c r="B46" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
@@ -2744,7 +2741,7 @@
         <v>17</v>
       </c>
       <c r="G46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
@@ -2763,33 +2760,33 @@
         <v>46168</v>
       </c>
       <c r="B47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D47" t="s">
         <v>12</v>
       </c>
       <c r="E47" t="s">
+        <v>104</v>
+      </c>
+      <c r="F47" t="s">
+        <v>104</v>
+      </c>
+      <c r="G47" t="s">
         <v>105</v>
       </c>
-      <c r="F47" t="s">
-        <v>105</v>
-      </c>
-      <c r="G47" t="s">
-        <v>106</v>
-      </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>No indexado</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
@@ -2797,10 +2794,10 @@
         <v>46168</v>
       </c>
       <c r="B48" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D48" t="s">
         <v>13</v>
@@ -2809,10 +2806,10 @@
         <v>23</v>
       </c>
       <c r="F48" t="s">
+        <v>114</v>
+      </c>
+      <c r="G48" t="s">
         <v>115</v>
-      </c>
-      <c r="G48" t="s">
-        <v>116</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
@@ -2831,10 +2828,10 @@
         <v>46168</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D49" t="s">
         <v>12</v>
@@ -2846,7 +2843,7 @@
         <v>26</v>
       </c>
       <c r="G49" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
@@ -2865,10 +2862,10 @@
         <v>46168</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -2880,7 +2877,7 @@
         <v>29</v>
       </c>
       <c r="G50" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
@@ -2899,10 +2896,10 @@
         <v>46168</v>
       </c>
       <c r="B51" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
@@ -2911,10 +2908,10 @@
         <v>16</v>
       </c>
       <c r="F51" t="s">
+        <v>169</v>
+      </c>
+      <c r="G51" t="s">
         <v>170</v>
-      </c>
-      <c r="G51" t="s">
-        <v>171</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
@@ -2933,10 +2930,10 @@
         <v>46168</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
@@ -2948,10 +2945,10 @@
         <v>24</v>
       </c>
       <c r="G52" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H52" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2967,10 +2964,10 @@
         <v>46168</v>
       </c>
       <c r="B53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D53" t="s">
         <v>13</v>
@@ -2982,10 +2979,10 @@
         <v>24</v>
       </c>
       <c r="G53" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H53" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3001,10 +2998,10 @@
         <v>46168</v>
       </c>
       <c r="B54" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
@@ -3013,10 +3010,10 @@
         <v>23</v>
       </c>
       <c r="F54" t="s">
+        <v>114</v>
+      </c>
+      <c r="G54" t="s">
         <v>115</v>
-      </c>
-      <c r="G54" t="s">
-        <v>116</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
@@ -3035,25 +3032,25 @@
         <v>46168</v>
       </c>
       <c r="B55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D55" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E55" t="s">
         <v>27</v>
       </c>
       <c r="F55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G55" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="H55" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3069,33 +3066,33 @@
         <v>46168</v>
       </c>
       <c r="B56" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
       </c>
       <c r="E56" t="s">
+        <v>104</v>
+      </c>
+      <c r="F56" t="s">
+        <v>104</v>
+      </c>
+      <c r="G56" t="s">
         <v>105</v>
       </c>
-      <c r="F56" t="s">
-        <v>105</v>
-      </c>
-      <c r="G56" t="s">
-        <v>106</v>
-      </c>
       <c r="H56" t="s">
         <v>11</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>No indexado</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
   </sheetData>
@@ -3128,21 +3125,21 @@
         <v>4</v>
       </c>
       <c r="E1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" t="s">
         <v>62</v>
-      </c>
-      <c r="B2" t="s">
-        <v>63</v>
       </c>
       <c r="D2" s="10" t="s">
         <v>19</v>
       </c>
       <c r="E2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -3153,10 +3150,10 @@
         <v>31</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>33</v>
+        <v>104</v>
       </c>
       <c r="E3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -3167,15 +3164,15 @@
         <v>32</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
         <v>10</v>
@@ -3184,49 +3181,49 @@
         <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
         <v>32</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
         <v>32</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -3237,10 +3234,10 @@
         <v>32</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -3259,63 +3256,63 @@
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
         <v>32</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B12" t="s">
         <v>32</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B13" t="s">
         <v>32</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B15" t="s">
         <v>32</v>
@@ -3324,7 +3321,7 @@
         <v>17</v>
       </c>
       <c r="E15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -3335,43 +3332,43 @@
         <v>32</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E16" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B17" t="s">
         <v>32</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
         <v>32</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E18" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" t="s">
         <v>10</v>
@@ -3380,35 +3377,35 @@
         <v>23</v>
       </c>
       <c r="E19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" t="s">
         <v>42</v>
-      </c>
-      <c r="B20" t="s">
-        <v>43</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>20</v>
       </c>
       <c r="E20" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>43</v>
+      </c>
+      <c r="B21" t="s">
         <v>44</v>
-      </c>
-      <c r="B21" t="s">
-        <v>45</v>
       </c>
       <c r="D21" s="9" t="s">
         <v>27</v>
       </c>
       <c r="E21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3416,13 +3413,13 @@
         <v>18</v>
       </c>
       <c r="B22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D22" s="10" t="s">
         <v>26</v>
       </c>
       <c r="E22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -3433,10 +3430,10 @@
         <v>32</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -3450,49 +3447,49 @@
         <v>15</v>
       </c>
       <c r="E24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>22</v>
       </c>
       <c r="E25" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E26" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>29</v>
       </c>
       <c r="E27" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3505,7 +3502,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B29" t="s">
         <v>32</v>
@@ -3513,10 +3510,10 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B30" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -3524,36 +3521,36 @@
         <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B32" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B33" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B35" t="s">
         <v>32</v>
@@ -3561,7 +3558,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B36" t="s">
         <v>32</v>
@@ -3601,7 +3598,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B41" t="s">
         <v>32</v>
@@ -3625,7 +3622,7 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B44" t="s">
         <v>32</v>
@@ -3633,7 +3630,7 @@
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B45" t="s">
         <v>10</v>
@@ -3641,7 +3638,7 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B46" t="s">
         <v>10</v>
@@ -3657,7 +3654,7 @@
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B48" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
REporte portadas 02 de junio
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DFCD130-9CA9-4B57-97D8-56D9DB2C9405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAE0E59F-11DE-4C62-9BD1-AC94A4EC115A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="643" uniqueCount="193">
   <si>
     <t>Fecha</t>
   </si>
@@ -258,18 +258,12 @@
     <t>Síntesis</t>
   </si>
   <si>
-    <t>Plaza Juárez</t>
-  </si>
-  <si>
     <t>Temas varios</t>
   </si>
   <si>
     <t>Pachuca Brilla</t>
   </si>
   <si>
-    <t>Tauromaquia</t>
-  </si>
-  <si>
     <t>La Jornada Hidalgo</t>
   </si>
   <si>
@@ -279,300 +273,45 @@
     <t>Mundial De Futbol</t>
   </si>
   <si>
-    <t>Titulación</t>
-  </si>
-  <si>
-    <t>Festival Cultural</t>
-  </si>
-  <si>
-    <t>Aniversario de la transformación</t>
-  </si>
-  <si>
     <t>Deportes</t>
   </si>
   <si>
-    <t>Plan B</t>
-  </si>
-  <si>
     <t>Alerta Meteorológica</t>
   </si>
   <si>
-    <t>Señalan que no hay para cuando en la obra</t>
-  </si>
-  <si>
-    <t>SICT</t>
-  </si>
-  <si>
-    <t>Tren México Querétaro</t>
-  </si>
-  <si>
-    <t>Conmemoran aniversario luctuoso de Jorge Márquez</t>
-  </si>
-  <si>
-    <t>Aniversario luctuoso</t>
-  </si>
-  <si>
-    <t>Prioriza defensa de la soberanía nacional</t>
-  </si>
-  <si>
-    <t>Hasta siete mdp por una casa en la Bella Airosa</t>
-  </si>
-  <si>
-    <t>Costo de vivienda</t>
-  </si>
-  <si>
-    <t>Anuncian el último depósito de becas</t>
-  </si>
-  <si>
-    <t>Becas</t>
-  </si>
-  <si>
     <t>El Universal Hidalgo</t>
   </si>
   <si>
-    <t>Respaldan a la presidenta Claudia Sheinbaum en la lucha por la soberanía</t>
-  </si>
-  <si>
-    <t>Defienden Santiagada</t>
-  </si>
-  <si>
-    <t>Invadidos de lirio y moscos</t>
-  </si>
-  <si>
-    <t>Conagua</t>
-  </si>
-  <si>
-    <t>Presa Endhó</t>
-  </si>
-  <si>
-    <t>Chofer se vuelve tendencia en web</t>
-  </si>
-  <si>
-    <t>Modernización transporte público</t>
-  </si>
-  <si>
-    <t>ANALIZA TSJEH P O ST E RG AC I Ó N Escanea este código y síguenos en las redes sociales de El Universal Hidalgo BA JO |3| RE SERVA DE ELECCIÓN</t>
-  </si>
-  <si>
-    <t>Elección Judicial</t>
-  </si>
-  <si>
     <t>Criterio</t>
   </si>
   <si>
-    <t>ABIERTA, POSIBILIDAD DE ALIANZA PANALH-MORENA</t>
-  </si>
-  <si>
     <t>Alianzas Electorales</t>
   </si>
   <si>
-    <t>Señalan cambio de uso de suelo en el cerro de Cubitos</t>
-  </si>
-  <si>
-    <t>Área Natural Protegida</t>
-  </si>
-  <si>
-    <t>Desde hoy, el gobierno administra el Tuzobús</t>
-  </si>
-  <si>
     <t>Sitmah</t>
   </si>
   <si>
     <t>Modernización Tuzobús</t>
   </si>
   <si>
-    <t>Morena llena Plaza Juárez en respaldo a Sheinbaum</t>
-  </si>
-  <si>
-    <t>México revela su lista para el Mundial 2026</t>
-  </si>
-  <si>
-    <t>“EXCELENTE”,  HACER ELECCIÓN  JUDICIAL HASTA  2028: ALADRO</t>
-  </si>
-  <si>
-    <t>Los adversarios están en camino</t>
-  </si>
-  <si>
-    <t>Sheinbaum llama a impedir que EU sea el gran elector en 2027</t>
-  </si>
-  <si>
-    <t>Posar con un gato es mala idea para ligar</t>
-  </si>
-  <si>
-    <t>Aumenta 87% comercio aéreo con China pese a los aranceles</t>
-  </si>
-  <si>
     <t>Temas internacionales</t>
   </si>
   <si>
-    <t>Buscan que se reconozca a víctimas masculinas</t>
-  </si>
-  <si>
-    <t>La lista de Aguirre</t>
-  </si>
-  <si>
-    <t>Tuzobús: es de 722 mdp la inversión para renovar el sistema de transporte</t>
-  </si>
-  <si>
-    <t>Prevén que desinsentivará el uso deiario del automóvil</t>
-  </si>
-  <si>
-    <t>Gobierno prevé 100 mdp para estaciones del Tuzobús</t>
-  </si>
-  <si>
-    <t>Con respaldo del pueblo, CSP rechaza presiones del extranjero y la derecha local</t>
-  </si>
-  <si>
-    <t>Más de 10 mil escuchan a la presidenta</t>
-  </si>
-  <si>
-    <t>Riña en penal de Culiacán deja siete muertos</t>
-  </si>
-  <si>
-    <t>Riña en penal</t>
-  </si>
-  <si>
-    <t>La “solución” planteada de revocar concesiones es apenas un parche  mediático que no atiende lo estructural. Mientras tanto, la titular de la  Secretaría de Movilidad y Transporte, Liz Robles, permanece omisa en sus  funciones, lo que también constituye un acto de corrupción”.</t>
-  </si>
-  <si>
-    <t>Deficiencias transporte público</t>
-  </si>
-  <si>
-    <t>Reconoce Menchaca papel de Sheinbaum frende a momentos difíciles para el país</t>
-  </si>
-  <si>
-    <t>Obtienen bomberos de Pachuca certificación internacional en materia de rescate</t>
-  </si>
-  <si>
-    <t>Certificación</t>
-  </si>
-  <si>
-    <t>Audio para pedir apoyo en redes sociales fue sacado de contexto: Miguel Moreno</t>
-  </si>
-  <si>
-    <t>Audioescándalo</t>
-  </si>
-  <si>
-    <t>Reúne Hidalgo a estudiantes de 18 estados en concurso escolar</t>
-  </si>
-  <si>
-    <t>Justa Académica</t>
-  </si>
-  <si>
-    <t>Las hidalguenses y los hidalguenses estamos con usted"": Menchaca a Sheinbaum</t>
-  </si>
-  <si>
-    <t>Se intensificaron reportes por fallas en servicio eléctrico en la cabecera</t>
-  </si>
-  <si>
-    <t>CFE</t>
-  </si>
-  <si>
-    <t>Falta de servicios públicos</t>
-  </si>
-  <si>
-    <t>Fortalece personal del ISSSTE hávibos de higiene bucal</t>
-  </si>
-  <si>
-    <t>ISSSTE</t>
-  </si>
-  <si>
-    <t>Salud bucal</t>
-  </si>
-  <si>
-    <t>TCNM realiza ceremonia de graduación y entrega de títulos profesionales</t>
-  </si>
-  <si>
-    <t>Se venció el plazo de declaraciones patrimoniales</t>
-  </si>
-  <si>
     <t>Declaración patrimonial</t>
   </si>
   <si>
-    <t>MC rechaza cambios a gubernatura de dos años</t>
-  </si>
-  <si>
-    <t>Reforma Electoral</t>
-  </si>
-  <si>
-    <t>La 4T de Hidalgo respalda a Sheinbaum</t>
-  </si>
-  <si>
-    <t>Elección judicial en 2028: más eficiente y menos costosa</t>
-  </si>
-  <si>
-    <t>Mantiene Hidalgo 26 fichas rojas activas</t>
-  </si>
-  <si>
-    <t>Ficha De Búsqueda</t>
-  </si>
-  <si>
-    <t>Pachuca descarta ampliar horarios en bares por Mundial</t>
-  </si>
-  <si>
-    <t>Congreso aprueba reducción de regidurías en Hidalgo</t>
-  </si>
-  <si>
     <t>Marfeca</t>
   </si>
   <si>
-    <t>Tren embiste a vehículo que intentó ganar el paso en Atitalaquia</t>
-  </si>
-  <si>
     <t>Cintillo</t>
   </si>
   <si>
     <t>Accidente Carretero</t>
   </si>
   <si>
-    <t>Los hidalguenses estamos con usted: reitera Menchaca a Sheinbaum</t>
-  </si>
-  <si>
-    <t>Bomberos de Pachuca obtienen certificación internacional y rescate fortalecen su capacidad de respuesta</t>
-  </si>
-  <si>
-    <t>Por unanimidad, 99.18% de socios reeligen a Víctor Velázquez Rangel al frente de la Cruz Azul</t>
-  </si>
-  <si>
-    <t>Cruz Azul</t>
-  </si>
-  <si>
-    <t>Con inversión superior a los 2MDP arrancan 2 obras de drenaje sanitario en Atotonilco de Tula</t>
-  </si>
-  <si>
-    <t>Drenaje</t>
-  </si>
-  <si>
-    <t>Realizan 1a edición "Lucha Cafe", festival que mezcló el café, luchas y música de rock</t>
-  </si>
-  <si>
-    <t>Hidalgo fortalece su promoción turística en el norte del país</t>
-  </si>
-  <si>
     <t>Promoción turística</t>
   </si>
   <si>
-    <t>Bomberos de Atitalaquia comparten información preventiva por temporada de lluvias</t>
-  </si>
-  <si>
-    <t>Prevención De Riesgos</t>
-  </si>
-  <si>
-    <t>Becas del Citnova impulsan a especialistas para el sector productivo</t>
-  </si>
-  <si>
-    <t>Citnova</t>
-  </si>
-  <si>
-    <t>Becas De Posgrado</t>
-  </si>
-  <si>
-    <t>Judocas Garza conquistan medallas en Certamen Nacional</t>
-  </si>
-  <si>
-    <t>Justa Deportiva</t>
-  </si>
-  <si>
     <t>Drones</t>
   </si>
   <si>
@@ -582,46 +321,301 @@
     <t>Videovigilancia</t>
   </si>
   <si>
-    <t>Menchaca refrenda apoyo de Hidalgo a Sheinbaum</t>
-  </si>
-  <si>
-    <t>Comienza nueva etapa del Tuzobús este lunes</t>
-  </si>
-  <si>
-    <t>Anuncian a los 26 jugadores de la selecció mexicana</t>
-  </si>
-  <si>
-    <t>BOMBEROS DE PACHUCA OBTIENEN CERTIFICACIÓN INTERNACIONAL DE RESCATE</t>
-  </si>
-  <si>
-    <t>Seguridad Pública de Pachuca refuerza profesionalización en detección de vehículos clonados</t>
-  </si>
-  <si>
-    <t>Profesionalización policial</t>
-  </si>
-  <si>
     <t>Impulso indígena</t>
   </si>
   <si>
     <t>Cedspi</t>
   </si>
   <si>
-    <t>Sheinbaum defiende con dignidad los intereses de México""</t>
-  </si>
-  <si>
-    <t>Claudia Sheinbaum: ""VAmos a defender la soberanía de México""</t>
-  </si>
-  <si>
-    <t>Hoy inicia temporada de ciclones tropicales</t>
-  </si>
-  <si>
-    <t>Rescatan cebaderos diversos acuerdos con Grupo Modelo</t>
-  </si>
-  <si>
-    <t>Cebaderos</t>
-  </si>
-  <si>
-    <t>Listos los 26 que representarán a México</t>
+    <t>En abandono dos inmuebles del SNTE</t>
+  </si>
+  <si>
+    <t>Abandono de obra</t>
+  </si>
+  <si>
+    <t>Venta de roba ligera aumenta en Pachuca</t>
+  </si>
+  <si>
+    <t>Destaca atracción de inversión urbana</t>
+  </si>
+  <si>
+    <t>Atracción De Inversiones</t>
+  </si>
+  <si>
+    <t>Crece demanda de monedas del mundial 2026</t>
+  </si>
+  <si>
+    <t>En marcha la flotilla, suman 80 nuevas unidades móviles</t>
+  </si>
+  <si>
+    <t>Arranca nuevo Sistema de Transporte Metropolitano</t>
+  </si>
+  <si>
+    <t>Dia de la Marina</t>
+  </si>
+  <si>
+    <t>Día de la Marina</t>
+  </si>
+  <si>
+    <t>Pachuca recibe a Sudáfrica</t>
+  </si>
+  <si>
+    <t>Nueve infestados por el gusano</t>
+  </si>
+  <si>
+    <t>Gusano barrenador</t>
+  </si>
+  <si>
+    <t>Dirigente de Morena ve derrotado al PRI</t>
+  </si>
+  <si>
+    <t>Elecciones</t>
+  </si>
+  <si>
+    <t>APLAZA CNHJ  RESOLUCIÓN AL CONFLICTO ENTRE EDILA Y REGIDOR</t>
+  </si>
+  <si>
+    <t>Juicio Político</t>
+  </si>
+  <si>
+    <t>Suman 9 casos de miasis por barrenador en humanos: SSH</t>
+  </si>
+  <si>
+    <t>COMENZARON OPERACIÓN 80 UNIDADES DEL TUZOBÚS</t>
+  </si>
+  <si>
+    <t>Ciclovía, en el olvido</t>
+  </si>
+  <si>
+    <t>Vialidad En Mal Estado</t>
+  </si>
+  <si>
+    <t>Hidalgo, con 30% de tomas clandestinas del país: IGAVIM</t>
+  </si>
+  <si>
+    <t>Huachicol</t>
+  </si>
+  <si>
+    <t>TRI ya tiene dorsales para el Mundial</t>
+  </si>
+  <si>
+    <t>El líder de Ecuador</t>
+  </si>
+  <si>
+    <t>Tuzobús estrena unidades: misma tarifa, cámaras, IA...</t>
+  </si>
+  <si>
+    <t>Reconocen que el sistema tiene 210 conductores de 351 necesarios</t>
+  </si>
+  <si>
+    <t>Tres mil funcionarios no cumplen con declaración patrimonial</t>
+  </si>
+  <si>
+    <t>Sheinbaum exime a Trump de la ofensiva: ""es la ultraderecha""</t>
+  </si>
+  <si>
+    <t>Intervención extranjera</t>
+  </si>
+  <si>
+    <t>Sir Paul vuelve al Liverpool de los años felices</t>
+  </si>
+  <si>
+    <t>Dan luz verde a megaproyecto fotovoltaico en Tecozautla</t>
+  </si>
+  <si>
+    <t>Parque Fotovoltaico</t>
+  </si>
+  <si>
+    <t>Luis García: Nos asomamos a la mesa, pero falta</t>
+  </si>
+  <si>
+    <t>Aprobación presidenta Claudia Sheinbaum</t>
+  </si>
+  <si>
+    <t>Aprobación Sheinbaum</t>
+  </si>
+  <si>
+    <t>Gobierno asume control del Tuzobús y estrena 148 unidades</t>
+  </si>
+  <si>
+    <t>Sheinbaum mantiene aval de 70.1%, a dos años de su triunfo</t>
+  </si>
+  <si>
+    <t>Comparece Mérida en corte de Nueva York</t>
+  </si>
+  <si>
+    <t>Programas del Bienestar beneficiarán a 42.8  millones de personas en 2026</t>
+  </si>
+  <si>
+    <t>Programas Del Bienestar</t>
+  </si>
+  <si>
+    <t>Porque la soberanía que se invoca hoy no es la del discurso decimonónico ni la de la autarquía. Es algo más  fino y más difícil: la autonomía de decisión dentro de la interdependencia”.</t>
+  </si>
+  <si>
+    <t>Descartan Salud muertes en humanos por gusano barrenador; hay nueve casos confirmados</t>
+  </si>
+  <si>
+    <t>Continúa búsqueda de seis personas en Tianguistengo tras lluvias atipicas</t>
+  </si>
+  <si>
+    <t>Huracán Priscilla</t>
+  </si>
+  <si>
+    <t>Transforman Tuzobús en Sistema de Transporte  Metropolitano; operan 80 unidades</t>
+  </si>
+  <si>
+    <t>Investiga organismo  electoral siete denuncias  por violencia política  contra mujeres</t>
+  </si>
+  <si>
+    <t>Violencia Política De Género</t>
+  </si>
+  <si>
+    <t>Invertirá Cuautepec más  de 19.2 millones de pesos  en infraestructura pública</t>
+  </si>
+  <si>
+    <t>infraestructura</t>
+  </si>
+  <si>
+    <t>Intensifican pláticas a motociclistas tras aumento de accidentes</t>
+  </si>
+  <si>
+    <t>Educación vial</t>
+  </si>
+  <si>
+    <t>Leyendas del futbol se reunirán en el partido México VS Sudáfrica</t>
+  </si>
+  <si>
+    <t>Confirman instalación del consejo político estatal del PRI en Hidlago</t>
+  </si>
+  <si>
+    <t>PRI</t>
+  </si>
+  <si>
+    <t>Instalación de comité</t>
+  </si>
+  <si>
+    <t>Conmemoran en Huejutla el Día de la Marina Nacional</t>
+  </si>
+  <si>
+    <t>Temporal de lluvias inicia este lunes 1 de junio</t>
+  </si>
+  <si>
+    <t>"iAdiós, Tuzobus! ibienvenido, Sistema de Transporte Metropolitano!"</t>
+  </si>
+  <si>
+    <t>La revolución del cascarón</t>
+  </si>
+  <si>
+    <t>Nueva Alianza, sin definir coalición con Morena</t>
+  </si>
+  <si>
+    <t>Adiós a los cobros arbitrarios</t>
+  </si>
+  <si>
+    <t>Abusos taxistas</t>
+  </si>
+  <si>
+    <t>Sin toma de nota, no hay dirigencia</t>
+  </si>
+  <si>
+    <t>Dirigencia SUTSPEEH</t>
+  </si>
+  <si>
+    <t>10 lesionados en fuerte accidente en la Jorobas - Tula</t>
+  </si>
+  <si>
+    <t>Fortalece DIF Hidalgo red municipal de protección a niñas, niños y adolescentes</t>
+  </si>
+  <si>
+    <t>Protección del menor</t>
+  </si>
+  <si>
+    <t>Menchaca transforma movilidad con nuevo Sistema de Transporte Metropolitano</t>
+  </si>
+  <si>
+    <t>Tezontepec de Aldama fortalece acciones preventivas ante temporada de lluvias y ciclones 2026</t>
+  </si>
+  <si>
+    <t>Prevención de inundaciones</t>
+  </si>
+  <si>
+    <t>Gabinete de Seguridad de Hidalgo frustra robo al transporte de carga</t>
+  </si>
+  <si>
+    <t>Reunión Gabinete De Seguridad</t>
+  </si>
+  <si>
+    <t>Sección 15 del SNTE impulsa el desarrollo profesional del magisterio hidalguense con nuevas asignaciones y promociones</t>
+  </si>
+  <si>
+    <t>¡Remojo! Dan estreno a nueva unidad del Tuzobús</t>
+  </si>
+  <si>
+    <t>Accidente Tuzobús</t>
+  </si>
+  <si>
+    <t>Con proximidad niños de la colonia Dendho conocen a bomberos de Atitalaquia</t>
+  </si>
+  <si>
+    <t>Respalda gobierno de Julio Menchaca a productores en el eDía Mundial de la leche</t>
+  </si>
+  <si>
+    <t>Producción lechera</t>
+  </si>
+  <si>
+    <t>Alberga UAEH etapa estatal de las Olimpiadas del conocimiento</t>
+  </si>
+  <si>
+    <t>Encuentro académico</t>
+  </si>
+  <si>
+    <t>Senderismo cerro de la Mesa</t>
+  </si>
+  <si>
+    <t>JULIO MENCHACA TRANSFORMA MOVILIDAD CON NUEVO SISTEMA DE TRANSPORTE METROPOLITANO</t>
+  </si>
+  <si>
+    <t>NATIVIDAD CASTREJÓN INAUGURA AULAS STEM EN COLEGIO DE CIUDAD SAHAGÚN</t>
+  </si>
+  <si>
+    <t>Laboratorio STEM</t>
+  </si>
+  <si>
+    <t>EXHORTAN A CUIDAR UNIDADES; PIDEN NO INVADIR CARRIL EXCLUSIVO</t>
+  </si>
+  <si>
+    <t>Carril confinado</t>
+  </si>
+  <si>
+    <t>La fiesta mundialista en Hidalgo: jugarán leyendas de Sudáfrica y de México</t>
+  </si>
+  <si>
+    <t>Camioneta impactó a unidad del transaporte sobre la Avenida Juárez</t>
+  </si>
+  <si>
+    <t>Los taxistas no pueden poner su propia tarifa: Semot</t>
+  </si>
+  <si>
+    <t>Tarifario de taxis</t>
+  </si>
+  <si>
+    <t>Comienza a operar el Sistema de Transporte Metropolitano</t>
+  </si>
+  <si>
+    <t>Denuncian presunto abuso sexual contra estudiante</t>
+  </si>
+  <si>
+    <t>Abuso Sexual</t>
+  </si>
+  <si>
+    <t>Camioneta choca contra nueva unidad de transporte</t>
+  </si>
+  <si>
+    <t>Era tiempo de poner un alto a los abusos de los taxistas en Pachuca, donde cobran lo que quieren ... la medida llega tarde, pero mas vale tarde que nunca.</t>
+  </si>
+  <si>
+    <t>Editorial</t>
   </si>
 </sst>
 </file>
@@ -868,8 +862,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J68" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J68" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J70" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J70" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1235,7 +1229,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1284,32 +1278,32 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B2" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="H2" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1318,32 +1312,32 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B3" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="H3" t="s">
         <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1352,47 +1346,47 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B4" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="H4" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B5" t="s">
         <v>68</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
@@ -1404,10 +1398,10 @@
         <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="H5" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1418,49 +1412,49 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B6" t="s">
         <v>68</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
         <v>13</v>
@@ -1472,7 +1466,7 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H7" t="s">
         <v>69</v>
@@ -1488,32 +1482,32 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B8" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="D8" t="s">
         <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G8" t="s">
-        <v>76</v>
+        <v>105</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1522,32 +1516,32 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B9" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>100</v>
+        <v>16</v>
       </c>
       <c r="G9" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="H9" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1556,149 +1550,149 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B10" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F10" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="G10" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" t="s">
+        <v>110</v>
+      </c>
+      <c r="H11" t="s">
+        <v>11</v>
+      </c>
+      <c r="I11" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J11" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B11" t="s">
-        <v>96</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="D11" t="s">
-        <v>12</v>
-      </c>
-      <c r="E11" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" t="s">
-        <v>105</v>
-      </c>
-      <c r="H11" t="s">
-        <v>11</v>
-      </c>
-      <c r="I11" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J11" t="str">
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" t="s">
+        <v>18</v>
+      </c>
+      <c r="G12" t="s">
+        <v>112</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+      <c r="I12" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" t="s">
-        <v>46</v>
-      </c>
-      <c r="F12" t="s">
-        <v>46</v>
-      </c>
-      <c r="G12" t="s">
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" t="s">
+        <v>15</v>
+      </c>
+      <c r="G13" t="s">
         <v>108</v>
       </c>
-      <c r="H12" t="s">
-        <v>11</v>
-      </c>
-      <c r="I12" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
-      </c>
-      <c r="J12" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B13" t="s">
-        <v>106</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" t="s">
-        <v>16</v>
-      </c>
-      <c r="F13" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" t="s">
-        <v>110</v>
-      </c>
       <c r="H13" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B14" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="D14" t="s">
         <v>13</v>
@@ -1707,10 +1701,10 @@
         <v>27</v>
       </c>
       <c r="F14" t="s">
-        <v>112</v>
+        <v>83</v>
       </c>
       <c r="G14" t="s">
-        <v>113</v>
+        <v>84</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
@@ -1726,93 +1720,93 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B15" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="D15" t="s">
         <v>9</v>
       </c>
       <c r="E15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G15" t="s">
-        <v>82</v>
+        <v>116</v>
       </c>
       <c r="H15" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B16" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
       </c>
       <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>17</v>
+      </c>
+      <c r="G16" t="s">
+        <v>118</v>
+      </c>
+      <c r="H16" t="s">
+        <v>70</v>
+      </c>
+      <c r="I16" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J16" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B17" t="s">
+        <v>81</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
         <v>10</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F17" t="s">
         <v>10</v>
       </c>
-      <c r="G16" t="s">
-        <v>83</v>
-      </c>
-      <c r="H16" t="s">
-        <v>11</v>
-      </c>
-      <c r="I16" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J16" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B17" t="s">
-        <v>106</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" t="s">
-        <v>58</v>
-      </c>
-      <c r="F17" t="s">
-        <v>2</v>
-      </c>
       <c r="G17" t="s">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
@@ -1828,13 +1822,13 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B18" t="s">
-        <v>106</v>
+        <v>81</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
@@ -1846,7 +1840,7 @@
         <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
@@ -1860,136 +1854,136 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B19" t="s">
         <v>67</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D19" t="s">
         <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F19" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G19" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H19" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B20" t="s">
         <v>67</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F20" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="G20" t="s">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B21" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="F21" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="G21" t="s">
-        <v>121</v>
+        <v>86</v>
       </c>
       <c r="H21" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B22" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F22" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>74</v>
+        <v>125</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1998,13 +1992,13 @@
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B23" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
@@ -2016,7 +2010,7 @@
         <v>10</v>
       </c>
       <c r="G23" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
@@ -2032,25 +2026,25 @@
     </row>
     <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B24" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="F24" t="s">
-        <v>112</v>
+        <v>54</v>
       </c>
       <c r="G24" t="s">
-        <v>113</v>
+        <v>128</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
@@ -2066,149 +2060,149 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B25" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>112</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>113</v>
+        <v>78</v>
       </c>
       <c r="H25" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B26" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E26" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F26" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G26" t="s">
-        <v>113</v>
+        <v>131</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>27</v>
+      </c>
+      <c r="F27" t="s">
+        <v>83</v>
+      </c>
+      <c r="G27" t="s">
+        <v>84</v>
+      </c>
+      <c r="H27" t="s">
+        <v>11</v>
+      </c>
+      <c r="I27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B28" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="D28" t="s">
         <v>13</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E28" t="s">
         <v>14</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F28" t="s">
         <v>14</v>
       </c>
-      <c r="G27" t="s">
-        <v>82</v>
-      </c>
-      <c r="H27" t="s">
-        <v>11</v>
-      </c>
-      <c r="I27" t="str">
+      <c r="G28" t="s">
+        <v>131</v>
+      </c>
+      <c r="H28" t="s">
+        <v>69</v>
+      </c>
+      <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Presidencia de la República</v>
       </c>
-      <c r="J27" t="str">
+      <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B28" t="s">
-        <v>77</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D28" t="s">
-        <v>9</v>
-      </c>
-      <c r="E28" t="s">
-        <v>24</v>
-      </c>
-      <c r="F28" t="s">
-        <v>24</v>
-      </c>
-      <c r="G28" t="s">
-        <v>82</v>
-      </c>
-      <c r="H28" t="s">
-        <v>11</v>
-      </c>
-      <c r="I28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
@@ -2220,10 +2214,10 @@
         <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="H29" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2234,117 +2228,117 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B30" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="F30" t="s">
+        <v>14</v>
+      </c>
+      <c r="G30" t="s">
+        <v>136</v>
+      </c>
+      <c r="H30" t="s">
+        <v>69</v>
+      </c>
+      <c r="I30" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J30" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B31" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="D31" t="s">
+        <v>12</v>
+      </c>
+      <c r="E31" t="s">
+        <v>47</v>
+      </c>
+      <c r="F31" t="s">
         <v>2</v>
       </c>
-      <c r="G30" t="s">
-        <v>132</v>
-      </c>
-      <c r="H30" t="s">
-        <v>70</v>
-      </c>
-      <c r="I30" t="str">
+      <c r="G31" t="s">
+        <v>125</v>
+      </c>
+      <c r="H31" t="s">
+        <v>11</v>
+      </c>
+      <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J30" t="str">
+      <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B31" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="D31" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" t="s">
-        <v>24</v>
-      </c>
-      <c r="F31" t="s">
-        <v>24</v>
-      </c>
-      <c r="G31" t="s">
-        <v>82</v>
-      </c>
-      <c r="H31" t="s">
-        <v>69</v>
-      </c>
-      <c r="I31" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J31" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B32" t="s">
         <v>72</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G32" t="s">
-        <v>135</v>
+        <v>108</v>
       </c>
       <c r="H32" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B33" t="s">
         <v>72</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
@@ -2356,7 +2350,7 @@
         <v>16</v>
       </c>
       <c r="G33" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
@@ -2372,25 +2366,25 @@
     </row>
     <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B34" t="s">
         <v>72</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F34" t="s">
-        <v>26</v>
+        <v>83</v>
       </c>
       <c r="G34" t="s">
-        <v>139</v>
+        <v>84</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
@@ -2406,100 +2400,100 @@
     </row>
     <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B35" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="D35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="F35" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="G35" t="s">
-        <v>82</v>
+        <v>143</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B36" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F36" t="s">
-        <v>142</v>
+        <v>16</v>
       </c>
       <c r="G36" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H36" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B37" t="s">
         <v>71</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D37" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E37" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F37" t="s">
-        <v>145</v>
+        <v>16</v>
       </c>
       <c r="G37" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2508,100 +2502,100 @@
     </row>
     <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B38" t="s">
         <v>71</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="F38" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="G38" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B39" t="s">
         <v>71</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D39" t="s">
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>34</v>
+        <v>150</v>
       </c>
       <c r="F39" t="s">
-        <v>34</v>
+        <v>150</v>
       </c>
       <c r="G39" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H39" t="s">
         <v>11</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Partidos</v>
       </c>
       <c r="J39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B40" t="s">
         <v>71</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="F40" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
       <c r="G40" t="s">
-        <v>151</v>
+        <v>105</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Partidos</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2610,109 +2604,109 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B41" t="s">
         <v>71</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F41" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="G41" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="H41" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B42" t="s">
         <v>71</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>58</v>
+        <v>27</v>
       </c>
       <c r="F42" t="s">
-        <v>2</v>
+        <v>83</v>
       </c>
       <c r="G42" t="s">
-        <v>105</v>
+        <v>84</v>
       </c>
       <c r="H42" t="s">
         <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B43" t="s">
         <v>71</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="F43" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="G43" t="s">
-        <v>155</v>
+        <v>73</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
       </c>
       <c r="I43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J43" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B44" t="s">
         <v>71</v>
@@ -2724,20 +2718,20 @@
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="F44" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="G44" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H44" t="s">
         <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Partidos</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2746,7 +2740,7 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B45" t="s">
         <v>71</v>
@@ -2758,171 +2752,171 @@
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F45" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G45" t="s">
-        <v>84</v>
+        <v>158</v>
       </c>
       <c r="H45" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B46" t="s">
-        <v>158</v>
+        <v>71</v>
       </c>
       <c r="C46" s="6" t="s">
         <v>159</v>
       </c>
       <c r="D46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>24</v>
+      </c>
+      <c r="F46" t="s">
+        <v>24</v>
+      </c>
+      <c r="G46" t="s">
         <v>160</v>
       </c>
-      <c r="E46" t="s">
+      <c r="H46" t="s">
+        <v>11</v>
+      </c>
+      <c r="I46" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J46" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B47" t="s">
+        <v>87</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="D47" t="s">
+        <v>88</v>
+      </c>
+      <c r="E47" t="s">
         <v>10</v>
       </c>
-      <c r="F46" t="s">
+      <c r="F47" t="s">
         <v>10</v>
       </c>
-      <c r="G46" t="s">
-        <v>161</v>
-      </c>
-      <c r="H46" t="s">
-        <v>11</v>
-      </c>
-      <c r="I46" t="str">
+      <c r="G47" t="s">
+        <v>89</v>
+      </c>
+      <c r="H47" t="s">
+        <v>11</v>
+      </c>
+      <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J46" t="str">
+      <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B47" t="s">
-        <v>158</v>
-      </c>
-      <c r="C47" s="6" t="s">
+    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B48" t="s">
+        <v>87</v>
+      </c>
+      <c r="C48" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="D47" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" t="s">
-        <v>24</v>
-      </c>
-      <c r="F47" t="s">
-        <v>24</v>
-      </c>
-      <c r="G47" t="s">
-        <v>82</v>
-      </c>
-      <c r="H47" t="s">
-        <v>11</v>
-      </c>
-      <c r="I47" t="str">
+      <c r="D48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" t="s">
+        <v>36</v>
+      </c>
+      <c r="F48" t="s">
+        <v>36</v>
+      </c>
+      <c r="G48" t="s">
+        <v>163</v>
+      </c>
+      <c r="H48" t="s">
+        <v>11</v>
+      </c>
+      <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A48" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B48" t="s">
-        <v>158</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D48" t="s">
-        <v>12</v>
-      </c>
-      <c r="E48" t="s">
-        <v>16</v>
-      </c>
-      <c r="F48" t="s">
-        <v>16</v>
-      </c>
-      <c r="G48" t="s">
-        <v>135</v>
-      </c>
-      <c r="H48" t="s">
-        <v>11</v>
-      </c>
-      <c r="I48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B49" t="s">
-        <v>158</v>
+        <v>87</v>
       </c>
       <c r="C49" s="6" t="s">
         <v>164</v>
       </c>
       <c r="D49" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E49" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F49" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G49" t="s">
-        <v>165</v>
+        <v>84</v>
       </c>
       <c r="H49" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B50" t="s">
-        <v>158</v>
+        <v>87</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
@@ -2934,7 +2928,7 @@
         <v>16</v>
       </c>
       <c r="G50" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
@@ -2950,44 +2944,44 @@
     </row>
     <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B51" t="s">
-        <v>158</v>
+        <v>87</v>
       </c>
       <c r="C51" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="D51" t="s">
+        <v>12</v>
+      </c>
+      <c r="E51" t="s">
+        <v>24</v>
+      </c>
+      <c r="F51" t="s">
+        <v>24</v>
+      </c>
+      <c r="G51" t="s">
         <v>168</v>
       </c>
-      <c r="D51" t="s">
-        <v>12</v>
-      </c>
-      <c r="E51" t="s">
-        <v>16</v>
-      </c>
-      <c r="F51" t="s">
-        <v>16</v>
-      </c>
-      <c r="G51" t="s">
-        <v>81</v>
-      </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B52" t="s">
-        <v>158</v>
+        <v>87</v>
       </c>
       <c r="C52" s="6" t="s">
         <v>169</v>
@@ -2996,84 +2990,84 @@
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>170</v>
+        <v>73</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B53" t="s">
-        <v>158</v>
+        <v>87</v>
       </c>
       <c r="C53" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>29</v>
+      </c>
+      <c r="F53" t="s">
+        <v>29</v>
+      </c>
+      <c r="G53" t="s">
+        <v>77</v>
+      </c>
+      <c r="H53" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B54" t="s">
+        <v>87</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>27</v>
+      </c>
+      <c r="F54" t="s">
+        <v>83</v>
+      </c>
+      <c r="G54" t="s">
         <v>171</v>
       </c>
-      <c r="D53" t="s">
-        <v>12</v>
-      </c>
-      <c r="E53" t="s">
-        <v>16</v>
-      </c>
-      <c r="F53" t="s">
-        <v>16</v>
-      </c>
-      <c r="G53" t="s">
-        <v>172</v>
-      </c>
-      <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A54" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B54" t="s">
-        <v>158</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D54" t="s">
-        <v>12</v>
-      </c>
-      <c r="E54" t="s">
-        <v>47</v>
-      </c>
-      <c r="F54" t="s">
-        <v>174</v>
-      </c>
-      <c r="G54" t="s">
-        <v>175</v>
-      </c>
       <c r="H54" t="s">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="I54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -3086,372 +3080,372 @@
     </row>
     <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B55" t="s">
-        <v>158</v>
+        <v>87</v>
       </c>
       <c r="C55" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>16</v>
+      </c>
+      <c r="F55" t="s">
+        <v>16</v>
+      </c>
+      <c r="G55" t="s">
+        <v>73</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A56" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B56" t="s">
+        <v>87</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>53</v>
+      </c>
+      <c r="F56" t="s">
+        <v>53</v>
+      </c>
+      <c r="G56" t="s">
+        <v>174</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A57" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B57" t="s">
+        <v>87</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>59</v>
+      </c>
+      <c r="F57" t="s">
+        <v>59</v>
+      </c>
+      <c r="G57" t="s">
         <v>176</v>
       </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>59</v>
-      </c>
-      <c r="F55" t="s">
-        <v>59</v>
-      </c>
-      <c r="G55" t="s">
-        <v>177</v>
-      </c>
-      <c r="H55" t="s">
-        <v>69</v>
-      </c>
-      <c r="I55" t="str">
+      <c r="H57" t="s">
+        <v>11</v>
+      </c>
+      <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J55" t="str">
+      <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B56" t="s">
-        <v>158</v>
-      </c>
-      <c r="C56" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="D56" t="s">
-        <v>179</v>
-      </c>
-      <c r="E56" t="s">
-        <v>16</v>
-      </c>
-      <c r="F56" t="s">
-        <v>16</v>
-      </c>
-      <c r="G56" t="s">
-        <v>180</v>
-      </c>
-      <c r="H56" t="s">
-        <v>11</v>
-      </c>
-      <c r="I56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J56" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B57" t="s">
-        <v>75</v>
-      </c>
-      <c r="C57" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="D57" t="s">
-        <v>13</v>
-      </c>
-      <c r="E57" t="s">
-        <v>24</v>
-      </c>
-      <c r="F57" t="s">
-        <v>24</v>
-      </c>
-      <c r="G57" t="s">
-        <v>82</v>
-      </c>
-      <c r="H57" t="s">
-        <v>11</v>
-      </c>
-      <c r="I57" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J57" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B58" t="s">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="D58" t="s">
-        <v>12</v>
+        <v>92</v>
       </c>
       <c r="E58" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F58" t="s">
-        <v>112</v>
+        <v>16</v>
       </c>
       <c r="G58" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="H58" t="s">
+        <v>11</v>
+      </c>
+      <c r="I58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A59" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B59" t="s">
+        <v>74</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="D59" t="s">
+        <v>13</v>
+      </c>
+      <c r="E59" t="s">
+        <v>24</v>
+      </c>
+      <c r="F59" t="s">
+        <v>24</v>
+      </c>
+      <c r="G59" t="s">
+        <v>84</v>
+      </c>
+      <c r="H59" t="s">
         <v>69</v>
       </c>
-      <c r="I58" t="str">
+      <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J58" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B59" t="s">
-        <v>75</v>
-      </c>
-      <c r="C59" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="D59" t="s">
-        <v>12</v>
-      </c>
-      <c r="E59" t="s">
-        <v>10</v>
-      </c>
-      <c r="F59" t="s">
-        <v>10</v>
-      </c>
-      <c r="G59" t="s">
-        <v>83</v>
-      </c>
-      <c r="H59" t="s">
-        <v>11</v>
-      </c>
-      <c r="I59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
       <c r="J59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B60" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="D60" t="s">
         <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F60" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="G60" t="s">
-        <v>135</v>
+        <v>180</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B61" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D61" t="s">
         <v>12</v>
       </c>
       <c r="E61" t="s">
+        <v>24</v>
+      </c>
+      <c r="F61" t="s">
+        <v>24</v>
+      </c>
+      <c r="G61" t="s">
+        <v>182</v>
+      </c>
+      <c r="H61" t="s">
+        <v>11</v>
+      </c>
+      <c r="I61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A62" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B62" t="s">
+        <v>74</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>29</v>
+      </c>
+      <c r="F62" t="s">
+        <v>29</v>
+      </c>
+      <c r="G62" t="s">
+        <v>77</v>
+      </c>
+      <c r="H62" t="s">
+        <v>11</v>
+      </c>
+      <c r="I62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A63" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B63" t="s">
+        <v>74</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>27</v>
+      </c>
+      <c r="F63" t="s">
+        <v>83</v>
+      </c>
+      <c r="G63" t="s">
+        <v>171</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+      <c r="I63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A64" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B64" t="s">
+        <v>74</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D64" t="s">
+        <v>92</v>
+      </c>
+      <c r="E64" t="s">
+        <v>47</v>
+      </c>
+      <c r="F64" t="s">
+        <v>95</v>
+      </c>
+      <c r="G64" t="s">
+        <v>77</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A65" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B65" t="s">
+        <v>74</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D65" t="s">
+        <v>92</v>
+      </c>
+      <c r="E65" t="s">
         <v>16</v>
       </c>
-      <c r="F61" t="s">
+      <c r="F65" t="s">
         <v>16</v>
       </c>
-      <c r="G61" t="s">
-        <v>186</v>
-      </c>
-      <c r="H61" t="s">
-        <v>11</v>
-      </c>
-      <c r="I61" t="str">
+      <c r="G65" t="s">
+        <v>93</v>
+      </c>
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Alcaldías</v>
-      </c>
-      <c r="J61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B62" t="s">
-        <v>75</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="D62" t="s">
-        <v>12</v>
-      </c>
-      <c r="E62" t="s">
-        <v>47</v>
-      </c>
-      <c r="F62" t="s">
-        <v>188</v>
-      </c>
-      <c r="G62" t="s">
-        <v>79</v>
-      </c>
-      <c r="H62" t="s">
-        <v>11</v>
-      </c>
-      <c r="I62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A63" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B63" t="s">
-        <v>75</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="D63" t="s">
-        <v>179</v>
-      </c>
-      <c r="E63" t="s">
-        <v>16</v>
-      </c>
-      <c r="F63" t="s">
-        <v>16</v>
-      </c>
-      <c r="G63" t="s">
-        <v>180</v>
-      </c>
-      <c r="H63" t="s">
-        <v>11</v>
-      </c>
-      <c r="I63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A64" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B64" t="s">
-        <v>73</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="D64" t="s">
-        <v>13</v>
-      </c>
-      <c r="E64" t="s">
-        <v>24</v>
-      </c>
-      <c r="F64" t="s">
-        <v>24</v>
-      </c>
-      <c r="G64" t="s">
-        <v>82</v>
-      </c>
-      <c r="H64" t="s">
-        <v>11</v>
-      </c>
-      <c r="I64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A65" s="5">
-        <v>46174</v>
-      </c>
-      <c r="B65" t="s">
-        <v>73</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="D65" t="s">
-        <v>12</v>
-      </c>
-      <c r="E65" t="s">
-        <v>14</v>
-      </c>
-      <c r="F65" t="s">
-        <v>14</v>
-      </c>
-      <c r="G65" t="s">
-        <v>82</v>
-      </c>
-      <c r="H65" t="s">
-        <v>11</v>
-      </c>
-      <c r="I65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
       </c>
       <c r="J65" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -3460,104 +3454,172 @@
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B66" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="D66" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E66" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F66" t="s">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="G66" t="s">
-        <v>85</v>
+        <v>186</v>
       </c>
       <c r="H66" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I66" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J66" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="67" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A67" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B67" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="D67" t="s">
         <v>12</v>
       </c>
       <c r="E67" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F67" t="s">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="G67" t="s">
-        <v>193</v>
+        <v>84</v>
       </c>
       <c r="H67" t="s">
         <v>11</v>
       </c>
       <c r="I67" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J67" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" s="5">
-        <v>46174</v>
+        <v>46175</v>
       </c>
       <c r="B68" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="D68" t="s">
         <v>12</v>
       </c>
       <c r="E68" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="F68" t="s">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="G68" t="s">
+        <v>189</v>
+      </c>
+      <c r="H68" t="s">
+        <v>70</v>
+      </c>
+      <c r="I68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A69" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B69" t="s">
+        <v>74</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>190</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" t="s">
+        <v>27</v>
+      </c>
+      <c r="F69" t="s">
         <v>83</v>
       </c>
-      <c r="H68" t="s">
-        <v>11</v>
-      </c>
-      <c r="I68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+      <c r="G69" t="s">
+        <v>171</v>
+      </c>
+      <c r="H69" t="s">
+        <v>11</v>
+      </c>
+      <c r="I69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A70" s="5">
+        <v>46175</v>
+      </c>
+      <c r="B70" t="s">
+        <v>74</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D70" t="s">
+        <v>192</v>
+      </c>
+      <c r="E70" t="s">
+        <v>27</v>
+      </c>
+      <c r="F70" t="s">
+        <v>27</v>
+      </c>
+      <c r="G70" t="s">
+        <v>158</v>
+      </c>
+      <c r="H70" t="s">
+        <v>69</v>
+      </c>
+      <c r="I70" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J70" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
       </c>
     </row>
   </sheetData>
@@ -3615,7 +3677,7 @@
         <v>31</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E3" t="s">
         <v>66</v>
@@ -3651,7 +3713,7 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
         <v>32</v>

</xml_diff>

<commit_message>
Reporte de portadas 050626
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Repositorios GitHub\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75FA5CED-9CD2-4A00-A946-353FF84D68AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31AA2082-0598-49CE-A3E7-046368FEC09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="650" uniqueCount="213">
   <si>
     <t>Fecha</t>
   </si>
@@ -276,24 +276,12 @@
     <t>Sitmah</t>
   </si>
   <si>
-    <t>Intervención extranjera</t>
-  </si>
-  <si>
-    <t>Protección del menor</t>
-  </si>
-  <si>
     <t>Carril confinado</t>
   </si>
   <si>
-    <t>Editorial</t>
-  </si>
-  <si>
     <t>Protesta sindical</t>
   </si>
   <si>
-    <t>CFE</t>
-  </si>
-  <si>
     <t>Effetá</t>
   </si>
   <si>
@@ -306,271 +294,388 @@
     <t>Plaza Juárez</t>
   </si>
   <si>
-    <t>Piden explicación sobre uso de predios al SNTE</t>
-  </si>
-  <si>
-    <t>Conflicto por predio</t>
-  </si>
-  <si>
-    <t>No está prohibida la vuelta a la izquierda</t>
-  </si>
-  <si>
-    <t>La CNTE llama a manifestarse en la entidad</t>
-  </si>
-  <si>
-    <t>Legisladores buscan regular reparto en moto</t>
-  </si>
-  <si>
     <t>Iniciativa</t>
   </si>
   <si>
-    <t>Hidalgo, cuarto lugar en economía informal</t>
-  </si>
-  <si>
-    <t>Informalidad laboral</t>
-  </si>
-  <si>
-    <t>Escuela de La Reforma trabaja con diablitos</t>
-  </si>
-  <si>
     <t>Básica</t>
   </si>
   <si>
-    <t>Infraestructura escolar</t>
-  </si>
-  <si>
-    <t>Entrenan en el Hidalgo</t>
-  </si>
-  <si>
-    <t>Programan caminos artesanales para 2026 en Hidalgo</t>
-  </si>
-  <si>
     <t>SICT</t>
   </si>
   <si>
     <t>Carretera artesanal</t>
   </si>
   <si>
-    <t>Formalizan protección a niñas y niños</t>
-  </si>
-  <si>
-    <t>Buscan cuidar a repartidores</t>
-  </si>
-  <si>
-    <t>Aumentan registros de programas</t>
-  </si>
-  <si>
-    <t>Programas Del Bienestar</t>
-  </si>
-  <si>
     <t>Criterio</t>
   </si>
   <si>
-    <t>Aumentarán a tres carriles el Felipe Ángeles, anuncia Sipdus</t>
-  </si>
-  <si>
     <t>Sipdus</t>
   </si>
   <si>
-    <t>IMCO: ocupa la Bella Airosa 5° lugar nacional en competitividad</t>
-  </si>
-  <si>
-    <t>índice de Competitividad Urbana</t>
-  </si>
-  <si>
-    <t>Pachuca, con el 50% de denuncias por tortura</t>
-  </si>
-  <si>
-    <t>Tortura</t>
-  </si>
-  <si>
-    <t>LA CAPITAL DA UNA TIBIA  BIENVENIDA A SELECCIÓN</t>
-  </si>
-  <si>
-    <t>Tuzos, a un año de la inundación que afectó a más de 200 casas</t>
-  </si>
-  <si>
-    <t>Afectaciones Por Lluvias</t>
-  </si>
-  <si>
-    <t>Sudáfrica cumple sueño de lucho en Pachuca</t>
-  </si>
-  <si>
-    <t>América cierra la era de jardine</t>
-  </si>
-  <si>
     <t>Deportes</t>
   </si>
   <si>
-    <t>Innovación y economía ponen a Pachuca en el top de competitividad</t>
-  </si>
-  <si>
-    <t>índice de competitividad</t>
-  </si>
-  <si>
-    <t>Semestre de crecimiento prevé SHCP</t>
-  </si>
-  <si>
-    <t>Crecimiento Económico</t>
-  </si>
-  <si>
-    <t>Reconoce EU la colaboración de México y respalda su soberanía</t>
-  </si>
-  <si>
     <t>Temas internacionales</t>
   </si>
   <si>
-    <t>AMLO: "por el bien de todos, que regrese el otro Trump"</t>
-  </si>
-  <si>
-    <t>Somos el rival que se quiere evitar""</t>
-  </si>
-  <si>
-    <t>Exhibirán en zona arqueológica pieza del juego de pelota</t>
-  </si>
-  <si>
     <t>INAH</t>
   </si>
   <si>
     <t>Zona Arqueológica</t>
   </si>
   <si>
-    <t>Realizan entrenamiento a puerta cerrada</t>
-  </si>
-  <si>
-    <t>Hidalgo, segundo en crecimiento de trabajo remunerado</t>
-  </si>
-  <si>
-    <t>Empleo formal</t>
-  </si>
-  <si>
-    <t>Gobierno de EU ofrece respeto a la soberanía</t>
-  </si>
-  <si>
-    <t>Tulancingo, último en competitividad urbana</t>
-  </si>
-  <si>
-    <t>Índice de competitividad</t>
-  </si>
-  <si>
-    <t>EU investiga a Durazo y Villarreal</t>
-  </si>
-  <si>
-    <t>Sudáfrica desata la euforia en Pachuca durante entrenamiento</t>
-  </si>
-  <si>
-    <t>Cuando un gobierno extranjero comienza a intervenir en la conversación política interna mexicana, lo que se requiere no es una fotografía bonita para redes sociales. Se necesita cohesión política, respaldo popular y lectura histórica</t>
-  </si>
-  <si>
-    <t>Suma gobierno federal al estado en programa de conservación carretera con inversiones millonarias</t>
-  </si>
-  <si>
-    <t>Rehabilitación carretera</t>
-  </si>
-  <si>
-    <t>Refuerza Hidalgo vigilancia sanitaria por el Mundial 2026; descartan casos de ébola en la entidad</t>
-  </si>
-  <si>
-    <t>Lanzan convocatoria para contratar choferes para el Sistema de Transporte Metropolitano</t>
-  </si>
-  <si>
     <t>Reclutamiento</t>
   </si>
   <si>
-    <t>Vive Pachuca fiebre mundialista con entrenamiento de Sudáfrica en estadio Hidalgo</t>
-  </si>
-  <si>
-    <t>ALcalde y supervisor de CFE se reúnen con comunidades</t>
-  </si>
-  <si>
-    <t>Reunión con funcionario federal</t>
-  </si>
-  <si>
-    <t>Destinó gobierno federal recursos históricos para carreteras</t>
-  </si>
-  <si>
-    <t>Apagón prolongado golpea al municipio de Huejutla</t>
-  </si>
-  <si>
-    <t>Apagones</t>
-  </si>
-  <si>
-    <t>Fortaleza a participación ciudadana y la rendicón de cuentas</t>
-  </si>
-  <si>
-    <t>Contraloría Social</t>
-  </si>
-  <si>
-    <t>Buscan frenar las entregas contrarreloj de apps en Hidalgo</t>
-  </si>
-  <si>
-    <t>Imprudencias involucran al Metropolitano en cuatro incidentes viales</t>
-  </si>
-  <si>
-    <t>Accidente Tuzobús</t>
-  </si>
-  <si>
-    <t>Teman nuevas tragedias</t>
-  </si>
-  <si>
     <t>Atlas de Riesgos</t>
   </si>
   <si>
-    <t>Hubo desaseo legislativo en recorte al IEEH</t>
-  </si>
-  <si>
-    <t>Presupuesto IEEH</t>
-  </si>
-  <si>
-    <t>Hidalgo tendrá siete caminos artesanales con recursos federales</t>
-  </si>
-  <si>
-    <t>Hidalgo, entre los líderes en generación de empleo</t>
-  </si>
-  <si>
-    <t>Generación De Empleo</t>
-  </si>
-  <si>
-    <t>Sudáfrica entrena en el Hidalgo; aficionados les dan bienvenida</t>
-  </si>
-  <si>
-    <t>Realiza IHE etapa estatal de la Olimpiada del Conocimiento Infantil</t>
-  </si>
-  <si>
-    <t>Justa Académica</t>
-  </si>
-  <si>
-    <t>Desazolva Río de las Avenidas ara evitar inundaciones en Los Tuzos</t>
-  </si>
-  <si>
-    <t>Desazolve</t>
-  </si>
-  <si>
-    <t>Día accidentado en Sistema de Transporte Metropolitano: 4 percances</t>
-  </si>
-  <si>
-    <t>Seguridad Pública de Pachuca fortalece acciones preventivas y de proximidad en los barrios altos</t>
-  </si>
-  <si>
     <t>Policía municipal</t>
   </si>
   <si>
     <t>Operativo de Seguridad</t>
   </si>
   <si>
-    <t>A menos de una semana de su lanzamiento, Chocan otra unidad del Transporte Metropolitano</t>
-  </si>
-  <si>
-    <t>Niegan gobemadores que se les haya retirado la visa</t>
-  </si>
-  <si>
-    <t>Siguen los incidentes con unidades nuevas de los llamados (antes) Tuzobuses, pareciera mala suerte, aunque la realidad es que falta respeto a los reglamentos por parte de los conductores, tanto de las unidades de servicio como de los autos en general</t>
-  </si>
-  <si>
-    <t>Exigen destitución de síndico procurador de Singuilucan</t>
-  </si>
-  <si>
     <t>Regidor ebrio</t>
+  </si>
+  <si>
+    <t>Quezada asume dirigencia del PRI en Hidalgo</t>
+  </si>
+  <si>
+    <t>PRI</t>
+  </si>
+  <si>
+    <t>Renovación De Dirigencia</t>
+  </si>
+  <si>
+    <t>El tricolor goleó 5-1 a Servia en amistoso</t>
+  </si>
+  <si>
+    <t>Continúa el problema de basura en Jaltocán</t>
+  </si>
+  <si>
+    <t>Disposición de basura</t>
+  </si>
+  <si>
+    <t>Leyendas: una hechicera del siglo XVIII en Omitlán</t>
+  </si>
+  <si>
+    <t>Temas varios</t>
+  </si>
+  <si>
+    <t>INAH exhibirá el histórico aro del juego de pelota</t>
+  </si>
+  <si>
+    <t>Inicia contienda por la dirigencia del SUTEUAEH</t>
+  </si>
+  <si>
+    <t>Tras detenciones, Tezontepec y Progreso se unen al Mando Coordinado</t>
+  </si>
+  <si>
+    <t>Mando Coordinado</t>
+  </si>
+  <si>
+    <t>Sobrevive tradición</t>
+  </si>
+  <si>
+    <t>“A dos años del triunfo electoral que dio origen al Segundo Piso de la Transformación, la presidenta Claudia Sheinbaum reiteró que México...”</t>
+  </si>
+  <si>
+    <t>Aniversario de la Transformación</t>
+  </si>
+  <si>
+    <t>EL ARBOLITO, ÚNICA ZONA DE RIESGO EN PACHUCA</t>
+  </si>
+  <si>
+    <t>Inversión en Santiago Tulantepec</t>
+  </si>
+  <si>
+    <t>Ruta de la Transformación</t>
+  </si>
+  <si>
+    <t>Sí habrá clases el día de inauguración</t>
+  </si>
+  <si>
+    <t>Capacitarán a funcionarios para erradicar trabajo infantil</t>
+  </si>
+  <si>
+    <t>Erradicación trabajo infantil</t>
+  </si>
+  <si>
+    <t>Adultos mayores irán a los Estados Unidos para ver a su hijo</t>
+  </si>
+  <si>
+    <t>Apoyo A Migrantes</t>
+  </si>
+  <si>
+    <t>Dos funcionarios, con retribuciones externas por más de $3 millones</t>
+  </si>
+  <si>
+    <t>Declaración patrimonial</t>
+  </si>
+  <si>
+    <t>GALARDONAN A  LUY, CARTONISTA  DE CRITERIO</t>
+  </si>
+  <si>
+    <t>Reconocimiento</t>
+  </si>
+  <si>
+    <t>Buscan que acciones afirmativas en las elecciones sean ley</t>
+  </si>
+  <si>
+    <t>Infaltables en la fiesta del futbol</t>
+  </si>
+  <si>
+    <t>Hidalgo gana en terreno arbitral</t>
+  </si>
+  <si>
+    <t>Mando coordinado: dos más se adhieren</t>
+  </si>
+  <si>
+    <t>Para unidades que no tienen seguro, sanciones severas</t>
+  </si>
+  <si>
+    <t>Supervisión de Transporte</t>
+  </si>
+  <si>
+    <t>Plan de desarrollo para la zona está en proceso</t>
+  </si>
+  <si>
+    <t>Tren México Querétaro</t>
+  </si>
+  <si>
+    <t>Se ve obligada a bajar sus precios tras señalamientos</t>
+  </si>
+  <si>
+    <t>Alerta al consumidor</t>
+  </si>
+  <si>
+    <t>Estrena IMSS un quirófano ""inteligente""</t>
+  </si>
+  <si>
+    <t>IMSS</t>
+  </si>
+  <si>
+    <t>Quirófano inteligente</t>
+  </si>
+  <si>
+    <t>Cómo sobrevivir al ""no era penal""</t>
+  </si>
+  <si>
+    <t>Así se habla de Pachuca en medios de Sudáfrica</t>
+  </si>
+  <si>
+    <t>"Negociar cara acara", exige Zelenski a Putin e invita a Estados Unidos y Europa</t>
+  </si>
+  <si>
+    <t>Marjane Satrapi, novelista gráfica, murió de tristeza</t>
+  </si>
+  <si>
+    <t>Cruz Azul regresará al Estadio Banorte</t>
+  </si>
+  <si>
+    <t>JMS condena amenazas del síndico de Singuilucan</t>
+  </si>
+  <si>
+    <t>Aumentan robos y hechos violentos en el Arco Norte</t>
+  </si>
+  <si>
+    <t>Coordinación interestatal</t>
+  </si>
+  <si>
+    <t>Estallido de pipas en Puebla deja tres heridos y 2 mil desalojados</t>
+  </si>
+  <si>
+    <t>La democracia deliberativa, como ejercicio de acción política e incidencia pública, requiere otros  elementos para engrosar el debate de la función gubernamental y contribuir a una rendición de  cuentas más puntual”.</t>
+  </si>
+  <si>
+    <t>Combate a la corrupción</t>
+  </si>
+  <si>
+    <t>Con 27 años de historia, Síntesis Hidalgo apuesta por la innovación con nueva plataforma digital</t>
+  </si>
+  <si>
+    <t>Conmemoración Aniversario</t>
+  </si>
+  <si>
+    <t>Estará lista en noviembre rehabilitación de la Casa del Niño en Pachuca</t>
+  </si>
+  <si>
+    <t>Rehabilitación de instalaciones</t>
+  </si>
+  <si>
+    <t>Se adhiere Progreso de Obregón al Mando Coordinado tras detención de nueve policías</t>
+  </si>
+  <si>
+    <t>Caasim despliega equipo especializado ante pronóstico de lluvias intensas</t>
+  </si>
+  <si>
+    <t>Caasim</t>
+  </si>
+  <si>
+    <t>Prevención de inundaciones</t>
+  </si>
+  <si>
+    <t>Bloquean carretera Huejutla-Tamazunchale</t>
+  </si>
+  <si>
+    <t>Protesta por obra</t>
+  </si>
+  <si>
+    <t>Realiazan aplicación de gelish a bajo costo</t>
+  </si>
+  <si>
+    <t>Católicos participan en multitudinaria procesión de Corpus</t>
+  </si>
+  <si>
+    <t>Llamado a respetar el carril exclusivo de Transporte Metropolitano</t>
+  </si>
+  <si>
+    <t>Predial verde: la propuesta de Naida  Reyna</t>
+  </si>
+  <si>
+    <t>Predial</t>
+  </si>
+  <si>
+    <t>Tras escándalos policiales, Progreso se suma al Mando Coordinado</t>
+  </si>
+  <si>
+    <t>Persecución de terror</t>
+  </si>
+  <si>
+    <t>Combate a la delincuencia</t>
+  </si>
+  <si>
+    <t>Más de 24 horas retenidos</t>
+  </si>
+  <si>
+    <t>Retención de funcionarios</t>
+  </si>
+  <si>
+    <t>Arco Norte: crece la presión vs concesionaria por inseguridad</t>
+  </si>
+  <si>
+    <t>Inseguridad Carretera</t>
+  </si>
+  <si>
+    <t>Marfeca</t>
+  </si>
+  <si>
+    <t>Guardia Nacional despliega operativo de seguridad en el Arco Norte</t>
+  </si>
+  <si>
+    <t>Cintillo</t>
+  </si>
+  <si>
+    <t>GN</t>
+  </si>
+  <si>
+    <t>Zamacona presenta ""Qué Será?"" y proyecta la música electrónica hidalguense hacia eI ámbito internacional</t>
+  </si>
+  <si>
+    <t>"seguimos en la ruta; vamos a redoblar esfuerzos", sostiene Julio Menchaca</t>
+  </si>
+  <si>
+    <t>Congreso de Puebla condecora a Víctor Velázquez por su impulso al deporte</t>
+  </si>
+  <si>
+    <t>Impulso al deporte</t>
+  </si>
+  <si>
+    <t>Atitalaquia presente en la 80 reunión de evaluación del Arco Norte</t>
+  </si>
+  <si>
+    <t>Secundaria Netzahualcóyotl de Tlahuelilpan celebrará medio siglo de historia con carrera atlética</t>
+  </si>
+  <si>
+    <t>Las obras en Tula se deciden con el pueblo y para el pueblo</t>
+  </si>
+  <si>
+    <t>Socialización de obra</t>
+  </si>
+  <si>
+    <t>Comisión de Honor definirá posible sanción a regidores de Morena en Huichapan: Marco Rico</t>
+  </si>
+  <si>
+    <t>Sanción a regidores</t>
+  </si>
+  <si>
+    <t>Atitalaquia vive un hecho histórico de inclusión</t>
+  </si>
+  <si>
+    <t>Lengua De Señas</t>
+  </si>
+  <si>
+    <t>Carretera Atotonilco-Progreso registra 30% de avance en su 2° etapa</t>
+  </si>
+  <si>
+    <t>Ejecución de obras</t>
+  </si>
+  <si>
+    <t>Refuerza Pachuca profesionalización en bienestar animal y conservación de fauna silvestre</t>
+  </si>
+  <si>
+    <t>Conservación Biodiversidad</t>
+  </si>
+  <si>
+    <t>Hidalgo libre de adicciones</t>
+  </si>
+  <si>
+    <t>Publicidad</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo llama a extremar precauciones ante pronóstico de lluvias intensas</t>
+  </si>
+  <si>
+    <t>PC</t>
+  </si>
+  <si>
+    <t>Alerta Meteorológica</t>
+  </si>
+  <si>
+    <t>Impulsa IHE alianzas estratégicas para fortalecer la alfabetización inicial en Hidalgo</t>
+  </si>
+  <si>
+    <t>Alfabetización</t>
+  </si>
+  <si>
+    <t>Refuerza Pachuca capacitación en bienestar animal</t>
+  </si>
+  <si>
+    <t>Protección Biodiversidad</t>
+  </si>
+  <si>
+    <t>¿Buscas trabajo? Abren convocatoria para choferes de transporte metropolitano</t>
+  </si>
+  <si>
+    <t>"Seguimos en la ruta; vamos a redoblar esfuerzos", sostiene Julio Menchaca</t>
+  </si>
+  <si>
+    <t>Construye tu camino</t>
+  </si>
+  <si>
+    <t>Ellos importan</t>
+  </si>
+  <si>
+    <t>Maltrato animal</t>
+  </si>
+  <si>
+    <t>En persecución recuperan tráiler y liberan a plagiado</t>
+  </si>
+  <si>
+    <t>Llama Sitmah a respetar el carril confinado</t>
+  </si>
+  <si>
+    <t>México lo da todo en amistoso contra Serbia</t>
+  </si>
+  <si>
+    <t>Tres lesionados en explosión de tanques de gas en una bodega</t>
+  </si>
+  <si>
+    <t>Explosión De Pipa</t>
+  </si>
+  <si>
+    <t>Califican de ""insuficientes"" las propuestas para el magisterio</t>
   </si>
 </sst>
 </file>
@@ -817,8 +922,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J55" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J55" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J71" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J71" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1184,7 +1289,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J55"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
@@ -1233,32 +1338,32 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B2" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>101</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="H2" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Partidos</v>
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1267,66 +1372,66 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B3" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
       <c r="D3" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
       <c r="F3" t="s">
-        <v>78</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H3" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B4" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>92</v>
+        <v>104</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>83</v>
+        <v>105</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1335,25 +1440,25 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B5" t="s">
         <v>68</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="D5" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="G5" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="H5" t="s">
         <v>11</v>
@@ -1369,164 +1474,164 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B6" t="s">
         <v>68</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>93</v>
       </c>
       <c r="G6" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H6" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B7" t="s">
         <v>68</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>59</v>
       </c>
       <c r="F7" t="s">
-        <v>98</v>
+        <v>59</v>
       </c>
       <c r="G7" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H7" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A8" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B8" t="s">
         <v>77</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="F8" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="G8" t="s">
-        <v>76</v>
+        <v>111</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B9" t="s">
         <v>77</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="D9" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E9" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="G9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B10" t="s">
         <v>77</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F10" t="s">
-        <v>36</v>
+        <v>2</v>
       </c>
       <c r="G10" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="H10" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1539,32 +1644,32 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B11" t="s">
         <v>77</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="F11" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="G11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1573,59 +1678,59 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B12" t="s">
         <v>77</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G12" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B13" t="s">
-        <v>108</v>
+        <v>77</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
       </c>
       <c r="E13" t="s">
-        <v>110</v>
+        <v>26</v>
       </c>
       <c r="F13" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="G13" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
@@ -1639,15 +1744,15 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="D14" t="s">
         <v>12</v>
@@ -1659,7 +1764,7 @@
         <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="H14" t="s">
         <v>11</v>
@@ -1675,100 +1780,100 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" t="s">
+        <v>122</v>
+      </c>
+      <c r="H15" t="s">
+        <v>11</v>
+      </c>
+      <c r="I15" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J15" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A16" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B16" t="s">
+        <v>89</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D16" t="s">
         <v>13</v>
       </c>
-      <c r="E15" t="s">
-        <v>17</v>
-      </c>
-      <c r="F15" t="s">
-        <v>17</v>
-      </c>
-      <c r="G15" t="s">
-        <v>114</v>
-      </c>
-      <c r="H15" t="s">
+      <c r="E16" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" t="s">
+        <v>38</v>
+      </c>
+      <c r="G16" t="s">
+        <v>124</v>
+      </c>
+      <c r="H16" t="s">
         <v>70</v>
       </c>
-      <c r="I15" t="str">
+      <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J15" t="str">
+      <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="5">
-        <v>46177</v>
-      </c>
-      <c r="B16" t="s">
-        <v>108</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="D16" t="s">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A17" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B17" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D17" t="s">
         <v>9</v>
       </c>
-      <c r="E16" t="s">
-        <v>10</v>
-      </c>
-      <c r="F16" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" t="s">
-        <v>76</v>
-      </c>
-      <c r="H16" t="s">
-        <v>11</v>
-      </c>
-      <c r="I16" t="str">
+      <c r="E17" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" t="s">
+        <v>126</v>
+      </c>
+      <c r="H17" t="s">
+        <v>11</v>
+      </c>
+      <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
-      </c>
-      <c r="J16" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A17" s="5">
-        <v>46177</v>
-      </c>
-      <c r="B17" t="s">
-        <v>108</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="D17" t="s">
-        <v>12</v>
-      </c>
-      <c r="E17" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" t="s">
-        <v>117</v>
-      </c>
-      <c r="H17" t="s">
-        <v>11</v>
-      </c>
-      <c r="I17" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1777,25 +1882,25 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B18" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F18" t="s">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G18" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="H18" t="s">
         <v>11</v>
@@ -1811,13 +1916,13 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B19" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="D19" t="s">
         <v>12</v>
@@ -1829,7 +1934,7 @@
         <v>10</v>
       </c>
       <c r="G19" t="s">
-        <v>120</v>
+        <v>76</v>
       </c>
       <c r="H19" t="s">
         <v>11</v>
@@ -1843,34 +1948,34 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B20" t="s">
-        <v>67</v>
+        <v>89</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="D20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G20" t="s">
-        <v>122</v>
+        <v>91</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1879,100 +1984,100 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B21" t="s">
         <v>67</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D21" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E21" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F21" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G21" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="H21" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B22" t="s">
         <v>67</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="D22" t="s">
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="F22" t="s">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="G22" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H22" t="s">
         <v>11</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B23" t="s">
         <v>67</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F23" t="s">
-        <v>10</v>
+        <v>87</v>
       </c>
       <c r="G23" t="s">
-        <v>79</v>
+        <v>134</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
       </c>
       <c r="I23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J23" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -1981,32 +2086,32 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B24" t="s">
         <v>67</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F24" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>76</v>
+        <v>136</v>
       </c>
       <c r="H24" t="s">
         <v>11</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2015,13 +2120,13 @@
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B25" t="s">
         <v>67</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="D25" t="s">
         <v>12</v>
@@ -2030,10 +2135,10 @@
         <v>14</v>
       </c>
       <c r="F25" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="G25" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="H25" t="s">
         <v>11</v>
@@ -2049,16 +2154,16 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B26" t="s">
         <v>67</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="D26" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E26" t="s">
         <v>10</v>
@@ -2083,66 +2188,66 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="D27" t="s">
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="F27" t="s">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="G27" t="s">
-        <v>134</v>
+        <v>76</v>
       </c>
       <c r="H27" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="D28" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G28" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="H28" t="s">
         <v>11</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2151,32 +2256,32 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
+        <v>67</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F29" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G29" t="s">
-        <v>137</v>
+        <v>107</v>
       </c>
       <c r="H29" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2185,195 +2290,195 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B30" t="s">
         <v>74</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="D30" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E30" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F30" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G30" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="H30" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B31" t="s">
         <v>74</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="D31" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F31" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G31" t="s">
-        <v>76</v>
+        <v>99</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B32" t="s">
         <v>74</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="D32" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E32" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="F32" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="G32" t="s">
-        <v>79</v>
+        <v>147</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A33" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F33" t="s">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="G33" t="s">
-        <v>142</v>
+        <v>107</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" ht="58" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="D34" t="s">
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F34" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G34" t="s">
-        <v>76</v>
+        <v>150</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="35" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B35" t="s">
         <v>72</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="D35" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="F35" t="s">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="G35" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
@@ -2389,127 +2494,127 @@
     </row>
     <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A36" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B36" t="s">
         <v>72</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="D36" t="s">
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="F36" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="G36" t="s">
-        <v>76</v>
+        <v>154</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
       </c>
       <c r="I36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A37" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="D37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F37" t="s">
-        <v>86</v>
+        <v>22</v>
       </c>
       <c r="G37" t="s">
-        <v>148</v>
+        <v>111</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A38" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B38" t="s">
         <v>71</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="D38" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E38" t="s">
-        <v>14</v>
+        <v>90</v>
       </c>
       <c r="F38" t="s">
-        <v>102</v>
+        <v>157</v>
       </c>
       <c r="G38" t="s">
-        <v>142</v>
+        <v>158</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B39" t="s">
         <v>71</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="D39" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E39" t="s">
         <v>14</v>
       </c>
       <c r="F39" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G39" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="H39" t="s">
         <v>70</v>
@@ -2525,59 +2630,59 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B40" t="s">
         <v>71</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="F40" t="s">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G40" t="s">
-        <v>153</v>
+        <v>107</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B41" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="F41" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="G41" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
@@ -2593,13 +2698,13 @@
     </row>
     <row r="42" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A42" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B42" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="D42" t="s">
         <v>12</v>
@@ -2611,10 +2716,10 @@
         <v>78</v>
       </c>
       <c r="G42" t="s">
-        <v>156</v>
+        <v>79</v>
       </c>
       <c r="H42" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2627,13 +2732,13 @@
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B43" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="D43" t="s">
         <v>12</v>
@@ -2645,7 +2750,7 @@
         <v>16</v>
       </c>
       <c r="G43" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="H43" t="s">
         <v>11</v>
@@ -2659,234 +2764,234 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A44" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B44" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="D44" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E44" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="F44" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="G44" t="s">
-        <v>160</v>
+        <v>111</v>
       </c>
       <c r="H44" t="s">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="I44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B45" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="D45" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E45" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F45" t="s">
-        <v>102</v>
+        <v>22</v>
       </c>
       <c r="G45" t="s">
-        <v>142</v>
+        <v>168</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B46" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>56</v>
+        <v>16</v>
       </c>
       <c r="F46" t="s">
-        <v>56</v>
+        <v>97</v>
       </c>
       <c r="G46" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="H46" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J46" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A47" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B47" t="s">
+        <v>81</v>
+      </c>
+      <c r="C47" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D47" t="s">
+        <v>12</v>
+      </c>
+      <c r="E47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F47" t="s">
+        <v>23</v>
+      </c>
+      <c r="G47" t="s">
+        <v>172</v>
+      </c>
+      <c r="H47" t="s">
+        <v>11</v>
+      </c>
+      <c r="I47" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J46" t="str">
+      <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A47" s="5">
-        <v>46177</v>
-      </c>
-      <c r="B47" t="s">
-        <v>73</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>164</v>
-      </c>
-      <c r="D47" t="s">
-        <v>13</v>
-      </c>
-      <c r="E47" t="s">
-        <v>10</v>
-      </c>
-      <c r="F47" t="s">
-        <v>10</v>
-      </c>
-      <c r="G47" t="s">
-        <v>76</v>
-      </c>
-      <c r="H47" t="s">
-        <v>11</v>
-      </c>
-      <c r="I47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
       </c>
     </row>
     <row r="48" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A48" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B48" t="s">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="D48" t="s">
-        <v>12</v>
+        <v>175</v>
       </c>
       <c r="E48" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="F48" t="s">
-        <v>87</v>
+        <v>176</v>
       </c>
       <c r="G48" t="s">
-        <v>166</v>
+        <v>98</v>
       </c>
       <c r="H48" t="s">
         <v>11</v>
       </c>
       <c r="I48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J48" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="49" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A49" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B49" t="s">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="D49" t="s">
         <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>110</v>
+        <v>10</v>
       </c>
       <c r="F49" t="s">
-        <v>110</v>
+        <v>10</v>
       </c>
       <c r="G49" t="s">
-        <v>168</v>
+        <v>107</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>otros</v>
       </c>
     </row>
     <row r="50" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="D50" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E50" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="F50" t="s">
-        <v>78</v>
+        <v>24</v>
       </c>
       <c r="G50" t="s">
-        <v>156</v>
+        <v>117</v>
       </c>
       <c r="H50" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2894,37 +2999,37 @@
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A51" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B51" t="s">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="D51" t="s">
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F51" t="s">
-        <v>171</v>
+        <v>10</v>
       </c>
       <c r="G51" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
@@ -2933,136 +3038,680 @@
     </row>
     <row r="52" spans="1:10" ht="29" x14ac:dyDescent="0.35">
       <c r="A52" s="5">
-        <v>46177</v>
+        <v>46178</v>
       </c>
       <c r="B52" t="s">
+        <v>173</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="D52" t="s">
+        <v>12</v>
+      </c>
+      <c r="E52" t="s">
+        <v>23</v>
+      </c>
+      <c r="F52" t="s">
+        <v>2</v>
+      </c>
+      <c r="G52" t="s">
+        <v>147</v>
+      </c>
+      <c r="H52" t="s">
+        <v>11</v>
+      </c>
+      <c r="I52" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J52" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A53" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B53" t="s">
+        <v>173</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D53" t="s">
+        <v>12</v>
+      </c>
+      <c r="E53" t="s">
+        <v>10</v>
+      </c>
+      <c r="F53" t="s">
+        <v>10</v>
+      </c>
+      <c r="G53" t="s">
+        <v>152</v>
+      </c>
+      <c r="H53" t="s">
+        <v>11</v>
+      </c>
+      <c r="I53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J53" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A54" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B54" t="s">
+        <v>173</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="D54" t="s">
+        <v>12</v>
+      </c>
+      <c r="E54" t="s">
+        <v>16</v>
+      </c>
+      <c r="F54" t="s">
+        <v>82</v>
+      </c>
+      <c r="G54" t="s">
+        <v>184</v>
+      </c>
+      <c r="H54" t="s">
+        <v>11</v>
+      </c>
+      <c r="I54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J54" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A55" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B55" t="s">
+        <v>173</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="D55" t="s">
+        <v>12</v>
+      </c>
+      <c r="E55" t="s">
+        <v>18</v>
+      </c>
+      <c r="F55" t="s">
+        <v>2</v>
+      </c>
+      <c r="G55" t="s">
+        <v>186</v>
+      </c>
+      <c r="H55" t="s">
+        <v>11</v>
+      </c>
+      <c r="I55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Partidos</v>
+      </c>
+      <c r="J55" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A56" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B56" t="s">
+        <v>173</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="D56" t="s">
+        <v>12</v>
+      </c>
+      <c r="E56" t="s">
+        <v>16</v>
+      </c>
+      <c r="F56" t="s">
+        <v>16</v>
+      </c>
+      <c r="G56" t="s">
+        <v>188</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="I56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J56" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A57" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B57" t="s">
+        <v>173</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>189</v>
+      </c>
+      <c r="D57" t="s">
+        <v>12</v>
+      </c>
+      <c r="E57" t="s">
+        <v>16</v>
+      </c>
+      <c r="F57" t="s">
+        <v>16</v>
+      </c>
+      <c r="G57" t="s">
+        <v>190</v>
+      </c>
+      <c r="H57" t="s">
+        <v>11</v>
+      </c>
+      <c r="I57" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J57" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A58" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B58" t="s">
+        <v>173</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="D58" t="s">
+        <v>12</v>
+      </c>
+      <c r="E58" t="s">
+        <v>16</v>
+      </c>
+      <c r="F58" t="s">
+        <v>16</v>
+      </c>
+      <c r="G58" t="s">
+        <v>192</v>
+      </c>
+      <c r="H58" t="s">
+        <v>11</v>
+      </c>
+      <c r="I58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J58" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A59" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B59" t="s">
+        <v>173</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="D59" t="s">
+        <v>194</v>
+      </c>
+      <c r="E59" t="s">
+        <v>22</v>
+      </c>
+      <c r="F59" t="s">
+        <v>22</v>
+      </c>
+      <c r="G59" t="s">
+        <v>98</v>
+      </c>
+      <c r="H59" t="s">
+        <v>11</v>
+      </c>
+      <c r="I59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A60" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B60" t="s">
+        <v>73</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D60" t="s">
+        <v>13</v>
+      </c>
+      <c r="E60" t="s">
+        <v>23</v>
+      </c>
+      <c r="F60" t="s">
+        <v>196</v>
+      </c>
+      <c r="G60" t="s">
+        <v>197</v>
+      </c>
+      <c r="H60" t="s">
+        <v>11</v>
+      </c>
+      <c r="I60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A61" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B61" t="s">
+        <v>73</v>
+      </c>
+      <c r="C61" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" t="s">
+        <v>26</v>
+      </c>
+      <c r="F61" t="s">
+        <v>83</v>
+      </c>
+      <c r="G61" t="s">
+        <v>199</v>
+      </c>
+      <c r="H61" t="s">
+        <v>11</v>
+      </c>
+      <c r="I61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J61" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A62" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B62" t="s">
+        <v>73</v>
+      </c>
+      <c r="C62" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="D62" t="s">
+        <v>12</v>
+      </c>
+      <c r="E62" t="s">
+        <v>16</v>
+      </c>
+      <c r="F62" t="s">
+        <v>16</v>
+      </c>
+      <c r="G62" t="s">
+        <v>201</v>
+      </c>
+      <c r="H62" t="s">
+        <v>11</v>
+      </c>
+      <c r="I62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J62" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A63" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B63" t="s">
+        <v>73</v>
+      </c>
+      <c r="C63" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="D63" t="s">
+        <v>12</v>
+      </c>
+      <c r="E63" t="s">
+        <v>27</v>
+      </c>
+      <c r="F63" t="s">
+        <v>78</v>
+      </c>
+      <c r="G63" t="s">
+        <v>95</v>
+      </c>
+      <c r="H63" t="s">
+        <v>11</v>
+      </c>
+      <c r="I63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J63" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A64" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B64" t="s">
+        <v>73</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="D64" t="s">
+        <v>12</v>
+      </c>
+      <c r="E64" t="s">
+        <v>24</v>
+      </c>
+      <c r="F64" t="s">
+        <v>24</v>
+      </c>
+      <c r="G64" t="s">
+        <v>117</v>
+      </c>
+      <c r="H64" t="s">
+        <v>11</v>
+      </c>
+      <c r="I64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J64" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A65" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B65" t="s">
+        <v>73</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="D65" t="s">
+        <v>194</v>
+      </c>
+      <c r="E65" t="s">
+        <v>90</v>
+      </c>
+      <c r="F65" t="s">
+        <v>90</v>
+      </c>
+      <c r="G65" t="s">
         <v>88</v>
       </c>
-      <c r="C52" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="D52" t="s">
+      <c r="H65" t="s">
+        <v>11</v>
+      </c>
+      <c r="I65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J65" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A66" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B66" t="s">
+        <v>73</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="D66" t="s">
+        <v>194</v>
+      </c>
+      <c r="E66" t="s">
+        <v>16</v>
+      </c>
+      <c r="F66" t="s">
+        <v>16</v>
+      </c>
+      <c r="G66" t="s">
+        <v>206</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="I66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J66" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A67" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B67" t="s">
+        <v>84</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="D67" t="s">
         <v>13</v>
       </c>
-      <c r="E52" t="s">
+      <c r="E67" t="s">
+        <v>22</v>
+      </c>
+      <c r="F67" t="s">
+        <v>22</v>
+      </c>
+      <c r="G67" t="s">
+        <v>168</v>
+      </c>
+      <c r="H67" t="s">
+        <v>69</v>
+      </c>
+      <c r="I67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J67" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A68" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B68" t="s">
+        <v>84</v>
+      </c>
+      <c r="C68" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="D68" t="s">
+        <v>12</v>
+      </c>
+      <c r="E68" t="s">
         <v>27</v>
       </c>
-      <c r="F52" t="s">
+      <c r="F68" t="s">
         <v>78</v>
       </c>
-      <c r="G52" t="s">
-        <v>156</v>
-      </c>
-      <c r="H52" t="s">
+      <c r="G68" t="s">
+        <v>79</v>
+      </c>
+      <c r="H68" t="s">
+        <v>11</v>
+      </c>
+      <c r="I68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J68" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A69" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B69" t="s">
+        <v>84</v>
+      </c>
+      <c r="C69" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="D69" t="s">
+        <v>12</v>
+      </c>
+      <c r="E69" t="s">
+        <v>10</v>
+      </c>
+      <c r="F69" t="s">
+        <v>10</v>
+      </c>
+      <c r="G69" t="s">
+        <v>76</v>
+      </c>
+      <c r="H69" t="s">
+        <v>11</v>
+      </c>
+      <c r="I69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J69" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A70" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B70" t="s">
+        <v>84</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="D70" t="s">
+        <v>12</v>
+      </c>
+      <c r="E70" t="s">
+        <v>10</v>
+      </c>
+      <c r="F70" t="s">
+        <v>10</v>
+      </c>
+      <c r="G70" t="s">
+        <v>211</v>
+      </c>
+      <c r="H70" t="s">
+        <v>11</v>
+      </c>
+      <c r="I70" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J70" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+      <c r="A71" s="5">
+        <v>46178</v>
+      </c>
+      <c r="B71" t="s">
+        <v>84</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D71" t="s">
+        <v>12</v>
+      </c>
+      <c r="E71" t="s">
+        <v>14</v>
+      </c>
+      <c r="F71" t="s">
+        <v>14</v>
+      </c>
+      <c r="G71" t="s">
+        <v>80</v>
+      </c>
+      <c r="H71" t="s">
         <v>70</v>
       </c>
-      <c r="I52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J52" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A53" s="5">
-        <v>46177</v>
-      </c>
-      <c r="B53" t="s">
-        <v>88</v>
-      </c>
-      <c r="C53" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="D53" t="s">
-        <v>12</v>
-      </c>
-      <c r="E53" t="s">
-        <v>10</v>
-      </c>
-      <c r="F53" t="s">
-        <v>10</v>
-      </c>
-      <c r="G53" t="s">
-        <v>79</v>
-      </c>
-      <c r="H53" t="s">
-        <v>11</v>
-      </c>
-      <c r="I53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J53" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="72.5" x14ac:dyDescent="0.35">
-      <c r="A54" s="5">
-        <v>46177</v>
-      </c>
-      <c r="B54" t="s">
-        <v>88</v>
-      </c>
-      <c r="C54" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="D54" t="s">
-        <v>82</v>
-      </c>
-      <c r="E54" t="s">
-        <v>27</v>
-      </c>
-      <c r="F54" t="s">
-        <v>78</v>
-      </c>
-      <c r="G54" t="s">
-        <v>156</v>
-      </c>
-      <c r="H54" t="s">
-        <v>11</v>
-      </c>
-      <c r="I54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J54" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A55" s="5">
-        <v>46177</v>
-      </c>
-      <c r="B55" t="s">
-        <v>88</v>
-      </c>
-      <c r="C55" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="D55" t="s">
-        <v>12</v>
-      </c>
-      <c r="E55" t="s">
-        <v>16</v>
-      </c>
-      <c r="F55" t="s">
-        <v>16</v>
-      </c>
-      <c r="G55" t="s">
-        <v>177</v>
-      </c>
-      <c r="H55" t="s">
-        <v>70</v>
-      </c>
-      <c r="I55" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J55" t="str">
+      <c r="I71" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Presidencia de la República</v>
+      </c>
+      <c r="J71" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>

</xml_diff>

<commit_message>
Reporte portadas que no envié
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Repositorios GitHub\Reporteportadas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC186A7E-F025-41E8-94C6-DEFBE7F7192B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ED9741C-4555-46D9-AD38-635B08FA2F49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="172">
   <si>
     <t>Fecha</t>
   </si>
@@ -276,18 +276,9 @@
     <t>El Universal Hidalgo</t>
   </si>
   <si>
-    <t>Sipdus</t>
-  </si>
-  <si>
     <t>Marfeca</t>
   </si>
   <si>
-    <t>Cintillo</t>
-  </si>
-  <si>
-    <t>Alcalde</t>
-  </si>
-  <si>
     <t>Relleno Sanitario</t>
   </si>
   <si>
@@ -297,397 +288,271 @@
     <t>Temas internacionales</t>
   </si>
   <si>
-    <t>Justa Deportiva</t>
-  </si>
-  <si>
     <t>Negativa</t>
   </si>
   <si>
-    <t>Parque Fotovoltaico</t>
-  </si>
-  <si>
     <t>CBPEH</t>
   </si>
   <si>
     <t>Búsqueda de personas</t>
   </si>
   <si>
-    <t>Básica</t>
-  </si>
-  <si>
-    <t>Inclusión</t>
-  </si>
-  <si>
-    <t>Tauromaquia</t>
-  </si>
-  <si>
     <t>Pachuca Brilla</t>
   </si>
   <si>
-    <t>Afectaciones Por Lluvias</t>
-  </si>
-  <si>
-    <t>OEEH</t>
-  </si>
-  <si>
-    <t>Feria Pachuca</t>
-  </si>
-  <si>
-    <t>Apuestas dañan la salud mental</t>
-  </si>
-  <si>
-    <t>Prevención De Adicciones</t>
-  </si>
-  <si>
-    <t>Paraguay elimina a Alemania 3-4</t>
-  </si>
-  <si>
-    <t>Piden concluir obras en vialidad</t>
-  </si>
-  <si>
-    <t>Obras públicas</t>
-  </si>
-  <si>
-    <t>Obra inconclusa</t>
-  </si>
-  <si>
-    <t>Hasta 80 pesos el kilo de aguacate y manzana</t>
-  </si>
-  <si>
-    <t>Inflación</t>
-  </si>
-  <si>
-    <t>SEPH ha autorizado más de 2 mil permisos</t>
-  </si>
-  <si>
     <t>Solicitud De Licencia</t>
   </si>
   <si>
-    <t>A revisión, concesiones sin uso</t>
-  </si>
-  <si>
-    <t>Concesiones transporte público</t>
-  </si>
-  <si>
-    <t>Altos mandos del INE se llevan $654 mil cada mes</t>
-  </si>
-  <si>
-    <t>Tabulador salarial</t>
-  </si>
-  <si>
-    <t>Topo hidalguense se suma a las labores de rescate en Venezuela</t>
-  </si>
-  <si>
-    <t>Ayuda humanitaria</t>
-  </si>
-  <si>
-    <t>Descubren tiradero ilegal en Tezontepec</t>
-  </si>
-  <si>
-    <t>Basurero Clandestino</t>
-  </si>
-  <si>
-    <t>Proeza guaraní elimina a Alemania</t>
-  </si>
-  <si>
-    <t>Trituradoras de lirio requieren 800 litros de diésel al día</t>
-  </si>
-  <si>
-    <t>Conagua</t>
-  </si>
-  <si>
-    <t>Control lirio acuático</t>
-  </si>
-  <si>
-    <t>Amplían búsqueda por trabajadores de la CFE</t>
-  </si>
-  <si>
-    <t>Autoridades estatales perfilan multas que podrían alcanzar hasta 1.2 millones de pesos por tiradero</t>
-  </si>
-  <si>
-    <t>Hoy, México vs Ecuador</t>
-  </si>
-  <si>
-    <t>México y Ecuador, choque de poder</t>
-  </si>
-  <si>
-    <t>Lucha comunidad vs parque fotovoltaico</t>
-  </si>
-  <si>
-    <t>Medio ambiente</t>
-  </si>
-  <si>
-    <t>Indagan tres quejas por uso arbitrario de la fuerza</t>
-  </si>
-  <si>
-    <t>Queja CNDH</t>
-  </si>
-  <si>
-    <t>Niega Ortigoza notificación legal de los colectivos por tauromaquia</t>
-  </si>
-  <si>
-    <t>Coesbioh</t>
-  </si>
-  <si>
-    <t>Destinarán 5.3 mdp para pavimentación de una calle en la colonia Periodistas</t>
-  </si>
-  <si>
     <t>Rehabilitación Vial</t>
   </si>
   <si>
-    <t>A todo caso de desaparición se le pone atención"": Julio Menchaca</t>
-  </si>
-  <si>
-    <t>Hidalgo es cuarto lugar nacional por jóvenes en conflicto con la ley</t>
-  </si>
-  <si>
-    <t>Incidencia Delictiva</t>
-  </si>
-  <si>
-    <t>Sanciones son por portación de armas y narcomenudeo</t>
-  </si>
-  <si>
-    <t>Identifican deficiencias en centros de internamiento</t>
-  </si>
-  <si>
-    <t>Deficiencias en penales</t>
-  </si>
-  <si>
-    <t>Impulsan a servidores con alguna discapacidad</t>
-  </si>
-  <si>
-    <t>Países Bajos y Alemania vuelven a casa</t>
-  </si>
-  <si>
-    <t>Cae 50% decomiso de armas por relajación de Estados Unidos y las nuevas rutas</t>
-  </si>
-  <si>
-    <t>Respaldan ciudadanos a Sheinbaum y militares</t>
-  </si>
-  <si>
-    <t>Respaldo a Sheinbaum</t>
-  </si>
-  <si>
-    <t>Los cárteles contaminan el futbol de barrio</t>
-  </si>
-  <si>
-    <t>CFE: refuerzan operativo para localizar a 2 de sus empleados</t>
-  </si>
-  <si>
-    <t>Continúa búsqueda de dos trabajadores de la CFE: Menchaca</t>
-  </si>
-  <si>
-    <t>Hallan tiradero clandestino de 5 hectáreas en Tezontepec</t>
-  </si>
-  <si>
-    <t>Sheinbaum exige ""todo el peso de la ley"" para director de Pemex</t>
-  </si>
-  <si>
-    <t>Violencia De Género</t>
-  </si>
-  <si>
-    <t>Vecinos bloquean el Minero; exigen reparar daños por inundaciones</t>
-  </si>
-  <si>
-    <t>La diferencia entre Colombia y México no es que uno tenga onda regresiva. La diferencia es que uno tiene  oposición real, aunque sea de derecha, y el otro tiene fragmentación, nostalgia y crítica sin respuestas”.</t>
-  </si>
-  <si>
-    <t>Coordinan Hidalgo y Puebla búsqueda de dos trabajadores desaparecidos de la CFE</t>
-  </si>
-  <si>
-    <t>Pachuca, sede de Congreso Nacional de personas Servidoras Públicas con Discapacidad</t>
-  </si>
-  <si>
-    <t>inclusión</t>
-  </si>
-  <si>
-    <t>Exhibe Semarnath tiraderos clandestinos en Tezontepec de Aldama</t>
-  </si>
-  <si>
-    <t>Fiscalizará Auditoría Superior del Estado recursos federales transferidos a municipios</t>
-  </si>
-  <si>
     <t>ASEH</t>
   </si>
   <si>
-    <t>Fiscalización</t>
-  </si>
-  <si>
-    <t>Alberga el Museo del Santo la exhibición ""El Rostro del Combate""</t>
-  </si>
-  <si>
-    <t>Exposición cultural</t>
-  </si>
-  <si>
-    <t>Gobierno de Hidalgo responde con inversión, ciencia y coordinación a los retos ambientales</t>
-  </si>
-  <si>
-    <t>Sembrando vida impulsa obras de captación de agua en la Región Huasteca</t>
-  </si>
-  <si>
-    <t>Captación De Agua</t>
-  </si>
-  <si>
-    <t>Padres exigen justicia para niños arrollados</t>
-  </si>
-  <si>
     <t>Atropellamiento</t>
   </si>
   <si>
-    <t>Dan mantenimiento al sistema pluvial del mercado</t>
-  </si>
-  <si>
-    <t>Infraestructura Hidráulica</t>
-  </si>
-  <si>
-    <t>Alertan por mayor infestación de gusano barrenador en perros callejeros</t>
-  </si>
-  <si>
-    <t>Gusano barrenador</t>
-  </si>
-  <si>
-    <t>Gabinete de seguridad de Hidalgo consolida atención a emergencias mediante el C5i</t>
-  </si>
-  <si>
-    <t>Reunión Gabinete De Seguridad</t>
-  </si>
-  <si>
-    <t>ASEH asume nuevas facultades para auditar recursos federales</t>
-  </si>
-  <si>
-    <t>Orgullo garza en Polonia</t>
-  </si>
-  <si>
-    <t>Intercambio académico</t>
-  </si>
-  <si>
-    <t>Tezontepec rechaza relleno sanitario, pero alberga tiraderos a cielo abierto</t>
-  </si>
-  <si>
-    <t>No todo ejercicio policial es represión"": Menchaca</t>
-  </si>
-  <si>
-    <t>Represión policial</t>
-  </si>
-  <si>
-    <t>Continúa operativo por trabajadores de CFE</t>
-  </si>
-  <si>
-    <t>Investigan tiraderos clandestinos de escombro</t>
-  </si>
-  <si>
-    <t>Créditos Infonavit ya se pueden pagar en Oxxo</t>
-  </si>
-  <si>
-    <t>Firma De Convenio</t>
-  </si>
-  <si>
-    <t>Descubren estructura de élite y lápidas toltecas grabadas en salvamento arqueológico</t>
-  </si>
-  <si>
     <t>INAH</t>
   </si>
   <si>
-    <t>Vestigios Arqueológicos</t>
-  </si>
-  <si>
-    <t>Julio Menchaca promueve un Hidalgo incluyente</t>
-  </si>
-  <si>
-    <t>Gabinete de seguridad de HIdalgo consolida atención a emergencias mediante el C5i</t>
-  </si>
-  <si>
-    <t>Tula se suma al Mundial Social 2026 con la rehabilitación y entrega de una cancha de futbol 5</t>
-  </si>
-  <si>
-    <t>Claudia Sandoval entrega a Congreso modificación a ley de ingresos, busca dar certeza al desarrollo urbano</t>
-  </si>
-  <si>
-    <t>Ley De Ingresos</t>
-  </si>
-  <si>
-    <t>Zitlaly Zúñiga impulsa coordinación con el DIFH para fortalecer los programas de asistencia</t>
-  </si>
-  <si>
-    <t>Coordinación Interinstitucional</t>
-  </si>
-  <si>
-    <t>Cabildo aprueba 2 reglamentos clave para dar certeza a empresas y proteger a las familias de Atitalaquia</t>
-  </si>
-  <si>
-    <t>Actualización de reglamentos</t>
-  </si>
-  <si>
-    <t>PC de Atitalaquia atiende accidente en la zona centro</t>
-  </si>
-  <si>
-    <t>Accidente Vial</t>
-  </si>
-  <si>
-    <t>Asegura policía de Pachuca a personas por presuntos delitos contra la salud</t>
-  </si>
-  <si>
     <t>Policía municipal</t>
   </si>
   <si>
-    <t>Combate Al Narcomenudeo</t>
-  </si>
-  <si>
-    <t>El deporte, el arte y la cultura fortalecen la unidad del magisterio hidalguense</t>
-  </si>
-  <si>
-    <t>Ellos importan, esteriliza</t>
-  </si>
-  <si>
-    <t>Bienestar Animal</t>
-  </si>
-  <si>
-    <t>Julio Menchaca promueve un estado incluyente</t>
-  </si>
-  <si>
-    <t>Hidalgo fortalece la protección de su riqueza natural</t>
-  </si>
-  <si>
-    <t>Protección ambiental</t>
-  </si>
-  <si>
-    <t>Enfrenta México a Ecuador en 16vos del Mundial</t>
-  </si>
-  <si>
-    <t>Grupo Firme, primeros confirmados al Palenque Pchuca 2026</t>
-  </si>
-  <si>
-    <t>Impulsa IHE acciones para fortalecer la educación inicial</t>
-  </si>
-  <si>
-    <t>IHE</t>
-  </si>
-  <si>
-    <t>Educación inicial</t>
-  </si>
-  <si>
     <t>Huracanes y ciclones</t>
   </si>
   <si>
     <t>Prevención De Riesgos</t>
   </si>
   <si>
-    <t>Por obras inconclusas, bloquean bulevares Minero y Colosio</t>
-  </si>
-  <si>
-    <t>Capturan a tres que robaban motocicletas en Pachuca</t>
-  </si>
-  <si>
     <t>Combate a la delincuencia</t>
   </si>
   <si>
-    <t>Postergan audiencia por caso de triple feminicidio</t>
-  </si>
-  <si>
-    <t>Exigen Esclarecer Feminicidio</t>
-  </si>
-  <si>
-    <t>Continúa búsqueda de dos trabajadores de CFE</t>
+    <t>México la rompe</t>
+  </si>
+  <si>
+    <t>Auditoría avala manejo fiscal en Hidalgo con resultado de 2025</t>
+  </si>
+  <si>
+    <t>Cuenta Pública</t>
+  </si>
+  <si>
+    <t>Reporta SEPH 32 trabajadores con licencia sin goce de sueldo</t>
+  </si>
+  <si>
+    <t>Preservan parte del antiguo Camino Real en Tepeji del Río</t>
+  </si>
+  <si>
+    <t>Conservación del Patrimonio Cultural</t>
+  </si>
+  <si>
+    <t>ASEH halla anomalías por $46.3 millones</t>
+  </si>
+  <si>
+    <t>Irregularidades ASEH</t>
+  </si>
+  <si>
+    <t>¡Y, sí!</t>
+  </si>
+  <si>
+    <t>Sin observaciones, la Cuenta Pública 2025 del estado de Hidalgo</t>
+  </si>
+  <si>
+    <t>Suman 18 túneles para traficar huachicol</t>
+  </si>
+  <si>
+    <t>Gabinete de seguridad</t>
+  </si>
+  <si>
+    <t>Huachitúnel</t>
+  </si>
+  <si>
+    <t>El robo del balneario Dios Padre asciende a $9 millones</t>
+  </si>
+  <si>
+    <t>Asalto a balneario</t>
+  </si>
+  <si>
+    <t>En cinco años, suman 61 denuncias por aborto</t>
+  </si>
+  <si>
+    <t>ILE</t>
+  </si>
+  <si>
+    <t>Por robo de $9 millones, habrá diálogo con los de Dios Padre</t>
+  </si>
+  <si>
+    <t>OBSERVA ASEH A ENTES MÁS DE $46 MILLONES</t>
+  </si>
+  <si>
+    <t>Observaciones ASEH</t>
+  </si>
+  <si>
+    <t>El Tri da el golpe</t>
+  </si>
+  <si>
+    <t>Autoridades destruyen huachitúnel en Pachuca</t>
+  </si>
+  <si>
+    <t>Celebran pachuqueños triunfo de México</t>
+  </si>
+  <si>
+    <t>Hidalgo, sin señalamientos en la cuenta pública 2025</t>
+  </si>
+  <si>
+    <t>Concentran municipios casi 70% de observaciones en 2025: ASEH</t>
+  </si>
+  <si>
+    <t>Corte preserva nacionalidad por nacimiento y frena a Trump</t>
+  </si>
+  <si>
+    <t>Detectan 18 estructuras en la entidad; serán derribadas</t>
+  </si>
+  <si>
+    <t>Imbatible. Un 2-0 sin tacha desata festejos apoteósicos</t>
+  </si>
+  <si>
+    <t>Prosiguen irregularidades en Tula; deberán aclarar destino de $17 millones</t>
+  </si>
+  <si>
+    <t>Van cuatro huachitúneles inhabilitados; aún faltan 14</t>
+  </si>
+  <si>
+    <t>El futuro del T-Mec está en manos de Trump</t>
+  </si>
+  <si>
+    <t>México tiene noche redonda y Jiménez la firma con su garra hidalguense</t>
+  </si>
+  <si>
+    <t>Ojalá que Adolfo y Marco Antonio regresen con vida. Ojalá que las autoridades esclarezcan los hechos y, ojalá, lo más pronto posible, la desaparición deje de ser una situación cotidiana en nuestra sociedad”.</t>
+  </si>
+  <si>
+    <t>¡Y sí! México invicto y en octavos de final</t>
+  </si>
+  <si>
+    <t>Emociona Selección Mexicana a la afición pachuqueña</t>
+  </si>
+  <si>
+    <t>Destruyen túnel utilizado para robo de hidrocarburo en Pachuca</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo sin observaciones por la ASF</t>
+  </si>
+  <si>
+    <t>Robo en balneario Dios Padre supera los 9 mdp: PGJEH</t>
+  </si>
+  <si>
+    <t>Obtiene Hidalgo resultados favorables sin observaciones de Auditoría Superior</t>
+  </si>
+  <si>
+    <t>Cuenta pública</t>
+  </si>
+  <si>
+    <t>Más de 17 millones de pesos para la secundaria 2 en Huejutla</t>
+  </si>
+  <si>
+    <t>Infraestructura escolar</t>
+  </si>
+  <si>
+    <t>Afición vibra en Plaza 21 de Mayo con triunfo del Tri</t>
+  </si>
+  <si>
+    <t>Registro de líneas telefónicas se realizará de forma escalonada</t>
+  </si>
+  <si>
+    <t>Registro de celulares</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo refrenda coordinación con la Guardia Nacional</t>
+  </si>
+  <si>
+    <t>Conmemoración Aniversario</t>
+  </si>
+  <si>
+    <t>Hidalgo plantea plan prospectivo rumbo a 2040</t>
+  </si>
+  <si>
+    <t>Plan 2040</t>
+  </si>
+  <si>
+    <t>Gabinete de Seguridad localiza 18 túneless huachicoleros en Hidalgo</t>
+  </si>
+  <si>
+    <t>Roban 9 millones al balneario Dios Padre</t>
+  </si>
+  <si>
+    <t>iforma</t>
+  </si>
+  <si>
+    <t>Sin observaciones, revisión de la ASF a Hidalgo</t>
+  </si>
+  <si>
+    <t>Congreso entra a la polémica del relleno sanitario de Tula</t>
+  </si>
+  <si>
+    <t>Video de persecución en Tizayuca contradice versión oficial</t>
+  </si>
+  <si>
+    <t>México pasa a octavos, con goles de Quiñones Raúl JIménez</t>
+  </si>
+  <si>
+    <t>Hidalgo obtiene resultados sin observaciones en la primera entrega de la Cuenta Pública 2025 de la ASF</t>
+  </si>
+  <si>
+    <t>Van por destrucción de 18 huachitúneles detectados en Hidalgo</t>
+  </si>
+  <si>
+    <t>Se gradúa la 16a generación de la Casa de la Mujer Hidalguense</t>
+  </si>
+  <si>
+    <t>Graduación</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo refrenda coordinación con la Guardia Nacional para fortalecer la paz y la seguridad</t>
+  </si>
+  <si>
+    <t>Anuncian rehabilitación del Bulevar Refinería con una inversión de 13 mdp en Tula</t>
+  </si>
+  <si>
+    <t>Policías de Pachuca auxilian a mujer en labor de parto</t>
+  </si>
+  <si>
+    <t>Atención a la ciudadanía</t>
+  </si>
+  <si>
+    <t>Víctor Velázquez confirma partido del Cruz Azul en Ciudad Deportiva</t>
+  </si>
+  <si>
+    <t>Cruz Azul</t>
+  </si>
+  <si>
+    <t>Identidad segura</t>
+  </si>
+  <si>
+    <t>Robo de identidad</t>
+  </si>
+  <si>
+    <t>Enloquecen pachuqueños con el triunfo del Tri</t>
+  </si>
+  <si>
+    <t>SSPH captura a presunto generador de violencia vinculado a hechos de alto impacto</t>
+  </si>
+  <si>
+    <t>Hidalgo, sin observaciones en la primera entrega de la Cuenta Pública 2025 de la ASF</t>
+  </si>
+  <si>
+    <t>¡A octavos! México deja fuera a Ecuador y siguen soñando</t>
+  </si>
+  <si>
+    <t>Ellos importan</t>
+  </si>
+  <si>
+    <t>Maltrato animal</t>
+  </si>
+  <si>
+    <t>¡Sí se pudo!</t>
+  </si>
+  <si>
+    <t>La Auditoría superior de la Federación fiscalizó más de 6 mil 657</t>
   </si>
 </sst>
 </file>
@@ -934,8 +799,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J74" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J74" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J60" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J60" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1301,22 +1166,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J74"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J60"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="50.7265625" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1348,18 +1213,18 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B2" t="s">
         <v>68</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E2" t="s">
         <v>10</v>
@@ -1368,10 +1233,10 @@
         <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1382,265 +1247,265 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B3" t="s">
         <v>68</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="G3" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
       <c r="H3" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J3" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B4" t="s">
         <v>68</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D4" t="s">
         <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>102</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s">
-        <v>103</v>
+        <v>87</v>
       </c>
       <c r="H4" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B5" t="s">
         <v>68</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F5" t="s">
-        <v>10</v>
+        <v>91</v>
       </c>
       <c r="G5" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H5" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="G6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
       </c>
       <c r="I6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J6" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B7" t="s">
-        <v>68</v>
+        <v>78</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="H7" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
       <c r="I7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J7" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B8" t="s">
         <v>78</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D8" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="F8" t="s">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="G8" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="H8" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="I8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B9" t="s">
         <v>78</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>10</v>
+        <v>107</v>
       </c>
       <c r="F9" t="s">
-        <v>10</v>
+        <v>107</v>
       </c>
       <c r="G9" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B10" t="s">
         <v>78</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
       </c>
       <c r="E10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="F10" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="H10" t="s">
         <v>11</v>
@@ -1654,185 +1519,185 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B11" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
       </c>
       <c r="E11" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F11" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
       </c>
       <c r="I11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J11" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
       </c>
       <c r="E12" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="F12" t="s">
-        <v>118</v>
+        <v>2</v>
       </c>
       <c r="G12" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="H12" t="s">
         <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="D13" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F13" t="s">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="G13" t="s">
-        <v>90</v>
+        <v>115</v>
       </c>
       <c r="H13" t="s">
         <v>11</v>
       </c>
       <c r="I13" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J13" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" t="s">
+        <v>74</v>
+      </c>
+      <c r="H14" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J14" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F15" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" t="s">
+        <v>108</v>
+      </c>
+      <c r="H15" t="s">
+        <v>69</v>
+      </c>
+      <c r="I15" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J13" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A14" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B14" t="s">
-        <v>78</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="D14" t="s">
-        <v>12</v>
-      </c>
-      <c r="E14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G14" t="s">
-        <v>115</v>
-      </c>
-      <c r="H14" t="s">
-        <v>11</v>
-      </c>
-      <c r="I14" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J14" t="str">
+      <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B15" t="s">
-        <v>78</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="D15" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" t="s">
-        <v>10</v>
-      </c>
-      <c r="F15" t="s">
-        <v>10</v>
-      </c>
-      <c r="G15" t="s">
-        <v>74</v>
-      </c>
-      <c r="H15" t="s">
-        <v>11</v>
-      </c>
-      <c r="I15" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J15" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B16" t="s">
         <v>76</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D16" t="s">
         <v>12</v>
@@ -1847,7 +1712,7 @@
         <v>74</v>
       </c>
       <c r="H16" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -1858,129 +1723,129 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B17" t="s">
         <v>76</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>38</v>
+      </c>
+      <c r="F17" t="s">
+        <v>38</v>
+      </c>
+      <c r="G17" t="s">
+        <v>98</v>
+      </c>
+      <c r="H17" t="s">
+        <v>69</v>
+      </c>
+      <c r="I17" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J17" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B18" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="D18" t="s">
         <v>13</v>
       </c>
-      <c r="E17" t="s">
-        <v>14</v>
-      </c>
-      <c r="F17" t="s">
-        <v>125</v>
-      </c>
-      <c r="G17" t="s">
-        <v>88</v>
-      </c>
-      <c r="H17" t="s">
-        <v>87</v>
-      </c>
-      <c r="I17" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J17" t="str">
+      <c r="E18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" t="s">
+        <v>89</v>
+      </c>
+      <c r="G18" t="s">
+        <v>115</v>
+      </c>
+      <c r="H18" t="s">
+        <v>11</v>
+      </c>
+      <c r="I18" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J18" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A18" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B18" t="s">
-        <v>76</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="D18" t="s">
-        <v>12</v>
-      </c>
-      <c r="E18" t="s">
-        <v>14</v>
-      </c>
-      <c r="F18" t="s">
-        <v>14</v>
-      </c>
-      <c r="G18" t="s">
-        <v>127</v>
-      </c>
-      <c r="H18" t="s">
-        <v>87</v>
-      </c>
-      <c r="I18" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J18" t="str">
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A19" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" t="s">
+        <v>82</v>
+      </c>
+      <c r="H19" t="s">
+        <v>69</v>
+      </c>
+      <c r="I19" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A19" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B19" t="s">
-        <v>76</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D19" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19" t="s">
-        <v>129</v>
-      </c>
-      <c r="G19" t="s">
-        <v>93</v>
-      </c>
-      <c r="H19" t="s">
-        <v>11</v>
-      </c>
-      <c r="I19" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J19" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="D20" t="s">
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="F20" t="s">
-        <v>79</v>
+        <v>107</v>
       </c>
       <c r="G20" t="s">
-        <v>131</v>
+        <v>108</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
@@ -1994,95 +1859,95 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>67</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E21" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="G21" t="s">
-        <v>90</v>
+        <v>74</v>
       </c>
       <c r="H21" t="s">
         <v>69</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B22" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="D22" t="s">
         <v>13</v>
       </c>
       <c r="E22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F22" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G22" t="s">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="H22" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B23" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="D23" t="s">
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>17</v>
+        <v>107</v>
       </c>
       <c r="F23" t="s">
-        <v>17</v>
+        <v>107</v>
       </c>
       <c r="G23" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="H23" t="s">
         <v>11</v>
@@ -2096,234 +1961,234 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="D24" t="s">
         <v>12</v>
       </c>
       <c r="E24" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F24" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
       <c r="H24" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="I24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J24" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B25" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="D25" t="s">
         <v>9</v>
       </c>
       <c r="E25" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F25" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="G25" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="H25" t="s">
         <v>69</v>
       </c>
       <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="60" x14ac:dyDescent="0.25">
       <c r="A26" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F26" t="s">
-        <v>10</v>
+        <v>84</v>
       </c>
       <c r="G26" t="s">
-        <v>74</v>
+        <v>85</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
       </c>
       <c r="I26" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J26" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B27" t="s">
+        <v>71</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" t="s">
+        <v>10</v>
+      </c>
+      <c r="F27" t="s">
+        <v>10</v>
+      </c>
+      <c r="G27" t="s">
+        <v>74</v>
+      </c>
+      <c r="H27" t="s">
+        <v>69</v>
+      </c>
+      <c r="I27" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Otros</v>
       </c>
-      <c r="J26" t="str">
+      <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A27" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B27" t="s">
-        <v>67</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="D27" t="s">
-        <v>12</v>
-      </c>
-      <c r="E27" t="s">
-        <v>10</v>
-      </c>
-      <c r="F27" t="s">
-        <v>10</v>
-      </c>
-      <c r="G27" t="s">
-        <v>85</v>
-      </c>
-      <c r="H27" t="s">
-        <v>87</v>
-      </c>
-      <c r="I27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J27" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B28" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="D28" t="s">
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F28" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="G28" t="s">
-        <v>142</v>
+        <v>74</v>
       </c>
       <c r="H28" t="s">
         <v>69</v>
       </c>
       <c r="I28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J28" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>143</v>
+        <v>131</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F29" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="G29" t="s">
-        <v>134</v>
+        <v>108</v>
       </c>
       <c r="H29" t="s">
-        <v>87</v>
+        <v>11</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B30" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>23</v>
+        <v>38</v>
       </c>
       <c r="F30" t="s">
-        <v>89</v>
+        <v>38</v>
       </c>
       <c r="G30" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="H30" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2334,27 +2199,27 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B31" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="D31" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="F31" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="G31" t="s">
-        <v>90</v>
+        <v>110</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
@@ -2365,33 +2230,33 @@
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="F32" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="G32" t="s">
-        <v>115</v>
+        <v>135</v>
       </c>
       <c r="H32" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
@@ -2402,129 +2267,129 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>147</v>
+        <v>136</v>
       </c>
       <c r="D33" t="s">
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="F33" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="G33" t="s">
-        <v>148</v>
+        <v>137</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A34" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B34" t="s">
+        <v>70</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+      <c r="E34" t="s">
+        <v>10</v>
+      </c>
+      <c r="F34" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" t="s">
+        <v>74</v>
+      </c>
+      <c r="H34" t="s">
+        <v>69</v>
+      </c>
+      <c r="I34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J34" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A34" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B34" t="s">
-        <v>72</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D34" t="s">
-        <v>9</v>
-      </c>
-      <c r="E34" t="s">
-        <v>16</v>
-      </c>
-      <c r="F34" t="s">
-        <v>102</v>
-      </c>
-      <c r="G34" t="s">
-        <v>95</v>
-      </c>
-      <c r="H34" t="s">
-        <v>87</v>
-      </c>
-      <c r="I34" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J34" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" ht="58" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>150</v>
+        <v>139</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="F35" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="G35" t="s">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
       </c>
       <c r="I35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J35" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B36" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="D36" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F36" t="s">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="G36" t="s">
-        <v>90</v>
+        <v>142</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
@@ -2535,30 +2400,30 @@
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B37" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="D37" t="s">
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="F37" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="G37" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
@@ -2569,30 +2434,30 @@
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B38" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>154</v>
+        <v>145</v>
       </c>
       <c r="D38" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E38" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="F38" t="s">
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="G38" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="H38" t="s">
         <v>11</v>
@@ -2606,265 +2471,265 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B39" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>155</v>
+        <v>146</v>
       </c>
       <c r="D39" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E39" t="s">
+        <v>17</v>
+      </c>
+      <c r="F39" t="s">
+        <v>17</v>
+      </c>
+      <c r="G39" t="s">
+        <v>110</v>
+      </c>
+      <c r="H39" t="s">
+        <v>147</v>
+      </c>
+      <c r="I39" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J39" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A40" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B40" t="s">
+        <v>75</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="D40" t="s">
+        <v>12</v>
+      </c>
+      <c r="E40" t="s">
+        <v>38</v>
+      </c>
+      <c r="F40" t="s">
+        <v>38</v>
+      </c>
+      <c r="G40" t="s">
+        <v>98</v>
+      </c>
+      <c r="H40" t="s">
+        <v>69</v>
+      </c>
+      <c r="I40" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J40" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A41" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B41" t="s">
+        <v>75</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D41" t="s">
+        <v>12</v>
+      </c>
+      <c r="E41" t="s">
         <v>33</v>
       </c>
-      <c r="F39" t="s">
-        <v>156</v>
-      </c>
-      <c r="G39" t="s">
-        <v>157</v>
-      </c>
-      <c r="H39" t="s">
-        <v>11</v>
-      </c>
-      <c r="I39" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J39" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A40" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B40" t="s">
-        <v>71</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="D40" t="s">
-        <v>12</v>
-      </c>
-      <c r="E40" t="s">
-        <v>16</v>
-      </c>
-      <c r="F40" t="s">
-        <v>16</v>
-      </c>
-      <c r="G40" t="s">
-        <v>159</v>
-      </c>
-      <c r="H40" t="s">
-        <v>11</v>
-      </c>
-      <c r="I40" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J40" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A41" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B41" t="s">
-        <v>70</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="D41" t="s">
-        <v>12</v>
-      </c>
-      <c r="E41" t="s">
-        <v>20</v>
-      </c>
       <c r="F41" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G41" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="H41" t="s">
         <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J41" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A42" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B42" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="D42" t="s">
+        <v>12</v>
+      </c>
+      <c r="E42" t="s">
+        <v>16</v>
+      </c>
+      <c r="F42" t="s">
+        <v>92</v>
+      </c>
+      <c r="G42" t="s">
+        <v>90</v>
+      </c>
+      <c r="H42" t="s">
+        <v>83</v>
+      </c>
+      <c r="I42" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J42" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A43" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B43" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" t="s">
+        <v>10</v>
+      </c>
+      <c r="G43" t="s">
+        <v>74</v>
+      </c>
+      <c r="H43" t="s">
+        <v>69</v>
+      </c>
+      <c r="I43" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Otros</v>
+      </c>
+      <c r="J43" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A44" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B44" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="D44" t="s">
+        <v>13</v>
+      </c>
+      <c r="E44" t="s">
+        <v>38</v>
+      </c>
+      <c r="F44" t="s">
+        <v>38</v>
+      </c>
+      <c r="G44" t="s">
+        <v>135</v>
+      </c>
+      <c r="H44" t="s">
+        <v>69</v>
+      </c>
+      <c r="I44" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J41" t="str">
+      <c r="J44" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="42" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A42" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B42" t="s">
-        <v>70</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="D42" t="s">
-        <v>12</v>
-      </c>
-      <c r="E42" t="s">
-        <v>14</v>
-      </c>
-      <c r="F42" t="s">
-        <v>14</v>
-      </c>
-      <c r="G42" t="s">
-        <v>162</v>
-      </c>
-      <c r="H42" t="s">
-        <v>11</v>
-      </c>
-      <c r="I42" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J42" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A43" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B43" t="s">
-        <v>70</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="D43" t="s">
-        <v>13</v>
-      </c>
-      <c r="E43" t="s">
-        <v>58</v>
-      </c>
-      <c r="F43" t="s">
-        <v>58</v>
-      </c>
-      <c r="G43" t="s">
-        <v>164</v>
-      </c>
-      <c r="H43" t="s">
-        <v>11</v>
-      </c>
-      <c r="I43" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J43" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A44" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B44" t="s">
-        <v>70</v>
-      </c>
-      <c r="C44" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="D44" t="s">
-        <v>12</v>
-      </c>
-      <c r="E44" t="s">
-        <v>16</v>
-      </c>
-      <c r="F44" t="s">
-        <v>16</v>
-      </c>
-      <c r="G44" t="s">
-        <v>166</v>
-      </c>
-      <c r="H44" t="s">
-        <v>11</v>
-      </c>
-      <c r="I44" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J44" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B45" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>167</v>
+        <v>153</v>
       </c>
       <c r="D45" t="s">
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="F45" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="G45" t="s">
-        <v>168</v>
+        <v>108</v>
       </c>
       <c r="H45" t="s">
         <v>11</v>
       </c>
       <c r="I45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J45" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A46" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B46" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="D46" t="s">
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="F46" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="G46" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="H46" t="s">
         <v>11</v>
@@ -2875,166 +2740,166 @@
       </c>
       <c r="J46" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B47" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
       <c r="D47" t="s">
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="F47" t="s">
-        <v>156</v>
+        <v>24</v>
       </c>
       <c r="G47" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="H47" t="s">
         <v>11</v>
       </c>
       <c r="I47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J47" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A48" s="5">
+        <v>46204</v>
+      </c>
+      <c r="B48" t="s">
+        <v>79</v>
+      </c>
+      <c r="C48" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="D48" t="s">
+        <v>12</v>
+      </c>
+      <c r="E48" t="s">
+        <v>16</v>
+      </c>
+      <c r="F48" t="s">
+        <v>16</v>
+      </c>
+      <c r="G48" t="s">
+        <v>88</v>
+      </c>
+      <c r="H48" t="s">
+        <v>11</v>
+      </c>
+      <c r="I48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A48" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B48" t="s">
-        <v>75</v>
-      </c>
-      <c r="C48" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="D48" t="s">
-        <v>9</v>
-      </c>
-      <c r="E48" t="s">
-        <v>59</v>
-      </c>
-      <c r="F48" t="s">
-        <v>59</v>
-      </c>
-      <c r="G48" t="s">
-        <v>173</v>
-      </c>
-      <c r="H48" t="s">
-        <v>69</v>
-      </c>
-      <c r="I48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B49" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="D49" t="s">
         <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F49" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
       <c r="G49" t="s">
-        <v>115</v>
+        <v>159</v>
       </c>
       <c r="H49" t="s">
         <v>11</v>
       </c>
       <c r="I49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J49" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A50" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B50" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="D50" t="s">
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F50" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="G50" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="H50" t="s">
         <v>11</v>
       </c>
       <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B51" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="D51" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="E51" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F51" t="s">
-        <v>89</v>
+        <v>22</v>
       </c>
       <c r="G51" t="s">
-        <v>90</v>
+        <v>163</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
@@ -3048,151 +2913,151 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B52" t="s">
-        <v>75</v>
+        <v>86</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>178</v>
+        <v>164</v>
       </c>
       <c r="D52" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E52" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>115</v>
+        <v>74</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A53" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B53" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="D53" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F53" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="G53" t="s">
-        <v>180</v>
+        <v>95</v>
       </c>
       <c r="H53" t="s">
         <v>11</v>
       </c>
       <c r="I53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B54" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="D54" t="s">
         <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="F54" t="s">
-        <v>182</v>
+        <v>38</v>
       </c>
       <c r="G54" t="s">
-        <v>183</v>
+        <v>135</v>
       </c>
       <c r="H54" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B55" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>184</v>
+        <v>167</v>
       </c>
       <c r="D55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="F55" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="G55" t="s">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="H55" t="s">
         <v>69</v>
       </c>
       <c r="I55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>otros</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B56" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>185</v>
+        <v>141</v>
       </c>
       <c r="D56" t="s">
         <v>12</v>
@@ -3204,7 +3069,7 @@
         <v>24</v>
       </c>
       <c r="G56" t="s">
-        <v>170</v>
+        <v>142</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
@@ -3218,61 +3083,61 @@
         <v>Gobernador</v>
       </c>
     </row>
-    <row r="57" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B57" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>186</v>
+        <v>93</v>
       </c>
       <c r="D57" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="E57" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F57" t="s">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="G57" t="s">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="H57" t="s">
         <v>11</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B58" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="D58" t="s">
-        <v>12</v>
+        <v>77</v>
       </c>
       <c r="E58" t="s">
         <v>16</v>
       </c>
       <c r="F58" t="s">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="G58" t="s">
-        <v>188</v>
+        <v>169</v>
       </c>
       <c r="H58" t="s">
         <v>11</v>
@@ -3286,546 +3151,70 @@
         <v>otros</v>
       </c>
     </row>
-    <row r="59" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B59" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>189</v>
+        <v>170</v>
       </c>
       <c r="D59" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E59" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F59" t="s">
-        <v>82</v>
+        <v>10</v>
       </c>
       <c r="G59" t="s">
-        <v>190</v>
+        <v>74</v>
       </c>
       <c r="H59" t="s">
-        <v>11</v>
+        <v>69</v>
       </c>
       <c r="I59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J59" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>otros</v>
       </c>
     </row>
-    <row r="60" spans="1:10" ht="29" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A60" s="5">
-        <v>46203</v>
+        <v>46204</v>
       </c>
       <c r="B60" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="D60" t="s">
         <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="F60" t="s">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="G60" t="s">
-        <v>192</v>
+        <v>135</v>
       </c>
       <c r="H60" t="s">
         <v>11</v>
       </c>
       <c r="I60" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J60" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A61" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B61" t="s">
-        <v>80</v>
-      </c>
-      <c r="C61" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="D61" t="s">
-        <v>12</v>
-      </c>
-      <c r="E61" t="s">
-        <v>16</v>
-      </c>
-      <c r="F61" t="s">
-        <v>16</v>
-      </c>
-      <c r="G61" t="s">
-        <v>194</v>
-      </c>
-      <c r="H61" t="s">
-        <v>11</v>
-      </c>
-      <c r="I61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J61" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A62" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B62" t="s">
-        <v>80</v>
-      </c>
-      <c r="C62" s="6" t="s">
-        <v>195</v>
-      </c>
-      <c r="D62" t="s">
-        <v>12</v>
-      </c>
-      <c r="E62" t="s">
-        <v>16</v>
-      </c>
-      <c r="F62" t="s">
-        <v>196</v>
-      </c>
-      <c r="G62" t="s">
-        <v>197</v>
-      </c>
-      <c r="H62" t="s">
-        <v>11</v>
-      </c>
-      <c r="I62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J62" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="29" x14ac:dyDescent="0.35">
-      <c r="A63" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B63" t="s">
-        <v>80</v>
-      </c>
-      <c r="C63" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="D63" t="s">
-        <v>12</v>
-      </c>
-      <c r="E63" t="s">
-        <v>10</v>
-      </c>
-      <c r="F63" t="s">
-        <v>10</v>
-      </c>
-      <c r="G63" t="s">
-        <v>86</v>
-      </c>
-      <c r="H63" t="s">
-        <v>11</v>
-      </c>
-      <c r="I63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J63" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A64" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B64" t="s">
-        <v>80</v>
-      </c>
-      <c r="C64" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="D64" t="s">
-        <v>77</v>
-      </c>
-      <c r="E64" t="s">
-        <v>16</v>
-      </c>
-      <c r="F64" t="s">
-        <v>16</v>
-      </c>
-      <c r="G64" t="s">
-        <v>200</v>
-      </c>
-      <c r="H64" t="s">
-        <v>11</v>
-      </c>
-      <c r="I64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J64" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A65" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B65" t="s">
-        <v>94</v>
-      </c>
-      <c r="C65" s="6" t="s">
-        <v>201</v>
-      </c>
-      <c r="D65" t="s">
-        <v>13</v>
-      </c>
-      <c r="E65" t="s">
-        <v>24</v>
-      </c>
-      <c r="F65" t="s">
-        <v>24</v>
-      </c>
-      <c r="G65" t="s">
-        <v>92</v>
-      </c>
-      <c r="H65" t="s">
-        <v>11</v>
-      </c>
-      <c r="I65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J65" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gobernador</v>
-      </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A66" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B66" t="s">
-        <v>94</v>
-      </c>
-      <c r="C66" s="6" t="s">
-        <v>202</v>
-      </c>
-      <c r="D66" t="s">
-        <v>12</v>
-      </c>
-      <c r="E66" t="s">
-        <v>20</v>
-      </c>
-      <c r="F66" t="s">
-        <v>20</v>
-      </c>
-      <c r="G66" t="s">
-        <v>203</v>
-      </c>
-      <c r="H66" t="s">
-        <v>11</v>
-      </c>
-      <c r="I66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J66" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A67" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B67" t="s">
-        <v>94</v>
-      </c>
-      <c r="C67" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="D67" t="s">
-        <v>12</v>
-      </c>
-      <c r="E67" t="s">
-        <v>10</v>
-      </c>
-      <c r="F67" t="s">
-        <v>10</v>
-      </c>
-      <c r="G67" t="s">
-        <v>74</v>
-      </c>
-      <c r="H67" t="s">
-        <v>11</v>
-      </c>
-      <c r="I67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J67" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A68" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B68" t="s">
-        <v>94</v>
-      </c>
-      <c r="C68" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="D68" t="s">
-        <v>12</v>
-      </c>
-      <c r="E68" t="s">
-        <v>29</v>
-      </c>
-      <c r="F68" t="s">
-        <v>96</v>
-      </c>
-      <c r="G68" t="s">
-        <v>97</v>
-      </c>
-      <c r="H68" t="s">
-        <v>11</v>
-      </c>
-      <c r="I68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J68" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A69" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B69" t="s">
-        <v>94</v>
-      </c>
-      <c r="C69" s="6" t="s">
-        <v>206</v>
-      </c>
-      <c r="D69" t="s">
-        <v>12</v>
-      </c>
-      <c r="E69" t="s">
-        <v>26</v>
-      </c>
-      <c r="F69" t="s">
-        <v>207</v>
-      </c>
-      <c r="G69" t="s">
-        <v>208</v>
-      </c>
-      <c r="H69" t="s">
-        <v>11</v>
-      </c>
-      <c r="I69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J69" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A70" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B70" t="s">
-        <v>94</v>
-      </c>
-      <c r="C70" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="D70" t="s">
-        <v>77</v>
-      </c>
-      <c r="E70" t="s">
-        <v>15</v>
-      </c>
-      <c r="F70" t="s">
-        <v>15</v>
-      </c>
-      <c r="G70" t="s">
-        <v>210</v>
-      </c>
-      <c r="H70" t="s">
-        <v>11</v>
-      </c>
-      <c r="I70" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J70" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A71" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B71" t="s">
-        <v>84</v>
-      </c>
-      <c r="C71" s="6" t="s">
-        <v>211</v>
-      </c>
-      <c r="D71" t="s">
-        <v>13</v>
-      </c>
-      <c r="E71" t="s">
-        <v>16</v>
-      </c>
-      <c r="F71" t="s">
-        <v>102</v>
-      </c>
-      <c r="G71" t="s">
-        <v>103</v>
-      </c>
-      <c r="H71" t="s">
-        <v>87</v>
-      </c>
-      <c r="I71" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J71" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A72" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B72" t="s">
-        <v>84</v>
-      </c>
-      <c r="C72" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="D72" t="s">
-        <v>12</v>
-      </c>
-      <c r="E72" t="s">
-        <v>22</v>
-      </c>
-      <c r="F72" t="s">
-        <v>22</v>
-      </c>
-      <c r="G72" t="s">
-        <v>213</v>
-      </c>
-      <c r="H72" t="s">
-        <v>11</v>
-      </c>
-      <c r="I72" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J72" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A73" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B73" t="s">
-        <v>84</v>
-      </c>
-      <c r="C73" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="D73" t="s">
-        <v>12</v>
-      </c>
-      <c r="E73" t="s">
-        <v>58</v>
-      </c>
-      <c r="F73" t="s">
-        <v>58</v>
-      </c>
-      <c r="G73" t="s">
-        <v>215</v>
-      </c>
-      <c r="H73" t="s">
-        <v>87</v>
-      </c>
-      <c r="I73" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Otros</v>
-      </c>
-      <c r="J73" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
-        <v>otros</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A74" s="5">
-        <v>46203</v>
-      </c>
-      <c r="B74" t="s">
-        <v>84</v>
-      </c>
-      <c r="C74" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="D74" t="s">
-        <v>12</v>
-      </c>
-      <c r="E74" t="s">
-        <v>23</v>
-      </c>
-      <c r="F74" t="s">
-        <v>89</v>
-      </c>
-      <c r="G74" t="s">
-        <v>90</v>
-      </c>
-      <c r="H74" t="s">
-        <v>11</v>
-      </c>
-      <c r="I74" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"No indexado")</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J74" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"otros",0)</f>
         <v>Gabinete</v>
       </c>
@@ -3842,14 +3231,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8151DEFD-FF29-4969-B1FC-DF47C7CD743C}">
   <dimension ref="A1:E48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -3863,7 +3252,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>61</v>
       </c>
@@ -3877,7 +3266,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -3891,7 +3280,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>19</v>
       </c>
@@ -3905,7 +3294,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>60</v>
       </c>
@@ -3919,7 +3308,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>73</v>
       </c>
@@ -3933,7 +3322,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -3947,7 +3336,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>34</v>
       </c>
@@ -3961,7 +3350,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -3975,7 +3364,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -3989,7 +3378,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>35</v>
       </c>
@@ -4003,7 +3392,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>36</v>
       </c>
@@ -4017,7 +3406,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>36</v>
       </c>
@@ -4031,7 +3420,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>63</v>
       </c>
@@ -4045,7 +3434,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -4059,7 +3448,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -4073,7 +3462,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>38</v>
       </c>
@@ -4087,7 +3476,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -4101,7 +3490,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -4115,7 +3504,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>41</v>
       </c>
@@ -4129,7 +3518,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>43</v>
       </c>
@@ -4143,7 +3532,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -4157,7 +3546,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -4171,7 +3560,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>10</v>
       </c>
@@ -4185,7 +3574,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>45</v>
       </c>
@@ -4199,7 +3588,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>46</v>
       </c>
@@ -4213,7 +3602,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>64</v>
       </c>
@@ -4227,7 +3616,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>17</v>
       </c>
@@ -4235,7 +3624,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -4243,7 +3632,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>48</v>
       </c>
@@ -4251,7 +3640,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
@@ -4259,7 +3648,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>50</v>
       </c>
@@ -4267,7 +3656,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>51</v>
       </c>
@@ -4275,7 +3664,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>52</v>
       </c>
@@ -4283,7 +3672,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>53</v>
       </c>
@@ -4291,7 +3680,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>54</v>
       </c>
@@ -4299,7 +3688,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>23</v>
       </c>
@@ -4307,7 +3696,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>20</v>
       </c>
@@ -4315,7 +3704,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>27</v>
       </c>
@@ -4323,7 +3712,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>26</v>
       </c>
@@ -4331,7 +3720,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>55</v>
       </c>
@@ -4339,7 +3728,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>15</v>
       </c>
@@ -4347,7 +3736,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>22</v>
       </c>
@@ -4355,7 +3744,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>56</v>
       </c>
@@ -4363,7 +3752,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>57</v>
       </c>
@@ -4371,7 +3760,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>58</v>
       </c>
@@ -4379,7 +3768,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>29</v>
       </c>
@@ -4387,7 +3776,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>59</v>
       </c>

</xml_diff>

<commit_message>
Reporte portadas en pptx
</commit_message>
<xml_diff>
--- a/MuestraPortadas.xlsx
+++ b/MuestraPortadas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vivie\Reporteportadas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B382CF9C-9D55-4673-A8D5-E7DB77C40C7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8868BC89-6E1E-4C1D-8F46-76226CAD4692}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56C16FF2-DC5E-4EA2-A3CB-6D506676B8B8}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="191">
   <si>
     <t>Fecha</t>
   </si>
@@ -285,9 +285,6 @@
     <t>Cintillo</t>
   </si>
   <si>
-    <t>Editorial</t>
-  </si>
-  <si>
     <t>Zunoticia</t>
   </si>
   <si>
@@ -300,30 +297,9 @@
     <t>Combate a trata de personas</t>
   </si>
   <si>
-    <t>Publicidad comercial</t>
-  </si>
-  <si>
-    <t>Radio Plaza Juárez</t>
-  </si>
-  <si>
-    <t>Homicidio de Policía</t>
-  </si>
-  <si>
-    <t>Combate a la corrupción</t>
-  </si>
-  <si>
     <t>Temas internacionales</t>
   </si>
   <si>
-    <t>Búsqueda de personas</t>
-  </si>
-  <si>
-    <t>Mega sorteo San Judas</t>
-  </si>
-  <si>
-    <t>Anuncian corte en red de agua</t>
-  </si>
-  <si>
     <t>Sipdus</t>
   </si>
   <si>
@@ -333,310 +309,307 @@
     <t>Abasto De Agua</t>
   </si>
   <si>
-    <t>Obra de tren afecta suministro hídrico</t>
-  </si>
-  <si>
-    <t>SICT</t>
-  </si>
-  <si>
-    <t>Tren México Querétaro</t>
-  </si>
-  <si>
-    <t>Pobladores de Tula, preocupados por lluvias</t>
-  </si>
-  <si>
-    <t>Monitoreo De Ríos</t>
-  </si>
-  <si>
-    <t>Lecheros piden frenar el producto externo</t>
-  </si>
-  <si>
-    <t>Producción lechera</t>
-  </si>
-  <si>
-    <t>Listos los cuartos de final</t>
-  </si>
-  <si>
-    <t>Asesinan, roban una camioneta y desatan persecución</t>
-  </si>
-  <si>
-    <t>C5i</t>
-  </si>
-  <si>
     <t>Combate a la delincuencia</t>
   </si>
   <si>
-    <t>Convierten una cárcel de Tizayuc en galería de arte</t>
-  </si>
-  <si>
-    <t>Cecultah</t>
-  </si>
-  <si>
-    <t>Exposición Artística</t>
-  </si>
-  <si>
-    <t>Absuelve INE al gobernador Julio Menchaca</t>
-  </si>
-  <si>
-    <t>Fiscalización INE</t>
-  </si>
-  <si>
-    <t>Messi manda a volar a los Faraones</t>
-  </si>
-  <si>
-    <t>Respaldan aplazar comicios judiciales a 2028</t>
-  </si>
-  <si>
-    <t>Elección Judicial</t>
-  </si>
-  <si>
-    <t>Remontada de campeón</t>
-  </si>
-  <si>
-    <t>Suiza elimina a Colombia</t>
-  </si>
-  <si>
-    <t>Hallaron culpable a un expolicía por asesinar a Rosaura</t>
-  </si>
-  <si>
-    <t>Sentencia Feminicida</t>
-  </si>
-  <si>
-    <t>Estudiantes de Cenhies crean app contra las desapariciones</t>
-  </si>
-  <si>
     <t>Personas desaparecidas</t>
   </si>
   <si>
-    <t>Acuan anomalías los alumnos de Intermédica en Pachuca de Soto</t>
-  </si>
-  <si>
-    <t>Anomalías</t>
-  </si>
-  <si>
-    <t>Suman diez quejas en la CDHEH por daños ecológicos en actual gestión</t>
-  </si>
-  <si>
-    <t>Queja CDHEH</t>
-  </si>
-  <si>
-    <t>Reitera la SEPH clases virtuales por Bullying</t>
-  </si>
-  <si>
-    <t>Bullying</t>
-  </si>
-  <si>
-    <t>Obesidad rebasa en seis meses las cifras de todo 2025</t>
-  </si>
-  <si>
-    <t>Salud</t>
-  </si>
-  <si>
-    <t>Obesidad</t>
-  </si>
-  <si>
-    <t>Endurecen medidas para frenar deterioro del Parque El Chico</t>
-  </si>
-  <si>
     <t>Área Natural Protegida</t>
   </si>
   <si>
-    <t>Información   sobre tema  de El Mayo, en   manos de FGR</t>
-  </si>
-  <si>
-    <t>FGR</t>
-  </si>
-  <si>
-    <t>Robo de patrulla genera intensa movilización policiaca</t>
-  </si>
-  <si>
-    <t>Robo de patrulla</t>
-  </si>
-  <si>
-    <t>Necesitamos urgentemente una reforma fiscal para que  las personas más ricas de este país paguen impuestos;  que, por cierto, no son las personas trabajadoras”.</t>
-  </si>
-  <si>
-    <t>Reforma fiscal</t>
-  </si>
-  <si>
-    <t>Declaran culpable a expolicía por feminicidio de Rosaura</t>
-  </si>
-  <si>
-    <t>Detectan 43 invasiones irregulares en el Parque Nacional</t>
-  </si>
-  <si>
-    <t>Prevén mantener en 100 mdp costo del nuevo Salón de Plenos</t>
-  </si>
-  <si>
-    <t>Junta de Gobierno</t>
-  </si>
-  <si>
-    <t>Salón De Plenos</t>
-  </si>
-  <si>
-    <t>SEPH entrega certificados de inglés a más de 22 m il estudiantes de bachillerato</t>
-  </si>
-  <si>
-    <t>Entrega De Certificados</t>
-  </si>
-  <si>
-    <t>Prevalecen enfrentamientos entre comuneros</t>
-  </si>
-  <si>
     <t>Enfrentamiento</t>
   </si>
   <si>
-    <t>Sebiso inicia operativos de entrega de tarjetas de los Programas del Pueblo</t>
-  </si>
-  <si>
-    <t>Programas Del Pueblo</t>
-  </si>
-  <si>
-    <t>Exdelegado pide regular topes en la carretera México-Tampico</t>
-  </si>
-  <si>
-    <t>Cuadrillas de CFE intensifican mantenimiento en infraestructura</t>
-  </si>
-  <si>
-    <t>CFE</t>
-  </si>
-  <si>
-    <t>Infraestructura en mal estado</t>
-  </si>
-  <si>
-    <t>Fortalecen acciones para proteger el Parque Nacional ""El Chico""</t>
-  </si>
-  <si>
-    <t>Detectan 43 construcciones irregulares en el Parque Nacional El Chico</t>
-  </si>
-  <si>
-    <t>¡Mega operativo por asesinato!</t>
-  </si>
-  <si>
-    <t>Descartan que cadáveres de Tlaxcala sean de CFE</t>
-  </si>
-  <si>
-    <t>Sancionan a dos policías por uso excesivo de la fuerza en protesta del ISSSTE</t>
-  </si>
-  <si>
-    <t>Abuso Policiaco</t>
-  </si>
-  <si>
-    <t>Asesinato de ministeriales: proceso entra a etapa decisiva</t>
-  </si>
-  <si>
-    <t>Declaran culpable a expolicía por el feminicidio de Rosaura</t>
-  </si>
-  <si>
-    <t>Contraloría acumula 95 denuncias por presuntos actos de corrupción en Hidalgo</t>
-  </si>
-  <si>
-    <t>Suman 76 animales devuertos a su hábitat en 2026 gracias a la Unidad de Rehabilitación de Fauna Silvestre</t>
-  </si>
-  <si>
-    <t>Liberación Fauna Silvestre</t>
-  </si>
-  <si>
-    <t>Entrega DIF Hidalgo 28 proyectos productivos y audas técnicas para familias del Valle de Tulancingo</t>
-  </si>
-  <si>
-    <t>Entrega de proyectos productivos</t>
-  </si>
-  <si>
-    <t>Despacho del Gobernador abre convocatoria para la sexta edición de Intervención Gráfica</t>
-  </si>
-  <si>
-    <t>Intervención Gráfica</t>
-  </si>
-  <si>
-    <t>Participación ciudadana fortalece la actualización del Plan Municipal de Desarrollo de Tula de Allende</t>
-  </si>
-  <si>
-    <t>Plan Municipal de Desarrollo</t>
-  </si>
-  <si>
-    <t>Ajacuba se suma a estrategia estatal para mejorar el aprovechamiento del agua en el sector agrícola</t>
-  </si>
-  <si>
-    <t>Captación De Agua</t>
-  </si>
-  <si>
-    <t>La jornada de bacheo sigue avanzando</t>
-  </si>
-  <si>
-    <t>Bacheo</t>
-  </si>
-  <si>
-    <t>Brigadas  de la salud acercarán atención médica gratuita</t>
-  </si>
-  <si>
-    <t>Brigadas De Salud</t>
-  </si>
-  <si>
-    <t>Carlos Montoya Romero: una vida marcada por la pasión y la tradición</t>
-  </si>
-  <si>
-    <t>Infonavit atenderá este domingo 12 de julio a las y los trabajadores en el Tec de Pachuca</t>
-  </si>
-  <si>
-    <t>Infonavit</t>
-  </si>
-  <si>
-    <t>Atención a la ciudadanía</t>
-  </si>
-  <si>
-    <t>Abre DIF Pachuca inscripciones para el Curso de Verano</t>
-  </si>
-  <si>
-    <t>Curso de verano</t>
-  </si>
-  <si>
-    <t>Publicidad gubernamental</t>
-  </si>
-  <si>
-    <t>Detienen a menor que asesinó a persona a la que compraría auto, en La Reforma</t>
-  </si>
-  <si>
-    <t>Unidad de Rehabilitación de Pachuca libera a 32 animales</t>
-  </si>
-  <si>
-    <t>Condenan a responsable de tres homicidios en Azoyatla</t>
-  </si>
-  <si>
-    <t>Despacho del Gobernador abre convocatoria para la Sexta Edición de Intervención Gráfica</t>
-  </si>
-  <si>
-    <t>SEPH entrega certificados de inglés a más de 22 mil estudiantes de bachillerato</t>
-  </si>
-  <si>
-    <t>Hióki</t>
-  </si>
-  <si>
-    <t>Una sola voz contra la trata de mujeres, niñas y niños</t>
-  </si>
-  <si>
-    <t>Condenan a expolicía por el asesinato de tres personas</t>
-  </si>
-  <si>
-    <t>Definidos los cuartos de final del Mundial</t>
-  </si>
-  <si>
-    <t>Se necesita hacer algo con urgencia para mejorar la movilidad en la Felipe Ángeles, en ambos sentidos, donde se registran "embotellamientos" permanentes</t>
-  </si>
-  <si>
-    <t>Infraestructura vial</t>
-  </si>
-  <si>
-    <t>Nunca vamos a hacer acuerdos con  la delincuencia organizada""</t>
-  </si>
-  <si>
-    <t>Crimen Organizado</t>
-  </si>
-  <si>
-    <t>Atenderán registro de Programa Vivienda para el Bienestar</t>
-  </si>
-  <si>
-    <t>Plan Nacional De Vivienda</t>
+    <t>Adiós casa de gobierno, ahora son oficinas</t>
+  </si>
+  <si>
+    <t>Casa De Gobierno</t>
+  </si>
+  <si>
+    <t>No investigarán la muerte del mexicano en EU</t>
+  </si>
+  <si>
+    <t>Muerte de migrante</t>
+  </si>
+  <si>
+    <t>Francia lista para ir por Marruecos</t>
+  </si>
+  <si>
+    <t>Solo reciben suministro de agua un par de días</t>
+  </si>
+  <si>
+    <t>Reforma de austeridad elimina 40 lugares de síndicos y regidores</t>
+  </si>
+  <si>
+    <t>Reforma De Ley</t>
+  </si>
+  <si>
+    <t>Homicida del Saucillo fingió ser un menor</t>
+  </si>
+  <si>
+    <t>De Casa de Gobernadores a oficinas de atención</t>
+  </si>
+  <si>
+    <t>Desarticulan banda de defraudadores</t>
+  </si>
+  <si>
+    <t>Policía municipal</t>
+  </si>
+  <si>
+    <t>Fraude</t>
+  </si>
+  <si>
+    <t>Rafael Márquez es el nuevo entrenador</t>
+  </si>
+  <si>
+    <t>Deportes</t>
+  </si>
+  <si>
+    <t>Visitan 35 mil Fan Fest Pachuca</t>
+  </si>
+  <si>
+    <t>El Káiser recibe las llaves del Tri</t>
+  </si>
+  <si>
+    <t>Por un boleto a semifinales</t>
+  </si>
+  <si>
+    <t>Destinan 45 mdp a 4 partidos con registro estatal</t>
+  </si>
+  <si>
+    <t>Financiamiento a Partidos</t>
+  </si>
+  <si>
+    <t>Planean hacer un bloqueo ante la falta de agua en Muixmí-Pitayas</t>
+  </si>
+  <si>
+    <t>Inauguran el centro administrativo, en la excasa del gobernador</t>
+  </si>
+  <si>
+    <t>Sin definir, ubicación del nuevo penal: JMS</t>
+  </si>
+  <si>
+    <t>Construcción de Cereso</t>
+  </si>
+  <si>
+    <t>Pone ASEH ojo al equipo que falta en RTH: auditor</t>
+  </si>
+  <si>
+    <t>RTVH</t>
+  </si>
+  <si>
+    <t>Observaciones ASEH</t>
+  </si>
+  <si>
+    <t>Milenio Hidalgo</t>
+  </si>
+  <si>
+    <t>Aseguran 1-3 millones de dosis; caen homicidios y extorsiones</t>
+  </si>
+  <si>
+    <t>"No era nuestro avión ni nuestra operación", dice Ken Salazar</t>
+  </si>
+  <si>
+    <t>Ya no es momento de frenarse""</t>
+  </si>
+  <si>
+    <t>Recuperan casa de exgobernadores</t>
+  </si>
+  <si>
+    <t>En la antigua Casa de Gobierno inauguran oficinas</t>
+  </si>
+  <si>
+    <t>inorma</t>
+  </si>
+  <si>
+    <t>Pachuca sumará 50 nuevos policías</t>
+  </si>
+  <si>
+    <t>Déficit policial</t>
+  </si>
+  <si>
+    <t>EU rechaza requerimientos de extradición de El Mayo</t>
+  </si>
+  <si>
+    <t>A once meses de la renovación de los 30 diputados locales y los 84 ayuntamientos, la efervescencia  política crece porque los resultados serán definitorios para las decisiones que habrán de tomar los doce  partidos políticos al año siguiente”.</t>
+  </si>
+  <si>
+    <t>Elecciones</t>
+  </si>
+  <si>
+    <t>Excasa de Gobierno pasa a la historia</t>
+  </si>
+  <si>
+    <t>Repatrian a 28 hidalguenses fallecidos en Estados Unidos este año</t>
+  </si>
+  <si>
+    <t>Repatriación</t>
+  </si>
+  <si>
+    <t>Salud estatal rebasa el 100% de cobertura en vacunas contra influenza y covid-19</t>
+  </si>
+  <si>
+    <t>Vacunación</t>
+  </si>
+  <si>
+    <t>Imputan por homicidio doloso y robo a detenido por caso Saucillo</t>
+  </si>
+  <si>
+    <t>Homicidios</t>
+  </si>
+  <si>
+    <t>Liberaron a retenidos en  Zocuitzintla al presentar problemas de salud</t>
+  </si>
+  <si>
+    <t>Julio Menchaca pide a municipios colaboración permanente en seguridad</t>
+  </si>
+  <si>
+    <t>Coordinación Interinstitucional</t>
+  </si>
+  <si>
+    <t>Por fuertes lluvias llaman a mantenerse informado y tomar precauciones</t>
+  </si>
+  <si>
+    <t>Alerta Meteorológica</t>
+  </si>
+  <si>
+    <t>Salud Pública exhorta a reforzar medidas contra la varicela</t>
+  </si>
+  <si>
+    <t>Vigilancia Epidemiológica</t>
+  </si>
+  <si>
+    <t>Natividad Castrejón encabeza recital poético Vida y Obra</t>
+  </si>
+  <si>
+    <t>Festival Cultural</t>
+  </si>
+  <si>
+    <t>De mansión de gobernadores a oficinas públicas; Menchaca inaugura complejo de 377 millones</t>
+  </si>
+  <si>
+    <t>Una encuesta en redes... no sirve de nada</t>
+  </si>
+  <si>
+    <t>Pachuca iluminará principales bulevares</t>
+  </si>
+  <si>
+    <t>alcald</t>
+  </si>
+  <si>
+    <t>Luminarias</t>
+  </si>
+  <si>
+    <t>Hallan hombre ejecutado y maniatado en la México-Tuxpan</t>
+  </si>
+  <si>
+    <t>Ejecuciones</t>
+  </si>
+  <si>
+    <t>Hidalgo, lugar 26 en empleo para mujeres: IMCO</t>
+  </si>
+  <si>
+    <t>Brecha de género</t>
+  </si>
+  <si>
+    <t>Hidalgo reporta 25 mil detenidos en casi cuatro años</t>
+  </si>
+  <si>
+    <t>Estrategia de seguridad</t>
+  </si>
+  <si>
+    <t>De mansión oficial a espacio de atención ciudadana: inauguran centro administrativo</t>
+  </si>
+  <si>
+    <t>Analizan hacer más estrictos exámenes para licencias de conducir</t>
+  </si>
+  <si>
+    <t>Licencia de conducir</t>
+  </si>
+  <si>
+    <t>Enner Valencia le dice adiós a los Tuzos</t>
+  </si>
+  <si>
+    <t>Natividad Castrejón encabeza recital poético en honor a Efrén Rebolledo</t>
+  </si>
+  <si>
+    <t>Juntos, terceros confirmados para el palenque 2026</t>
+  </si>
+  <si>
+    <t>OEEH</t>
+  </si>
+  <si>
+    <t>Feria Pachuca</t>
+  </si>
+  <si>
+    <t>Tu seguridad no es un juego</t>
+  </si>
+  <si>
+    <t>CBPEH</t>
+  </si>
+  <si>
+    <t>Una sola voz contra la trata</t>
+  </si>
+  <si>
+    <t>Avalan reformas para regular cobro de agua</t>
+  </si>
+  <si>
+    <t>Termina un lugar de privilegios; se abre un lugar para la ciudadanía</t>
+  </si>
+  <si>
+    <t>EE.UU. sigue sin enviar ""pruebas"" para detener a Rocha Moya</t>
+  </si>
+  <si>
+    <t>Trump da por acabado el alto al fuego tras ataques iraníes en Ormuz</t>
+  </si>
+  <si>
+    <t>De casa del gobernador a Casa del Pueblo</t>
+  </si>
+  <si>
+    <t>Detectan 43 construcciones irregulares dentro del Parque Nacional El Chico</t>
+  </si>
+  <si>
+    <t>Menchaca pide extremar precauciones en compra-venta de autos tras homicidio y persecución</t>
+  </si>
+  <si>
+    <t>Alerta De Fraude</t>
+  </si>
+  <si>
+    <t>Claudia Sandoval presenta a nuevo director de Seguridad</t>
+  </si>
+  <si>
+    <t>Nombramientos</t>
+  </si>
+  <si>
+    <t>Tezontepec de Aldama fortalece su estrategia de seguridad con convenio de videovigilancia</t>
+  </si>
+  <si>
+    <t>Videovigilancia</t>
+  </si>
+  <si>
+    <t>iforma</t>
+  </si>
+  <si>
+    <t>Julio Menchaca pide a municipios colaboración permanente para fortalecer acciones en materia de seguridad</t>
+  </si>
+  <si>
+    <t>Bienestar animal impulsa la producción pecuaria rentable y sostenible</t>
+  </si>
+  <si>
+    <t>Bienestar Animal</t>
+  </si>
+  <si>
+    <t>Contraloría de Hidalgo lleva el padrón de proveedores y contratistas al mundo digital</t>
+  </si>
+  <si>
+    <t>Padrón de proveedores</t>
+  </si>
+  <si>
+    <t>Gobierno de Hidalgo, federación y municipios fortalecen acciones para proteger el Parque Nacional El Chico</t>
+  </si>
+  <si>
+    <t>Supera Hidalgo metas de vacunación y fortalece la prevención de enfermedades</t>
   </si>
 </sst>
 </file>
@@ -883,8 +856,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J63" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
-  <autoFilter ref="A1:J63" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}" name="Tabla1" displayName="Tabla1" ref="A1:J62" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+  <autoFilter ref="A1:J62" xr:uid="{5593606E-308D-4113-AE3C-6E714B763B6E}"/>
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{9D9ACAF2-1710-400E-A0E5-0A5BB378D4A0}" name="Fecha" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{03A139BE-A997-45E6-81E6-5F7467162FC5}" name="Medio"/>
@@ -1250,7 +1223,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F590D41B-EE15-4091-8762-C3A670C9D896}">
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:J62"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -1299,7 +1272,7 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B2" t="s">
         <v>67</v>
@@ -1308,17 +1281,17 @@
         <v>94</v>
       </c>
       <c r="D2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
         <v>95</v>
       </c>
-      <c r="F2" t="s">
-        <v>96</v>
-      </c>
-      <c r="G2" t="s">
-        <v>97</v>
-      </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
@@ -1328,18 +1301,18 @@
       </c>
       <c r="J2" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B3" t="s">
         <v>67</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
@@ -1348,10 +1321,10 @@
         <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>99</v>
+        <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="H3" t="s">
         <v>78</v>
@@ -1367,93 +1340,93 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B4" t="s">
         <v>67</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="F4" t="s">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="G4" t="s">
-        <v>102</v>
+        <v>72</v>
       </c>
       <c r="H4" t="s">
         <v>11</v>
       </c>
       <c r="I4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J4" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B5" t="s">
         <v>67</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="F5" t="s">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="G5" t="s">
-        <v>104</v>
+        <v>89</v>
       </c>
       <c r="H5" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="I5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J5" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E6" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="F6" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="G6" t="s">
-        <v>72</v>
+        <v>101</v>
       </c>
       <c r="H6" t="s">
         <v>11</v>
@@ -1469,25 +1442,25 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B7" t="s">
         <v>75</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="D7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="F7" t="s">
-        <v>107</v>
+        <v>17</v>
       </c>
       <c r="G7" t="s">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="H7" t="s">
         <v>11</v>
@@ -1503,25 +1476,25 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B8" t="s">
         <v>75</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="D8" t="s">
         <v>9</v>
       </c>
       <c r="E8" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="F8" t="s">
-        <v>110</v>
+        <v>24</v>
       </c>
       <c r="G8" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="H8" t="s">
         <v>11</v>
@@ -1532,52 +1505,52 @@
       </c>
       <c r="J8" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B9" t="s">
         <v>75</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="D9" t="s">
         <v>12</v>
       </c>
       <c r="E9" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>105</v>
       </c>
       <c r="G9" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="H9" t="s">
         <v>11</v>
       </c>
       <c r="I9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J9" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gobernador</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B10" t="s">
         <v>75</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="D10" t="s">
         <v>12</v>
@@ -1589,10 +1562,10 @@
         <v>10</v>
       </c>
       <c r="G10" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="H10" t="s">
-        <v>78</v>
+        <v>11</v>
       </c>
       <c r="I10" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -1605,13 +1578,13 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B11" t="s">
         <v>75</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
         <v>12</v>
@@ -1623,7 +1596,7 @@
         <v>10</v>
       </c>
       <c r="G11" t="s">
-        <v>116</v>
+        <v>72</v>
       </c>
       <c r="H11" t="s">
         <v>11</v>
@@ -1639,13 +1612,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B12" t="s">
         <v>74</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
         <v>12</v>
@@ -1657,10 +1630,10 @@
         <v>10</v>
       </c>
       <c r="G12" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="H12" t="s">
-        <v>78</v>
+        <v>11</v>
       </c>
       <c r="I12" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -1673,13 +1646,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B13" t="s">
         <v>74</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
         <v>12</v>
@@ -1705,163 +1678,163 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A14" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B14" t="s">
         <v>74</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="D14" t="s">
         <v>13</v>
       </c>
       <c r="E14" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="F14" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="G14" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="H14" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="I14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J14" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="D15" t="s">
         <v>12</v>
       </c>
       <c r="E15" t="s">
-        <v>10</v>
+        <v>87</v>
       </c>
       <c r="F15" t="s">
-        <v>10</v>
+        <v>88</v>
       </c>
       <c r="G15" t="s">
-        <v>122</v>
+        <v>89</v>
       </c>
       <c r="H15" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="I15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J15" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B16" t="s">
         <v>74</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D16" t="s">
         <v>9</v>
       </c>
       <c r="E16" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G16" t="s">
-        <v>124</v>
+        <v>95</v>
       </c>
       <c r="H16" t="s">
-        <v>78</v>
+        <v>11</v>
       </c>
       <c r="I16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J16" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A17" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B17" t="s">
         <v>74</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="D17" t="s">
         <v>12</v>
       </c>
       <c r="E17" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="F17" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="G17" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="H17" t="s">
         <v>11</v>
       </c>
       <c r="I17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J17" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A18" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B18" t="s">
         <v>74</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="D18" t="s">
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="F18" t="s">
-        <v>26</v>
+        <v>119</v>
       </c>
       <c r="G18" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="H18" t="s">
         <v>78</v>
@@ -1875,102 +1848,102 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B19" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D19" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E19" t="s">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="F19" t="s">
-        <v>130</v>
+        <v>22</v>
       </c>
       <c r="G19" t="s">
-        <v>131</v>
+        <v>90</v>
       </c>
       <c r="H19" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="I19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Presidencia de la República</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J19" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B20" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="D20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F20" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="G20" t="s">
-        <v>133</v>
+        <v>86</v>
       </c>
       <c r="H20" t="s">
         <v>11</v>
       </c>
       <c r="I20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J20" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B21" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="D21" t="s">
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F21" t="s">
-        <v>135</v>
+        <v>10</v>
       </c>
       <c r="G21" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="H21" t="s">
         <v>11</v>
       </c>
       <c r="I21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J21" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
@@ -1979,28 +1952,28 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B22" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="D22" t="s">
         <v>9</v>
       </c>
       <c r="E22" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F22" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G22" t="s">
-        <v>137</v>
+        <v>95</v>
       </c>
       <c r="H22" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="I22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2008,132 +1981,132 @@
       </c>
       <c r="J22" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B23" t="s">
         <v>70</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="D23" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E23" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" t="s">
+        <v>95</v>
+      </c>
+      <c r="H23" t="s">
+        <v>127</v>
+      </c>
+      <c r="I23" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J23" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A24" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B24" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>16</v>
+      </c>
+      <c r="F24" t="s">
+        <v>16</v>
+      </c>
+      <c r="G24" t="s">
+        <v>129</v>
+      </c>
+      <c r="H24" t="s">
+        <v>11</v>
+      </c>
+      <c r="I24" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J24" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B25" t="s">
+        <v>70</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
         <v>14</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F25" t="s">
         <v>14</v>
       </c>
-      <c r="G23" t="s">
-        <v>139</v>
-      </c>
-      <c r="H23" t="s">
-        <v>78</v>
-      </c>
-      <c r="I23" t="str">
+      <c r="G25" t="s">
+        <v>86</v>
+      </c>
+      <c r="H25" t="s">
+        <v>11</v>
+      </c>
+      <c r="I25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Presidencia de la República</v>
       </c>
-      <c r="J23" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A24" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B24" t="s">
-        <v>69</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="D24" t="s">
-        <v>13</v>
-      </c>
-      <c r="E24" t="s">
-        <v>17</v>
-      </c>
-      <c r="F24" t="s">
-        <v>17</v>
-      </c>
-      <c r="G24" t="s">
-        <v>120</v>
-      </c>
-      <c r="H24" t="s">
-        <v>68</v>
-      </c>
-      <c r="I24" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
-      <c r="J24" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B25" t="s">
-        <v>69</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="D25" t="s">
-        <v>12</v>
-      </c>
-      <c r="E25" t="s">
-        <v>23</v>
-      </c>
-      <c r="F25" t="s">
-        <v>23</v>
-      </c>
-      <c r="G25" t="s">
-        <v>133</v>
-      </c>
-      <c r="H25" t="s">
-        <v>11</v>
-      </c>
-      <c r="I25" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
-      </c>
       <c r="J25" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="75" x14ac:dyDescent="0.25">
       <c r="A26" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B26" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
       <c r="D26" t="s">
         <v>12</v>
       </c>
       <c r="E26" t="s">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="F26" t="s">
-        <v>143</v>
+        <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="H26" t="s">
         <v>11</v>
@@ -2147,30 +2120,30 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B27" t="s">
         <v>69</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="D27" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E27" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G27" t="s">
-        <v>146</v>
+        <v>95</v>
       </c>
       <c r="H27" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="I27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2178,67 +2151,67 @@
       </c>
       <c r="J27" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B28" t="s">
+        <v>69</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D28" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" t="s">
+        <v>19</v>
+      </c>
+      <c r="G28" t="s">
+        <v>135</v>
+      </c>
+      <c r="H28" t="s">
+        <v>11</v>
+      </c>
+      <c r="I28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J28" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A28" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B28" t="s">
-        <v>83</v>
-      </c>
-      <c r="C28" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="D28" t="s">
-        <v>13</v>
-      </c>
-      <c r="E28" t="s">
-        <v>10</v>
-      </c>
-      <c r="F28" t="s">
-        <v>10</v>
-      </c>
-      <c r="G28" t="s">
-        <v>148</v>
-      </c>
-      <c r="H28" t="s">
-        <v>78</v>
-      </c>
-      <c r="I28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
-      <c r="J28" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
       </c>
     </row>
     <row r="29" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B29" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="D29" t="s">
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="F29" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G29" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="H29" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="I29" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2251,66 +2224,66 @@
     </row>
     <row r="30" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B30" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="D30" t="s">
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="F30" t="s">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="G30" t="s">
-        <v>79</v>
+        <v>139</v>
       </c>
       <c r="H30" t="s">
         <v>11</v>
       </c>
       <c r="I30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J30" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gabinete</v>
       </c>
     </row>
     <row r="31" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>152</v>
+        <v>140</v>
       </c>
       <c r="D31" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E31" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F31" t="s">
-        <v>153</v>
+        <v>10</v>
       </c>
       <c r="G31" t="s">
-        <v>154</v>
+        <v>93</v>
       </c>
       <c r="H31" t="s">
         <v>11</v>
       </c>
       <c r="I31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Presidencia de la República</v>
+        <v>Otros</v>
       </c>
       <c r="J31" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
@@ -2319,25 +2292,25 @@
     </row>
     <row r="32" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="D32" t="s">
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F32" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G32" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="H32" t="s">
         <v>11</v>
@@ -2348,98 +2321,98 @@
       </c>
       <c r="J32" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="33" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>156</v>
+        <v>143</v>
       </c>
       <c r="D33" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F33" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="G33" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="H33" t="s">
         <v>11</v>
       </c>
       <c r="I33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J33" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>157</v>
+        <v>145</v>
       </c>
       <c r="D34" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="F34" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="G34" t="s">
-        <v>108</v>
+        <v>146</v>
       </c>
       <c r="H34" t="s">
         <v>11</v>
       </c>
       <c r="I34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J34" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B35" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>158</v>
+        <v>147</v>
       </c>
       <c r="D35" t="s">
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="F35" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="G35" t="s">
-        <v>92</v>
+        <v>148</v>
       </c>
       <c r="H35" t="s">
         <v>11</v>
@@ -2455,25 +2428,25 @@
     </row>
     <row r="36" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A36" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B36" t="s">
         <v>73</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="D36" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E36" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F36" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G36" t="s">
-        <v>160</v>
+        <v>95</v>
       </c>
       <c r="H36" t="s">
         <v>11</v>
@@ -2484,101 +2457,101 @@
       </c>
       <c r="J36" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B37" t="s">
         <v>73</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>161</v>
+        <v>150</v>
       </c>
       <c r="D37" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E37" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="F37" t="s">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="G37" t="s">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H37" t="s">
         <v>11</v>
       </c>
       <c r="I37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Otros</v>
       </c>
       <c r="J37" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B38" t="s">
         <v>73</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="D38" t="s">
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F38" t="s">
-        <v>17</v>
+        <v>152</v>
       </c>
       <c r="G38" t="s">
-        <v>120</v>
+        <v>153</v>
       </c>
       <c r="H38" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="I38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J38" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="39" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A39" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B39" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
       <c r="D39" t="s">
-        <v>81</v>
+        <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="F39" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G39" t="s">
-        <v>90</v>
+        <v>155</v>
       </c>
       <c r="H39" t="s">
-        <v>11</v>
+        <v>78</v>
       </c>
       <c r="I39" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2589,64 +2562,64 @@
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B40" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D40" t="s">
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="F40" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="G40" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="H40" t="s">
         <v>11</v>
       </c>
       <c r="I40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
+        <v>Gobierno del estado</v>
       </c>
       <c r="J40" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B41" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D41" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="F41" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="G41" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="H41" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="I41" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2659,28 +2632,28 @@
     </row>
     <row r="42" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B42" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
       <c r="D42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E42" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="F42" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="G42" t="s">
-        <v>169</v>
+        <v>95</v>
       </c>
       <c r="H42" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="I42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -2688,370 +2661,370 @@
       </c>
       <c r="J42" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="43" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A43" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B43" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="C43" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="D43" t="s">
+        <v>12</v>
+      </c>
+      <c r="E43" t="s">
+        <v>24</v>
+      </c>
+      <c r="F43" t="s">
+        <v>24</v>
+      </c>
+      <c r="G43" t="s">
+        <v>162</v>
+      </c>
+      <c r="H43" t="s">
+        <v>11</v>
+      </c>
+      <c r="I43" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J43" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A44" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B44" t="s">
+        <v>83</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D44" t="s">
+        <v>12</v>
+      </c>
+      <c r="E44" t="s">
+        <v>10</v>
+      </c>
+      <c r="F44" t="s">
+        <v>10</v>
+      </c>
+      <c r="G44" t="s">
+        <v>108</v>
+      </c>
+      <c r="H44" t="s">
+        <v>11</v>
+      </c>
+      <c r="I44" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J44" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B45" t="s">
+        <v>83</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="D45" t="s">
+        <v>12</v>
+      </c>
+      <c r="E45" t="s">
+        <v>26</v>
+      </c>
+      <c r="F45" t="s">
+        <v>2</v>
+      </c>
+      <c r="G45" t="s">
+        <v>148</v>
+      </c>
+      <c r="H45" t="s">
+        <v>11</v>
+      </c>
+      <c r="I45" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J45" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A46" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B46" t="s">
+        <v>83</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>165</v>
+      </c>
+      <c r="D46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E46" t="s">
+        <v>29</v>
+      </c>
+      <c r="F46" t="s">
+        <v>166</v>
+      </c>
+      <c r="G46" t="s">
+        <v>167</v>
+      </c>
+      <c r="H46" t="s">
+        <v>11</v>
+      </c>
+      <c r="I46" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J46" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A47" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B47" t="s">
+        <v>83</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="D47" t="s">
+        <v>84</v>
+      </c>
+      <c r="E47" t="s">
+        <v>23</v>
+      </c>
+      <c r="F47" t="s">
+        <v>169</v>
+      </c>
+      <c r="G47" t="s">
+        <v>91</v>
+      </c>
+      <c r="H47" t="s">
+        <v>11</v>
+      </c>
+      <c r="I47" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J47" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gabinete</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A48" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B48" t="s">
+        <v>83</v>
+      </c>
+      <c r="C48" s="5" t="s">
         <v>170</v>
       </c>
-      <c r="D43" t="s">
-        <v>12</v>
-      </c>
-      <c r="E43" t="s">
+      <c r="D48" t="s">
+        <v>84</v>
+      </c>
+      <c r="E48" t="s">
         <v>16</v>
       </c>
-      <c r="F43" t="s">
-        <v>80</v>
-      </c>
-      <c r="G43" t="s">
+      <c r="F48" t="s">
+        <v>16</v>
+      </c>
+      <c r="G48" t="s">
+        <v>85</v>
+      </c>
+      <c r="H48" t="s">
+        <v>11</v>
+      </c>
+      <c r="I48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Alcaldías</v>
+      </c>
+      <c r="J48" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A49" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B49" t="s">
+        <v>77</v>
+      </c>
+      <c r="C49" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="H43" t="s">
-        <v>11</v>
-      </c>
-      <c r="I43" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J43" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A44" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B44" t="s">
-        <v>76</v>
-      </c>
-      <c r="C44" s="5" t="s">
+      <c r="D49" t="s">
+        <v>13</v>
+      </c>
+      <c r="E49" t="s">
+        <v>33</v>
+      </c>
+      <c r="F49" t="s">
+        <v>33</v>
+      </c>
+      <c r="G49" t="s">
+        <v>101</v>
+      </c>
+      <c r="H49" t="s">
+        <v>11</v>
+      </c>
+      <c r="I49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J49" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A50" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B50" t="s">
+        <v>77</v>
+      </c>
+      <c r="C50" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="D44" t="s">
-        <v>12</v>
-      </c>
-      <c r="E44" t="s">
-        <v>53</v>
-      </c>
-      <c r="F44" t="s">
-        <v>2</v>
-      </c>
-      <c r="G44" t="s">
-        <v>173</v>
-      </c>
-      <c r="H44" t="s">
-        <v>11</v>
-      </c>
-      <c r="I44" t="str">
+      <c r="D50" t="s">
+        <v>12</v>
+      </c>
+      <c r="E50" t="s">
+        <v>24</v>
+      </c>
+      <c r="F50" t="s">
+        <v>24</v>
+      </c>
+      <c r="G50" t="s">
+        <v>95</v>
+      </c>
+      <c r="H50" t="s">
+        <v>68</v>
+      </c>
+      <c r="I50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J44" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B45" t="s">
-        <v>76</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="D45" t="s">
-        <v>12</v>
-      </c>
-      <c r="E45" t="s">
-        <v>16</v>
-      </c>
-      <c r="F45" t="s">
-        <v>16</v>
-      </c>
-      <c r="G45" t="s">
-        <v>175</v>
-      </c>
-      <c r="H45" t="s">
-        <v>11</v>
-      </c>
-      <c r="I45" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J45" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A46" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B46" t="s">
-        <v>76</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="D46" t="s">
-        <v>12</v>
-      </c>
-      <c r="E46" t="s">
-        <v>16</v>
-      </c>
-      <c r="F46" t="s">
-        <v>16</v>
-      </c>
-      <c r="G46" t="s">
-        <v>177</v>
-      </c>
-      <c r="H46" t="s">
-        <v>11</v>
-      </c>
-      <c r="I46" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J46" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B47" t="s">
-        <v>76</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="D47" t="s">
-        <v>12</v>
-      </c>
-      <c r="E47" t="s">
-        <v>10</v>
-      </c>
-      <c r="F47" t="s">
-        <v>10</v>
-      </c>
-      <c r="G47" t="s">
-        <v>79</v>
-      </c>
-      <c r="H47" t="s">
-        <v>11</v>
-      </c>
-      <c r="I47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
-      <c r="J47" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B48" t="s">
-        <v>76</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="D48" t="s">
-        <v>12</v>
-      </c>
-      <c r="E48" t="s">
-        <v>14</v>
-      </c>
-      <c r="F48" t="s">
-        <v>180</v>
-      </c>
-      <c r="G48" t="s">
-        <v>181</v>
-      </c>
-      <c r="H48" t="s">
-        <v>11</v>
-      </c>
-      <c r="I48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Presidencia de la República</v>
-      </c>
-      <c r="J48" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A49" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B49" t="s">
-        <v>76</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="D49" t="s">
-        <v>12</v>
-      </c>
-      <c r="E49" t="s">
-        <v>16</v>
-      </c>
-      <c r="F49" t="s">
-        <v>16</v>
-      </c>
-      <c r="G49" t="s">
-        <v>183</v>
-      </c>
-      <c r="H49" t="s">
-        <v>11</v>
-      </c>
-      <c r="I49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
-      </c>
-      <c r="J49" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B50" t="s">
-        <v>76</v>
-      </c>
-      <c r="C50" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="D50" t="s">
-        <v>85</v>
-      </c>
-      <c r="E50" t="s">
-        <v>10</v>
-      </c>
-      <c r="F50" t="s">
-        <v>10</v>
-      </c>
-      <c r="G50" t="s">
-        <v>184</v>
-      </c>
-      <c r="H50" t="s">
-        <v>11</v>
-      </c>
-      <c r="I50" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
       <c r="J50" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="51" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A51" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B51" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="D51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="F51" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="G51" t="s">
-        <v>108</v>
+        <v>86</v>
       </c>
       <c r="H51" t="s">
         <v>11</v>
       </c>
       <c r="I51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Presidencia de la República</v>
       </c>
       <c r="J51" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Otros</v>
       </c>
     </row>
     <row r="52" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A52" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B52" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="D52" t="s">
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="F52" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G52" t="s">
-        <v>165</v>
+        <v>86</v>
       </c>
       <c r="H52" t="s">
         <v>11</v>
       </c>
       <c r="I52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Alcaldías</v>
+        <v>Otros</v>
       </c>
       <c r="J52" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
         <v>Otros</v>
       </c>
     </row>
-    <row r="53" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B53" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="D53" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E53" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F53" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G53" t="s">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="H53" t="s">
         <v>68</v>
@@ -3062,30 +3035,30 @@
       </c>
       <c r="J53" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="54" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A54" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B54" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="D54" t="s">
-        <v>12</v>
+        <v>81</v>
       </c>
       <c r="E54" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="F54" t="s">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="G54" t="s">
-        <v>169</v>
+        <v>92</v>
       </c>
       <c r="H54" t="s">
         <v>11</v>
@@ -3096,30 +3069,30 @@
       </c>
       <c r="J54" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
+        <v>Gobernador</v>
       </c>
     </row>
     <row r="55" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A55" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B55" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>189</v>
+        <v>177</v>
       </c>
       <c r="D55" t="s">
         <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F55" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G55" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
       <c r="H55" t="s">
         <v>11</v>
@@ -3130,55 +3103,55 @@
       </c>
       <c r="J55" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A56" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B56" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>190</v>
+        <v>179</v>
       </c>
       <c r="D56" t="s">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>35</v>
+        <v>16</v>
       </c>
       <c r="F56" t="s">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="G56" t="s">
-        <v>169</v>
+        <v>180</v>
       </c>
       <c r="H56" t="s">
         <v>11</v>
       </c>
       <c r="I56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Gobierno del estado</v>
+        <v>Alcaldías</v>
       </c>
       <c r="J56" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B57" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C57" s="5" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D57" t="s">
-        <v>85</v>
+        <v>12</v>
       </c>
       <c r="E57" t="s">
         <v>16</v>
@@ -3187,10 +3160,10 @@
         <v>16</v>
       </c>
       <c r="G57" t="s">
-        <v>86</v>
+        <v>182</v>
       </c>
       <c r="H57" t="s">
-        <v>11</v>
+        <v>183</v>
       </c>
       <c r="I57" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -3201,30 +3174,30 @@
         <v>Otros</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" ht="45" x14ac:dyDescent="0.25">
       <c r="A58" s="11">
-        <v>46211</v>
+        <v>46212</v>
       </c>
       <c r="B58" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C58" s="5" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="D58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="F58" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="G58" t="s">
-        <v>120</v>
+        <v>142</v>
       </c>
       <c r="H58" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="I58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
@@ -3232,177 +3205,143 @@
       </c>
       <c r="J58" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Gobernador</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A59" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B59" t="s">
+        <v>76</v>
+      </c>
+      <c r="C59" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="D59" t="s">
+        <v>12</v>
+      </c>
+      <c r="E59" t="s">
+        <v>59</v>
+      </c>
+      <c r="F59" t="s">
+        <v>59</v>
+      </c>
+      <c r="G59" t="s">
+        <v>186</v>
+      </c>
+      <c r="H59" t="s">
+        <v>11</v>
+      </c>
+      <c r="I59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Otros</v>
+      </c>
+      <c r="J59" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
+        <v>Otros</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A60" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B60" t="s">
+        <v>76</v>
+      </c>
+      <c r="C60" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="D60" t="s">
+        <v>12</v>
+      </c>
+      <c r="E60" t="s">
+        <v>34</v>
+      </c>
+      <c r="F60" t="s">
+        <v>34</v>
+      </c>
+      <c r="G60" t="s">
+        <v>188</v>
+      </c>
+      <c r="H60" t="s">
+        <v>11</v>
+      </c>
+      <c r="I60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
+        <v>Gobierno del estado</v>
+      </c>
+      <c r="J60" t="str">
+        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
         <v>Gabinete</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B59" t="s">
-        <v>77</v>
-      </c>
-      <c r="C59" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="D59" t="s">
-        <v>12</v>
-      </c>
-      <c r="E59" t="s">
-        <v>10</v>
-      </c>
-      <c r="F59" t="s">
-        <v>10</v>
-      </c>
-      <c r="G59" t="s">
-        <v>72</v>
-      </c>
-      <c r="H59" t="s">
-        <v>11</v>
-      </c>
-      <c r="I59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
-        <v>Otros</v>
-      </c>
-      <c r="J59" t="str">
-        <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
-        <v>Otros</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" ht="45" x14ac:dyDescent="0.25">
-      <c r="A60" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B60" t="s">
-        <v>77</v>
-      </c>
-      <c r="C60" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="D60" t="s">
-        <v>82</v>
-      </c>
-      <c r="E60" t="s">
-        <v>95</v>
-      </c>
-      <c r="F60" t="s">
-        <v>95</v>
-      </c>
-      <c r="G60" t="s">
-        <v>195</v>
-      </c>
-      <c r="H60" t="s">
-        <v>78</v>
-      </c>
-      <c r="I60" t="str">
+    <row r="61" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="A61" s="11">
+        <v>46212</v>
+      </c>
+      <c r="B61" t="s">
+        <v>76</v>
+      </c>
+      <c r="C61" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="D61" t="s">
+        <v>12</v>
+      </c>
+      <c r="E61" t="s">
+        <v>23</v>
+      </c>
+      <c r="F61" t="s">
+        <v>2</v>
+      </c>
+      <c r="G61" t="s">
+        <v>92</v>
+      </c>
+      <c r="H61" t="s">
+        <v>11</v>
+      </c>
+      <c r="I61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla2[Dependencia],Tabla2[Clasificación],"XXX",0)</f>
         <v>Gobierno del estado</v>
       </c>
-      <c r="J60" t="str">
+      <c r="J61" t="str">
         <f>_xlfn.XLOOKUP(Tabla1[[#This Row],[Dependencia]],Tabla3[Dependencia],Tabla3[Nivel],"Otros",0)</f>
         <v>Gabinete</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" ht="30" x14ac:dyDescent="0.25">
-      <c r="A61" s="11">
-        <v>46211</v>
-      </c>
-      <c r="B61" t="s">
-        <v>77</v>
-      </c>
-      <c r="C61" s="5" t="s">
-        <v>